<commit_message>
Atualização automática: devolucoes (10/07/2026 18:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -25105,18 +25105,62 @@
           <t>326</t>
         </is>
       </c>
-      <c r="B326" t="inlineStr"/>
-      <c r="C326" t="inlineStr"/>
-      <c r="D326" t="inlineStr"/>
-      <c r="E326" t="inlineStr"/>
-      <c r="F326" t="inlineStr"/>
+      <c r="B326" t="inlineStr">
+        <is>
+          <t>S3326-2RX</t>
+        </is>
+      </c>
+      <c r="C326" t="inlineStr">
+        <is>
+          <t>INDICATOR, GYRO-HORIZON</t>
+        </is>
+      </c>
+      <c r="D326" t="inlineStr">
+        <is>
+          <t>T94079Q</t>
+        </is>
+      </c>
+      <c r="E326" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F326" t="inlineStr">
+        <is>
+          <t>01 EA</t>
+        </is>
+      </c>
       <c r="G326" t="inlineStr"/>
-      <c r="H326" t="inlineStr"/>
-      <c r="I326" t="inlineStr"/>
-      <c r="J326" t="inlineStr"/>
-      <c r="K326" t="inlineStr"/>
-      <c r="L326" t="inlineStr"/>
-      <c r="M326" t="inlineStr"/>
+      <c r="H326" t="inlineStr">
+        <is>
+          <t>17880693</t>
+        </is>
+      </c>
+      <c r="I326" t="inlineStr">
+        <is>
+          <t>Atender necessidade informada pelo 2S Gabriel em 03/07/26.</t>
+        </is>
+      </c>
+      <c r="J326" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="K326" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="L326" t="inlineStr">
+        <is>
+          <t>2743</t>
+        </is>
+      </c>
+      <c r="M326" t="inlineStr">
+        <is>
+          <t>BACO</t>
+        </is>
+      </c>
       <c r="N326" t="inlineStr"/>
       <c r="O326" t="inlineStr"/>
       <c r="P326" t="inlineStr"/>
@@ -25138,18 +25182,62 @@
           <t>327</t>
         </is>
       </c>
-      <c r="B327" t="inlineStr"/>
-      <c r="C327" t="inlineStr"/>
-      <c r="D327" t="inlineStr"/>
-      <c r="E327" t="inlineStr"/>
-      <c r="F327" t="inlineStr"/>
+      <c r="B327" t="inlineStr">
+        <is>
+          <t>799-1</t>
+        </is>
+      </c>
+      <c r="C327" t="inlineStr">
+        <is>
+          <t>TRANSDUCER</t>
+        </is>
+      </c>
+      <c r="D327" t="inlineStr">
+        <is>
+          <t>207572-10</t>
+        </is>
+      </c>
+      <c r="E327" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F327" t="inlineStr">
+        <is>
+          <t>01 EA</t>
+        </is>
+      </c>
       <c r="G327" t="inlineStr"/>
-      <c r="H327" t="inlineStr"/>
-      <c r="I327" t="inlineStr"/>
-      <c r="J327" t="inlineStr"/>
-      <c r="K327" t="inlineStr"/>
-      <c r="L327" t="inlineStr"/>
-      <c r="M327" t="inlineStr"/>
+      <c r="H327" t="inlineStr">
+        <is>
+          <t>17647315</t>
+        </is>
+      </c>
+      <c r="I327" t="inlineStr">
+        <is>
+          <t>Atender necessidade informada pelo 2S Gabriel em 03/07/26.</t>
+        </is>
+      </c>
+      <c r="J327" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="K327" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="L327" t="inlineStr">
+        <is>
+          <t>2743</t>
+        </is>
+      </c>
+      <c r="M327" t="inlineStr">
+        <is>
+          <t>BACO</t>
+        </is>
+      </c>
       <c r="N327" t="inlineStr"/>
       <c r="O327" t="inlineStr"/>
       <c r="P327" t="inlineStr"/>
@@ -25171,18 +25259,58 @@
           <t>328</t>
         </is>
       </c>
-      <c r="B328" t="inlineStr"/>
-      <c r="C328" t="inlineStr"/>
-      <c r="D328" t="inlineStr"/>
-      <c r="E328" t="inlineStr"/>
-      <c r="F328" t="inlineStr"/>
+      <c r="B328" t="inlineStr">
+        <is>
+          <t>060-0017-00</t>
+        </is>
+      </c>
+      <c r="C328" t="inlineStr">
+        <is>
+          <t>IND DE COMANDO DE VOO</t>
+        </is>
+      </c>
+      <c r="D328" t="inlineStr">
+        <is>
+          <t>19796</t>
+        </is>
+      </c>
+      <c r="E328" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F328" t="inlineStr">
+        <is>
+          <t>01 EA</t>
+        </is>
+      </c>
       <c r="G328" t="inlineStr"/>
       <c r="H328" t="inlineStr"/>
-      <c r="I328" t="inlineStr"/>
-      <c r="J328" t="inlineStr"/>
-      <c r="K328" t="inlineStr"/>
-      <c r="L328" t="inlineStr"/>
-      <c r="M328" t="inlineStr"/>
+      <c r="I328" t="inlineStr">
+        <is>
+          <t>Atender demanda do 2703 e 2708 da BABE para a BANT</t>
+        </is>
+      </c>
+      <c r="J328" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="K328" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="L328" t="inlineStr">
+        <is>
+          <t>2703</t>
+        </is>
+      </c>
+      <c r="M328" t="inlineStr">
+        <is>
+          <t>BANT</t>
+        </is>
+      </c>
       <c r="N328" t="inlineStr"/>
       <c r="O328" t="inlineStr"/>
       <c r="P328" t="inlineStr"/>
@@ -25204,18 +25332,58 @@
           <t>329</t>
         </is>
       </c>
-      <c r="B329" t="inlineStr"/>
-      <c r="C329" t="inlineStr"/>
-      <c r="D329" t="inlineStr"/>
-      <c r="E329" t="inlineStr"/>
-      <c r="F329" t="inlineStr"/>
+      <c r="B329" t="inlineStr">
+        <is>
+          <t>060-0017-00</t>
+        </is>
+      </c>
+      <c r="C329" t="inlineStr">
+        <is>
+          <t>IND DE COMANDO DE VOO</t>
+        </is>
+      </c>
+      <c r="D329" t="inlineStr">
+        <is>
+          <t>R17062</t>
+        </is>
+      </c>
+      <c r="E329" t="inlineStr">
+        <is>
+          <t>R</t>
+        </is>
+      </c>
+      <c r="F329" t="inlineStr">
+        <is>
+          <t>01 EA</t>
+        </is>
+      </c>
       <c r="G329" t="inlineStr"/>
       <c r="H329" t="inlineStr"/>
-      <c r="I329" t="inlineStr"/>
-      <c r="J329" t="inlineStr"/>
-      <c r="K329" t="inlineStr"/>
-      <c r="L329" t="inlineStr"/>
-      <c r="M329" t="inlineStr"/>
+      <c r="I329" t="inlineStr">
+        <is>
+          <t>Atender demanda do 2703 e 2708 da BABE para a BANT</t>
+        </is>
+      </c>
+      <c r="J329" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="K329" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="L329" t="inlineStr">
+        <is>
+          <t>2708</t>
+        </is>
+      </c>
+      <c r="M329" t="inlineStr">
+        <is>
+          <t>BANT</t>
+        </is>
+      </c>
       <c r="N329" t="inlineStr"/>
       <c r="O329" t="inlineStr"/>
       <c r="P329" t="inlineStr"/>
@@ -25237,18 +25405,58 @@
           <t>330</t>
         </is>
       </c>
-      <c r="B330" t="inlineStr"/>
-      <c r="C330" t="inlineStr"/>
+      <c r="B330" t="inlineStr">
+        <is>
+          <t>4002HS</t>
+        </is>
+      </c>
+      <c r="C330" t="inlineStr">
+        <is>
+          <t>EYELET,TURNLOCK FASTENER</t>
+        </is>
+      </c>
       <c r="D330" t="inlineStr"/>
-      <c r="E330" t="inlineStr"/>
-      <c r="F330" t="inlineStr"/>
+      <c r="E330" t="inlineStr">
+        <is>
+          <t>C</t>
+        </is>
+      </c>
+      <c r="F330" t="inlineStr">
+        <is>
+          <t>10 EA</t>
+        </is>
+      </c>
       <c r="G330" t="inlineStr"/>
-      <c r="H330" t="inlineStr"/>
-      <c r="I330" t="inlineStr"/>
-      <c r="J330" t="inlineStr"/>
-      <c r="K330" t="inlineStr"/>
-      <c r="L330" t="inlineStr"/>
-      <c r="M330" t="inlineStr"/>
+      <c r="H330" t="inlineStr">
+        <is>
+          <t>17926773</t>
+        </is>
+      </c>
+      <c r="I330" t="inlineStr">
+        <is>
+          <t>Atender demanda do C-98 solicitada pelo CP Souto e acordada pelo SO Cláduio no grupo do Whats App</t>
+        </is>
+      </c>
+      <c r="J330" t="inlineStr">
+        <is>
+          <t>U8</t>
+        </is>
+      </c>
+      <c r="K330" t="inlineStr">
+        <is>
+          <t>10/07/2026</t>
+        </is>
+      </c>
+      <c r="L330" t="inlineStr">
+        <is>
+          <t>2709</t>
+        </is>
+      </c>
+      <c r="M330" t="inlineStr">
+        <is>
+          <t>BABR</t>
+        </is>
+      </c>
       <c r="N330" t="inlineStr"/>
       <c r="O330" t="inlineStr"/>
       <c r="P330" t="inlineStr"/>

</xml_diff>

<commit_message>
Atualização automática: devolucoes (10/07/2026 22:40)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,117 +421,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_ordem</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>part_number</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>sn_lt</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>quantidade_texto</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>pedido_emg</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>motivo</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>pj</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>pedido_envio</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>anv</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>destino</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>nf_gmm</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>rastreio</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>pn_devolvido</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>detalhe_entrega</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>numero_rc</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>nf_devolucao_vee_one</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>data_devolucao</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>observacao_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>observacao_empresa</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -598,7 +586,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>45730</v>
       </c>
       <c r="L2" t="inlineStr">
@@ -675,7 +663,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>45735</v>
       </c>
       <c r="L3" t="inlineStr">
@@ -752,7 +740,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>45737</v>
       </c>
       <c r="L4" t="inlineStr">
@@ -829,7 +817,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L5" t="inlineStr">
@@ -914,7 +902,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L6" t="inlineStr">
@@ -995,7 +983,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L7" t="inlineStr">
@@ -1076,7 +1064,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L8" t="inlineStr">
@@ -1157,7 +1145,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L9" t="inlineStr">
@@ -1238,7 +1226,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L10" t="inlineStr">
@@ -1319,7 +1307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L11" t="inlineStr">
@@ -1400,7 +1388,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L12" t="inlineStr">
@@ -1477,7 +1465,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>45762</v>
       </c>
       <c r="L13" t="inlineStr">
@@ -1554,7 +1542,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>45763</v>
       </c>
       <c r="L14" t="inlineStr">
@@ -1631,7 +1619,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>45763</v>
       </c>
       <c r="L15" t="inlineStr">
@@ -1708,7 +1696,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="1" t="n">
         <v>45783</v>
       </c>
       <c r="L16" t="inlineStr">
@@ -1785,7 +1773,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="K17" s="1" t="n">
         <v>45783</v>
       </c>
       <c r="L17" t="inlineStr">
@@ -1862,7 +1850,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="K18" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L18" t="inlineStr">
@@ -1893,7 +1881,7 @@
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" s="2" t="n">
+      <c r="T18" s="1" t="n">
         <v>45845</v>
       </c>
       <c r="U18" t="inlineStr">
@@ -1957,7 +1945,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="K19" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L19" t="inlineStr">
@@ -2034,7 +2022,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="K20" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L20" t="inlineStr">
@@ -2111,7 +2099,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K21" s="2" t="n">
+      <c r="K21" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L21" t="inlineStr">
@@ -2142,7 +2130,7 @@
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
-      <c r="T21" s="2" t="n">
+      <c r="T21" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="U21" t="inlineStr">
@@ -2206,7 +2194,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="K22" s="1" t="n">
         <v>45789</v>
       </c>
       <c r="L22" t="inlineStr">
@@ -2237,7 +2225,7 @@
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
-      <c r="T22" s="2" t="n">
+      <c r="T22" s="1" t="n">
         <v>45868</v>
       </c>
       <c r="U22" t="inlineStr">
@@ -2301,7 +2289,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K23" s="2" t="n">
+      <c r="K23" s="1" t="n">
         <v>45789</v>
       </c>
       <c r="L23" t="inlineStr">
@@ -2332,7 +2320,7 @@
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
-      <c r="T23" s="2" t="n">
+      <c r="T23" s="1" t="n">
         <v>45982</v>
       </c>
       <c r="U23" t="inlineStr">
@@ -2396,7 +2384,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="K24" s="1" t="n">
         <v>45791</v>
       </c>
       <c r="L24" t="inlineStr">
@@ -2473,7 +2461,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="K25" s="1" t="n">
         <v>45814</v>
       </c>
       <c r="L25" t="inlineStr">
@@ -2546,7 +2534,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="K26" s="1" t="n">
         <v>45819</v>
       </c>
       <c r="L26" t="inlineStr">
@@ -2619,7 +2607,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K27" s="2" t="n">
+      <c r="K27" s="1" t="n">
         <v>45821</v>
       </c>
       <c r="L27" t="inlineStr">
@@ -2650,7 +2638,7 @@
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" s="2" t="n">
+      <c r="T27" s="1" t="n">
         <v>45876</v>
       </c>
       <c r="U27" t="inlineStr">
@@ -2714,7 +2702,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="K28" s="1" t="n">
         <v>45824</v>
       </c>
       <c r="L28" t="inlineStr">
@@ -2791,7 +2779,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K29" s="2" t="n">
+      <c r="K29" s="1" t="n">
         <v>45825</v>
       </c>
       <c r="L29" t="inlineStr">
@@ -2868,7 +2856,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K30" s="2" t="n">
+      <c r="K30" s="1" t="n">
         <v>45836</v>
       </c>
       <c r="L30" t="inlineStr">
@@ -2945,7 +2933,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K31" s="2" t="n">
+      <c r="K31" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="L31" t="inlineStr">
@@ -2976,7 +2964,7 @@
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" s="2" t="n">
+      <c r="T31" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U31" t="inlineStr">
@@ -3040,7 +3028,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="K32" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="L32" t="inlineStr">
@@ -3117,7 +3105,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="K33" s="1" t="n">
         <v>45845</v>
       </c>
       <c r="L33" t="inlineStr">
@@ -3148,7 +3136,7 @@
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" s="2" t="n">
+      <c r="T33" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U33" t="inlineStr">
@@ -3212,7 +3200,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="K34" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L34" t="inlineStr">
@@ -3289,7 +3277,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="K35" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L35" t="inlineStr">
@@ -3320,7 +3308,7 @@
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
-      <c r="T35" s="2" t="n">
+      <c r="T35" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U35" t="inlineStr">
@@ -3384,7 +3372,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="K36" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L36" t="inlineStr">
@@ -3415,7 +3403,7 @@
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
-      <c r="T36" s="2" t="n">
+      <c r="T36" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U36" t="inlineStr">
@@ -3479,7 +3467,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K37" s="2" t="n">
+      <c r="K37" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L37" t="inlineStr">
@@ -3510,7 +3498,7 @@
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
-      <c r="T37" s="2" t="n">
+      <c r="T37" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U37" t="inlineStr">
@@ -3574,7 +3562,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K38" s="2" t="n">
+      <c r="K38" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L38" t="inlineStr">
@@ -3605,7 +3593,7 @@
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
-      <c r="T38" s="2" t="n">
+      <c r="T38" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U38" t="inlineStr">
@@ -3669,7 +3657,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K39" s="2" t="n">
+      <c r="K39" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L39" t="inlineStr">
@@ -3700,7 +3688,7 @@
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
-      <c r="T39" s="2" t="n">
+      <c r="T39" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U39" t="inlineStr">
@@ -3764,7 +3752,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K40" s="2" t="n">
+      <c r="K40" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L40" t="inlineStr">
@@ -3795,7 +3783,7 @@
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
-      <c r="T40" s="2" t="n">
+      <c r="T40" s="1" t="n">
         <v>45916</v>
       </c>
       <c r="U40" t="inlineStr">
@@ -3859,7 +3847,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K41" s="2" t="n">
+      <c r="K41" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L41" t="inlineStr">
@@ -3936,7 +3924,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="K42" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L42" t="inlineStr">
@@ -3967,7 +3955,7 @@
         </is>
       </c>
       <c r="S42" t="inlineStr"/>
-      <c r="T42" s="2" t="n">
+      <c r="T42" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U42" t="inlineStr">
@@ -4031,7 +4019,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K43" s="2" t="n">
+      <c r="K43" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L43" t="inlineStr">
@@ -4108,7 +4096,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K44" s="2" t="n">
+      <c r="K44" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L44" t="inlineStr">
@@ -4139,7 +4127,7 @@
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
-      <c r="T44" s="2" t="n">
+      <c r="T44" s="1" t="n">
         <v>46002</v>
       </c>
       <c r="U44" t="inlineStr">
@@ -4203,7 +4191,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K45" s="2" t="n">
+      <c r="K45" s="1" t="n">
         <v>45882</v>
       </c>
       <c r="L45" t="inlineStr">
@@ -4280,7 +4268,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K46" s="2" t="n">
+      <c r="K46" s="1" t="n">
         <v>45882</v>
       </c>
       <c r="L46" t="inlineStr">
@@ -4357,7 +4345,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K47" s="2" t="n">
+      <c r="K47" s="1" t="n">
         <v>45890</v>
       </c>
       <c r="L47" t="inlineStr">
@@ -4388,7 +4376,7 @@
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
-      <c r="T47" s="2" t="n">
+      <c r="T47" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="U47" t="inlineStr">
@@ -4452,7 +4440,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="K48" s="1" t="n">
         <v>45903</v>
       </c>
       <c r="L48" t="inlineStr">
@@ -4529,7 +4517,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K49" s="2" t="n">
+      <c r="K49" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="L49" t="inlineStr">
@@ -4606,7 +4594,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K50" s="2" t="n">
+      <c r="K50" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="L50" t="inlineStr">
@@ -4683,7 +4671,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K51" s="2" t="n">
+      <c r="K51" s="1" t="n">
         <v>45925</v>
       </c>
       <c r="L51" t="inlineStr">
@@ -4764,7 +4752,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K52" s="2" t="n">
+      <c r="K52" s="1" t="n">
         <v>45924</v>
       </c>
       <c r="L52" t="inlineStr">
@@ -4841,7 +4829,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K53" s="2" t="n">
+      <c r="K53" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="L53" t="inlineStr">
@@ -4918,7 +4906,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K54" s="2" t="n">
+      <c r="K54" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="L54" t="inlineStr">
@@ -4995,7 +4983,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K55" s="2" t="n">
+      <c r="K55" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L55" t="inlineStr">
@@ -5080,7 +5068,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="K56" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L56" t="inlineStr">
@@ -5169,7 +5157,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K57" s="2" t="n">
+      <c r="K57" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L57" t="inlineStr">
@@ -5254,7 +5242,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K58" s="2" t="n">
+      <c r="K58" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L58" t="inlineStr">
@@ -5339,7 +5327,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="K59" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="L59" t="inlineStr">
@@ -5370,7 +5358,7 @@
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
-      <c r="T59" s="2" t="n">
+      <c r="T59" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="U59" t="inlineStr">
@@ -5434,7 +5422,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="K60" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="L60" t="inlineStr">
@@ -5511,7 +5499,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K61" s="2" t="n">
+      <c r="K61" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="L61" t="inlineStr">
@@ -5588,7 +5576,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K62" s="2" t="n">
+      <c r="K62" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="L62" t="inlineStr">
@@ -5665,7 +5653,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K63" s="2" t="n">
+      <c r="K63" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="L63" t="inlineStr">
@@ -5742,7 +5730,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K64" s="2" t="n">
+      <c r="K64" s="1" t="n">
         <v>45940</v>
       </c>
       <c r="L64" t="inlineStr">
@@ -5819,7 +5807,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K65" s="2" t="n">
+      <c r="K65" s="1" t="n">
         <v>45943</v>
       </c>
       <c r="L65" t="inlineStr">
@@ -5900,7 +5888,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K66" s="2" t="n">
+      <c r="K66" s="1" t="n">
         <v>45943</v>
       </c>
       <c r="L66" t="inlineStr">
@@ -5977,7 +5965,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K67" s="2" t="n">
+      <c r="K67" s="1" t="n">
         <v>45943</v>
       </c>
       <c r="L67" t="inlineStr">
@@ -6054,7 +6042,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K68" s="2" t="n">
+      <c r="K68" s="1" t="n">
         <v>45961</v>
       </c>
       <c r="L68" t="inlineStr">
@@ -6081,7 +6069,7 @@
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
-      <c r="T68" s="2" t="n">
+      <c r="T68" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U68" t="inlineStr">
@@ -6149,7 +6137,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K69" s="2" t="n">
+      <c r="K69" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="L69" t="inlineStr">
@@ -6226,7 +6214,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K70" s="2" t="n">
+      <c r="K70" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="L70" t="inlineStr">
@@ -6303,7 +6291,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K71" s="2" t="n">
+      <c r="K71" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="L71" t="inlineStr">
@@ -6380,7 +6368,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K72" s="2" t="n">
+      <c r="K72" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L72" t="inlineStr">
@@ -6457,7 +6445,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K73" s="2" t="n">
+      <c r="K73" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L73" t="inlineStr">
@@ -6534,7 +6522,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K74" s="2" t="n">
+      <c r="K74" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L74" t="inlineStr">
@@ -6611,7 +6599,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K75" s="2" t="n">
+      <c r="K75" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L75" t="inlineStr">
@@ -6688,7 +6676,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K76" s="2" t="n">
+      <c r="K76" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L76" t="inlineStr">
@@ -6765,7 +6753,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K77" s="2" t="n">
+      <c r="K77" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L77" t="inlineStr">
@@ -6842,7 +6830,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K78" s="2" t="n">
+      <c r="K78" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L78" t="inlineStr">
@@ -6919,7 +6907,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K79" s="2" t="n">
+      <c r="K79" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L79" t="inlineStr">
@@ -6996,7 +6984,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K80" s="2" t="n">
+      <c r="K80" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L80" t="inlineStr">
@@ -7073,7 +7061,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K81" s="2" t="n">
+      <c r="K81" s="1" t="n">
         <v>45973</v>
       </c>
       <c r="L81" t="inlineStr">
@@ -7150,7 +7138,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K82" s="2" t="n">
+      <c r="K82" s="1" t="n">
         <v>45974</v>
       </c>
       <c r="L82" t="inlineStr">
@@ -7227,7 +7215,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K83" s="2" t="n">
+      <c r="K83" s="1" t="n">
         <v>45975</v>
       </c>
       <c r="L83" t="inlineStr">
@@ -7304,7 +7292,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K84" s="2" t="n">
+      <c r="K84" s="1" t="n">
         <v>45975</v>
       </c>
       <c r="L84" t="inlineStr">
@@ -7381,7 +7369,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K85" s="2" t="n">
+      <c r="K85" s="1" t="n">
         <v>45982</v>
       </c>
       <c r="L85" t="inlineStr">
@@ -7458,7 +7446,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K86" s="2" t="n">
+      <c r="K86" s="1" t="n">
         <v>45982</v>
       </c>
       <c r="L86" t="inlineStr">
@@ -7535,7 +7523,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K87" s="2" t="n">
+      <c r="K87" s="1" t="n">
         <v>45985</v>
       </c>
       <c r="L87" t="inlineStr">
@@ -7612,7 +7600,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K88" s="2" t="n">
+      <c r="K88" s="1" t="n">
         <v>45985</v>
       </c>
       <c r="L88" t="inlineStr">
@@ -7689,7 +7677,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K89" s="2" t="n">
+      <c r="K89" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="L89" t="inlineStr">
@@ -7762,7 +7750,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K90" s="2" t="n">
+      <c r="K90" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="L90" t="inlineStr">
@@ -7835,7 +7823,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K91" s="2" t="n">
+      <c r="K91" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="L91" t="inlineStr">
@@ -7912,7 +7900,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K92" s="2" t="n">
+      <c r="K92" s="1" t="n">
         <v>45996</v>
       </c>
       <c r="L92" t="inlineStr">
@@ -7947,7 +7935,7 @@
         </is>
       </c>
       <c r="S92" t="inlineStr"/>
-      <c r="T92" s="2" t="n">
+      <c r="T92" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="U92" t="inlineStr">
@@ -8011,7 +7999,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K93" s="2" t="n">
+      <c r="K93" s="1" t="n">
         <v>46002</v>
       </c>
       <c r="L93" t="inlineStr">
@@ -8084,7 +8072,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K94" s="2" t="n">
+      <c r="K94" s="1" t="n">
         <v>46007</v>
       </c>
       <c r="L94" t="inlineStr">
@@ -8161,7 +8149,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K95" s="2" t="n">
+      <c r="K95" s="1" t="n">
         <v>46007</v>
       </c>
       <c r="L95" t="inlineStr">
@@ -8238,7 +8226,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K96" s="2" t="n">
+      <c r="K96" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="L96" t="inlineStr">
@@ -8319,7 +8307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K97" s="2" t="n">
+      <c r="K97" s="1" t="n">
         <v>46029</v>
       </c>
       <c r="L97" t="inlineStr">
@@ -8346,7 +8334,7 @@
         </is>
       </c>
       <c r="S97" t="inlineStr"/>
-      <c r="T97" s="2" t="n">
+      <c r="T97" s="1" t="n">
         <v>46030</v>
       </c>
       <c r="U97" t="inlineStr">
@@ -8410,7 +8398,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K98" s="2" t="n">
+      <c r="K98" s="1" t="n">
         <v>46029</v>
       </c>
       <c r="L98" t="inlineStr">
@@ -8487,7 +8475,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K99" s="2" t="n">
+      <c r="K99" s="1" t="n">
         <v>46034</v>
       </c>
       <c r="L99" t="inlineStr">
@@ -8564,7 +8552,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K100" s="2" t="n">
+      <c r="K100" s="1" t="n">
         <v>46034</v>
       </c>
       <c r="L100" t="inlineStr">
@@ -8637,7 +8625,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K101" s="2" t="n">
+      <c r="K101" s="1" t="n">
         <v>46035</v>
       </c>
       <c r="L101" t="inlineStr">
@@ -8710,7 +8698,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K102" s="2" t="n">
+      <c r="K102" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L102" t="inlineStr">
@@ -8783,7 +8771,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K103" s="2" t="n">
+      <c r="K103" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L103" t="inlineStr">
@@ -8856,7 +8844,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K104" s="2" t="n">
+      <c r="K104" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L104" t="inlineStr">
@@ -8929,7 +8917,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K105" s="2" t="n">
+      <c r="K105" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L105" t="inlineStr">
@@ -9002,7 +8990,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K106" s="2" t="n">
+      <c r="K106" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L106" t="inlineStr">
@@ -9075,7 +9063,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K107" s="2" t="n">
+      <c r="K107" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L107" t="inlineStr">
@@ -9148,7 +9136,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K108" s="2" t="n">
+      <c r="K108" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L108" t="inlineStr">
@@ -9221,7 +9209,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K109" s="2" t="n">
+      <c r="K109" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L109" t="inlineStr">
@@ -9294,7 +9282,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K110" s="2" t="n">
+      <c r="K110" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L110" t="inlineStr">
@@ -9325,7 +9313,7 @@
         </is>
       </c>
       <c r="S110" t="inlineStr"/>
-      <c r="T110" s="2" t="n">
+      <c r="T110" s="1" t="n">
         <v>45805</v>
       </c>
       <c r="U110" t="inlineStr">
@@ -9385,7 +9373,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K111" s="2" t="n">
+      <c r="K111" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L111" t="inlineStr">
@@ -9416,7 +9404,7 @@
         </is>
       </c>
       <c r="S111" t="inlineStr"/>
-      <c r="T111" s="2" t="n">
+      <c r="T111" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="U111" t="inlineStr">
@@ -9476,7 +9464,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K112" s="2" t="n">
+      <c r="K112" s="1" t="n">
         <v>46044</v>
       </c>
       <c r="L112" t="inlineStr">
@@ -9507,7 +9495,7 @@
         </is>
       </c>
       <c r="S112" t="inlineStr"/>
-      <c r="T112" s="2" t="n">
+      <c r="T112" s="1" t="n">
         <v>46052</v>
       </c>
       <c r="U112" t="inlineStr">
@@ -9571,7 +9559,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K113" s="2" t="n">
+      <c r="K113" s="1" t="n">
         <v>46049</v>
       </c>
       <c r="L113" t="inlineStr">
@@ -9648,7 +9636,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K114" s="2" t="n">
+      <c r="K114" s="1" t="n">
         <v>46049</v>
       </c>
       <c r="L114" t="inlineStr">
@@ -9725,7 +9713,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K115" s="2" t="n">
+      <c r="K115" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="L115" t="inlineStr">
@@ -9802,7 +9790,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K116" s="2" t="n">
+      <c r="K116" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="L116" t="inlineStr">
@@ -9833,7 +9821,7 @@
         </is>
       </c>
       <c r="S116" t="inlineStr"/>
-      <c r="T116" s="2" t="n">
+      <c r="T116" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="U116" t="inlineStr">
@@ -9897,7 +9885,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K117" s="2" t="n">
+      <c r="K117" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="L117" t="inlineStr">
@@ -9974,7 +9962,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K118" s="2" t="n">
+      <c r="K118" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="L118" t="inlineStr">
@@ -10055,7 +10043,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K119" s="2" t="n">
+      <c r="K119" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="L119" t="inlineStr">
@@ -10126,7 +10114,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K120" s="2" t="n">
+      <c r="K120" s="1" t="n">
         <v>46062</v>
       </c>
       <c r="L120" t="inlineStr">
@@ -10203,7 +10191,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K121" s="2" t="n">
+      <c r="K121" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L121" t="inlineStr">
@@ -10280,7 +10268,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K122" s="2" t="n">
+      <c r="K122" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L122" t="inlineStr">
@@ -10365,7 +10353,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K123" s="2" t="n">
+      <c r="K123" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L123" t="inlineStr">
@@ -10442,7 +10430,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K124" s="2" t="n">
+      <c r="K124" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L124" t="inlineStr">
@@ -10519,7 +10507,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K125" s="2" t="n">
+      <c r="K125" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="L125" t="inlineStr">
@@ -10592,7 +10580,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K126" s="2" t="n">
+      <c r="K126" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L126" t="inlineStr">
@@ -10665,7 +10653,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K127" s="2" t="n">
+      <c r="K127" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L127" t="inlineStr">
@@ -10696,7 +10684,7 @@
         </is>
       </c>
       <c r="S127" t="inlineStr"/>
-      <c r="T127" s="2" t="n">
+      <c r="T127" s="1" t="n">
         <v>45889</v>
       </c>
       <c r="U127" t="inlineStr">
@@ -10756,7 +10744,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K128" s="2" t="n">
+      <c r="K128" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L128" t="inlineStr">
@@ -10829,7 +10817,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K129" s="2" t="n">
+      <c r="K129" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L129" t="inlineStr">
@@ -10902,7 +10890,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K130" s="2" t="n">
+      <c r="K130" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L130" t="inlineStr">
@@ -10975,7 +10963,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K131" s="2" t="n">
+      <c r="K131" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L131" t="inlineStr">
@@ -11052,7 +11040,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K132" s="2" t="n">
+      <c r="K132" s="1" t="n">
         <v>46077</v>
       </c>
       <c r="L132" t="inlineStr">
@@ -11125,7 +11113,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K133" s="2" t="n">
+      <c r="K133" s="1" t="n">
         <v>46079</v>
       </c>
       <c r="L133" t="inlineStr">
@@ -11198,7 +11186,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K134" s="2" t="n">
+      <c r="K134" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L134" t="inlineStr">
@@ -11271,7 +11259,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K135" s="2" t="n">
+      <c r="K135" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L135" t="inlineStr">
@@ -11344,7 +11332,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K136" s="2" t="n">
+      <c r="K136" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L136" t="inlineStr">
@@ -11417,7 +11405,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K137" s="2" t="n">
+      <c r="K137" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L137" t="inlineStr">
@@ -11490,7 +11478,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K138" s="2" t="n">
+      <c r="K138" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L138" t="inlineStr">
@@ -11563,7 +11551,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K139" s="2" t="n">
+      <c r="K139" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="L139" t="inlineStr">
@@ -11644,7 +11632,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K140" s="2" t="n">
+      <c r="K140" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L140" t="inlineStr">
@@ -11717,7 +11705,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K141" s="2" t="n">
+      <c r="K141" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L141" t="inlineStr">
@@ -11790,7 +11778,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K142" s="2" t="n">
+      <c r="K142" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L142" t="inlineStr">
@@ -11867,7 +11855,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K143" s="2" t="n">
+      <c r="K143" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L143" t="inlineStr">
@@ -11940,7 +11928,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K144" s="2" t="n">
+      <c r="K144" s="1" t="n">
         <v>46090</v>
       </c>
       <c r="L144" t="inlineStr">
@@ -12013,7 +12001,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K145" s="2" t="n">
+      <c r="K145" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="L145" t="inlineStr">
@@ -12086,7 +12074,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K146" s="2" t="n">
+      <c r="K146" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="L146" t="inlineStr">
@@ -12159,7 +12147,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K147" s="2" t="n">
+      <c r="K147" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="L147" t="inlineStr">
@@ -12232,7 +12220,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K148" s="2" t="n">
+      <c r="K148" s="1" t="n">
         <v>46097</v>
       </c>
       <c r="L148" t="inlineStr">
@@ -12305,7 +12293,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K149" s="2" t="n">
+      <c r="K149" s="1" t="n">
         <v>46097</v>
       </c>
       <c r="L149" t="inlineStr">
@@ -12378,7 +12366,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K150" s="2" t="n">
+      <c r="K150" s="1" t="n">
         <v>46098</v>
       </c>
       <c r="L150" t="inlineStr">
@@ -12451,7 +12439,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K151" s="2" t="n">
+      <c r="K151" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="L151" t="inlineStr">
@@ -12524,7 +12512,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K152" s="2" t="n">
+      <c r="K152" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="L152" t="inlineStr">
@@ -12597,7 +12585,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K153" s="2" t="n">
+      <c r="K153" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="L153" t="inlineStr">
@@ -12616,7 +12604,7 @@
       <c r="Q153" t="inlineStr"/>
       <c r="R153" t="inlineStr"/>
       <c r="S153" t="inlineStr"/>
-      <c r="T153" s="2" t="n">
+      <c r="T153" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U153" t="inlineStr">
@@ -12680,7 +12668,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K154" s="2" t="n">
+      <c r="K154" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L154" t="inlineStr">
@@ -12753,7 +12741,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K155" s="2" t="n">
+      <c r="K155" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L155" t="inlineStr">
@@ -12826,7 +12814,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K156" s="2" t="n">
+      <c r="K156" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L156" t="inlineStr">
@@ -12899,7 +12887,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K157" s="2" t="n">
+      <c r="K157" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L157" t="inlineStr">
@@ -12972,7 +12960,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K158" s="2" t="n">
+      <c r="K158" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L158" t="inlineStr">
@@ -13045,7 +13033,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K159" s="2" t="n">
+      <c r="K159" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L159" t="inlineStr">
@@ -13118,7 +13106,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K160" s="2" t="n">
+      <c r="K160" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L160" t="inlineStr">
@@ -13191,7 +13179,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K161" s="2" t="n">
+      <c r="K161" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L161" t="inlineStr">
@@ -13264,7 +13252,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K162" s="2" t="n">
+      <c r="K162" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="L162" t="inlineStr">
@@ -13337,7 +13325,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K163" s="2" t="n">
+      <c r="K163" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L163" t="inlineStr">
@@ -13410,7 +13398,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K164" s="2" t="n">
+      <c r="K164" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L164" t="inlineStr">
@@ -13483,7 +13471,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K165" s="2" t="n">
+      <c r="K165" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L165" t="inlineStr">
@@ -13556,7 +13544,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K166" s="2" t="n">
+      <c r="K166" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L166" t="inlineStr">
@@ -13629,7 +13617,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K167" s="2" t="n">
+      <c r="K167" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L167" t="inlineStr">
@@ -13706,7 +13694,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K168" s="2" t="n">
+      <c r="K168" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L168" t="inlineStr">
@@ -13783,7 +13771,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K169" s="2" t="n">
+      <c r="K169" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L169" t="inlineStr">
@@ -13856,7 +13844,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K170" s="2" t="n">
+      <c r="K170" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L170" t="inlineStr">
@@ -13929,7 +13917,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K171" s="2" t="n">
+      <c r="K171" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L171" t="inlineStr">
@@ -14002,7 +13990,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K172" s="2" t="n">
+      <c r="K172" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L172" t="inlineStr">
@@ -14075,7 +14063,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K173" s="2" t="n">
+      <c r="K173" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L173" t="inlineStr">
@@ -14148,7 +14136,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K174" s="2" t="n">
+      <c r="K174" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L174" t="inlineStr">
@@ -14221,7 +14209,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K175" s="2" t="n">
+      <c r="K175" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L175" t="inlineStr">
@@ -14294,7 +14282,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K176" s="2" t="n">
+      <c r="K176" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L176" t="inlineStr">
@@ -14367,7 +14355,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K177" s="2" t="n">
+      <c r="K177" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L177" t="inlineStr">
@@ -14440,7 +14428,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K178" s="2" t="n">
+      <c r="K178" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L178" t="inlineStr">
@@ -14513,7 +14501,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K179" s="2" t="n">
+      <c r="K179" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L179" t="inlineStr">
@@ -14532,7 +14520,7 @@
       <c r="Q179" t="inlineStr"/>
       <c r="R179" t="inlineStr"/>
       <c r="S179" t="inlineStr"/>
-      <c r="T179" s="2" t="n">
+      <c r="T179" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U179" t="inlineStr">
@@ -14596,7 +14584,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K180" s="2" t="n">
+      <c r="K180" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L180" t="inlineStr">
@@ -14669,7 +14657,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K181" s="2" t="n">
+      <c r="K181" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L181" t="inlineStr">
@@ -14742,7 +14730,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K182" s="2" t="n">
+      <c r="K182" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L182" t="inlineStr">
@@ -14815,7 +14803,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K183" s="2" t="n">
+      <c r="K183" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L183" t="inlineStr">
@@ -14888,7 +14876,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K184" s="2" t="n">
+      <c r="K184" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L184" t="inlineStr">
@@ -14961,7 +14949,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K185" s="2" t="n">
+      <c r="K185" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L185" t="inlineStr">
@@ -15034,7 +15022,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K186" s="2" t="n">
+      <c r="K186" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L186" t="inlineStr">
@@ -15107,7 +15095,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K187" s="2" t="n">
+      <c r="K187" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L187" t="inlineStr">
@@ -15180,7 +15168,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K188" s="2" t="n">
+      <c r="K188" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L188" t="inlineStr">
@@ -15253,7 +15241,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K189" s="2" t="n">
+      <c r="K189" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L189" t="inlineStr">
@@ -15326,7 +15314,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K190" s="2" t="n">
+      <c r="K190" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L190" t="inlineStr">
@@ -15399,7 +15387,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K191" s="2" t="n">
+      <c r="K191" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L191" t="inlineStr">
@@ -15472,7 +15460,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K192" s="2" t="n">
+      <c r="K192" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L192" t="inlineStr">
@@ -15545,7 +15533,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K193" s="2" t="n">
+      <c r="K193" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L193" t="inlineStr">
@@ -15618,7 +15606,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K194" s="2" t="n">
+      <c r="K194" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L194" t="inlineStr">
@@ -15691,7 +15679,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K195" s="2" t="n">
+      <c r="K195" s="1" t="n">
         <v>46126</v>
       </c>
       <c r="L195" t="inlineStr">
@@ -15766,7 +15754,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K196" s="2" t="n">
+      <c r="K196" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="L196" t="inlineStr">
@@ -15841,7 +15829,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K197" s="2" t="n">
+      <c r="K197" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="L197" t="inlineStr">
@@ -15912,7 +15900,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K198" s="2" t="n">
+      <c r="K198" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="L198" t="inlineStr">
@@ -15983,7 +15971,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K199" s="2" t="n">
+      <c r="K199" s="1" t="n">
         <v>46129</v>
       </c>
       <c r="L199" t="inlineStr">
@@ -16054,7 +16042,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K200" s="2" t="n">
+      <c r="K200" s="1" t="n">
         <v>46135</v>
       </c>
       <c r="L200" t="inlineStr">
@@ -16125,7 +16113,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K201" s="2" t="n">
+      <c r="K201" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L201" t="inlineStr">
@@ -16196,7 +16184,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K202" s="2" t="n">
+      <c r="K202" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L202" t="inlineStr">
@@ -16267,7 +16255,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K203" s="2" t="n">
+      <c r="K203" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L203" t="inlineStr">
@@ -16338,7 +16326,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K204" s="2" t="n">
+      <c r="K204" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L204" t="inlineStr">
@@ -16413,7 +16401,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K205" s="2" t="n">
+      <c r="K205" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L205" t="inlineStr">
@@ -16488,7 +16476,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K206" s="2" t="n">
+      <c r="K206" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L206" t="inlineStr">
@@ -16559,7 +16547,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K207" s="2" t="n">
+      <c r="K207" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L207" t="inlineStr">
@@ -16630,7 +16618,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K208" s="2" t="n">
+      <c r="K208" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L208" t="inlineStr">
@@ -16701,7 +16689,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K209" s="2" t="n">
+      <c r="K209" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L209" t="inlineStr">
@@ -16772,7 +16760,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K210" s="2" t="n">
+      <c r="K210" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L210" t="inlineStr">
@@ -16843,7 +16831,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K211" s="2" t="n">
+      <c r="K211" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L211" t="inlineStr">
@@ -16914,7 +16902,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K212" s="2" t="n">
+      <c r="K212" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L212" t="inlineStr">
@@ -16985,7 +16973,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K213" s="2" t="n">
+      <c r="K213" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L213" t="inlineStr">
@@ -17056,7 +17044,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K214" s="2" t="n">
+      <c r="K214" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L214" t="inlineStr">
@@ -17127,7 +17115,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K215" s="2" t="n">
+      <c r="K215" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="L215" t="inlineStr">
@@ -17198,7 +17186,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K216" s="2" t="n">
+      <c r="K216" s="1" t="n">
         <v>46146</v>
       </c>
       <c r="L216" t="inlineStr">
@@ -17269,7 +17257,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K217" s="2" t="n">
+      <c r="K217" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L217" t="inlineStr">
@@ -17340,7 +17328,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K218" s="2" t="n">
+      <c r="K218" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L218" t="inlineStr">
@@ -17411,7 +17399,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K219" s="2" t="n">
+      <c r="K219" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L219" t="inlineStr">
@@ -17482,7 +17470,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K220" s="2" t="n">
+      <c r="K220" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L220" t="inlineStr">
@@ -17553,7 +17541,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K221" s="2" t="n">
+      <c r="K221" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L221" t="inlineStr">
@@ -17624,7 +17612,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K222" s="2" t="n">
+      <c r="K222" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L222" t="inlineStr">
@@ -17695,7 +17683,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K223" s="2" t="n">
+      <c r="K223" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L223" t="inlineStr">
@@ -17766,7 +17754,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K224" s="2" t="n">
+      <c r="K224" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L224" t="inlineStr">
@@ -17837,7 +17825,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K225" s="2" t="n">
+      <c r="K225" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L225" t="inlineStr">
@@ -17908,7 +17896,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K226" s="2" t="n">
+      <c r="K226" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L226" t="inlineStr">
@@ -17979,7 +17967,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K227" s="2" t="n">
+      <c r="K227" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L227" t="inlineStr">
@@ -18050,7 +18038,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K228" s="2" t="n">
+      <c r="K228" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L228" t="inlineStr">
@@ -18121,7 +18109,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K229" s="2" t="n">
+      <c r="K229" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L229" t="inlineStr">
@@ -18192,7 +18180,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K230" s="2" t="n">
+      <c r="K230" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L230" t="inlineStr">
@@ -18263,7 +18251,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K231" s="2" t="n">
+      <c r="K231" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L231" t="inlineStr">
@@ -18334,7 +18322,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K232" s="2" t="n">
+      <c r="K232" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L232" t="inlineStr">
@@ -18405,7 +18393,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K233" s="2" t="n">
+      <c r="K233" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L233" t="inlineStr">
@@ -18476,7 +18464,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K234" s="2" t="n">
+      <c r="K234" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L234" t="inlineStr">
@@ -18547,7 +18535,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K235" s="2" t="n">
+      <c r="K235" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L235" t="inlineStr">
@@ -18618,7 +18606,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K236" s="2" t="n">
+      <c r="K236" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L236" t="inlineStr">
@@ -18689,7 +18677,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K237" s="2" t="n">
+      <c r="K237" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L237" t="inlineStr">
@@ -18760,7 +18748,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K238" s="2" t="n">
+      <c r="K238" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L238" t="inlineStr">
@@ -18831,7 +18819,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K239" s="2" t="n">
+      <c r="K239" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L239" t="inlineStr">
@@ -18902,7 +18890,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K240" s="2" t="n">
+      <c r="K240" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L240" t="inlineStr">
@@ -18973,7 +18961,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K241" s="2" t="n">
+      <c r="K241" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L241" t="inlineStr">
@@ -19044,7 +19032,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K242" s="2" t="n">
+      <c r="K242" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L242" t="inlineStr">
@@ -19115,7 +19103,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K243" s="2" t="n">
+      <c r="K243" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L243" t="inlineStr">
@@ -19186,7 +19174,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K244" s="2" t="n">
+      <c r="K244" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L244" t="inlineStr">
@@ -19257,7 +19245,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K245" s="2" t="n">
+      <c r="K245" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L245" t="inlineStr">
@@ -19328,7 +19316,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K246" s="2" t="n">
+      <c r="K246" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L246" t="inlineStr">
@@ -19399,7 +19387,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K247" s="2" t="n">
+      <c r="K247" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L247" t="inlineStr">
@@ -19470,7 +19458,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K248" s="2" t="n">
+      <c r="K248" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L248" t="inlineStr">
@@ -19541,7 +19529,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K249" s="2" t="n">
+      <c r="K249" s="1" t="n">
         <v>46150</v>
       </c>
       <c r="L249" t="inlineStr">
@@ -19612,7 +19600,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K250" s="2" t="n">
+      <c r="K250" s="1" t="n">
         <v>46155</v>
       </c>
       <c r="L250" t="inlineStr">
@@ -19683,7 +19671,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K251" s="2" t="n">
+      <c r="K251" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="L251" t="inlineStr">
@@ -19754,7 +19742,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K252" s="2" t="n">
+      <c r="K252" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="L252" t="inlineStr">
@@ -19825,7 +19813,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K253" s="2" t="n">
+      <c r="K253" s="1" t="n">
         <v>46162</v>
       </c>
       <c r="L253" t="inlineStr">
@@ -19900,7 +19888,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K254" s="2" t="n">
+      <c r="K254" s="1" t="n">
         <v>46162</v>
       </c>
       <c r="L254" t="inlineStr">
@@ -19971,7 +19959,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K255" s="2" t="n">
+      <c r="K255" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="L255" t="inlineStr">
@@ -20042,7 +20030,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K256" s="2" t="n">
+      <c r="K256" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="L256" t="inlineStr">
@@ -20117,7 +20105,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K257" s="2" t="n">
+      <c r="K257" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="L257" t="inlineStr">
@@ -20136,7 +20124,7 @@
       <c r="Q257" t="inlineStr"/>
       <c r="R257" t="inlineStr"/>
       <c r="S257" t="inlineStr"/>
-      <c r="T257" s="2" t="n">
+      <c r="T257" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U257" t="inlineStr">
@@ -20202,7 +20190,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K258" s="2" t="n">
+      <c r="K258" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="L258" t="inlineStr">
@@ -20277,7 +20265,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K259" s="2" t="n">
+      <c r="K259" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L259" t="inlineStr">
@@ -20352,7 +20340,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K260" s="2" t="n">
+      <c r="K260" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L260" t="inlineStr">
@@ -20371,7 +20359,7 @@
       <c r="Q260" t="inlineStr"/>
       <c r="R260" t="inlineStr"/>
       <c r="S260" t="inlineStr"/>
-      <c r="T260" s="2" t="n">
+      <c r="T260" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U260" t="inlineStr">
@@ -20437,7 +20425,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K261" s="2" t="n">
+      <c r="K261" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L261" t="inlineStr">
@@ -20512,7 +20500,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K262" s="2" t="n">
+      <c r="K262" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L262" t="inlineStr">
@@ -20587,7 +20575,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K263" s="2" t="n">
+      <c r="K263" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L263" t="inlineStr">
@@ -20606,7 +20594,7 @@
       <c r="Q263" t="inlineStr"/>
       <c r="R263" t="inlineStr"/>
       <c r="S263" t="inlineStr"/>
-      <c r="T263" s="2" t="n">
+      <c r="T263" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U263" t="inlineStr">
@@ -20672,7 +20660,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K264" s="2" t="n">
+      <c r="K264" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L264" t="inlineStr">
@@ -20743,7 +20731,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K265" s="2" t="n">
+      <c r="K265" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L265" t="inlineStr">
@@ -20814,7 +20802,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K266" s="2" t="n">
+      <c r="K266" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L266" t="inlineStr">
@@ -20885,7 +20873,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K267" s="2" t="n">
+      <c r="K267" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L267" t="inlineStr">
@@ -20960,7 +20948,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K268" s="2" t="n">
+      <c r="K268" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L268" t="inlineStr">
@@ -21031,7 +21019,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K269" s="2" t="n">
+      <c r="K269" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L269" t="inlineStr">
@@ -21102,7 +21090,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K270" s="2" t="n">
+      <c r="K270" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L270" t="inlineStr">
@@ -21173,7 +21161,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K271" s="2" t="n">
+      <c r="K271" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L271" t="inlineStr">
@@ -21244,7 +21232,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K272" s="2" t="n">
+      <c r="K272" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L272" t="inlineStr">
@@ -21319,7 +21307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K273" s="2" t="n">
+      <c r="K273" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L273" t="inlineStr">
@@ -21394,7 +21382,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K274" s="2" t="n">
+      <c r="K274" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L274" t="inlineStr">
@@ -21465,7 +21453,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K275" s="2" t="n">
+      <c r="K275" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L275" t="inlineStr">
@@ -21536,7 +21524,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K276" s="2" t="n">
+      <c r="K276" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L276" t="inlineStr">
@@ -21607,7 +21595,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K277" s="2" t="n">
+      <c r="K277" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L277" t="inlineStr">
@@ -21678,7 +21666,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K278" s="2" t="n">
+      <c r="K278" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L278" t="inlineStr">
@@ -21749,7 +21737,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K279" s="2" t="n">
+      <c r="K279" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L279" t="inlineStr">
@@ -21820,7 +21808,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K280" s="2" t="n">
+      <c r="K280" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L280" t="inlineStr">
@@ -21891,7 +21879,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K281" s="2" t="n">
+      <c r="K281" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L281" t="inlineStr">
@@ -21962,7 +21950,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K282" s="2" t="n">
+      <c r="K282" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L282" t="inlineStr">
@@ -22033,7 +22021,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K283" s="2" t="n">
+      <c r="K283" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L283" t="inlineStr">
@@ -22104,7 +22092,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K284" s="2" t="n">
+      <c r="K284" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L284" t="inlineStr">
@@ -22175,7 +22163,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K285" s="2" t="n">
+      <c r="K285" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L285" t="inlineStr">
@@ -22246,7 +22234,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K286" s="2" t="n">
+      <c r="K286" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L286" t="inlineStr">
@@ -22317,7 +22305,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K287" s="2" t="n">
+      <c r="K287" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L287" t="inlineStr">
@@ -22388,7 +22376,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K288" s="2" t="n">
+      <c r="K288" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="L288" t="inlineStr">
@@ -22459,7 +22447,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K289" s="2" t="n">
+      <c r="K289" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="L289" t="inlineStr">
@@ -22530,7 +22518,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K290" s="2" t="n">
+      <c r="K290" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="L290" t="inlineStr">
@@ -22601,7 +22589,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K291" s="2" t="n">
+      <c r="K291" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="L291" t="inlineStr">
@@ -22672,7 +22660,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K292" s="2" t="n">
+      <c r="K292" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L292" t="inlineStr">
@@ -22743,7 +22731,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K293" s="2" t="n">
+      <c r="K293" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L293" t="inlineStr">
@@ -22814,7 +22802,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K294" s="2" t="n">
+      <c r="K294" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L294" t="inlineStr">
@@ -22885,7 +22873,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K295" s="2" t="n">
+      <c r="K295" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L295" t="inlineStr">
@@ -22960,7 +22948,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K296" s="2" t="n">
+      <c r="K296" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L296" t="inlineStr">
@@ -23035,7 +23023,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K297" s="2" t="n">
+      <c r="K297" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L297" t="inlineStr">
@@ -23106,7 +23094,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K298" s="2" t="n">
+      <c r="K298" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L298" t="inlineStr">
@@ -23177,7 +23165,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K299" s="2" t="n">
+      <c r="K299" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L299" t="inlineStr">
@@ -23248,7 +23236,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K300" s="2" t="n">
+      <c r="K300" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L300" t="inlineStr">
@@ -23319,7 +23307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K301" s="2" t="n">
+      <c r="K301" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L301" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (10/07/2026 20:02)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -20,13 +20,16 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
+    </font>
+    <font>
+      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -37,7 +40,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -45,12 +48,21 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin"/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -421,117 +433,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" t="inlineStr">
+      <c r="A1" s="1" t="inlineStr">
         <is>
           <t>numero_ordem</t>
         </is>
       </c>
-      <c r="B1" t="inlineStr">
+      <c r="B1" s="1" t="inlineStr">
         <is>
           <t>part_number</t>
         </is>
       </c>
-      <c r="C1" t="inlineStr">
+      <c r="C1" s="1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="D1" t="inlineStr">
+      <c r="D1" s="1" t="inlineStr">
         <is>
           <t>sn_lt</t>
         </is>
       </c>
-      <c r="E1" t="inlineStr">
+      <c r="E1" s="1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="F1" t="inlineStr">
+      <c r="F1" s="1" t="inlineStr">
         <is>
           <t>quantidade_texto</t>
         </is>
       </c>
-      <c r="G1" t="inlineStr">
+      <c r="G1" s="1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="H1" t="inlineStr">
+      <c r="H1" s="1" t="inlineStr">
         <is>
           <t>pedido_emg</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
+      <c r="I1" s="1" t="inlineStr">
         <is>
           <t>motivo</t>
         </is>
       </c>
-      <c r="J1" t="inlineStr">
+      <c r="J1" s="1" t="inlineStr">
         <is>
           <t>pj</t>
         </is>
       </c>
-      <c r="K1" t="inlineStr">
+      <c r="K1" s="1" t="inlineStr">
         <is>
           <t>pedido_envio</t>
         </is>
       </c>
-      <c r="L1" t="inlineStr">
+      <c r="L1" s="1" t="inlineStr">
         <is>
           <t>anv</t>
         </is>
       </c>
-      <c r="M1" t="inlineStr">
+      <c r="M1" s="1" t="inlineStr">
         <is>
           <t>destino</t>
         </is>
       </c>
-      <c r="N1" t="inlineStr">
+      <c r="N1" s="1" t="inlineStr">
         <is>
           <t>nf_gmm</t>
         </is>
       </c>
-      <c r="O1" t="inlineStr">
+      <c r="O1" s="1" t="inlineStr">
         <is>
           <t>rastreio</t>
         </is>
       </c>
-      <c r="P1" t="inlineStr">
+      <c r="P1" s="1" t="inlineStr">
         <is>
           <t>pn_devolvido</t>
         </is>
       </c>
-      <c r="Q1" t="inlineStr">
+      <c r="Q1" s="1" t="inlineStr">
         <is>
           <t>detalhe_entrega</t>
         </is>
       </c>
-      <c r="R1" t="inlineStr">
+      <c r="R1" s="1" t="inlineStr">
         <is>
           <t>numero_rc</t>
         </is>
       </c>
-      <c r="S1" t="inlineStr">
+      <c r="S1" s="1" t="inlineStr">
         <is>
           <t>nf_devolucao_vee_one</t>
         </is>
       </c>
-      <c r="T1" t="inlineStr">
+      <c r="T1" s="1" t="inlineStr">
         <is>
           <t>data_devolucao</t>
         </is>
       </c>
-      <c r="U1" t="inlineStr">
+      <c r="U1" s="1" t="inlineStr">
         <is>
           <t>observacao_fiscal</t>
         </is>
       </c>
-      <c r="V1" t="inlineStr">
+      <c r="V1" s="1" t="inlineStr">
         <is>
           <t>observacao_empresa</t>
         </is>
       </c>
-      <c r="W1" t="inlineStr">
+      <c r="W1" s="1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -586,7 +598,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K2" s="1" t="n">
+      <c r="K2" s="2" t="n">
         <v>45730</v>
       </c>
       <c r="L2" t="inlineStr">
@@ -663,7 +675,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K3" s="1" t="n">
+      <c r="K3" s="2" t="n">
         <v>45735</v>
       </c>
       <c r="L3" t="inlineStr">
@@ -740,7 +752,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K4" s="1" t="n">
+      <c r="K4" s="2" t="n">
         <v>45737</v>
       </c>
       <c r="L4" t="inlineStr">
@@ -817,7 +829,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K5" s="1" t="n">
+      <c r="K5" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L5" t="inlineStr">
@@ -902,7 +914,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K6" s="1" t="n">
+      <c r="K6" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L6" t="inlineStr">
@@ -983,7 +995,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K7" s="1" t="n">
+      <c r="K7" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L7" t="inlineStr">
@@ -1064,7 +1076,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K8" s="1" t="n">
+      <c r="K8" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L8" t="inlineStr">
@@ -1145,7 +1157,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K9" s="1" t="n">
+      <c r="K9" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L9" t="inlineStr">
@@ -1226,7 +1238,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K10" s="1" t="n">
+      <c r="K10" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L10" t="inlineStr">
@@ -1307,7 +1319,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K11" s="1" t="n">
+      <c r="K11" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L11" t="inlineStr">
@@ -1388,7 +1400,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K12" s="1" t="n">
+      <c r="K12" s="2" t="n">
         <v>45747</v>
       </c>
       <c r="L12" t="inlineStr">
@@ -1465,7 +1477,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K13" s="1" t="n">
+      <c r="K13" s="2" t="n">
         <v>45762</v>
       </c>
       <c r="L13" t="inlineStr">
@@ -1542,7 +1554,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K14" s="1" t="n">
+      <c r="K14" s="2" t="n">
         <v>45763</v>
       </c>
       <c r="L14" t="inlineStr">
@@ -1619,7 +1631,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K15" s="1" t="n">
+      <c r="K15" s="2" t="n">
         <v>45763</v>
       </c>
       <c r="L15" t="inlineStr">
@@ -1696,7 +1708,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K16" s="1" t="n">
+      <c r="K16" s="2" t="n">
         <v>45783</v>
       </c>
       <c r="L16" t="inlineStr">
@@ -1773,7 +1785,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K17" s="1" t="n">
+      <c r="K17" s="2" t="n">
         <v>45783</v>
       </c>
       <c r="L17" t="inlineStr">
@@ -1850,7 +1862,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K18" s="1" t="n">
+      <c r="K18" s="2" t="n">
         <v>45784</v>
       </c>
       <c r="L18" t="inlineStr">
@@ -1881,7 +1893,7 @@
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" s="1" t="n">
+      <c r="T18" s="2" t="n">
         <v>45845</v>
       </c>
       <c r="U18" t="inlineStr">
@@ -1945,7 +1957,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K19" s="1" t="n">
+      <c r="K19" s="2" t="n">
         <v>45784</v>
       </c>
       <c r="L19" t="inlineStr">
@@ -2022,7 +2034,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K20" s="1" t="n">
+      <c r="K20" s="2" t="n">
         <v>45784</v>
       </c>
       <c r="L20" t="inlineStr">
@@ -2099,7 +2111,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K21" s="1" t="n">
+      <c r="K21" s="2" t="n">
         <v>45784</v>
       </c>
       <c r="L21" t="inlineStr">
@@ -2130,7 +2142,7 @@
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
-      <c r="T21" s="1" t="n">
+      <c r="T21" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="U21" t="inlineStr">
@@ -2194,7 +2206,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K22" s="1" t="n">
+      <c r="K22" s="2" t="n">
         <v>45789</v>
       </c>
       <c r="L22" t="inlineStr">
@@ -2225,7 +2237,7 @@
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
-      <c r="T22" s="1" t="n">
+      <c r="T22" s="2" t="n">
         <v>45868</v>
       </c>
       <c r="U22" t="inlineStr">
@@ -2289,7 +2301,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K23" s="1" t="n">
+      <c r="K23" s="2" t="n">
         <v>45789</v>
       </c>
       <c r="L23" t="inlineStr">
@@ -2320,7 +2332,7 @@
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
-      <c r="T23" s="1" t="n">
+      <c r="T23" s="2" t="n">
         <v>45982</v>
       </c>
       <c r="U23" t="inlineStr">
@@ -2384,7 +2396,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K24" s="1" t="n">
+      <c r="K24" s="2" t="n">
         <v>45791</v>
       </c>
       <c r="L24" t="inlineStr">
@@ -2461,7 +2473,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K25" s="1" t="n">
+      <c r="K25" s="2" t="n">
         <v>45814</v>
       </c>
       <c r="L25" t="inlineStr">
@@ -2534,7 +2546,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K26" s="1" t="n">
+      <c r="K26" s="2" t="n">
         <v>45819</v>
       </c>
       <c r="L26" t="inlineStr">
@@ -2607,7 +2619,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K27" s="1" t="n">
+      <c r="K27" s="2" t="n">
         <v>45821</v>
       </c>
       <c r="L27" t="inlineStr">
@@ -2638,7 +2650,7 @@
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" s="1" t="n">
+      <c r="T27" s="2" t="n">
         <v>45876</v>
       </c>
       <c r="U27" t="inlineStr">
@@ -2702,7 +2714,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K28" s="1" t="n">
+      <c r="K28" s="2" t="n">
         <v>45824</v>
       </c>
       <c r="L28" t="inlineStr">
@@ -2779,7 +2791,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K29" s="1" t="n">
+      <c r="K29" s="2" t="n">
         <v>45825</v>
       </c>
       <c r="L29" t="inlineStr">
@@ -2856,7 +2868,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K30" s="1" t="n">
+      <c r="K30" s="2" t="n">
         <v>45836</v>
       </c>
       <c r="L30" t="inlineStr">
@@ -2933,7 +2945,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K31" s="1" t="n">
+      <c r="K31" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="L31" t="inlineStr">
@@ -2964,7 +2976,7 @@
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" s="1" t="n">
+      <c r="T31" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U31" t="inlineStr">
@@ -3028,7 +3040,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K32" s="1" t="n">
+      <c r="K32" s="2" t="n">
         <v>45839</v>
       </c>
       <c r="L32" t="inlineStr">
@@ -3105,7 +3117,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K33" s="1" t="n">
+      <c r="K33" s="2" t="n">
         <v>45845</v>
       </c>
       <c r="L33" t="inlineStr">
@@ -3136,7 +3148,7 @@
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" s="1" t="n">
+      <c r="T33" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U33" t="inlineStr">
@@ -3200,7 +3212,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K34" s="1" t="n">
+      <c r="K34" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="L34" t="inlineStr">
@@ -3277,7 +3289,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K35" s="1" t="n">
+      <c r="K35" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="L35" t="inlineStr">
@@ -3308,7 +3320,7 @@
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
-      <c r="T35" s="1" t="n">
+      <c r="T35" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U35" t="inlineStr">
@@ -3372,7 +3384,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K36" s="1" t="n">
+      <c r="K36" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="L36" t="inlineStr">
@@ -3403,7 +3415,7 @@
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
-      <c r="T36" s="1" t="n">
+      <c r="T36" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U36" t="inlineStr">
@@ -3467,7 +3479,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K37" s="1" t="n">
+      <c r="K37" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="L37" t="inlineStr">
@@ -3498,7 +3510,7 @@
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
-      <c r="T37" s="1" t="n">
+      <c r="T37" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U37" t="inlineStr">
@@ -3562,7 +3574,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K38" s="1" t="n">
+      <c r="K38" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="L38" t="inlineStr">
@@ -3593,7 +3605,7 @@
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
-      <c r="T38" s="1" t="n">
+      <c r="T38" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U38" t="inlineStr">
@@ -3657,7 +3669,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K39" s="1" t="n">
+      <c r="K39" s="2" t="n">
         <v>45856</v>
       </c>
       <c r="L39" t="inlineStr">
@@ -3688,7 +3700,7 @@
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
-      <c r="T39" s="1" t="n">
+      <c r="T39" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U39" t="inlineStr">
@@ -3752,7 +3764,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K40" s="1" t="n">
+      <c r="K40" s="2" t="n">
         <v>45866</v>
       </c>
       <c r="L40" t="inlineStr">
@@ -3783,7 +3795,7 @@
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
-      <c r="T40" s="1" t="n">
+      <c r="T40" s="2" t="n">
         <v>45916</v>
       </c>
       <c r="U40" t="inlineStr">
@@ -3847,7 +3859,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K41" s="1" t="n">
+      <c r="K41" s="2" t="n">
         <v>45866</v>
       </c>
       <c r="L41" t="inlineStr">
@@ -3924,7 +3936,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K42" s="1" t="n">
+      <c r="K42" s="2" t="n">
         <v>45866</v>
       </c>
       <c r="L42" t="inlineStr">
@@ -3955,7 +3967,7 @@
         </is>
       </c>
       <c r="S42" t="inlineStr"/>
-      <c r="T42" s="1" t="n">
+      <c r="T42" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="U42" t="inlineStr">
@@ -4019,7 +4031,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K43" s="1" t="n">
+      <c r="K43" s="2" t="n">
         <v>45866</v>
       </c>
       <c r="L43" t="inlineStr">
@@ -4096,7 +4108,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K44" s="1" t="n">
+      <c r="K44" s="2" t="n">
         <v>45866</v>
       </c>
       <c r="L44" t="inlineStr">
@@ -4127,7 +4139,7 @@
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
-      <c r="T44" s="1" t="n">
+      <c r="T44" s="2" t="n">
         <v>46002</v>
       </c>
       <c r="U44" t="inlineStr">
@@ -4191,7 +4203,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K45" s="1" t="n">
+      <c r="K45" s="2" t="n">
         <v>45882</v>
       </c>
       <c r="L45" t="inlineStr">
@@ -4268,7 +4280,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K46" s="1" t="n">
+      <c r="K46" s="2" t="n">
         <v>45882</v>
       </c>
       <c r="L46" t="inlineStr">
@@ -4345,7 +4357,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K47" s="1" t="n">
+      <c r="K47" s="2" t="n">
         <v>45890</v>
       </c>
       <c r="L47" t="inlineStr">
@@ -4376,7 +4388,7 @@
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
-      <c r="T47" s="1" t="n">
+      <c r="T47" s="2" t="n">
         <v>45944</v>
       </c>
       <c r="U47" t="inlineStr">
@@ -4440,7 +4452,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K48" s="1" t="n">
+      <c r="K48" s="2" t="n">
         <v>45903</v>
       </c>
       <c r="L48" t="inlineStr">
@@ -4517,7 +4529,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K49" s="1" t="n">
+      <c r="K49" s="2" t="n">
         <v>45904</v>
       </c>
       <c r="L49" t="inlineStr">
@@ -4594,7 +4606,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K50" s="1" t="n">
+      <c r="K50" s="2" t="n">
         <v>45912</v>
       </c>
       <c r="L50" t="inlineStr">
@@ -4671,7 +4683,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K51" s="1" t="n">
+      <c r="K51" s="2" t="n">
         <v>45925</v>
       </c>
       <c r="L51" t="inlineStr">
@@ -4752,7 +4764,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K52" s="1" t="n">
+      <c r="K52" s="2" t="n">
         <v>45924</v>
       </c>
       <c r="L52" t="inlineStr">
@@ -4829,7 +4841,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K53" s="1" t="n">
+      <c r="K53" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="L53" t="inlineStr">
@@ -4906,7 +4918,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K54" s="1" t="n">
+      <c r="K54" s="2" t="n">
         <v>45930</v>
       </c>
       <c r="L54" t="inlineStr">
@@ -4983,7 +4995,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K55" s="1" t="n">
+      <c r="K55" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="L55" t="inlineStr">
@@ -5068,7 +5080,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K56" s="1" t="n">
+      <c r="K56" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="L56" t="inlineStr">
@@ -5157,7 +5169,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K57" s="1" t="n">
+      <c r="K57" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="L57" t="inlineStr">
@@ -5242,7 +5254,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K58" s="1" t="n">
+      <c r="K58" s="2" t="n">
         <v>45931</v>
       </c>
       <c r="L58" t="inlineStr">
@@ -5327,7 +5339,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K59" s="1" t="n">
+      <c r="K59" s="2" t="n">
         <v>45937</v>
       </c>
       <c r="L59" t="inlineStr">
@@ -5358,7 +5370,7 @@
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
-      <c r="T59" s="1" t="n">
+      <c r="T59" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="U59" t="inlineStr">
@@ -5422,7 +5434,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K60" s="1" t="n">
+      <c r="K60" s="2" t="n">
         <v>45938</v>
       </c>
       <c r="L60" t="inlineStr">
@@ -5499,7 +5511,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K61" s="1" t="n">
+      <c r="K61" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="L61" t="inlineStr">
@@ -5576,7 +5588,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K62" s="1" t="n">
+      <c r="K62" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="L62" t="inlineStr">
@@ -5653,7 +5665,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K63" s="1" t="n">
+      <c r="K63" s="2" t="n">
         <v>45939</v>
       </c>
       <c r="L63" t="inlineStr">
@@ -5730,7 +5742,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K64" s="1" t="n">
+      <c r="K64" s="2" t="n">
         <v>45940</v>
       </c>
       <c r="L64" t="inlineStr">
@@ -5807,7 +5819,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K65" s="1" t="n">
+      <c r="K65" s="2" t="n">
         <v>45943</v>
       </c>
       <c r="L65" t="inlineStr">
@@ -5888,7 +5900,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K66" s="1" t="n">
+      <c r="K66" s="2" t="n">
         <v>45943</v>
       </c>
       <c r="L66" t="inlineStr">
@@ -5965,7 +5977,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K67" s="1" t="n">
+      <c r="K67" s="2" t="n">
         <v>45943</v>
       </c>
       <c r="L67" t="inlineStr">
@@ -6042,7 +6054,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K68" s="1" t="n">
+      <c r="K68" s="2" t="n">
         <v>45961</v>
       </c>
       <c r="L68" t="inlineStr">
@@ -6069,7 +6081,7 @@
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
-      <c r="T68" s="1" t="n">
+      <c r="T68" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="U68" t="inlineStr">
@@ -6137,7 +6149,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K69" s="1" t="n">
+      <c r="K69" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="L69" t="inlineStr">
@@ -6214,7 +6226,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K70" s="1" t="n">
+      <c r="K70" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="L70" t="inlineStr">
@@ -6291,7 +6303,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K71" s="1" t="n">
+      <c r="K71" s="2" t="n">
         <v>45965</v>
       </c>
       <c r="L71" t="inlineStr">
@@ -6368,7 +6380,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K72" s="1" t="n">
+      <c r="K72" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="L72" t="inlineStr">
@@ -6445,7 +6457,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K73" s="1" t="n">
+      <c r="K73" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="L73" t="inlineStr">
@@ -6522,7 +6534,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K74" s="1" t="n">
+      <c r="K74" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="L74" t="inlineStr">
@@ -6599,7 +6611,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K75" s="1" t="n">
+      <c r="K75" s="2" t="n">
         <v>45967</v>
       </c>
       <c r="L75" t="inlineStr">
@@ -6676,7 +6688,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K76" s="1" t="n">
+      <c r="K76" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="L76" t="inlineStr">
@@ -6753,7 +6765,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K77" s="1" t="n">
+      <c r="K77" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="L77" t="inlineStr">
@@ -6830,7 +6842,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K78" s="1" t="n">
+      <c r="K78" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="L78" t="inlineStr">
@@ -6907,7 +6919,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K79" s="1" t="n">
+      <c r="K79" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="L79" t="inlineStr">
@@ -6984,7 +6996,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K80" s="1" t="n">
+      <c r="K80" s="2" t="n">
         <v>45968</v>
       </c>
       <c r="L80" t="inlineStr">
@@ -7061,7 +7073,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K81" s="1" t="n">
+      <c r="K81" s="2" t="n">
         <v>45973</v>
       </c>
       <c r="L81" t="inlineStr">
@@ -7138,7 +7150,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K82" s="1" t="n">
+      <c r="K82" s="2" t="n">
         <v>45974</v>
       </c>
       <c r="L82" t="inlineStr">
@@ -7215,7 +7227,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K83" s="1" t="n">
+      <c r="K83" s="2" t="n">
         <v>45975</v>
       </c>
       <c r="L83" t="inlineStr">
@@ -7292,7 +7304,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K84" s="1" t="n">
+      <c r="K84" s="2" t="n">
         <v>45975</v>
       </c>
       <c r="L84" t="inlineStr">
@@ -7369,7 +7381,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K85" s="1" t="n">
+      <c r="K85" s="2" t="n">
         <v>45982</v>
       </c>
       <c r="L85" t="inlineStr">
@@ -7446,7 +7458,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K86" s="1" t="n">
+      <c r="K86" s="2" t="n">
         <v>45982</v>
       </c>
       <c r="L86" t="inlineStr">
@@ -7523,7 +7535,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K87" s="1" t="n">
+      <c r="K87" s="2" t="n">
         <v>45985</v>
       </c>
       <c r="L87" t="inlineStr">
@@ -7600,7 +7612,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K88" s="1" t="n">
+      <c r="K88" s="2" t="n">
         <v>45985</v>
       </c>
       <c r="L88" t="inlineStr">
@@ -7677,7 +7689,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K89" s="1" t="n">
+      <c r="K89" s="2" t="n">
         <v>45986</v>
       </c>
       <c r="L89" t="inlineStr">
@@ -7750,7 +7762,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K90" s="1" t="n">
+      <c r="K90" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="L90" t="inlineStr">
@@ -7823,7 +7835,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K91" s="1" t="n">
+      <c r="K91" s="2" t="n">
         <v>45992</v>
       </c>
       <c r="L91" t="inlineStr">
@@ -7900,7 +7912,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K92" s="1" t="n">
+      <c r="K92" s="2" t="n">
         <v>45996</v>
       </c>
       <c r="L92" t="inlineStr">
@@ -7935,7 +7947,7 @@
         </is>
       </c>
       <c r="S92" t="inlineStr"/>
-      <c r="T92" s="1" t="n">
+      <c r="T92" s="2" t="n">
         <v>45979</v>
       </c>
       <c r="U92" t="inlineStr">
@@ -7999,7 +8011,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K93" s="1" t="n">
+      <c r="K93" s="2" t="n">
         <v>46002</v>
       </c>
       <c r="L93" t="inlineStr">
@@ -8072,7 +8084,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K94" s="1" t="n">
+      <c r="K94" s="2" t="n">
         <v>46007</v>
       </c>
       <c r="L94" t="inlineStr">
@@ -8149,7 +8161,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K95" s="1" t="n">
+      <c r="K95" s="2" t="n">
         <v>46007</v>
       </c>
       <c r="L95" t="inlineStr">
@@ -8226,7 +8238,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K96" s="1" t="n">
+      <c r="K96" s="2" t="n">
         <v>46008</v>
       </c>
       <c r="L96" t="inlineStr">
@@ -8307,7 +8319,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K97" s="1" t="n">
+      <c r="K97" s="2" t="n">
         <v>46029</v>
       </c>
       <c r="L97" t="inlineStr">
@@ -8334,7 +8346,7 @@
         </is>
       </c>
       <c r="S97" t="inlineStr"/>
-      <c r="T97" s="1" t="n">
+      <c r="T97" s="2" t="n">
         <v>46030</v>
       </c>
       <c r="U97" t="inlineStr">
@@ -8398,7 +8410,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K98" s="1" t="n">
+      <c r="K98" s="2" t="n">
         <v>46029</v>
       </c>
       <c r="L98" t="inlineStr">
@@ -8475,7 +8487,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K99" s="1" t="n">
+      <c r="K99" s="2" t="n">
         <v>46034</v>
       </c>
       <c r="L99" t="inlineStr">
@@ -8552,7 +8564,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K100" s="1" t="n">
+      <c r="K100" s="2" t="n">
         <v>46034</v>
       </c>
       <c r="L100" t="inlineStr">
@@ -8625,7 +8637,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K101" s="1" t="n">
+      <c r="K101" s="2" t="n">
         <v>46035</v>
       </c>
       <c r="L101" t="inlineStr">
@@ -8698,7 +8710,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K102" s="1" t="n">
+      <c r="K102" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="L102" t="inlineStr">
@@ -8771,7 +8783,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K103" s="1" t="n">
+      <c r="K103" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="L103" t="inlineStr">
@@ -8844,7 +8856,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K104" s="1" t="n">
+      <c r="K104" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="L104" t="inlineStr">
@@ -8917,7 +8929,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K105" s="1" t="n">
+      <c r="K105" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="L105" t="inlineStr">
@@ -8990,7 +9002,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K106" s="1" t="n">
+      <c r="K106" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="L106" t="inlineStr">
@@ -9063,7 +9075,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K107" s="1" t="n">
+      <c r="K107" s="2" t="n">
         <v>46036</v>
       </c>
       <c r="L107" t="inlineStr">
@@ -9136,7 +9148,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K108" s="1" t="n">
+      <c r="K108" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="L108" t="inlineStr">
@@ -9209,7 +9221,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K109" s="1" t="n">
+      <c r="K109" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="L109" t="inlineStr">
@@ -9282,7 +9294,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K110" s="1" t="n">
+      <c r="K110" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="L110" t="inlineStr">
@@ -9313,7 +9325,7 @@
         </is>
       </c>
       <c r="S110" t="inlineStr"/>
-      <c r="T110" s="1" t="n">
+      <c r="T110" s="2" t="n">
         <v>45805</v>
       </c>
       <c r="U110" t="inlineStr">
@@ -9373,7 +9385,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K111" s="1" t="n">
+      <c r="K111" s="2" t="n">
         <v>46043</v>
       </c>
       <c r="L111" t="inlineStr">
@@ -9404,7 +9416,7 @@
         </is>
       </c>
       <c r="S111" t="inlineStr"/>
-      <c r="T111" s="1" t="n">
+      <c r="T111" s="2" t="n">
         <v>45959</v>
       </c>
       <c r="U111" t="inlineStr">
@@ -9464,7 +9476,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K112" s="1" t="n">
+      <c r="K112" s="2" t="n">
         <v>46044</v>
       </c>
       <c r="L112" t="inlineStr">
@@ -9495,7 +9507,7 @@
         </is>
       </c>
       <c r="S112" t="inlineStr"/>
-      <c r="T112" s="1" t="n">
+      <c r="T112" s="2" t="n">
         <v>46052</v>
       </c>
       <c r="U112" t="inlineStr">
@@ -9559,7 +9571,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K113" s="1" t="n">
+      <c r="K113" s="2" t="n">
         <v>46049</v>
       </c>
       <c r="L113" t="inlineStr">
@@ -9636,7 +9648,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K114" s="1" t="n">
+      <c r="K114" s="2" t="n">
         <v>46049</v>
       </c>
       <c r="L114" t="inlineStr">
@@ -9713,7 +9725,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K115" s="1" t="n">
+      <c r="K115" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="L115" t="inlineStr">
@@ -9790,7 +9802,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K116" s="1" t="n">
+      <c r="K116" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="L116" t="inlineStr">
@@ -9821,7 +9833,7 @@
         </is>
       </c>
       <c r="S116" t="inlineStr"/>
-      <c r="T116" s="1" t="n">
+      <c r="T116" s="2" t="n">
         <v>46048</v>
       </c>
       <c r="U116" t="inlineStr">
@@ -9885,7 +9897,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K117" s="1" t="n">
+      <c r="K117" s="2" t="n">
         <v>46050</v>
       </c>
       <c r="L117" t="inlineStr">
@@ -9962,7 +9974,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K118" s="1" t="n">
+      <c r="K118" s="2" t="n">
         <v>46063</v>
       </c>
       <c r="L118" t="inlineStr">
@@ -10043,7 +10055,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K119" s="1" t="n">
+      <c r="K119" s="2" t="n">
         <v>46028</v>
       </c>
       <c r="L119" t="inlineStr">
@@ -10114,7 +10126,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K120" s="1" t="n">
+      <c r="K120" s="2" t="n">
         <v>46062</v>
       </c>
       <c r="L120" t="inlineStr">
@@ -10191,7 +10203,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K121" s="1" t="n">
+      <c r="K121" s="2" t="n">
         <v>46065</v>
       </c>
       <c r="L121" t="inlineStr">
@@ -10268,7 +10280,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K122" s="1" t="n">
+      <c r="K122" s="2" t="n">
         <v>46065</v>
       </c>
       <c r="L122" t="inlineStr">
@@ -10353,7 +10365,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K123" s="1" t="n">
+      <c r="K123" s="2" t="n">
         <v>46065</v>
       </c>
       <c r="L123" t="inlineStr">
@@ -10430,7 +10442,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K124" s="1" t="n">
+      <c r="K124" s="2" t="n">
         <v>46065</v>
       </c>
       <c r="L124" t="inlineStr">
@@ -10507,7 +10519,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K125" s="1" t="n">
+      <c r="K125" s="2" t="n">
         <v>46066</v>
       </c>
       <c r="L125" t="inlineStr">
@@ -10580,7 +10592,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K126" s="1" t="n">
+      <c r="K126" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="L126" t="inlineStr">
@@ -10653,7 +10665,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K127" s="1" t="n">
+      <c r="K127" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="L127" t="inlineStr">
@@ -10684,7 +10696,7 @@
         </is>
       </c>
       <c r="S127" t="inlineStr"/>
-      <c r="T127" s="1" t="n">
+      <c r="T127" s="2" t="n">
         <v>45889</v>
       </c>
       <c r="U127" t="inlineStr">
@@ -10744,7 +10756,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K128" s="1" t="n">
+      <c r="K128" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="L128" t="inlineStr">
@@ -10817,7 +10829,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K129" s="1" t="n">
+      <c r="K129" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="L129" t="inlineStr">
@@ -10890,7 +10902,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K130" s="1" t="n">
+      <c r="K130" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="L130" t="inlineStr">
@@ -10963,7 +10975,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K131" s="1" t="n">
+      <c r="K131" s="2" t="n">
         <v>46073</v>
       </c>
       <c r="L131" t="inlineStr">
@@ -11040,7 +11052,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K132" s="1" t="n">
+      <c r="K132" s="2" t="n">
         <v>46077</v>
       </c>
       <c r="L132" t="inlineStr">
@@ -11113,7 +11125,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K133" s="1" t="n">
+      <c r="K133" s="2" t="n">
         <v>46079</v>
       </c>
       <c r="L133" t="inlineStr">
@@ -11186,7 +11198,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K134" s="1" t="n">
+      <c r="K134" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L134" t="inlineStr">
@@ -11259,7 +11271,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K135" s="1" t="n">
+      <c r="K135" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L135" t="inlineStr">
@@ -11332,7 +11344,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K136" s="1" t="n">
+      <c r="K136" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L136" t="inlineStr">
@@ -11405,7 +11417,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K137" s="1" t="n">
+      <c r="K137" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L137" t="inlineStr">
@@ -11478,7 +11490,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K138" s="1" t="n">
+      <c r="K138" s="2" t="n">
         <v>46080</v>
       </c>
       <c r="L138" t="inlineStr">
@@ -11551,7 +11563,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K139" s="1" t="n">
+      <c r="K139" s="2" t="n">
         <v>46078</v>
       </c>
       <c r="L139" t="inlineStr">
@@ -11632,7 +11644,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K140" s="1" t="n">
+      <c r="K140" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="L140" t="inlineStr">
@@ -11705,7 +11717,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K141" s="1" t="n">
+      <c r="K141" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="L141" t="inlineStr">
@@ -11778,7 +11790,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K142" s="1" t="n">
+      <c r="K142" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="L142" t="inlineStr">
@@ -11855,7 +11867,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K143" s="1" t="n">
+      <c r="K143" s="2" t="n">
         <v>46092</v>
       </c>
       <c r="L143" t="inlineStr">
@@ -11928,7 +11940,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K144" s="1" t="n">
+      <c r="K144" s="2" t="n">
         <v>46090</v>
       </c>
       <c r="L144" t="inlineStr">
@@ -12001,7 +12013,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K145" s="1" t="n">
+      <c r="K145" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="L145" t="inlineStr">
@@ -12074,7 +12086,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K146" s="1" t="n">
+      <c r="K146" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="L146" t="inlineStr">
@@ -12147,7 +12159,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K147" s="1" t="n">
+      <c r="K147" s="2" t="n">
         <v>46094</v>
       </c>
       <c r="L147" t="inlineStr">
@@ -12220,7 +12232,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K148" s="1" t="n">
+      <c r="K148" s="2" t="n">
         <v>46097</v>
       </c>
       <c r="L148" t="inlineStr">
@@ -12293,7 +12305,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K149" s="1" t="n">
+      <c r="K149" s="2" t="n">
         <v>46097</v>
       </c>
       <c r="L149" t="inlineStr">
@@ -12366,7 +12378,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K150" s="1" t="n">
+      <c r="K150" s="2" t="n">
         <v>46098</v>
       </c>
       <c r="L150" t="inlineStr">
@@ -12439,7 +12451,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K151" s="1" t="n">
+      <c r="K151" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="L151" t="inlineStr">
@@ -12512,7 +12524,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K152" s="1" t="n">
+      <c r="K152" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="L152" t="inlineStr">
@@ -12585,7 +12597,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K153" s="1" t="n">
+      <c r="K153" s="2" t="n">
         <v>46100</v>
       </c>
       <c r="L153" t="inlineStr">
@@ -12604,7 +12616,7 @@
       <c r="Q153" t="inlineStr"/>
       <c r="R153" t="inlineStr"/>
       <c r="S153" t="inlineStr"/>
-      <c r="T153" s="1" t="n">
+      <c r="T153" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="U153" t="inlineStr">
@@ -12668,7 +12680,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K154" s="1" t="n">
+      <c r="K154" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L154" t="inlineStr">
@@ -12741,7 +12753,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K155" s="1" t="n">
+      <c r="K155" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L155" t="inlineStr">
@@ -12814,7 +12826,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K156" s="1" t="n">
+      <c r="K156" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L156" t="inlineStr">
@@ -12887,7 +12899,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K157" s="1" t="n">
+      <c r="K157" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L157" t="inlineStr">
@@ -12960,7 +12972,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K158" s="1" t="n">
+      <c r="K158" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L158" t="inlineStr">
@@ -13033,7 +13045,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K159" s="1" t="n">
+      <c r="K159" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L159" t="inlineStr">
@@ -13106,7 +13118,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K160" s="1" t="n">
+      <c r="K160" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L160" t="inlineStr">
@@ -13179,7 +13191,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K161" s="1" t="n">
+      <c r="K161" s="2" t="n">
         <v>46101</v>
       </c>
       <c r="L161" t="inlineStr">
@@ -13252,7 +13264,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K162" s="1" t="n">
+      <c r="K162" s="2" t="n">
         <v>46113</v>
       </c>
       <c r="L162" t="inlineStr">
@@ -13325,7 +13337,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K163" s="1" t="n">
+      <c r="K163" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="L163" t="inlineStr">
@@ -13398,7 +13410,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K164" s="1" t="n">
+      <c r="K164" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="L164" t="inlineStr">
@@ -13471,7 +13483,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K165" s="1" t="n">
+      <c r="K165" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="L165" t="inlineStr">
@@ -13544,7 +13556,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K166" s="1" t="n">
+      <c r="K166" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="L166" t="inlineStr">
@@ -13617,7 +13629,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K167" s="1" t="n">
+      <c r="K167" s="2" t="n">
         <v>46119</v>
       </c>
       <c r="L167" t="inlineStr">
@@ -13694,7 +13706,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K168" s="1" t="n">
+      <c r="K168" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L168" t="inlineStr">
@@ -13771,7 +13783,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K169" s="1" t="n">
+      <c r="K169" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L169" t="inlineStr">
@@ -13844,7 +13856,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K170" s="1" t="n">
+      <c r="K170" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L170" t="inlineStr">
@@ -13917,7 +13929,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K171" s="1" t="n">
+      <c r="K171" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L171" t="inlineStr">
@@ -13990,7 +14002,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K172" s="1" t="n">
+      <c r="K172" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L172" t="inlineStr">
@@ -14063,7 +14075,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K173" s="1" t="n">
+      <c r="K173" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L173" t="inlineStr">
@@ -14136,7 +14148,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K174" s="1" t="n">
+      <c r="K174" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L174" t="inlineStr">
@@ -14209,7 +14221,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K175" s="1" t="n">
+      <c r="K175" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L175" t="inlineStr">
@@ -14282,7 +14294,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K176" s="1" t="n">
+      <c r="K176" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L176" t="inlineStr">
@@ -14355,7 +14367,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K177" s="1" t="n">
+      <c r="K177" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L177" t="inlineStr">
@@ -14428,7 +14440,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K178" s="1" t="n">
+      <c r="K178" s="2" t="n">
         <v>46120</v>
       </c>
       <c r="L178" t="inlineStr">
@@ -14501,7 +14513,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K179" s="1" t="n">
+      <c r="K179" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="L179" t="inlineStr">
@@ -14520,7 +14532,7 @@
       <c r="Q179" t="inlineStr"/>
       <c r="R179" t="inlineStr"/>
       <c r="S179" t="inlineStr"/>
-      <c r="T179" s="1" t="n">
+      <c r="T179" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="U179" t="inlineStr">
@@ -14584,7 +14596,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K180" s="1" t="n">
+      <c r="K180" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="L180" t="inlineStr">
@@ -14657,7 +14669,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K181" s="1" t="n">
+      <c r="K181" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="L181" t="inlineStr">
@@ -14730,7 +14742,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K182" s="1" t="n">
+      <c r="K182" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="L182" t="inlineStr">
@@ -14803,7 +14815,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K183" s="1" t="n">
+      <c r="K183" s="2" t="n">
         <v>46121</v>
       </c>
       <c r="L183" t="inlineStr">
@@ -14876,7 +14888,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K184" s="1" t="n">
+      <c r="K184" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L184" t="inlineStr">
@@ -14949,7 +14961,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K185" s="1" t="n">
+      <c r="K185" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L185" t="inlineStr">
@@ -15022,7 +15034,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K186" s="1" t="n">
+      <c r="K186" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L186" t="inlineStr">
@@ -15095,7 +15107,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K187" s="1" t="n">
+      <c r="K187" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L187" t="inlineStr">
@@ -15168,7 +15180,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K188" s="1" t="n">
+      <c r="K188" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L188" t="inlineStr">
@@ -15241,7 +15253,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K189" s="1" t="n">
+      <c r="K189" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L189" t="inlineStr">
@@ -15314,7 +15326,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K190" s="1" t="n">
+      <c r="K190" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L190" t="inlineStr">
@@ -15387,7 +15399,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K191" s="1" t="n">
+      <c r="K191" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L191" t="inlineStr">
@@ -15460,7 +15472,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K192" s="1" t="n">
+      <c r="K192" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L192" t="inlineStr">
@@ -15533,7 +15545,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K193" s="1" t="n">
+      <c r="K193" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L193" t="inlineStr">
@@ -15606,7 +15618,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K194" s="1" t="n">
+      <c r="K194" s="2" t="n">
         <v>46122</v>
       </c>
       <c r="L194" t="inlineStr">
@@ -15679,7 +15691,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K195" s="1" t="n">
+      <c r="K195" s="2" t="n">
         <v>46126</v>
       </c>
       <c r="L195" t="inlineStr">
@@ -15754,7 +15766,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K196" s="1" t="n">
+      <c r="K196" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="L196" t="inlineStr">
@@ -15829,7 +15841,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K197" s="1" t="n">
+      <c r="K197" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="L197" t="inlineStr">
@@ -15900,7 +15912,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K198" s="1" t="n">
+      <c r="K198" s="2" t="n">
         <v>46128</v>
       </c>
       <c r="L198" t="inlineStr">
@@ -15971,7 +15983,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K199" s="1" t="n">
+      <c r="K199" s="2" t="n">
         <v>46129</v>
       </c>
       <c r="L199" t="inlineStr">
@@ -16042,7 +16054,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K200" s="1" t="n">
+      <c r="K200" s="2" t="n">
         <v>46135</v>
       </c>
       <c r="L200" t="inlineStr">
@@ -16113,7 +16125,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K201" s="1" t="n">
+      <c r="K201" s="2" t="n">
         <v>46139</v>
       </c>
       <c r="L201" t="inlineStr">
@@ -16184,7 +16196,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K202" s="1" t="n">
+      <c r="K202" s="2" t="n">
         <v>46139</v>
       </c>
       <c r="L202" t="inlineStr">
@@ -16255,7 +16267,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K203" s="1" t="n">
+      <c r="K203" s="2" t="n">
         <v>46139</v>
       </c>
       <c r="L203" t="inlineStr">
@@ -16326,7 +16338,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K204" s="1" t="n">
+      <c r="K204" s="2" t="n">
         <v>46139</v>
       </c>
       <c r="L204" t="inlineStr">
@@ -16401,7 +16413,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K205" s="1" t="n">
+      <c r="K205" s="2" t="n">
         <v>46139</v>
       </c>
       <c r="L205" t="inlineStr">
@@ -16476,7 +16488,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K206" s="1" t="n">
+      <c r="K206" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L206" t="inlineStr">
@@ -16547,7 +16559,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K207" s="1" t="n">
+      <c r="K207" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L207" t="inlineStr">
@@ -16618,7 +16630,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K208" s="1" t="n">
+      <c r="K208" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L208" t="inlineStr">
@@ -16689,7 +16701,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K209" s="1" t="n">
+      <c r="K209" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L209" t="inlineStr">
@@ -16760,7 +16772,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K210" s="1" t="n">
+      <c r="K210" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L210" t="inlineStr">
@@ -16831,7 +16843,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K211" s="1" t="n">
+      <c r="K211" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L211" t="inlineStr">
@@ -16902,7 +16914,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K212" s="1" t="n">
+      <c r="K212" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L212" t="inlineStr">
@@ -16973,7 +16985,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K213" s="1" t="n">
+      <c r="K213" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L213" t="inlineStr">
@@ -17044,7 +17056,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K214" s="1" t="n">
+      <c r="K214" s="2" t="n">
         <v>46141</v>
       </c>
       <c r="L214" t="inlineStr">
@@ -17115,7 +17127,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K215" s="1" t="n">
+      <c r="K215" s="2" t="n">
         <v>46142</v>
       </c>
       <c r="L215" t="inlineStr">
@@ -17186,7 +17198,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K216" s="1" t="n">
+      <c r="K216" s="2" t="n">
         <v>46146</v>
       </c>
       <c r="L216" t="inlineStr">
@@ -17257,7 +17269,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K217" s="1" t="n">
+      <c r="K217" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L217" t="inlineStr">
@@ -17328,7 +17340,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K218" s="1" t="n">
+      <c r="K218" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L218" t="inlineStr">
@@ -17399,7 +17411,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K219" s="1" t="n">
+      <c r="K219" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L219" t="inlineStr">
@@ -17470,7 +17482,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K220" s="1" t="n">
+      <c r="K220" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L220" t="inlineStr">
@@ -17541,7 +17553,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K221" s="1" t="n">
+      <c r="K221" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L221" t="inlineStr">
@@ -17612,7 +17624,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K222" s="1" t="n">
+      <c r="K222" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L222" t="inlineStr">
@@ -17683,7 +17695,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K223" s="1" t="n">
+      <c r="K223" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L223" t="inlineStr">
@@ -17754,7 +17766,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K224" s="1" t="n">
+      <c r="K224" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L224" t="inlineStr">
@@ -17825,7 +17837,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K225" s="1" t="n">
+      <c r="K225" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L225" t="inlineStr">
@@ -17896,7 +17908,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K226" s="1" t="n">
+      <c r="K226" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L226" t="inlineStr">
@@ -17967,7 +17979,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K227" s="1" t="n">
+      <c r="K227" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L227" t="inlineStr">
@@ -18038,7 +18050,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K228" s="1" t="n">
+      <c r="K228" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L228" t="inlineStr">
@@ -18109,7 +18121,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K229" s="1" t="n">
+      <c r="K229" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L229" t="inlineStr">
@@ -18180,7 +18192,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K230" s="1" t="n">
+      <c r="K230" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L230" t="inlineStr">
@@ -18251,7 +18263,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K231" s="1" t="n">
+      <c r="K231" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L231" t="inlineStr">
@@ -18322,7 +18334,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K232" s="1" t="n">
+      <c r="K232" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L232" t="inlineStr">
@@ -18393,7 +18405,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K233" s="1" t="n">
+      <c r="K233" s="2" t="n">
         <v>46148</v>
       </c>
       <c r="L233" t="inlineStr">
@@ -18464,7 +18476,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K234" s="1" t="n">
+      <c r="K234" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L234" t="inlineStr">
@@ -18535,7 +18547,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K235" s="1" t="n">
+      <c r="K235" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L235" t="inlineStr">
@@ -18606,7 +18618,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K236" s="1" t="n">
+      <c r="K236" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L236" t="inlineStr">
@@ -18677,7 +18689,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K237" s="1" t="n">
+      <c r="K237" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L237" t="inlineStr">
@@ -18748,7 +18760,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K238" s="1" t="n">
+      <c r="K238" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L238" t="inlineStr">
@@ -18819,7 +18831,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K239" s="1" t="n">
+      <c r="K239" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L239" t="inlineStr">
@@ -18890,7 +18902,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K240" s="1" t="n">
+      <c r="K240" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L240" t="inlineStr">
@@ -18961,7 +18973,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K241" s="1" t="n">
+      <c r="K241" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L241" t="inlineStr">
@@ -19032,7 +19044,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K242" s="1" t="n">
+      <c r="K242" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L242" t="inlineStr">
@@ -19103,7 +19115,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K243" s="1" t="n">
+      <c r="K243" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L243" t="inlineStr">
@@ -19174,7 +19186,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K244" s="1" t="n">
+      <c r="K244" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L244" t="inlineStr">
@@ -19245,7 +19257,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K245" s="1" t="n">
+      <c r="K245" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L245" t="inlineStr">
@@ -19316,7 +19328,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K246" s="1" t="n">
+      <c r="K246" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L246" t="inlineStr">
@@ -19387,7 +19399,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K247" s="1" t="n">
+      <c r="K247" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L247" t="inlineStr">
@@ -19458,7 +19470,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K248" s="1" t="n">
+      <c r="K248" s="2" t="n">
         <v>46149</v>
       </c>
       <c r="L248" t="inlineStr">
@@ -19529,7 +19541,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K249" s="1" t="n">
+      <c r="K249" s="2" t="n">
         <v>46150</v>
       </c>
       <c r="L249" t="inlineStr">
@@ -19600,7 +19612,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K250" s="1" t="n">
+      <c r="K250" s="2" t="n">
         <v>46155</v>
       </c>
       <c r="L250" t="inlineStr">
@@ -19671,7 +19683,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K251" s="1" t="n">
+      <c r="K251" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="L251" t="inlineStr">
@@ -19742,7 +19754,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K252" s="1" t="n">
+      <c r="K252" s="2" t="n">
         <v>46161</v>
       </c>
       <c r="L252" t="inlineStr">
@@ -19813,7 +19825,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K253" s="1" t="n">
+      <c r="K253" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="L253" t="inlineStr">
@@ -19888,7 +19900,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K254" s="1" t="n">
+      <c r="K254" s="2" t="n">
         <v>46162</v>
       </c>
       <c r="L254" t="inlineStr">
@@ -19959,7 +19971,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K255" s="1" t="n">
+      <c r="K255" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="L255" t="inlineStr">
@@ -20030,7 +20042,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K256" s="1" t="n">
+      <c r="K256" s="2" t="n">
         <v>46163</v>
       </c>
       <c r="L256" t="inlineStr">
@@ -20105,7 +20117,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K257" s="1" t="n">
+      <c r="K257" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="L257" t="inlineStr">
@@ -20124,7 +20136,7 @@
       <c r="Q257" t="inlineStr"/>
       <c r="R257" t="inlineStr"/>
       <c r="S257" t="inlineStr"/>
-      <c r="T257" s="1" t="n">
+      <c r="T257" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="U257" t="inlineStr">
@@ -20190,7 +20202,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K258" s="1" t="n">
+      <c r="K258" s="2" t="n">
         <v>46170</v>
       </c>
       <c r="L258" t="inlineStr">
@@ -20265,7 +20277,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K259" s="1" t="n">
+      <c r="K259" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="L259" t="inlineStr">
@@ -20340,7 +20352,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K260" s="1" t="n">
+      <c r="K260" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="L260" t="inlineStr">
@@ -20359,7 +20371,7 @@
       <c r="Q260" t="inlineStr"/>
       <c r="R260" t="inlineStr"/>
       <c r="S260" t="inlineStr"/>
-      <c r="T260" s="1" t="n">
+      <c r="T260" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="U260" t="inlineStr">
@@ -20425,7 +20437,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K261" s="1" t="n">
+      <c r="K261" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="L261" t="inlineStr">
@@ -20500,7 +20512,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K262" s="1" t="n">
+      <c r="K262" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="L262" t="inlineStr">
@@ -20575,7 +20587,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K263" s="1" t="n">
+      <c r="K263" s="2" t="n">
         <v>46171</v>
       </c>
       <c r="L263" t="inlineStr">
@@ -20594,7 +20606,7 @@
       <c r="Q263" t="inlineStr"/>
       <c r="R263" t="inlineStr"/>
       <c r="S263" t="inlineStr"/>
-      <c r="T263" s="1" t="n">
+      <c r="T263" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="U263" t="inlineStr">
@@ -20660,7 +20672,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K264" s="1" t="n">
+      <c r="K264" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L264" t="inlineStr">
@@ -20731,7 +20743,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K265" s="1" t="n">
+      <c r="K265" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L265" t="inlineStr">
@@ -20802,7 +20814,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K266" s="1" t="n">
+      <c r="K266" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L266" t="inlineStr">
@@ -20873,7 +20885,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K267" s="1" t="n">
+      <c r="K267" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L267" t="inlineStr">
@@ -20948,7 +20960,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K268" s="1" t="n">
+      <c r="K268" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L268" t="inlineStr">
@@ -21019,7 +21031,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K269" s="1" t="n">
+      <c r="K269" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L269" t="inlineStr">
@@ -21090,7 +21102,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K270" s="1" t="n">
+      <c r="K270" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L270" t="inlineStr">
@@ -21161,7 +21173,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K271" s="1" t="n">
+      <c r="K271" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L271" t="inlineStr">
@@ -21232,7 +21244,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K272" s="1" t="n">
+      <c r="K272" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L272" t="inlineStr">
@@ -21307,7 +21319,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K273" s="1" t="n">
+      <c r="K273" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L273" t="inlineStr">
@@ -21382,7 +21394,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K274" s="1" t="n">
+      <c r="K274" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L274" t="inlineStr">
@@ -21453,7 +21465,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K275" s="1" t="n">
+      <c r="K275" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L275" t="inlineStr">
@@ -21524,7 +21536,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K276" s="1" t="n">
+      <c r="K276" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L276" t="inlineStr">
@@ -21595,7 +21607,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K277" s="1" t="n">
+      <c r="K277" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L277" t="inlineStr">
@@ -21666,7 +21678,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K278" s="1" t="n">
+      <c r="K278" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L278" t="inlineStr">
@@ -21737,7 +21749,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K279" s="1" t="n">
+      <c r="K279" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L279" t="inlineStr">
@@ -21808,7 +21820,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K280" s="1" t="n">
+      <c r="K280" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L280" t="inlineStr">
@@ -21879,7 +21891,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K281" s="1" t="n">
+      <c r="K281" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L281" t="inlineStr">
@@ -21950,7 +21962,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K282" s="1" t="n">
+      <c r="K282" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L282" t="inlineStr">
@@ -22021,7 +22033,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K283" s="1" t="n">
+      <c r="K283" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L283" t="inlineStr">
@@ -22092,7 +22104,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K284" s="1" t="n">
+      <c r="K284" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L284" t="inlineStr">
@@ -22163,7 +22175,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K285" s="1" t="n">
+      <c r="K285" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L285" t="inlineStr">
@@ -22234,7 +22246,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K286" s="1" t="n">
+      <c r="K286" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L286" t="inlineStr">
@@ -22305,7 +22317,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K287" s="1" t="n">
+      <c r="K287" s="2" t="n">
         <v>46174</v>
       </c>
       <c r="L287" t="inlineStr">
@@ -22376,7 +22388,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K288" s="1" t="n">
+      <c r="K288" s="2" t="n">
         <v>46176</v>
       </c>
       <c r="L288" t="inlineStr">
@@ -22447,7 +22459,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K289" s="1" t="n">
+      <c r="K289" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="L289" t="inlineStr">
@@ -22518,7 +22530,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K290" s="1" t="n">
+      <c r="K290" s="2" t="n">
         <v>46182</v>
       </c>
       <c r="L290" t="inlineStr">
@@ -22589,7 +22601,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K291" s="1" t="n">
+      <c r="K291" s="2" t="n">
         <v>46183</v>
       </c>
       <c r="L291" t="inlineStr">
@@ -22660,7 +22672,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K292" s="1" t="n">
+      <c r="K292" s="2" t="n">
         <v>46185</v>
       </c>
       <c r="L292" t="inlineStr">
@@ -22731,7 +22743,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K293" s="1" t="n">
+      <c r="K293" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L293" t="inlineStr">
@@ -22802,7 +22814,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K294" s="1" t="n">
+      <c r="K294" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L294" t="inlineStr">
@@ -22873,7 +22885,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K295" s="1" t="n">
+      <c r="K295" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L295" t="inlineStr">
@@ -22948,7 +22960,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K296" s="1" t="n">
+      <c r="K296" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L296" t="inlineStr">
@@ -23023,7 +23035,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K297" s="1" t="n">
+      <c r="K297" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L297" t="inlineStr">
@@ -23094,7 +23106,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K298" s="1" t="n">
+      <c r="K298" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L298" t="inlineStr">
@@ -23165,7 +23177,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K299" s="1" t="n">
+      <c r="K299" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L299" t="inlineStr">
@@ -23236,7 +23248,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K300" s="1" t="n">
+      <c r="K300" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L300" t="inlineStr">
@@ -23307,7 +23319,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K301" s="1" t="n">
+      <c r="K301" s="2" t="n">
         <v>46192</v>
       </c>
       <c r="L301" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (11/07/2026 07:21)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -20,16 +20,13 @@
     <numFmt numFmtId="164" formatCode="yyyy-mm-dd h:mm:ss"/>
     <numFmt numFmtId="165" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
       <name val="Calibri"/>
       <family val="2"/>
       <color theme="1"/>
       <sz val="11"/>
       <scheme val="minor"/>
-    </font>
-    <font>
-      <b val="1"/>
     </font>
   </fonts>
   <fills count="2">
@@ -40,7 +37,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -48,21 +45,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="165" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -433,117 +421,117 @@
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
-      <c r="A1" s="1" t="inlineStr">
+      <c r="A1" t="inlineStr">
         <is>
           <t>numero_ordem</t>
         </is>
       </c>
-      <c r="B1" s="1" t="inlineStr">
+      <c r="B1" t="inlineStr">
         <is>
           <t>part_number</t>
         </is>
       </c>
-      <c r="C1" s="1" t="inlineStr">
+      <c r="C1" t="inlineStr">
         <is>
           <t>descricao</t>
         </is>
       </c>
-      <c r="D1" s="1" t="inlineStr">
+      <c r="D1" t="inlineStr">
         <is>
           <t>sn_lt</t>
         </is>
       </c>
-      <c r="E1" s="1" t="inlineStr">
+      <c r="E1" t="inlineStr">
         <is>
           <t>categoria</t>
         </is>
       </c>
-      <c r="F1" s="1" t="inlineStr">
+      <c r="F1" t="inlineStr">
         <is>
           <t>quantidade_texto</t>
         </is>
       </c>
-      <c r="G1" s="1" t="inlineStr">
+      <c r="G1" t="inlineStr">
         <is>
           <t>quantidade</t>
         </is>
       </c>
-      <c r="H1" s="1" t="inlineStr">
+      <c r="H1" t="inlineStr">
         <is>
           <t>pedido_emg</t>
         </is>
       </c>
-      <c r="I1" s="1" t="inlineStr">
+      <c r="I1" t="inlineStr">
         <is>
           <t>motivo</t>
         </is>
       </c>
-      <c r="J1" s="1" t="inlineStr">
+      <c r="J1" t="inlineStr">
         <is>
           <t>pj</t>
         </is>
       </c>
-      <c r="K1" s="1" t="inlineStr">
+      <c r="K1" t="inlineStr">
         <is>
           <t>pedido_envio</t>
         </is>
       </c>
-      <c r="L1" s="1" t="inlineStr">
+      <c r="L1" t="inlineStr">
         <is>
           <t>anv</t>
         </is>
       </c>
-      <c r="M1" s="1" t="inlineStr">
+      <c r="M1" t="inlineStr">
         <is>
           <t>destino</t>
         </is>
       </c>
-      <c r="N1" s="1" t="inlineStr">
+      <c r="N1" t="inlineStr">
         <is>
           <t>nf_gmm</t>
         </is>
       </c>
-      <c r="O1" s="1" t="inlineStr">
+      <c r="O1" t="inlineStr">
         <is>
           <t>rastreio</t>
         </is>
       </c>
-      <c r="P1" s="1" t="inlineStr">
+      <c r="P1" t="inlineStr">
         <is>
           <t>pn_devolvido</t>
         </is>
       </c>
-      <c r="Q1" s="1" t="inlineStr">
+      <c r="Q1" t="inlineStr">
         <is>
           <t>detalhe_entrega</t>
         </is>
       </c>
-      <c r="R1" s="1" t="inlineStr">
+      <c r="R1" t="inlineStr">
         <is>
           <t>numero_rc</t>
         </is>
       </c>
-      <c r="S1" s="1" t="inlineStr">
+      <c r="S1" t="inlineStr">
         <is>
           <t>nf_devolucao_vee_one</t>
         </is>
       </c>
-      <c r="T1" s="1" t="inlineStr">
+      <c r="T1" t="inlineStr">
         <is>
           <t>data_devolucao</t>
         </is>
       </c>
-      <c r="U1" s="1" t="inlineStr">
+      <c r="U1" t="inlineStr">
         <is>
           <t>observacao_fiscal</t>
         </is>
       </c>
-      <c r="V1" s="1" t="inlineStr">
+      <c r="V1" t="inlineStr">
         <is>
           <t>observacao_empresa</t>
         </is>
       </c>
-      <c r="W1" s="1" t="inlineStr">
+      <c r="W1" t="inlineStr">
         <is>
           <t>status</t>
         </is>
@@ -598,7 +586,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K2" s="2" t="n">
+      <c r="K2" s="1" t="n">
         <v>45730</v>
       </c>
       <c r="L2" t="inlineStr">
@@ -675,7 +663,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K3" s="2" t="n">
+      <c r="K3" s="1" t="n">
         <v>45735</v>
       </c>
       <c r="L3" t="inlineStr">
@@ -752,7 +740,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K4" s="2" t="n">
+      <c r="K4" s="1" t="n">
         <v>45737</v>
       </c>
       <c r="L4" t="inlineStr">
@@ -829,7 +817,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K5" s="2" t="n">
+      <c r="K5" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L5" t="inlineStr">
@@ -914,7 +902,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K6" s="2" t="n">
+      <c r="K6" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L6" t="inlineStr">
@@ -995,7 +983,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K7" s="2" t="n">
+      <c r="K7" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L7" t="inlineStr">
@@ -1076,7 +1064,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K8" s="2" t="n">
+      <c r="K8" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L8" t="inlineStr">
@@ -1157,7 +1145,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K9" s="2" t="n">
+      <c r="K9" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L9" t="inlineStr">
@@ -1238,7 +1226,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K10" s="2" t="n">
+      <c r="K10" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L10" t="inlineStr">
@@ -1319,7 +1307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K11" s="2" t="n">
+      <c r="K11" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L11" t="inlineStr">
@@ -1400,7 +1388,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K12" s="2" t="n">
+      <c r="K12" s="1" t="n">
         <v>45747</v>
       </c>
       <c r="L12" t="inlineStr">
@@ -1477,7 +1465,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K13" s="2" t="n">
+      <c r="K13" s="1" t="n">
         <v>45762</v>
       </c>
       <c r="L13" t="inlineStr">
@@ -1554,7 +1542,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K14" s="2" t="n">
+      <c r="K14" s="1" t="n">
         <v>45763</v>
       </c>
       <c r="L14" t="inlineStr">
@@ -1631,7 +1619,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K15" s="2" t="n">
+      <c r="K15" s="1" t="n">
         <v>45763</v>
       </c>
       <c r="L15" t="inlineStr">
@@ -1708,7 +1696,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K16" s="2" t="n">
+      <c r="K16" s="1" t="n">
         <v>45783</v>
       </c>
       <c r="L16" t="inlineStr">
@@ -1785,7 +1773,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K17" s="2" t="n">
+      <c r="K17" s="1" t="n">
         <v>45783</v>
       </c>
       <c r="L17" t="inlineStr">
@@ -1862,7 +1850,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K18" s="2" t="n">
+      <c r="K18" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L18" t="inlineStr">
@@ -1893,7 +1881,7 @@
         </is>
       </c>
       <c r="S18" t="inlineStr"/>
-      <c r="T18" s="2" t="n">
+      <c r="T18" s="1" t="n">
         <v>45845</v>
       </c>
       <c r="U18" t="inlineStr">
@@ -1957,7 +1945,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K19" s="2" t="n">
+      <c r="K19" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L19" t="inlineStr">
@@ -2034,7 +2022,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K20" s="2" t="n">
+      <c r="K20" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L20" t="inlineStr">
@@ -2111,7 +2099,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K21" s="2" t="n">
+      <c r="K21" s="1" t="n">
         <v>45784</v>
       </c>
       <c r="L21" t="inlineStr">
@@ -2142,7 +2130,7 @@
         </is>
       </c>
       <c r="S21" t="inlineStr"/>
-      <c r="T21" s="2" t="n">
+      <c r="T21" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="U21" t="inlineStr">
@@ -2206,7 +2194,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K22" s="2" t="n">
+      <c r="K22" s="1" t="n">
         <v>45789</v>
       </c>
       <c r="L22" t="inlineStr">
@@ -2237,7 +2225,7 @@
         </is>
       </c>
       <c r="S22" t="inlineStr"/>
-      <c r="T22" s="2" t="n">
+      <c r="T22" s="1" t="n">
         <v>45868</v>
       </c>
       <c r="U22" t="inlineStr">
@@ -2301,7 +2289,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K23" s="2" t="n">
+      <c r="K23" s="1" t="n">
         <v>45789</v>
       </c>
       <c r="L23" t="inlineStr">
@@ -2332,7 +2320,7 @@
         </is>
       </c>
       <c r="S23" t="inlineStr"/>
-      <c r="T23" s="2" t="n">
+      <c r="T23" s="1" t="n">
         <v>45982</v>
       </c>
       <c r="U23" t="inlineStr">
@@ -2396,7 +2384,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K24" s="2" t="n">
+      <c r="K24" s="1" t="n">
         <v>45791</v>
       </c>
       <c r="L24" t="inlineStr">
@@ -2473,7 +2461,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K25" s="2" t="n">
+      <c r="K25" s="1" t="n">
         <v>45814</v>
       </c>
       <c r="L25" t="inlineStr">
@@ -2546,7 +2534,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K26" s="2" t="n">
+      <c r="K26" s="1" t="n">
         <v>45819</v>
       </c>
       <c r="L26" t="inlineStr">
@@ -2619,7 +2607,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K27" s="2" t="n">
+      <c r="K27" s="1" t="n">
         <v>45821</v>
       </c>
       <c r="L27" t="inlineStr">
@@ -2650,7 +2638,7 @@
         </is>
       </c>
       <c r="S27" t="inlineStr"/>
-      <c r="T27" s="2" t="n">
+      <c r="T27" s="1" t="n">
         <v>45876</v>
       </c>
       <c r="U27" t="inlineStr">
@@ -2714,7 +2702,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K28" s="2" t="n">
+      <c r="K28" s="1" t="n">
         <v>45824</v>
       </c>
       <c r="L28" t="inlineStr">
@@ -2791,7 +2779,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K29" s="2" t="n">
+      <c r="K29" s="1" t="n">
         <v>45825</v>
       </c>
       <c r="L29" t="inlineStr">
@@ -2868,7 +2856,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K30" s="2" t="n">
+      <c r="K30" s="1" t="n">
         <v>45836</v>
       </c>
       <c r="L30" t="inlineStr">
@@ -2945,7 +2933,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K31" s="2" t="n">
+      <c r="K31" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="L31" t="inlineStr">
@@ -2976,7 +2964,7 @@
         </is>
       </c>
       <c r="S31" t="inlineStr"/>
-      <c r="T31" s="2" t="n">
+      <c r="T31" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U31" t="inlineStr">
@@ -3040,7 +3028,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K32" s="2" t="n">
+      <c r="K32" s="1" t="n">
         <v>45839</v>
       </c>
       <c r="L32" t="inlineStr">
@@ -3117,7 +3105,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K33" s="2" t="n">
+      <c r="K33" s="1" t="n">
         <v>45845</v>
       </c>
       <c r="L33" t="inlineStr">
@@ -3148,7 +3136,7 @@
         </is>
       </c>
       <c r="S33" t="inlineStr"/>
-      <c r="T33" s="2" t="n">
+      <c r="T33" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U33" t="inlineStr">
@@ -3212,7 +3200,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K34" s="2" t="n">
+      <c r="K34" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L34" t="inlineStr">
@@ -3289,7 +3277,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K35" s="2" t="n">
+      <c r="K35" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L35" t="inlineStr">
@@ -3320,7 +3308,7 @@
         </is>
       </c>
       <c r="S35" t="inlineStr"/>
-      <c r="T35" s="2" t="n">
+      <c r="T35" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U35" t="inlineStr">
@@ -3384,7 +3372,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K36" s="2" t="n">
+      <c r="K36" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L36" t="inlineStr">
@@ -3415,7 +3403,7 @@
         </is>
       </c>
       <c r="S36" t="inlineStr"/>
-      <c r="T36" s="2" t="n">
+      <c r="T36" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U36" t="inlineStr">
@@ -3479,7 +3467,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K37" s="2" t="n">
+      <c r="K37" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L37" t="inlineStr">
@@ -3510,7 +3498,7 @@
         </is>
       </c>
       <c r="S37" t="inlineStr"/>
-      <c r="T37" s="2" t="n">
+      <c r="T37" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U37" t="inlineStr">
@@ -3574,7 +3562,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K38" s="2" t="n">
+      <c r="K38" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L38" t="inlineStr">
@@ -3605,7 +3593,7 @@
         </is>
       </c>
       <c r="S38" t="inlineStr"/>
-      <c r="T38" s="2" t="n">
+      <c r="T38" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U38" t="inlineStr">
@@ -3669,7 +3657,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K39" s="2" t="n">
+      <c r="K39" s="1" t="n">
         <v>45856</v>
       </c>
       <c r="L39" t="inlineStr">
@@ -3700,7 +3688,7 @@
         </is>
       </c>
       <c r="S39" t="inlineStr"/>
-      <c r="T39" s="2" t="n">
+      <c r="T39" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U39" t="inlineStr">
@@ -3764,7 +3752,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K40" s="2" t="n">
+      <c r="K40" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L40" t="inlineStr">
@@ -3795,7 +3783,7 @@
         </is>
       </c>
       <c r="S40" t="inlineStr"/>
-      <c r="T40" s="2" t="n">
+      <c r="T40" s="1" t="n">
         <v>45916</v>
       </c>
       <c r="U40" t="inlineStr">
@@ -3859,7 +3847,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K41" s="2" t="n">
+      <c r="K41" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L41" t="inlineStr">
@@ -3936,7 +3924,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K42" s="2" t="n">
+      <c r="K42" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L42" t="inlineStr">
@@ -3967,7 +3955,7 @@
         </is>
       </c>
       <c r="S42" t="inlineStr"/>
-      <c r="T42" s="2" t="n">
+      <c r="T42" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="U42" t="inlineStr">
@@ -4031,7 +4019,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K43" s="2" t="n">
+      <c r="K43" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L43" t="inlineStr">
@@ -4108,7 +4096,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K44" s="2" t="n">
+      <c r="K44" s="1" t="n">
         <v>45866</v>
       </c>
       <c r="L44" t="inlineStr">
@@ -4139,7 +4127,7 @@
         </is>
       </c>
       <c r="S44" t="inlineStr"/>
-      <c r="T44" s="2" t="n">
+      <c r="T44" s="1" t="n">
         <v>46002</v>
       </c>
       <c r="U44" t="inlineStr">
@@ -4203,7 +4191,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K45" s="2" t="n">
+      <c r="K45" s="1" t="n">
         <v>45882</v>
       </c>
       <c r="L45" t="inlineStr">
@@ -4280,7 +4268,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K46" s="2" t="n">
+      <c r="K46" s="1" t="n">
         <v>45882</v>
       </c>
       <c r="L46" t="inlineStr">
@@ -4357,7 +4345,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K47" s="2" t="n">
+      <c r="K47" s="1" t="n">
         <v>45890</v>
       </c>
       <c r="L47" t="inlineStr">
@@ -4388,7 +4376,7 @@
         </is>
       </c>
       <c r="S47" t="inlineStr"/>
-      <c r="T47" s="2" t="n">
+      <c r="T47" s="1" t="n">
         <v>45944</v>
       </c>
       <c r="U47" t="inlineStr">
@@ -4452,7 +4440,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K48" s="2" t="n">
+      <c r="K48" s="1" t="n">
         <v>45903</v>
       </c>
       <c r="L48" t="inlineStr">
@@ -4529,7 +4517,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K49" s="2" t="n">
+      <c r="K49" s="1" t="n">
         <v>45904</v>
       </c>
       <c r="L49" t="inlineStr">
@@ -4606,7 +4594,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K50" s="2" t="n">
+      <c r="K50" s="1" t="n">
         <v>45912</v>
       </c>
       <c r="L50" t="inlineStr">
@@ -4683,7 +4671,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K51" s="2" t="n">
+      <c r="K51" s="1" t="n">
         <v>45925</v>
       </c>
       <c r="L51" t="inlineStr">
@@ -4764,7 +4752,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K52" s="2" t="n">
+      <c r="K52" s="1" t="n">
         <v>45924</v>
       </c>
       <c r="L52" t="inlineStr">
@@ -4841,7 +4829,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K53" s="2" t="n">
+      <c r="K53" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="L53" t="inlineStr">
@@ -4918,7 +4906,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K54" s="2" t="n">
+      <c r="K54" s="1" t="n">
         <v>45930</v>
       </c>
       <c r="L54" t="inlineStr">
@@ -4995,7 +4983,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K55" s="2" t="n">
+      <c r="K55" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L55" t="inlineStr">
@@ -5080,7 +5068,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K56" s="2" t="n">
+      <c r="K56" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L56" t="inlineStr">
@@ -5169,7 +5157,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K57" s="2" t="n">
+      <c r="K57" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L57" t="inlineStr">
@@ -5254,7 +5242,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K58" s="2" t="n">
+      <c r="K58" s="1" t="n">
         <v>45931</v>
       </c>
       <c r="L58" t="inlineStr">
@@ -5339,7 +5327,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K59" s="2" t="n">
+      <c r="K59" s="1" t="n">
         <v>45937</v>
       </c>
       <c r="L59" t="inlineStr">
@@ -5370,7 +5358,7 @@
         </is>
       </c>
       <c r="S59" t="inlineStr"/>
-      <c r="T59" s="2" t="n">
+      <c r="T59" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="U59" t="inlineStr">
@@ -5434,7 +5422,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K60" s="2" t="n">
+      <c r="K60" s="1" t="n">
         <v>45938</v>
       </c>
       <c r="L60" t="inlineStr">
@@ -5511,7 +5499,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K61" s="2" t="n">
+      <c r="K61" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="L61" t="inlineStr">
@@ -5588,7 +5576,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K62" s="2" t="n">
+      <c r="K62" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="L62" t="inlineStr">
@@ -5665,7 +5653,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K63" s="2" t="n">
+      <c r="K63" s="1" t="n">
         <v>45939</v>
       </c>
       <c r="L63" t="inlineStr">
@@ -5742,7 +5730,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K64" s="2" t="n">
+      <c r="K64" s="1" t="n">
         <v>45940</v>
       </c>
       <c r="L64" t="inlineStr">
@@ -5819,7 +5807,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K65" s="2" t="n">
+      <c r="K65" s="1" t="n">
         <v>45943</v>
       </c>
       <c r="L65" t="inlineStr">
@@ -5900,7 +5888,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K66" s="2" t="n">
+      <c r="K66" s="1" t="n">
         <v>45943</v>
       </c>
       <c r="L66" t="inlineStr">
@@ -5977,7 +5965,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K67" s="2" t="n">
+      <c r="K67" s="1" t="n">
         <v>45943</v>
       </c>
       <c r="L67" t="inlineStr">
@@ -6054,7 +6042,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K68" s="2" t="n">
+      <c r="K68" s="1" t="n">
         <v>45961</v>
       </c>
       <c r="L68" t="inlineStr">
@@ -6081,7 +6069,7 @@
       <c r="Q68" t="inlineStr"/>
       <c r="R68" t="inlineStr"/>
       <c r="S68" t="inlineStr"/>
-      <c r="T68" s="2" t="n">
+      <c r="T68" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U68" t="inlineStr">
@@ -6149,7 +6137,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K69" s="2" t="n">
+      <c r="K69" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="L69" t="inlineStr">
@@ -6226,7 +6214,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K70" s="2" t="n">
+      <c r="K70" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="L70" t="inlineStr">
@@ -6303,7 +6291,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K71" s="2" t="n">
+      <c r="K71" s="1" t="n">
         <v>45965</v>
       </c>
       <c r="L71" t="inlineStr">
@@ -6380,7 +6368,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K72" s="2" t="n">
+      <c r="K72" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L72" t="inlineStr">
@@ -6457,7 +6445,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K73" s="2" t="n">
+      <c r="K73" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L73" t="inlineStr">
@@ -6534,7 +6522,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K74" s="2" t="n">
+      <c r="K74" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L74" t="inlineStr">
@@ -6611,7 +6599,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K75" s="2" t="n">
+      <c r="K75" s="1" t="n">
         <v>45967</v>
       </c>
       <c r="L75" t="inlineStr">
@@ -6688,7 +6676,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K76" s="2" t="n">
+      <c r="K76" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L76" t="inlineStr">
@@ -6765,7 +6753,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K77" s="2" t="n">
+      <c r="K77" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L77" t="inlineStr">
@@ -6842,7 +6830,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K78" s="2" t="n">
+      <c r="K78" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L78" t="inlineStr">
@@ -6919,7 +6907,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K79" s="2" t="n">
+      <c r="K79" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L79" t="inlineStr">
@@ -6996,7 +6984,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K80" s="2" t="n">
+      <c r="K80" s="1" t="n">
         <v>45968</v>
       </c>
       <c r="L80" t="inlineStr">
@@ -7073,7 +7061,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K81" s="2" t="n">
+      <c r="K81" s="1" t="n">
         <v>45973</v>
       </c>
       <c r="L81" t="inlineStr">
@@ -7150,7 +7138,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K82" s="2" t="n">
+      <c r="K82" s="1" t="n">
         <v>45974</v>
       </c>
       <c r="L82" t="inlineStr">
@@ -7227,7 +7215,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K83" s="2" t="n">
+      <c r="K83" s="1" t="n">
         <v>45975</v>
       </c>
       <c r="L83" t="inlineStr">
@@ -7304,7 +7292,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K84" s="2" t="n">
+      <c r="K84" s="1" t="n">
         <v>45975</v>
       </c>
       <c r="L84" t="inlineStr">
@@ -7381,7 +7369,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K85" s="2" t="n">
+      <c r="K85" s="1" t="n">
         <v>45982</v>
       </c>
       <c r="L85" t="inlineStr">
@@ -7458,7 +7446,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K86" s="2" t="n">
+      <c r="K86" s="1" t="n">
         <v>45982</v>
       </c>
       <c r="L86" t="inlineStr">
@@ -7535,7 +7523,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K87" s="2" t="n">
+      <c r="K87" s="1" t="n">
         <v>45985</v>
       </c>
       <c r="L87" t="inlineStr">
@@ -7612,7 +7600,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K88" s="2" t="n">
+      <c r="K88" s="1" t="n">
         <v>45985</v>
       </c>
       <c r="L88" t="inlineStr">
@@ -7689,7 +7677,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K89" s="2" t="n">
+      <c r="K89" s="1" t="n">
         <v>45986</v>
       </c>
       <c r="L89" t="inlineStr">
@@ -7762,7 +7750,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K90" s="2" t="n">
+      <c r="K90" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="L90" t="inlineStr">
@@ -7835,7 +7823,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K91" s="2" t="n">
+      <c r="K91" s="1" t="n">
         <v>45992</v>
       </c>
       <c r="L91" t="inlineStr">
@@ -7912,7 +7900,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K92" s="2" t="n">
+      <c r="K92" s="1" t="n">
         <v>45996</v>
       </c>
       <c r="L92" t="inlineStr">
@@ -7947,7 +7935,7 @@
         </is>
       </c>
       <c r="S92" t="inlineStr"/>
-      <c r="T92" s="2" t="n">
+      <c r="T92" s="1" t="n">
         <v>45979</v>
       </c>
       <c r="U92" t="inlineStr">
@@ -8011,7 +7999,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K93" s="2" t="n">
+      <c r="K93" s="1" t="n">
         <v>46002</v>
       </c>
       <c r="L93" t="inlineStr">
@@ -8084,7 +8072,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K94" s="2" t="n">
+      <c r="K94" s="1" t="n">
         <v>46007</v>
       </c>
       <c r="L94" t="inlineStr">
@@ -8161,7 +8149,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K95" s="2" t="n">
+      <c r="K95" s="1" t="n">
         <v>46007</v>
       </c>
       <c r="L95" t="inlineStr">
@@ -8238,7 +8226,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K96" s="2" t="n">
+      <c r="K96" s="1" t="n">
         <v>46008</v>
       </c>
       <c r="L96" t="inlineStr">
@@ -8319,7 +8307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K97" s="2" t="n">
+      <c r="K97" s="1" t="n">
         <v>46029</v>
       </c>
       <c r="L97" t="inlineStr">
@@ -8346,7 +8334,7 @@
         </is>
       </c>
       <c r="S97" t="inlineStr"/>
-      <c r="T97" s="2" t="n">
+      <c r="T97" s="1" t="n">
         <v>46030</v>
       </c>
       <c r="U97" t="inlineStr">
@@ -8410,7 +8398,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K98" s="2" t="n">
+      <c r="K98" s="1" t="n">
         <v>46029</v>
       </c>
       <c r="L98" t="inlineStr">
@@ -8487,7 +8475,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K99" s="2" t="n">
+      <c r="K99" s="1" t="n">
         <v>46034</v>
       </c>
       <c r="L99" t="inlineStr">
@@ -8564,7 +8552,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K100" s="2" t="n">
+      <c r="K100" s="1" t="n">
         <v>46034</v>
       </c>
       <c r="L100" t="inlineStr">
@@ -8637,7 +8625,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K101" s="2" t="n">
+      <c r="K101" s="1" t="n">
         <v>46035</v>
       </c>
       <c r="L101" t="inlineStr">
@@ -8710,7 +8698,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K102" s="2" t="n">
+      <c r="K102" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L102" t="inlineStr">
@@ -8783,7 +8771,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K103" s="2" t="n">
+      <c r="K103" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L103" t="inlineStr">
@@ -8856,7 +8844,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K104" s="2" t="n">
+      <c r="K104" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L104" t="inlineStr">
@@ -8929,7 +8917,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K105" s="2" t="n">
+      <c r="K105" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L105" t="inlineStr">
@@ -9002,7 +8990,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K106" s="2" t="n">
+      <c r="K106" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L106" t="inlineStr">
@@ -9075,7 +9063,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K107" s="2" t="n">
+      <c r="K107" s="1" t="n">
         <v>46036</v>
       </c>
       <c r="L107" t="inlineStr">
@@ -9148,7 +9136,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K108" s="2" t="n">
+      <c r="K108" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L108" t="inlineStr">
@@ -9221,7 +9209,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K109" s="2" t="n">
+      <c r="K109" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L109" t="inlineStr">
@@ -9294,7 +9282,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K110" s="2" t="n">
+      <c r="K110" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L110" t="inlineStr">
@@ -9325,7 +9313,7 @@
         </is>
       </c>
       <c r="S110" t="inlineStr"/>
-      <c r="T110" s="2" t="n">
+      <c r="T110" s="1" t="n">
         <v>45805</v>
       </c>
       <c r="U110" t="inlineStr">
@@ -9385,7 +9373,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K111" s="2" t="n">
+      <c r="K111" s="1" t="n">
         <v>46043</v>
       </c>
       <c r="L111" t="inlineStr">
@@ -9416,7 +9404,7 @@
         </is>
       </c>
       <c r="S111" t="inlineStr"/>
-      <c r="T111" s="2" t="n">
+      <c r="T111" s="1" t="n">
         <v>45959</v>
       </c>
       <c r="U111" t="inlineStr">
@@ -9476,7 +9464,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K112" s="2" t="n">
+      <c r="K112" s="1" t="n">
         <v>46044</v>
       </c>
       <c r="L112" t="inlineStr">
@@ -9507,7 +9495,7 @@
         </is>
       </c>
       <c r="S112" t="inlineStr"/>
-      <c r="T112" s="2" t="n">
+      <c r="T112" s="1" t="n">
         <v>46052</v>
       </c>
       <c r="U112" t="inlineStr">
@@ -9571,7 +9559,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K113" s="2" t="n">
+      <c r="K113" s="1" t="n">
         <v>46049</v>
       </c>
       <c r="L113" t="inlineStr">
@@ -9648,7 +9636,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K114" s="2" t="n">
+      <c r="K114" s="1" t="n">
         <v>46049</v>
       </c>
       <c r="L114" t="inlineStr">
@@ -9725,7 +9713,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K115" s="2" t="n">
+      <c r="K115" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="L115" t="inlineStr">
@@ -9802,7 +9790,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K116" s="2" t="n">
+      <c r="K116" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="L116" t="inlineStr">
@@ -9833,7 +9821,7 @@
         </is>
       </c>
       <c r="S116" t="inlineStr"/>
-      <c r="T116" s="2" t="n">
+      <c r="T116" s="1" t="n">
         <v>46048</v>
       </c>
       <c r="U116" t="inlineStr">
@@ -9897,7 +9885,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K117" s="2" t="n">
+      <c r="K117" s="1" t="n">
         <v>46050</v>
       </c>
       <c r="L117" t="inlineStr">
@@ -9974,7 +9962,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K118" s="2" t="n">
+      <c r="K118" s="1" t="n">
         <v>46063</v>
       </c>
       <c r="L118" t="inlineStr">
@@ -10055,7 +10043,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K119" s="2" t="n">
+      <c r="K119" s="1" t="n">
         <v>46028</v>
       </c>
       <c r="L119" t="inlineStr">
@@ -10126,7 +10114,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K120" s="2" t="n">
+      <c r="K120" s="1" t="n">
         <v>46062</v>
       </c>
       <c r="L120" t="inlineStr">
@@ -10203,7 +10191,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K121" s="2" t="n">
+      <c r="K121" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L121" t="inlineStr">
@@ -10280,7 +10268,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K122" s="2" t="n">
+      <c r="K122" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L122" t="inlineStr">
@@ -10365,7 +10353,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K123" s="2" t="n">
+      <c r="K123" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L123" t="inlineStr">
@@ -10442,7 +10430,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K124" s="2" t="n">
+      <c r="K124" s="1" t="n">
         <v>46065</v>
       </c>
       <c r="L124" t="inlineStr">
@@ -10519,7 +10507,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K125" s="2" t="n">
+      <c r="K125" s="1" t="n">
         <v>46066</v>
       </c>
       <c r="L125" t="inlineStr">
@@ -10592,7 +10580,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K126" s="2" t="n">
+      <c r="K126" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L126" t="inlineStr">
@@ -10665,7 +10653,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K127" s="2" t="n">
+      <c r="K127" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L127" t="inlineStr">
@@ -10696,7 +10684,7 @@
         </is>
       </c>
       <c r="S127" t="inlineStr"/>
-      <c r="T127" s="2" t="n">
+      <c r="T127" s="1" t="n">
         <v>45889</v>
       </c>
       <c r="U127" t="inlineStr">
@@ -10756,7 +10744,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K128" s="2" t="n">
+      <c r="K128" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L128" t="inlineStr">
@@ -10829,7 +10817,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K129" s="2" t="n">
+      <c r="K129" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L129" t="inlineStr">
@@ -10902,7 +10890,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K130" s="2" t="n">
+      <c r="K130" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L130" t="inlineStr">
@@ -10975,7 +10963,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K131" s="2" t="n">
+      <c r="K131" s="1" t="n">
         <v>46073</v>
       </c>
       <c r="L131" t="inlineStr">
@@ -11052,7 +11040,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K132" s="2" t="n">
+      <c r="K132" s="1" t="n">
         <v>46077</v>
       </c>
       <c r="L132" t="inlineStr">
@@ -11125,7 +11113,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K133" s="2" t="n">
+      <c r="K133" s="1" t="n">
         <v>46079</v>
       </c>
       <c r="L133" t="inlineStr">
@@ -11198,7 +11186,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K134" s="2" t="n">
+      <c r="K134" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L134" t="inlineStr">
@@ -11271,7 +11259,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K135" s="2" t="n">
+      <c r="K135" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L135" t="inlineStr">
@@ -11344,7 +11332,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K136" s="2" t="n">
+      <c r="K136" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L136" t="inlineStr">
@@ -11417,7 +11405,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K137" s="2" t="n">
+      <c r="K137" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L137" t="inlineStr">
@@ -11490,7 +11478,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K138" s="2" t="n">
+      <c r="K138" s="1" t="n">
         <v>46080</v>
       </c>
       <c r="L138" t="inlineStr">
@@ -11563,7 +11551,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K139" s="2" t="n">
+      <c r="K139" s="1" t="n">
         <v>46078</v>
       </c>
       <c r="L139" t="inlineStr">
@@ -11644,7 +11632,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K140" s="2" t="n">
+      <c r="K140" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L140" t="inlineStr">
@@ -11717,7 +11705,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K141" s="2" t="n">
+      <c r="K141" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L141" t="inlineStr">
@@ -11790,7 +11778,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K142" s="2" t="n">
+      <c r="K142" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L142" t="inlineStr">
@@ -11867,7 +11855,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K143" s="2" t="n">
+      <c r="K143" s="1" t="n">
         <v>46092</v>
       </c>
       <c r="L143" t="inlineStr">
@@ -11940,7 +11928,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K144" s="2" t="n">
+      <c r="K144" s="1" t="n">
         <v>46090</v>
       </c>
       <c r="L144" t="inlineStr">
@@ -12013,7 +12001,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K145" s="2" t="n">
+      <c r="K145" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="L145" t="inlineStr">
@@ -12086,7 +12074,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K146" s="2" t="n">
+      <c r="K146" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="L146" t="inlineStr">
@@ -12159,7 +12147,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K147" s="2" t="n">
+      <c r="K147" s="1" t="n">
         <v>46094</v>
       </c>
       <c r="L147" t="inlineStr">
@@ -12232,7 +12220,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K148" s="2" t="n">
+      <c r="K148" s="1" t="n">
         <v>46097</v>
       </c>
       <c r="L148" t="inlineStr">
@@ -12305,7 +12293,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K149" s="2" t="n">
+      <c r="K149" s="1" t="n">
         <v>46097</v>
       </c>
       <c r="L149" t="inlineStr">
@@ -12378,7 +12366,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K150" s="2" t="n">
+      <c r="K150" s="1" t="n">
         <v>46098</v>
       </c>
       <c r="L150" t="inlineStr">
@@ -12451,7 +12439,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K151" s="2" t="n">
+      <c r="K151" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="L151" t="inlineStr">
@@ -12524,7 +12512,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K152" s="2" t="n">
+      <c r="K152" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="L152" t="inlineStr">
@@ -12597,7 +12585,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K153" s="2" t="n">
+      <c r="K153" s="1" t="n">
         <v>46100</v>
       </c>
       <c r="L153" t="inlineStr">
@@ -12616,7 +12604,7 @@
       <c r="Q153" t="inlineStr"/>
       <c r="R153" t="inlineStr"/>
       <c r="S153" t="inlineStr"/>
-      <c r="T153" s="2" t="n">
+      <c r="T153" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U153" t="inlineStr">
@@ -12680,7 +12668,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K154" s="2" t="n">
+      <c r="K154" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L154" t="inlineStr">
@@ -12753,7 +12741,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K155" s="2" t="n">
+      <c r="K155" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L155" t="inlineStr">
@@ -12826,7 +12814,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K156" s="2" t="n">
+      <c r="K156" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L156" t="inlineStr">
@@ -12899,7 +12887,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K157" s="2" t="n">
+      <c r="K157" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L157" t="inlineStr">
@@ -12972,7 +12960,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K158" s="2" t="n">
+      <c r="K158" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L158" t="inlineStr">
@@ -13045,7 +13033,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K159" s="2" t="n">
+      <c r="K159" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L159" t="inlineStr">
@@ -13118,7 +13106,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K160" s="2" t="n">
+      <c r="K160" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L160" t="inlineStr">
@@ -13191,7 +13179,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K161" s="2" t="n">
+      <c r="K161" s="1" t="n">
         <v>46101</v>
       </c>
       <c r="L161" t="inlineStr">
@@ -13264,7 +13252,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K162" s="2" t="n">
+      <c r="K162" s="1" t="n">
         <v>46113</v>
       </c>
       <c r="L162" t="inlineStr">
@@ -13337,7 +13325,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K163" s="2" t="n">
+      <c r="K163" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L163" t="inlineStr">
@@ -13410,7 +13398,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K164" s="2" t="n">
+      <c r="K164" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L164" t="inlineStr">
@@ -13483,7 +13471,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K165" s="2" t="n">
+      <c r="K165" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L165" t="inlineStr">
@@ -13556,7 +13544,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K166" s="2" t="n">
+      <c r="K166" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L166" t="inlineStr">
@@ -13629,7 +13617,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K167" s="2" t="n">
+      <c r="K167" s="1" t="n">
         <v>46119</v>
       </c>
       <c r="L167" t="inlineStr">
@@ -13706,7 +13694,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K168" s="2" t="n">
+      <c r="K168" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L168" t="inlineStr">
@@ -13783,7 +13771,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K169" s="2" t="n">
+      <c r="K169" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L169" t="inlineStr">
@@ -13856,7 +13844,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K170" s="2" t="n">
+      <c r="K170" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L170" t="inlineStr">
@@ -13929,7 +13917,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K171" s="2" t="n">
+      <c r="K171" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L171" t="inlineStr">
@@ -14002,7 +13990,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K172" s="2" t="n">
+      <c r="K172" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L172" t="inlineStr">
@@ -14075,7 +14063,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K173" s="2" t="n">
+      <c r="K173" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L173" t="inlineStr">
@@ -14148,7 +14136,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K174" s="2" t="n">
+      <c r="K174" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L174" t="inlineStr">
@@ -14221,7 +14209,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K175" s="2" t="n">
+      <c r="K175" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L175" t="inlineStr">
@@ -14294,7 +14282,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K176" s="2" t="n">
+      <c r="K176" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L176" t="inlineStr">
@@ -14367,7 +14355,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K177" s="2" t="n">
+      <c r="K177" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L177" t="inlineStr">
@@ -14440,7 +14428,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K178" s="2" t="n">
+      <c r="K178" s="1" t="n">
         <v>46120</v>
       </c>
       <c r="L178" t="inlineStr">
@@ -14513,7 +14501,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K179" s="2" t="n">
+      <c r="K179" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L179" t="inlineStr">
@@ -14532,7 +14520,7 @@
       <c r="Q179" t="inlineStr"/>
       <c r="R179" t="inlineStr"/>
       <c r="S179" t="inlineStr"/>
-      <c r="T179" s="2" t="n">
+      <c r="T179" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U179" t="inlineStr">
@@ -14596,7 +14584,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K180" s="2" t="n">
+      <c r="K180" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L180" t="inlineStr">
@@ -14669,7 +14657,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K181" s="2" t="n">
+      <c r="K181" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L181" t="inlineStr">
@@ -14742,7 +14730,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K182" s="2" t="n">
+      <c r="K182" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L182" t="inlineStr">
@@ -14815,7 +14803,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K183" s="2" t="n">
+      <c r="K183" s="1" t="n">
         <v>46121</v>
       </c>
       <c r="L183" t="inlineStr">
@@ -14888,7 +14876,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K184" s="2" t="n">
+      <c r="K184" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L184" t="inlineStr">
@@ -14961,7 +14949,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K185" s="2" t="n">
+      <c r="K185" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L185" t="inlineStr">
@@ -15034,7 +15022,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K186" s="2" t="n">
+      <c r="K186" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L186" t="inlineStr">
@@ -15107,7 +15095,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K187" s="2" t="n">
+      <c r="K187" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L187" t="inlineStr">
@@ -15180,7 +15168,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K188" s="2" t="n">
+      <c r="K188" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L188" t="inlineStr">
@@ -15253,7 +15241,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K189" s="2" t="n">
+      <c r="K189" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L189" t="inlineStr">
@@ -15326,7 +15314,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K190" s="2" t="n">
+      <c r="K190" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L190" t="inlineStr">
@@ -15399,7 +15387,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K191" s="2" t="n">
+      <c r="K191" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L191" t="inlineStr">
@@ -15472,7 +15460,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K192" s="2" t="n">
+      <c r="K192" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L192" t="inlineStr">
@@ -15545,7 +15533,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K193" s="2" t="n">
+      <c r="K193" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L193" t="inlineStr">
@@ -15618,7 +15606,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K194" s="2" t="n">
+      <c r="K194" s="1" t="n">
         <v>46122</v>
       </c>
       <c r="L194" t="inlineStr">
@@ -15691,7 +15679,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K195" s="2" t="n">
+      <c r="K195" s="1" t="n">
         <v>46126</v>
       </c>
       <c r="L195" t="inlineStr">
@@ -15766,7 +15754,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K196" s="2" t="n">
+      <c r="K196" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="L196" t="inlineStr">
@@ -15841,7 +15829,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K197" s="2" t="n">
+      <c r="K197" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="L197" t="inlineStr">
@@ -15912,7 +15900,7 @@
           <t>A7</t>
         </is>
       </c>
-      <c r="K198" s="2" t="n">
+      <c r="K198" s="1" t="n">
         <v>46128</v>
       </c>
       <c r="L198" t="inlineStr">
@@ -15983,7 +15971,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K199" s="2" t="n">
+      <c r="K199" s="1" t="n">
         <v>46129</v>
       </c>
       <c r="L199" t="inlineStr">
@@ -16054,7 +16042,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K200" s="2" t="n">
+      <c r="K200" s="1" t="n">
         <v>46135</v>
       </c>
       <c r="L200" t="inlineStr">
@@ -16125,7 +16113,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K201" s="2" t="n">
+      <c r="K201" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L201" t="inlineStr">
@@ -16196,7 +16184,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K202" s="2" t="n">
+      <c r="K202" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L202" t="inlineStr">
@@ -16267,7 +16255,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K203" s="2" t="n">
+      <c r="K203" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L203" t="inlineStr">
@@ -16338,7 +16326,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K204" s="2" t="n">
+      <c r="K204" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L204" t="inlineStr">
@@ -16413,7 +16401,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K205" s="2" t="n">
+      <c r="K205" s="1" t="n">
         <v>46139</v>
       </c>
       <c r="L205" t="inlineStr">
@@ -16488,7 +16476,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K206" s="2" t="n">
+      <c r="K206" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L206" t="inlineStr">
@@ -16559,7 +16547,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K207" s="2" t="n">
+      <c r="K207" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L207" t="inlineStr">
@@ -16630,7 +16618,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K208" s="2" t="n">
+      <c r="K208" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L208" t="inlineStr">
@@ -16701,7 +16689,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K209" s="2" t="n">
+      <c r="K209" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L209" t="inlineStr">
@@ -16772,7 +16760,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K210" s="2" t="n">
+      <c r="K210" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L210" t="inlineStr">
@@ -16843,7 +16831,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K211" s="2" t="n">
+      <c r="K211" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L211" t="inlineStr">
@@ -16914,7 +16902,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K212" s="2" t="n">
+      <c r="K212" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L212" t="inlineStr">
@@ -16985,7 +16973,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K213" s="2" t="n">
+      <c r="K213" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L213" t="inlineStr">
@@ -17056,7 +17044,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K214" s="2" t="n">
+      <c r="K214" s="1" t="n">
         <v>46141</v>
       </c>
       <c r="L214" t="inlineStr">
@@ -17127,7 +17115,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K215" s="2" t="n">
+      <c r="K215" s="1" t="n">
         <v>46142</v>
       </c>
       <c r="L215" t="inlineStr">
@@ -17198,7 +17186,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K216" s="2" t="n">
+      <c r="K216" s="1" t="n">
         <v>46146</v>
       </c>
       <c r="L216" t="inlineStr">
@@ -17269,7 +17257,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K217" s="2" t="n">
+      <c r="K217" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L217" t="inlineStr">
@@ -17340,7 +17328,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K218" s="2" t="n">
+      <c r="K218" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L218" t="inlineStr">
@@ -17411,7 +17399,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K219" s="2" t="n">
+      <c r="K219" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L219" t="inlineStr">
@@ -17482,7 +17470,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K220" s="2" t="n">
+      <c r="K220" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L220" t="inlineStr">
@@ -17553,7 +17541,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K221" s="2" t="n">
+      <c r="K221" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L221" t="inlineStr">
@@ -17624,7 +17612,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K222" s="2" t="n">
+      <c r="K222" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L222" t="inlineStr">
@@ -17695,7 +17683,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K223" s="2" t="n">
+      <c r="K223" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L223" t="inlineStr">
@@ -17766,7 +17754,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K224" s="2" t="n">
+      <c r="K224" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L224" t="inlineStr">
@@ -17837,7 +17825,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K225" s="2" t="n">
+      <c r="K225" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L225" t="inlineStr">
@@ -17908,7 +17896,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K226" s="2" t="n">
+      <c r="K226" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L226" t="inlineStr">
@@ -17979,7 +17967,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K227" s="2" t="n">
+      <c r="K227" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L227" t="inlineStr">
@@ -18050,7 +18038,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K228" s="2" t="n">
+      <c r="K228" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L228" t="inlineStr">
@@ -18121,7 +18109,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K229" s="2" t="n">
+      <c r="K229" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L229" t="inlineStr">
@@ -18192,7 +18180,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K230" s="2" t="n">
+      <c r="K230" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L230" t="inlineStr">
@@ -18263,7 +18251,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K231" s="2" t="n">
+      <c r="K231" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L231" t="inlineStr">
@@ -18334,7 +18322,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K232" s="2" t="n">
+      <c r="K232" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L232" t="inlineStr">
@@ -18405,7 +18393,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K233" s="2" t="n">
+      <c r="K233" s="1" t="n">
         <v>46148</v>
       </c>
       <c r="L233" t="inlineStr">
@@ -18476,7 +18464,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K234" s="2" t="n">
+      <c r="K234" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L234" t="inlineStr">
@@ -18547,7 +18535,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K235" s="2" t="n">
+      <c r="K235" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L235" t="inlineStr">
@@ -18618,7 +18606,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K236" s="2" t="n">
+      <c r="K236" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L236" t="inlineStr">
@@ -18689,7 +18677,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K237" s="2" t="n">
+      <c r="K237" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L237" t="inlineStr">
@@ -18760,7 +18748,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K238" s="2" t="n">
+      <c r="K238" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L238" t="inlineStr">
@@ -18831,7 +18819,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K239" s="2" t="n">
+      <c r="K239" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L239" t="inlineStr">
@@ -18902,7 +18890,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K240" s="2" t="n">
+      <c r="K240" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L240" t="inlineStr">
@@ -18973,7 +18961,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K241" s="2" t="n">
+      <c r="K241" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L241" t="inlineStr">
@@ -19044,7 +19032,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K242" s="2" t="n">
+      <c r="K242" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L242" t="inlineStr">
@@ -19115,7 +19103,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K243" s="2" t="n">
+      <c r="K243" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L243" t="inlineStr">
@@ -19186,7 +19174,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K244" s="2" t="n">
+      <c r="K244" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L244" t="inlineStr">
@@ -19257,7 +19245,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K245" s="2" t="n">
+      <c r="K245" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L245" t="inlineStr">
@@ -19328,7 +19316,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K246" s="2" t="n">
+      <c r="K246" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L246" t="inlineStr">
@@ -19399,7 +19387,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K247" s="2" t="n">
+      <c r="K247" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L247" t="inlineStr">
@@ -19470,7 +19458,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K248" s="2" t="n">
+      <c r="K248" s="1" t="n">
         <v>46149</v>
       </c>
       <c r="L248" t="inlineStr">
@@ -19541,7 +19529,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K249" s="2" t="n">
+      <c r="K249" s="1" t="n">
         <v>46150</v>
       </c>
       <c r="L249" t="inlineStr">
@@ -19612,7 +19600,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K250" s="2" t="n">
+      <c r="K250" s="1" t="n">
         <v>46155</v>
       </c>
       <c r="L250" t="inlineStr">
@@ -19683,7 +19671,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K251" s="2" t="n">
+      <c r="K251" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="L251" t="inlineStr">
@@ -19754,7 +19742,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K252" s="2" t="n">
+      <c r="K252" s="1" t="n">
         <v>46161</v>
       </c>
       <c r="L252" t="inlineStr">
@@ -19825,7 +19813,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K253" s="2" t="n">
+      <c r="K253" s="1" t="n">
         <v>46162</v>
       </c>
       <c r="L253" t="inlineStr">
@@ -19900,7 +19888,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K254" s="2" t="n">
+      <c r="K254" s="1" t="n">
         <v>46162</v>
       </c>
       <c r="L254" t="inlineStr">
@@ -19971,7 +19959,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K255" s="2" t="n">
+      <c r="K255" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="L255" t="inlineStr">
@@ -20042,7 +20030,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K256" s="2" t="n">
+      <c r="K256" s="1" t="n">
         <v>46163</v>
       </c>
       <c r="L256" t="inlineStr">
@@ -20117,7 +20105,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K257" s="2" t="n">
+      <c r="K257" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="L257" t="inlineStr">
@@ -20136,7 +20124,7 @@
       <c r="Q257" t="inlineStr"/>
       <c r="R257" t="inlineStr"/>
       <c r="S257" t="inlineStr"/>
-      <c r="T257" s="2" t="n">
+      <c r="T257" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U257" t="inlineStr">
@@ -20202,7 +20190,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K258" s="2" t="n">
+      <c r="K258" s="1" t="n">
         <v>46170</v>
       </c>
       <c r="L258" t="inlineStr">
@@ -20277,7 +20265,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K259" s="2" t="n">
+      <c r="K259" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L259" t="inlineStr">
@@ -20352,7 +20340,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K260" s="2" t="n">
+      <c r="K260" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L260" t="inlineStr">
@@ -20371,7 +20359,7 @@
       <c r="Q260" t="inlineStr"/>
       <c r="R260" t="inlineStr"/>
       <c r="S260" t="inlineStr"/>
-      <c r="T260" s="2" t="n">
+      <c r="T260" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U260" t="inlineStr">
@@ -20437,7 +20425,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K261" s="2" t="n">
+      <c r="K261" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L261" t="inlineStr">
@@ -20512,7 +20500,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K262" s="2" t="n">
+      <c r="K262" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L262" t="inlineStr">
@@ -20587,7 +20575,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K263" s="2" t="n">
+      <c r="K263" s="1" t="n">
         <v>46171</v>
       </c>
       <c r="L263" t="inlineStr">
@@ -20606,7 +20594,7 @@
       <c r="Q263" t="inlineStr"/>
       <c r="R263" t="inlineStr"/>
       <c r="S263" t="inlineStr"/>
-      <c r="T263" s="2" t="n">
+      <c r="T263" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="U263" t="inlineStr">
@@ -20672,7 +20660,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K264" s="2" t="n">
+      <c r="K264" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L264" t="inlineStr">
@@ -20743,7 +20731,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K265" s="2" t="n">
+      <c r="K265" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L265" t="inlineStr">
@@ -20814,7 +20802,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K266" s="2" t="n">
+      <c r="K266" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L266" t="inlineStr">
@@ -20885,7 +20873,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K267" s="2" t="n">
+      <c r="K267" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L267" t="inlineStr">
@@ -20960,7 +20948,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K268" s="2" t="n">
+      <c r="K268" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L268" t="inlineStr">
@@ -21031,7 +21019,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K269" s="2" t="n">
+      <c r="K269" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L269" t="inlineStr">
@@ -21102,7 +21090,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K270" s="2" t="n">
+      <c r="K270" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L270" t="inlineStr">
@@ -21173,7 +21161,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K271" s="2" t="n">
+      <c r="K271" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L271" t="inlineStr">
@@ -21244,7 +21232,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K272" s="2" t="n">
+      <c r="K272" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L272" t="inlineStr">
@@ -21319,7 +21307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K273" s="2" t="n">
+      <c r="K273" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L273" t="inlineStr">
@@ -21394,7 +21382,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K274" s="2" t="n">
+      <c r="K274" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L274" t="inlineStr">
@@ -21465,7 +21453,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K275" s="2" t="n">
+      <c r="K275" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L275" t="inlineStr">
@@ -21536,7 +21524,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K276" s="2" t="n">
+      <c r="K276" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L276" t="inlineStr">
@@ -21607,7 +21595,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K277" s="2" t="n">
+      <c r="K277" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L277" t="inlineStr">
@@ -21678,7 +21666,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K278" s="2" t="n">
+      <c r="K278" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L278" t="inlineStr">
@@ -21749,7 +21737,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K279" s="2" t="n">
+      <c r="K279" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L279" t="inlineStr">
@@ -21820,7 +21808,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K280" s="2" t="n">
+      <c r="K280" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L280" t="inlineStr">
@@ -21891,7 +21879,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K281" s="2" t="n">
+      <c r="K281" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L281" t="inlineStr">
@@ -21962,7 +21950,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K282" s="2" t="n">
+      <c r="K282" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L282" t="inlineStr">
@@ -22033,7 +22021,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K283" s="2" t="n">
+      <c r="K283" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L283" t="inlineStr">
@@ -22104,7 +22092,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K284" s="2" t="n">
+      <c r="K284" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L284" t="inlineStr">
@@ -22175,7 +22163,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K285" s="2" t="n">
+      <c r="K285" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L285" t="inlineStr">
@@ -22246,7 +22234,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K286" s="2" t="n">
+      <c r="K286" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L286" t="inlineStr">
@@ -22317,7 +22305,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K287" s="2" t="n">
+      <c r="K287" s="1" t="n">
         <v>46174</v>
       </c>
       <c r="L287" t="inlineStr">
@@ -22388,7 +22376,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K288" s="2" t="n">
+      <c r="K288" s="1" t="n">
         <v>46176</v>
       </c>
       <c r="L288" t="inlineStr">
@@ -22459,7 +22447,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K289" s="2" t="n">
+      <c r="K289" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="L289" t="inlineStr">
@@ -22530,7 +22518,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K290" s="2" t="n">
+      <c r="K290" s="1" t="n">
         <v>46182</v>
       </c>
       <c r="L290" t="inlineStr">
@@ -22601,7 +22589,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K291" s="2" t="n">
+      <c r="K291" s="1" t="n">
         <v>46183</v>
       </c>
       <c r="L291" t="inlineStr">
@@ -22672,7 +22660,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K292" s="2" t="n">
+      <c r="K292" s="1" t="n">
         <v>46185</v>
       </c>
       <c r="L292" t="inlineStr">
@@ -22743,7 +22731,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K293" s="2" t="n">
+      <c r="K293" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L293" t="inlineStr">
@@ -22814,7 +22802,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K294" s="2" t="n">
+      <c r="K294" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L294" t="inlineStr">
@@ -22885,7 +22873,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K295" s="2" t="n">
+      <c r="K295" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L295" t="inlineStr">
@@ -22960,7 +22948,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K296" s="2" t="n">
+      <c r="K296" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L296" t="inlineStr">
@@ -23035,7 +23023,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K297" s="2" t="n">
+      <c r="K297" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L297" t="inlineStr">
@@ -23106,7 +23094,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K298" s="2" t="n">
+      <c r="K298" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L298" t="inlineStr">
@@ -23177,7 +23165,7 @@
           <t>T1</t>
         </is>
       </c>
-      <c r="K299" s="2" t="n">
+      <c r="K299" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L299" t="inlineStr">
@@ -23248,7 +23236,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K300" s="2" t="n">
+      <c r="K300" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L300" t="inlineStr">
@@ -23319,7 +23307,7 @@
           <t>U8</t>
         </is>
       </c>
-      <c r="K301" s="2" t="n">
+      <c r="K301" s="1" t="n">
         <v>46192</v>
       </c>
       <c r="L301" t="inlineStr">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (15/07/2026 20:42)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -19373,6 +19373,9 @@
       <c r="F331" t="s">
         <v>869</v>
       </c>
+      <c r="G331">
+        <v>1</v>
+      </c>
       <c r="H331" t="s">
         <v>1219</v>
       </c>
@@ -19411,6 +19414,9 @@
       <c r="F332" t="s">
         <v>869</v>
       </c>
+      <c r="G332">
+        <v>1</v>
+      </c>
       <c r="H332" t="s">
         <v>1220</v>
       </c>
@@ -19449,6 +19455,9 @@
       <c r="F333" t="s">
         <v>869</v>
       </c>
+      <c r="G333">
+        <v>1</v>
+      </c>
       <c r="H333" t="s">
         <v>1221</v>
       </c>
@@ -19487,6 +19496,9 @@
       <c r="F334" t="s">
         <v>869</v>
       </c>
+      <c r="G334">
+        <v>1</v>
+      </c>
       <c r="H334" t="s">
         <v>1222</v>
       </c>
@@ -19525,6 +19537,9 @@
       <c r="F335" t="s">
         <v>869</v>
       </c>
+      <c r="G335">
+        <v>1</v>
+      </c>
       <c r="H335" t="s">
         <v>1223</v>
       </c>
@@ -19563,6 +19578,9 @@
       <c r="F336" t="s">
         <v>869</v>
       </c>
+      <c r="G336">
+        <v>1</v>
+      </c>
       <c r="H336" t="s">
         <v>1224</v>
       </c>
@@ -19601,6 +19619,9 @@
       <c r="F337" t="s">
         <v>884</v>
       </c>
+      <c r="G337">
+        <v>5</v>
+      </c>
       <c r="H337" t="s">
         <v>1225</v>
       </c>
@@ -19639,6 +19660,9 @@
       <c r="F338" t="s">
         <v>869</v>
       </c>
+      <c r="G338">
+        <v>1</v>
+      </c>
       <c r="H338" t="s">
         <v>1226</v>
       </c>
@@ -19676,6 +19700,9 @@
       </c>
       <c r="F339" t="s">
         <v>869</v>
+      </c>
+      <c r="G339">
+        <v>1</v>
       </c>
       <c r="H339" t="s">
         <v>1227</v>

</xml_diff>

<commit_message>
Atualização automática: devolucoes (22/07/2026 12:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -4616,8 +4616,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -4633,7 +4641,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -4641,12 +4649,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4946,73 +4972,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5047,7 +5073,7 @@
       <c r="J2" t="s">
         <v>1388</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5091,7 +5117,7 @@
       <c r="J3" t="s">
         <v>1388</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5135,7 +5161,7 @@
       <c r="J4" t="s">
         <v>1388</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5179,7 +5205,7 @@
       <c r="J5" t="s">
         <v>1389</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5229,7 +5255,7 @@
       <c r="J6" t="s">
         <v>1388</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5276,7 +5302,7 @@
       <c r="J7" t="s">
         <v>1388</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5323,7 +5349,7 @@
       <c r="J8" t="s">
         <v>1388</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5370,7 +5396,7 @@
       <c r="J9" t="s">
         <v>1388</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5417,7 +5443,7 @@
       <c r="J10" t="s">
         <v>1388</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -5464,7 +5490,7 @@
       <c r="J11" t="s">
         <v>1388</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -5511,7 +5537,7 @@
       <c r="J12" t="s">
         <v>1388</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -5555,7 +5581,7 @@
       <c r="J13" t="s">
         <v>1388</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -5599,7 +5625,7 @@
       <c r="J14" t="s">
         <v>1388</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -5643,7 +5669,7 @@
       <c r="J15" t="s">
         <v>1388</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -5687,7 +5713,7 @@
       <c r="J16" t="s">
         <v>1388</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -5731,7 +5757,7 @@
       <c r="J17" t="s">
         <v>1388</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -5775,7 +5801,7 @@
       <c r="J18" t="s">
         <v>1388</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -5793,7 +5819,7 @@
       <c r="R18" t="s">
         <v>1479</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -5834,7 +5860,7 @@
       <c r="J19" t="s">
         <v>1388</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -5878,7 +5904,7 @@
       <c r="J20" t="s">
         <v>1388</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -5922,7 +5948,7 @@
       <c r="J21" t="s">
         <v>1388</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -5940,7 +5966,7 @@
       <c r="R21" t="s">
         <v>1480</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -5981,7 +6007,7 @@
       <c r="J22" t="s">
         <v>1388</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -5999,7 +6025,7 @@
       <c r="R22" t="s">
         <v>1481</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6040,7 +6066,7 @@
       <c r="J23" t="s">
         <v>1388</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6058,7 +6084,7 @@
       <c r="R23" t="s">
         <v>1482</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6099,7 +6125,7 @@
       <c r="J24" t="s">
         <v>1388</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6143,7 +6169,7 @@
       <c r="J25" t="s">
         <v>1388</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6184,7 +6210,7 @@
       <c r="J26" t="s">
         <v>1390</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6225,7 +6251,7 @@
       <c r="J27" t="s">
         <v>1388</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6243,7 +6269,7 @@
       <c r="R27" t="s">
         <v>1483</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6284,7 +6310,7 @@
       <c r="J28" t="s">
         <v>1388</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6328,7 +6354,7 @@
       <c r="J29" t="s">
         <v>1388</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6372,7 +6398,7 @@
       <c r="J30" t="s">
         <v>1388</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -6416,7 +6442,7 @@
       <c r="J31" t="s">
         <v>1388</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -6434,7 +6460,7 @@
       <c r="R31" t="s">
         <v>1484</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -6475,7 +6501,7 @@
       <c r="J32" t="s">
         <v>1388</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -6519,7 +6545,7 @@
       <c r="J33" t="s">
         <v>1388</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -6537,7 +6563,7 @@
       <c r="R33" t="s">
         <v>1485</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -6578,7 +6604,7 @@
       <c r="J34" t="s">
         <v>1388</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -6622,7 +6648,7 @@
       <c r="J35" t="s">
         <v>1388</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -6640,7 +6666,7 @@
       <c r="R35" t="s">
         <v>1486</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -6681,7 +6707,7 @@
       <c r="J36" t="s">
         <v>1388</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -6699,7 +6725,7 @@
       <c r="R36" t="s">
         <v>1486</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -6740,7 +6766,7 @@
       <c r="J37" t="s">
         <v>1388</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -6758,7 +6784,7 @@
       <c r="R37" t="s">
         <v>1486</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -6799,7 +6825,7 @@
       <c r="J38" t="s">
         <v>1388</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -6817,7 +6843,7 @@
       <c r="R38" t="s">
         <v>1486</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -6858,7 +6884,7 @@
       <c r="J39" t="s">
         <v>1388</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -6876,7 +6902,7 @@
       <c r="R39" t="s">
         <v>1486</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -6917,7 +6943,7 @@
       <c r="J40" t="s">
         <v>1388</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -6935,7 +6961,7 @@
       <c r="R40" t="s">
         <v>1487</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -6976,7 +7002,7 @@
       <c r="J41" t="s">
         <v>1388</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7020,7 +7046,7 @@
       <c r="J42" t="s">
         <v>1388</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7038,7 +7064,7 @@
       <c r="R42" t="s">
         <v>1486</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7079,7 +7105,7 @@
       <c r="J43" t="s">
         <v>1388</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7123,7 +7149,7 @@
       <c r="J44" t="s">
         <v>1388</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7141,7 +7167,7 @@
       <c r="R44" t="s">
         <v>1488</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7182,7 +7208,7 @@
       <c r="J45" t="s">
         <v>1388</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7226,7 +7252,7 @@
       <c r="J46" t="s">
         <v>1388</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7270,7 +7296,7 @@
       <c r="J47" t="s">
         <v>1388</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7288,7 +7314,7 @@
       <c r="R47" t="s">
         <v>1489</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7329,7 +7355,7 @@
       <c r="J48" t="s">
         <v>1388</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -7373,7 +7399,7 @@
       <c r="J49" t="s">
         <v>1388</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -7417,7 +7443,7 @@
       <c r="J50" t="s">
         <v>1388</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -7461,7 +7487,7 @@
       <c r="J51" t="s">
         <v>1388</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -7508,7 +7534,7 @@
       <c r="J52" t="s">
         <v>1388</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -7552,7 +7578,7 @@
       <c r="J53" t="s">
         <v>1388</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -7596,7 +7622,7 @@
       <c r="J54" t="s">
         <v>1388</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -7640,7 +7666,7 @@
       <c r="J55" t="s">
         <v>1388</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -7690,7 +7716,7 @@
       <c r="J56" t="s">
         <v>1388</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -7743,7 +7769,7 @@
       <c r="J57" t="s">
         <v>1388</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -7793,7 +7819,7 @@
       <c r="J58" t="s">
         <v>1388</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -7843,7 +7869,7 @@
       <c r="J59" t="s">
         <v>1388</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -7861,7 +7887,7 @@
       <c r="R59" t="s">
         <v>1490</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -7902,7 +7928,7 @@
       <c r="J60" t="s">
         <v>1388</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -7946,7 +7972,7 @@
       <c r="J61" t="s">
         <v>1388</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -7990,7 +8016,7 @@
       <c r="J62" t="s">
         <v>1388</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8034,7 +8060,7 @@
       <c r="J63" t="s">
         <v>1388</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8078,7 +8104,7 @@
       <c r="J64" t="s">
         <v>1388</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8122,7 +8148,7 @@
       <c r="J65" t="s">
         <v>1388</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8169,7 +8195,7 @@
       <c r="J66" t="s">
         <v>1388</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8213,7 +8239,7 @@
       <c r="J67" t="s">
         <v>1388</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8257,7 +8283,7 @@
       <c r="J68" t="s">
         <v>1388</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8272,7 +8298,7 @@
       <c r="O68" t="s">
         <v>1455</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8316,7 +8342,7 @@
       <c r="J69" t="s">
         <v>1390</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -8360,7 +8386,7 @@
       <c r="J70" t="s">
         <v>1388</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -8404,7 +8430,7 @@
       <c r="J71" t="s">
         <v>1388</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -8448,7 +8474,7 @@
       <c r="J72" t="s">
         <v>1388</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -8492,7 +8518,7 @@
       <c r="J73" t="s">
         <v>1388</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -8536,7 +8562,7 @@
       <c r="J74" t="s">
         <v>1388</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -8580,7 +8606,7 @@
       <c r="J75" t="s">
         <v>1388</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -8624,7 +8650,7 @@
       <c r="J76" t="s">
         <v>1388</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -8668,7 +8694,7 @@
       <c r="J77" t="s">
         <v>1388</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -8712,7 +8738,7 @@
       <c r="J78" t="s">
         <v>1388</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -8756,7 +8782,7 @@
       <c r="J79" t="s">
         <v>1388</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -8800,7 +8826,7 @@
       <c r="J80" t="s">
         <v>1388</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -8844,7 +8870,7 @@
       <c r="J81" t="s">
         <v>1388</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -8888,7 +8914,7 @@
       <c r="J82" t="s">
         <v>1388</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -8932,7 +8958,7 @@
       <c r="J83" t="s">
         <v>1388</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -8976,7 +9002,7 @@
       <c r="J84" t="s">
         <v>1388</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9020,7 +9046,7 @@
       <c r="J85" t="s">
         <v>1388</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9064,7 +9090,7 @@
       <c r="J86" t="s">
         <v>1388</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9108,7 +9134,7 @@
       <c r="J87" t="s">
         <v>1388</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9152,7 +9178,7 @@
       <c r="J88" t="s">
         <v>1388</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9196,7 +9222,7 @@
       <c r="J89" t="s">
         <v>1388</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9237,7 +9263,7 @@
       <c r="J90" t="s">
         <v>1388</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -9278,7 +9304,7 @@
       <c r="J91" t="s">
         <v>1388</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -9322,7 +9348,7 @@
       <c r="J92" t="s">
         <v>1388</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -9343,7 +9369,7 @@
       <c r="R92" t="s">
         <v>1482</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -9384,7 +9410,7 @@
       <c r="J93" t="s">
         <v>1388</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -9425,7 +9451,7 @@
       <c r="J94" t="s">
         <v>1388</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -9469,7 +9495,7 @@
       <c r="J95" t="s">
         <v>1388</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -9513,7 +9539,7 @@
       <c r="J96" t="s">
         <v>1388</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -9560,7 +9586,7 @@
       <c r="J97" t="s">
         <v>1388</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -9575,7 +9601,7 @@
       <c r="R97" t="s">
         <v>1491</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -9616,7 +9642,7 @@
       <c r="J98" t="s">
         <v>1388</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -9660,7 +9686,7 @@
       <c r="J99" t="s">
         <v>1388</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -9704,7 +9730,7 @@
       <c r="J100" t="s">
         <v>1388</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -9745,7 +9771,7 @@
       <c r="J101" t="s">
         <v>1388</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -9786,7 +9812,7 @@
       <c r="J102" t="s">
         <v>1388</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -9827,7 +9853,7 @@
       <c r="J103" t="s">
         <v>1388</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -9868,7 +9894,7 @@
       <c r="J104" t="s">
         <v>1388</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -9909,7 +9935,7 @@
       <c r="J105" t="s">
         <v>1388</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -9950,7 +9976,7 @@
       <c r="J106" t="s">
         <v>1388</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -9991,7 +10017,7 @@
       <c r="J107" t="s">
         <v>1388</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10032,7 +10058,7 @@
       <c r="J108" t="s">
         <v>1388</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10073,7 +10099,7 @@
       <c r="J109" t="s">
         <v>1388</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10114,7 +10140,7 @@
       <c r="J110" t="s">
         <v>1388</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10132,7 +10158,7 @@
       <c r="R110" t="s">
         <v>1492</v>
       </c>
-      <c r="T110" s="1">
+      <c r="T110" s="2">
         <v>45805</v>
       </c>
       <c r="U110" t="s">
@@ -10170,7 +10196,7 @@
       <c r="J111" t="s">
         <v>1388</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -10188,7 +10214,7 @@
       <c r="R111" t="s">
         <v>1493</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -10226,7 +10252,7 @@
       <c r="J112" t="s">
         <v>1388</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -10244,7 +10270,7 @@
       <c r="R112" t="s">
         <v>1494</v>
       </c>
-      <c r="T112" s="1">
+      <c r="T112" s="2">
         <v>46052</v>
       </c>
       <c r="U112" t="s">
@@ -10285,7 +10311,7 @@
       <c r="J113" t="s">
         <v>1388</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -10329,7 +10355,7 @@
       <c r="J114" t="s">
         <v>1388</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -10373,7 +10399,7 @@
       <c r="J115" t="s">
         <v>1388</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -10417,7 +10443,7 @@
       <c r="J116" t="s">
         <v>1388</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -10435,7 +10461,7 @@
       <c r="R116" t="s">
         <v>1495</v>
       </c>
-      <c r="T116" s="1">
+      <c r="T116" s="2">
         <v>46048</v>
       </c>
       <c r="U116" t="s">
@@ -10476,7 +10502,7 @@
       <c r="J117" t="s">
         <v>1388</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -10520,7 +10546,7 @@
       <c r="J118" t="s">
         <v>1388</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -10567,7 +10593,7 @@
       <c r="J119" t="s">
         <v>1388</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -10608,7 +10634,7 @@
       <c r="J120" t="s">
         <v>1388</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -10652,7 +10678,7 @@
       <c r="J121" t="s">
         <v>1388</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -10696,7 +10722,7 @@
       <c r="J122" t="s">
         <v>1388</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -10746,7 +10772,7 @@
       <c r="J123" t="s">
         <v>1388</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -10790,7 +10816,7 @@
       <c r="J124" t="s">
         <v>1388</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -10834,7 +10860,7 @@
       <c r="J125" t="s">
         <v>1388</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -10875,7 +10901,7 @@
       <c r="J126" t="s">
         <v>1388</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -10916,7 +10942,7 @@
       <c r="J127" t="s">
         <v>1388</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -10934,7 +10960,7 @@
       <c r="R127" t="s">
         <v>1497</v>
       </c>
-      <c r="T127" s="1">
+      <c r="T127" s="2">
         <v>45889</v>
       </c>
       <c r="U127" t="s">
@@ -10972,7 +10998,7 @@
       <c r="J128" t="s">
         <v>1388</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11013,7 +11039,7 @@
       <c r="J129" t="s">
         <v>1388</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11054,7 +11080,7 @@
       <c r="J130" t="s">
         <v>1388</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11095,7 +11121,7 @@
       <c r="J131" t="s">
         <v>1388</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11139,7 +11165,7 @@
       <c r="J132" t="s">
         <v>1388</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -11180,7 +11206,7 @@
       <c r="J133" t="s">
         <v>1388</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -11221,7 +11247,7 @@
       <c r="J134" t="s">
         <v>1388</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -11262,7 +11288,7 @@
       <c r="J135" t="s">
         <v>1388</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -11303,7 +11329,7 @@
       <c r="J136" t="s">
         <v>1388</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -11344,7 +11370,7 @@
       <c r="J137" t="s">
         <v>1388</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -11385,7 +11411,7 @@
       <c r="J138" t="s">
         <v>1388</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -11426,7 +11452,7 @@
       <c r="J139" t="s">
         <v>1388</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -11473,7 +11499,7 @@
       <c r="J140" t="s">
         <v>1388</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -11514,7 +11540,7 @@
       <c r="J141" t="s">
         <v>1388</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -11555,7 +11581,7 @@
       <c r="J142" t="s">
         <v>1388</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -11599,7 +11625,7 @@
       <c r="J143" t="s">
         <v>1388</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -11640,7 +11666,7 @@
       <c r="J144" t="s">
         <v>1388</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -11681,7 +11707,7 @@
       <c r="J145" t="s">
         <v>1388</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -11722,7 +11748,7 @@
       <c r="J146" t="s">
         <v>1388</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -11763,7 +11789,7 @@
       <c r="J147" t="s">
         <v>1388</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -11804,7 +11830,7 @@
       <c r="J148" t="s">
         <v>1388</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -11845,7 +11871,7 @@
       <c r="J149" t="s">
         <v>1388</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -11886,7 +11912,7 @@
       <c r="J150" t="s">
         <v>1388</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -11927,7 +11953,7 @@
       <c r="J151" t="s">
         <v>1388</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -11968,7 +11994,7 @@
       <c r="J152" t="s">
         <v>1388</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12009,7 +12035,7 @@
       <c r="J153" t="s">
         <v>1388</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -12018,7 +12044,7 @@
       <c r="M153" t="s">
         <v>1446</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -12059,7 +12085,7 @@
       <c r="J154" t="s">
         <v>1388</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -12100,7 +12126,7 @@
       <c r="J155" t="s">
         <v>1388</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -12141,7 +12167,7 @@
       <c r="J156" t="s">
         <v>1388</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -12182,7 +12208,7 @@
       <c r="J157" t="s">
         <v>1388</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -12223,7 +12249,7 @@
       <c r="J158" t="s">
         <v>1388</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -12264,7 +12290,7 @@
       <c r="J159" t="s">
         <v>1388</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -12305,7 +12331,7 @@
       <c r="J160" t="s">
         <v>1388</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -12346,7 +12372,7 @@
       <c r="J161" t="s">
         <v>1388</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -12387,7 +12413,7 @@
       <c r="J162" t="s">
         <v>1388</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -12428,7 +12454,7 @@
       <c r="J163" t="s">
         <v>1388</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -12469,7 +12495,7 @@
       <c r="J164" t="s">
         <v>1388</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -12510,7 +12536,7 @@
       <c r="J165" t="s">
         <v>1388</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -12551,7 +12577,7 @@
       <c r="J166" t="s">
         <v>1388</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -12592,7 +12618,7 @@
       <c r="J167" t="s">
         <v>1388</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -12636,7 +12662,7 @@
       <c r="J168" t="s">
         <v>1388</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -12680,7 +12706,7 @@
       <c r="J169" t="s">
         <v>1388</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -12721,7 +12747,7 @@
       <c r="J170" t="s">
         <v>1388</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -12762,7 +12788,7 @@
       <c r="J171" t="s">
         <v>1388</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -12803,7 +12829,7 @@
       <c r="J172" t="s">
         <v>1388</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -12844,7 +12870,7 @@
       <c r="J173" t="s">
         <v>1388</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -12885,7 +12911,7 @@
       <c r="J174" t="s">
         <v>1388</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -12926,7 +12952,7 @@
       <c r="J175" t="s">
         <v>1388</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -12967,7 +12993,7 @@
       <c r="J176" t="s">
         <v>1388</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -13008,7 +13034,7 @@
       <c r="J177" t="s">
         <v>1388</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -13049,7 +13075,7 @@
       <c r="J178" t="s">
         <v>1388</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -13090,7 +13116,7 @@
       <c r="J179" t="s">
         <v>1388</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -13099,7 +13125,7 @@
       <c r="M179" t="s">
         <v>1443</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -13140,7 +13166,7 @@
       <c r="J180" t="s">
         <v>1388</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -13181,7 +13207,7 @@
       <c r="J181" t="s">
         <v>1388</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -13222,7 +13248,7 @@
       <c r="J182" t="s">
         <v>1388</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -13263,7 +13289,7 @@
       <c r="J183" t="s">
         <v>1388</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -13304,7 +13330,7 @@
       <c r="J184" t="s">
         <v>1388</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -13345,7 +13371,7 @@
       <c r="J185" t="s">
         <v>1388</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -13386,7 +13412,7 @@
       <c r="J186" t="s">
         <v>1388</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -13427,7 +13453,7 @@
       <c r="J187" t="s">
         <v>1388</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -13468,7 +13494,7 @@
       <c r="J188" t="s">
         <v>1388</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -13509,7 +13535,7 @@
       <c r="J189" t="s">
         <v>1388</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -13550,7 +13576,7 @@
       <c r="J190" t="s">
         <v>1388</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -13591,7 +13617,7 @@
       <c r="J191" t="s">
         <v>1388</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -13632,7 +13658,7 @@
       <c r="J192" t="s">
         <v>1388</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -13673,7 +13699,7 @@
       <c r="J193" t="s">
         <v>1388</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -13714,7 +13740,7 @@
       <c r="J194" t="s">
         <v>1388</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -13755,7 +13781,7 @@
       <c r="J195" t="s">
         <v>1388</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -13799,7 +13825,7 @@
       <c r="J196" t="s">
         <v>1388</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -13843,7 +13869,7 @@
       <c r="J197" t="s">
         <v>1388</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -13884,7 +13910,7 @@
       <c r="J198" t="s">
         <v>1390</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -13925,7 +13951,7 @@
       <c r="J199" t="s">
         <v>1389</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -13966,7 +13992,7 @@
       <c r="J200" t="s">
         <v>1388</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -14007,7 +14033,7 @@
       <c r="J201" t="s">
         <v>1388</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -14048,7 +14074,7 @@
       <c r="J202" t="s">
         <v>1388</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -14089,7 +14115,7 @@
       <c r="J203" t="s">
         <v>1388</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -14130,7 +14156,7 @@
       <c r="J204" t="s">
         <v>1388</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -14174,7 +14200,7 @@
       <c r="J205" t="s">
         <v>1388</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -14218,7 +14244,7 @@
       <c r="J206" t="s">
         <v>1388</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -14259,7 +14285,7 @@
       <c r="J207" t="s">
         <v>1388</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -14300,7 +14326,7 @@
       <c r="J208" t="s">
         <v>1388</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -14341,7 +14367,7 @@
       <c r="J209" t="s">
         <v>1388</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -14382,7 +14408,7 @@
       <c r="J210" t="s">
         <v>1388</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -14423,7 +14449,7 @@
       <c r="J211" t="s">
         <v>1388</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -14464,7 +14490,7 @@
       <c r="J212" t="s">
         <v>1388</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -14505,7 +14531,7 @@
       <c r="J213" t="s">
         <v>1388</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -14546,7 +14572,7 @@
       <c r="J214" t="s">
         <v>1388</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -14587,7 +14613,7 @@
       <c r="J215" t="s">
         <v>1388</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -14628,7 +14654,7 @@
       <c r="J216" t="s">
         <v>1388</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -14669,7 +14695,7 @@
       <c r="J217" t="s">
         <v>1388</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -14710,7 +14736,7 @@
       <c r="J218" t="s">
         <v>1388</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -14751,7 +14777,7 @@
       <c r="J219" t="s">
         <v>1388</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -14792,7 +14818,7 @@
       <c r="J220" t="s">
         <v>1388</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -14833,7 +14859,7 @@
       <c r="J221" t="s">
         <v>1388</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -14874,7 +14900,7 @@
       <c r="J222" t="s">
         <v>1388</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -14915,7 +14941,7 @@
       <c r="J223" t="s">
         <v>1388</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -14956,7 +14982,7 @@
       <c r="J224" t="s">
         <v>1388</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -14997,7 +15023,7 @@
       <c r="J225" t="s">
         <v>1388</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -15038,7 +15064,7 @@
       <c r="J226" t="s">
         <v>1388</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -15079,7 +15105,7 @@
       <c r="J227" t="s">
         <v>1388</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -15120,7 +15146,7 @@
       <c r="J228" t="s">
         <v>1388</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -15161,7 +15187,7 @@
       <c r="J229" t="s">
         <v>1388</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -15202,7 +15228,7 @@
       <c r="J230" t="s">
         <v>1388</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -15243,7 +15269,7 @@
       <c r="J231" t="s">
         <v>1388</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -15284,7 +15310,7 @@
       <c r="J232" t="s">
         <v>1388</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -15325,7 +15351,7 @@
       <c r="J233" t="s">
         <v>1388</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -15366,7 +15392,7 @@
       <c r="J234" t="s">
         <v>1388</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -15407,7 +15433,7 @@
       <c r="J235" t="s">
         <v>1388</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -15448,7 +15474,7 @@
       <c r="J236" t="s">
         <v>1388</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -15489,7 +15515,7 @@
       <c r="J237" t="s">
         <v>1388</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -15530,7 +15556,7 @@
       <c r="J238" t="s">
         <v>1388</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -15571,7 +15597,7 @@
       <c r="J239" t="s">
         <v>1388</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -15612,7 +15638,7 @@
       <c r="J240" t="s">
         <v>1388</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -15653,7 +15679,7 @@
       <c r="J241" t="s">
         <v>1388</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -15694,7 +15720,7 @@
       <c r="J242" t="s">
         <v>1388</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -15735,7 +15761,7 @@
       <c r="J243" t="s">
         <v>1388</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -15776,7 +15802,7 @@
       <c r="J244" t="s">
         <v>1388</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -15817,7 +15843,7 @@
       <c r="J245" t="s">
         <v>1388</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -15858,7 +15884,7 @@
       <c r="J246" t="s">
         <v>1388</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -15899,7 +15925,7 @@
       <c r="J247" t="s">
         <v>1388</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -15940,7 +15966,7 @@
       <c r="J248" t="s">
         <v>1388</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -15981,7 +16007,7 @@
       <c r="J249" t="s">
         <v>1388</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -16022,7 +16048,7 @@
       <c r="J250" t="s">
         <v>1388</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -16063,7 +16089,7 @@
       <c r="J251" t="s">
         <v>1388</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -16104,7 +16130,7 @@
       <c r="J252" t="s">
         <v>1388</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -16145,7 +16171,7 @@
       <c r="J253" t="s">
         <v>1388</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -16189,7 +16215,7 @@
       <c r="J254" t="s">
         <v>1388</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -16230,7 +16256,7 @@
       <c r="J255" t="s">
         <v>1388</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -16271,7 +16297,7 @@
       <c r="J256" t="s">
         <v>1388</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -16315,7 +16341,7 @@
       <c r="J257" t="s">
         <v>1388</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -16324,7 +16350,7 @@
       <c r="M257" t="s">
         <v>1443</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -16368,7 +16394,7 @@
       <c r="J258" t="s">
         <v>1388</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -16412,7 +16438,7 @@
       <c r="J259" t="s">
         <v>1388</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -16456,7 +16482,7 @@
       <c r="J260" t="s">
         <v>1388</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -16465,7 +16491,7 @@
       <c r="M260" t="s">
         <v>1437</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -16509,7 +16535,7 @@
       <c r="J261" t="s">
         <v>1388</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -16553,7 +16579,7 @@
       <c r="J262" t="s">
         <v>1388</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -16597,7 +16623,7 @@
       <c r="J263" t="s">
         <v>1388</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -16606,7 +16632,7 @@
       <c r="M263" t="s">
         <v>1437</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -16650,7 +16676,7 @@
       <c r="J264" t="s">
         <v>1388</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -16691,7 +16717,7 @@
       <c r="J265" t="s">
         <v>1388</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -16732,7 +16758,7 @@
       <c r="J266" t="s">
         <v>1388</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -16773,7 +16799,7 @@
       <c r="J267" t="s">
         <v>1388</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -16817,7 +16843,7 @@
       <c r="J268" t="s">
         <v>1388</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -16858,7 +16884,7 @@
       <c r="J269" t="s">
         <v>1388</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -16899,7 +16925,7 @@
       <c r="J270" t="s">
         <v>1388</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -16940,7 +16966,7 @@
       <c r="J271" t="s">
         <v>1388</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -16981,7 +17007,7 @@
       <c r="J272" t="s">
         <v>1388</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -17025,7 +17051,7 @@
       <c r="J273" t="s">
         <v>1388</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -17069,7 +17095,7 @@
       <c r="J274" t="s">
         <v>1388</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -17110,7 +17136,7 @@
       <c r="J275" t="s">
         <v>1388</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -17151,7 +17177,7 @@
       <c r="J276" t="s">
         <v>1388</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -17192,7 +17218,7 @@
       <c r="J277" t="s">
         <v>1388</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -17233,7 +17259,7 @@
       <c r="J278" t="s">
         <v>1388</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -17274,7 +17300,7 @@
       <c r="J279" t="s">
         <v>1388</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -17315,7 +17341,7 @@
       <c r="J280" t="s">
         <v>1388</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -17356,7 +17382,7 @@
       <c r="J281" t="s">
         <v>1388</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -17397,7 +17423,7 @@
       <c r="J282" t="s">
         <v>1388</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -17438,7 +17464,7 @@
       <c r="J283" t="s">
         <v>1388</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -17479,7 +17505,7 @@
       <c r="J284" t="s">
         <v>1388</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -17520,7 +17546,7 @@
       <c r="J285" t="s">
         <v>1388</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -17561,7 +17587,7 @@
       <c r="J286" t="s">
         <v>1388</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -17602,7 +17628,7 @@
       <c r="J287" t="s">
         <v>1388</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -17643,7 +17669,7 @@
       <c r="J288" t="s">
         <v>1388</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -17684,7 +17710,7 @@
       <c r="J289" t="s">
         <v>1388</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -17725,7 +17751,7 @@
       <c r="J290" t="s">
         <v>1388</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -17766,7 +17792,7 @@
       <c r="J291" t="s">
         <v>1388</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -17807,7 +17833,7 @@
       <c r="J292" t="s">
         <v>1388</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -17848,7 +17874,7 @@
       <c r="J293" t="s">
         <v>1388</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -17889,7 +17915,7 @@
       <c r="J294" t="s">
         <v>1388</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -17930,7 +17956,7 @@
       <c r="J295" t="s">
         <v>1388</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -17974,7 +18000,7 @@
       <c r="J296" t="s">
         <v>1388</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -18018,7 +18044,7 @@
       <c r="J297" t="s">
         <v>1388</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -18059,7 +18085,7 @@
       <c r="J298" t="s">
         <v>1388</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -18100,7 +18126,7 @@
       <c r="J299" t="s">
         <v>1389</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -18141,7 +18167,7 @@
       <c r="J300" t="s">
         <v>1388</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -18182,7 +18208,7 @@
       <c r="J301" t="s">
         <v>1388</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (22/07/2026 16:11)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -4616,16 +4616,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -4641,7 +4633,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -4649,30 +4641,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4972,73 +4946,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5073,7 +5047,7 @@
       <c r="J2" t="s">
         <v>1388</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5117,7 +5091,7 @@
       <c r="J3" t="s">
         <v>1388</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5161,7 +5135,7 @@
       <c r="J4" t="s">
         <v>1388</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5205,7 +5179,7 @@
       <c r="J5" t="s">
         <v>1389</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5255,7 +5229,7 @@
       <c r="J6" t="s">
         <v>1388</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5302,7 +5276,7 @@
       <c r="J7" t="s">
         <v>1388</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5349,7 +5323,7 @@
       <c r="J8" t="s">
         <v>1388</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5396,7 +5370,7 @@
       <c r="J9" t="s">
         <v>1388</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5443,7 +5417,7 @@
       <c r="J10" t="s">
         <v>1388</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -5490,7 +5464,7 @@
       <c r="J11" t="s">
         <v>1388</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -5537,7 +5511,7 @@
       <c r="J12" t="s">
         <v>1388</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -5581,7 +5555,7 @@
       <c r="J13" t="s">
         <v>1388</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -5625,7 +5599,7 @@
       <c r="J14" t="s">
         <v>1388</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -5669,7 +5643,7 @@
       <c r="J15" t="s">
         <v>1388</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -5713,7 +5687,7 @@
       <c r="J16" t="s">
         <v>1388</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -5757,7 +5731,7 @@
       <c r="J17" t="s">
         <v>1388</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -5801,7 +5775,7 @@
       <c r="J18" t="s">
         <v>1388</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -5819,7 +5793,7 @@
       <c r="R18" t="s">
         <v>1479</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -5860,7 +5834,7 @@
       <c r="J19" t="s">
         <v>1388</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -5904,7 +5878,7 @@
       <c r="J20" t="s">
         <v>1388</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -5948,7 +5922,7 @@
       <c r="J21" t="s">
         <v>1388</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -5966,7 +5940,7 @@
       <c r="R21" t="s">
         <v>1480</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6007,7 +5981,7 @@
       <c r="J22" t="s">
         <v>1388</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6025,7 +5999,7 @@
       <c r="R22" t="s">
         <v>1481</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6066,7 +6040,7 @@
       <c r="J23" t="s">
         <v>1388</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6084,7 +6058,7 @@
       <c r="R23" t="s">
         <v>1482</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6125,7 +6099,7 @@
       <c r="J24" t="s">
         <v>1388</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6169,7 +6143,7 @@
       <c r="J25" t="s">
         <v>1388</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6210,7 +6184,7 @@
       <c r="J26" t="s">
         <v>1390</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6251,7 +6225,7 @@
       <c r="J27" t="s">
         <v>1388</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6269,7 +6243,7 @@
       <c r="R27" t="s">
         <v>1483</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6310,7 +6284,7 @@
       <c r="J28" t="s">
         <v>1388</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6354,7 +6328,7 @@
       <c r="J29" t="s">
         <v>1388</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6398,7 +6372,7 @@
       <c r="J30" t="s">
         <v>1388</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -6442,7 +6416,7 @@
       <c r="J31" t="s">
         <v>1388</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -6460,7 +6434,7 @@
       <c r="R31" t="s">
         <v>1484</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -6501,7 +6475,7 @@
       <c r="J32" t="s">
         <v>1388</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -6545,7 +6519,7 @@
       <c r="J33" t="s">
         <v>1388</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -6563,7 +6537,7 @@
       <c r="R33" t="s">
         <v>1485</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -6604,7 +6578,7 @@
       <c r="J34" t="s">
         <v>1388</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -6648,7 +6622,7 @@
       <c r="J35" t="s">
         <v>1388</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -6666,7 +6640,7 @@
       <c r="R35" t="s">
         <v>1486</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -6707,7 +6681,7 @@
       <c r="J36" t="s">
         <v>1388</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -6725,7 +6699,7 @@
       <c r="R36" t="s">
         <v>1486</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -6766,7 +6740,7 @@
       <c r="J37" t="s">
         <v>1388</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -6784,7 +6758,7 @@
       <c r="R37" t="s">
         <v>1486</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -6825,7 +6799,7 @@
       <c r="J38" t="s">
         <v>1388</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -6843,7 +6817,7 @@
       <c r="R38" t="s">
         <v>1486</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -6884,7 +6858,7 @@
       <c r="J39" t="s">
         <v>1388</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -6902,7 +6876,7 @@
       <c r="R39" t="s">
         <v>1486</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -6943,7 +6917,7 @@
       <c r="J40" t="s">
         <v>1388</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -6961,7 +6935,7 @@
       <c r="R40" t="s">
         <v>1487</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7002,7 +6976,7 @@
       <c r="J41" t="s">
         <v>1388</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7046,7 +7020,7 @@
       <c r="J42" t="s">
         <v>1388</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7064,7 +7038,7 @@
       <c r="R42" t="s">
         <v>1486</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7105,7 +7079,7 @@
       <c r="J43" t="s">
         <v>1388</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7149,7 +7123,7 @@
       <c r="J44" t="s">
         <v>1388</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7167,7 +7141,7 @@
       <c r="R44" t="s">
         <v>1488</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7208,7 +7182,7 @@
       <c r="J45" t="s">
         <v>1388</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7252,7 +7226,7 @@
       <c r="J46" t="s">
         <v>1388</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7296,7 +7270,7 @@
       <c r="J47" t="s">
         <v>1388</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7314,7 +7288,7 @@
       <c r="R47" t="s">
         <v>1489</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7355,7 +7329,7 @@
       <c r="J48" t="s">
         <v>1388</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -7399,7 +7373,7 @@
       <c r="J49" t="s">
         <v>1388</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -7443,7 +7417,7 @@
       <c r="J50" t="s">
         <v>1388</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -7487,7 +7461,7 @@
       <c r="J51" t="s">
         <v>1388</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -7534,7 +7508,7 @@
       <c r="J52" t="s">
         <v>1388</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -7578,7 +7552,7 @@
       <c r="J53" t="s">
         <v>1388</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -7622,7 +7596,7 @@
       <c r="J54" t="s">
         <v>1388</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -7666,7 +7640,7 @@
       <c r="J55" t="s">
         <v>1388</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -7716,7 +7690,7 @@
       <c r="J56" t="s">
         <v>1388</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -7769,7 +7743,7 @@
       <c r="J57" t="s">
         <v>1388</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -7819,7 +7793,7 @@
       <c r="J58" t="s">
         <v>1388</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -7869,7 +7843,7 @@
       <c r="J59" t="s">
         <v>1388</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -7887,7 +7861,7 @@
       <c r="R59" t="s">
         <v>1490</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -7928,7 +7902,7 @@
       <c r="J60" t="s">
         <v>1388</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -7972,7 +7946,7 @@
       <c r="J61" t="s">
         <v>1388</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8016,7 +7990,7 @@
       <c r="J62" t="s">
         <v>1388</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8060,7 +8034,7 @@
       <c r="J63" t="s">
         <v>1388</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8104,7 +8078,7 @@
       <c r="J64" t="s">
         <v>1388</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8148,7 +8122,7 @@
       <c r="J65" t="s">
         <v>1388</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8195,7 +8169,7 @@
       <c r="J66" t="s">
         <v>1388</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8239,7 +8213,7 @@
       <c r="J67" t="s">
         <v>1388</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8283,7 +8257,7 @@
       <c r="J68" t="s">
         <v>1388</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8298,7 +8272,7 @@
       <c r="O68" t="s">
         <v>1455</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8342,7 +8316,7 @@
       <c r="J69" t="s">
         <v>1390</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -8386,7 +8360,7 @@
       <c r="J70" t="s">
         <v>1388</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -8430,7 +8404,7 @@
       <c r="J71" t="s">
         <v>1388</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -8474,7 +8448,7 @@
       <c r="J72" t="s">
         <v>1388</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -8518,7 +8492,7 @@
       <c r="J73" t="s">
         <v>1388</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -8562,7 +8536,7 @@
       <c r="J74" t="s">
         <v>1388</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -8606,7 +8580,7 @@
       <c r="J75" t="s">
         <v>1388</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -8650,7 +8624,7 @@
       <c r="J76" t="s">
         <v>1388</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -8694,7 +8668,7 @@
       <c r="J77" t="s">
         <v>1388</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -8738,7 +8712,7 @@
       <c r="J78" t="s">
         <v>1388</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -8782,7 +8756,7 @@
       <c r="J79" t="s">
         <v>1388</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -8826,7 +8800,7 @@
       <c r="J80" t="s">
         <v>1388</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -8870,7 +8844,7 @@
       <c r="J81" t="s">
         <v>1388</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -8914,7 +8888,7 @@
       <c r="J82" t="s">
         <v>1388</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -8958,7 +8932,7 @@
       <c r="J83" t="s">
         <v>1388</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9002,7 +8976,7 @@
       <c r="J84" t="s">
         <v>1388</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9046,7 +9020,7 @@
       <c r="J85" t="s">
         <v>1388</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9090,7 +9064,7 @@
       <c r="J86" t="s">
         <v>1388</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9134,7 +9108,7 @@
       <c r="J87" t="s">
         <v>1388</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9178,7 +9152,7 @@
       <c r="J88" t="s">
         <v>1388</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9222,7 +9196,7 @@
       <c r="J89" t="s">
         <v>1388</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9263,7 +9237,7 @@
       <c r="J90" t="s">
         <v>1388</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -9304,7 +9278,7 @@
       <c r="J91" t="s">
         <v>1388</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -9348,7 +9322,7 @@
       <c r="J92" t="s">
         <v>1388</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -9369,7 +9343,7 @@
       <c r="R92" t="s">
         <v>1482</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -9410,7 +9384,7 @@
       <c r="J93" t="s">
         <v>1388</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -9451,7 +9425,7 @@
       <c r="J94" t="s">
         <v>1388</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -9495,7 +9469,7 @@
       <c r="J95" t="s">
         <v>1388</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -9539,7 +9513,7 @@
       <c r="J96" t="s">
         <v>1388</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -9586,7 +9560,7 @@
       <c r="J97" t="s">
         <v>1388</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -9601,7 +9575,7 @@
       <c r="R97" t="s">
         <v>1491</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -9642,7 +9616,7 @@
       <c r="J98" t="s">
         <v>1388</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -9686,7 +9660,7 @@
       <c r="J99" t="s">
         <v>1388</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -9730,7 +9704,7 @@
       <c r="J100" t="s">
         <v>1388</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -9771,7 +9745,7 @@
       <c r="J101" t="s">
         <v>1388</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -9812,7 +9786,7 @@
       <c r="J102" t="s">
         <v>1388</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -9853,7 +9827,7 @@
       <c r="J103" t="s">
         <v>1388</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -9894,7 +9868,7 @@
       <c r="J104" t="s">
         <v>1388</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -9935,7 +9909,7 @@
       <c r="J105" t="s">
         <v>1388</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -9976,7 +9950,7 @@
       <c r="J106" t="s">
         <v>1388</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10017,7 +9991,7 @@
       <c r="J107" t="s">
         <v>1388</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10058,7 +10032,7 @@
       <c r="J108" t="s">
         <v>1388</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10099,7 +10073,7 @@
       <c r="J109" t="s">
         <v>1388</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10140,7 +10114,7 @@
       <c r="J110" t="s">
         <v>1388</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10158,7 +10132,7 @@
       <c r="R110" t="s">
         <v>1492</v>
       </c>
-      <c r="T110" s="2">
+      <c r="T110" s="1">
         <v>45805</v>
       </c>
       <c r="U110" t="s">
@@ -10196,7 +10170,7 @@
       <c r="J111" t="s">
         <v>1388</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -10214,7 +10188,7 @@
       <c r="R111" t="s">
         <v>1493</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -10252,7 +10226,7 @@
       <c r="J112" t="s">
         <v>1388</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -10270,7 +10244,7 @@
       <c r="R112" t="s">
         <v>1494</v>
       </c>
-      <c r="T112" s="2">
+      <c r="T112" s="1">
         <v>46052</v>
       </c>
       <c r="U112" t="s">
@@ -10311,7 +10285,7 @@
       <c r="J113" t="s">
         <v>1388</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -10355,7 +10329,7 @@
       <c r="J114" t="s">
         <v>1388</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -10399,7 +10373,7 @@
       <c r="J115" t="s">
         <v>1388</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -10443,7 +10417,7 @@
       <c r="J116" t="s">
         <v>1388</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -10461,7 +10435,7 @@
       <c r="R116" t="s">
         <v>1495</v>
       </c>
-      <c r="T116" s="2">
+      <c r="T116" s="1">
         <v>46048</v>
       </c>
       <c r="U116" t="s">
@@ -10502,7 +10476,7 @@
       <c r="J117" t="s">
         <v>1388</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -10546,7 +10520,7 @@
       <c r="J118" t="s">
         <v>1388</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -10593,7 +10567,7 @@
       <c r="J119" t="s">
         <v>1388</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -10634,7 +10608,7 @@
       <c r="J120" t="s">
         <v>1388</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -10678,7 +10652,7 @@
       <c r="J121" t="s">
         <v>1388</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -10722,7 +10696,7 @@
       <c r="J122" t="s">
         <v>1388</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -10772,7 +10746,7 @@
       <c r="J123" t="s">
         <v>1388</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -10816,7 +10790,7 @@
       <c r="J124" t="s">
         <v>1388</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -10860,7 +10834,7 @@
       <c r="J125" t="s">
         <v>1388</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -10901,7 +10875,7 @@
       <c r="J126" t="s">
         <v>1388</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -10942,7 +10916,7 @@
       <c r="J127" t="s">
         <v>1388</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -10960,7 +10934,7 @@
       <c r="R127" t="s">
         <v>1497</v>
       </c>
-      <c r="T127" s="2">
+      <c r="T127" s="1">
         <v>45889</v>
       </c>
       <c r="U127" t="s">
@@ -10998,7 +10972,7 @@
       <c r="J128" t="s">
         <v>1388</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11039,7 +11013,7 @@
       <c r="J129" t="s">
         <v>1388</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11080,7 +11054,7 @@
       <c r="J130" t="s">
         <v>1388</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11121,7 +11095,7 @@
       <c r="J131" t="s">
         <v>1388</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11165,7 +11139,7 @@
       <c r="J132" t="s">
         <v>1388</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -11206,7 +11180,7 @@
       <c r="J133" t="s">
         <v>1388</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -11247,7 +11221,7 @@
       <c r="J134" t="s">
         <v>1388</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -11288,7 +11262,7 @@
       <c r="J135" t="s">
         <v>1388</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -11329,7 +11303,7 @@
       <c r="J136" t="s">
         <v>1388</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -11370,7 +11344,7 @@
       <c r="J137" t="s">
         <v>1388</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -11411,7 +11385,7 @@
       <c r="J138" t="s">
         <v>1388</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -11452,7 +11426,7 @@
       <c r="J139" t="s">
         <v>1388</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -11499,7 +11473,7 @@
       <c r="J140" t="s">
         <v>1388</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -11540,7 +11514,7 @@
       <c r="J141" t="s">
         <v>1388</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -11581,7 +11555,7 @@
       <c r="J142" t="s">
         <v>1388</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -11625,7 +11599,7 @@
       <c r="J143" t="s">
         <v>1388</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -11666,7 +11640,7 @@
       <c r="J144" t="s">
         <v>1388</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -11707,7 +11681,7 @@
       <c r="J145" t="s">
         <v>1388</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -11748,7 +11722,7 @@
       <c r="J146" t="s">
         <v>1388</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -11789,7 +11763,7 @@
       <c r="J147" t="s">
         <v>1388</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -11830,7 +11804,7 @@
       <c r="J148" t="s">
         <v>1388</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -11871,7 +11845,7 @@
       <c r="J149" t="s">
         <v>1388</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -11912,7 +11886,7 @@
       <c r="J150" t="s">
         <v>1388</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -11953,7 +11927,7 @@
       <c r="J151" t="s">
         <v>1388</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -11994,7 +11968,7 @@
       <c r="J152" t="s">
         <v>1388</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12035,7 +12009,7 @@
       <c r="J153" t="s">
         <v>1388</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -12044,7 +12018,7 @@
       <c r="M153" t="s">
         <v>1446</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -12085,7 +12059,7 @@
       <c r="J154" t="s">
         <v>1388</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -12126,7 +12100,7 @@
       <c r="J155" t="s">
         <v>1388</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -12167,7 +12141,7 @@
       <c r="J156" t="s">
         <v>1388</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -12208,7 +12182,7 @@
       <c r="J157" t="s">
         <v>1388</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -12249,7 +12223,7 @@
       <c r="J158" t="s">
         <v>1388</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -12290,7 +12264,7 @@
       <c r="J159" t="s">
         <v>1388</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -12331,7 +12305,7 @@
       <c r="J160" t="s">
         <v>1388</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -12372,7 +12346,7 @@
       <c r="J161" t="s">
         <v>1388</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -12413,7 +12387,7 @@
       <c r="J162" t="s">
         <v>1388</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -12454,7 +12428,7 @@
       <c r="J163" t="s">
         <v>1388</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -12495,7 +12469,7 @@
       <c r="J164" t="s">
         <v>1388</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -12536,7 +12510,7 @@
       <c r="J165" t="s">
         <v>1388</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -12577,7 +12551,7 @@
       <c r="J166" t="s">
         <v>1388</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -12618,7 +12592,7 @@
       <c r="J167" t="s">
         <v>1388</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -12662,7 +12636,7 @@
       <c r="J168" t="s">
         <v>1388</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -12706,7 +12680,7 @@
       <c r="J169" t="s">
         <v>1388</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -12747,7 +12721,7 @@
       <c r="J170" t="s">
         <v>1388</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -12788,7 +12762,7 @@
       <c r="J171" t="s">
         <v>1388</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -12829,7 +12803,7 @@
       <c r="J172" t="s">
         <v>1388</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -12870,7 +12844,7 @@
       <c r="J173" t="s">
         <v>1388</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -12911,7 +12885,7 @@
       <c r="J174" t="s">
         <v>1388</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -12952,7 +12926,7 @@
       <c r="J175" t="s">
         <v>1388</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -12993,7 +12967,7 @@
       <c r="J176" t="s">
         <v>1388</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -13034,7 +13008,7 @@
       <c r="J177" t="s">
         <v>1388</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -13075,7 +13049,7 @@
       <c r="J178" t="s">
         <v>1388</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -13116,7 +13090,7 @@
       <c r="J179" t="s">
         <v>1388</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -13125,7 +13099,7 @@
       <c r="M179" t="s">
         <v>1443</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -13166,7 +13140,7 @@
       <c r="J180" t="s">
         <v>1388</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -13207,7 +13181,7 @@
       <c r="J181" t="s">
         <v>1388</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -13248,7 +13222,7 @@
       <c r="J182" t="s">
         <v>1388</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -13289,7 +13263,7 @@
       <c r="J183" t="s">
         <v>1388</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -13330,7 +13304,7 @@
       <c r="J184" t="s">
         <v>1388</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -13371,7 +13345,7 @@
       <c r="J185" t="s">
         <v>1388</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -13412,7 +13386,7 @@
       <c r="J186" t="s">
         <v>1388</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -13453,7 +13427,7 @@
       <c r="J187" t="s">
         <v>1388</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -13494,7 +13468,7 @@
       <c r="J188" t="s">
         <v>1388</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -13535,7 +13509,7 @@
       <c r="J189" t="s">
         <v>1388</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -13576,7 +13550,7 @@
       <c r="J190" t="s">
         <v>1388</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -13617,7 +13591,7 @@
       <c r="J191" t="s">
         <v>1388</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -13658,7 +13632,7 @@
       <c r="J192" t="s">
         <v>1388</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -13699,7 +13673,7 @@
       <c r="J193" t="s">
         <v>1388</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -13740,7 +13714,7 @@
       <c r="J194" t="s">
         <v>1388</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -13781,7 +13755,7 @@
       <c r="J195" t="s">
         <v>1388</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -13825,7 +13799,7 @@
       <c r="J196" t="s">
         <v>1388</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -13869,7 +13843,7 @@
       <c r="J197" t="s">
         <v>1388</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -13910,7 +13884,7 @@
       <c r="J198" t="s">
         <v>1390</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -13951,7 +13925,7 @@
       <c r="J199" t="s">
         <v>1389</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -13992,7 +13966,7 @@
       <c r="J200" t="s">
         <v>1388</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -14033,7 +14007,7 @@
       <c r="J201" t="s">
         <v>1388</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -14074,7 +14048,7 @@
       <c r="J202" t="s">
         <v>1388</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -14115,7 +14089,7 @@
       <c r="J203" t="s">
         <v>1388</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -14156,7 +14130,7 @@
       <c r="J204" t="s">
         <v>1388</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -14200,7 +14174,7 @@
       <c r="J205" t="s">
         <v>1388</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -14244,7 +14218,7 @@
       <c r="J206" t="s">
         <v>1388</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -14285,7 +14259,7 @@
       <c r="J207" t="s">
         <v>1388</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -14326,7 +14300,7 @@
       <c r="J208" t="s">
         <v>1388</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -14367,7 +14341,7 @@
       <c r="J209" t="s">
         <v>1388</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -14408,7 +14382,7 @@
       <c r="J210" t="s">
         <v>1388</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -14449,7 +14423,7 @@
       <c r="J211" t="s">
         <v>1388</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -14490,7 +14464,7 @@
       <c r="J212" t="s">
         <v>1388</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -14531,7 +14505,7 @@
       <c r="J213" t="s">
         <v>1388</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -14572,7 +14546,7 @@
       <c r="J214" t="s">
         <v>1388</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -14613,7 +14587,7 @@
       <c r="J215" t="s">
         <v>1388</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -14654,7 +14628,7 @@
       <c r="J216" t="s">
         <v>1388</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -14695,7 +14669,7 @@
       <c r="J217" t="s">
         <v>1388</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -14736,7 +14710,7 @@
       <c r="J218" t="s">
         <v>1388</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -14777,7 +14751,7 @@
       <c r="J219" t="s">
         <v>1388</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -14818,7 +14792,7 @@
       <c r="J220" t="s">
         <v>1388</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -14859,7 +14833,7 @@
       <c r="J221" t="s">
         <v>1388</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -14900,7 +14874,7 @@
       <c r="J222" t="s">
         <v>1388</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -14941,7 +14915,7 @@
       <c r="J223" t="s">
         <v>1388</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -14982,7 +14956,7 @@
       <c r="J224" t="s">
         <v>1388</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -15023,7 +14997,7 @@
       <c r="J225" t="s">
         <v>1388</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -15064,7 +15038,7 @@
       <c r="J226" t="s">
         <v>1388</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -15105,7 +15079,7 @@
       <c r="J227" t="s">
         <v>1388</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -15146,7 +15120,7 @@
       <c r="J228" t="s">
         <v>1388</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -15187,7 +15161,7 @@
       <c r="J229" t="s">
         <v>1388</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -15228,7 +15202,7 @@
       <c r="J230" t="s">
         <v>1388</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -15269,7 +15243,7 @@
       <c r="J231" t="s">
         <v>1388</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -15310,7 +15284,7 @@
       <c r="J232" t="s">
         <v>1388</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -15351,7 +15325,7 @@
       <c r="J233" t="s">
         <v>1388</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -15392,7 +15366,7 @@
       <c r="J234" t="s">
         <v>1388</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -15433,7 +15407,7 @@
       <c r="J235" t="s">
         <v>1388</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -15474,7 +15448,7 @@
       <c r="J236" t="s">
         <v>1388</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -15515,7 +15489,7 @@
       <c r="J237" t="s">
         <v>1388</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -15556,7 +15530,7 @@
       <c r="J238" t="s">
         <v>1388</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -15597,7 +15571,7 @@
       <c r="J239" t="s">
         <v>1388</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -15638,7 +15612,7 @@
       <c r="J240" t="s">
         <v>1388</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -15679,7 +15653,7 @@
       <c r="J241" t="s">
         <v>1388</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -15720,7 +15694,7 @@
       <c r="J242" t="s">
         <v>1388</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -15761,7 +15735,7 @@
       <c r="J243" t="s">
         <v>1388</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -15802,7 +15776,7 @@
       <c r="J244" t="s">
         <v>1388</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -15843,7 +15817,7 @@
       <c r="J245" t="s">
         <v>1388</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -15884,7 +15858,7 @@
       <c r="J246" t="s">
         <v>1388</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -15925,7 +15899,7 @@
       <c r="J247" t="s">
         <v>1388</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -15966,7 +15940,7 @@
       <c r="J248" t="s">
         <v>1388</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -16007,7 +15981,7 @@
       <c r="J249" t="s">
         <v>1388</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -16048,7 +16022,7 @@
       <c r="J250" t="s">
         <v>1388</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -16089,7 +16063,7 @@
       <c r="J251" t="s">
         <v>1388</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -16130,7 +16104,7 @@
       <c r="J252" t="s">
         <v>1388</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -16171,7 +16145,7 @@
       <c r="J253" t="s">
         <v>1388</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -16215,7 +16189,7 @@
       <c r="J254" t="s">
         <v>1388</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -16256,7 +16230,7 @@
       <c r="J255" t="s">
         <v>1388</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -16297,7 +16271,7 @@
       <c r="J256" t="s">
         <v>1388</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -16341,7 +16315,7 @@
       <c r="J257" t="s">
         <v>1388</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -16350,7 +16324,7 @@
       <c r="M257" t="s">
         <v>1443</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -16394,7 +16368,7 @@
       <c r="J258" t="s">
         <v>1388</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -16438,7 +16412,7 @@
       <c r="J259" t="s">
         <v>1388</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -16482,7 +16456,7 @@
       <c r="J260" t="s">
         <v>1388</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -16491,7 +16465,7 @@
       <c r="M260" t="s">
         <v>1437</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -16535,7 +16509,7 @@
       <c r="J261" t="s">
         <v>1388</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -16579,7 +16553,7 @@
       <c r="J262" t="s">
         <v>1388</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -16623,7 +16597,7 @@
       <c r="J263" t="s">
         <v>1388</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -16632,7 +16606,7 @@
       <c r="M263" t="s">
         <v>1437</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -16676,7 +16650,7 @@
       <c r="J264" t="s">
         <v>1388</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -16717,7 +16691,7 @@
       <c r="J265" t="s">
         <v>1388</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -16758,7 +16732,7 @@
       <c r="J266" t="s">
         <v>1388</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -16799,7 +16773,7 @@
       <c r="J267" t="s">
         <v>1388</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -16843,7 +16817,7 @@
       <c r="J268" t="s">
         <v>1388</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -16884,7 +16858,7 @@
       <c r="J269" t="s">
         <v>1388</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -16925,7 +16899,7 @@
       <c r="J270" t="s">
         <v>1388</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -16966,7 +16940,7 @@
       <c r="J271" t="s">
         <v>1388</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -17007,7 +16981,7 @@
       <c r="J272" t="s">
         <v>1388</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -17051,7 +17025,7 @@
       <c r="J273" t="s">
         <v>1388</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -17095,7 +17069,7 @@
       <c r="J274" t="s">
         <v>1388</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -17136,7 +17110,7 @@
       <c r="J275" t="s">
         <v>1388</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -17177,7 +17151,7 @@
       <c r="J276" t="s">
         <v>1388</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -17218,7 +17192,7 @@
       <c r="J277" t="s">
         <v>1388</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -17259,7 +17233,7 @@
       <c r="J278" t="s">
         <v>1388</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -17300,7 +17274,7 @@
       <c r="J279" t="s">
         <v>1388</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -17341,7 +17315,7 @@
       <c r="J280" t="s">
         <v>1388</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -17382,7 +17356,7 @@
       <c r="J281" t="s">
         <v>1388</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -17423,7 +17397,7 @@
       <c r="J282" t="s">
         <v>1388</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -17464,7 +17438,7 @@
       <c r="J283" t="s">
         <v>1388</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -17505,7 +17479,7 @@
       <c r="J284" t="s">
         <v>1388</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -17546,7 +17520,7 @@
       <c r="J285" t="s">
         <v>1388</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -17587,7 +17561,7 @@
       <c r="J286" t="s">
         <v>1388</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -17628,7 +17602,7 @@
       <c r="J287" t="s">
         <v>1388</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -17669,7 +17643,7 @@
       <c r="J288" t="s">
         <v>1388</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -17710,7 +17684,7 @@
       <c r="J289" t="s">
         <v>1388</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -17751,7 +17725,7 @@
       <c r="J290" t="s">
         <v>1388</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -17792,7 +17766,7 @@
       <c r="J291" t="s">
         <v>1388</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -17833,7 +17807,7 @@
       <c r="J292" t="s">
         <v>1388</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -17874,7 +17848,7 @@
       <c r="J293" t="s">
         <v>1388</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -17915,7 +17889,7 @@
       <c r="J294" t="s">
         <v>1388</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -17956,7 +17930,7 @@
       <c r="J295" t="s">
         <v>1388</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -18000,7 +17974,7 @@
       <c r="J296" t="s">
         <v>1388</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -18044,7 +18018,7 @@
       <c r="J297" t="s">
         <v>1388</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -18085,7 +18059,7 @@
       <c r="J298" t="s">
         <v>1388</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -18126,7 +18100,7 @@
       <c r="J299" t="s">
         <v>1389</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -18167,7 +18141,7 @@
       <c r="J300" t="s">
         <v>1388</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -18208,7 +18182,7 @@
       <c r="J301" t="s">
         <v>1388</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (23/07/2026 11:42)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -4616,8 +4616,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -4633,7 +4641,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -4641,12 +4649,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4946,73 +4972,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5047,7 +5073,7 @@
       <c r="J2" t="s">
         <v>1388</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5091,7 +5117,7 @@
       <c r="J3" t="s">
         <v>1388</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5135,7 +5161,7 @@
       <c r="J4" t="s">
         <v>1388</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5179,7 +5205,7 @@
       <c r="J5" t="s">
         <v>1389</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5229,7 +5255,7 @@
       <c r="J6" t="s">
         <v>1388</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5276,7 +5302,7 @@
       <c r="J7" t="s">
         <v>1388</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5323,7 +5349,7 @@
       <c r="J8" t="s">
         <v>1388</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5370,7 +5396,7 @@
       <c r="J9" t="s">
         <v>1388</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5417,7 +5443,7 @@
       <c r="J10" t="s">
         <v>1388</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -5464,7 +5490,7 @@
       <c r="J11" t="s">
         <v>1388</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -5511,7 +5537,7 @@
       <c r="J12" t="s">
         <v>1388</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -5555,7 +5581,7 @@
       <c r="J13" t="s">
         <v>1388</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -5599,7 +5625,7 @@
       <c r="J14" t="s">
         <v>1388</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -5643,7 +5669,7 @@
       <c r="J15" t="s">
         <v>1388</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -5687,7 +5713,7 @@
       <c r="J16" t="s">
         <v>1388</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -5731,7 +5757,7 @@
       <c r="J17" t="s">
         <v>1388</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -5775,7 +5801,7 @@
       <c r="J18" t="s">
         <v>1388</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -5793,7 +5819,7 @@
       <c r="R18" t="s">
         <v>1479</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -5834,7 +5860,7 @@
       <c r="J19" t="s">
         <v>1388</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -5878,7 +5904,7 @@
       <c r="J20" t="s">
         <v>1388</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -5922,7 +5948,7 @@
       <c r="J21" t="s">
         <v>1388</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -5940,7 +5966,7 @@
       <c r="R21" t="s">
         <v>1480</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -5981,7 +6007,7 @@
       <c r="J22" t="s">
         <v>1388</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -5999,7 +6025,7 @@
       <c r="R22" t="s">
         <v>1481</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6040,7 +6066,7 @@
       <c r="J23" t="s">
         <v>1388</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6058,7 +6084,7 @@
       <c r="R23" t="s">
         <v>1482</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6099,7 +6125,7 @@
       <c r="J24" t="s">
         <v>1388</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6143,7 +6169,7 @@
       <c r="J25" t="s">
         <v>1388</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6184,7 +6210,7 @@
       <c r="J26" t="s">
         <v>1390</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6225,7 +6251,7 @@
       <c r="J27" t="s">
         <v>1388</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6243,7 +6269,7 @@
       <c r="R27" t="s">
         <v>1483</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6284,7 +6310,7 @@
       <c r="J28" t="s">
         <v>1388</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6328,7 +6354,7 @@
       <c r="J29" t="s">
         <v>1388</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6372,7 +6398,7 @@
       <c r="J30" t="s">
         <v>1388</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -6416,7 +6442,7 @@
       <c r="J31" t="s">
         <v>1388</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -6434,7 +6460,7 @@
       <c r="R31" t="s">
         <v>1484</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -6475,7 +6501,7 @@
       <c r="J32" t="s">
         <v>1388</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -6519,7 +6545,7 @@
       <c r="J33" t="s">
         <v>1388</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -6537,7 +6563,7 @@
       <c r="R33" t="s">
         <v>1485</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -6578,7 +6604,7 @@
       <c r="J34" t="s">
         <v>1388</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -6622,7 +6648,7 @@
       <c r="J35" t="s">
         <v>1388</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -6640,7 +6666,7 @@
       <c r="R35" t="s">
         <v>1486</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -6681,7 +6707,7 @@
       <c r="J36" t="s">
         <v>1388</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -6699,7 +6725,7 @@
       <c r="R36" t="s">
         <v>1486</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -6740,7 +6766,7 @@
       <c r="J37" t="s">
         <v>1388</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -6758,7 +6784,7 @@
       <c r="R37" t="s">
         <v>1486</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -6799,7 +6825,7 @@
       <c r="J38" t="s">
         <v>1388</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -6817,7 +6843,7 @@
       <c r="R38" t="s">
         <v>1486</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -6858,7 +6884,7 @@
       <c r="J39" t="s">
         <v>1388</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -6876,7 +6902,7 @@
       <c r="R39" t="s">
         <v>1486</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -6917,7 +6943,7 @@
       <c r="J40" t="s">
         <v>1388</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -6935,7 +6961,7 @@
       <c r="R40" t="s">
         <v>1487</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -6976,7 +7002,7 @@
       <c r="J41" t="s">
         <v>1388</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7020,7 +7046,7 @@
       <c r="J42" t="s">
         <v>1388</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7038,7 +7064,7 @@
       <c r="R42" t="s">
         <v>1486</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7079,7 +7105,7 @@
       <c r="J43" t="s">
         <v>1388</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7123,7 +7149,7 @@
       <c r="J44" t="s">
         <v>1388</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7141,7 +7167,7 @@
       <c r="R44" t="s">
         <v>1488</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7182,7 +7208,7 @@
       <c r="J45" t="s">
         <v>1388</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7226,7 +7252,7 @@
       <c r="J46" t="s">
         <v>1388</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7270,7 +7296,7 @@
       <c r="J47" t="s">
         <v>1388</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7288,7 +7314,7 @@
       <c r="R47" t="s">
         <v>1489</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7329,7 +7355,7 @@
       <c r="J48" t="s">
         <v>1388</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -7373,7 +7399,7 @@
       <c r="J49" t="s">
         <v>1388</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -7417,7 +7443,7 @@
       <c r="J50" t="s">
         <v>1388</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -7461,7 +7487,7 @@
       <c r="J51" t="s">
         <v>1388</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -7508,7 +7534,7 @@
       <c r="J52" t="s">
         <v>1388</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -7552,7 +7578,7 @@
       <c r="J53" t="s">
         <v>1388</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -7596,7 +7622,7 @@
       <c r="J54" t="s">
         <v>1388</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -7640,7 +7666,7 @@
       <c r="J55" t="s">
         <v>1388</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -7690,7 +7716,7 @@
       <c r="J56" t="s">
         <v>1388</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -7743,7 +7769,7 @@
       <c r="J57" t="s">
         <v>1388</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -7793,7 +7819,7 @@
       <c r="J58" t="s">
         <v>1388</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -7843,7 +7869,7 @@
       <c r="J59" t="s">
         <v>1388</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -7861,7 +7887,7 @@
       <c r="R59" t="s">
         <v>1490</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -7902,7 +7928,7 @@
       <c r="J60" t="s">
         <v>1388</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -7946,7 +7972,7 @@
       <c r="J61" t="s">
         <v>1388</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -7990,7 +8016,7 @@
       <c r="J62" t="s">
         <v>1388</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8034,7 +8060,7 @@
       <c r="J63" t="s">
         <v>1388</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8078,7 +8104,7 @@
       <c r="J64" t="s">
         <v>1388</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8122,7 +8148,7 @@
       <c r="J65" t="s">
         <v>1388</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8169,7 +8195,7 @@
       <c r="J66" t="s">
         <v>1388</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8213,7 +8239,7 @@
       <c r="J67" t="s">
         <v>1388</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8257,7 +8283,7 @@
       <c r="J68" t="s">
         <v>1388</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8272,7 +8298,7 @@
       <c r="O68" t="s">
         <v>1455</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8316,7 +8342,7 @@
       <c r="J69" t="s">
         <v>1390</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -8360,7 +8386,7 @@
       <c r="J70" t="s">
         <v>1388</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -8404,7 +8430,7 @@
       <c r="J71" t="s">
         <v>1388</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -8448,7 +8474,7 @@
       <c r="J72" t="s">
         <v>1388</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -8492,7 +8518,7 @@
       <c r="J73" t="s">
         <v>1388</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -8536,7 +8562,7 @@
       <c r="J74" t="s">
         <v>1388</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -8580,7 +8606,7 @@
       <c r="J75" t="s">
         <v>1388</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -8624,7 +8650,7 @@
       <c r="J76" t="s">
         <v>1388</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -8668,7 +8694,7 @@
       <c r="J77" t="s">
         <v>1388</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -8712,7 +8738,7 @@
       <c r="J78" t="s">
         <v>1388</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -8756,7 +8782,7 @@
       <c r="J79" t="s">
         <v>1388</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -8800,7 +8826,7 @@
       <c r="J80" t="s">
         <v>1388</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -8844,7 +8870,7 @@
       <c r="J81" t="s">
         <v>1388</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -8888,7 +8914,7 @@
       <c r="J82" t="s">
         <v>1388</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -8932,7 +8958,7 @@
       <c r="J83" t="s">
         <v>1388</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -8976,7 +9002,7 @@
       <c r="J84" t="s">
         <v>1388</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9020,7 +9046,7 @@
       <c r="J85" t="s">
         <v>1388</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9064,7 +9090,7 @@
       <c r="J86" t="s">
         <v>1388</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9108,7 +9134,7 @@
       <c r="J87" t="s">
         <v>1388</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9152,7 +9178,7 @@
       <c r="J88" t="s">
         <v>1388</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9196,7 +9222,7 @@
       <c r="J89" t="s">
         <v>1388</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9237,7 +9263,7 @@
       <c r="J90" t="s">
         <v>1388</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -9278,7 +9304,7 @@
       <c r="J91" t="s">
         <v>1388</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -9322,7 +9348,7 @@
       <c r="J92" t="s">
         <v>1388</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -9343,7 +9369,7 @@
       <c r="R92" t="s">
         <v>1482</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -9384,7 +9410,7 @@
       <c r="J93" t="s">
         <v>1388</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -9425,7 +9451,7 @@
       <c r="J94" t="s">
         <v>1388</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -9469,7 +9495,7 @@
       <c r="J95" t="s">
         <v>1388</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -9513,7 +9539,7 @@
       <c r="J96" t="s">
         <v>1388</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -9560,7 +9586,7 @@
       <c r="J97" t="s">
         <v>1388</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -9575,7 +9601,7 @@
       <c r="R97" t="s">
         <v>1491</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -9616,7 +9642,7 @@
       <c r="J98" t="s">
         <v>1388</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -9660,7 +9686,7 @@
       <c r="J99" t="s">
         <v>1388</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -9704,7 +9730,7 @@
       <c r="J100" t="s">
         <v>1388</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -9745,7 +9771,7 @@
       <c r="J101" t="s">
         <v>1388</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -9786,7 +9812,7 @@
       <c r="J102" t="s">
         <v>1388</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -9827,7 +9853,7 @@
       <c r="J103" t="s">
         <v>1388</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -9868,7 +9894,7 @@
       <c r="J104" t="s">
         <v>1388</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -9909,7 +9935,7 @@
       <c r="J105" t="s">
         <v>1388</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -9950,7 +9976,7 @@
       <c r="J106" t="s">
         <v>1388</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -9991,7 +10017,7 @@
       <c r="J107" t="s">
         <v>1388</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10032,7 +10058,7 @@
       <c r="J108" t="s">
         <v>1388</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10073,7 +10099,7 @@
       <c r="J109" t="s">
         <v>1388</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10114,7 +10140,7 @@
       <c r="J110" t="s">
         <v>1388</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10132,7 +10158,7 @@
       <c r="R110" t="s">
         <v>1492</v>
       </c>
-      <c r="T110" s="1">
+      <c r="T110" s="2">
         <v>45805</v>
       </c>
       <c r="U110" t="s">
@@ -10170,7 +10196,7 @@
       <c r="J111" t="s">
         <v>1388</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -10188,7 +10214,7 @@
       <c r="R111" t="s">
         <v>1493</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -10226,7 +10252,7 @@
       <c r="J112" t="s">
         <v>1388</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -10244,7 +10270,7 @@
       <c r="R112" t="s">
         <v>1494</v>
       </c>
-      <c r="T112" s="1">
+      <c r="T112" s="2">
         <v>46052</v>
       </c>
       <c r="U112" t="s">
@@ -10285,7 +10311,7 @@
       <c r="J113" t="s">
         <v>1388</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -10329,7 +10355,7 @@
       <c r="J114" t="s">
         <v>1388</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -10373,7 +10399,7 @@
       <c r="J115" t="s">
         <v>1388</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -10417,7 +10443,7 @@
       <c r="J116" t="s">
         <v>1388</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -10435,7 +10461,7 @@
       <c r="R116" t="s">
         <v>1495</v>
       </c>
-      <c r="T116" s="1">
+      <c r="T116" s="2">
         <v>46048</v>
       </c>
       <c r="U116" t="s">
@@ -10476,7 +10502,7 @@
       <c r="J117" t="s">
         <v>1388</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -10520,7 +10546,7 @@
       <c r="J118" t="s">
         <v>1388</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -10567,7 +10593,7 @@
       <c r="J119" t="s">
         <v>1388</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -10608,7 +10634,7 @@
       <c r="J120" t="s">
         <v>1388</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -10652,7 +10678,7 @@
       <c r="J121" t="s">
         <v>1388</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -10696,7 +10722,7 @@
       <c r="J122" t="s">
         <v>1388</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -10746,7 +10772,7 @@
       <c r="J123" t="s">
         <v>1388</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -10790,7 +10816,7 @@
       <c r="J124" t="s">
         <v>1388</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -10834,7 +10860,7 @@
       <c r="J125" t="s">
         <v>1388</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -10875,7 +10901,7 @@
       <c r="J126" t="s">
         <v>1388</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -10916,7 +10942,7 @@
       <c r="J127" t="s">
         <v>1388</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -10934,7 +10960,7 @@
       <c r="R127" t="s">
         <v>1497</v>
       </c>
-      <c r="T127" s="1">
+      <c r="T127" s="2">
         <v>45889</v>
       </c>
       <c r="U127" t="s">
@@ -10972,7 +10998,7 @@
       <c r="J128" t="s">
         <v>1388</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11013,7 +11039,7 @@
       <c r="J129" t="s">
         <v>1388</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11054,7 +11080,7 @@
       <c r="J130" t="s">
         <v>1388</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11095,7 +11121,7 @@
       <c r="J131" t="s">
         <v>1388</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11139,7 +11165,7 @@
       <c r="J132" t="s">
         <v>1388</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -11180,7 +11206,7 @@
       <c r="J133" t="s">
         <v>1388</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -11221,7 +11247,7 @@
       <c r="J134" t="s">
         <v>1388</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -11262,7 +11288,7 @@
       <c r="J135" t="s">
         <v>1388</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -11303,7 +11329,7 @@
       <c r="J136" t="s">
         <v>1388</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -11344,7 +11370,7 @@
       <c r="J137" t="s">
         <v>1388</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -11385,7 +11411,7 @@
       <c r="J138" t="s">
         <v>1388</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -11426,7 +11452,7 @@
       <c r="J139" t="s">
         <v>1388</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -11473,7 +11499,7 @@
       <c r="J140" t="s">
         <v>1388</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -11514,7 +11540,7 @@
       <c r="J141" t="s">
         <v>1388</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -11555,7 +11581,7 @@
       <c r="J142" t="s">
         <v>1388</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -11599,7 +11625,7 @@
       <c r="J143" t="s">
         <v>1388</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -11640,7 +11666,7 @@
       <c r="J144" t="s">
         <v>1388</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -11681,7 +11707,7 @@
       <c r="J145" t="s">
         <v>1388</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -11722,7 +11748,7 @@
       <c r="J146" t="s">
         <v>1388</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -11763,7 +11789,7 @@
       <c r="J147" t="s">
         <v>1388</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -11804,7 +11830,7 @@
       <c r="J148" t="s">
         <v>1388</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -11845,7 +11871,7 @@
       <c r="J149" t="s">
         <v>1388</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -11886,7 +11912,7 @@
       <c r="J150" t="s">
         <v>1388</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -11927,7 +11953,7 @@
       <c r="J151" t="s">
         <v>1388</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -11968,7 +11994,7 @@
       <c r="J152" t="s">
         <v>1388</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12009,7 +12035,7 @@
       <c r="J153" t="s">
         <v>1388</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -12018,7 +12044,7 @@
       <c r="M153" t="s">
         <v>1446</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -12059,7 +12085,7 @@
       <c r="J154" t="s">
         <v>1388</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -12100,7 +12126,7 @@
       <c r="J155" t="s">
         <v>1388</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -12141,7 +12167,7 @@
       <c r="J156" t="s">
         <v>1388</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -12182,7 +12208,7 @@
       <c r="J157" t="s">
         <v>1388</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -12223,7 +12249,7 @@
       <c r="J158" t="s">
         <v>1388</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -12264,7 +12290,7 @@
       <c r="J159" t="s">
         <v>1388</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -12305,7 +12331,7 @@
       <c r="J160" t="s">
         <v>1388</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -12346,7 +12372,7 @@
       <c r="J161" t="s">
         <v>1388</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -12387,7 +12413,7 @@
       <c r="J162" t="s">
         <v>1388</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -12428,7 +12454,7 @@
       <c r="J163" t="s">
         <v>1388</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -12469,7 +12495,7 @@
       <c r="J164" t="s">
         <v>1388</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -12510,7 +12536,7 @@
       <c r="J165" t="s">
         <v>1388</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -12551,7 +12577,7 @@
       <c r="J166" t="s">
         <v>1388</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -12592,7 +12618,7 @@
       <c r="J167" t="s">
         <v>1388</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -12636,7 +12662,7 @@
       <c r="J168" t="s">
         <v>1388</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -12680,7 +12706,7 @@
       <c r="J169" t="s">
         <v>1388</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -12721,7 +12747,7 @@
       <c r="J170" t="s">
         <v>1388</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -12762,7 +12788,7 @@
       <c r="J171" t="s">
         <v>1388</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -12803,7 +12829,7 @@
       <c r="J172" t="s">
         <v>1388</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -12844,7 +12870,7 @@
       <c r="J173" t="s">
         <v>1388</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -12885,7 +12911,7 @@
       <c r="J174" t="s">
         <v>1388</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -12926,7 +12952,7 @@
       <c r="J175" t="s">
         <v>1388</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -12967,7 +12993,7 @@
       <c r="J176" t="s">
         <v>1388</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -13008,7 +13034,7 @@
       <c r="J177" t="s">
         <v>1388</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -13049,7 +13075,7 @@
       <c r="J178" t="s">
         <v>1388</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -13090,7 +13116,7 @@
       <c r="J179" t="s">
         <v>1388</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -13099,7 +13125,7 @@
       <c r="M179" t="s">
         <v>1443</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -13140,7 +13166,7 @@
       <c r="J180" t="s">
         <v>1388</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -13181,7 +13207,7 @@
       <c r="J181" t="s">
         <v>1388</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -13222,7 +13248,7 @@
       <c r="J182" t="s">
         <v>1388</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -13263,7 +13289,7 @@
       <c r="J183" t="s">
         <v>1388</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -13304,7 +13330,7 @@
       <c r="J184" t="s">
         <v>1388</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -13345,7 +13371,7 @@
       <c r="J185" t="s">
         <v>1388</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -13386,7 +13412,7 @@
       <c r="J186" t="s">
         <v>1388</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -13427,7 +13453,7 @@
       <c r="J187" t="s">
         <v>1388</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -13468,7 +13494,7 @@
       <c r="J188" t="s">
         <v>1388</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -13509,7 +13535,7 @@
       <c r="J189" t="s">
         <v>1388</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -13550,7 +13576,7 @@
       <c r="J190" t="s">
         <v>1388</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -13591,7 +13617,7 @@
       <c r="J191" t="s">
         <v>1388</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -13632,7 +13658,7 @@
       <c r="J192" t="s">
         <v>1388</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -13673,7 +13699,7 @@
       <c r="J193" t="s">
         <v>1388</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -13714,7 +13740,7 @@
       <c r="J194" t="s">
         <v>1388</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -13755,7 +13781,7 @@
       <c r="J195" t="s">
         <v>1388</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -13799,7 +13825,7 @@
       <c r="J196" t="s">
         <v>1388</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -13843,7 +13869,7 @@
       <c r="J197" t="s">
         <v>1388</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -13884,7 +13910,7 @@
       <c r="J198" t="s">
         <v>1390</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -13925,7 +13951,7 @@
       <c r="J199" t="s">
         <v>1389</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -13966,7 +13992,7 @@
       <c r="J200" t="s">
         <v>1388</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -14007,7 +14033,7 @@
       <c r="J201" t="s">
         <v>1388</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -14048,7 +14074,7 @@
       <c r="J202" t="s">
         <v>1388</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -14089,7 +14115,7 @@
       <c r="J203" t="s">
         <v>1388</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -14130,7 +14156,7 @@
       <c r="J204" t="s">
         <v>1388</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -14174,7 +14200,7 @@
       <c r="J205" t="s">
         <v>1388</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -14218,7 +14244,7 @@
       <c r="J206" t="s">
         <v>1388</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -14259,7 +14285,7 @@
       <c r="J207" t="s">
         <v>1388</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -14300,7 +14326,7 @@
       <c r="J208" t="s">
         <v>1388</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -14341,7 +14367,7 @@
       <c r="J209" t="s">
         <v>1388</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -14382,7 +14408,7 @@
       <c r="J210" t="s">
         <v>1388</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -14423,7 +14449,7 @@
       <c r="J211" t="s">
         <v>1388</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -14464,7 +14490,7 @@
       <c r="J212" t="s">
         <v>1388</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -14505,7 +14531,7 @@
       <c r="J213" t="s">
         <v>1388</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -14546,7 +14572,7 @@
       <c r="J214" t="s">
         <v>1388</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -14587,7 +14613,7 @@
       <c r="J215" t="s">
         <v>1388</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -14628,7 +14654,7 @@
       <c r="J216" t="s">
         <v>1388</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -14669,7 +14695,7 @@
       <c r="J217" t="s">
         <v>1388</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -14710,7 +14736,7 @@
       <c r="J218" t="s">
         <v>1388</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -14751,7 +14777,7 @@
       <c r="J219" t="s">
         <v>1388</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -14792,7 +14818,7 @@
       <c r="J220" t="s">
         <v>1388</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -14833,7 +14859,7 @@
       <c r="J221" t="s">
         <v>1388</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -14874,7 +14900,7 @@
       <c r="J222" t="s">
         <v>1388</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -14915,7 +14941,7 @@
       <c r="J223" t="s">
         <v>1388</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -14956,7 +14982,7 @@
       <c r="J224" t="s">
         <v>1388</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -14997,7 +15023,7 @@
       <c r="J225" t="s">
         <v>1388</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -15038,7 +15064,7 @@
       <c r="J226" t="s">
         <v>1388</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -15079,7 +15105,7 @@
       <c r="J227" t="s">
         <v>1388</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -15120,7 +15146,7 @@
       <c r="J228" t="s">
         <v>1388</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -15161,7 +15187,7 @@
       <c r="J229" t="s">
         <v>1388</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -15202,7 +15228,7 @@
       <c r="J230" t="s">
         <v>1388</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -15243,7 +15269,7 @@
       <c r="J231" t="s">
         <v>1388</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -15284,7 +15310,7 @@
       <c r="J232" t="s">
         <v>1388</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -15325,7 +15351,7 @@
       <c r="J233" t="s">
         <v>1388</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -15366,7 +15392,7 @@
       <c r="J234" t="s">
         <v>1388</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -15407,7 +15433,7 @@
       <c r="J235" t="s">
         <v>1388</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -15448,7 +15474,7 @@
       <c r="J236" t="s">
         <v>1388</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -15489,7 +15515,7 @@
       <c r="J237" t="s">
         <v>1388</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -15530,7 +15556,7 @@
       <c r="J238" t="s">
         <v>1388</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -15571,7 +15597,7 @@
       <c r="J239" t="s">
         <v>1388</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -15612,7 +15638,7 @@
       <c r="J240" t="s">
         <v>1388</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -15653,7 +15679,7 @@
       <c r="J241" t="s">
         <v>1388</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -15694,7 +15720,7 @@
       <c r="J242" t="s">
         <v>1388</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -15735,7 +15761,7 @@
       <c r="J243" t="s">
         <v>1388</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -15776,7 +15802,7 @@
       <c r="J244" t="s">
         <v>1388</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -15817,7 +15843,7 @@
       <c r="J245" t="s">
         <v>1388</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -15858,7 +15884,7 @@
       <c r="J246" t="s">
         <v>1388</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -15899,7 +15925,7 @@
       <c r="J247" t="s">
         <v>1388</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -15940,7 +15966,7 @@
       <c r="J248" t="s">
         <v>1388</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -15981,7 +16007,7 @@
       <c r="J249" t="s">
         <v>1388</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -16022,7 +16048,7 @@
       <c r="J250" t="s">
         <v>1388</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -16063,7 +16089,7 @@
       <c r="J251" t="s">
         <v>1388</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -16104,7 +16130,7 @@
       <c r="J252" t="s">
         <v>1388</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -16145,7 +16171,7 @@
       <c r="J253" t="s">
         <v>1388</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -16189,7 +16215,7 @@
       <c r="J254" t="s">
         <v>1388</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -16230,7 +16256,7 @@
       <c r="J255" t="s">
         <v>1388</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -16271,7 +16297,7 @@
       <c r="J256" t="s">
         <v>1388</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -16315,7 +16341,7 @@
       <c r="J257" t="s">
         <v>1388</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -16324,7 +16350,7 @@
       <c r="M257" t="s">
         <v>1443</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -16368,7 +16394,7 @@
       <c r="J258" t="s">
         <v>1388</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -16412,7 +16438,7 @@
       <c r="J259" t="s">
         <v>1388</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -16456,7 +16482,7 @@
       <c r="J260" t="s">
         <v>1388</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -16465,7 +16491,7 @@
       <c r="M260" t="s">
         <v>1437</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -16509,7 +16535,7 @@
       <c r="J261" t="s">
         <v>1388</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -16553,7 +16579,7 @@
       <c r="J262" t="s">
         <v>1388</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -16597,7 +16623,7 @@
       <c r="J263" t="s">
         <v>1388</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -16606,7 +16632,7 @@
       <c r="M263" t="s">
         <v>1437</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -16650,7 +16676,7 @@
       <c r="J264" t="s">
         <v>1388</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -16691,7 +16717,7 @@
       <c r="J265" t="s">
         <v>1388</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -16732,7 +16758,7 @@
       <c r="J266" t="s">
         <v>1388</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -16773,7 +16799,7 @@
       <c r="J267" t="s">
         <v>1388</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -16817,7 +16843,7 @@
       <c r="J268" t="s">
         <v>1388</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -16858,7 +16884,7 @@
       <c r="J269" t="s">
         <v>1388</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -16899,7 +16925,7 @@
       <c r="J270" t="s">
         <v>1388</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -16940,7 +16966,7 @@
       <c r="J271" t="s">
         <v>1388</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -16981,7 +17007,7 @@
       <c r="J272" t="s">
         <v>1388</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -17025,7 +17051,7 @@
       <c r="J273" t="s">
         <v>1388</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -17069,7 +17095,7 @@
       <c r="J274" t="s">
         <v>1388</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -17110,7 +17136,7 @@
       <c r="J275" t="s">
         <v>1388</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -17151,7 +17177,7 @@
       <c r="J276" t="s">
         <v>1388</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -17192,7 +17218,7 @@
       <c r="J277" t="s">
         <v>1388</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -17233,7 +17259,7 @@
       <c r="J278" t="s">
         <v>1388</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -17274,7 +17300,7 @@
       <c r="J279" t="s">
         <v>1388</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -17315,7 +17341,7 @@
       <c r="J280" t="s">
         <v>1388</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -17356,7 +17382,7 @@
       <c r="J281" t="s">
         <v>1388</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -17397,7 +17423,7 @@
       <c r="J282" t="s">
         <v>1388</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -17438,7 +17464,7 @@
       <c r="J283" t="s">
         <v>1388</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -17479,7 +17505,7 @@
       <c r="J284" t="s">
         <v>1388</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -17520,7 +17546,7 @@
       <c r="J285" t="s">
         <v>1388</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -17561,7 +17587,7 @@
       <c r="J286" t="s">
         <v>1388</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -17602,7 +17628,7 @@
       <c r="J287" t="s">
         <v>1388</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -17643,7 +17669,7 @@
       <c r="J288" t="s">
         <v>1388</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -17684,7 +17710,7 @@
       <c r="J289" t="s">
         <v>1388</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -17725,7 +17751,7 @@
       <c r="J290" t="s">
         <v>1388</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -17766,7 +17792,7 @@
       <c r="J291" t="s">
         <v>1388</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -17807,7 +17833,7 @@
       <c r="J292" t="s">
         <v>1388</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -17848,7 +17874,7 @@
       <c r="J293" t="s">
         <v>1388</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -17889,7 +17915,7 @@
       <c r="J294" t="s">
         <v>1388</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -17930,7 +17956,7 @@
       <c r="J295" t="s">
         <v>1388</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -17974,7 +18000,7 @@
       <c r="J296" t="s">
         <v>1388</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -18018,7 +18044,7 @@
       <c r="J297" t="s">
         <v>1388</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -18059,7 +18085,7 @@
       <c r="J298" t="s">
         <v>1388</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -18100,7 +18126,7 @@
       <c r="J299" t="s">
         <v>1389</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -18141,7 +18167,7 @@
       <c r="J300" t="s">
         <v>1388</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -18182,7 +18208,7 @@
       <c r="J301" t="s">
         <v>1388</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (23/07/2026 16:18)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -4616,16 +4616,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -4641,7 +4633,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -4649,30 +4641,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -4972,73 +4946,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5073,7 +5047,7 @@
       <c r="J2" t="s">
         <v>1388</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5117,7 +5091,7 @@
       <c r="J3" t="s">
         <v>1388</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5161,7 +5135,7 @@
       <c r="J4" t="s">
         <v>1388</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5205,7 +5179,7 @@
       <c r="J5" t="s">
         <v>1389</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5255,7 +5229,7 @@
       <c r="J6" t="s">
         <v>1388</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5302,7 +5276,7 @@
       <c r="J7" t="s">
         <v>1388</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5349,7 +5323,7 @@
       <c r="J8" t="s">
         <v>1388</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5396,7 +5370,7 @@
       <c r="J9" t="s">
         <v>1388</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5443,7 +5417,7 @@
       <c r="J10" t="s">
         <v>1388</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -5490,7 +5464,7 @@
       <c r="J11" t="s">
         <v>1388</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -5537,7 +5511,7 @@
       <c r="J12" t="s">
         <v>1388</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -5581,7 +5555,7 @@
       <c r="J13" t="s">
         <v>1388</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -5625,7 +5599,7 @@
       <c r="J14" t="s">
         <v>1388</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -5669,7 +5643,7 @@
       <c r="J15" t="s">
         <v>1388</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -5713,7 +5687,7 @@
       <c r="J16" t="s">
         <v>1388</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -5757,7 +5731,7 @@
       <c r="J17" t="s">
         <v>1388</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -5801,7 +5775,7 @@
       <c r="J18" t="s">
         <v>1388</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -5819,7 +5793,7 @@
       <c r="R18" t="s">
         <v>1479</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -5860,7 +5834,7 @@
       <c r="J19" t="s">
         <v>1388</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -5904,7 +5878,7 @@
       <c r="J20" t="s">
         <v>1388</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -5948,7 +5922,7 @@
       <c r="J21" t="s">
         <v>1388</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -5966,7 +5940,7 @@
       <c r="R21" t="s">
         <v>1480</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6007,7 +5981,7 @@
       <c r="J22" t="s">
         <v>1388</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6025,7 +5999,7 @@
       <c r="R22" t="s">
         <v>1481</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6066,7 +6040,7 @@
       <c r="J23" t="s">
         <v>1388</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6084,7 +6058,7 @@
       <c r="R23" t="s">
         <v>1482</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6125,7 +6099,7 @@
       <c r="J24" t="s">
         <v>1388</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6169,7 +6143,7 @@
       <c r="J25" t="s">
         <v>1388</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6210,7 +6184,7 @@
       <c r="J26" t="s">
         <v>1390</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6251,7 +6225,7 @@
       <c r="J27" t="s">
         <v>1388</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6269,7 +6243,7 @@
       <c r="R27" t="s">
         <v>1483</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6310,7 +6284,7 @@
       <c r="J28" t="s">
         <v>1388</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6354,7 +6328,7 @@
       <c r="J29" t="s">
         <v>1388</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6398,7 +6372,7 @@
       <c r="J30" t="s">
         <v>1388</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -6442,7 +6416,7 @@
       <c r="J31" t="s">
         <v>1388</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -6460,7 +6434,7 @@
       <c r="R31" t="s">
         <v>1484</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -6501,7 +6475,7 @@
       <c r="J32" t="s">
         <v>1388</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -6545,7 +6519,7 @@
       <c r="J33" t="s">
         <v>1388</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -6563,7 +6537,7 @@
       <c r="R33" t="s">
         <v>1485</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -6604,7 +6578,7 @@
       <c r="J34" t="s">
         <v>1388</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -6648,7 +6622,7 @@
       <c r="J35" t="s">
         <v>1388</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -6666,7 +6640,7 @@
       <c r="R35" t="s">
         <v>1486</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -6707,7 +6681,7 @@
       <c r="J36" t="s">
         <v>1388</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -6725,7 +6699,7 @@
       <c r="R36" t="s">
         <v>1486</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -6766,7 +6740,7 @@
       <c r="J37" t="s">
         <v>1388</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -6784,7 +6758,7 @@
       <c r="R37" t="s">
         <v>1486</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -6825,7 +6799,7 @@
       <c r="J38" t="s">
         <v>1388</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -6843,7 +6817,7 @@
       <c r="R38" t="s">
         <v>1486</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -6884,7 +6858,7 @@
       <c r="J39" t="s">
         <v>1388</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -6902,7 +6876,7 @@
       <c r="R39" t="s">
         <v>1486</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -6943,7 +6917,7 @@
       <c r="J40" t="s">
         <v>1388</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -6961,7 +6935,7 @@
       <c r="R40" t="s">
         <v>1487</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7002,7 +6976,7 @@
       <c r="J41" t="s">
         <v>1388</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7046,7 +7020,7 @@
       <c r="J42" t="s">
         <v>1388</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7064,7 +7038,7 @@
       <c r="R42" t="s">
         <v>1486</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7105,7 +7079,7 @@
       <c r="J43" t="s">
         <v>1388</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7149,7 +7123,7 @@
       <c r="J44" t="s">
         <v>1388</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7167,7 +7141,7 @@
       <c r="R44" t="s">
         <v>1488</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7208,7 +7182,7 @@
       <c r="J45" t="s">
         <v>1388</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7252,7 +7226,7 @@
       <c r="J46" t="s">
         <v>1388</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7296,7 +7270,7 @@
       <c r="J47" t="s">
         <v>1388</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7314,7 +7288,7 @@
       <c r="R47" t="s">
         <v>1489</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7355,7 +7329,7 @@
       <c r="J48" t="s">
         <v>1388</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -7399,7 +7373,7 @@
       <c r="J49" t="s">
         <v>1388</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -7443,7 +7417,7 @@
       <c r="J50" t="s">
         <v>1388</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -7487,7 +7461,7 @@
       <c r="J51" t="s">
         <v>1388</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -7534,7 +7508,7 @@
       <c r="J52" t="s">
         <v>1388</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -7578,7 +7552,7 @@
       <c r="J53" t="s">
         <v>1388</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -7622,7 +7596,7 @@
       <c r="J54" t="s">
         <v>1388</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -7666,7 +7640,7 @@
       <c r="J55" t="s">
         <v>1388</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -7716,7 +7690,7 @@
       <c r="J56" t="s">
         <v>1388</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -7769,7 +7743,7 @@
       <c r="J57" t="s">
         <v>1388</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -7819,7 +7793,7 @@
       <c r="J58" t="s">
         <v>1388</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -7869,7 +7843,7 @@
       <c r="J59" t="s">
         <v>1388</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -7887,7 +7861,7 @@
       <c r="R59" t="s">
         <v>1490</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -7928,7 +7902,7 @@
       <c r="J60" t="s">
         <v>1388</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -7972,7 +7946,7 @@
       <c r="J61" t="s">
         <v>1388</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8016,7 +7990,7 @@
       <c r="J62" t="s">
         <v>1388</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8060,7 +8034,7 @@
       <c r="J63" t="s">
         <v>1388</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8104,7 +8078,7 @@
       <c r="J64" t="s">
         <v>1388</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8148,7 +8122,7 @@
       <c r="J65" t="s">
         <v>1388</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8195,7 +8169,7 @@
       <c r="J66" t="s">
         <v>1388</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8239,7 +8213,7 @@
       <c r="J67" t="s">
         <v>1388</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8283,7 +8257,7 @@
       <c r="J68" t="s">
         <v>1388</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8298,7 +8272,7 @@
       <c r="O68" t="s">
         <v>1455</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8342,7 +8316,7 @@
       <c r="J69" t="s">
         <v>1390</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -8386,7 +8360,7 @@
       <c r="J70" t="s">
         <v>1388</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -8430,7 +8404,7 @@
       <c r="J71" t="s">
         <v>1388</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -8474,7 +8448,7 @@
       <c r="J72" t="s">
         <v>1388</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -8518,7 +8492,7 @@
       <c r="J73" t="s">
         <v>1388</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -8562,7 +8536,7 @@
       <c r="J74" t="s">
         <v>1388</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -8606,7 +8580,7 @@
       <c r="J75" t="s">
         <v>1388</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -8650,7 +8624,7 @@
       <c r="J76" t="s">
         <v>1388</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -8694,7 +8668,7 @@
       <c r="J77" t="s">
         <v>1388</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -8738,7 +8712,7 @@
       <c r="J78" t="s">
         <v>1388</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -8782,7 +8756,7 @@
       <c r="J79" t="s">
         <v>1388</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -8826,7 +8800,7 @@
       <c r="J80" t="s">
         <v>1388</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -8870,7 +8844,7 @@
       <c r="J81" t="s">
         <v>1388</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -8914,7 +8888,7 @@
       <c r="J82" t="s">
         <v>1388</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -8958,7 +8932,7 @@
       <c r="J83" t="s">
         <v>1388</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9002,7 +8976,7 @@
       <c r="J84" t="s">
         <v>1388</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9046,7 +9020,7 @@
       <c r="J85" t="s">
         <v>1388</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9090,7 +9064,7 @@
       <c r="J86" t="s">
         <v>1388</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9134,7 +9108,7 @@
       <c r="J87" t="s">
         <v>1388</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9178,7 +9152,7 @@
       <c r="J88" t="s">
         <v>1388</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9222,7 +9196,7 @@
       <c r="J89" t="s">
         <v>1388</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9263,7 +9237,7 @@
       <c r="J90" t="s">
         <v>1388</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -9304,7 +9278,7 @@
       <c r="J91" t="s">
         <v>1388</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -9348,7 +9322,7 @@
       <c r="J92" t="s">
         <v>1388</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -9369,7 +9343,7 @@
       <c r="R92" t="s">
         <v>1482</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -9410,7 +9384,7 @@
       <c r="J93" t="s">
         <v>1388</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -9451,7 +9425,7 @@
       <c r="J94" t="s">
         <v>1388</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -9495,7 +9469,7 @@
       <c r="J95" t="s">
         <v>1388</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -9539,7 +9513,7 @@
       <c r="J96" t="s">
         <v>1388</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -9586,7 +9560,7 @@
       <c r="J97" t="s">
         <v>1388</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -9601,7 +9575,7 @@
       <c r="R97" t="s">
         <v>1491</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -9642,7 +9616,7 @@
       <c r="J98" t="s">
         <v>1388</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -9686,7 +9660,7 @@
       <c r="J99" t="s">
         <v>1388</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -9730,7 +9704,7 @@
       <c r="J100" t="s">
         <v>1388</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -9771,7 +9745,7 @@
       <c r="J101" t="s">
         <v>1388</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -9812,7 +9786,7 @@
       <c r="J102" t="s">
         <v>1388</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -9853,7 +9827,7 @@
       <c r="J103" t="s">
         <v>1388</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -9894,7 +9868,7 @@
       <c r="J104" t="s">
         <v>1388</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -9935,7 +9909,7 @@
       <c r="J105" t="s">
         <v>1388</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -9976,7 +9950,7 @@
       <c r="J106" t="s">
         <v>1388</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10017,7 +9991,7 @@
       <c r="J107" t="s">
         <v>1388</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10058,7 +10032,7 @@
       <c r="J108" t="s">
         <v>1388</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10099,7 +10073,7 @@
       <c r="J109" t="s">
         <v>1388</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10140,7 +10114,7 @@
       <c r="J110" t="s">
         <v>1388</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10158,7 +10132,7 @@
       <c r="R110" t="s">
         <v>1492</v>
       </c>
-      <c r="T110" s="2">
+      <c r="T110" s="1">
         <v>45805</v>
       </c>
       <c r="U110" t="s">
@@ -10196,7 +10170,7 @@
       <c r="J111" t="s">
         <v>1388</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -10214,7 +10188,7 @@
       <c r="R111" t="s">
         <v>1493</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -10252,7 +10226,7 @@
       <c r="J112" t="s">
         <v>1388</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -10270,7 +10244,7 @@
       <c r="R112" t="s">
         <v>1494</v>
       </c>
-      <c r="T112" s="2">
+      <c r="T112" s="1">
         <v>46052</v>
       </c>
       <c r="U112" t="s">
@@ -10311,7 +10285,7 @@
       <c r="J113" t="s">
         <v>1388</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -10355,7 +10329,7 @@
       <c r="J114" t="s">
         <v>1388</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -10399,7 +10373,7 @@
       <c r="J115" t="s">
         <v>1388</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -10443,7 +10417,7 @@
       <c r="J116" t="s">
         <v>1388</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -10461,7 +10435,7 @@
       <c r="R116" t="s">
         <v>1495</v>
       </c>
-      <c r="T116" s="2">
+      <c r="T116" s="1">
         <v>46048</v>
       </c>
       <c r="U116" t="s">
@@ -10502,7 +10476,7 @@
       <c r="J117" t="s">
         <v>1388</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -10546,7 +10520,7 @@
       <c r="J118" t="s">
         <v>1388</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -10593,7 +10567,7 @@
       <c r="J119" t="s">
         <v>1388</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -10634,7 +10608,7 @@
       <c r="J120" t="s">
         <v>1388</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -10678,7 +10652,7 @@
       <c r="J121" t="s">
         <v>1388</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -10722,7 +10696,7 @@
       <c r="J122" t="s">
         <v>1388</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -10772,7 +10746,7 @@
       <c r="J123" t="s">
         <v>1388</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -10816,7 +10790,7 @@
       <c r="J124" t="s">
         <v>1388</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -10860,7 +10834,7 @@
       <c r="J125" t="s">
         <v>1388</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -10901,7 +10875,7 @@
       <c r="J126" t="s">
         <v>1388</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -10942,7 +10916,7 @@
       <c r="J127" t="s">
         <v>1388</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -10960,7 +10934,7 @@
       <c r="R127" t="s">
         <v>1497</v>
       </c>
-      <c r="T127" s="2">
+      <c r="T127" s="1">
         <v>45889</v>
       </c>
       <c r="U127" t="s">
@@ -10998,7 +10972,7 @@
       <c r="J128" t="s">
         <v>1388</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11039,7 +11013,7 @@
       <c r="J129" t="s">
         <v>1388</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11080,7 +11054,7 @@
       <c r="J130" t="s">
         <v>1388</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11121,7 +11095,7 @@
       <c r="J131" t="s">
         <v>1388</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11165,7 +11139,7 @@
       <c r="J132" t="s">
         <v>1388</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -11206,7 +11180,7 @@
       <c r="J133" t="s">
         <v>1388</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -11247,7 +11221,7 @@
       <c r="J134" t="s">
         <v>1388</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -11288,7 +11262,7 @@
       <c r="J135" t="s">
         <v>1388</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -11329,7 +11303,7 @@
       <c r="J136" t="s">
         <v>1388</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -11370,7 +11344,7 @@
       <c r="J137" t="s">
         <v>1388</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -11411,7 +11385,7 @@
       <c r="J138" t="s">
         <v>1388</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -11452,7 +11426,7 @@
       <c r="J139" t="s">
         <v>1388</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -11499,7 +11473,7 @@
       <c r="J140" t="s">
         <v>1388</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -11540,7 +11514,7 @@
       <c r="J141" t="s">
         <v>1388</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -11581,7 +11555,7 @@
       <c r="J142" t="s">
         <v>1388</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -11625,7 +11599,7 @@
       <c r="J143" t="s">
         <v>1388</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -11666,7 +11640,7 @@
       <c r="J144" t="s">
         <v>1388</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -11707,7 +11681,7 @@
       <c r="J145" t="s">
         <v>1388</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -11748,7 +11722,7 @@
       <c r="J146" t="s">
         <v>1388</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -11789,7 +11763,7 @@
       <c r="J147" t="s">
         <v>1388</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -11830,7 +11804,7 @@
       <c r="J148" t="s">
         <v>1388</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -11871,7 +11845,7 @@
       <c r="J149" t="s">
         <v>1388</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -11912,7 +11886,7 @@
       <c r="J150" t="s">
         <v>1388</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -11953,7 +11927,7 @@
       <c r="J151" t="s">
         <v>1388</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -11994,7 +11968,7 @@
       <c r="J152" t="s">
         <v>1388</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12035,7 +12009,7 @@
       <c r="J153" t="s">
         <v>1388</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -12044,7 +12018,7 @@
       <c r="M153" t="s">
         <v>1446</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -12085,7 +12059,7 @@
       <c r="J154" t="s">
         <v>1388</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -12126,7 +12100,7 @@
       <c r="J155" t="s">
         <v>1388</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -12167,7 +12141,7 @@
       <c r="J156" t="s">
         <v>1388</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -12208,7 +12182,7 @@
       <c r="J157" t="s">
         <v>1388</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -12249,7 +12223,7 @@
       <c r="J158" t="s">
         <v>1388</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -12290,7 +12264,7 @@
       <c r="J159" t="s">
         <v>1388</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -12331,7 +12305,7 @@
       <c r="J160" t="s">
         <v>1388</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -12372,7 +12346,7 @@
       <c r="J161" t="s">
         <v>1388</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -12413,7 +12387,7 @@
       <c r="J162" t="s">
         <v>1388</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -12454,7 +12428,7 @@
       <c r="J163" t="s">
         <v>1388</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -12495,7 +12469,7 @@
       <c r="J164" t="s">
         <v>1388</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -12536,7 +12510,7 @@
       <c r="J165" t="s">
         <v>1388</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -12577,7 +12551,7 @@
       <c r="J166" t="s">
         <v>1388</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -12618,7 +12592,7 @@
       <c r="J167" t="s">
         <v>1388</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -12662,7 +12636,7 @@
       <c r="J168" t="s">
         <v>1388</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -12706,7 +12680,7 @@
       <c r="J169" t="s">
         <v>1388</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -12747,7 +12721,7 @@
       <c r="J170" t="s">
         <v>1388</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -12788,7 +12762,7 @@
       <c r="J171" t="s">
         <v>1388</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -12829,7 +12803,7 @@
       <c r="J172" t="s">
         <v>1388</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -12870,7 +12844,7 @@
       <c r="J173" t="s">
         <v>1388</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -12911,7 +12885,7 @@
       <c r="J174" t="s">
         <v>1388</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -12952,7 +12926,7 @@
       <c r="J175" t="s">
         <v>1388</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -12993,7 +12967,7 @@
       <c r="J176" t="s">
         <v>1388</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -13034,7 +13008,7 @@
       <c r="J177" t="s">
         <v>1388</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -13075,7 +13049,7 @@
       <c r="J178" t="s">
         <v>1388</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -13116,7 +13090,7 @@
       <c r="J179" t="s">
         <v>1388</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -13125,7 +13099,7 @@
       <c r="M179" t="s">
         <v>1443</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -13166,7 +13140,7 @@
       <c r="J180" t="s">
         <v>1388</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -13207,7 +13181,7 @@
       <c r="J181" t="s">
         <v>1388</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -13248,7 +13222,7 @@
       <c r="J182" t="s">
         <v>1388</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -13289,7 +13263,7 @@
       <c r="J183" t="s">
         <v>1388</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -13330,7 +13304,7 @@
       <c r="J184" t="s">
         <v>1388</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -13371,7 +13345,7 @@
       <c r="J185" t="s">
         <v>1388</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -13412,7 +13386,7 @@
       <c r="J186" t="s">
         <v>1388</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -13453,7 +13427,7 @@
       <c r="J187" t="s">
         <v>1388</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -13494,7 +13468,7 @@
       <c r="J188" t="s">
         <v>1388</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -13535,7 +13509,7 @@
       <c r="J189" t="s">
         <v>1388</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -13576,7 +13550,7 @@
       <c r="J190" t="s">
         <v>1388</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -13617,7 +13591,7 @@
       <c r="J191" t="s">
         <v>1388</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -13658,7 +13632,7 @@
       <c r="J192" t="s">
         <v>1388</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -13699,7 +13673,7 @@
       <c r="J193" t="s">
         <v>1388</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -13740,7 +13714,7 @@
       <c r="J194" t="s">
         <v>1388</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -13781,7 +13755,7 @@
       <c r="J195" t="s">
         <v>1388</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -13825,7 +13799,7 @@
       <c r="J196" t="s">
         <v>1388</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -13869,7 +13843,7 @@
       <c r="J197" t="s">
         <v>1388</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -13910,7 +13884,7 @@
       <c r="J198" t="s">
         <v>1390</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -13951,7 +13925,7 @@
       <c r="J199" t="s">
         <v>1389</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -13992,7 +13966,7 @@
       <c r="J200" t="s">
         <v>1388</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -14033,7 +14007,7 @@
       <c r="J201" t="s">
         <v>1388</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -14074,7 +14048,7 @@
       <c r="J202" t="s">
         <v>1388</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -14115,7 +14089,7 @@
       <c r="J203" t="s">
         <v>1388</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -14156,7 +14130,7 @@
       <c r="J204" t="s">
         <v>1388</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -14200,7 +14174,7 @@
       <c r="J205" t="s">
         <v>1388</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -14244,7 +14218,7 @@
       <c r="J206" t="s">
         <v>1388</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -14285,7 +14259,7 @@
       <c r="J207" t="s">
         <v>1388</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -14326,7 +14300,7 @@
       <c r="J208" t="s">
         <v>1388</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -14367,7 +14341,7 @@
       <c r="J209" t="s">
         <v>1388</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -14408,7 +14382,7 @@
       <c r="J210" t="s">
         <v>1388</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -14449,7 +14423,7 @@
       <c r="J211" t="s">
         <v>1388</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -14490,7 +14464,7 @@
       <c r="J212" t="s">
         <v>1388</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -14531,7 +14505,7 @@
       <c r="J213" t="s">
         <v>1388</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -14572,7 +14546,7 @@
       <c r="J214" t="s">
         <v>1388</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -14613,7 +14587,7 @@
       <c r="J215" t="s">
         <v>1388</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -14654,7 +14628,7 @@
       <c r="J216" t="s">
         <v>1388</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -14695,7 +14669,7 @@
       <c r="J217" t="s">
         <v>1388</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -14736,7 +14710,7 @@
       <c r="J218" t="s">
         <v>1388</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -14777,7 +14751,7 @@
       <c r="J219" t="s">
         <v>1388</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -14818,7 +14792,7 @@
       <c r="J220" t="s">
         <v>1388</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -14859,7 +14833,7 @@
       <c r="J221" t="s">
         <v>1388</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -14900,7 +14874,7 @@
       <c r="J222" t="s">
         <v>1388</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -14941,7 +14915,7 @@
       <c r="J223" t="s">
         <v>1388</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -14982,7 +14956,7 @@
       <c r="J224" t="s">
         <v>1388</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -15023,7 +14997,7 @@
       <c r="J225" t="s">
         <v>1388</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -15064,7 +15038,7 @@
       <c r="J226" t="s">
         <v>1388</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -15105,7 +15079,7 @@
       <c r="J227" t="s">
         <v>1388</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -15146,7 +15120,7 @@
       <c r="J228" t="s">
         <v>1388</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -15187,7 +15161,7 @@
       <c r="J229" t="s">
         <v>1388</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -15228,7 +15202,7 @@
       <c r="J230" t="s">
         <v>1388</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -15269,7 +15243,7 @@
       <c r="J231" t="s">
         <v>1388</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -15310,7 +15284,7 @@
       <c r="J232" t="s">
         <v>1388</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -15351,7 +15325,7 @@
       <c r="J233" t="s">
         <v>1388</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -15392,7 +15366,7 @@
       <c r="J234" t="s">
         <v>1388</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -15433,7 +15407,7 @@
       <c r="J235" t="s">
         <v>1388</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -15474,7 +15448,7 @@
       <c r="J236" t="s">
         <v>1388</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -15515,7 +15489,7 @@
       <c r="J237" t="s">
         <v>1388</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -15556,7 +15530,7 @@
       <c r="J238" t="s">
         <v>1388</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -15597,7 +15571,7 @@
       <c r="J239" t="s">
         <v>1388</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -15638,7 +15612,7 @@
       <c r="J240" t="s">
         <v>1388</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -15679,7 +15653,7 @@
       <c r="J241" t="s">
         <v>1388</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -15720,7 +15694,7 @@
       <c r="J242" t="s">
         <v>1388</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -15761,7 +15735,7 @@
       <c r="J243" t="s">
         <v>1388</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -15802,7 +15776,7 @@
       <c r="J244" t="s">
         <v>1388</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -15843,7 +15817,7 @@
       <c r="J245" t="s">
         <v>1388</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -15884,7 +15858,7 @@
       <c r="J246" t="s">
         <v>1388</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -15925,7 +15899,7 @@
       <c r="J247" t="s">
         <v>1388</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -15966,7 +15940,7 @@
       <c r="J248" t="s">
         <v>1388</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -16007,7 +15981,7 @@
       <c r="J249" t="s">
         <v>1388</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -16048,7 +16022,7 @@
       <c r="J250" t="s">
         <v>1388</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -16089,7 +16063,7 @@
       <c r="J251" t="s">
         <v>1388</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -16130,7 +16104,7 @@
       <c r="J252" t="s">
         <v>1388</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -16171,7 +16145,7 @@
       <c r="J253" t="s">
         <v>1388</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -16215,7 +16189,7 @@
       <c r="J254" t="s">
         <v>1388</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -16256,7 +16230,7 @@
       <c r="J255" t="s">
         <v>1388</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -16297,7 +16271,7 @@
       <c r="J256" t="s">
         <v>1388</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -16341,7 +16315,7 @@
       <c r="J257" t="s">
         <v>1388</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -16350,7 +16324,7 @@
       <c r="M257" t="s">
         <v>1443</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -16394,7 +16368,7 @@
       <c r="J258" t="s">
         <v>1388</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -16438,7 +16412,7 @@
       <c r="J259" t="s">
         <v>1388</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -16482,7 +16456,7 @@
       <c r="J260" t="s">
         <v>1388</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -16491,7 +16465,7 @@
       <c r="M260" t="s">
         <v>1437</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -16535,7 +16509,7 @@
       <c r="J261" t="s">
         <v>1388</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -16579,7 +16553,7 @@
       <c r="J262" t="s">
         <v>1388</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -16623,7 +16597,7 @@
       <c r="J263" t="s">
         <v>1388</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -16632,7 +16606,7 @@
       <c r="M263" t="s">
         <v>1437</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -16676,7 +16650,7 @@
       <c r="J264" t="s">
         <v>1388</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -16717,7 +16691,7 @@
       <c r="J265" t="s">
         <v>1388</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -16758,7 +16732,7 @@
       <c r="J266" t="s">
         <v>1388</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -16799,7 +16773,7 @@
       <c r="J267" t="s">
         <v>1388</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -16843,7 +16817,7 @@
       <c r="J268" t="s">
         <v>1388</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -16884,7 +16858,7 @@
       <c r="J269" t="s">
         <v>1388</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -16925,7 +16899,7 @@
       <c r="J270" t="s">
         <v>1388</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -16966,7 +16940,7 @@
       <c r="J271" t="s">
         <v>1388</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -17007,7 +16981,7 @@
       <c r="J272" t="s">
         <v>1388</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -17051,7 +17025,7 @@
       <c r="J273" t="s">
         <v>1388</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -17095,7 +17069,7 @@
       <c r="J274" t="s">
         <v>1388</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -17136,7 +17110,7 @@
       <c r="J275" t="s">
         <v>1388</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -17177,7 +17151,7 @@
       <c r="J276" t="s">
         <v>1388</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -17218,7 +17192,7 @@
       <c r="J277" t="s">
         <v>1388</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -17259,7 +17233,7 @@
       <c r="J278" t="s">
         <v>1388</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -17300,7 +17274,7 @@
       <c r="J279" t="s">
         <v>1388</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -17341,7 +17315,7 @@
       <c r="J280" t="s">
         <v>1388</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -17382,7 +17356,7 @@
       <c r="J281" t="s">
         <v>1388</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -17423,7 +17397,7 @@
       <c r="J282" t="s">
         <v>1388</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -17464,7 +17438,7 @@
       <c r="J283" t="s">
         <v>1388</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -17505,7 +17479,7 @@
       <c r="J284" t="s">
         <v>1388</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -17546,7 +17520,7 @@
       <c r="J285" t="s">
         <v>1388</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -17587,7 +17561,7 @@
       <c r="J286" t="s">
         <v>1388</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -17628,7 +17602,7 @@
       <c r="J287" t="s">
         <v>1388</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -17669,7 +17643,7 @@
       <c r="J288" t="s">
         <v>1388</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -17710,7 +17684,7 @@
       <c r="J289" t="s">
         <v>1388</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -17751,7 +17725,7 @@
       <c r="J290" t="s">
         <v>1388</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -17792,7 +17766,7 @@
       <c r="J291" t="s">
         <v>1388</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -17833,7 +17807,7 @@
       <c r="J292" t="s">
         <v>1388</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -17874,7 +17848,7 @@
       <c r="J293" t="s">
         <v>1388</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -17915,7 +17889,7 @@
       <c r="J294" t="s">
         <v>1388</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -17956,7 +17930,7 @@
       <c r="J295" t="s">
         <v>1388</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -18000,7 +17974,7 @@
       <c r="J296" t="s">
         <v>1388</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -18044,7 +18018,7 @@
       <c r="J297" t="s">
         <v>1388</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -18085,7 +18059,7 @@
       <c r="J298" t="s">
         <v>1388</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -18126,7 +18100,7 @@
       <c r="J299" t="s">
         <v>1389</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -18167,7 +18141,7 @@
       <c r="J300" t="s">
         <v>1388</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -18208,7 +18182,7 @@
       <c r="J301" t="s">
         <v>1388</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (12/08/2026 13:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4309" uniqueCount="1612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4381" uniqueCount="1612">
   <si>
     <t>numero_ordem</t>
   </si>
@@ -4840,16 +4840,16 @@
     <t>ENTREGUE NO 03-06-2026 VIA RECIBO 438/FAB/2026</t>
   </si>
   <si>
-    <t>esse item foi reparado pela VeeOne e enviado ao estoque do PAMALS</t>
+    <t>200SGL119Q</t>
+  </si>
+  <si>
+    <t>324843-2020</t>
+  </si>
+  <si>
+    <t>#N/A</t>
   </si>
   <si>
     <t>Pendente</t>
-  </si>
-  <si>
-    <t>Desconsiderado</t>
-  </si>
-  <si>
-    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -5300,7 +5300,7 @@
         <v>1516</v>
       </c>
       <c r="W2" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -5344,7 +5344,7 @@
         <v>1517</v>
       </c>
       <c r="W3" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -5387,8 +5387,11 @@
       <c r="M4" t="s">
         <v>1518</v>
       </c>
+      <c r="V4" t="s">
+        <v>384</v>
+      </c>
       <c r="W4" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -5438,7 +5441,7 @@
         <v>1606</v>
       </c>
       <c r="W5" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="6" spans="1:23">
@@ -5485,7 +5488,7 @@
         <v>1580</v>
       </c>
       <c r="W6" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="7" spans="1:23">
@@ -5532,7 +5535,7 @@
         <v>1580</v>
       </c>
       <c r="W7" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="8" spans="1:23">
@@ -5579,7 +5582,7 @@
         <v>1580</v>
       </c>
       <c r="W8" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="9" spans="1:23">
@@ -5626,7 +5629,7 @@
         <v>1580</v>
       </c>
       <c r="W9" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="10" spans="1:23">
@@ -5673,7 +5676,7 @@
         <v>1580</v>
       </c>
       <c r="W10" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="11" spans="1:23">
@@ -5720,7 +5723,7 @@
         <v>1580</v>
       </c>
       <c r="W11" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="12" spans="1:23">
@@ -5764,7 +5767,7 @@
         <v>1519</v>
       </c>
       <c r="W12" t="s">
-        <v>1610</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="13" spans="1:23">
@@ -5807,8 +5810,11 @@
       <c r="M13" t="s">
         <v>1519</v>
       </c>
+      <c r="V13" t="s">
+        <v>393</v>
+      </c>
       <c r="W13" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -5851,8 +5857,11 @@
       <c r="M14" t="s">
         <v>1518</v>
       </c>
+      <c r="V14" t="s">
+        <v>394</v>
+      </c>
       <c r="W14" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="15" spans="1:23">
@@ -5895,8 +5904,11 @@
       <c r="M15" t="s">
         <v>1518</v>
       </c>
+      <c r="V15" t="s">
+        <v>394</v>
+      </c>
       <c r="W15" t="s">
-        <v>1609</v>
+        <v>1610</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -5940,7 +5952,7 @@
         <v>1520</v>
       </c>
       <c r="W16" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="17" spans="1:23">
@@ -5984,7 +5996,7 @@
         <v>1520</v>
       </c>
       <c r="W17" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="18" spans="1:23">
@@ -6087,7 +6099,7 @@
         <v>1518</v>
       </c>
       <c r="W19" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="20" spans="1:23">
@@ -6131,7 +6143,7 @@
         <v>1518</v>
       </c>
       <c r="W20" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -6352,7 +6364,7 @@
         <v>1521</v>
       </c>
       <c r="W24" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="25" spans="1:23">
@@ -6396,7 +6408,7 @@
         <v>1517</v>
       </c>
       <c r="W25" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="26" spans="1:23">
@@ -6436,8 +6448,11 @@
       <c r="M26" t="s">
         <v>1518</v>
       </c>
+      <c r="V26" t="s">
+        <v>405</v>
+      </c>
       <c r="W26" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="27" spans="1:23">
@@ -6537,7 +6552,7 @@
         <v>1517</v>
       </c>
       <c r="W28" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="29" spans="1:23">
@@ -6581,7 +6596,7 @@
         <v>1520</v>
       </c>
       <c r="W29" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="30" spans="1:23">
@@ -6625,7 +6640,7 @@
         <v>1517</v>
       </c>
       <c r="W30" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="31" spans="1:23">
@@ -6728,7 +6743,7 @@
         <v>1519</v>
       </c>
       <c r="W32" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="33" spans="1:23">
@@ -6831,7 +6846,7 @@
         <v>1520</v>
       </c>
       <c r="W34" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="35" spans="1:23">
@@ -7228,8 +7243,11 @@
       <c r="M41" t="s">
         <v>1520</v>
       </c>
+      <c r="V41" t="s">
+        <v>394</v>
+      </c>
       <c r="W41" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="42" spans="1:23">
@@ -7332,7 +7350,7 @@
         <v>1520</v>
       </c>
       <c r="W43" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="44" spans="1:23">
@@ -7434,8 +7452,11 @@
       <c r="M45" t="s">
         <v>1517</v>
       </c>
+      <c r="V45" t="s">
+        <v>422</v>
+      </c>
       <c r="W45" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="46" spans="1:23">
@@ -7479,7 +7500,7 @@
         <v>1520</v>
       </c>
       <c r="W46" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="47" spans="1:23">
@@ -7582,7 +7603,7 @@
         <v>1517</v>
       </c>
       <c r="W48" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="49" spans="1:23">
@@ -7626,7 +7647,7 @@
         <v>1518</v>
       </c>
       <c r="W49" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="50" spans="1:23">
@@ -7670,7 +7691,7 @@
         <v>1518</v>
       </c>
       <c r="W50" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="51" spans="1:23">
@@ -7717,7 +7738,7 @@
         <v>1593</v>
       </c>
       <c r="W51" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="52" spans="1:23">
@@ -7761,7 +7782,7 @@
         <v>1517</v>
       </c>
       <c r="W52" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="53" spans="1:23">
@@ -7805,7 +7826,7 @@
         <v>1517</v>
       </c>
       <c r="W53" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="54" spans="1:23">
@@ -7849,7 +7870,7 @@
         <v>1518</v>
       </c>
       <c r="W54" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="55" spans="1:23">
@@ -7899,7 +7920,7 @@
         <v>1534</v>
       </c>
       <c r="W55" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="56" spans="1:23">
@@ -7952,7 +7973,7 @@
         <v>1594</v>
       </c>
       <c r="W56" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="57" spans="1:23">
@@ -8002,7 +8023,7 @@
         <v>1534</v>
       </c>
       <c r="W57" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="58" spans="1:23">
@@ -8052,7 +8073,7 @@
         <v>1535</v>
       </c>
       <c r="W58" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="59" spans="1:23">
@@ -8155,7 +8176,7 @@
         <v>1517</v>
       </c>
       <c r="W60" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="61" spans="1:23">
@@ -8199,7 +8220,7 @@
         <v>1518</v>
       </c>
       <c r="W61" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="62" spans="1:23">
@@ -8243,7 +8264,7 @@
         <v>1518</v>
       </c>
       <c r="W62" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="63" spans="1:23">
@@ -8287,7 +8308,7 @@
         <v>1518</v>
       </c>
       <c r="W63" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="64" spans="1:23">
@@ -8331,7 +8352,7 @@
         <v>1518</v>
       </c>
       <c r="W64" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="65" spans="1:23">
@@ -8378,7 +8399,7 @@
         <v>1596</v>
       </c>
       <c r="W65" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="66" spans="1:23">
@@ -8421,8 +8442,11 @@
       <c r="M66" t="s">
         <v>1518</v>
       </c>
+      <c r="V66" t="s">
+        <v>442</v>
+      </c>
       <c r="W66" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="67" spans="1:23">
@@ -8466,7 +8490,7 @@
         <v>1520</v>
       </c>
       <c r="W67" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="68" spans="1:23">
@@ -8569,7 +8593,7 @@
         <v>1526</v>
       </c>
       <c r="W69" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="70" spans="1:23">
@@ -8613,7 +8637,7 @@
         <v>1526</v>
       </c>
       <c r="W70" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="71" spans="1:23">
@@ -8657,7 +8681,7 @@
         <v>1524</v>
       </c>
       <c r="W71" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="72" spans="1:23">
@@ -8701,7 +8725,7 @@
         <v>1520</v>
       </c>
       <c r="W72" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="73" spans="1:23">
@@ -8745,7 +8769,7 @@
         <v>1518</v>
       </c>
       <c r="W73" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="74" spans="1:23">
@@ -8789,7 +8813,7 @@
         <v>1518</v>
       </c>
       <c r="W74" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="75" spans="1:23">
@@ -8833,7 +8857,7 @@
         <v>1517</v>
       </c>
       <c r="W75" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="76" spans="1:23">
@@ -8876,8 +8900,11 @@
       <c r="M76" t="s">
         <v>1518</v>
       </c>
+      <c r="V76" t="s">
+        <v>452</v>
+      </c>
       <c r="W76" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="77" spans="1:23">
@@ -8920,8 +8947,11 @@
       <c r="M77" t="s">
         <v>1518</v>
       </c>
+      <c r="V77" t="s">
+        <v>453</v>
+      </c>
       <c r="W77" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="78" spans="1:23">
@@ -8964,8 +8994,11 @@
       <c r="M78" t="s">
         <v>1518</v>
       </c>
+      <c r="V78" t="s">
+        <v>454</v>
+      </c>
       <c r="W78" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="79" spans="1:23">
@@ -9008,8 +9041,11 @@
       <c r="M79" t="s">
         <v>1518</v>
       </c>
+      <c r="V79" t="s">
+        <v>455</v>
+      </c>
       <c r="W79" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="80" spans="1:23">
@@ -9053,7 +9089,7 @@
         <v>1518</v>
       </c>
       <c r="W80" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="81" spans="1:23">
@@ -9097,7 +9133,7 @@
         <v>1517</v>
       </c>
       <c r="W81" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="82" spans="1:23">
@@ -9141,7 +9177,7 @@
         <v>1527</v>
       </c>
       <c r="W82" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="83" spans="1:23">
@@ -9185,7 +9221,7 @@
         <v>1518</v>
       </c>
       <c r="W83" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="84" spans="1:23">
@@ -9229,7 +9265,7 @@
         <v>1518</v>
       </c>
       <c r="W84" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="85" spans="1:23">
@@ -9272,8 +9308,11 @@
       <c r="M85" t="s">
         <v>1523</v>
       </c>
+      <c r="V85" t="s">
+        <v>461</v>
+      </c>
       <c r="W85" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="86" spans="1:23">
@@ -9317,7 +9356,7 @@
         <v>1523</v>
       </c>
       <c r="W86" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="87" spans="1:23">
@@ -9360,8 +9399,11 @@
       <c r="M87" t="s">
         <v>1520</v>
       </c>
+      <c r="V87" t="s">
+        <v>463</v>
+      </c>
       <c r="W87" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="88" spans="1:23">
@@ -9405,7 +9447,7 @@
         <v>1519</v>
       </c>
       <c r="W88" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="89" spans="1:23">
@@ -9448,8 +9490,11 @@
       <c r="M89" t="s">
         <v>1520</v>
       </c>
+      <c r="V89" t="s">
+        <v>461</v>
+      </c>
       <c r="W89" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="90" spans="1:23">
@@ -9489,8 +9534,11 @@
       <c r="M90" t="s">
         <v>1518</v>
       </c>
+      <c r="V90" t="s">
+        <v>464</v>
+      </c>
       <c r="W90" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="91" spans="1:23">
@@ -9530,8 +9578,11 @@
       <c r="M91" t="s">
         <v>1526</v>
       </c>
+      <c r="V91" t="s">
+        <v>466</v>
+      </c>
       <c r="W91" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="92" spans="1:23">
@@ -9637,7 +9688,7 @@
         <v>1527</v>
       </c>
       <c r="W93" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="94" spans="1:23">
@@ -9678,7 +9729,7 @@
         <v>1524</v>
       </c>
       <c r="W94" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="95" spans="1:23">
@@ -9722,7 +9773,7 @@
         <v>1524</v>
       </c>
       <c r="W95" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="96" spans="1:23">
@@ -9768,8 +9819,11 @@
       <c r="O96" t="s">
         <v>1537</v>
       </c>
+      <c r="V96" t="s">
+        <v>471</v>
+      </c>
       <c r="W96" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="97" spans="1:23">
@@ -9868,8 +9922,11 @@
       <c r="M98" t="s">
         <v>1517</v>
       </c>
+      <c r="V98" t="s">
+        <v>473</v>
+      </c>
       <c r="W98" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="99" spans="1:23">
@@ -9912,8 +9969,11 @@
       <c r="M99" t="s">
         <v>1520</v>
       </c>
+      <c r="V99" t="s">
+        <v>474</v>
+      </c>
       <c r="W99" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="100" spans="1:23">
@@ -9957,7 +10017,7 @@
         <v>1519</v>
       </c>
       <c r="W100" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="101" spans="1:23">
@@ -9998,7 +10058,7 @@
         <v>1520</v>
       </c>
       <c r="W101" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="102" spans="1:23">
@@ -10039,7 +10099,7 @@
         <v>1526</v>
       </c>
       <c r="W102" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="103" spans="1:23">
@@ -10080,7 +10140,7 @@
         <v>1526</v>
       </c>
       <c r="W103" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="104" spans="1:23">
@@ -10121,7 +10181,7 @@
         <v>1519</v>
       </c>
       <c r="W104" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="105" spans="1:23">
@@ -10162,7 +10222,7 @@
         <v>1517</v>
       </c>
       <c r="W105" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="106" spans="1:23">
@@ -10203,7 +10263,7 @@
         <v>1517</v>
       </c>
       <c r="W106" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="107" spans="1:23">
@@ -10244,7 +10304,7 @@
         <v>1520</v>
       </c>
       <c r="W107" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="108" spans="1:23">
@@ -10285,7 +10345,7 @@
         <v>1519</v>
       </c>
       <c r="W108" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="109" spans="1:23">
@@ -10325,8 +10385,11 @@
       <c r="M109" t="s">
         <v>1520</v>
       </c>
+      <c r="V109" t="s">
+        <v>482</v>
+      </c>
       <c r="W109" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="110" spans="1:23">
@@ -10381,8 +10444,11 @@
       <c r="U110" t="s">
         <v>1600</v>
       </c>
+      <c r="V110" t="s">
+        <v>465</v>
+      </c>
       <c r="W110" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="111" spans="1:23">
@@ -10494,7 +10560,7 @@
         <v>1602</v>
       </c>
       <c r="W112" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="113" spans="1:23">
@@ -10538,7 +10604,7 @@
         <v>1526</v>
       </c>
       <c r="W113" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="114" spans="1:23">
@@ -10582,7 +10648,7 @@
         <v>1524</v>
       </c>
       <c r="W114" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="115" spans="1:23">
@@ -10625,8 +10691,11 @@
       <c r="M115" t="s">
         <v>1524</v>
       </c>
+      <c r="V115" t="s">
+        <v>488</v>
+      </c>
       <c r="W115" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="116" spans="1:23">
@@ -10685,7 +10754,7 @@
         <v>1603</v>
       </c>
       <c r="W116" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="117" spans="1:23">
@@ -10729,7 +10798,7 @@
         <v>1524</v>
       </c>
       <c r="W117" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="118" spans="1:23">
@@ -10776,7 +10845,7 @@
         <v>1532</v>
       </c>
       <c r="W118" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="119" spans="1:23">
@@ -10820,7 +10889,7 @@
         <v>1517</v>
       </c>
       <c r="W119" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="120" spans="1:23">
@@ -10861,7 +10930,7 @@
         <v>1517</v>
       </c>
       <c r="W120" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="121" spans="1:23">
@@ -10905,7 +10974,7 @@
         <v>1518</v>
       </c>
       <c r="W121" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="122" spans="1:23">
@@ -10951,11 +11020,8 @@
       <c r="R122" t="s">
         <v>1577</v>
       </c>
-      <c r="V122" t="s">
-        <v>1608</v>
-      </c>
       <c r="W122" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="123" spans="1:23">
@@ -10999,7 +11065,7 @@
         <v>1518</v>
       </c>
       <c r="W123" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="124" spans="1:23">
@@ -11043,7 +11109,7 @@
         <v>1518</v>
       </c>
       <c r="W124" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="125" spans="1:23">
@@ -11086,8 +11152,11 @@
       <c r="M125" t="s">
         <v>1520</v>
       </c>
+      <c r="V125" t="s">
+        <v>497</v>
+      </c>
       <c r="W125" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="126" spans="1:23">
@@ -11127,8 +11196,11 @@
       <c r="M126" t="s">
         <v>1527</v>
       </c>
+      <c r="V126" t="s">
+        <v>452</v>
+      </c>
       <c r="W126" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="127" spans="1:23">
@@ -11183,8 +11255,11 @@
       <c r="U127" t="s">
         <v>1604</v>
       </c>
+      <c r="V127" t="s">
+        <v>453</v>
+      </c>
       <c r="W127" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="128" spans="1:23">
@@ -11225,7 +11300,7 @@
         <v>1520</v>
       </c>
       <c r="W128" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="129" spans="1:23">
@@ -11266,7 +11341,7 @@
         <v>1520</v>
       </c>
       <c r="W129" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="130" spans="1:23">
@@ -11307,7 +11382,7 @@
         <v>1520</v>
       </c>
       <c r="W130" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="131" spans="1:23">
@@ -11348,7 +11423,7 @@
         <v>1520</v>
       </c>
       <c r="W131" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="132" spans="1:23">
@@ -11392,7 +11467,7 @@
         <v>1528</v>
       </c>
       <c r="W132" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="133" spans="1:23">
@@ -11432,8 +11507,11 @@
       <c r="M133" t="s">
         <v>1517</v>
       </c>
+      <c r="V133" t="s">
+        <v>454</v>
+      </c>
       <c r="W133" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="134" spans="1:23">
@@ -11473,8 +11551,11 @@
       <c r="M134" t="s">
         <v>1527</v>
       </c>
+      <c r="V134" t="s">
+        <v>455</v>
+      </c>
       <c r="W134" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="135" spans="1:23">
@@ -11515,7 +11596,7 @@
         <v>1527</v>
       </c>
       <c r="W135" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="136" spans="1:23">
@@ -11556,7 +11637,7 @@
         <v>1527</v>
       </c>
       <c r="W136" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="137" spans="1:23">
@@ -11597,7 +11678,7 @@
         <v>1518</v>
       </c>
       <c r="W137" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="138" spans="1:23">
@@ -11638,7 +11719,7 @@
         <v>1518</v>
       </c>
       <c r="W138" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="139" spans="1:23">
@@ -11685,7 +11766,7 @@
         <v>1605</v>
       </c>
       <c r="W139" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="140" spans="1:23">
@@ -11726,7 +11807,7 @@
         <v>1519</v>
       </c>
       <c r="W140" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="141" spans="1:23">
@@ -11767,7 +11848,7 @@
         <v>1519</v>
       </c>
       <c r="W141" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="142" spans="1:23">
@@ -11808,7 +11889,7 @@
         <v>1519</v>
       </c>
       <c r="W142" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="143" spans="1:23">
@@ -11851,8 +11932,11 @@
       <c r="M143" t="s">
         <v>1519</v>
       </c>
+      <c r="V143" t="s">
+        <v>454</v>
+      </c>
       <c r="W143" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="144" spans="1:23">
@@ -11892,8 +11976,11 @@
       <c r="M144" t="s">
         <v>1520</v>
       </c>
+      <c r="V144" t="s">
+        <v>455</v>
+      </c>
       <c r="W144" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="145" spans="1:23">
@@ -11933,8 +12020,11 @@
       <c r="M145" t="s">
         <v>1524</v>
       </c>
+      <c r="V145" t="s">
+        <v>510</v>
+      </c>
       <c r="W145" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="146" spans="1:23">
@@ -11974,8 +12064,11 @@
       <c r="M146" t="s">
         <v>1524</v>
       </c>
+      <c r="V146" t="s">
+        <v>482</v>
+      </c>
       <c r="W146" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="147" spans="1:23">
@@ -12015,8 +12108,11 @@
       <c r="M147" t="s">
         <v>1524</v>
       </c>
+      <c r="V147" t="s">
+        <v>483</v>
+      </c>
       <c r="W147" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="148" spans="1:23">
@@ -12057,7 +12153,7 @@
         <v>1520</v>
       </c>
       <c r="W148" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="149" spans="1:23">
@@ -12097,8 +12193,11 @@
       <c r="M149" t="s">
         <v>1520</v>
       </c>
+      <c r="V149" t="s">
+        <v>454</v>
+      </c>
       <c r="W149" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="150" spans="1:23">
@@ -12138,8 +12237,11 @@
       <c r="M150" t="s">
         <v>1519</v>
       </c>
+      <c r="V150" t="s">
+        <v>455</v>
+      </c>
       <c r="W150" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="151" spans="1:23">
@@ -12179,8 +12281,11 @@
       <c r="M151" t="s">
         <v>1518</v>
       </c>
+      <c r="V151" t="s">
+        <v>512</v>
+      </c>
       <c r="W151" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="152" spans="1:23">
@@ -12220,8 +12325,11 @@
       <c r="M152" t="s">
         <v>1518</v>
       </c>
+      <c r="V152" t="s">
+        <v>513</v>
+      </c>
       <c r="W152" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="153" spans="1:23">
@@ -12312,7 +12420,7 @@
         <v>1523</v>
       </c>
       <c r="W154" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="155" spans="1:23">
@@ -12353,7 +12461,7 @@
         <v>1523</v>
       </c>
       <c r="W155" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="156" spans="1:23">
@@ -12394,7 +12502,7 @@
         <v>1523</v>
       </c>
       <c r="W156" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="157" spans="1:23">
@@ -12435,7 +12543,7 @@
         <v>1519</v>
       </c>
       <c r="W157" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="158" spans="1:23">
@@ -12476,7 +12584,7 @@
         <v>1518</v>
       </c>
       <c r="W158" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="159" spans="1:23">
@@ -12517,7 +12625,7 @@
         <v>1518</v>
       </c>
       <c r="W159" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="160" spans="1:23">
@@ -12558,7 +12666,7 @@
         <v>1518</v>
       </c>
       <c r="W160" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="161" spans="1:23">
@@ -12599,7 +12707,7 @@
         <v>1518</v>
       </c>
       <c r="W161" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="162" spans="1:23">
@@ -12639,8 +12747,11 @@
       <c r="M162" t="s">
         <v>1519</v>
       </c>
+      <c r="V162" t="s">
+        <v>461</v>
+      </c>
       <c r="W162" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="163" spans="1:23">
@@ -12680,8 +12791,11 @@
       <c r="M163" t="s">
         <v>1518</v>
       </c>
+      <c r="V163" t="s">
+        <v>520</v>
+      </c>
       <c r="W163" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="164" spans="1:23">
@@ -12722,7 +12836,7 @@
         <v>1518</v>
       </c>
       <c r="W164" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="165" spans="1:23">
@@ -12763,7 +12877,7 @@
         <v>1518</v>
       </c>
       <c r="W165" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="166" spans="1:23">
@@ -12803,8 +12917,11 @@
       <c r="M166" t="s">
         <v>1518</v>
       </c>
+      <c r="V166" t="s">
+        <v>522</v>
+      </c>
       <c r="W166" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="167" spans="1:23">
@@ -12845,7 +12962,7 @@
         <v>1518</v>
       </c>
       <c r="W167" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="168" spans="1:23">
@@ -12889,7 +13006,7 @@
         <v>1528</v>
       </c>
       <c r="W168" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="169" spans="1:23">
@@ -12933,7 +13050,7 @@
         <v>1528</v>
       </c>
       <c r="W169" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="170" spans="1:23">
@@ -12974,7 +13091,7 @@
         <v>1528</v>
       </c>
       <c r="W170" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="171" spans="1:23">
@@ -13015,7 +13132,7 @@
         <v>1528</v>
       </c>
       <c r="W171" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="172" spans="1:23">
@@ -13056,7 +13173,7 @@
         <v>1528</v>
       </c>
       <c r="W172" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="173" spans="1:23">
@@ -13097,7 +13214,7 @@
         <v>1528</v>
       </c>
       <c r="W173" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="174" spans="1:23">
@@ -13138,7 +13255,7 @@
         <v>1528</v>
       </c>
       <c r="W174" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="175" spans="1:23">
@@ -13179,7 +13296,7 @@
         <v>1528</v>
       </c>
       <c r="W175" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="176" spans="1:23">
@@ -13220,7 +13337,7 @@
         <v>1528</v>
       </c>
       <c r="W176" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="177" spans="1:23">
@@ -13261,7 +13378,7 @@
         <v>1528</v>
       </c>
       <c r="W177" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="178" spans="1:23">
@@ -13301,8 +13418,11 @@
       <c r="M178" t="s">
         <v>1528</v>
       </c>
+      <c r="V178" t="s">
+        <v>512</v>
+      </c>
       <c r="W178" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="179" spans="1:23">
@@ -13393,7 +13513,7 @@
         <v>1518</v>
       </c>
       <c r="W180" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="181" spans="1:23">
@@ -13433,8 +13553,11 @@
       <c r="M181" t="s">
         <v>1518</v>
       </c>
+      <c r="V181" t="s">
+        <v>533</v>
+      </c>
       <c r="W181" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="182" spans="1:23">
@@ -13475,7 +13598,7 @@
         <v>1518</v>
       </c>
       <c r="W182" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="183" spans="1:23">
@@ -13516,7 +13639,7 @@
         <v>1518</v>
       </c>
       <c r="W183" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="184" spans="1:23">
@@ -13557,7 +13680,7 @@
         <v>1520</v>
       </c>
       <c r="W184" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="185" spans="1:23">
@@ -13598,7 +13721,7 @@
         <v>1520</v>
       </c>
       <c r="W185" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="186" spans="1:23">
@@ -13639,7 +13762,7 @@
         <v>1520</v>
       </c>
       <c r="W186" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="187" spans="1:23">
@@ -13680,7 +13803,7 @@
         <v>1528</v>
       </c>
       <c r="W187" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="188" spans="1:23">
@@ -13721,7 +13844,7 @@
         <v>1528</v>
       </c>
       <c r="W188" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="189" spans="1:23">
@@ -13762,7 +13885,7 @@
         <v>1528</v>
       </c>
       <c r="W189" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="190" spans="1:23">
@@ -13803,7 +13926,7 @@
         <v>1528</v>
       </c>
       <c r="W190" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="191" spans="1:23">
@@ -13844,7 +13967,7 @@
         <v>1528</v>
       </c>
       <c r="W191" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="192" spans="1:23">
@@ -13885,7 +14008,7 @@
         <v>1528</v>
       </c>
       <c r="W192" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="193" spans="1:23">
@@ -13926,7 +14049,7 @@
         <v>1528</v>
       </c>
       <c r="W193" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="194" spans="1:23">
@@ -13967,7 +14090,7 @@
         <v>1528</v>
       </c>
       <c r="W194" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="195" spans="1:23">
@@ -14007,8 +14130,11 @@
       <c r="M195" t="s">
         <v>1517</v>
       </c>
+      <c r="V195" t="s">
+        <v>465</v>
+      </c>
       <c r="W195" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="196" spans="1:23">
@@ -14051,8 +14177,11 @@
       <c r="M196" t="s">
         <v>1523</v>
       </c>
+      <c r="V196" t="s">
+        <v>483</v>
+      </c>
       <c r="W196" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="197" spans="1:23">
@@ -14096,7 +14225,7 @@
         <v>1520</v>
       </c>
       <c r="W197" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="198" spans="1:23">
@@ -14137,7 +14266,7 @@
         <v>1519</v>
       </c>
       <c r="W198" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="199" spans="1:23">
@@ -14178,7 +14307,7 @@
         <v>1519</v>
       </c>
       <c r="W199" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="200" spans="1:23">
@@ -14219,7 +14348,7 @@
         <v>1518</v>
       </c>
       <c r="W200" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="201" spans="1:23">
@@ -14260,7 +14389,7 @@
         <v>1526</v>
       </c>
       <c r="W201" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="202" spans="1:23">
@@ -14300,8 +14429,11 @@
       <c r="M202" t="s">
         <v>1526</v>
       </c>
+      <c r="V202" t="s">
+        <v>520</v>
+      </c>
       <c r="W202" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="203" spans="1:23">
@@ -14341,8 +14473,11 @@
       <c r="M203" t="s">
         <v>1520</v>
       </c>
+      <c r="V203" t="s">
+        <v>549</v>
+      </c>
       <c r="W203" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="204" spans="1:23">
@@ -14383,7 +14518,7 @@
         <v>1520</v>
       </c>
       <c r="W204" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="205" spans="1:23">
@@ -14426,8 +14561,11 @@
       <c r="M205" t="s">
         <v>1518</v>
       </c>
+      <c r="V205" t="s">
+        <v>521</v>
+      </c>
       <c r="W205" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="206" spans="1:23">
@@ -14470,8 +14608,11 @@
       <c r="M206" t="s">
         <v>1518</v>
       </c>
+      <c r="V206" t="s">
+        <v>466</v>
+      </c>
       <c r="W206" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="207" spans="1:23">
@@ -14512,7 +14653,7 @@
         <v>1518</v>
       </c>
       <c r="W207" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="208" spans="1:23">
@@ -14553,7 +14694,7 @@
         <v>1518</v>
       </c>
       <c r="W208" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="209" spans="1:23">
@@ -14594,7 +14735,7 @@
         <v>1518</v>
       </c>
       <c r="W209" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="210" spans="1:23">
@@ -14635,7 +14776,7 @@
         <v>1518</v>
       </c>
       <c r="W210" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="211" spans="1:23">
@@ -14676,7 +14817,7 @@
         <v>1518</v>
       </c>
       <c r="W211" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="212" spans="1:23">
@@ -14717,7 +14858,7 @@
         <v>1518</v>
       </c>
       <c r="W212" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="213" spans="1:23">
@@ -14758,7 +14899,7 @@
         <v>1518</v>
       </c>
       <c r="W213" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="214" spans="1:23">
@@ -14798,8 +14939,11 @@
       <c r="M214" t="s">
         <v>1518</v>
       </c>
+      <c r="V214" t="s">
+        <v>401</v>
+      </c>
       <c r="W214" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="215" spans="1:23">
@@ -14840,7 +14984,7 @@
         <v>1517</v>
       </c>
       <c r="W215" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="216" spans="1:23">
@@ -14881,7 +15025,7 @@
         <v>1519</v>
       </c>
       <c r="W216" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="217" spans="1:23">
@@ -14922,7 +15066,7 @@
         <v>1520</v>
       </c>
       <c r="W217" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="218" spans="1:23">
@@ -14963,7 +15107,7 @@
         <v>1520</v>
       </c>
       <c r="W218" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="219" spans="1:23">
@@ -15004,7 +15148,7 @@
         <v>1520</v>
       </c>
       <c r="W219" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="220" spans="1:23">
@@ -15045,7 +15189,7 @@
         <v>1524</v>
       </c>
       <c r="W220" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="221" spans="1:23">
@@ -15086,7 +15230,7 @@
         <v>1524</v>
       </c>
       <c r="W221" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="222" spans="1:23">
@@ -15127,7 +15271,7 @@
         <v>1524</v>
       </c>
       <c r="W222" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="223" spans="1:23">
@@ -15168,7 +15312,7 @@
         <v>1524</v>
       </c>
       <c r="W223" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="224" spans="1:23">
@@ -15209,7 +15353,7 @@
         <v>1524</v>
       </c>
       <c r="W224" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="225" spans="1:23">
@@ -15250,7 +15394,7 @@
         <v>1524</v>
       </c>
       <c r="W225" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="226" spans="1:23">
@@ -15291,7 +15435,7 @@
         <v>1524</v>
       </c>
       <c r="W226" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="227" spans="1:23">
@@ -15332,7 +15476,7 @@
         <v>1524</v>
       </c>
       <c r="W227" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="228" spans="1:23">
@@ -15373,7 +15517,7 @@
         <v>1524</v>
       </c>
       <c r="W228" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="229" spans="1:23">
@@ -15414,7 +15558,7 @@
         <v>1524</v>
       </c>
       <c r="W229" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="230" spans="1:23">
@@ -15455,7 +15599,7 @@
         <v>1524</v>
       </c>
       <c r="W230" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="231" spans="1:23">
@@ -15496,7 +15640,7 @@
         <v>1524</v>
       </c>
       <c r="W231" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="232" spans="1:23">
@@ -15537,7 +15681,7 @@
         <v>1524</v>
       </c>
       <c r="W232" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="233" spans="1:23">
@@ -15578,7 +15722,7 @@
         <v>1524</v>
       </c>
       <c r="W233" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="234" spans="1:23">
@@ -15619,7 +15763,7 @@
         <v>1518</v>
       </c>
       <c r="W234" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="235" spans="1:23">
@@ -15660,7 +15804,7 @@
         <v>1518</v>
       </c>
       <c r="W235" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="236" spans="1:23">
@@ -15701,7 +15845,7 @@
         <v>1518</v>
       </c>
       <c r="W236" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="237" spans="1:23">
@@ -15742,7 +15886,7 @@
         <v>1518</v>
       </c>
       <c r="W237" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="238" spans="1:23">
@@ -15783,7 +15927,7 @@
         <v>1518</v>
       </c>
       <c r="W238" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="239" spans="1:23">
@@ -15823,8 +15967,11 @@
       <c r="M239" t="s">
         <v>1518</v>
       </c>
+      <c r="V239" t="s">
+        <v>570</v>
+      </c>
       <c r="W239" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="240" spans="1:23">
@@ -15865,7 +16012,7 @@
         <v>1518</v>
       </c>
       <c r="W240" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="241" spans="1:23">
@@ -15906,7 +16053,7 @@
         <v>1518</v>
       </c>
       <c r="W241" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="242" spans="1:23">
@@ -15946,8 +16093,11 @@
       <c r="M242" t="s">
         <v>1518</v>
       </c>
+      <c r="V242" t="s">
+        <v>482</v>
+      </c>
       <c r="W242" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="243" spans="1:23">
@@ -15988,7 +16138,7 @@
         <v>1518</v>
       </c>
       <c r="W243" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="244" spans="1:23">
@@ -16029,7 +16179,7 @@
         <v>1518</v>
       </c>
       <c r="W244" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="245" spans="1:23">
@@ -16070,7 +16220,7 @@
         <v>1518</v>
       </c>
       <c r="W245" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="246" spans="1:23">
@@ -16110,8 +16260,11 @@
       <c r="M246" t="s">
         <v>1518</v>
       </c>
+      <c r="V246" t="s">
+        <v>466</v>
+      </c>
       <c r="W246" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="247" spans="1:23">
@@ -16152,7 +16305,7 @@
         <v>1518</v>
       </c>
       <c r="W247" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="248" spans="1:23">
@@ -16193,7 +16346,7 @@
         <v>1518</v>
       </c>
       <c r="W248" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="249" spans="1:23">
@@ -16234,7 +16387,7 @@
         <v>1526</v>
       </c>
       <c r="W249" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="250" spans="1:23">
@@ -16275,7 +16428,7 @@
         <v>1518</v>
       </c>
       <c r="W250" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="251" spans="1:23">
@@ -16316,7 +16469,7 @@
         <v>1520</v>
       </c>
       <c r="W251" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="252" spans="1:23">
@@ -16357,7 +16510,7 @@
         <v>1519</v>
       </c>
       <c r="W252" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="253" spans="1:23">
@@ -16397,8 +16550,11 @@
       <c r="M253" t="s">
         <v>1526</v>
       </c>
+      <c r="V253" t="s">
+        <v>579</v>
+      </c>
       <c r="W253" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="254" spans="1:23">
@@ -16442,7 +16598,7 @@
         <v>1519</v>
       </c>
       <c r="W254" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="255" spans="1:23">
@@ -16483,7 +16639,7 @@
         <v>1523</v>
       </c>
       <c r="W255" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="256" spans="1:23">
@@ -16524,7 +16680,7 @@
         <v>1523</v>
       </c>
       <c r="W256" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="257" spans="1:23">
@@ -16620,8 +16776,11 @@
       <c r="M258" t="s">
         <v>1520</v>
       </c>
+      <c r="V258" t="s">
+        <v>453</v>
+      </c>
       <c r="W258" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="259" spans="1:23">
@@ -16664,8 +16823,11 @@
       <c r="M259" t="s">
         <v>1518</v>
       </c>
+      <c r="V259" t="s">
+        <v>1608</v>
+      </c>
       <c r="W259" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="260" spans="1:23">
@@ -16761,8 +16923,11 @@
       <c r="M261" t="s">
         <v>1518</v>
       </c>
+      <c r="V261" t="s">
+        <v>584</v>
+      </c>
       <c r="W261" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="262" spans="1:23">
@@ -16805,8 +16970,11 @@
       <c r="M262" t="s">
         <v>1518</v>
       </c>
+      <c r="V262" t="s">
+        <v>512</v>
+      </c>
       <c r="W262" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="263" spans="1:23">
@@ -16903,7 +17071,7 @@
         <v>1519</v>
       </c>
       <c r="W264" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="265" spans="1:23">
@@ -16944,7 +17112,7 @@
         <v>1519</v>
       </c>
       <c r="W265" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="266" spans="1:23">
@@ -16985,7 +17153,7 @@
         <v>1519</v>
       </c>
       <c r="W266" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="267" spans="1:23">
@@ -17026,7 +17194,7 @@
         <v>1517</v>
       </c>
       <c r="W267" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="268" spans="1:23">
@@ -17070,7 +17238,7 @@
         <v>1520</v>
       </c>
       <c r="W268" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="269" spans="1:23">
@@ -17111,7 +17279,7 @@
         <v>1520</v>
       </c>
       <c r="W269" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="270" spans="1:23">
@@ -17152,7 +17320,7 @@
         <v>1520</v>
       </c>
       <c r="W270" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="271" spans="1:23">
@@ -17193,7 +17361,7 @@
         <v>1520</v>
       </c>
       <c r="W271" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="272" spans="1:23">
@@ -17233,8 +17401,11 @@
       <c r="M272" t="s">
         <v>1520</v>
       </c>
+      <c r="V272" t="s">
+        <v>590</v>
+      </c>
       <c r="W272" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="273" spans="1:23">
@@ -17278,7 +17449,7 @@
         <v>1520</v>
       </c>
       <c r="W273" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="274" spans="1:23">
@@ -17322,7 +17493,7 @@
         <v>1520</v>
       </c>
       <c r="W274" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="275" spans="1:23">
@@ -17363,7 +17534,7 @@
         <v>1520</v>
       </c>
       <c r="W275" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="276" spans="1:23">
@@ -17404,7 +17575,7 @@
         <v>1520</v>
       </c>
       <c r="W276" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="277" spans="1:23">
@@ -17445,7 +17616,7 @@
         <v>1520</v>
       </c>
       <c r="W277" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="278" spans="1:23">
@@ -17486,7 +17657,7 @@
         <v>1520</v>
       </c>
       <c r="W278" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="279" spans="1:23">
@@ -17527,7 +17698,7 @@
         <v>1520</v>
       </c>
       <c r="W279" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="280" spans="1:23">
@@ -17568,7 +17739,7 @@
         <v>1520</v>
       </c>
       <c r="W280" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="281" spans="1:23">
@@ -17609,7 +17780,7 @@
         <v>1520</v>
       </c>
       <c r="W281" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="282" spans="1:23">
@@ -17650,7 +17821,7 @@
         <v>1520</v>
       </c>
       <c r="W282" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="283" spans="1:23">
@@ -17691,7 +17862,7 @@
         <v>1520</v>
       </c>
       <c r="W283" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="284" spans="1:23">
@@ -17732,7 +17903,7 @@
         <v>1520</v>
       </c>
       <c r="W284" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="285" spans="1:23">
@@ -17773,7 +17944,7 @@
         <v>1520</v>
       </c>
       <c r="W285" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="286" spans="1:23">
@@ -17814,7 +17985,7 @@
         <v>1520</v>
       </c>
       <c r="W286" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="287" spans="1:23">
@@ -17855,7 +18026,7 @@
         <v>1519</v>
       </c>
       <c r="W287" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="288" spans="1:23">
@@ -17896,7 +18067,7 @@
         <v>1517</v>
       </c>
       <c r="W288" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="289" spans="1:23">
@@ -17937,7 +18108,7 @@
         <v>1520</v>
       </c>
       <c r="W289" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="290" spans="1:23">
@@ -17978,7 +18149,7 @@
         <v>1520</v>
       </c>
       <c r="W290" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="291" spans="1:23">
@@ -18019,7 +18190,7 @@
         <v>1517</v>
       </c>
       <c r="W291" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="292" spans="1:23">
@@ -18060,7 +18231,7 @@
         <v>1517</v>
       </c>
       <c r="W292" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="293" spans="1:23">
@@ -18101,7 +18272,7 @@
         <v>1519</v>
       </c>
       <c r="W293" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="294" spans="1:23">
@@ -18142,7 +18313,7 @@
         <v>1518</v>
       </c>
       <c r="W294" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="295" spans="1:23">
@@ -18182,8 +18353,11 @@
       <c r="M295" t="s">
         <v>1518</v>
       </c>
+      <c r="V295" t="s">
+        <v>605</v>
+      </c>
       <c r="W295" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="296" spans="1:23">
@@ -18226,8 +18400,11 @@
       <c r="M296" t="s">
         <v>1518</v>
       </c>
+      <c r="V296" t="s">
+        <v>606</v>
+      </c>
       <c r="W296" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="297" spans="1:23">
@@ -18271,7 +18448,7 @@
         <v>1527</v>
       </c>
       <c r="W297" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="298" spans="1:23">
@@ -18312,7 +18489,7 @@
         <v>1527</v>
       </c>
       <c r="W298" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="299" spans="1:23">
@@ -18353,7 +18530,7 @@
         <v>1527</v>
       </c>
       <c r="W299" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="300" spans="1:23">
@@ -18394,7 +18571,7 @@
         <v>1527</v>
       </c>
       <c r="W300" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="301" spans="1:23">
@@ -18435,7 +18612,7 @@
         <v>1527</v>
       </c>
       <c r="W301" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="302" spans="1:23">
@@ -18476,7 +18653,7 @@
         <v>1519</v>
       </c>
       <c r="W302" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="303" spans="1:23">
@@ -18517,7 +18694,7 @@
         <v>1519</v>
       </c>
       <c r="W303" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="304" spans="1:23">
@@ -18558,7 +18735,7 @@
         <v>1519</v>
       </c>
       <c r="W304" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="305" spans="1:23">
@@ -18599,7 +18776,7 @@
         <v>1519</v>
       </c>
       <c r="W305" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="306" spans="1:23">
@@ -18640,7 +18817,7 @@
         <v>1520</v>
       </c>
       <c r="W306" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="307" spans="1:23">
@@ -18681,7 +18858,7 @@
         <v>1520</v>
       </c>
       <c r="W307" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="308" spans="1:23">
@@ -18722,7 +18899,7 @@
         <v>1520</v>
       </c>
       <c r="W308" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="309" spans="1:23">
@@ -18763,7 +18940,7 @@
         <v>1520</v>
       </c>
       <c r="W309" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="310" spans="1:23">
@@ -18804,7 +18981,7 @@
         <v>1520</v>
       </c>
       <c r="W310" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="311" spans="1:23">
@@ -18845,7 +19022,7 @@
         <v>1520</v>
       </c>
       <c r="W311" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="312" spans="1:23">
@@ -18886,7 +19063,7 @@
         <v>1520</v>
       </c>
       <c r="W312" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="313" spans="1:23">
@@ -18927,7 +19104,7 @@
         <v>1517</v>
       </c>
       <c r="W313" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="314" spans="1:23">
@@ -18968,7 +19145,7 @@
         <v>1517</v>
       </c>
       <c r="W314" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="315" spans="1:23">
@@ -19009,7 +19186,7 @@
         <v>1518</v>
       </c>
       <c r="W315" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="316" spans="1:23">
@@ -19050,7 +19227,7 @@
         <v>1518</v>
       </c>
       <c r="W316" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="317" spans="1:23">
@@ -19091,7 +19268,7 @@
         <v>1518</v>
       </c>
       <c r="W317" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="318" spans="1:23">
@@ -19132,7 +19309,7 @@
         <v>1518</v>
       </c>
       <c r="W318" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="319" spans="1:23">
@@ -19173,7 +19350,7 @@
         <v>1518</v>
       </c>
       <c r="W319" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="320" spans="1:23">
@@ -19214,7 +19391,7 @@
         <v>1518</v>
       </c>
       <c r="W320" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="321" spans="1:23">
@@ -19254,8 +19431,11 @@
       <c r="M321" t="s">
         <v>1518</v>
       </c>
+      <c r="V321" t="s">
+        <v>398</v>
+      </c>
       <c r="W321" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="322" spans="1:23">
@@ -19296,7 +19476,7 @@
         <v>1518</v>
       </c>
       <c r="W322" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="323" spans="1:23">
@@ -19337,7 +19517,7 @@
         <v>1523</v>
       </c>
       <c r="W323" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="324" spans="1:23">
@@ -19378,7 +19558,7 @@
         <v>1523</v>
       </c>
       <c r="W324" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="325" spans="1:23">
@@ -19419,7 +19599,7 @@
         <v>1523</v>
       </c>
       <c r="W325" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="326" spans="1:23">
@@ -19462,8 +19642,11 @@
       <c r="M326" t="s">
         <v>1524</v>
       </c>
+      <c r="V326" t="s">
+        <v>629</v>
+      </c>
       <c r="W326" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="327" spans="1:23">
@@ -19507,7 +19690,7 @@
         <v>1524</v>
       </c>
       <c r="W327" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="328" spans="1:23">
@@ -19548,7 +19731,7 @@
         <v>1518</v>
       </c>
       <c r="W328" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="329" spans="1:23">
@@ -19589,7 +19772,7 @@
         <v>1518</v>
       </c>
       <c r="W329" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="330" spans="1:23">
@@ -19630,7 +19813,7 @@
         <v>1520</v>
       </c>
       <c r="W330" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="331" spans="1:23">
@@ -19671,7 +19854,7 @@
         <v>1526</v>
       </c>
       <c r="W331" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="332" spans="1:23">
@@ -19712,7 +19895,7 @@
         <v>1518</v>
       </c>
       <c r="W332" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="333" spans="1:23">
@@ -19753,7 +19936,7 @@
         <v>1518</v>
       </c>
       <c r="W333" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="334" spans="1:23">
@@ -19794,7 +19977,7 @@
         <v>1518</v>
       </c>
       <c r="W334" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="335" spans="1:23">
@@ -19835,7 +20018,7 @@
         <v>1518</v>
       </c>
       <c r="W335" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="336" spans="1:23">
@@ -19876,7 +20059,7 @@
         <v>1518</v>
       </c>
       <c r="W336" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="337" spans="1:23">
@@ -19917,7 +20100,7 @@
         <v>1518</v>
       </c>
       <c r="W337" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="338" spans="1:23">
@@ -19958,7 +20141,7 @@
         <v>1518</v>
       </c>
       <c r="W338" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="339" spans="1:23">
@@ -19999,7 +20182,7 @@
         <v>1518</v>
       </c>
       <c r="W339" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="340" spans="1:23">
@@ -20040,7 +20223,7 @@
         <v>1517</v>
       </c>
       <c r="W340" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="341" spans="1:23">
@@ -20081,7 +20264,7 @@
         <v>1518</v>
       </c>
       <c r="W341" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="342" spans="1:23">
@@ -20122,7 +20305,7 @@
         <v>1518</v>
       </c>
       <c r="W342" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="343" spans="1:23">
@@ -20163,7 +20346,7 @@
         <v>1524</v>
       </c>
       <c r="W343" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="344" spans="1:23">
@@ -20204,7 +20387,7 @@
         <v>1524</v>
       </c>
       <c r="W344" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="345" spans="1:23">
@@ -20245,7 +20428,7 @@
         <v>1524</v>
       </c>
       <c r="W345" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="346" spans="1:23">
@@ -20285,8 +20468,11 @@
       <c r="M346" t="s">
         <v>1519</v>
       </c>
+      <c r="V346" t="s">
+        <v>1609</v>
+      </c>
       <c r="W346" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="347" spans="1:23">
@@ -20327,7 +20513,7 @@
         <v>1517</v>
       </c>
       <c r="W347" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="348" spans="1:23">
@@ -20371,7 +20557,7 @@
         <v>1519</v>
       </c>
       <c r="W348" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="349" spans="1:23">
@@ -20412,7 +20598,7 @@
         <v>1527</v>
       </c>
       <c r="W349" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="350" spans="1:23">
@@ -20453,7 +20639,7 @@
         <v>1520</v>
       </c>
       <c r="W350" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="351" spans="1:23">
@@ -20494,7 +20680,7 @@
         <v>1520</v>
       </c>
       <c r="W351" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="352" spans="1:23">
@@ -20534,8 +20720,11 @@
       <c r="M352" t="s">
         <v>1519</v>
       </c>
+      <c r="V352" t="s">
+        <v>1610</v>
+      </c>
       <c r="W352" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="353" spans="1:23">
@@ -20575,8 +20764,11 @@
       <c r="M353" t="s">
         <v>1520</v>
       </c>
+      <c r="V353" t="s">
+        <v>1610</v>
+      </c>
       <c r="W353" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="354" spans="1:23">
@@ -20616,8 +20808,11 @@
       <c r="M354" t="s">
         <v>1519</v>
       </c>
+      <c r="V354" t="s">
+        <v>1610</v>
+      </c>
       <c r="W354" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="355" spans="1:23">
@@ -20657,8 +20852,11 @@
       <c r="M355" t="s">
         <v>1523</v>
       </c>
+      <c r="V355" t="s">
+        <v>1610</v>
+      </c>
       <c r="W355" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="356" spans="1:23">
@@ -20698,8 +20896,11 @@
       <c r="M356" t="s">
         <v>1523</v>
       </c>
+      <c r="V356" t="s">
+        <v>1610</v>
+      </c>
       <c r="W356" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="357" spans="1:23">
@@ -20739,8 +20940,11 @@
       <c r="M357" t="s">
         <v>1523</v>
       </c>
+      <c r="V357" t="s">
+        <v>1610</v>
+      </c>
       <c r="W357" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="358" spans="1:23">
@@ -20780,8 +20984,11 @@
       <c r="M358" t="s">
         <v>1523</v>
       </c>
+      <c r="V358" t="s">
+        <v>1610</v>
+      </c>
       <c r="W358" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="359" spans="1:23">
@@ -20821,8 +21028,11 @@
       <c r="M359" t="s">
         <v>1520</v>
       </c>
+      <c r="V359" t="s">
+        <v>1610</v>
+      </c>
       <c r="W359" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="360" spans="1:23">
@@ -20862,8 +21072,11 @@
       <c r="M360" t="s">
         <v>1520</v>
       </c>
+      <c r="V360" t="s">
+        <v>1610</v>
+      </c>
       <c r="W360" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
     <row r="361" spans="1:23">
@@ -20903,8 +21116,11 @@
       <c r="M361" t="s">
         <v>1518</v>
       </c>
+      <c r="V361" t="s">
+        <v>1610</v>
+      </c>
       <c r="W361" t="s">
-        <v>1609</v>
+        <v>1611</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualização automática: devolucoes (12/08/2026 15:03)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4381" uniqueCount="1612">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4496" uniqueCount="1695">
   <si>
     <t>numero_ordem</t>
   </si>
@@ -4636,6 +4636,21 @@
     <t>51539-012M</t>
   </si>
   <si>
+    <t>200SGL119Q</t>
+  </si>
+  <si>
+    <t>324843-2020</t>
+  </si>
+  <si>
+    <t>ENTREGUE NA BANT SERIAL KAS297B-A23223</t>
+  </si>
+  <si>
+    <t>ENTREGUE NA BABE SERIAL 471591</t>
+  </si>
+  <si>
+    <t>ENTREGUE NA BANT COMO ESTOQUE 8EA</t>
+  </si>
+  <si>
     <t>ENTREGUE NO PAMALS SERIAL 53850</t>
   </si>
   <si>
@@ -4648,6 +4663,9 @@
     <t>ENTREGUE NO PAMALS</t>
   </si>
   <si>
+    <t>ENVIAMOS UM TOTAL DE 95 EA COMO MAPEM PARA A ANV 2719</t>
+  </si>
+  <si>
     <t>ENTREGUE NO PAMALS SERIAL 322</t>
   </si>
   <si>
@@ -4675,12 +4693,48 @@
     <t>ENTREGUE NO PAMALS SERIAL 8320</t>
   </si>
   <si>
+    <t>ENTREGUE NA BABE SERIAL 22007425</t>
+  </si>
+  <si>
     <t>ENTREGUE NA BABR AWB 127-0209 6522</t>
   </si>
   <si>
+    <t>ENTREGUE NA BABR SERIAL 9599</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAS 965, UNK01, 03, 482, B4H-018, 39</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 01B</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL LSEAM3269</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 772</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL KA51B43711</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL T25814</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 23091</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 37853</t>
+  </si>
+  <si>
     <t>entregue 2 ea seriais 21890, 21990</t>
   </si>
   <si>
+    <t>ENTREGUE NA BANT SERIAL 1439</t>
+  </si>
+  <si>
+    <t>ESSE ITEM FOI REPARADO PELA VEEONE O.S 3040252159</t>
+  </si>
+  <si>
     <t>já tinha sido entregue 1 ea serial 1570 em estoque</t>
   </si>
   <si>
@@ -4693,21 +4747,148 @@
     <t>mapem</t>
   </si>
   <si>
+    <t>ENTREGUE NO PAMALS SERIAL T3011</t>
+  </si>
+  <si>
     <t>foram entregues no pamals 3 ea desse PN</t>
   </si>
   <si>
+    <t>ENTREGUE NO PAMALS SERIAL 795</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 48</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL LSEAM3218</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL LSEAM3167</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 3367-5</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 1570</t>
+  </si>
+  <si>
+    <t>ENTREUE NO PAMALS SERIAL 4144, 4118</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 784</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL LSEAM3168</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL X-330978</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS O SERIAL 90566</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 30435</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL T35158</t>
+  </si>
+  <si>
+    <t>PRECISA INFORMAR
+ O SERIAL</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 92A0049A</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL X-412785</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIA 6708</t>
+  </si>
+  <si>
+    <t>ESSE ITEM FOI REPARADO PELA VEEONE</t>
+  </si>
+  <si>
+    <t>ENTREUE NO PAMALS SERIAL 4741</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL T35507</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 0215-217</t>
+  </si>
+  <si>
+    <t>ESSE TEM FOI REVISADO PELA VEEONE O.S.3040250795</t>
+  </si>
+  <si>
+    <t>ESSE TEM FOI REVISADO PELA VEEONE O.S.3040250230</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 24890</t>
+  </si>
+  <si>
+    <t>ENTREGUE NA BABR SERIAL L1082</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 1874</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 7077</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 21990</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 374579</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL B4H-018</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 2691-5</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO DACTAII SERIAL 1023481-005</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL B-10811721</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 22A805</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 8317</t>
+  </si>
+  <si>
+    <t>ENTREGUE NO PAMALS SERIAL 4134</t>
+  </si>
+  <si>
+    <t>ENTREGUE NA BANT SERIAL 148515-04</t>
+  </si>
+  <si>
+    <t>ENTREGUE NA BAMN SERIAL 070407983320094AE</t>
+  </si>
+  <si>
+    <t>599/FAB/26</t>
+  </si>
+  <si>
+    <t>128/FAB/26</t>
+  </si>
+  <si>
+    <t>135/FAB/25</t>
+  </si>
+  <si>
     <t>1028/LS-C98/2025</t>
   </si>
   <si>
-    <t>135/FAB/25</t>
-  </si>
-  <si>
     <t>133/C 98/2025</t>
   </si>
   <si>
     <t>1088/PAMALS/2025</t>
   </si>
   <si>
+    <t>469/FAB/26</t>
+  </si>
+  <si>
     <t>143/C98/2025</t>
   </si>
   <si>
@@ -4726,15 +4907,42 @@
     <t>1100/LS-C-98/2025</t>
   </si>
   <si>
+    <t>258/FAB/26</t>
+  </si>
+  <si>
     <t>156/FAB/25</t>
   </si>
   <si>
     <t>1082/LS-C98/2025</t>
   </si>
   <si>
+    <t>488/FAB/2026</t>
+  </si>
+  <si>
+    <t>598/FAB/26</t>
+  </si>
+  <si>
+    <t>1098/LS-C98/2025</t>
+  </si>
+  <si>
+    <t>1099/LS-C98/2025</t>
+  </si>
+  <si>
+    <t>1102/LS-C-98/2025</t>
+  </si>
+  <si>
+    <t>1103/C98/2025</t>
+  </si>
+  <si>
     <t>016/FAB/26</t>
   </si>
   <si>
+    <t>1116/LS-C-98/2026</t>
+  </si>
+  <si>
+    <t>1100/FAB/2025</t>
+  </si>
+  <si>
     <t>045/C98/2025</t>
   </si>
   <si>
@@ -4750,9 +4958,51 @@
     <t>1071/LS-C-98/2025</t>
   </si>
   <si>
+    <t>45/C98/2025</t>
+  </si>
+  <si>
     <t>159/C98/2025, 160/c98/2025</t>
   </si>
   <si>
+    <t>1085/PAMALS/2025</t>
+  </si>
+  <si>
+    <t>438/FAB/2026</t>
+  </si>
+  <si>
+    <t>1013/LS-C98/2025</t>
+  </si>
+  <si>
+    <t>055/C98/2025</t>
+  </si>
+  <si>
+    <t>161/C98/2025</t>
+  </si>
+  <si>
+    <t>1007/FAB/2025</t>
+  </si>
+  <si>
+    <t>569/FAB/26</t>
+  </si>
+  <si>
+    <t>189/FAB/26</t>
+  </si>
+  <si>
+    <t>133/FAB/25</t>
+  </si>
+  <si>
+    <t>1065/LS-C98/2025</t>
+  </si>
+  <si>
+    <t>103/C98/2025</t>
+  </si>
+  <si>
+    <t>641/FAB/26</t>
+  </si>
+  <si>
+    <t>5/28/2025</t>
+  </si>
+  <si>
     <t>Lembro da empresa comentar algo sobre esses itens. Favor escrever o motivo. 04.02</t>
   </si>
   <si>
@@ -4840,16 +5090,16 @@
     <t>ENTREGUE NO 03-06-2026 VIA RECIBO 438/FAB/2026</t>
   </si>
   <si>
-    <t>200SGL119Q</t>
-  </si>
-  <si>
-    <t>324843-2020</t>
-  </si>
-  <si>
-    <t>#N/A</t>
+    <t>esse item foi reparado pela VeeOne e enviado ao estoque do PAMALS</t>
   </si>
   <si>
     <t>Pendente</t>
+  </si>
+  <si>
+    <t>Desconsiderado</t>
+  </si>
+  <si>
+    <t>OK</t>
   </si>
 </sst>
 </file>
@@ -5300,7 +5550,7 @@
         <v>1516</v>
       </c>
       <c r="W2" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="3" spans="1:23">
@@ -5344,7 +5594,7 @@
         <v>1517</v>
       </c>
       <c r="W3" t="s">
-        <v>1610</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="4" spans="1:23">
@@ -5387,11 +5637,20 @@
       <c r="M4" t="s">
         <v>1518</v>
       </c>
-      <c r="V4" t="s">
+      <c r="P4" t="s">
         <v>384</v>
       </c>
+      <c r="Q4" t="s">
+        <v>1542</v>
+      </c>
+      <c r="R4" t="s">
+        <v>1617</v>
+      </c>
+      <c r="T4" s="1">
+        <v>46227</v>
+      </c>
       <c r="W4" t="s">
-        <v>1610</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="5" spans="1:23">
@@ -5435,13 +5694,13 @@
         <v>1519</v>
       </c>
       <c r="U5" t="s">
-        <v>1579</v>
+        <v>1662</v>
       </c>
       <c r="V5" t="s">
-        <v>1606</v>
+        <v>1689</v>
       </c>
       <c r="W5" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="6" spans="1:23">
@@ -5485,10 +5744,10 @@
         <v>1519</v>
       </c>
       <c r="U6" t="s">
-        <v>1580</v>
+        <v>1663</v>
       </c>
       <c r="W6" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="7" spans="1:23">
@@ -5532,10 +5791,10 @@
         <v>1519</v>
       </c>
       <c r="U7" t="s">
-        <v>1580</v>
+        <v>1663</v>
       </c>
       <c r="W7" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="8" spans="1:23">
@@ -5579,10 +5838,10 @@
         <v>1519</v>
       </c>
       <c r="U8" t="s">
-        <v>1580</v>
+        <v>1663</v>
       </c>
       <c r="W8" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="9" spans="1:23">
@@ -5626,10 +5885,10 @@
         <v>1519</v>
       </c>
       <c r="U9" t="s">
-        <v>1580</v>
+        <v>1663</v>
       </c>
       <c r="W9" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="10" spans="1:23">
@@ -5673,10 +5932,10 @@
         <v>1519</v>
       </c>
       <c r="U10" t="s">
-        <v>1580</v>
+        <v>1663</v>
       </c>
       <c r="W10" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="11" spans="1:23">
@@ -5720,10 +5979,10 @@
         <v>1519</v>
       </c>
       <c r="U11" t="s">
-        <v>1580</v>
+        <v>1663</v>
       </c>
       <c r="W11" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="12" spans="1:23">
@@ -5767,7 +6026,7 @@
         <v>1519</v>
       </c>
       <c r="W12" t="s">
-        <v>1611</v>
+        <v>1693</v>
       </c>
     </row>
     <row r="13" spans="1:23">
@@ -5810,11 +6069,20 @@
       <c r="M13" t="s">
         <v>1519</v>
       </c>
-      <c r="V13" t="s">
+      <c r="P13" t="s">
         <v>393</v>
       </c>
+      <c r="Q13" t="s">
+        <v>1543</v>
+      </c>
+      <c r="R13" t="s">
+        <v>1618</v>
+      </c>
+      <c r="T13" s="1">
+        <v>46080</v>
+      </c>
       <c r="W13" t="s">
-        <v>1610</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="14" spans="1:23">
@@ -5857,11 +6125,20 @@
       <c r="M14" t="s">
         <v>1518</v>
       </c>
-      <c r="V14" t="s">
+      <c r="P14" t="s">
         <v>394</v>
       </c>
+      <c r="Q14" t="s">
+        <v>1544</v>
+      </c>
+      <c r="R14" t="s">
+        <v>1619</v>
+      </c>
+      <c r="T14" s="1">
+        <v>45938</v>
+      </c>
       <c r="W14" t="s">
-        <v>1610</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="15" spans="1:23">
@@ -5904,11 +6181,20 @@
       <c r="M15" t="s">
         <v>1518</v>
       </c>
-      <c r="V15" t="s">
+      <c r="P15" t="s">
         <v>394</v>
       </c>
+      <c r="Q15" t="s">
+        <v>1544</v>
+      </c>
+      <c r="R15" t="s">
+        <v>1619</v>
+      </c>
+      <c r="T15" s="1">
+        <v>45938</v>
+      </c>
       <c r="W15" t="s">
-        <v>1610</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="16" spans="1:23">
@@ -5952,7 +6238,7 @@
         <v>1520</v>
       </c>
       <c r="W16" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="17" spans="1:23">
@@ -5996,7 +6282,7 @@
         <v>1520</v>
       </c>
       <c r="W17" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="18" spans="1:23">
@@ -6043,19 +6329,19 @@
         <v>398</v>
       </c>
       <c r="Q18" t="s">
-        <v>1540</v>
+        <v>1545</v>
       </c>
       <c r="R18" t="s">
-        <v>1560</v>
+        <v>1620</v>
       </c>
       <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
-        <v>1581</v>
+        <v>1664</v>
       </c>
       <c r="W18" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="19" spans="1:23">
@@ -6099,7 +6385,7 @@
         <v>1518</v>
       </c>
       <c r="W19" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="20" spans="1:23">
@@ -6143,7 +6429,7 @@
         <v>1518</v>
       </c>
       <c r="W20" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="21" spans="1:23">
@@ -6190,19 +6476,19 @@
         <v>561</v>
       </c>
       <c r="Q21" t="s">
-        <v>1541</v>
+        <v>1546</v>
       </c>
       <c r="R21" t="s">
-        <v>1561</v>
+        <v>1619</v>
       </c>
       <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
-        <v>1582</v>
+        <v>1665</v>
       </c>
       <c r="W21" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="22" spans="1:23">
@@ -6249,19 +6535,19 @@
         <v>401</v>
       </c>
       <c r="Q22" t="s">
-        <v>1542</v>
+        <v>1547</v>
       </c>
       <c r="R22" t="s">
-        <v>1562</v>
+        <v>1621</v>
       </c>
       <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
-        <v>1583</v>
+        <v>1666</v>
       </c>
       <c r="W22" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="23" spans="1:23">
@@ -6308,19 +6594,19 @@
         <v>402</v>
       </c>
       <c r="Q23" t="s">
-        <v>1543</v>
+        <v>1548</v>
       </c>
       <c r="R23" t="s">
-        <v>1563</v>
+        <v>1622</v>
       </c>
       <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
-        <v>1584</v>
+        <v>1667</v>
       </c>
       <c r="W23" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="24" spans="1:23">
@@ -6364,7 +6650,7 @@
         <v>1521</v>
       </c>
       <c r="W24" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="25" spans="1:23">
@@ -6408,7 +6694,7 @@
         <v>1517</v>
       </c>
       <c r="W25" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="26" spans="1:23">
@@ -6448,11 +6734,20 @@
       <c r="M26" t="s">
         <v>1518</v>
       </c>
-      <c r="V26" t="s">
+      <c r="P26" t="s">
         <v>405</v>
       </c>
+      <c r="Q26" t="s">
+        <v>1549</v>
+      </c>
+      <c r="R26" t="s">
+        <v>1623</v>
+      </c>
+      <c r="T26" s="1">
+        <v>46185</v>
+      </c>
       <c r="W26" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="27" spans="1:23">
@@ -6496,19 +6791,19 @@
         <v>1538</v>
       </c>
       <c r="Q27" t="s">
-        <v>1544</v>
+        <v>1550</v>
       </c>
       <c r="R27" t="s">
-        <v>1564</v>
+        <v>1624</v>
       </c>
       <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
-        <v>1585</v>
+        <v>1668</v>
       </c>
       <c r="W27" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="28" spans="1:23">
@@ -6552,7 +6847,7 @@
         <v>1517</v>
       </c>
       <c r="W28" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="29" spans="1:23">
@@ -6596,7 +6891,7 @@
         <v>1520</v>
       </c>
       <c r="W29" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="30" spans="1:23">
@@ -6640,7 +6935,7 @@
         <v>1517</v>
       </c>
       <c r="W30" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="31" spans="1:23">
@@ -6687,19 +6982,19 @@
         <v>524</v>
       </c>
       <c r="Q31" t="s">
-        <v>1545</v>
+        <v>1551</v>
       </c>
       <c r="R31" t="s">
-        <v>1565</v>
+        <v>1625</v>
       </c>
       <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
-        <v>1586</v>
+        <v>1669</v>
       </c>
       <c r="W31" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="32" spans="1:23">
@@ -6743,7 +7038,7 @@
         <v>1519</v>
       </c>
       <c r="W32" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="33" spans="1:23">
@@ -6790,19 +7085,19 @@
         <v>412</v>
       </c>
       <c r="Q33" t="s">
-        <v>1546</v>
+        <v>1552</v>
       </c>
       <c r="R33" t="s">
-        <v>1566</v>
+        <v>1626</v>
       </c>
       <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
-        <v>1587</v>
+        <v>1670</v>
       </c>
       <c r="W33" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="34" spans="1:23">
@@ -6846,7 +7141,7 @@
         <v>1520</v>
       </c>
       <c r="W34" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="35" spans="1:23">
@@ -6893,19 +7188,19 @@
         <v>414</v>
       </c>
       <c r="Q35" t="s">
-        <v>1547</v>
+        <v>1553</v>
       </c>
       <c r="R35" t="s">
-        <v>1567</v>
+        <v>1627</v>
       </c>
       <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
-        <v>1588</v>
+        <v>1671</v>
       </c>
       <c r="W35" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="36" spans="1:23">
@@ -6952,19 +7247,19 @@
         <v>415</v>
       </c>
       <c r="Q36" t="s">
-        <v>1548</v>
+        <v>1554</v>
       </c>
       <c r="R36" t="s">
-        <v>1567</v>
+        <v>1627</v>
       </c>
       <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
-        <v>1588</v>
+        <v>1671</v>
       </c>
       <c r="W36" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="37" spans="1:23">
@@ -7011,19 +7306,19 @@
         <v>416</v>
       </c>
       <c r="Q37" t="s">
-        <v>1549</v>
+        <v>1555</v>
       </c>
       <c r="R37" t="s">
-        <v>1567</v>
+        <v>1627</v>
       </c>
       <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
-        <v>1588</v>
+        <v>1671</v>
       </c>
       <c r="W37" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="38" spans="1:23">
@@ -7070,19 +7365,19 @@
         <v>417</v>
       </c>
       <c r="Q38" t="s">
-        <v>1550</v>
+        <v>1556</v>
       </c>
       <c r="R38" t="s">
-        <v>1567</v>
+        <v>1627</v>
       </c>
       <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
-        <v>1588</v>
+        <v>1671</v>
       </c>
       <c r="W38" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="39" spans="1:23">
@@ -7129,19 +7424,19 @@
         <v>418</v>
       </c>
       <c r="Q39" t="s">
-        <v>1547</v>
+        <v>1553</v>
       </c>
       <c r="R39" t="s">
-        <v>1567</v>
+        <v>1627</v>
       </c>
       <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
-        <v>1588</v>
+        <v>1671</v>
       </c>
       <c r="W39" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="40" spans="1:23">
@@ -7188,19 +7483,19 @@
         <v>419</v>
       </c>
       <c r="Q40" t="s">
-        <v>1551</v>
+        <v>1557</v>
       </c>
       <c r="R40" t="s">
-        <v>1568</v>
+        <v>1628</v>
       </c>
       <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
-        <v>1589</v>
+        <v>1672</v>
       </c>
       <c r="W40" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="41" spans="1:23">
@@ -7243,11 +7538,20 @@
       <c r="M41" t="s">
         <v>1520</v>
       </c>
-      <c r="V41" t="s">
+      <c r="P41" t="s">
         <v>394</v>
       </c>
+      <c r="Q41" t="s">
+        <v>1544</v>
+      </c>
+      <c r="R41" t="s">
+        <v>1619</v>
+      </c>
+      <c r="T41" s="1">
+        <v>45938</v>
+      </c>
       <c r="W41" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="42" spans="1:23">
@@ -7294,19 +7598,19 @@
         <v>418</v>
       </c>
       <c r="Q42" t="s">
-        <v>1547</v>
+        <v>1553</v>
       </c>
       <c r="R42" t="s">
-        <v>1567</v>
+        <v>1627</v>
       </c>
       <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
-        <v>1590</v>
+        <v>1673</v>
       </c>
       <c r="W42" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="43" spans="1:23">
@@ -7350,7 +7654,7 @@
         <v>1520</v>
       </c>
       <c r="W43" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="44" spans="1:23">
@@ -7397,19 +7701,19 @@
         <v>605</v>
       </c>
       <c r="Q44" t="s">
-        <v>1552</v>
+        <v>1558</v>
       </c>
       <c r="R44" t="s">
-        <v>1569</v>
+        <v>1629</v>
       </c>
       <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
-        <v>1591</v>
+        <v>1674</v>
       </c>
       <c r="W44" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="45" spans="1:23">
@@ -7452,11 +7756,20 @@
       <c r="M45" t="s">
         <v>1517</v>
       </c>
-      <c r="V45" t="s">
+      <c r="P45" t="s">
         <v>422</v>
       </c>
+      <c r="Q45" t="s">
+        <v>1559</v>
+      </c>
+      <c r="R45" t="s">
+        <v>1630</v>
+      </c>
+      <c r="T45" s="1">
+        <v>46112</v>
+      </c>
       <c r="W45" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="46" spans="1:23">
@@ -7500,7 +7813,7 @@
         <v>1520</v>
       </c>
       <c r="W46" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="47" spans="1:23">
@@ -7547,19 +7860,19 @@
         <v>498</v>
       </c>
       <c r="Q47" t="s">
-        <v>1543</v>
+        <v>1548</v>
       </c>
       <c r="R47" t="s">
-        <v>1570</v>
+        <v>1631</v>
       </c>
       <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
-        <v>1592</v>
+        <v>1675</v>
       </c>
       <c r="W47" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="48" spans="1:23">
@@ -7603,7 +7916,7 @@
         <v>1517</v>
       </c>
       <c r="W48" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="49" spans="1:23">
@@ -7647,7 +7960,7 @@
         <v>1518</v>
       </c>
       <c r="W49" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="50" spans="1:23">
@@ -7691,7 +8004,7 @@
         <v>1518</v>
       </c>
       <c r="W50" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="51" spans="1:23">
@@ -7735,10 +8048,10 @@
         <v>1524</v>
       </c>
       <c r="U51" t="s">
-        <v>1593</v>
+        <v>1676</v>
       </c>
       <c r="W51" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="52" spans="1:23">
@@ -7782,7 +8095,7 @@
         <v>1517</v>
       </c>
       <c r="W52" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="53" spans="1:23">
@@ -7826,7 +8139,7 @@
         <v>1517</v>
       </c>
       <c r="W53" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="54" spans="1:23">
@@ -7870,7 +8183,7 @@
         <v>1518</v>
       </c>
       <c r="W54" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="55" spans="1:23">
@@ -7920,7 +8233,7 @@
         <v>1534</v>
       </c>
       <c r="W55" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="56" spans="1:23">
@@ -7970,10 +8283,10 @@
         <v>1534</v>
       </c>
       <c r="U56" t="s">
-        <v>1594</v>
+        <v>1677</v>
       </c>
       <c r="W56" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="57" spans="1:23">
@@ -8023,7 +8336,7 @@
         <v>1534</v>
       </c>
       <c r="W57" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="58" spans="1:23">
@@ -8073,7 +8386,7 @@
         <v>1535</v>
       </c>
       <c r="W58" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="59" spans="1:23">
@@ -8120,19 +8433,19 @@
         <v>436</v>
       </c>
       <c r="Q59" t="s">
-        <v>1553</v>
+        <v>1560</v>
       </c>
       <c r="R59" t="s">
-        <v>1571</v>
+        <v>1632</v>
       </c>
       <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
-        <v>1595</v>
+        <v>1678</v>
       </c>
       <c r="W59" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="60" spans="1:23">
@@ -8176,7 +8489,7 @@
         <v>1517</v>
       </c>
       <c r="W60" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="61" spans="1:23">
@@ -8220,7 +8533,7 @@
         <v>1518</v>
       </c>
       <c r="W61" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="62" spans="1:23">
@@ -8264,7 +8577,7 @@
         <v>1518</v>
       </c>
       <c r="W62" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="63" spans="1:23">
@@ -8308,7 +8621,7 @@
         <v>1518</v>
       </c>
       <c r="W63" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="64" spans="1:23">
@@ -8352,7 +8665,7 @@
         <v>1518</v>
       </c>
       <c r="W64" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="65" spans="1:23">
@@ -8396,10 +8709,10 @@
         <v>1524</v>
       </c>
       <c r="U65" t="s">
-        <v>1596</v>
+        <v>1679</v>
       </c>
       <c r="W65" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="66" spans="1:23">
@@ -8442,11 +8755,20 @@
       <c r="M66" t="s">
         <v>1518</v>
       </c>
-      <c r="V66" t="s">
+      <c r="P66" t="s">
         <v>442</v>
       </c>
+      <c r="Q66" t="s">
+        <v>1561</v>
+      </c>
+      <c r="R66" t="s">
+        <v>1633</v>
+      </c>
+      <c r="T66" s="1">
+        <v>46191</v>
+      </c>
       <c r="W66" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="67" spans="1:23">
@@ -8490,7 +8812,7 @@
         <v>1520</v>
       </c>
       <c r="W67" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="68" spans="1:23">
@@ -8543,13 +8865,13 @@
         <v>46176</v>
       </c>
       <c r="U68" t="s">
-        <v>1597</v>
+        <v>1680</v>
       </c>
       <c r="V68" t="s">
-        <v>1607</v>
+        <v>1690</v>
       </c>
       <c r="W68" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="69" spans="1:23">
@@ -8593,7 +8915,7 @@
         <v>1526</v>
       </c>
       <c r="W69" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="70" spans="1:23">
@@ -8637,7 +8959,7 @@
         <v>1526</v>
       </c>
       <c r="W70" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="71" spans="1:23">
@@ -8681,7 +9003,7 @@
         <v>1524</v>
       </c>
       <c r="W71" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="72" spans="1:23">
@@ -8725,7 +9047,7 @@
         <v>1520</v>
       </c>
       <c r="W72" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="73" spans="1:23">
@@ -8769,7 +9091,7 @@
         <v>1518</v>
       </c>
       <c r="W73" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="74" spans="1:23">
@@ -8813,7 +9135,7 @@
         <v>1518</v>
       </c>
       <c r="W74" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="75" spans="1:23">
@@ -8857,7 +9179,7 @@
         <v>1517</v>
       </c>
       <c r="W75" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="76" spans="1:23">
@@ -8900,11 +9222,20 @@
       <c r="M76" t="s">
         <v>1518</v>
       </c>
-      <c r="V76" t="s">
+      <c r="P76" t="s">
         <v>452</v>
       </c>
+      <c r="Q76" t="s">
+        <v>1562</v>
+      </c>
+      <c r="R76" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T76" s="1">
+        <v>46230</v>
+      </c>
       <c r="W76" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="77" spans="1:23">
@@ -8947,11 +9278,20 @@
       <c r="M77" t="s">
         <v>1518</v>
       </c>
-      <c r="V77" t="s">
+      <c r="P77" t="s">
         <v>453</v>
       </c>
+      <c r="Q77" t="s">
+        <v>1563</v>
+      </c>
+      <c r="R77" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T77" s="1">
+        <v>46230</v>
+      </c>
       <c r="W77" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="78" spans="1:23">
@@ -8994,11 +9334,20 @@
       <c r="M78" t="s">
         <v>1518</v>
       </c>
-      <c r="V78" t="s">
+      <c r="P78" t="s">
         <v>454</v>
       </c>
+      <c r="Q78" t="s">
+        <v>1564</v>
+      </c>
+      <c r="R78" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T78" s="1">
+        <v>46230</v>
+      </c>
       <c r="W78" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="79" spans="1:23">
@@ -9041,11 +9390,20 @@
       <c r="M79" t="s">
         <v>1518</v>
       </c>
-      <c r="V79" t="s">
+      <c r="P79" t="s">
         <v>455</v>
       </c>
+      <c r="Q79" t="s">
+        <v>1565</v>
+      </c>
+      <c r="R79" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T79" s="1">
+        <v>46230</v>
+      </c>
       <c r="W79" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="80" spans="1:23">
@@ -9089,7 +9447,7 @@
         <v>1518</v>
       </c>
       <c r="W80" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="81" spans="1:23">
@@ -9133,7 +9491,7 @@
         <v>1517</v>
       </c>
       <c r="W81" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="82" spans="1:23">
@@ -9177,7 +9535,7 @@
         <v>1527</v>
       </c>
       <c r="W82" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="83" spans="1:23">
@@ -9221,7 +9579,7 @@
         <v>1518</v>
       </c>
       <c r="W83" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="84" spans="1:23">
@@ -9265,7 +9623,7 @@
         <v>1518</v>
       </c>
       <c r="W84" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="85" spans="1:23">
@@ -9308,11 +9666,20 @@
       <c r="M85" t="s">
         <v>1523</v>
       </c>
-      <c r="V85" t="s">
+      <c r="P85" t="s">
         <v>461</v>
       </c>
+      <c r="Q85" t="s">
+        <v>1566</v>
+      </c>
+      <c r="R85" t="s">
+        <v>1635</v>
+      </c>
+      <c r="T85" s="1">
+        <v>45989</v>
+      </c>
       <c r="W85" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="86" spans="1:23">
@@ -9356,7 +9723,7 @@
         <v>1523</v>
       </c>
       <c r="W86" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="87" spans="1:23">
@@ -9399,11 +9766,20 @@
       <c r="M87" t="s">
         <v>1520</v>
       </c>
-      <c r="V87" t="s">
+      <c r="P87" t="s">
         <v>463</v>
       </c>
+      <c r="Q87" t="s">
+        <v>1567</v>
+      </c>
+      <c r="R87" t="s">
+        <v>1636</v>
+      </c>
+      <c r="T87" s="1">
+        <v>46001</v>
+      </c>
       <c r="W87" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="88" spans="1:23">
@@ -9447,7 +9823,7 @@
         <v>1519</v>
       </c>
       <c r="W88" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="89" spans="1:23">
@@ -9490,11 +9866,20 @@
       <c r="M89" t="s">
         <v>1520</v>
       </c>
-      <c r="V89" t="s">
+      <c r="P89" t="s">
         <v>461</v>
       </c>
+      <c r="Q89" t="s">
+        <v>1568</v>
+      </c>
+      <c r="R89" t="s">
+        <v>1637</v>
+      </c>
+      <c r="T89" s="1">
+        <v>46006</v>
+      </c>
       <c r="W89" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="90" spans="1:23">
@@ -9534,11 +9919,20 @@
       <c r="M90" t="s">
         <v>1518</v>
       </c>
-      <c r="V90" t="s">
+      <c r="P90" t="s">
         <v>464</v>
       </c>
+      <c r="Q90" t="s">
+        <v>1569</v>
+      </c>
+      <c r="R90" t="s">
+        <v>1638</v>
+      </c>
+      <c r="T90" s="1">
+        <v>46007</v>
+      </c>
       <c r="W90" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="91" spans="1:23">
@@ -9578,11 +9972,20 @@
       <c r="M91" t="s">
         <v>1526</v>
       </c>
-      <c r="V91" t="s">
+      <c r="P91" t="s">
         <v>466</v>
       </c>
+      <c r="Q91" t="s">
+        <v>1570</v>
+      </c>
+      <c r="R91" t="s">
+        <v>1622</v>
+      </c>
+      <c r="T91" s="1">
+        <v>45979</v>
+      </c>
       <c r="W91" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="92" spans="1:23">
@@ -9632,19 +10035,19 @@
         <v>466</v>
       </c>
       <c r="Q92" t="s">
-        <v>1554</v>
+        <v>1570</v>
       </c>
       <c r="R92" t="s">
-        <v>1563</v>
+        <v>1622</v>
       </c>
       <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
-        <v>1598</v>
+        <v>1681</v>
       </c>
       <c r="W92" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="93" spans="1:23">
@@ -9688,7 +10091,7 @@
         <v>1527</v>
       </c>
       <c r="W93" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="94" spans="1:23">
@@ -9729,7 +10132,7 @@
         <v>1524</v>
       </c>
       <c r="W94" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="95" spans="1:23">
@@ -9773,7 +10176,7 @@
         <v>1524</v>
       </c>
       <c r="W95" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="96" spans="1:23">
@@ -9819,11 +10222,17 @@
       <c r="O96" t="s">
         <v>1537</v>
       </c>
-      <c r="V96" t="s">
+      <c r="P96" t="s">
         <v>471</v>
       </c>
+      <c r="R96" t="s">
+        <v>1639</v>
+      </c>
+      <c r="T96" s="1">
+        <v>46030</v>
+      </c>
       <c r="W96" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="97" spans="1:23">
@@ -9870,16 +10279,16 @@
         <v>471</v>
       </c>
       <c r="R97" t="s">
-        <v>1572</v>
+        <v>1639</v>
       </c>
       <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
-        <v>1599</v>
+        <v>1682</v>
       </c>
       <c r="W97" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="98" spans="1:23">
@@ -9922,11 +10331,20 @@
       <c r="M98" t="s">
         <v>1517</v>
       </c>
-      <c r="V98" t="s">
+      <c r="P98" t="s">
         <v>473</v>
       </c>
+      <c r="Q98" t="s">
+        <v>1571</v>
+      </c>
+      <c r="R98" t="s">
+        <v>1640</v>
+      </c>
+      <c r="T98" s="1">
+        <v>46050</v>
+      </c>
       <c r="W98" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="99" spans="1:23">
@@ -9969,11 +10387,20 @@
       <c r="M99" t="s">
         <v>1520</v>
       </c>
-      <c r="V99" t="s">
+      <c r="P99" t="s">
         <v>474</v>
       </c>
+      <c r="Q99" t="s">
+        <v>1572</v>
+      </c>
+      <c r="R99" t="s">
+        <v>1641</v>
+      </c>
+      <c r="T99" s="1">
+        <v>45869</v>
+      </c>
       <c r="W99" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="100" spans="1:23">
@@ -10017,7 +10444,7 @@
         <v>1519</v>
       </c>
       <c r="W100" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="101" spans="1:23">
@@ -10058,7 +10485,7 @@
         <v>1520</v>
       </c>
       <c r="W101" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="102" spans="1:23">
@@ -10099,7 +10526,7 @@
         <v>1526</v>
       </c>
       <c r="W102" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="103" spans="1:23">
@@ -10140,7 +10567,7 @@
         <v>1526</v>
       </c>
       <c r="W103" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="104" spans="1:23">
@@ -10181,7 +10608,7 @@
         <v>1519</v>
       </c>
       <c r="W104" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="105" spans="1:23">
@@ -10222,7 +10649,7 @@
         <v>1517</v>
       </c>
       <c r="W105" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="106" spans="1:23">
@@ -10263,7 +10690,7 @@
         <v>1517</v>
       </c>
       <c r="W106" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="107" spans="1:23">
@@ -10304,7 +10731,7 @@
         <v>1520</v>
       </c>
       <c r="W107" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="108" spans="1:23">
@@ -10345,7 +10772,7 @@
         <v>1519</v>
       </c>
       <c r="W108" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="109" spans="1:23">
@@ -10385,11 +10812,20 @@
       <c r="M109" t="s">
         <v>1520</v>
       </c>
-      <c r="V109" t="s">
+      <c r="P109" t="s">
         <v>482</v>
       </c>
+      <c r="Q109" t="s">
+        <v>1573</v>
+      </c>
+      <c r="R109" t="s">
+        <v>1642</v>
+      </c>
+      <c r="T109" t="s">
+        <v>1661</v>
+      </c>
       <c r="W109" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="110" spans="1:23">
@@ -10433,22 +10869,19 @@
         <v>482</v>
       </c>
       <c r="Q110" t="s">
-        <v>1555</v>
+        <v>1573</v>
       </c>
       <c r="R110" t="s">
-        <v>1573</v>
-      </c>
-      <c r="T110" s="1">
+        <v>1642</v>
+      </c>
+      <c r="T110">
         <v>45805</v>
       </c>
       <c r="U110" t="s">
-        <v>1600</v>
-      </c>
-      <c r="V110" t="s">
-        <v>465</v>
+        <v>1683</v>
       </c>
       <c r="W110" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="111" spans="1:23">
@@ -10492,19 +10925,19 @@
         <v>465</v>
       </c>
       <c r="Q111" t="s">
-        <v>1556</v>
+        <v>1574</v>
       </c>
       <c r="R111" t="s">
-        <v>1574</v>
+        <v>1643</v>
       </c>
       <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
-        <v>1601</v>
+        <v>1684</v>
       </c>
       <c r="W111" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="112" spans="1:23">
@@ -10548,19 +10981,19 @@
         <v>1539</v>
       </c>
       <c r="Q112" t="s">
-        <v>1557</v>
+        <v>1575</v>
       </c>
       <c r="R112" t="s">
-        <v>1575</v>
-      </c>
-      <c r="T112" s="1">
+        <v>1644</v>
+      </c>
+      <c r="T112">
         <v>46052</v>
       </c>
       <c r="U112" t="s">
-        <v>1602</v>
+        <v>1685</v>
       </c>
       <c r="W112" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="113" spans="1:23">
@@ -10604,7 +11037,7 @@
         <v>1526</v>
       </c>
       <c r="W113" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="114" spans="1:23">
@@ -10648,7 +11081,7 @@
         <v>1524</v>
       </c>
       <c r="W114" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="115" spans="1:23">
@@ -10691,11 +11124,20 @@
       <c r="M115" t="s">
         <v>1524</v>
       </c>
-      <c r="V115" t="s">
+      <c r="P115" t="s">
         <v>488</v>
       </c>
+      <c r="Q115" t="s">
+        <v>1576</v>
+      </c>
+      <c r="R115" t="s">
+        <v>1645</v>
+      </c>
+      <c r="T115" s="1">
+        <v>46048</v>
+      </c>
       <c r="W115" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="116" spans="1:23">
@@ -10742,19 +11184,19 @@
         <v>488</v>
       </c>
       <c r="Q116" t="s">
-        <v>1558</v>
+        <v>1576</v>
       </c>
       <c r="R116" t="s">
-        <v>1576</v>
-      </c>
-      <c r="T116" s="1">
+        <v>1645</v>
+      </c>
+      <c r="T116">
         <v>46048</v>
       </c>
       <c r="U116" t="s">
-        <v>1603</v>
+        <v>1686</v>
       </c>
       <c r="W116" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="117" spans="1:23">
@@ -10798,7 +11240,7 @@
         <v>1524</v>
       </c>
       <c r="W117" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="118" spans="1:23">
@@ -10845,7 +11287,7 @@
         <v>1532</v>
       </c>
       <c r="W118" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="119" spans="1:23">
@@ -10889,7 +11331,7 @@
         <v>1517</v>
       </c>
       <c r="W119" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="120" spans="1:23">
@@ -10930,7 +11372,7 @@
         <v>1517</v>
       </c>
       <c r="W120" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="121" spans="1:23">
@@ -10973,8 +11415,11 @@
       <c r="M121" t="s">
         <v>1518</v>
       </c>
+      <c r="R121" t="s">
+        <v>1646</v>
+      </c>
       <c r="W121" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="122" spans="1:23">
@@ -11018,10 +11463,13 @@
         <v>1518</v>
       </c>
       <c r="R122" t="s">
-        <v>1577</v>
+        <v>1646</v>
+      </c>
+      <c r="V122" t="s">
+        <v>1691</v>
       </c>
       <c r="W122" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="123" spans="1:23">
@@ -11065,7 +11513,7 @@
         <v>1518</v>
       </c>
       <c r="W123" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="124" spans="1:23">
@@ -11109,7 +11557,7 @@
         <v>1518</v>
       </c>
       <c r="W124" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="125" spans="1:23">
@@ -11152,11 +11600,20 @@
       <c r="M125" t="s">
         <v>1520</v>
       </c>
-      <c r="V125" t="s">
+      <c r="P125" t="s">
         <v>497</v>
       </c>
+      <c r="Q125" t="s">
+        <v>1577</v>
+      </c>
+      <c r="R125" t="s">
+        <v>1647</v>
+      </c>
+      <c r="T125" s="1">
+        <v>45800</v>
+      </c>
       <c r="W125" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="126" spans="1:23">
@@ -11196,11 +11653,20 @@
       <c r="M126" t="s">
         <v>1527</v>
       </c>
-      <c r="V126" t="s">
+      <c r="P126" t="s">
         <v>452</v>
       </c>
+      <c r="Q126" t="s">
+        <v>1578</v>
+      </c>
+      <c r="R126" t="s">
+        <v>1648</v>
+      </c>
+      <c r="T126" s="1">
+        <v>45889</v>
+      </c>
       <c r="W126" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="127" spans="1:23">
@@ -11244,22 +11710,19 @@
         <v>452</v>
       </c>
       <c r="Q127" t="s">
-        <v>1559</v>
+        <v>1578</v>
       </c>
       <c r="R127" t="s">
-        <v>1578</v>
-      </c>
-      <c r="T127" s="1">
+        <v>1648</v>
+      </c>
+      <c r="T127">
         <v>45889</v>
       </c>
       <c r="U127" t="s">
-        <v>1604</v>
-      </c>
-      <c r="V127" t="s">
-        <v>453</v>
+        <v>1687</v>
       </c>
       <c r="W127" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="128" spans="1:23">
@@ -11300,7 +11763,7 @@
         <v>1520</v>
       </c>
       <c r="W128" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="129" spans="1:23">
@@ -11341,7 +11804,7 @@
         <v>1520</v>
       </c>
       <c r="W129" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="130" spans="1:23">
@@ -11382,7 +11845,7 @@
         <v>1520</v>
       </c>
       <c r="W130" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="131" spans="1:23">
@@ -11423,7 +11886,7 @@
         <v>1520</v>
       </c>
       <c r="W131" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="132" spans="1:23">
@@ -11467,7 +11930,7 @@
         <v>1528</v>
       </c>
       <c r="W132" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="133" spans="1:23">
@@ -11507,11 +11970,20 @@
       <c r="M133" t="s">
         <v>1517</v>
       </c>
-      <c r="V133" t="s">
+      <c r="P133" t="s">
         <v>454</v>
       </c>
+      <c r="Q133" t="s">
+        <v>1579</v>
+      </c>
+      <c r="R133" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T133" s="1">
+        <v>46230</v>
+      </c>
       <c r="W133" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="134" spans="1:23">
@@ -11551,11 +12023,20 @@
       <c r="M134" t="s">
         <v>1527</v>
       </c>
-      <c r="V134" t="s">
+      <c r="P134" t="s">
         <v>455</v>
       </c>
+      <c r="Q134" t="s">
+        <v>1580</v>
+      </c>
+      <c r="R134" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T134" s="1">
+        <v>46230</v>
+      </c>
       <c r="W134" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="135" spans="1:23">
@@ -11596,7 +12077,7 @@
         <v>1527</v>
       </c>
       <c r="W135" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="136" spans="1:23">
@@ -11637,7 +12118,7 @@
         <v>1527</v>
       </c>
       <c r="W136" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="137" spans="1:23">
@@ -11678,7 +12159,7 @@
         <v>1518</v>
       </c>
       <c r="W137" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="138" spans="1:23">
@@ -11719,7 +12200,7 @@
         <v>1518</v>
       </c>
       <c r="W138" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="139" spans="1:23">
@@ -11763,10 +12244,10 @@
         <v>1533</v>
       </c>
       <c r="U139" t="s">
-        <v>1605</v>
+        <v>1688</v>
       </c>
       <c r="W139" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="140" spans="1:23">
@@ -11807,7 +12288,7 @@
         <v>1519</v>
       </c>
       <c r="W140" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="141" spans="1:23">
@@ -11848,7 +12329,7 @@
         <v>1519</v>
       </c>
       <c r="W141" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="142" spans="1:23">
@@ -11889,7 +12370,7 @@
         <v>1519</v>
       </c>
       <c r="W142" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="143" spans="1:23">
@@ -11932,11 +12413,20 @@
       <c r="M143" t="s">
         <v>1519</v>
       </c>
-      <c r="V143" t="s">
+      <c r="P143" t="s">
         <v>454</v>
       </c>
+      <c r="Q143" t="s">
+        <v>1581</v>
+      </c>
+      <c r="R143" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T143" s="1">
+        <v>46230</v>
+      </c>
       <c r="W143" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="144" spans="1:23">
@@ -11976,11 +12466,20 @@
       <c r="M144" t="s">
         <v>1520</v>
       </c>
-      <c r="V144" t="s">
+      <c r="P144" t="s">
         <v>455</v>
       </c>
+      <c r="Q144" t="s">
+        <v>1582</v>
+      </c>
+      <c r="R144" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T144" s="1">
+        <v>46230</v>
+      </c>
       <c r="W144" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="145" spans="1:23">
@@ -12020,11 +12519,20 @@
       <c r="M145" t="s">
         <v>1524</v>
       </c>
-      <c r="V145" t="s">
+      <c r="P145" t="s">
         <v>510</v>
       </c>
+      <c r="Q145" t="s">
+        <v>1583</v>
+      </c>
+      <c r="R145" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T145" s="1">
+        <v>46230</v>
+      </c>
       <c r="W145" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="146" spans="1:23">
@@ -12064,11 +12572,20 @@
       <c r="M146" t="s">
         <v>1524</v>
       </c>
-      <c r="V146" t="s">
+      <c r="P146" t="s">
         <v>482</v>
       </c>
+      <c r="Q146" t="s">
+        <v>1584</v>
+      </c>
+      <c r="R146" t="s">
+        <v>1642</v>
+      </c>
+      <c r="T146" s="1">
+        <v>45805</v>
+      </c>
       <c r="W146" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="147" spans="1:23">
@@ -12108,11 +12625,20 @@
       <c r="M147" t="s">
         <v>1524</v>
       </c>
-      <c r="V147" t="s">
+      <c r="P147" t="s">
         <v>483</v>
       </c>
+      <c r="Q147" t="s">
+        <v>1585</v>
+      </c>
+      <c r="R147" t="s">
+        <v>1649</v>
+      </c>
+      <c r="T147" s="1">
+        <v>45971</v>
+      </c>
       <c r="W147" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="148" spans="1:23">
@@ -12153,7 +12679,7 @@
         <v>1520</v>
       </c>
       <c r="W148" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="149" spans="1:23">
@@ -12193,11 +12719,20 @@
       <c r="M149" t="s">
         <v>1520</v>
       </c>
-      <c r="V149" t="s">
+      <c r="P149" t="s">
         <v>454</v>
       </c>
+      <c r="Q149" t="s">
+        <v>1586</v>
+      </c>
+      <c r="R149" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T149" s="1">
+        <v>46230</v>
+      </c>
       <c r="W149" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="150" spans="1:23">
@@ -12237,11 +12772,20 @@
       <c r="M150" t="s">
         <v>1519</v>
       </c>
-      <c r="V150" t="s">
+      <c r="P150" t="s">
         <v>455</v>
       </c>
+      <c r="Q150" t="s">
+        <v>1587</v>
+      </c>
+      <c r="R150" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T150" s="1">
+        <v>46230</v>
+      </c>
       <c r="W150" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="151" spans="1:23">
@@ -12281,11 +12825,20 @@
       <c r="M151" t="s">
         <v>1518</v>
       </c>
-      <c r="V151" t="s">
+      <c r="P151" t="s">
         <v>512</v>
       </c>
+      <c r="Q151" t="s">
+        <v>1588</v>
+      </c>
+      <c r="R151" t="s">
+        <v>1650</v>
+      </c>
+      <c r="T151" s="1">
+        <v>46176</v>
+      </c>
       <c r="W151" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="152" spans="1:23">
@@ -12325,11 +12878,20 @@
       <c r="M152" t="s">
         <v>1518</v>
       </c>
-      <c r="V152" t="s">
+      <c r="P152" t="s">
         <v>513</v>
       </c>
+      <c r="Q152" t="s">
+        <v>1589</v>
+      </c>
+      <c r="R152" t="s">
+        <v>1651</v>
+      </c>
+      <c r="T152" s="1">
+        <v>45769</v>
+      </c>
       <c r="W152" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="153" spans="1:23">
@@ -12373,13 +12935,13 @@
         <v>46176</v>
       </c>
       <c r="U153" t="s">
-        <v>1597</v>
+        <v>1680</v>
       </c>
       <c r="V153" t="s">
-        <v>1607</v>
+        <v>1690</v>
       </c>
       <c r="W153" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="154" spans="1:23">
@@ -12420,7 +12982,7 @@
         <v>1523</v>
       </c>
       <c r="W154" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="155" spans="1:23">
@@ -12461,7 +13023,7 @@
         <v>1523</v>
       </c>
       <c r="W155" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="156" spans="1:23">
@@ -12502,7 +13064,7 @@
         <v>1523</v>
       </c>
       <c r="W156" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="157" spans="1:23">
@@ -12543,7 +13105,7 @@
         <v>1519</v>
       </c>
       <c r="W157" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="158" spans="1:23">
@@ -12584,7 +13146,7 @@
         <v>1518</v>
       </c>
       <c r="W158" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="159" spans="1:23">
@@ -12625,7 +13187,7 @@
         <v>1518</v>
       </c>
       <c r="W159" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="160" spans="1:23">
@@ -12666,7 +13228,7 @@
         <v>1518</v>
       </c>
       <c r="W160" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="161" spans="1:23">
@@ -12707,7 +13269,7 @@
         <v>1518</v>
       </c>
       <c r="W161" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="162" spans="1:23">
@@ -12747,11 +13309,20 @@
       <c r="M162" t="s">
         <v>1519</v>
       </c>
-      <c r="V162" t="s">
+      <c r="P162" t="s">
         <v>461</v>
       </c>
+      <c r="Q162" t="s">
+        <v>1590</v>
+      </c>
+      <c r="R162" t="s">
+        <v>1637</v>
+      </c>
+      <c r="T162" s="1">
+        <v>46006</v>
+      </c>
       <c r="W162" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="163" spans="1:23">
@@ -12791,11 +13362,20 @@
       <c r="M163" t="s">
         <v>1518</v>
       </c>
-      <c r="V163" t="s">
+      <c r="P163" t="s">
         <v>520</v>
       </c>
+      <c r="Q163" t="s">
+        <v>1591</v>
+      </c>
+      <c r="R163" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T163" s="1">
+        <v>46230</v>
+      </c>
       <c r="W163" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="164" spans="1:23">
@@ -12835,8 +13415,11 @@
       <c r="M164" t="s">
         <v>1518</v>
       </c>
+      <c r="Q164" t="s">
+        <v>1592</v>
+      </c>
       <c r="W164" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="165" spans="1:23">
@@ -12877,7 +13460,7 @@
         <v>1518</v>
       </c>
       <c r="W165" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="166" spans="1:23">
@@ -12917,11 +13500,20 @@
       <c r="M166" t="s">
         <v>1518</v>
       </c>
-      <c r="V166" t="s">
+      <c r="P166" t="s">
         <v>522</v>
       </c>
+      <c r="Q166" t="s">
+        <v>1593</v>
+      </c>
+      <c r="R166" t="s">
+        <v>1652</v>
+      </c>
+      <c r="T166" s="1">
+        <v>45817</v>
+      </c>
       <c r="W166" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="167" spans="1:23">
@@ -12962,7 +13554,7 @@
         <v>1518</v>
       </c>
       <c r="W167" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="168" spans="1:23">
@@ -13006,7 +13598,7 @@
         <v>1528</v>
       </c>
       <c r="W168" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="169" spans="1:23">
@@ -13050,7 +13642,7 @@
         <v>1528</v>
       </c>
       <c r="W169" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="170" spans="1:23">
@@ -13091,7 +13683,7 @@
         <v>1528</v>
       </c>
       <c r="W170" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="171" spans="1:23">
@@ -13132,7 +13724,7 @@
         <v>1528</v>
       </c>
       <c r="W171" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="172" spans="1:23">
@@ -13173,7 +13765,7 @@
         <v>1528</v>
       </c>
       <c r="W172" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="173" spans="1:23">
@@ -13214,7 +13806,7 @@
         <v>1528</v>
       </c>
       <c r="W173" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="174" spans="1:23">
@@ -13255,7 +13847,7 @@
         <v>1528</v>
       </c>
       <c r="W174" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="175" spans="1:23">
@@ -13296,7 +13888,7 @@
         <v>1528</v>
       </c>
       <c r="W175" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="176" spans="1:23">
@@ -13337,7 +13929,7 @@
         <v>1528</v>
       </c>
       <c r="W176" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="177" spans="1:23">
@@ -13378,7 +13970,7 @@
         <v>1528</v>
       </c>
       <c r="W177" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="178" spans="1:23">
@@ -13418,11 +14010,20 @@
       <c r="M178" t="s">
         <v>1528</v>
       </c>
-      <c r="V178" t="s">
+      <c r="P178" t="s">
         <v>512</v>
       </c>
+      <c r="Q178" t="s">
+        <v>1594</v>
+      </c>
+      <c r="R178" t="s">
+        <v>1650</v>
+      </c>
+      <c r="T178" s="1">
+        <v>46176</v>
+      </c>
       <c r="W178" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="179" spans="1:23">
@@ -13466,13 +14067,13 @@
         <v>46176</v>
       </c>
       <c r="U179" t="s">
-        <v>1597</v>
+        <v>1680</v>
       </c>
       <c r="V179" t="s">
-        <v>1607</v>
+        <v>1690</v>
       </c>
       <c r="W179" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="180" spans="1:23">
@@ -13513,7 +14114,7 @@
         <v>1518</v>
       </c>
       <c r="W180" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="181" spans="1:23">
@@ -13553,11 +14154,20 @@
       <c r="M181" t="s">
         <v>1518</v>
       </c>
-      <c r="V181" t="s">
+      <c r="P181" t="s">
         <v>533</v>
       </c>
+      <c r="Q181" t="s">
+        <v>1595</v>
+      </c>
+      <c r="R181" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T181" s="1">
+        <v>46230</v>
+      </c>
       <c r="W181" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="182" spans="1:23">
@@ -13598,7 +14208,7 @@
         <v>1518</v>
       </c>
       <c r="W182" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="183" spans="1:23">
@@ -13639,7 +14249,7 @@
         <v>1518</v>
       </c>
       <c r="W183" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="184" spans="1:23">
@@ -13680,7 +14290,7 @@
         <v>1520</v>
       </c>
       <c r="W184" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="185" spans="1:23">
@@ -13721,7 +14331,7 @@
         <v>1520</v>
       </c>
       <c r="W185" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="186" spans="1:23">
@@ -13762,7 +14372,7 @@
         <v>1520</v>
       </c>
       <c r="W186" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="187" spans="1:23">
@@ -13803,7 +14413,7 @@
         <v>1528</v>
       </c>
       <c r="W187" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="188" spans="1:23">
@@ -13844,7 +14454,7 @@
         <v>1528</v>
       </c>
       <c r="W188" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="189" spans="1:23">
@@ -13885,7 +14495,7 @@
         <v>1528</v>
       </c>
       <c r="W189" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="190" spans="1:23">
@@ -13926,7 +14536,7 @@
         <v>1528</v>
       </c>
       <c r="W190" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="191" spans="1:23">
@@ -13967,7 +14577,7 @@
         <v>1528</v>
       </c>
       <c r="W191" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="192" spans="1:23">
@@ -14008,7 +14618,7 @@
         <v>1528</v>
       </c>
       <c r="W192" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="193" spans="1:23">
@@ -14049,7 +14659,7 @@
         <v>1528</v>
       </c>
       <c r="W193" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="194" spans="1:23">
@@ -14090,7 +14700,7 @@
         <v>1528</v>
       </c>
       <c r="W194" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="195" spans="1:23">
@@ -14130,11 +14740,20 @@
       <c r="M195" t="s">
         <v>1517</v>
       </c>
-      <c r="V195" t="s">
+      <c r="P195" t="s">
         <v>465</v>
       </c>
+      <c r="Q195" t="s">
+        <v>1596</v>
+      </c>
+      <c r="R195" t="s">
+        <v>1643</v>
+      </c>
+      <c r="T195" s="1">
+        <v>45959</v>
+      </c>
       <c r="W195" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="196" spans="1:23">
@@ -14177,11 +14796,20 @@
       <c r="M196" t="s">
         <v>1523</v>
       </c>
-      <c r="V196" t="s">
+      <c r="P196" t="s">
         <v>483</v>
       </c>
+      <c r="Q196" t="s">
+        <v>1597</v>
+      </c>
+      <c r="R196" t="s">
+        <v>1649</v>
+      </c>
+      <c r="T196" s="1">
+        <v>45971</v>
+      </c>
       <c r="W196" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="197" spans="1:23">
@@ -14225,7 +14853,7 @@
         <v>1520</v>
       </c>
       <c r="W197" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="198" spans="1:23">
@@ -14266,7 +14894,7 @@
         <v>1519</v>
       </c>
       <c r="W198" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="199" spans="1:23">
@@ -14307,7 +14935,7 @@
         <v>1519</v>
       </c>
       <c r="W199" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="200" spans="1:23">
@@ -14348,7 +14976,7 @@
         <v>1518</v>
       </c>
       <c r="W200" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="201" spans="1:23">
@@ -14389,7 +15017,7 @@
         <v>1526</v>
       </c>
       <c r="W201" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="202" spans="1:23">
@@ -14429,11 +15057,20 @@
       <c r="M202" t="s">
         <v>1526</v>
       </c>
-      <c r="V202" t="s">
+      <c r="P202" t="s">
         <v>520</v>
       </c>
+      <c r="Q202" t="s">
+        <v>1598</v>
+      </c>
+      <c r="R202" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T202" s="1">
+        <v>46230</v>
+      </c>
       <c r="W202" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="203" spans="1:23">
@@ -14473,11 +15110,20 @@
       <c r="M203" t="s">
         <v>1520</v>
       </c>
-      <c r="V203" t="s">
+      <c r="P203" t="s">
         <v>549</v>
       </c>
+      <c r="Q203" t="s">
+        <v>1599</v>
+      </c>
+      <c r="R203" t="s">
+        <v>1642</v>
+      </c>
+      <c r="T203" s="1">
+        <v>45805</v>
+      </c>
       <c r="W203" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="204" spans="1:23">
@@ -14517,8 +15163,17 @@
       <c r="M204" t="s">
         <v>1520</v>
       </c>
+      <c r="Q204" t="s">
+        <v>1600</v>
+      </c>
+      <c r="R204" t="s">
+        <v>1653</v>
+      </c>
+      <c r="T204" s="1">
+        <v>45889</v>
+      </c>
       <c r="W204" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="205" spans="1:23">
@@ -14561,11 +15216,20 @@
       <c r="M205" t="s">
         <v>1518</v>
       </c>
-      <c r="V205" t="s">
+      <c r="P205" t="s">
         <v>521</v>
       </c>
+      <c r="Q205" t="s">
+        <v>1601</v>
+      </c>
+      <c r="R205" t="s">
+        <v>1654</v>
+      </c>
+      <c r="T205" s="1">
+        <v>45762</v>
+      </c>
       <c r="W205" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="206" spans="1:23">
@@ -14608,11 +15272,20 @@
       <c r="M206" t="s">
         <v>1518</v>
       </c>
-      <c r="V206" t="s">
+      <c r="P206" t="s">
         <v>466</v>
       </c>
+      <c r="Q206" t="s">
+        <v>1602</v>
+      </c>
+      <c r="R206" t="s">
+        <v>1622</v>
+      </c>
+      <c r="T206" s="1">
+        <v>45979</v>
+      </c>
       <c r="W206" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="207" spans="1:23">
@@ -14653,7 +15326,7 @@
         <v>1518</v>
       </c>
       <c r="W207" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="208" spans="1:23">
@@ -14694,7 +15367,7 @@
         <v>1518</v>
       </c>
       <c r="W208" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="209" spans="1:23">
@@ -14735,7 +15408,7 @@
         <v>1518</v>
       </c>
       <c r="W209" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="210" spans="1:23">
@@ -14776,7 +15449,7 @@
         <v>1518</v>
       </c>
       <c r="W210" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="211" spans="1:23">
@@ -14817,7 +15490,7 @@
         <v>1518</v>
       </c>
       <c r="W211" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="212" spans="1:23">
@@ -14858,7 +15531,7 @@
         <v>1518</v>
       </c>
       <c r="W212" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="213" spans="1:23">
@@ -14899,7 +15572,7 @@
         <v>1518</v>
       </c>
       <c r="W213" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="214" spans="1:23">
@@ -14939,11 +15612,20 @@
       <c r="M214" t="s">
         <v>1518</v>
       </c>
-      <c r="V214" t="s">
+      <c r="P214" t="s">
         <v>401</v>
       </c>
+      <c r="Q214" t="s">
+        <v>1603</v>
+      </c>
+      <c r="R214" t="s">
+        <v>1655</v>
+      </c>
+      <c r="T214" s="1">
+        <v>46216</v>
+      </c>
       <c r="W214" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="215" spans="1:23">
@@ -14984,7 +15666,7 @@
         <v>1517</v>
       </c>
       <c r="W215" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="216" spans="1:23">
@@ -15025,7 +15707,7 @@
         <v>1519</v>
       </c>
       <c r="W216" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="217" spans="1:23">
@@ -15066,7 +15748,7 @@
         <v>1520</v>
       </c>
       <c r="W217" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="218" spans="1:23">
@@ -15107,7 +15789,7 @@
         <v>1520</v>
       </c>
       <c r="W218" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="219" spans="1:23">
@@ -15148,7 +15830,7 @@
         <v>1520</v>
       </c>
       <c r="W219" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="220" spans="1:23">
@@ -15189,7 +15871,7 @@
         <v>1524</v>
       </c>
       <c r="W220" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="221" spans="1:23">
@@ -15230,7 +15912,7 @@
         <v>1524</v>
       </c>
       <c r="W221" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="222" spans="1:23">
@@ -15271,7 +15953,7 @@
         <v>1524</v>
       </c>
       <c r="W222" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="223" spans="1:23">
@@ -15312,7 +15994,7 @@
         <v>1524</v>
       </c>
       <c r="W223" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="224" spans="1:23">
@@ -15353,7 +16035,7 @@
         <v>1524</v>
       </c>
       <c r="W224" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="225" spans="1:23">
@@ -15394,7 +16076,7 @@
         <v>1524</v>
       </c>
       <c r="W225" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="226" spans="1:23">
@@ -15435,7 +16117,7 @@
         <v>1524</v>
       </c>
       <c r="W226" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="227" spans="1:23">
@@ -15476,7 +16158,7 @@
         <v>1524</v>
       </c>
       <c r="W227" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="228" spans="1:23">
@@ -15517,7 +16199,7 @@
         <v>1524</v>
       </c>
       <c r="W228" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="229" spans="1:23">
@@ -15558,7 +16240,7 @@
         <v>1524</v>
       </c>
       <c r="W229" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="230" spans="1:23">
@@ -15599,7 +16281,7 @@
         <v>1524</v>
       </c>
       <c r="W230" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="231" spans="1:23">
@@ -15640,7 +16322,7 @@
         <v>1524</v>
       </c>
       <c r="W231" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="232" spans="1:23">
@@ -15681,7 +16363,7 @@
         <v>1524</v>
       </c>
       <c r="W232" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="233" spans="1:23">
@@ -15722,7 +16404,7 @@
         <v>1524</v>
       </c>
       <c r="W233" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="234" spans="1:23">
@@ -15763,7 +16445,7 @@
         <v>1518</v>
       </c>
       <c r="W234" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="235" spans="1:23">
@@ -15804,7 +16486,7 @@
         <v>1518</v>
       </c>
       <c r="W235" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="236" spans="1:23">
@@ -15845,7 +16527,7 @@
         <v>1518</v>
       </c>
       <c r="W236" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="237" spans="1:23">
@@ -15886,7 +16568,7 @@
         <v>1518</v>
       </c>
       <c r="W237" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="238" spans="1:23">
@@ -15927,7 +16609,7 @@
         <v>1518</v>
       </c>
       <c r="W238" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="239" spans="1:23">
@@ -15967,11 +16649,20 @@
       <c r="M239" t="s">
         <v>1518</v>
       </c>
-      <c r="V239" t="s">
+      <c r="P239" t="s">
         <v>570</v>
       </c>
+      <c r="Q239" t="s">
+        <v>1604</v>
+      </c>
+      <c r="R239" t="s">
+        <v>1649</v>
+      </c>
+      <c r="T239" s="1">
+        <v>45971</v>
+      </c>
       <c r="W239" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="240" spans="1:23">
@@ -16012,7 +16703,7 @@
         <v>1518</v>
       </c>
       <c r="W240" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="241" spans="1:23">
@@ -16053,7 +16744,7 @@
         <v>1518</v>
       </c>
       <c r="W241" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="242" spans="1:23">
@@ -16093,11 +16784,20 @@
       <c r="M242" t="s">
         <v>1518</v>
       </c>
-      <c r="V242" t="s">
+      <c r="P242" t="s">
         <v>482</v>
       </c>
+      <c r="Q242" t="s">
+        <v>1605</v>
+      </c>
+      <c r="R242" t="s">
+        <v>1642</v>
+      </c>
+      <c r="T242" s="1">
+        <v>45805</v>
+      </c>
       <c r="W242" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="243" spans="1:23">
@@ -16138,7 +16838,7 @@
         <v>1518</v>
       </c>
       <c r="W243" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="244" spans="1:23">
@@ -16179,7 +16879,7 @@
         <v>1518</v>
       </c>
       <c r="W244" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="245" spans="1:23">
@@ -16220,7 +16920,7 @@
         <v>1518</v>
       </c>
       <c r="W245" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="246" spans="1:23">
@@ -16260,11 +16960,20 @@
       <c r="M246" t="s">
         <v>1518</v>
       </c>
-      <c r="V246" t="s">
+      <c r="P246" t="s">
         <v>466</v>
       </c>
+      <c r="Q246" t="s">
+        <v>1606</v>
+      </c>
+      <c r="R246" t="s">
+        <v>1622</v>
+      </c>
+      <c r="T246" s="1">
+        <v>45979</v>
+      </c>
       <c r="W246" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="247" spans="1:23">
@@ -16305,7 +17014,7 @@
         <v>1518</v>
       </c>
       <c r="W247" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="248" spans="1:23">
@@ -16346,7 +17055,7 @@
         <v>1518</v>
       </c>
       <c r="W248" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="249" spans="1:23">
@@ -16387,7 +17096,7 @@
         <v>1526</v>
       </c>
       <c r="W249" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="250" spans="1:23">
@@ -16428,7 +17137,7 @@
         <v>1518</v>
       </c>
       <c r="W250" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="251" spans="1:23">
@@ -16469,7 +17178,7 @@
         <v>1520</v>
       </c>
       <c r="W251" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="252" spans="1:23">
@@ -16510,7 +17219,7 @@
         <v>1519</v>
       </c>
       <c r="W252" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="253" spans="1:23">
@@ -16550,11 +17259,20 @@
       <c r="M253" t="s">
         <v>1526</v>
       </c>
-      <c r="V253" t="s">
+      <c r="P253" t="s">
         <v>579</v>
       </c>
+      <c r="Q253" t="s">
+        <v>1607</v>
+      </c>
+      <c r="R253" t="s">
+        <v>1652</v>
+      </c>
+      <c r="T253" s="1">
+        <v>45817</v>
+      </c>
       <c r="W253" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="254" spans="1:23">
@@ -16598,7 +17316,7 @@
         <v>1519</v>
       </c>
       <c r="W254" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="255" spans="1:23">
@@ -16639,7 +17357,7 @@
         <v>1523</v>
       </c>
       <c r="W255" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="256" spans="1:23">
@@ -16679,8 +17397,11 @@
       <c r="M256" t="s">
         <v>1523</v>
       </c>
+      <c r="T256" s="1">
+        <v>46176</v>
+      </c>
       <c r="W256" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="257" spans="1:23">
@@ -16727,13 +17448,13 @@
         <v>46176</v>
       </c>
       <c r="U257" t="s">
-        <v>1597</v>
+        <v>1680</v>
       </c>
       <c r="V257" t="s">
-        <v>1607</v>
+        <v>1690</v>
       </c>
       <c r="W257" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="258" spans="1:23">
@@ -16776,11 +17497,20 @@
       <c r="M258" t="s">
         <v>1520</v>
       </c>
-      <c r="V258" t="s">
+      <c r="P258" t="s">
         <v>453</v>
       </c>
+      <c r="Q258" t="s">
+        <v>1608</v>
+      </c>
+      <c r="R258" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T258" s="1">
+        <v>46230</v>
+      </c>
       <c r="W258" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="259" spans="1:23">
@@ -16823,11 +17553,20 @@
       <c r="M259" t="s">
         <v>1518</v>
       </c>
-      <c r="V259" t="s">
-        <v>1608</v>
+      <c r="P259" t="s">
+        <v>1540</v>
+      </c>
+      <c r="Q259" t="s">
+        <v>1609</v>
+      </c>
+      <c r="R259" t="s">
+        <v>1650</v>
+      </c>
+      <c r="T259" s="1">
+        <v>46176</v>
       </c>
       <c r="W259" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="260" spans="1:23">
@@ -16874,13 +17613,13 @@
         <v>46176</v>
       </c>
       <c r="U260" t="s">
-        <v>1597</v>
+        <v>1680</v>
       </c>
       <c r="V260" t="s">
-        <v>1607</v>
+        <v>1690</v>
       </c>
       <c r="W260" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="261" spans="1:23">
@@ -16923,11 +17662,20 @@
       <c r="M261" t="s">
         <v>1518</v>
       </c>
-      <c r="V261" t="s">
+      <c r="P261" t="s">
         <v>584</v>
       </c>
+      <c r="Q261" t="s">
+        <v>1610</v>
+      </c>
+      <c r="R261" t="s">
+        <v>1656</v>
+      </c>
+      <c r="T261" s="1">
+        <v>46094</v>
+      </c>
       <c r="W261" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="262" spans="1:23">
@@ -16970,11 +17718,20 @@
       <c r="M262" t="s">
         <v>1518</v>
       </c>
-      <c r="V262" t="s">
+      <c r="P262" t="s">
         <v>512</v>
       </c>
+      <c r="Q262" t="s">
+        <v>1611</v>
+      </c>
+      <c r="R262" t="s">
+        <v>1650</v>
+      </c>
+      <c r="T262" s="1">
+        <v>46176</v>
+      </c>
       <c r="W262" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="263" spans="1:23">
@@ -17021,13 +17778,13 @@
         <v>46176</v>
       </c>
       <c r="U263" t="s">
-        <v>1597</v>
+        <v>1680</v>
       </c>
       <c r="V263" t="s">
-        <v>1607</v>
+        <v>1690</v>
       </c>
       <c r="W263" t="s">
-        <v>1611</v>
+        <v>1694</v>
       </c>
     </row>
     <row r="264" spans="1:23">
@@ -17071,7 +17828,7 @@
         <v>1519</v>
       </c>
       <c r="W264" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="265" spans="1:23">
@@ -17112,7 +17869,7 @@
         <v>1519</v>
       </c>
       <c r="W265" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="266" spans="1:23">
@@ -17153,7 +17910,7 @@
         <v>1519</v>
       </c>
       <c r="W266" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="267" spans="1:23">
@@ -17194,7 +17951,7 @@
         <v>1517</v>
       </c>
       <c r="W267" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="268" spans="1:23">
@@ -17238,7 +17995,7 @@
         <v>1520</v>
       </c>
       <c r="W268" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="269" spans="1:23">
@@ -17279,7 +18036,7 @@
         <v>1520</v>
       </c>
       <c r="W269" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="270" spans="1:23">
@@ -17320,7 +18077,7 @@
         <v>1520</v>
       </c>
       <c r="W270" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="271" spans="1:23">
@@ -17361,7 +18118,7 @@
         <v>1520</v>
       </c>
       <c r="W271" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="272" spans="1:23">
@@ -17401,11 +18158,20 @@
       <c r="M272" t="s">
         <v>1520</v>
       </c>
-      <c r="V272" t="s">
+      <c r="P272" t="s">
         <v>590</v>
       </c>
+      <c r="Q272" t="s">
+        <v>1612</v>
+      </c>
+      <c r="R272" t="s">
+        <v>1657</v>
+      </c>
+      <c r="T272" s="1">
+        <v>46168</v>
+      </c>
       <c r="W272" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="273" spans="1:23">
@@ -17449,7 +18215,7 @@
         <v>1520</v>
       </c>
       <c r="W273" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="274" spans="1:23">
@@ -17493,7 +18259,7 @@
         <v>1520</v>
       </c>
       <c r="W274" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="275" spans="1:23">
@@ -17534,7 +18300,7 @@
         <v>1520</v>
       </c>
       <c r="W275" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="276" spans="1:23">
@@ -17575,7 +18341,7 @@
         <v>1520</v>
       </c>
       <c r="W276" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="277" spans="1:23">
@@ -17616,7 +18382,7 @@
         <v>1520</v>
       </c>
       <c r="W277" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="278" spans="1:23">
@@ -17657,7 +18423,7 @@
         <v>1520</v>
       </c>
       <c r="W278" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="279" spans="1:23">
@@ -17698,7 +18464,7 @@
         <v>1520</v>
       </c>
       <c r="W279" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="280" spans="1:23">
@@ -17739,7 +18505,7 @@
         <v>1520</v>
       </c>
       <c r="W280" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="281" spans="1:23">
@@ -17780,7 +18546,7 @@
         <v>1520</v>
       </c>
       <c r="W281" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="282" spans="1:23">
@@ -17821,7 +18587,7 @@
         <v>1520</v>
       </c>
       <c r="W282" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="283" spans="1:23">
@@ -17862,7 +18628,7 @@
         <v>1520</v>
       </c>
       <c r="W283" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="284" spans="1:23">
@@ -17903,7 +18669,7 @@
         <v>1520</v>
       </c>
       <c r="W284" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="285" spans="1:23">
@@ -17944,7 +18710,7 @@
         <v>1520</v>
       </c>
       <c r="W285" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="286" spans="1:23">
@@ -17985,7 +18751,7 @@
         <v>1520</v>
       </c>
       <c r="W286" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="287" spans="1:23">
@@ -18026,7 +18792,7 @@
         <v>1519</v>
       </c>
       <c r="W287" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="288" spans="1:23">
@@ -18067,7 +18833,7 @@
         <v>1517</v>
       </c>
       <c r="W288" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="289" spans="1:23">
@@ -18108,7 +18874,7 @@
         <v>1520</v>
       </c>
       <c r="W289" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="290" spans="1:23">
@@ -18149,7 +18915,7 @@
         <v>1520</v>
       </c>
       <c r="W290" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="291" spans="1:23">
@@ -18190,7 +18956,7 @@
         <v>1517</v>
       </c>
       <c r="W291" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="292" spans="1:23">
@@ -18231,7 +18997,7 @@
         <v>1517</v>
       </c>
       <c r="W292" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="293" spans="1:23">
@@ -18272,7 +19038,7 @@
         <v>1519</v>
       </c>
       <c r="W293" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="294" spans="1:23">
@@ -18313,7 +19079,7 @@
         <v>1518</v>
       </c>
       <c r="W294" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="295" spans="1:23">
@@ -18353,11 +19119,20 @@
       <c r="M295" t="s">
         <v>1518</v>
       </c>
-      <c r="V295" t="s">
+      <c r="P295" t="s">
         <v>605</v>
       </c>
+      <c r="Q295" t="s">
+        <v>1613</v>
+      </c>
+      <c r="R295" t="s">
+        <v>1658</v>
+      </c>
+      <c r="T295" s="1">
+        <v>45912</v>
+      </c>
       <c r="W295" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="296" spans="1:23">
@@ -18400,11 +19175,20 @@
       <c r="M296" t="s">
         <v>1518</v>
       </c>
-      <c r="V296" t="s">
+      <c r="P296" t="s">
         <v>606</v>
       </c>
+      <c r="Q296" t="s">
+        <v>1614</v>
+      </c>
+      <c r="R296" t="s">
+        <v>1634</v>
+      </c>
+      <c r="T296" s="1">
+        <v>46230</v>
+      </c>
       <c r="W296" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="297" spans="1:23">
@@ -18448,7 +19232,7 @@
         <v>1527</v>
       </c>
       <c r="W297" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="298" spans="1:23">
@@ -18489,7 +19273,7 @@
         <v>1527</v>
       </c>
       <c r="W298" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="299" spans="1:23">
@@ -18530,7 +19314,7 @@
         <v>1527</v>
       </c>
       <c r="W299" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="300" spans="1:23">
@@ -18571,7 +19355,7 @@
         <v>1527</v>
       </c>
       <c r="W300" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="301" spans="1:23">
@@ -18612,7 +19396,7 @@
         <v>1527</v>
       </c>
       <c r="W301" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="302" spans="1:23">
@@ -18653,7 +19437,7 @@
         <v>1519</v>
       </c>
       <c r="W302" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="303" spans="1:23">
@@ -18694,7 +19478,7 @@
         <v>1519</v>
       </c>
       <c r="W303" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="304" spans="1:23">
@@ -18735,7 +19519,7 @@
         <v>1519</v>
       </c>
       <c r="W304" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="305" spans="1:23">
@@ -18776,7 +19560,7 @@
         <v>1519</v>
       </c>
       <c r="W305" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="306" spans="1:23">
@@ -18817,7 +19601,7 @@
         <v>1520</v>
       </c>
       <c r="W306" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="307" spans="1:23">
@@ -18858,7 +19642,7 @@
         <v>1520</v>
       </c>
       <c r="W307" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="308" spans="1:23">
@@ -18899,7 +19683,7 @@
         <v>1520</v>
       </c>
       <c r="W308" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="309" spans="1:23">
@@ -18940,7 +19724,7 @@
         <v>1520</v>
       </c>
       <c r="W309" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="310" spans="1:23">
@@ -18981,7 +19765,7 @@
         <v>1520</v>
       </c>
       <c r="W310" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="311" spans="1:23">
@@ -19022,7 +19806,7 @@
         <v>1520</v>
       </c>
       <c r="W311" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="312" spans="1:23">
@@ -19063,7 +19847,7 @@
         <v>1520</v>
       </c>
       <c r="W312" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="313" spans="1:23">
@@ -19104,7 +19888,7 @@
         <v>1517</v>
       </c>
       <c r="W313" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="314" spans="1:23">
@@ -19145,7 +19929,7 @@
         <v>1517</v>
       </c>
       <c r="W314" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="315" spans="1:23">
@@ -19186,7 +19970,7 @@
         <v>1518</v>
       </c>
       <c r="W315" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="316" spans="1:23">
@@ -19227,7 +20011,7 @@
         <v>1518</v>
       </c>
       <c r="W316" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="317" spans="1:23">
@@ -19268,7 +20052,7 @@
         <v>1518</v>
       </c>
       <c r="W317" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="318" spans="1:23">
@@ -19309,7 +20093,7 @@
         <v>1518</v>
       </c>
       <c r="W318" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="319" spans="1:23">
@@ -19350,7 +20134,7 @@
         <v>1518</v>
       </c>
       <c r="W319" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="320" spans="1:23">
@@ -19391,7 +20175,7 @@
         <v>1518</v>
       </c>
       <c r="W320" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="321" spans="1:23">
@@ -19431,11 +20215,20 @@
       <c r="M321" t="s">
         <v>1518</v>
       </c>
-      <c r="V321" t="s">
+      <c r="P321" t="s">
         <v>398</v>
       </c>
+      <c r="Q321" t="s">
+        <v>1545</v>
+      </c>
+      <c r="R321" t="s">
+        <v>1620</v>
+      </c>
+      <c r="T321" s="1">
+        <v>45845</v>
+      </c>
       <c r="W321" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="322" spans="1:23">
@@ -19476,7 +20269,7 @@
         <v>1518</v>
       </c>
       <c r="W322" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="323" spans="1:23">
@@ -19517,7 +20310,7 @@
         <v>1523</v>
       </c>
       <c r="W323" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="324" spans="1:23">
@@ -19558,7 +20351,7 @@
         <v>1523</v>
       </c>
       <c r="W324" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="325" spans="1:23">
@@ -19599,7 +20392,7 @@
         <v>1523</v>
       </c>
       <c r="W325" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="326" spans="1:23">
@@ -19642,11 +20435,20 @@
       <c r="M326" t="s">
         <v>1524</v>
       </c>
-      <c r="V326" t="s">
+      <c r="P326" t="s">
         <v>629</v>
       </c>
+      <c r="Q326" t="s">
+        <v>1615</v>
+      </c>
+      <c r="R326" t="s">
+        <v>1659</v>
+      </c>
+      <c r="T326" s="1">
+        <v>45848</v>
+      </c>
       <c r="W326" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="327" spans="1:23">
@@ -19690,7 +20492,7 @@
         <v>1524</v>
       </c>
       <c r="W327" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="328" spans="1:23">
@@ -19731,7 +20533,7 @@
         <v>1518</v>
       </c>
       <c r="W328" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="329" spans="1:23">
@@ -19772,7 +20574,7 @@
         <v>1518</v>
       </c>
       <c r="W329" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="330" spans="1:23">
@@ -19813,7 +20615,7 @@
         <v>1520</v>
       </c>
       <c r="W330" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="331" spans="1:23">
@@ -19854,7 +20656,7 @@
         <v>1526</v>
       </c>
       <c r="W331" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="332" spans="1:23">
@@ -19895,7 +20697,7 @@
         <v>1518</v>
       </c>
       <c r="W332" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="333" spans="1:23">
@@ -19936,7 +20738,7 @@
         <v>1518</v>
       </c>
       <c r="W333" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="334" spans="1:23">
@@ -19977,7 +20779,7 @@
         <v>1518</v>
       </c>
       <c r="W334" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="335" spans="1:23">
@@ -20018,7 +20820,7 @@
         <v>1518</v>
       </c>
       <c r="W335" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="336" spans="1:23">
@@ -20059,7 +20861,7 @@
         <v>1518</v>
       </c>
       <c r="W336" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="337" spans="1:23">
@@ -20100,7 +20902,7 @@
         <v>1518</v>
       </c>
       <c r="W337" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="338" spans="1:23">
@@ -20141,7 +20943,7 @@
         <v>1518</v>
       </c>
       <c r="W338" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="339" spans="1:23">
@@ -20182,7 +20984,7 @@
         <v>1518</v>
       </c>
       <c r="W339" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="340" spans="1:23">
@@ -20223,7 +21025,7 @@
         <v>1517</v>
       </c>
       <c r="W340" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="341" spans="1:23">
@@ -20264,7 +21066,7 @@
         <v>1518</v>
       </c>
       <c r="W341" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="342" spans="1:23">
@@ -20305,7 +21107,7 @@
         <v>1518</v>
       </c>
       <c r="W342" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="343" spans="1:23">
@@ -20346,7 +21148,7 @@
         <v>1524</v>
       </c>
       <c r="W343" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="344" spans="1:23">
@@ -20387,7 +21189,7 @@
         <v>1524</v>
       </c>
       <c r="W344" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="345" spans="1:23">
@@ -20428,7 +21230,7 @@
         <v>1524</v>
       </c>
       <c r="W345" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="346" spans="1:23">
@@ -20468,11 +21270,20 @@
       <c r="M346" t="s">
         <v>1519</v>
       </c>
-      <c r="V346" t="s">
-        <v>1609</v>
+      <c r="P346" t="s">
+        <v>1541</v>
+      </c>
+      <c r="Q346" t="s">
+        <v>1616</v>
+      </c>
+      <c r="R346" t="s">
+        <v>1660</v>
+      </c>
+      <c r="T346" s="1">
+        <v>46234</v>
       </c>
       <c r="W346" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="347" spans="1:23">
@@ -20513,7 +21324,7 @@
         <v>1517</v>
       </c>
       <c r="W347" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="348" spans="1:23">
@@ -20557,7 +21368,7 @@
         <v>1519</v>
       </c>
       <c r="W348" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="349" spans="1:23">
@@ -20598,7 +21409,7 @@
         <v>1527</v>
       </c>
       <c r="W349" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="350" spans="1:23">
@@ -20639,7 +21450,7 @@
         <v>1520</v>
       </c>
       <c r="W350" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="351" spans="1:23">
@@ -20680,7 +21491,7 @@
         <v>1520</v>
       </c>
       <c r="W351" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="352" spans="1:23">
@@ -20720,11 +21531,8 @@
       <c r="M352" t="s">
         <v>1519</v>
       </c>
-      <c r="V352" t="s">
-        <v>1610</v>
-      </c>
       <c r="W352" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="353" spans="1:23">
@@ -20764,11 +21572,8 @@
       <c r="M353" t="s">
         <v>1520</v>
       </c>
-      <c r="V353" t="s">
-        <v>1610</v>
-      </c>
       <c r="W353" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="354" spans="1:23">
@@ -20808,11 +21613,8 @@
       <c r="M354" t="s">
         <v>1519</v>
       </c>
-      <c r="V354" t="s">
-        <v>1610</v>
-      </c>
       <c r="W354" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="355" spans="1:23">
@@ -20852,11 +21654,8 @@
       <c r="M355" t="s">
         <v>1523</v>
       </c>
-      <c r="V355" t="s">
-        <v>1610</v>
-      </c>
       <c r="W355" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="356" spans="1:23">
@@ -20896,11 +21695,8 @@
       <c r="M356" t="s">
         <v>1523</v>
       </c>
-      <c r="V356" t="s">
-        <v>1610</v>
-      </c>
       <c r="W356" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="357" spans="1:23">
@@ -20940,11 +21736,8 @@
       <c r="M357" t="s">
         <v>1523</v>
       </c>
-      <c r="V357" t="s">
-        <v>1610</v>
-      </c>
       <c r="W357" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="358" spans="1:23">
@@ -20984,11 +21777,8 @@
       <c r="M358" t="s">
         <v>1523</v>
       </c>
-      <c r="V358" t="s">
-        <v>1610</v>
-      </c>
       <c r="W358" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="359" spans="1:23">
@@ -21028,11 +21818,8 @@
       <c r="M359" t="s">
         <v>1520</v>
       </c>
-      <c r="V359" t="s">
-        <v>1610</v>
-      </c>
       <c r="W359" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="360" spans="1:23">
@@ -21072,11 +21859,8 @@
       <c r="M360" t="s">
         <v>1520</v>
       </c>
-      <c r="V360" t="s">
-        <v>1610</v>
-      </c>
       <c r="W360" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
     <row r="361" spans="1:23">
@@ -21116,11 +21900,8 @@
       <c r="M361" t="s">
         <v>1518</v>
       </c>
-      <c r="V361" t="s">
-        <v>1610</v>
-      </c>
       <c r="W361" t="s">
-        <v>1611</v>
+        <v>1692</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Atualiza Empréstimos (Devoluções) — 360 itens
Sem inconsistências. Status: 326 Pendente, 26 OK, 8 Desconsiderado — mesma
contagem de OK que já havia antes (não é isso que explica o '0' visto no
site, investigando à parte).

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5109,8 +5109,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5126,7 +5134,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5134,12 +5142,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5439,73 +5465,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5540,7 +5566,7 @@
       <c r="J2" t="s">
         <v>1463</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5584,7 +5610,7 @@
       <c r="J3" t="s">
         <v>1463</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5628,7 +5654,7 @@
       <c r="J4" t="s">
         <v>1463</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5646,7 +5672,7 @@
       <c r="R4" t="s">
         <v>1617</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5684,7 +5710,7 @@
       <c r="J5" t="s">
         <v>1464</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5734,7 +5760,7 @@
       <c r="J6" t="s">
         <v>1463</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5781,7 +5807,7 @@
       <c r="J7" t="s">
         <v>1463</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5828,7 +5854,7 @@
       <c r="J8" t="s">
         <v>1463</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5875,7 +5901,7 @@
       <c r="J9" t="s">
         <v>1463</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5922,7 +5948,7 @@
       <c r="J10" t="s">
         <v>1463</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -5969,7 +5995,7 @@
       <c r="J11" t="s">
         <v>1463</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6016,7 +6042,7 @@
       <c r="J12" t="s">
         <v>1463</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6060,7 +6086,7 @@
       <c r="J13" t="s">
         <v>1463</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6078,7 +6104,7 @@
       <c r="R13" t="s">
         <v>1618</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6116,7 +6142,7 @@
       <c r="J14" t="s">
         <v>1463</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6134,7 +6160,7 @@
       <c r="R14" t="s">
         <v>1619</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6172,7 +6198,7 @@
       <c r="J15" t="s">
         <v>1463</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6190,7 +6216,7 @@
       <c r="R15" t="s">
         <v>1619</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6228,7 +6254,7 @@
       <c r="J16" t="s">
         <v>1463</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6272,7 +6298,7 @@
       <c r="J17" t="s">
         <v>1463</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6316,7 +6342,7 @@
       <c r="J18" t="s">
         <v>1463</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6334,7 +6360,7 @@
       <c r="R18" t="s">
         <v>1620</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6375,7 +6401,7 @@
       <c r="J19" t="s">
         <v>1463</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6419,7 +6445,7 @@
       <c r="J20" t="s">
         <v>1463</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6463,7 +6489,7 @@
       <c r="J21" t="s">
         <v>1463</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6481,7 +6507,7 @@
       <c r="R21" t="s">
         <v>1619</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6522,7 +6548,7 @@
       <c r="J22" t="s">
         <v>1463</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6540,7 +6566,7 @@
       <c r="R22" t="s">
         <v>1621</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6581,7 +6607,7 @@
       <c r="J23" t="s">
         <v>1463</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6599,7 +6625,7 @@
       <c r="R23" t="s">
         <v>1622</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6640,7 +6666,7 @@
       <c r="J24" t="s">
         <v>1463</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6684,7 +6710,7 @@
       <c r="J25" t="s">
         <v>1463</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6725,7 +6751,7 @@
       <c r="J26" t="s">
         <v>1465</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6743,7 +6769,7 @@
       <c r="R26" t="s">
         <v>1623</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6778,7 +6804,7 @@
       <c r="J27" t="s">
         <v>1463</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6796,7 +6822,7 @@
       <c r="R27" t="s">
         <v>1624</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6837,7 +6863,7 @@
       <c r="J28" t="s">
         <v>1463</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6881,7 +6907,7 @@
       <c r="J29" t="s">
         <v>1463</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6925,7 +6951,7 @@
       <c r="J30" t="s">
         <v>1463</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -6969,7 +6995,7 @@
       <c r="J31" t="s">
         <v>1463</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -6987,7 +7013,7 @@
       <c r="R31" t="s">
         <v>1625</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7028,7 +7054,7 @@
       <c r="J32" t="s">
         <v>1463</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7072,7 +7098,7 @@
       <c r="J33" t="s">
         <v>1463</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7090,7 +7116,7 @@
       <c r="R33" t="s">
         <v>1626</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7131,7 +7157,7 @@
       <c r="J34" t="s">
         <v>1463</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7175,7 +7201,7 @@
       <c r="J35" t="s">
         <v>1463</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7193,7 +7219,7 @@
       <c r="R35" t="s">
         <v>1627</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7234,7 +7260,7 @@
       <c r="J36" t="s">
         <v>1463</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7252,7 +7278,7 @@
       <c r="R36" t="s">
         <v>1627</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7293,7 +7319,7 @@
       <c r="J37" t="s">
         <v>1463</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7311,7 +7337,7 @@
       <c r="R37" t="s">
         <v>1627</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7352,7 +7378,7 @@
       <c r="J38" t="s">
         <v>1463</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7370,7 +7396,7 @@
       <c r="R38" t="s">
         <v>1627</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7411,7 +7437,7 @@
       <c r="J39" t="s">
         <v>1463</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7429,7 +7455,7 @@
       <c r="R39" t="s">
         <v>1627</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7470,7 +7496,7 @@
       <c r="J40" t="s">
         <v>1463</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7488,7 +7514,7 @@
       <c r="R40" t="s">
         <v>1628</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7529,7 +7555,7 @@
       <c r="J41" t="s">
         <v>1463</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7547,7 +7573,7 @@
       <c r="R41" t="s">
         <v>1619</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7585,7 +7611,7 @@
       <c r="J42" t="s">
         <v>1463</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7603,7 +7629,7 @@
       <c r="R42" t="s">
         <v>1627</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7644,7 +7670,7 @@
       <c r="J43" t="s">
         <v>1463</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7688,7 +7714,7 @@
       <c r="J44" t="s">
         <v>1463</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7706,7 +7732,7 @@
       <c r="R44" t="s">
         <v>1629</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7747,7 +7773,7 @@
       <c r="J45" t="s">
         <v>1463</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7765,7 +7791,7 @@
       <c r="R45" t="s">
         <v>1630</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7803,7 +7829,7 @@
       <c r="J46" t="s">
         <v>1463</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7847,7 +7873,7 @@
       <c r="J47" t="s">
         <v>1463</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7865,7 +7891,7 @@
       <c r="R47" t="s">
         <v>1631</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7906,7 +7932,7 @@
       <c r="J48" t="s">
         <v>1463</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -7950,7 +7976,7 @@
       <c r="J49" t="s">
         <v>1463</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -7994,7 +8020,7 @@
       <c r="J50" t="s">
         <v>1463</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8038,7 +8064,7 @@
       <c r="J51" t="s">
         <v>1463</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8085,7 +8111,7 @@
       <c r="J52" t="s">
         <v>1463</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8129,7 +8155,7 @@
       <c r="J53" t="s">
         <v>1463</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8173,7 +8199,7 @@
       <c r="J54" t="s">
         <v>1463</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8217,7 +8243,7 @@
       <c r="J55" t="s">
         <v>1463</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8267,7 +8293,7 @@
       <c r="J56" t="s">
         <v>1463</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8320,7 +8346,7 @@
       <c r="J57" t="s">
         <v>1463</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8370,7 +8396,7 @@
       <c r="J58" t="s">
         <v>1463</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8420,7 +8446,7 @@
       <c r="J59" t="s">
         <v>1463</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8438,7 +8464,7 @@
       <c r="R59" t="s">
         <v>1632</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8479,7 +8505,7 @@
       <c r="J60" t="s">
         <v>1463</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8523,7 +8549,7 @@
       <c r="J61" t="s">
         <v>1463</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8567,7 +8593,7 @@
       <c r="J62" t="s">
         <v>1463</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8611,7 +8637,7 @@
       <c r="J63" t="s">
         <v>1463</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8655,7 +8681,7 @@
       <c r="J64" t="s">
         <v>1463</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8699,7 +8725,7 @@
       <c r="J65" t="s">
         <v>1463</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8746,7 +8772,7 @@
       <c r="J66" t="s">
         <v>1463</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8764,7 +8790,7 @@
       <c r="R66" t="s">
         <v>1633</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8802,7 +8828,7 @@
       <c r="J67" t="s">
         <v>1463</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8846,7 +8872,7 @@
       <c r="J68" t="s">
         <v>1463</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8861,7 +8887,7 @@
       <c r="O68" t="s">
         <v>1536</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8905,7 +8931,7 @@
       <c r="J69" t="s">
         <v>1465</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -8949,7 +8975,7 @@
       <c r="J70" t="s">
         <v>1463</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -8993,7 +9019,7 @@
       <c r="J71" t="s">
         <v>1463</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9037,7 +9063,7 @@
       <c r="J72" t="s">
         <v>1463</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9081,7 +9107,7 @@
       <c r="J73" t="s">
         <v>1463</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9125,7 +9151,7 @@
       <c r="J74" t="s">
         <v>1463</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9169,7 +9195,7 @@
       <c r="J75" t="s">
         <v>1463</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9213,7 +9239,7 @@
       <c r="J76" t="s">
         <v>1463</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9231,7 +9257,7 @@
       <c r="R76" t="s">
         <v>1634</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9269,7 +9295,7 @@
       <c r="J77" t="s">
         <v>1463</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9287,7 +9313,7 @@
       <c r="R77" t="s">
         <v>1634</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9325,7 +9351,7 @@
       <c r="J78" t="s">
         <v>1463</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9343,7 +9369,7 @@
       <c r="R78" t="s">
         <v>1634</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9381,7 +9407,7 @@
       <c r="J79" t="s">
         <v>1463</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9399,7 +9425,7 @@
       <c r="R79" t="s">
         <v>1634</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9437,7 +9463,7 @@
       <c r="J80" t="s">
         <v>1463</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9481,7 +9507,7 @@
       <c r="J81" t="s">
         <v>1463</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9525,7 +9551,7 @@
       <c r="J82" t="s">
         <v>1463</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9569,7 +9595,7 @@
       <c r="J83" t="s">
         <v>1463</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9613,7 +9639,7 @@
       <c r="J84" t="s">
         <v>1463</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9657,7 +9683,7 @@
       <c r="J85" t="s">
         <v>1463</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9675,7 +9701,7 @@
       <c r="R85" t="s">
         <v>1635</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9713,7 +9739,7 @@
       <c r="J86" t="s">
         <v>1463</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9757,7 +9783,7 @@
       <c r="J87" t="s">
         <v>1463</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9775,7 +9801,7 @@
       <c r="R87" t="s">
         <v>1636</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9813,7 +9839,7 @@
       <c r="J88" t="s">
         <v>1463</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9857,7 +9883,7 @@
       <c r="J89" t="s">
         <v>1463</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9875,7 +9901,7 @@
       <c r="R89" t="s">
         <v>1637</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -9910,7 +9936,7 @@
       <c r="J90" t="s">
         <v>1463</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -9928,7 +9954,7 @@
       <c r="R90" t="s">
         <v>1638</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -9963,7 +9989,7 @@
       <c r="J91" t="s">
         <v>1463</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -9981,7 +10007,7 @@
       <c r="R91" t="s">
         <v>1622</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10019,7 +10045,7 @@
       <c r="J92" t="s">
         <v>1463</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10040,7 +10066,7 @@
       <c r="R92" t="s">
         <v>1622</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10081,7 +10107,7 @@
       <c r="J93" t="s">
         <v>1463</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10122,7 +10148,7 @@
       <c r="J94" t="s">
         <v>1463</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10166,7 +10192,7 @@
       <c r="J95" t="s">
         <v>1463</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10210,7 +10236,7 @@
       <c r="J96" t="s">
         <v>1463</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10228,7 +10254,7 @@
       <c r="R96" t="s">
         <v>1639</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10266,7 +10292,7 @@
       <c r="J97" t="s">
         <v>1463</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10281,7 +10307,7 @@
       <c r="R97" t="s">
         <v>1639</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10322,7 +10348,7 @@
       <c r="J98" t="s">
         <v>1463</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10340,7 +10366,7 @@
       <c r="R98" t="s">
         <v>1640</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10378,7 +10404,7 @@
       <c r="J99" t="s">
         <v>1463</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10396,7 +10422,7 @@
       <c r="R99" t="s">
         <v>1641</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10434,7 +10460,7 @@
       <c r="J100" t="s">
         <v>1463</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10475,7 +10501,7 @@
       <c r="J101" t="s">
         <v>1463</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10516,7 +10542,7 @@
       <c r="J102" t="s">
         <v>1463</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10557,7 +10583,7 @@
       <c r="J103" t="s">
         <v>1463</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10598,7 +10624,7 @@
       <c r="J104" t="s">
         <v>1463</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10639,7 +10665,7 @@
       <c r="J105" t="s">
         <v>1463</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10680,7 +10706,7 @@
       <c r="J106" t="s">
         <v>1463</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10721,7 +10747,7 @@
       <c r="J107" t="s">
         <v>1463</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10762,7 +10788,7 @@
       <c r="J108" t="s">
         <v>1463</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10803,7 +10829,7 @@
       <c r="J109" t="s">
         <v>1463</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10856,7 +10882,7 @@
       <c r="J110" t="s">
         <v>1463</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10912,7 +10938,7 @@
       <c r="J111" t="s">
         <v>1463</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -10930,7 +10956,7 @@
       <c r="R111" t="s">
         <v>1643</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -10968,7 +10994,7 @@
       <c r="J112" t="s">
         <v>1463</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11027,7 +11053,7 @@
       <c r="J113" t="s">
         <v>1463</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11071,7 +11097,7 @@
       <c r="J114" t="s">
         <v>1463</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11115,7 +11141,7 @@
       <c r="J115" t="s">
         <v>1463</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11133,7 +11159,7 @@
       <c r="R115" t="s">
         <v>1645</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11171,7 +11197,7 @@
       <c r="J116" t="s">
         <v>1463</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11230,7 +11256,7 @@
       <c r="J117" t="s">
         <v>1463</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11274,7 +11300,7 @@
       <c r="J118" t="s">
         <v>1463</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11321,7 +11347,7 @@
       <c r="J119" t="s">
         <v>1463</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11362,7 +11388,7 @@
       <c r="J120" t="s">
         <v>1463</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11406,7 +11432,7 @@
       <c r="J121" t="s">
         <v>1463</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11453,7 +11479,7 @@
       <c r="J122" t="s">
         <v>1463</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11503,7 +11529,7 @@
       <c r="J123" t="s">
         <v>1463</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11547,7 +11573,7 @@
       <c r="J124" t="s">
         <v>1463</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11591,7 +11617,7 @@
       <c r="J125" t="s">
         <v>1463</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11609,7 +11635,7 @@
       <c r="R125" t="s">
         <v>1647</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11644,7 +11670,7 @@
       <c r="J126" t="s">
         <v>1463</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11662,7 +11688,7 @@
       <c r="R126" t="s">
         <v>1648</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11697,7 +11723,7 @@
       <c r="J127" t="s">
         <v>1463</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11753,7 +11779,7 @@
       <c r="J128" t="s">
         <v>1463</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11794,7 +11820,7 @@
       <c r="J129" t="s">
         <v>1463</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11835,7 +11861,7 @@
       <c r="J130" t="s">
         <v>1463</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11876,7 +11902,7 @@
       <c r="J131" t="s">
         <v>1463</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11920,7 +11946,7 @@
       <c r="J132" t="s">
         <v>1463</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -11961,7 +11987,7 @@
       <c r="J133" t="s">
         <v>1463</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -11979,7 +12005,7 @@
       <c r="R133" t="s">
         <v>1634</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12014,7 +12040,7 @@
       <c r="J134" t="s">
         <v>1463</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12032,7 +12058,7 @@
       <c r="R134" t="s">
         <v>1634</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12067,7 +12093,7 @@
       <c r="J135" t="s">
         <v>1463</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12108,7 +12134,7 @@
       <c r="J136" t="s">
         <v>1463</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12149,7 +12175,7 @@
       <c r="J137" t="s">
         <v>1463</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12190,7 +12216,7 @@
       <c r="J138" t="s">
         <v>1463</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12231,7 +12257,7 @@
       <c r="J139" t="s">
         <v>1463</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12278,7 +12304,7 @@
       <c r="J140" t="s">
         <v>1463</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12319,7 +12345,7 @@
       <c r="J141" t="s">
         <v>1463</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12360,7 +12386,7 @@
       <c r="J142" t="s">
         <v>1463</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12404,7 +12430,7 @@
       <c r="J143" t="s">
         <v>1463</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12422,7 +12448,7 @@
       <c r="R143" t="s">
         <v>1634</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12457,7 +12483,7 @@
       <c r="J144" t="s">
         <v>1463</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12475,7 +12501,7 @@
       <c r="R144" t="s">
         <v>1634</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12510,7 +12536,7 @@
       <c r="J145" t="s">
         <v>1463</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12528,7 +12554,7 @@
       <c r="R145" t="s">
         <v>1634</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12563,7 +12589,7 @@
       <c r="J146" t="s">
         <v>1463</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12581,7 +12607,7 @@
       <c r="R146" t="s">
         <v>1642</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12616,7 +12642,7 @@
       <c r="J147" t="s">
         <v>1463</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12634,7 +12660,7 @@
       <c r="R147" t="s">
         <v>1649</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12669,7 +12695,7 @@
       <c r="J148" t="s">
         <v>1463</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12710,7 +12736,7 @@
       <c r="J149" t="s">
         <v>1463</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12728,7 +12754,7 @@
       <c r="R149" t="s">
         <v>1634</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12763,7 +12789,7 @@
       <c r="J150" t="s">
         <v>1463</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12781,7 +12807,7 @@
       <c r="R150" t="s">
         <v>1634</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12816,7 +12842,7 @@
       <c r="J151" t="s">
         <v>1463</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12834,7 +12860,7 @@
       <c r="R151" t="s">
         <v>1650</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12869,7 +12895,7 @@
       <c r="J152" t="s">
         <v>1463</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12887,7 +12913,7 @@
       <c r="R152" t="s">
         <v>1651</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -12922,7 +12948,7 @@
       <c r="J153" t="s">
         <v>1463</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -12931,7 +12957,7 @@
       <c r="M153" t="s">
         <v>1527</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -12972,7 +12998,7 @@
       <c r="J154" t="s">
         <v>1463</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13013,7 +13039,7 @@
       <c r="J155" t="s">
         <v>1463</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13054,7 +13080,7 @@
       <c r="J156" t="s">
         <v>1463</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13095,7 +13121,7 @@
       <c r="J157" t="s">
         <v>1463</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13136,7 +13162,7 @@
       <c r="J158" t="s">
         <v>1463</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13177,7 +13203,7 @@
       <c r="J159" t="s">
         <v>1463</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13218,7 +13244,7 @@
       <c r="J160" t="s">
         <v>1463</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13259,7 +13285,7 @@
       <c r="J161" t="s">
         <v>1463</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13300,7 +13326,7 @@
       <c r="J162" t="s">
         <v>1463</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13318,7 +13344,7 @@
       <c r="R162" t="s">
         <v>1637</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13353,7 +13379,7 @@
       <c r="J163" t="s">
         <v>1463</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13371,7 +13397,7 @@
       <c r="R163" t="s">
         <v>1634</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13406,7 +13432,7 @@
       <c r="J164" t="s">
         <v>1463</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13450,7 +13476,7 @@
       <c r="J165" t="s">
         <v>1463</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13491,7 +13517,7 @@
       <c r="J166" t="s">
         <v>1463</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13509,7 +13535,7 @@
       <c r="R166" t="s">
         <v>1652</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13544,7 +13570,7 @@
       <c r="J167" t="s">
         <v>1463</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13588,7 +13614,7 @@
       <c r="J168" t="s">
         <v>1463</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13632,7 +13658,7 @@
       <c r="J169" t="s">
         <v>1463</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13673,7 +13699,7 @@
       <c r="J170" t="s">
         <v>1463</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13714,7 +13740,7 @@
       <c r="J171" t="s">
         <v>1463</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13755,7 +13781,7 @@
       <c r="J172" t="s">
         <v>1463</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13796,7 +13822,7 @@
       <c r="J173" t="s">
         <v>1463</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13837,7 +13863,7 @@
       <c r="J174" t="s">
         <v>1463</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13878,7 +13904,7 @@
       <c r="J175" t="s">
         <v>1463</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -13919,7 +13945,7 @@
       <c r="J176" t="s">
         <v>1463</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -13960,7 +13986,7 @@
       <c r="J177" t="s">
         <v>1463</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14001,7 +14027,7 @@
       <c r="J178" t="s">
         <v>1463</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14019,7 +14045,7 @@
       <c r="R178" t="s">
         <v>1650</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14054,7 +14080,7 @@
       <c r="J179" t="s">
         <v>1463</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14063,7 +14089,7 @@
       <c r="M179" t="s">
         <v>1524</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14104,7 +14130,7 @@
       <c r="J180" t="s">
         <v>1463</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14145,7 +14171,7 @@
       <c r="J181" t="s">
         <v>1463</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14163,7 +14189,7 @@
       <c r="R181" t="s">
         <v>1634</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14198,7 +14224,7 @@
       <c r="J182" t="s">
         <v>1463</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14239,7 +14265,7 @@
       <c r="J183" t="s">
         <v>1463</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14280,7 +14306,7 @@
       <c r="J184" t="s">
         <v>1463</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14321,7 +14347,7 @@
       <c r="J185" t="s">
         <v>1463</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14362,7 +14388,7 @@
       <c r="J186" t="s">
         <v>1463</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14403,7 +14429,7 @@
       <c r="J187" t="s">
         <v>1463</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14444,7 +14470,7 @@
       <c r="J188" t="s">
         <v>1463</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14485,7 +14511,7 @@
       <c r="J189" t="s">
         <v>1463</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14526,7 +14552,7 @@
       <c r="J190" t="s">
         <v>1463</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14567,7 +14593,7 @@
       <c r="J191" t="s">
         <v>1463</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14608,7 +14634,7 @@
       <c r="J192" t="s">
         <v>1463</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14649,7 +14675,7 @@
       <c r="J193" t="s">
         <v>1463</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14690,7 +14716,7 @@
       <c r="J194" t="s">
         <v>1463</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14731,7 +14757,7 @@
       <c r="J195" t="s">
         <v>1463</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14749,7 +14775,7 @@
       <c r="R195" t="s">
         <v>1643</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14787,7 +14813,7 @@
       <c r="J196" t="s">
         <v>1463</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14805,7 +14831,7 @@
       <c r="R196" t="s">
         <v>1649</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14843,7 +14869,7 @@
       <c r="J197" t="s">
         <v>1463</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14884,7 +14910,7 @@
       <c r="J198" t="s">
         <v>1465</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -14925,7 +14951,7 @@
       <c r="J199" t="s">
         <v>1464</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -14966,7 +14992,7 @@
       <c r="J200" t="s">
         <v>1463</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15007,7 +15033,7 @@
       <c r="J201" t="s">
         <v>1463</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15048,7 +15074,7 @@
       <c r="J202" t="s">
         <v>1463</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15066,7 +15092,7 @@
       <c r="R202" t="s">
         <v>1634</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15101,7 +15127,7 @@
       <c r="J203" t="s">
         <v>1463</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15119,7 +15145,7 @@
       <c r="R203" t="s">
         <v>1642</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15154,7 +15180,7 @@
       <c r="J204" t="s">
         <v>1463</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15169,7 +15195,7 @@
       <c r="R204" t="s">
         <v>1653</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15207,7 +15233,7 @@
       <c r="J205" t="s">
         <v>1463</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15225,7 +15251,7 @@
       <c r="R205" t="s">
         <v>1654</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15263,7 +15289,7 @@
       <c r="J206" t="s">
         <v>1463</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15281,7 +15307,7 @@
       <c r="R206" t="s">
         <v>1622</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15316,7 +15342,7 @@
       <c r="J207" t="s">
         <v>1463</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15357,7 +15383,7 @@
       <c r="J208" t="s">
         <v>1463</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15398,7 +15424,7 @@
       <c r="J209" t="s">
         <v>1463</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15439,7 +15465,7 @@
       <c r="J210" t="s">
         <v>1463</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15480,7 +15506,7 @@
       <c r="J211" t="s">
         <v>1463</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15521,7 +15547,7 @@
       <c r="J212" t="s">
         <v>1463</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15562,7 +15588,7 @@
       <c r="J213" t="s">
         <v>1463</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15603,7 +15629,7 @@
       <c r="J214" t="s">
         <v>1463</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15621,7 +15647,7 @@
       <c r="R214" t="s">
         <v>1655</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15656,7 +15682,7 @@
       <c r="J215" t="s">
         <v>1463</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15697,7 +15723,7 @@
       <c r="J216" t="s">
         <v>1463</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15738,7 +15764,7 @@
       <c r="J217" t="s">
         <v>1463</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15779,7 +15805,7 @@
       <c r="J218" t="s">
         <v>1463</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15820,7 +15846,7 @@
       <c r="J219" t="s">
         <v>1463</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15861,7 +15887,7 @@
       <c r="J220" t="s">
         <v>1463</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -15902,7 +15928,7 @@
       <c r="J221" t="s">
         <v>1463</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -15943,7 +15969,7 @@
       <c r="J222" t="s">
         <v>1463</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -15984,7 +16010,7 @@
       <c r="J223" t="s">
         <v>1463</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16025,7 +16051,7 @@
       <c r="J224" t="s">
         <v>1463</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16066,7 +16092,7 @@
       <c r="J225" t="s">
         <v>1463</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16107,7 +16133,7 @@
       <c r="J226" t="s">
         <v>1463</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16148,7 +16174,7 @@
       <c r="J227" t="s">
         <v>1463</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16189,7 +16215,7 @@
       <c r="J228" t="s">
         <v>1463</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16230,7 +16256,7 @@
       <c r="J229" t="s">
         <v>1463</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16271,7 +16297,7 @@
       <c r="J230" t="s">
         <v>1463</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16312,7 +16338,7 @@
       <c r="J231" t="s">
         <v>1463</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16353,7 +16379,7 @@
       <c r="J232" t="s">
         <v>1463</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16394,7 +16420,7 @@
       <c r="J233" t="s">
         <v>1463</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16435,7 +16461,7 @@
       <c r="J234" t="s">
         <v>1463</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16476,7 +16502,7 @@
       <c r="J235" t="s">
         <v>1463</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16517,7 +16543,7 @@
       <c r="J236" t="s">
         <v>1463</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16558,7 +16584,7 @@
       <c r="J237" t="s">
         <v>1463</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16599,7 +16625,7 @@
       <c r="J238" t="s">
         <v>1463</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16640,7 +16666,7 @@
       <c r="J239" t="s">
         <v>1463</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16658,7 +16684,7 @@
       <c r="R239" t="s">
         <v>1649</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16693,7 +16719,7 @@
       <c r="J240" t="s">
         <v>1463</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16734,7 +16760,7 @@
       <c r="J241" t="s">
         <v>1463</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16775,7 +16801,7 @@
       <c r="J242" t="s">
         <v>1463</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16793,7 +16819,7 @@
       <c r="R242" t="s">
         <v>1642</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16828,7 +16854,7 @@
       <c r="J243" t="s">
         <v>1463</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16869,7 +16895,7 @@
       <c r="J244" t="s">
         <v>1463</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -16910,7 +16936,7 @@
       <c r="J245" t="s">
         <v>1463</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -16951,7 +16977,7 @@
       <c r="J246" t="s">
         <v>1463</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -16969,7 +16995,7 @@
       <c r="R246" t="s">
         <v>1622</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17004,7 +17030,7 @@
       <c r="J247" t="s">
         <v>1463</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17045,7 +17071,7 @@
       <c r="J248" t="s">
         <v>1463</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17086,7 +17112,7 @@
       <c r="J249" t="s">
         <v>1463</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17127,7 +17153,7 @@
       <c r="J250" t="s">
         <v>1463</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17168,7 +17194,7 @@
       <c r="J251" t="s">
         <v>1463</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17209,7 +17235,7 @@
       <c r="J252" t="s">
         <v>1463</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17250,7 +17276,7 @@
       <c r="J253" t="s">
         <v>1463</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17268,7 +17294,7 @@
       <c r="R253" t="s">
         <v>1652</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17306,7 +17332,7 @@
       <c r="J254" t="s">
         <v>1463</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17347,7 +17373,7 @@
       <c r="J255" t="s">
         <v>1463</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17388,7 +17414,7 @@
       <c r="J256" t="s">
         <v>1463</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17397,7 +17423,7 @@
       <c r="M256" t="s">
         <v>1523</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17435,7 +17461,7 @@
       <c r="J257" t="s">
         <v>1463</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17444,7 +17470,7 @@
       <c r="M257" t="s">
         <v>1524</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17488,7 +17514,7 @@
       <c r="J258" t="s">
         <v>1463</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17506,7 +17532,7 @@
       <c r="R258" t="s">
         <v>1634</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17544,7 +17570,7 @@
       <c r="J259" t="s">
         <v>1463</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17562,7 +17588,7 @@
       <c r="R259" t="s">
         <v>1650</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17600,7 +17626,7 @@
       <c r="J260" t="s">
         <v>1463</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17609,7 +17635,7 @@
       <c r="M260" t="s">
         <v>1518</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17653,7 +17679,7 @@
       <c r="J261" t="s">
         <v>1463</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17671,7 +17697,7 @@
       <c r="R261" t="s">
         <v>1656</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17709,7 +17735,7 @@
       <c r="J262" t="s">
         <v>1463</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17727,7 +17753,7 @@
       <c r="R262" t="s">
         <v>1650</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17765,7 +17791,7 @@
       <c r="J263" t="s">
         <v>1463</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17774,7 +17800,7 @@
       <c r="M263" t="s">
         <v>1518</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17818,7 +17844,7 @@
       <c r="J264" t="s">
         <v>1463</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17859,7 +17885,7 @@
       <c r="J265" t="s">
         <v>1463</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17900,7 +17926,7 @@
       <c r="J266" t="s">
         <v>1463</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -17941,7 +17967,7 @@
       <c r="J267" t="s">
         <v>1463</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -17985,7 +18011,7 @@
       <c r="J268" t="s">
         <v>1463</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18026,7 +18052,7 @@
       <c r="J269" t="s">
         <v>1463</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18067,7 +18093,7 @@
       <c r="J270" t="s">
         <v>1463</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18108,7 +18134,7 @@
       <c r="J271" t="s">
         <v>1463</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18149,7 +18175,7 @@
       <c r="J272" t="s">
         <v>1463</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18167,7 +18193,7 @@
       <c r="R272" t="s">
         <v>1657</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18205,7 +18231,7 @@
       <c r="J273" t="s">
         <v>1463</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18249,7 +18275,7 @@
       <c r="J274" t="s">
         <v>1463</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18290,7 +18316,7 @@
       <c r="J275" t="s">
         <v>1463</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18331,7 +18357,7 @@
       <c r="J276" t="s">
         <v>1463</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18372,7 +18398,7 @@
       <c r="J277" t="s">
         <v>1463</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18413,7 +18439,7 @@
       <c r="J278" t="s">
         <v>1463</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18454,7 +18480,7 @@
       <c r="J279" t="s">
         <v>1463</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18495,7 +18521,7 @@
       <c r="J280" t="s">
         <v>1463</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18536,7 +18562,7 @@
       <c r="J281" t="s">
         <v>1463</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18577,7 +18603,7 @@
       <c r="J282" t="s">
         <v>1463</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18618,7 +18644,7 @@
       <c r="J283" t="s">
         <v>1463</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18659,7 +18685,7 @@
       <c r="J284" t="s">
         <v>1463</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18700,7 +18726,7 @@
       <c r="J285" t="s">
         <v>1463</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18741,7 +18767,7 @@
       <c r="J286" t="s">
         <v>1463</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18782,7 +18808,7 @@
       <c r="J287" t="s">
         <v>1463</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18823,7 +18849,7 @@
       <c r="J288" t="s">
         <v>1463</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18864,7 +18890,7 @@
       <c r="J289" t="s">
         <v>1463</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -18905,7 +18931,7 @@
       <c r="J290" t="s">
         <v>1463</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -18946,7 +18972,7 @@
       <c r="J291" t="s">
         <v>1463</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -18987,7 +19013,7 @@
       <c r="J292" t="s">
         <v>1463</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19028,7 +19054,7 @@
       <c r="J293" t="s">
         <v>1463</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19069,7 +19095,7 @@
       <c r="J294" t="s">
         <v>1463</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19110,7 +19136,7 @@
       <c r="J295" t="s">
         <v>1463</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19128,7 +19154,7 @@
       <c r="R295" t="s">
         <v>1658</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19166,7 +19192,7 @@
       <c r="J296" t="s">
         <v>1463</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19184,7 +19210,7 @@
       <c r="R296" t="s">
         <v>1634</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19222,7 +19248,7 @@
       <c r="J297" t="s">
         <v>1463</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19263,7 +19289,7 @@
       <c r="J298" t="s">
         <v>1463</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19304,7 +19330,7 @@
       <c r="J299" t="s">
         <v>1464</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19345,7 +19371,7 @@
       <c r="J300" t="s">
         <v>1463</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19386,7 +19412,7 @@
       <c r="J301" t="s">
         <v>1463</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20224,7 +20250,7 @@
       <c r="R321" t="s">
         <v>1620</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20444,7 +20470,7 @@
       <c r="R326" t="s">
         <v>1659</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21279,7 +21305,7 @@
       <c r="R346" t="s">
         <v>1660</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (13/08/2026 13:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5109,16 +5109,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5134,7 +5126,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5142,30 +5134,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5465,73 +5439,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5566,7 +5540,7 @@
       <c r="J2" t="s">
         <v>1463</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5610,7 +5584,7 @@
       <c r="J3" t="s">
         <v>1463</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5654,7 +5628,7 @@
       <c r="J4" t="s">
         <v>1463</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5672,7 +5646,7 @@
       <c r="R4" t="s">
         <v>1617</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5710,7 +5684,7 @@
       <c r="J5" t="s">
         <v>1464</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5760,7 +5734,7 @@
       <c r="J6" t="s">
         <v>1463</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5807,7 +5781,7 @@
       <c r="J7" t="s">
         <v>1463</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5854,7 +5828,7 @@
       <c r="J8" t="s">
         <v>1463</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5901,7 +5875,7 @@
       <c r="J9" t="s">
         <v>1463</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5948,7 +5922,7 @@
       <c r="J10" t="s">
         <v>1463</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -5995,7 +5969,7 @@
       <c r="J11" t="s">
         <v>1463</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6042,7 +6016,7 @@
       <c r="J12" t="s">
         <v>1463</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6086,7 +6060,7 @@
       <c r="J13" t="s">
         <v>1463</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6104,7 +6078,7 @@
       <c r="R13" t="s">
         <v>1618</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6142,7 +6116,7 @@
       <c r="J14" t="s">
         <v>1463</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6160,7 +6134,7 @@
       <c r="R14" t="s">
         <v>1619</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6198,7 +6172,7 @@
       <c r="J15" t="s">
         <v>1463</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6216,7 +6190,7 @@
       <c r="R15" t="s">
         <v>1619</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6254,7 +6228,7 @@
       <c r="J16" t="s">
         <v>1463</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6298,7 +6272,7 @@
       <c r="J17" t="s">
         <v>1463</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6342,7 +6316,7 @@
       <c r="J18" t="s">
         <v>1463</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6360,7 +6334,7 @@
       <c r="R18" t="s">
         <v>1620</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6401,7 +6375,7 @@
       <c r="J19" t="s">
         <v>1463</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6445,7 +6419,7 @@
       <c r="J20" t="s">
         <v>1463</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6489,7 +6463,7 @@
       <c r="J21" t="s">
         <v>1463</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6507,7 +6481,7 @@
       <c r="R21" t="s">
         <v>1619</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6548,7 +6522,7 @@
       <c r="J22" t="s">
         <v>1463</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6566,7 +6540,7 @@
       <c r="R22" t="s">
         <v>1621</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6607,7 +6581,7 @@
       <c r="J23" t="s">
         <v>1463</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6625,7 +6599,7 @@
       <c r="R23" t="s">
         <v>1622</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6666,7 +6640,7 @@
       <c r="J24" t="s">
         <v>1463</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6710,7 +6684,7 @@
       <c r="J25" t="s">
         <v>1463</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6751,7 +6725,7 @@
       <c r="J26" t="s">
         <v>1465</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6769,7 +6743,7 @@
       <c r="R26" t="s">
         <v>1623</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6804,7 +6778,7 @@
       <c r="J27" t="s">
         <v>1463</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6822,7 +6796,7 @@
       <c r="R27" t="s">
         <v>1624</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6863,7 +6837,7 @@
       <c r="J28" t="s">
         <v>1463</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6907,7 +6881,7 @@
       <c r="J29" t="s">
         <v>1463</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6951,7 +6925,7 @@
       <c r="J30" t="s">
         <v>1463</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -6995,7 +6969,7 @@
       <c r="J31" t="s">
         <v>1463</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7013,7 +6987,7 @@
       <c r="R31" t="s">
         <v>1625</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7054,7 +7028,7 @@
       <c r="J32" t="s">
         <v>1463</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7098,7 +7072,7 @@
       <c r="J33" t="s">
         <v>1463</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7116,7 +7090,7 @@
       <c r="R33" t="s">
         <v>1626</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7157,7 +7131,7 @@
       <c r="J34" t="s">
         <v>1463</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7201,7 +7175,7 @@
       <c r="J35" t="s">
         <v>1463</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7219,7 +7193,7 @@
       <c r="R35" t="s">
         <v>1627</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7260,7 +7234,7 @@
       <c r="J36" t="s">
         <v>1463</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7278,7 +7252,7 @@
       <c r="R36" t="s">
         <v>1627</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7319,7 +7293,7 @@
       <c r="J37" t="s">
         <v>1463</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7337,7 +7311,7 @@
       <c r="R37" t="s">
         <v>1627</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7378,7 +7352,7 @@
       <c r="J38" t="s">
         <v>1463</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7396,7 +7370,7 @@
       <c r="R38" t="s">
         <v>1627</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7437,7 +7411,7 @@
       <c r="J39" t="s">
         <v>1463</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7455,7 +7429,7 @@
       <c r="R39" t="s">
         <v>1627</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7496,7 +7470,7 @@
       <c r="J40" t="s">
         <v>1463</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7514,7 +7488,7 @@
       <c r="R40" t="s">
         <v>1628</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7555,7 +7529,7 @@
       <c r="J41" t="s">
         <v>1463</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7573,7 +7547,7 @@
       <c r="R41" t="s">
         <v>1619</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7611,7 +7585,7 @@
       <c r="J42" t="s">
         <v>1463</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7629,7 +7603,7 @@
       <c r="R42" t="s">
         <v>1627</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7670,7 +7644,7 @@
       <c r="J43" t="s">
         <v>1463</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7714,7 +7688,7 @@
       <c r="J44" t="s">
         <v>1463</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7732,7 +7706,7 @@
       <c r="R44" t="s">
         <v>1629</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7773,7 +7747,7 @@
       <c r="J45" t="s">
         <v>1463</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7791,7 +7765,7 @@
       <c r="R45" t="s">
         <v>1630</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7829,7 +7803,7 @@
       <c r="J46" t="s">
         <v>1463</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7873,7 +7847,7 @@
       <c r="J47" t="s">
         <v>1463</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7891,7 +7865,7 @@
       <c r="R47" t="s">
         <v>1631</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7932,7 +7906,7 @@
       <c r="J48" t="s">
         <v>1463</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -7976,7 +7950,7 @@
       <c r="J49" t="s">
         <v>1463</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8020,7 +7994,7 @@
       <c r="J50" t="s">
         <v>1463</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8064,7 +8038,7 @@
       <c r="J51" t="s">
         <v>1463</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8111,7 +8085,7 @@
       <c r="J52" t="s">
         <v>1463</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8155,7 +8129,7 @@
       <c r="J53" t="s">
         <v>1463</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8199,7 +8173,7 @@
       <c r="J54" t="s">
         <v>1463</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8243,7 +8217,7 @@
       <c r="J55" t="s">
         <v>1463</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8293,7 +8267,7 @@
       <c r="J56" t="s">
         <v>1463</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8346,7 +8320,7 @@
       <c r="J57" t="s">
         <v>1463</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8396,7 +8370,7 @@
       <c r="J58" t="s">
         <v>1463</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8446,7 +8420,7 @@
       <c r="J59" t="s">
         <v>1463</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8464,7 +8438,7 @@
       <c r="R59" t="s">
         <v>1632</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8505,7 +8479,7 @@
       <c r="J60" t="s">
         <v>1463</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8549,7 +8523,7 @@
       <c r="J61" t="s">
         <v>1463</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8593,7 +8567,7 @@
       <c r="J62" t="s">
         <v>1463</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8637,7 +8611,7 @@
       <c r="J63" t="s">
         <v>1463</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8681,7 +8655,7 @@
       <c r="J64" t="s">
         <v>1463</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8725,7 +8699,7 @@
       <c r="J65" t="s">
         <v>1463</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8772,7 +8746,7 @@
       <c r="J66" t="s">
         <v>1463</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8790,7 +8764,7 @@
       <c r="R66" t="s">
         <v>1633</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8828,7 +8802,7 @@
       <c r="J67" t="s">
         <v>1463</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8872,7 +8846,7 @@
       <c r="J68" t="s">
         <v>1463</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8887,7 +8861,7 @@
       <c r="O68" t="s">
         <v>1536</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8931,7 +8905,7 @@
       <c r="J69" t="s">
         <v>1465</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -8975,7 +8949,7 @@
       <c r="J70" t="s">
         <v>1463</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9019,7 +8993,7 @@
       <c r="J71" t="s">
         <v>1463</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9063,7 +9037,7 @@
       <c r="J72" t="s">
         <v>1463</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9107,7 +9081,7 @@
       <c r="J73" t="s">
         <v>1463</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9151,7 +9125,7 @@
       <c r="J74" t="s">
         <v>1463</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9195,7 +9169,7 @@
       <c r="J75" t="s">
         <v>1463</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9239,7 +9213,7 @@
       <c r="J76" t="s">
         <v>1463</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9257,7 +9231,7 @@
       <c r="R76" t="s">
         <v>1634</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9295,7 +9269,7 @@
       <c r="J77" t="s">
         <v>1463</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9313,7 +9287,7 @@
       <c r="R77" t="s">
         <v>1634</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9351,7 +9325,7 @@
       <c r="J78" t="s">
         <v>1463</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9369,7 +9343,7 @@
       <c r="R78" t="s">
         <v>1634</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9407,7 +9381,7 @@
       <c r="J79" t="s">
         <v>1463</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9425,7 +9399,7 @@
       <c r="R79" t="s">
         <v>1634</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9463,7 +9437,7 @@
       <c r="J80" t="s">
         <v>1463</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9507,7 +9481,7 @@
       <c r="J81" t="s">
         <v>1463</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9551,7 +9525,7 @@
       <c r="J82" t="s">
         <v>1463</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9595,7 +9569,7 @@
       <c r="J83" t="s">
         <v>1463</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9639,7 +9613,7 @@
       <c r="J84" t="s">
         <v>1463</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9683,7 +9657,7 @@
       <c r="J85" t="s">
         <v>1463</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9701,7 +9675,7 @@
       <c r="R85" t="s">
         <v>1635</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9739,7 +9713,7 @@
       <c r="J86" t="s">
         <v>1463</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9783,7 +9757,7 @@
       <c r="J87" t="s">
         <v>1463</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9801,7 +9775,7 @@
       <c r="R87" t="s">
         <v>1636</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9839,7 +9813,7 @@
       <c r="J88" t="s">
         <v>1463</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9883,7 +9857,7 @@
       <c r="J89" t="s">
         <v>1463</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9901,7 +9875,7 @@
       <c r="R89" t="s">
         <v>1637</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -9936,7 +9910,7 @@
       <c r="J90" t="s">
         <v>1463</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -9954,7 +9928,7 @@
       <c r="R90" t="s">
         <v>1638</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -9989,7 +9963,7 @@
       <c r="J91" t="s">
         <v>1463</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10007,7 +9981,7 @@
       <c r="R91" t="s">
         <v>1622</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10045,7 +10019,7 @@
       <c r="J92" t="s">
         <v>1463</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10066,7 +10040,7 @@
       <c r="R92" t="s">
         <v>1622</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10107,7 +10081,7 @@
       <c r="J93" t="s">
         <v>1463</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10148,7 +10122,7 @@
       <c r="J94" t="s">
         <v>1463</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10192,7 +10166,7 @@
       <c r="J95" t="s">
         <v>1463</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10236,7 +10210,7 @@
       <c r="J96" t="s">
         <v>1463</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10254,7 +10228,7 @@
       <c r="R96" t="s">
         <v>1639</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10292,7 +10266,7 @@
       <c r="J97" t="s">
         <v>1463</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10307,7 +10281,7 @@
       <c r="R97" t="s">
         <v>1639</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10348,7 +10322,7 @@
       <c r="J98" t="s">
         <v>1463</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10366,7 +10340,7 @@
       <c r="R98" t="s">
         <v>1640</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10404,7 +10378,7 @@
       <c r="J99" t="s">
         <v>1463</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10422,7 +10396,7 @@
       <c r="R99" t="s">
         <v>1641</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10460,7 +10434,7 @@
       <c r="J100" t="s">
         <v>1463</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10501,7 +10475,7 @@
       <c r="J101" t="s">
         <v>1463</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10542,7 +10516,7 @@
       <c r="J102" t="s">
         <v>1463</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10583,7 +10557,7 @@
       <c r="J103" t="s">
         <v>1463</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10624,7 +10598,7 @@
       <c r="J104" t="s">
         <v>1463</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10665,7 +10639,7 @@
       <c r="J105" t="s">
         <v>1463</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10706,7 +10680,7 @@
       <c r="J106" t="s">
         <v>1463</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10747,7 +10721,7 @@
       <c r="J107" t="s">
         <v>1463</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10788,7 +10762,7 @@
       <c r="J108" t="s">
         <v>1463</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10829,7 +10803,7 @@
       <c r="J109" t="s">
         <v>1463</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10882,7 +10856,7 @@
       <c r="J110" t="s">
         <v>1463</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10938,7 +10912,7 @@
       <c r="J111" t="s">
         <v>1463</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -10956,7 +10930,7 @@
       <c r="R111" t="s">
         <v>1643</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -10994,7 +10968,7 @@
       <c r="J112" t="s">
         <v>1463</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11053,7 +11027,7 @@
       <c r="J113" t="s">
         <v>1463</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11097,7 +11071,7 @@
       <c r="J114" t="s">
         <v>1463</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11141,7 +11115,7 @@
       <c r="J115" t="s">
         <v>1463</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11159,7 +11133,7 @@
       <c r="R115" t="s">
         <v>1645</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11197,7 +11171,7 @@
       <c r="J116" t="s">
         <v>1463</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11256,7 +11230,7 @@
       <c r="J117" t="s">
         <v>1463</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11300,7 +11274,7 @@
       <c r="J118" t="s">
         <v>1463</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11347,7 +11321,7 @@
       <c r="J119" t="s">
         <v>1463</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11388,7 +11362,7 @@
       <c r="J120" t="s">
         <v>1463</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11432,7 +11406,7 @@
       <c r="J121" t="s">
         <v>1463</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11479,7 +11453,7 @@
       <c r="J122" t="s">
         <v>1463</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11529,7 +11503,7 @@
       <c r="J123" t="s">
         <v>1463</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11573,7 +11547,7 @@
       <c r="J124" t="s">
         <v>1463</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11617,7 +11591,7 @@
       <c r="J125" t="s">
         <v>1463</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11635,7 +11609,7 @@
       <c r="R125" t="s">
         <v>1647</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11670,7 +11644,7 @@
       <c r="J126" t="s">
         <v>1463</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11688,7 +11662,7 @@
       <c r="R126" t="s">
         <v>1648</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11723,7 +11697,7 @@
       <c r="J127" t="s">
         <v>1463</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11779,7 +11753,7 @@
       <c r="J128" t="s">
         <v>1463</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11820,7 +11794,7 @@
       <c r="J129" t="s">
         <v>1463</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11861,7 +11835,7 @@
       <c r="J130" t="s">
         <v>1463</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11902,7 +11876,7 @@
       <c r="J131" t="s">
         <v>1463</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11946,7 +11920,7 @@
       <c r="J132" t="s">
         <v>1463</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -11987,7 +11961,7 @@
       <c r="J133" t="s">
         <v>1463</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12005,7 +11979,7 @@
       <c r="R133" t="s">
         <v>1634</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12040,7 +12014,7 @@
       <c r="J134" t="s">
         <v>1463</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12058,7 +12032,7 @@
       <c r="R134" t="s">
         <v>1634</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12093,7 +12067,7 @@
       <c r="J135" t="s">
         <v>1463</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12134,7 +12108,7 @@
       <c r="J136" t="s">
         <v>1463</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12175,7 +12149,7 @@
       <c r="J137" t="s">
         <v>1463</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12216,7 +12190,7 @@
       <c r="J138" t="s">
         <v>1463</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12257,7 +12231,7 @@
       <c r="J139" t="s">
         <v>1463</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12304,7 +12278,7 @@
       <c r="J140" t="s">
         <v>1463</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12345,7 +12319,7 @@
       <c r="J141" t="s">
         <v>1463</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12386,7 +12360,7 @@
       <c r="J142" t="s">
         <v>1463</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12430,7 +12404,7 @@
       <c r="J143" t="s">
         <v>1463</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12448,7 +12422,7 @@
       <c r="R143" t="s">
         <v>1634</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12483,7 +12457,7 @@
       <c r="J144" t="s">
         <v>1463</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12501,7 +12475,7 @@
       <c r="R144" t="s">
         <v>1634</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12536,7 +12510,7 @@
       <c r="J145" t="s">
         <v>1463</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12554,7 +12528,7 @@
       <c r="R145" t="s">
         <v>1634</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12589,7 +12563,7 @@
       <c r="J146" t="s">
         <v>1463</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12607,7 +12581,7 @@
       <c r="R146" t="s">
         <v>1642</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12642,7 +12616,7 @@
       <c r="J147" t="s">
         <v>1463</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12660,7 +12634,7 @@
       <c r="R147" t="s">
         <v>1649</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12695,7 +12669,7 @@
       <c r="J148" t="s">
         <v>1463</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12736,7 +12710,7 @@
       <c r="J149" t="s">
         <v>1463</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12754,7 +12728,7 @@
       <c r="R149" t="s">
         <v>1634</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12789,7 +12763,7 @@
       <c r="J150" t="s">
         <v>1463</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12807,7 +12781,7 @@
       <c r="R150" t="s">
         <v>1634</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12842,7 +12816,7 @@
       <c r="J151" t="s">
         <v>1463</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12860,7 +12834,7 @@
       <c r="R151" t="s">
         <v>1650</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12895,7 +12869,7 @@
       <c r="J152" t="s">
         <v>1463</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12913,7 +12887,7 @@
       <c r="R152" t="s">
         <v>1651</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -12948,7 +12922,7 @@
       <c r="J153" t="s">
         <v>1463</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -12957,7 +12931,7 @@
       <c r="M153" t="s">
         <v>1527</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -12998,7 +12972,7 @@
       <c r="J154" t="s">
         <v>1463</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13039,7 +13013,7 @@
       <c r="J155" t="s">
         <v>1463</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13080,7 +13054,7 @@
       <c r="J156" t="s">
         <v>1463</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13121,7 +13095,7 @@
       <c r="J157" t="s">
         <v>1463</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13162,7 +13136,7 @@
       <c r="J158" t="s">
         <v>1463</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13203,7 +13177,7 @@
       <c r="J159" t="s">
         <v>1463</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13244,7 +13218,7 @@
       <c r="J160" t="s">
         <v>1463</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13285,7 +13259,7 @@
       <c r="J161" t="s">
         <v>1463</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13326,7 +13300,7 @@
       <c r="J162" t="s">
         <v>1463</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13344,7 +13318,7 @@
       <c r="R162" t="s">
         <v>1637</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13379,7 +13353,7 @@
       <c r="J163" t="s">
         <v>1463</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13397,7 +13371,7 @@
       <c r="R163" t="s">
         <v>1634</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13432,7 +13406,7 @@
       <c r="J164" t="s">
         <v>1463</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13476,7 +13450,7 @@
       <c r="J165" t="s">
         <v>1463</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13517,7 +13491,7 @@
       <c r="J166" t="s">
         <v>1463</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13535,7 +13509,7 @@
       <c r="R166" t="s">
         <v>1652</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13570,7 +13544,7 @@
       <c r="J167" t="s">
         <v>1463</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13614,7 +13588,7 @@
       <c r="J168" t="s">
         <v>1463</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13658,7 +13632,7 @@
       <c r="J169" t="s">
         <v>1463</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13699,7 +13673,7 @@
       <c r="J170" t="s">
         <v>1463</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13740,7 +13714,7 @@
       <c r="J171" t="s">
         <v>1463</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13781,7 +13755,7 @@
       <c r="J172" t="s">
         <v>1463</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13822,7 +13796,7 @@
       <c r="J173" t="s">
         <v>1463</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13863,7 +13837,7 @@
       <c r="J174" t="s">
         <v>1463</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13904,7 +13878,7 @@
       <c r="J175" t="s">
         <v>1463</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -13945,7 +13919,7 @@
       <c r="J176" t="s">
         <v>1463</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -13986,7 +13960,7 @@
       <c r="J177" t="s">
         <v>1463</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14027,7 +14001,7 @@
       <c r="J178" t="s">
         <v>1463</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14045,7 +14019,7 @@
       <c r="R178" t="s">
         <v>1650</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14080,7 +14054,7 @@
       <c r="J179" t="s">
         <v>1463</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14089,7 +14063,7 @@
       <c r="M179" t="s">
         <v>1524</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14130,7 +14104,7 @@
       <c r="J180" t="s">
         <v>1463</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14171,7 +14145,7 @@
       <c r="J181" t="s">
         <v>1463</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14189,7 +14163,7 @@
       <c r="R181" t="s">
         <v>1634</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14224,7 +14198,7 @@
       <c r="J182" t="s">
         <v>1463</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14265,7 +14239,7 @@
       <c r="J183" t="s">
         <v>1463</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14306,7 +14280,7 @@
       <c r="J184" t="s">
         <v>1463</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14347,7 +14321,7 @@
       <c r="J185" t="s">
         <v>1463</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14388,7 +14362,7 @@
       <c r="J186" t="s">
         <v>1463</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14429,7 +14403,7 @@
       <c r="J187" t="s">
         <v>1463</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14470,7 +14444,7 @@
       <c r="J188" t="s">
         <v>1463</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14511,7 +14485,7 @@
       <c r="J189" t="s">
         <v>1463</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14552,7 +14526,7 @@
       <c r="J190" t="s">
         <v>1463</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14593,7 +14567,7 @@
       <c r="J191" t="s">
         <v>1463</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14634,7 +14608,7 @@
       <c r="J192" t="s">
         <v>1463</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14675,7 +14649,7 @@
       <c r="J193" t="s">
         <v>1463</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14716,7 +14690,7 @@
       <c r="J194" t="s">
         <v>1463</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14757,7 +14731,7 @@
       <c r="J195" t="s">
         <v>1463</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14775,7 +14749,7 @@
       <c r="R195" t="s">
         <v>1643</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14813,7 +14787,7 @@
       <c r="J196" t="s">
         <v>1463</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14831,7 +14805,7 @@
       <c r="R196" t="s">
         <v>1649</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14869,7 +14843,7 @@
       <c r="J197" t="s">
         <v>1463</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14910,7 +14884,7 @@
       <c r="J198" t="s">
         <v>1465</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -14951,7 +14925,7 @@
       <c r="J199" t="s">
         <v>1464</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -14992,7 +14966,7 @@
       <c r="J200" t="s">
         <v>1463</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15033,7 +15007,7 @@
       <c r="J201" t="s">
         <v>1463</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15074,7 +15048,7 @@
       <c r="J202" t="s">
         <v>1463</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15092,7 +15066,7 @@
       <c r="R202" t="s">
         <v>1634</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15127,7 +15101,7 @@
       <c r="J203" t="s">
         <v>1463</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15145,7 +15119,7 @@
       <c r="R203" t="s">
         <v>1642</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15180,7 +15154,7 @@
       <c r="J204" t="s">
         <v>1463</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15195,7 +15169,7 @@
       <c r="R204" t="s">
         <v>1653</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15233,7 +15207,7 @@
       <c r="J205" t="s">
         <v>1463</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15251,7 +15225,7 @@
       <c r="R205" t="s">
         <v>1654</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15289,7 +15263,7 @@
       <c r="J206" t="s">
         <v>1463</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15307,7 +15281,7 @@
       <c r="R206" t="s">
         <v>1622</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15342,7 +15316,7 @@
       <c r="J207" t="s">
         <v>1463</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15383,7 +15357,7 @@
       <c r="J208" t="s">
         <v>1463</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15424,7 +15398,7 @@
       <c r="J209" t="s">
         <v>1463</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15465,7 +15439,7 @@
       <c r="J210" t="s">
         <v>1463</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15506,7 +15480,7 @@
       <c r="J211" t="s">
         <v>1463</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15547,7 +15521,7 @@
       <c r="J212" t="s">
         <v>1463</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15588,7 +15562,7 @@
       <c r="J213" t="s">
         <v>1463</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15629,7 +15603,7 @@
       <c r="J214" t="s">
         <v>1463</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15647,7 +15621,7 @@
       <c r="R214" t="s">
         <v>1655</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15682,7 +15656,7 @@
       <c r="J215" t="s">
         <v>1463</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15723,7 +15697,7 @@
       <c r="J216" t="s">
         <v>1463</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15764,7 +15738,7 @@
       <c r="J217" t="s">
         <v>1463</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15805,7 +15779,7 @@
       <c r="J218" t="s">
         <v>1463</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15846,7 +15820,7 @@
       <c r="J219" t="s">
         <v>1463</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15887,7 +15861,7 @@
       <c r="J220" t="s">
         <v>1463</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -15928,7 +15902,7 @@
       <c r="J221" t="s">
         <v>1463</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -15969,7 +15943,7 @@
       <c r="J222" t="s">
         <v>1463</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16010,7 +15984,7 @@
       <c r="J223" t="s">
         <v>1463</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16051,7 +16025,7 @@
       <c r="J224" t="s">
         <v>1463</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16092,7 +16066,7 @@
       <c r="J225" t="s">
         <v>1463</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16133,7 +16107,7 @@
       <c r="J226" t="s">
         <v>1463</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16174,7 +16148,7 @@
       <c r="J227" t="s">
         <v>1463</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16215,7 +16189,7 @@
       <c r="J228" t="s">
         <v>1463</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16256,7 +16230,7 @@
       <c r="J229" t="s">
         <v>1463</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16297,7 +16271,7 @@
       <c r="J230" t="s">
         <v>1463</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16338,7 +16312,7 @@
       <c r="J231" t="s">
         <v>1463</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16379,7 +16353,7 @@
       <c r="J232" t="s">
         <v>1463</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16420,7 +16394,7 @@
       <c r="J233" t="s">
         <v>1463</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16461,7 +16435,7 @@
       <c r="J234" t="s">
         <v>1463</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16502,7 +16476,7 @@
       <c r="J235" t="s">
         <v>1463</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16543,7 +16517,7 @@
       <c r="J236" t="s">
         <v>1463</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16584,7 +16558,7 @@
       <c r="J237" t="s">
         <v>1463</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16625,7 +16599,7 @@
       <c r="J238" t="s">
         <v>1463</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16666,7 +16640,7 @@
       <c r="J239" t="s">
         <v>1463</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16684,7 +16658,7 @@
       <c r="R239" t="s">
         <v>1649</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16719,7 +16693,7 @@
       <c r="J240" t="s">
         <v>1463</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16760,7 +16734,7 @@
       <c r="J241" t="s">
         <v>1463</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16801,7 +16775,7 @@
       <c r="J242" t="s">
         <v>1463</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16819,7 +16793,7 @@
       <c r="R242" t="s">
         <v>1642</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16854,7 +16828,7 @@
       <c r="J243" t="s">
         <v>1463</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16895,7 +16869,7 @@
       <c r="J244" t="s">
         <v>1463</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -16936,7 +16910,7 @@
       <c r="J245" t="s">
         <v>1463</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -16977,7 +16951,7 @@
       <c r="J246" t="s">
         <v>1463</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -16995,7 +16969,7 @@
       <c r="R246" t="s">
         <v>1622</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17030,7 +17004,7 @@
       <c r="J247" t="s">
         <v>1463</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17071,7 +17045,7 @@
       <c r="J248" t="s">
         <v>1463</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17112,7 +17086,7 @@
       <c r="J249" t="s">
         <v>1463</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17153,7 +17127,7 @@
       <c r="J250" t="s">
         <v>1463</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17194,7 +17168,7 @@
       <c r="J251" t="s">
         <v>1463</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17235,7 +17209,7 @@
       <c r="J252" t="s">
         <v>1463</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17276,7 +17250,7 @@
       <c r="J253" t="s">
         <v>1463</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17294,7 +17268,7 @@
       <c r="R253" t="s">
         <v>1652</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17332,7 +17306,7 @@
       <c r="J254" t="s">
         <v>1463</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17373,7 +17347,7 @@
       <c r="J255" t="s">
         <v>1463</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17414,7 +17388,7 @@
       <c r="J256" t="s">
         <v>1463</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17423,7 +17397,7 @@
       <c r="M256" t="s">
         <v>1523</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17461,7 +17435,7 @@
       <c r="J257" t="s">
         <v>1463</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17470,7 +17444,7 @@
       <c r="M257" t="s">
         <v>1524</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17514,7 +17488,7 @@
       <c r="J258" t="s">
         <v>1463</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17532,7 +17506,7 @@
       <c r="R258" t="s">
         <v>1634</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17570,7 +17544,7 @@
       <c r="J259" t="s">
         <v>1463</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17588,7 +17562,7 @@
       <c r="R259" t="s">
         <v>1650</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17626,7 +17600,7 @@
       <c r="J260" t="s">
         <v>1463</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17635,7 +17609,7 @@
       <c r="M260" t="s">
         <v>1518</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17679,7 +17653,7 @@
       <c r="J261" t="s">
         <v>1463</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17697,7 +17671,7 @@
       <c r="R261" t="s">
         <v>1656</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17735,7 +17709,7 @@
       <c r="J262" t="s">
         <v>1463</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17753,7 +17727,7 @@
       <c r="R262" t="s">
         <v>1650</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17791,7 +17765,7 @@
       <c r="J263" t="s">
         <v>1463</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17800,7 +17774,7 @@
       <c r="M263" t="s">
         <v>1518</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17844,7 +17818,7 @@
       <c r="J264" t="s">
         <v>1463</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17885,7 +17859,7 @@
       <c r="J265" t="s">
         <v>1463</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17926,7 +17900,7 @@
       <c r="J266" t="s">
         <v>1463</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -17967,7 +17941,7 @@
       <c r="J267" t="s">
         <v>1463</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18011,7 +17985,7 @@
       <c r="J268" t="s">
         <v>1463</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18052,7 +18026,7 @@
       <c r="J269" t="s">
         <v>1463</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18093,7 +18067,7 @@
       <c r="J270" t="s">
         <v>1463</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18134,7 +18108,7 @@
       <c r="J271" t="s">
         <v>1463</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18175,7 +18149,7 @@
       <c r="J272" t="s">
         <v>1463</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18193,7 +18167,7 @@
       <c r="R272" t="s">
         <v>1657</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18231,7 +18205,7 @@
       <c r="J273" t="s">
         <v>1463</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18275,7 +18249,7 @@
       <c r="J274" t="s">
         <v>1463</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18316,7 +18290,7 @@
       <c r="J275" t="s">
         <v>1463</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18357,7 +18331,7 @@
       <c r="J276" t="s">
         <v>1463</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18398,7 +18372,7 @@
       <c r="J277" t="s">
         <v>1463</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18439,7 +18413,7 @@
       <c r="J278" t="s">
         <v>1463</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18480,7 +18454,7 @@
       <c r="J279" t="s">
         <v>1463</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18521,7 +18495,7 @@
       <c r="J280" t="s">
         <v>1463</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18562,7 +18536,7 @@
       <c r="J281" t="s">
         <v>1463</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18603,7 +18577,7 @@
       <c r="J282" t="s">
         <v>1463</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18644,7 +18618,7 @@
       <c r="J283" t="s">
         <v>1463</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18685,7 +18659,7 @@
       <c r="J284" t="s">
         <v>1463</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18726,7 +18700,7 @@
       <c r="J285" t="s">
         <v>1463</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18767,7 +18741,7 @@
       <c r="J286" t="s">
         <v>1463</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18808,7 +18782,7 @@
       <c r="J287" t="s">
         <v>1463</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18849,7 +18823,7 @@
       <c r="J288" t="s">
         <v>1463</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18890,7 +18864,7 @@
       <c r="J289" t="s">
         <v>1463</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -18931,7 +18905,7 @@
       <c r="J290" t="s">
         <v>1463</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -18972,7 +18946,7 @@
       <c r="J291" t="s">
         <v>1463</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19013,7 +18987,7 @@
       <c r="J292" t="s">
         <v>1463</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19054,7 +19028,7 @@
       <c r="J293" t="s">
         <v>1463</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19095,7 +19069,7 @@
       <c r="J294" t="s">
         <v>1463</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19136,7 +19110,7 @@
       <c r="J295" t="s">
         <v>1463</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19154,7 +19128,7 @@
       <c r="R295" t="s">
         <v>1658</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19192,7 +19166,7 @@
       <c r="J296" t="s">
         <v>1463</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19210,7 +19184,7 @@
       <c r="R296" t="s">
         <v>1634</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19248,7 +19222,7 @@
       <c r="J297" t="s">
         <v>1463</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19289,7 +19263,7 @@
       <c r="J298" t="s">
         <v>1463</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19330,7 +19304,7 @@
       <c r="J299" t="s">
         <v>1464</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19371,7 +19345,7 @@
       <c r="J300" t="s">
         <v>1463</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19412,7 +19386,7 @@
       <c r="J301" t="s">
         <v>1463</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20250,7 +20224,7 @@
       <c r="R321" t="s">
         <v>1620</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20470,7 +20444,7 @@
       <c r="R326" t="s">
         <v>1659</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21305,7 +21279,7 @@
       <c r="R346" t="s">
         <v>1660</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (18/08/2026 12:33)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5181,8 +5181,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5198,7 +5206,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5206,12 +5214,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5511,73 +5537,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="J2" t="s">
         <v>1484</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5656,7 +5682,7 @@
       <c r="J3" t="s">
         <v>1484</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5700,7 +5726,7 @@
       <c r="J4" t="s">
         <v>1484</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5718,7 +5744,7 @@
       <c r="R4" t="s">
         <v>1641</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5756,7 +5782,7 @@
       <c r="J5" t="s">
         <v>1485</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5806,7 +5832,7 @@
       <c r="J6" t="s">
         <v>1484</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5853,7 +5879,7 @@
       <c r="J7" t="s">
         <v>1484</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5900,7 +5926,7 @@
       <c r="J8" t="s">
         <v>1484</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5947,7 +5973,7 @@
       <c r="J9" t="s">
         <v>1484</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5994,7 +6020,7 @@
       <c r="J10" t="s">
         <v>1484</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6041,7 +6067,7 @@
       <c r="J11" t="s">
         <v>1484</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6088,7 +6114,7 @@
       <c r="J12" t="s">
         <v>1484</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6132,7 +6158,7 @@
       <c r="J13" t="s">
         <v>1484</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6150,7 +6176,7 @@
       <c r="R13" t="s">
         <v>1642</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6188,7 +6214,7 @@
       <c r="J14" t="s">
         <v>1484</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6206,7 +6232,7 @@
       <c r="R14" t="s">
         <v>1643</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6244,7 +6270,7 @@
       <c r="J15" t="s">
         <v>1484</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6262,7 +6288,7 @@
       <c r="R15" t="s">
         <v>1643</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6300,7 +6326,7 @@
       <c r="J16" t="s">
         <v>1484</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6344,7 +6370,7 @@
       <c r="J17" t="s">
         <v>1484</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6388,7 +6414,7 @@
       <c r="J18" t="s">
         <v>1484</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6406,7 +6432,7 @@
       <c r="R18" t="s">
         <v>1644</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6447,7 +6473,7 @@
       <c r="J19" t="s">
         <v>1484</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6491,7 +6517,7 @@
       <c r="J20" t="s">
         <v>1484</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6535,7 +6561,7 @@
       <c r="J21" t="s">
         <v>1484</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6553,7 +6579,7 @@
       <c r="R21" t="s">
         <v>1643</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6594,7 +6620,7 @@
       <c r="J22" t="s">
         <v>1484</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6612,7 +6638,7 @@
       <c r="R22" t="s">
         <v>1645</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6653,7 +6679,7 @@
       <c r="J23" t="s">
         <v>1484</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6671,7 +6697,7 @@
       <c r="R23" t="s">
         <v>1646</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6712,7 +6738,7 @@
       <c r="J24" t="s">
         <v>1484</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6756,7 +6782,7 @@
       <c r="J25" t="s">
         <v>1484</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6797,7 +6823,7 @@
       <c r="J26" t="s">
         <v>1486</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6815,7 +6841,7 @@
       <c r="R26" t="s">
         <v>1647</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6850,7 +6876,7 @@
       <c r="J27" t="s">
         <v>1484</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6868,7 +6894,7 @@
       <c r="R27" t="s">
         <v>1648</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6909,7 +6935,7 @@
       <c r="J28" t="s">
         <v>1484</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6953,7 +6979,7 @@
       <c r="J29" t="s">
         <v>1484</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6997,7 +7023,7 @@
       <c r="J30" t="s">
         <v>1484</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7041,7 +7067,7 @@
       <c r="J31" t="s">
         <v>1484</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7059,7 +7085,7 @@
       <c r="R31" t="s">
         <v>1649</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7100,7 +7126,7 @@
       <c r="J32" t="s">
         <v>1484</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7144,7 +7170,7 @@
       <c r="J33" t="s">
         <v>1484</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7162,7 +7188,7 @@
       <c r="R33" t="s">
         <v>1650</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7203,7 +7229,7 @@
       <c r="J34" t="s">
         <v>1484</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7247,7 +7273,7 @@
       <c r="J35" t="s">
         <v>1484</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7265,7 +7291,7 @@
       <c r="R35" t="s">
         <v>1651</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7306,7 +7332,7 @@
       <c r="J36" t="s">
         <v>1484</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7324,7 +7350,7 @@
       <c r="R36" t="s">
         <v>1651</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7365,7 +7391,7 @@
       <c r="J37" t="s">
         <v>1484</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7383,7 +7409,7 @@
       <c r="R37" t="s">
         <v>1651</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7424,7 +7450,7 @@
       <c r="J38" t="s">
         <v>1484</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7442,7 +7468,7 @@
       <c r="R38" t="s">
         <v>1651</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7483,7 +7509,7 @@
       <c r="J39" t="s">
         <v>1484</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7501,7 +7527,7 @@
       <c r="R39" t="s">
         <v>1651</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7542,7 +7568,7 @@
       <c r="J40" t="s">
         <v>1484</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7560,7 +7586,7 @@
       <c r="R40" t="s">
         <v>1652</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7601,7 +7627,7 @@
       <c r="J41" t="s">
         <v>1484</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7619,7 +7645,7 @@
       <c r="R41" t="s">
         <v>1643</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7657,7 +7683,7 @@
       <c r="J42" t="s">
         <v>1484</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7675,7 +7701,7 @@
       <c r="R42" t="s">
         <v>1651</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7716,7 +7742,7 @@
       <c r="J43" t="s">
         <v>1484</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7760,7 +7786,7 @@
       <c r="J44" t="s">
         <v>1484</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7778,7 +7804,7 @@
       <c r="R44" t="s">
         <v>1653</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7819,7 +7845,7 @@
       <c r="J45" t="s">
         <v>1484</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7837,7 +7863,7 @@
       <c r="R45" t="s">
         <v>1654</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7875,7 +7901,7 @@
       <c r="J46" t="s">
         <v>1484</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7919,7 +7945,7 @@
       <c r="J47" t="s">
         <v>1484</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7937,7 +7963,7 @@
       <c r="R47" t="s">
         <v>1655</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7978,7 +8004,7 @@
       <c r="J48" t="s">
         <v>1484</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8022,7 +8048,7 @@
       <c r="J49" t="s">
         <v>1484</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8066,7 +8092,7 @@
       <c r="J50" t="s">
         <v>1484</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8110,7 +8136,7 @@
       <c r="J51" t="s">
         <v>1484</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8157,7 +8183,7 @@
       <c r="J52" t="s">
         <v>1484</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8201,7 +8227,7 @@
       <c r="J53" t="s">
         <v>1484</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8245,7 +8271,7 @@
       <c r="J54" t="s">
         <v>1484</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8289,7 +8315,7 @@
       <c r="J55" t="s">
         <v>1484</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8339,7 +8365,7 @@
       <c r="J56" t="s">
         <v>1484</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8392,7 +8418,7 @@
       <c r="J57" t="s">
         <v>1484</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8442,7 +8468,7 @@
       <c r="J58" t="s">
         <v>1484</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8492,7 +8518,7 @@
       <c r="J59" t="s">
         <v>1484</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8510,7 +8536,7 @@
       <c r="R59" t="s">
         <v>1656</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8551,7 +8577,7 @@
       <c r="J60" t="s">
         <v>1484</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8595,7 +8621,7 @@
       <c r="J61" t="s">
         <v>1484</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8639,7 +8665,7 @@
       <c r="J62" t="s">
         <v>1484</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8683,7 +8709,7 @@
       <c r="J63" t="s">
         <v>1484</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8727,7 +8753,7 @@
       <c r="J64" t="s">
         <v>1484</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8771,7 +8797,7 @@
       <c r="J65" t="s">
         <v>1484</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8818,7 +8844,7 @@
       <c r="J66" t="s">
         <v>1484</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8836,7 +8862,7 @@
       <c r="R66" t="s">
         <v>1657</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8874,7 +8900,7 @@
       <c r="J67" t="s">
         <v>1484</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8918,7 +8944,7 @@
       <c r="J68" t="s">
         <v>1484</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8933,7 +8959,7 @@
       <c r="O68" t="s">
         <v>1560</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8977,7 +9003,7 @@
       <c r="J69" t="s">
         <v>1486</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9021,7 +9047,7 @@
       <c r="J70" t="s">
         <v>1484</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9065,7 +9091,7 @@
       <c r="J71" t="s">
         <v>1484</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9109,7 +9135,7 @@
       <c r="J72" t="s">
         <v>1484</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9153,7 +9179,7 @@
       <c r="J73" t="s">
         <v>1484</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9197,7 +9223,7 @@
       <c r="J74" t="s">
         <v>1484</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9241,7 +9267,7 @@
       <c r="J75" t="s">
         <v>1484</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9285,7 +9311,7 @@
       <c r="J76" t="s">
         <v>1484</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9303,7 +9329,7 @@
       <c r="R76" t="s">
         <v>1658</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9341,7 +9367,7 @@
       <c r="J77" t="s">
         <v>1484</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9359,7 +9385,7 @@
       <c r="R77" t="s">
         <v>1658</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9397,7 +9423,7 @@
       <c r="J78" t="s">
         <v>1484</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9415,7 +9441,7 @@
       <c r="R78" t="s">
         <v>1658</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9453,7 +9479,7 @@
       <c r="J79" t="s">
         <v>1484</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9471,7 +9497,7 @@
       <c r="R79" t="s">
         <v>1658</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9509,7 +9535,7 @@
       <c r="J80" t="s">
         <v>1484</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9553,7 +9579,7 @@
       <c r="J81" t="s">
         <v>1484</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9597,7 +9623,7 @@
       <c r="J82" t="s">
         <v>1484</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9641,7 +9667,7 @@
       <c r="J83" t="s">
         <v>1484</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9685,7 +9711,7 @@
       <c r="J84" t="s">
         <v>1484</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9729,7 +9755,7 @@
       <c r="J85" t="s">
         <v>1484</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9747,7 +9773,7 @@
       <c r="R85" t="s">
         <v>1659</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9785,7 +9811,7 @@
       <c r="J86" t="s">
         <v>1484</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9829,7 +9855,7 @@
       <c r="J87" t="s">
         <v>1484</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9847,7 +9873,7 @@
       <c r="R87" t="s">
         <v>1660</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9885,7 +9911,7 @@
       <c r="J88" t="s">
         <v>1484</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9929,7 +9955,7 @@
       <c r="J89" t="s">
         <v>1484</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9947,7 +9973,7 @@
       <c r="R89" t="s">
         <v>1661</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -9982,7 +10008,7 @@
       <c r="J90" t="s">
         <v>1484</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10000,7 +10026,7 @@
       <c r="R90" t="s">
         <v>1662</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10035,7 +10061,7 @@
       <c r="J91" t="s">
         <v>1484</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10053,7 +10079,7 @@
       <c r="R91" t="s">
         <v>1646</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10091,7 +10117,7 @@
       <c r="J92" t="s">
         <v>1484</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10112,7 +10138,7 @@
       <c r="R92" t="s">
         <v>1646</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10153,7 +10179,7 @@
       <c r="J93" t="s">
         <v>1484</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10194,7 +10220,7 @@
       <c r="J94" t="s">
         <v>1484</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10238,7 +10264,7 @@
       <c r="J95" t="s">
         <v>1484</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10282,7 +10308,7 @@
       <c r="J96" t="s">
         <v>1484</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10300,7 +10326,7 @@
       <c r="R96" t="s">
         <v>1663</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10338,7 +10364,7 @@
       <c r="J97" t="s">
         <v>1484</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10353,7 +10379,7 @@
       <c r="R97" t="s">
         <v>1663</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10394,7 +10420,7 @@
       <c r="J98" t="s">
         <v>1484</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10412,7 +10438,7 @@
       <c r="R98" t="s">
         <v>1664</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10450,7 +10476,7 @@
       <c r="J99" t="s">
         <v>1484</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10468,7 +10494,7 @@
       <c r="R99" t="s">
         <v>1665</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10506,7 +10532,7 @@
       <c r="J100" t="s">
         <v>1484</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10547,7 +10573,7 @@
       <c r="J101" t="s">
         <v>1484</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10588,7 +10614,7 @@
       <c r="J102" t="s">
         <v>1484</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10629,7 +10655,7 @@
       <c r="J103" t="s">
         <v>1484</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10670,7 +10696,7 @@
       <c r="J104" t="s">
         <v>1484</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10711,7 +10737,7 @@
       <c r="J105" t="s">
         <v>1484</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10752,7 +10778,7 @@
       <c r="J106" t="s">
         <v>1484</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10793,7 +10819,7 @@
       <c r="J107" t="s">
         <v>1484</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10834,7 +10860,7 @@
       <c r="J108" t="s">
         <v>1484</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10875,7 +10901,7 @@
       <c r="J109" t="s">
         <v>1484</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10928,7 +10954,7 @@
       <c r="J110" t="s">
         <v>1484</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10984,7 +11010,7 @@
       <c r="J111" t="s">
         <v>1484</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11002,7 +11028,7 @@
       <c r="R111" t="s">
         <v>1667</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11040,7 +11066,7 @@
       <c r="J112" t="s">
         <v>1484</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11099,7 +11125,7 @@
       <c r="J113" t="s">
         <v>1484</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11143,7 +11169,7 @@
       <c r="J114" t="s">
         <v>1484</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11187,7 +11213,7 @@
       <c r="J115" t="s">
         <v>1484</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11205,7 +11231,7 @@
       <c r="R115" t="s">
         <v>1669</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11243,7 +11269,7 @@
       <c r="J116" t="s">
         <v>1484</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11302,7 +11328,7 @@
       <c r="J117" t="s">
         <v>1484</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11346,7 +11372,7 @@
       <c r="J118" t="s">
         <v>1484</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11393,7 +11419,7 @@
       <c r="J119" t="s">
         <v>1484</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11434,7 +11460,7 @@
       <c r="J120" t="s">
         <v>1484</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11478,7 +11504,7 @@
       <c r="J121" t="s">
         <v>1484</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11525,7 +11551,7 @@
       <c r="J122" t="s">
         <v>1484</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11575,7 +11601,7 @@
       <c r="J123" t="s">
         <v>1484</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11619,7 +11645,7 @@
       <c r="J124" t="s">
         <v>1484</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11663,7 +11689,7 @@
       <c r="J125" t="s">
         <v>1484</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11681,7 +11707,7 @@
       <c r="R125" t="s">
         <v>1671</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11716,7 +11742,7 @@
       <c r="J126" t="s">
         <v>1484</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11734,7 +11760,7 @@
       <c r="R126" t="s">
         <v>1672</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11769,7 +11795,7 @@
       <c r="J127" t="s">
         <v>1484</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11825,7 +11851,7 @@
       <c r="J128" t="s">
         <v>1484</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11866,7 +11892,7 @@
       <c r="J129" t="s">
         <v>1484</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11907,7 +11933,7 @@
       <c r="J130" t="s">
         <v>1484</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11948,7 +11974,7 @@
       <c r="J131" t="s">
         <v>1484</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11992,7 +12018,7 @@
       <c r="J132" t="s">
         <v>1484</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12033,7 +12059,7 @@
       <c r="J133" t="s">
         <v>1484</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12051,7 +12077,7 @@
       <c r="R133" t="s">
         <v>1658</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12086,7 +12112,7 @@
       <c r="J134" t="s">
         <v>1484</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12104,7 +12130,7 @@
       <c r="R134" t="s">
         <v>1658</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12139,7 +12165,7 @@
       <c r="J135" t="s">
         <v>1484</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12180,7 +12206,7 @@
       <c r="J136" t="s">
         <v>1484</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12221,7 +12247,7 @@
       <c r="J137" t="s">
         <v>1484</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12262,7 +12288,7 @@
       <c r="J138" t="s">
         <v>1484</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12303,7 +12329,7 @@
       <c r="J139" t="s">
         <v>1484</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12350,7 +12376,7 @@
       <c r="J140" t="s">
         <v>1484</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12391,7 +12417,7 @@
       <c r="J141" t="s">
         <v>1484</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12432,7 +12458,7 @@
       <c r="J142" t="s">
         <v>1484</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12476,7 +12502,7 @@
       <c r="J143" t="s">
         <v>1484</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12494,7 +12520,7 @@
       <c r="R143" t="s">
         <v>1658</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12529,7 +12555,7 @@
       <c r="J144" t="s">
         <v>1484</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12547,7 +12573,7 @@
       <c r="R144" t="s">
         <v>1658</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12582,7 +12608,7 @@
       <c r="J145" t="s">
         <v>1484</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12600,7 +12626,7 @@
       <c r="R145" t="s">
         <v>1658</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12635,7 +12661,7 @@
       <c r="J146" t="s">
         <v>1484</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12653,7 +12679,7 @@
       <c r="R146" t="s">
         <v>1666</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12688,7 +12714,7 @@
       <c r="J147" t="s">
         <v>1484</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12706,7 +12732,7 @@
       <c r="R147" t="s">
         <v>1673</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12741,7 +12767,7 @@
       <c r="J148" t="s">
         <v>1484</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12782,7 +12808,7 @@
       <c r="J149" t="s">
         <v>1484</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12800,7 +12826,7 @@
       <c r="R149" t="s">
         <v>1658</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12835,7 +12861,7 @@
       <c r="J150" t="s">
         <v>1484</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12853,7 +12879,7 @@
       <c r="R150" t="s">
         <v>1658</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12888,7 +12914,7 @@
       <c r="J151" t="s">
         <v>1484</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12906,7 +12932,7 @@
       <c r="R151" t="s">
         <v>1674</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12941,7 +12967,7 @@
       <c r="J152" t="s">
         <v>1484</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12959,7 +12985,7 @@
       <c r="R152" t="s">
         <v>1675</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -12994,7 +13020,7 @@
       <c r="J153" t="s">
         <v>1484</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13003,7 +13029,7 @@
       <c r="M153" t="s">
         <v>1551</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13044,7 +13070,7 @@
       <c r="J154" t="s">
         <v>1484</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13085,7 +13111,7 @@
       <c r="J155" t="s">
         <v>1484</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13126,7 +13152,7 @@
       <c r="J156" t="s">
         <v>1484</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13167,7 +13193,7 @@
       <c r="J157" t="s">
         <v>1484</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13208,7 +13234,7 @@
       <c r="J158" t="s">
         <v>1484</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13249,7 +13275,7 @@
       <c r="J159" t="s">
         <v>1484</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13290,7 +13316,7 @@
       <c r="J160" t="s">
         <v>1484</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13331,7 +13357,7 @@
       <c r="J161" t="s">
         <v>1484</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13372,7 +13398,7 @@
       <c r="J162" t="s">
         <v>1484</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13390,7 +13416,7 @@
       <c r="R162" t="s">
         <v>1661</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13425,7 +13451,7 @@
       <c r="J163" t="s">
         <v>1484</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13443,7 +13469,7 @@
       <c r="R163" t="s">
         <v>1658</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13478,7 +13504,7 @@
       <c r="J164" t="s">
         <v>1484</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13522,7 +13548,7 @@
       <c r="J165" t="s">
         <v>1484</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13563,7 +13589,7 @@
       <c r="J166" t="s">
         <v>1484</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13581,7 +13607,7 @@
       <c r="R166" t="s">
         <v>1676</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13616,7 +13642,7 @@
       <c r="J167" t="s">
         <v>1484</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13660,7 +13686,7 @@
       <c r="J168" t="s">
         <v>1484</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13704,7 +13730,7 @@
       <c r="J169" t="s">
         <v>1484</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13745,7 +13771,7 @@
       <c r="J170" t="s">
         <v>1484</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13786,7 +13812,7 @@
       <c r="J171" t="s">
         <v>1484</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13827,7 +13853,7 @@
       <c r="J172" t="s">
         <v>1484</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13868,7 +13894,7 @@
       <c r="J173" t="s">
         <v>1484</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13909,7 +13935,7 @@
       <c r="J174" t="s">
         <v>1484</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13950,7 +13976,7 @@
       <c r="J175" t="s">
         <v>1484</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -13991,7 +14017,7 @@
       <c r="J176" t="s">
         <v>1484</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14032,7 +14058,7 @@
       <c r="J177" t="s">
         <v>1484</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14073,7 +14099,7 @@
       <c r="J178" t="s">
         <v>1484</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14091,7 +14117,7 @@
       <c r="R178" t="s">
         <v>1674</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14126,7 +14152,7 @@
       <c r="J179" t="s">
         <v>1484</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14135,7 +14161,7 @@
       <c r="M179" t="s">
         <v>1548</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14176,7 +14202,7 @@
       <c r="J180" t="s">
         <v>1484</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14217,7 +14243,7 @@
       <c r="J181" t="s">
         <v>1484</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14235,7 +14261,7 @@
       <c r="R181" t="s">
         <v>1658</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14270,7 +14296,7 @@
       <c r="J182" t="s">
         <v>1484</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14311,7 +14337,7 @@
       <c r="J183" t="s">
         <v>1484</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14352,7 +14378,7 @@
       <c r="J184" t="s">
         <v>1484</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14393,7 +14419,7 @@
       <c r="J185" t="s">
         <v>1484</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14434,7 +14460,7 @@
       <c r="J186" t="s">
         <v>1484</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14475,7 +14501,7 @@
       <c r="J187" t="s">
         <v>1484</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14516,7 +14542,7 @@
       <c r="J188" t="s">
         <v>1484</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14557,7 +14583,7 @@
       <c r="J189" t="s">
         <v>1484</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14598,7 +14624,7 @@
       <c r="J190" t="s">
         <v>1484</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14639,7 +14665,7 @@
       <c r="J191" t="s">
         <v>1484</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14680,7 +14706,7 @@
       <c r="J192" t="s">
         <v>1484</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14721,7 +14747,7 @@
       <c r="J193" t="s">
         <v>1484</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14762,7 +14788,7 @@
       <c r="J194" t="s">
         <v>1484</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14803,7 +14829,7 @@
       <c r="J195" t="s">
         <v>1484</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14821,7 +14847,7 @@
       <c r="R195" t="s">
         <v>1667</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14859,7 +14885,7 @@
       <c r="J196" t="s">
         <v>1484</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14877,7 +14903,7 @@
       <c r="R196" t="s">
         <v>1673</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14915,7 +14941,7 @@
       <c r="J197" t="s">
         <v>1484</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14956,7 +14982,7 @@
       <c r="J198" t="s">
         <v>1486</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -14997,7 +15023,7 @@
       <c r="J199" t="s">
         <v>1485</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15038,7 +15064,7 @@
       <c r="J200" t="s">
         <v>1484</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15079,7 +15105,7 @@
       <c r="J201" t="s">
         <v>1484</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15120,7 +15146,7 @@
       <c r="J202" t="s">
         <v>1484</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15138,7 +15164,7 @@
       <c r="R202" t="s">
         <v>1658</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15173,7 +15199,7 @@
       <c r="J203" t="s">
         <v>1484</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15191,7 +15217,7 @@
       <c r="R203" t="s">
         <v>1666</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15226,7 +15252,7 @@
       <c r="J204" t="s">
         <v>1484</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15241,7 +15267,7 @@
       <c r="R204" t="s">
         <v>1677</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15279,7 +15305,7 @@
       <c r="J205" t="s">
         <v>1484</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15297,7 +15323,7 @@
       <c r="R205" t="s">
         <v>1678</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15335,7 +15361,7 @@
       <c r="J206" t="s">
         <v>1484</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15353,7 +15379,7 @@
       <c r="R206" t="s">
         <v>1646</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15388,7 +15414,7 @@
       <c r="J207" t="s">
         <v>1484</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15429,7 +15455,7 @@
       <c r="J208" t="s">
         <v>1484</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15470,7 +15496,7 @@
       <c r="J209" t="s">
         <v>1484</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15511,7 +15537,7 @@
       <c r="J210" t="s">
         <v>1484</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15552,7 +15578,7 @@
       <c r="J211" t="s">
         <v>1484</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15593,7 +15619,7 @@
       <c r="J212" t="s">
         <v>1484</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15634,7 +15660,7 @@
       <c r="J213" t="s">
         <v>1484</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15675,7 +15701,7 @@
       <c r="J214" t="s">
         <v>1484</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15693,7 +15719,7 @@
       <c r="R214" t="s">
         <v>1679</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15728,7 +15754,7 @@
       <c r="J215" t="s">
         <v>1484</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15769,7 +15795,7 @@
       <c r="J216" t="s">
         <v>1484</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15810,7 +15836,7 @@
       <c r="J217" t="s">
         <v>1484</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15851,7 +15877,7 @@
       <c r="J218" t="s">
         <v>1484</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15892,7 +15918,7 @@
       <c r="J219" t="s">
         <v>1484</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15933,7 +15959,7 @@
       <c r="J220" t="s">
         <v>1484</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -15974,7 +16000,7 @@
       <c r="J221" t="s">
         <v>1484</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16015,7 +16041,7 @@
       <c r="J222" t="s">
         <v>1484</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16056,7 +16082,7 @@
       <c r="J223" t="s">
         <v>1484</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16097,7 +16123,7 @@
       <c r="J224" t="s">
         <v>1484</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16138,7 +16164,7 @@
       <c r="J225" t="s">
         <v>1484</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16179,7 +16205,7 @@
       <c r="J226" t="s">
         <v>1484</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16220,7 +16246,7 @@
       <c r="J227" t="s">
         <v>1484</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16261,7 +16287,7 @@
       <c r="J228" t="s">
         <v>1484</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16302,7 +16328,7 @@
       <c r="J229" t="s">
         <v>1484</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16343,7 +16369,7 @@
       <c r="J230" t="s">
         <v>1484</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16384,7 +16410,7 @@
       <c r="J231" t="s">
         <v>1484</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16425,7 +16451,7 @@
       <c r="J232" t="s">
         <v>1484</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16466,7 +16492,7 @@
       <c r="J233" t="s">
         <v>1484</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16507,7 +16533,7 @@
       <c r="J234" t="s">
         <v>1484</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16548,7 +16574,7 @@
       <c r="J235" t="s">
         <v>1484</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16589,7 +16615,7 @@
       <c r="J236" t="s">
         <v>1484</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16630,7 +16656,7 @@
       <c r="J237" t="s">
         <v>1484</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16671,7 +16697,7 @@
       <c r="J238" t="s">
         <v>1484</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16712,7 +16738,7 @@
       <c r="J239" t="s">
         <v>1484</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16730,7 +16756,7 @@
       <c r="R239" t="s">
         <v>1673</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16765,7 +16791,7 @@
       <c r="J240" t="s">
         <v>1484</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16806,7 +16832,7 @@
       <c r="J241" t="s">
         <v>1484</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16847,7 +16873,7 @@
       <c r="J242" t="s">
         <v>1484</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16865,7 +16891,7 @@
       <c r="R242" t="s">
         <v>1666</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16900,7 +16926,7 @@
       <c r="J243" t="s">
         <v>1484</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16941,7 +16967,7 @@
       <c r="J244" t="s">
         <v>1484</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -16982,7 +17008,7 @@
       <c r="J245" t="s">
         <v>1484</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17023,7 +17049,7 @@
       <c r="J246" t="s">
         <v>1484</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17041,7 +17067,7 @@
       <c r="R246" t="s">
         <v>1646</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17076,7 +17102,7 @@
       <c r="J247" t="s">
         <v>1484</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17117,7 +17143,7 @@
       <c r="J248" t="s">
         <v>1484</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17158,7 +17184,7 @@
       <c r="J249" t="s">
         <v>1484</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17199,7 +17225,7 @@
       <c r="J250" t="s">
         <v>1484</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17240,7 +17266,7 @@
       <c r="J251" t="s">
         <v>1484</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17281,7 +17307,7 @@
       <c r="J252" t="s">
         <v>1484</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17322,7 +17348,7 @@
       <c r="J253" t="s">
         <v>1484</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17340,7 +17366,7 @@
       <c r="R253" t="s">
         <v>1676</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17378,7 +17404,7 @@
       <c r="J254" t="s">
         <v>1484</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17419,7 +17445,7 @@
       <c r="J255" t="s">
         <v>1484</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17460,7 +17486,7 @@
       <c r="J256" t="s">
         <v>1484</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17469,7 +17495,7 @@
       <c r="M256" t="s">
         <v>1547</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17507,7 +17533,7 @@
       <c r="J257" t="s">
         <v>1484</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17516,7 +17542,7 @@
       <c r="M257" t="s">
         <v>1548</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17560,7 +17586,7 @@
       <c r="J258" t="s">
         <v>1484</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17578,7 +17604,7 @@
       <c r="R258" t="s">
         <v>1658</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17616,7 +17642,7 @@
       <c r="J259" t="s">
         <v>1484</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17634,7 +17660,7 @@
       <c r="R259" t="s">
         <v>1674</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17672,7 +17698,7 @@
       <c r="J260" t="s">
         <v>1484</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17681,7 +17707,7 @@
       <c r="M260" t="s">
         <v>1542</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17725,7 +17751,7 @@
       <c r="J261" t="s">
         <v>1484</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17743,7 +17769,7 @@
       <c r="R261" t="s">
         <v>1680</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17781,7 +17807,7 @@
       <c r="J262" t="s">
         <v>1484</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17799,7 +17825,7 @@
       <c r="R262" t="s">
         <v>1674</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17837,7 +17863,7 @@
       <c r="J263" t="s">
         <v>1484</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17846,7 +17872,7 @@
       <c r="M263" t="s">
         <v>1542</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17890,7 +17916,7 @@
       <c r="J264" t="s">
         <v>1484</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17931,7 +17957,7 @@
       <c r="J265" t="s">
         <v>1484</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17972,7 +17998,7 @@
       <c r="J266" t="s">
         <v>1484</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18013,7 +18039,7 @@
       <c r="J267" t="s">
         <v>1484</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18057,7 +18083,7 @@
       <c r="J268" t="s">
         <v>1484</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18098,7 +18124,7 @@
       <c r="J269" t="s">
         <v>1484</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18139,7 +18165,7 @@
       <c r="J270" t="s">
         <v>1484</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18180,7 +18206,7 @@
       <c r="J271" t="s">
         <v>1484</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18221,7 +18247,7 @@
       <c r="J272" t="s">
         <v>1484</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18239,7 +18265,7 @@
       <c r="R272" t="s">
         <v>1681</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18277,7 +18303,7 @@
       <c r="J273" t="s">
         <v>1484</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18321,7 +18347,7 @@
       <c r="J274" t="s">
         <v>1484</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18362,7 +18388,7 @@
       <c r="J275" t="s">
         <v>1484</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18403,7 +18429,7 @@
       <c r="J276" t="s">
         <v>1484</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18444,7 +18470,7 @@
       <c r="J277" t="s">
         <v>1484</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18485,7 +18511,7 @@
       <c r="J278" t="s">
         <v>1484</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18526,7 +18552,7 @@
       <c r="J279" t="s">
         <v>1484</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18567,7 +18593,7 @@
       <c r="J280" t="s">
         <v>1484</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18608,7 +18634,7 @@
       <c r="J281" t="s">
         <v>1484</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18649,7 +18675,7 @@
       <c r="J282" t="s">
         <v>1484</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18690,7 +18716,7 @@
       <c r="J283" t="s">
         <v>1484</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18731,7 +18757,7 @@
       <c r="J284" t="s">
         <v>1484</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18772,7 +18798,7 @@
       <c r="J285" t="s">
         <v>1484</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18813,7 +18839,7 @@
       <c r="J286" t="s">
         <v>1484</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18854,7 +18880,7 @@
       <c r="J287" t="s">
         <v>1484</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18895,7 +18921,7 @@
       <c r="J288" t="s">
         <v>1484</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18936,7 +18962,7 @@
       <c r="J289" t="s">
         <v>1484</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -18977,7 +19003,7 @@
       <c r="J290" t="s">
         <v>1484</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19018,7 +19044,7 @@
       <c r="J291" t="s">
         <v>1484</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19059,7 +19085,7 @@
       <c r="J292" t="s">
         <v>1484</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19100,7 +19126,7 @@
       <c r="J293" t="s">
         <v>1484</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19141,7 +19167,7 @@
       <c r="J294" t="s">
         <v>1484</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19182,7 +19208,7 @@
       <c r="J295" t="s">
         <v>1484</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19200,7 +19226,7 @@
       <c r="R295" t="s">
         <v>1682</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19238,7 +19264,7 @@
       <c r="J296" t="s">
         <v>1484</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19256,7 +19282,7 @@
       <c r="R296" t="s">
         <v>1658</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19294,7 +19320,7 @@
       <c r="J297" t="s">
         <v>1484</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19335,7 +19361,7 @@
       <c r="J298" t="s">
         <v>1484</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19376,7 +19402,7 @@
       <c r="J299" t="s">
         <v>1485</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19417,7 +19443,7 @@
       <c r="J300" t="s">
         <v>1484</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19458,7 +19484,7 @@
       <c r="J301" t="s">
         <v>1484</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20296,7 +20322,7 @@
       <c r="R321" t="s">
         <v>1644</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20516,7 +20542,7 @@
       <c r="R326" t="s">
         <v>1683</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21351,7 +21377,7 @@
       <c r="R346" t="s">
         <v>1684</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (18/08/2026 12:41)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5181,16 +5181,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5206,7 +5198,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5214,30 +5206,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5537,73 +5511,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="J2" t="s">
         <v>1484</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5682,7 +5656,7 @@
       <c r="J3" t="s">
         <v>1484</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5726,7 +5700,7 @@
       <c r="J4" t="s">
         <v>1484</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5744,7 +5718,7 @@
       <c r="R4" t="s">
         <v>1641</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5782,7 +5756,7 @@
       <c r="J5" t="s">
         <v>1485</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5832,7 +5806,7 @@
       <c r="J6" t="s">
         <v>1484</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5879,7 +5853,7 @@
       <c r="J7" t="s">
         <v>1484</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5926,7 +5900,7 @@
       <c r="J8" t="s">
         <v>1484</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5973,7 +5947,7 @@
       <c r="J9" t="s">
         <v>1484</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6020,7 +5994,7 @@
       <c r="J10" t="s">
         <v>1484</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6067,7 +6041,7 @@
       <c r="J11" t="s">
         <v>1484</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6114,7 +6088,7 @@
       <c r="J12" t="s">
         <v>1484</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6158,7 +6132,7 @@
       <c r="J13" t="s">
         <v>1484</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6176,7 +6150,7 @@
       <c r="R13" t="s">
         <v>1642</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6214,7 +6188,7 @@
       <c r="J14" t="s">
         <v>1484</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6232,7 +6206,7 @@
       <c r="R14" t="s">
         <v>1643</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6270,7 +6244,7 @@
       <c r="J15" t="s">
         <v>1484</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6288,7 +6262,7 @@
       <c r="R15" t="s">
         <v>1643</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6326,7 +6300,7 @@
       <c r="J16" t="s">
         <v>1484</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6370,7 +6344,7 @@
       <c r="J17" t="s">
         <v>1484</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6414,7 +6388,7 @@
       <c r="J18" t="s">
         <v>1484</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6432,7 +6406,7 @@
       <c r="R18" t="s">
         <v>1644</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6473,7 +6447,7 @@
       <c r="J19" t="s">
         <v>1484</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6517,7 +6491,7 @@
       <c r="J20" t="s">
         <v>1484</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6561,7 +6535,7 @@
       <c r="J21" t="s">
         <v>1484</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6579,7 +6553,7 @@
       <c r="R21" t="s">
         <v>1643</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6620,7 +6594,7 @@
       <c r="J22" t="s">
         <v>1484</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6638,7 +6612,7 @@
       <c r="R22" t="s">
         <v>1645</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6679,7 +6653,7 @@
       <c r="J23" t="s">
         <v>1484</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6697,7 +6671,7 @@
       <c r="R23" t="s">
         <v>1646</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6738,7 +6712,7 @@
       <c r="J24" t="s">
         <v>1484</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6782,7 +6756,7 @@
       <c r="J25" t="s">
         <v>1484</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6823,7 +6797,7 @@
       <c r="J26" t="s">
         <v>1486</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6841,7 +6815,7 @@
       <c r="R26" t="s">
         <v>1647</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6876,7 +6850,7 @@
       <c r="J27" t="s">
         <v>1484</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6894,7 +6868,7 @@
       <c r="R27" t="s">
         <v>1648</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6935,7 +6909,7 @@
       <c r="J28" t="s">
         <v>1484</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6979,7 +6953,7 @@
       <c r="J29" t="s">
         <v>1484</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7023,7 +6997,7 @@
       <c r="J30" t="s">
         <v>1484</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7067,7 +7041,7 @@
       <c r="J31" t="s">
         <v>1484</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7085,7 +7059,7 @@
       <c r="R31" t="s">
         <v>1649</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7126,7 +7100,7 @@
       <c r="J32" t="s">
         <v>1484</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7170,7 +7144,7 @@
       <c r="J33" t="s">
         <v>1484</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7188,7 +7162,7 @@
       <c r="R33" t="s">
         <v>1650</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7229,7 +7203,7 @@
       <c r="J34" t="s">
         <v>1484</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7273,7 +7247,7 @@
       <c r="J35" t="s">
         <v>1484</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7291,7 +7265,7 @@
       <c r="R35" t="s">
         <v>1651</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7332,7 +7306,7 @@
       <c r="J36" t="s">
         <v>1484</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7350,7 +7324,7 @@
       <c r="R36" t="s">
         <v>1651</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7391,7 +7365,7 @@
       <c r="J37" t="s">
         <v>1484</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7409,7 +7383,7 @@
       <c r="R37" t="s">
         <v>1651</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7450,7 +7424,7 @@
       <c r="J38" t="s">
         <v>1484</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7468,7 +7442,7 @@
       <c r="R38" t="s">
         <v>1651</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7509,7 +7483,7 @@
       <c r="J39" t="s">
         <v>1484</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7527,7 +7501,7 @@
       <c r="R39" t="s">
         <v>1651</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7568,7 +7542,7 @@
       <c r="J40" t="s">
         <v>1484</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7586,7 +7560,7 @@
       <c r="R40" t="s">
         <v>1652</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7627,7 +7601,7 @@
       <c r="J41" t="s">
         <v>1484</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7645,7 +7619,7 @@
       <c r="R41" t="s">
         <v>1643</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7683,7 +7657,7 @@
       <c r="J42" t="s">
         <v>1484</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7701,7 +7675,7 @@
       <c r="R42" t="s">
         <v>1651</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7742,7 +7716,7 @@
       <c r="J43" t="s">
         <v>1484</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7786,7 +7760,7 @@
       <c r="J44" t="s">
         <v>1484</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7804,7 +7778,7 @@
       <c r="R44" t="s">
         <v>1653</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7845,7 +7819,7 @@
       <c r="J45" t="s">
         <v>1484</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7863,7 +7837,7 @@
       <c r="R45" t="s">
         <v>1654</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7901,7 +7875,7 @@
       <c r="J46" t="s">
         <v>1484</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7945,7 +7919,7 @@
       <c r="J47" t="s">
         <v>1484</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7963,7 +7937,7 @@
       <c r="R47" t="s">
         <v>1655</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8004,7 +7978,7 @@
       <c r="J48" t="s">
         <v>1484</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8048,7 +8022,7 @@
       <c r="J49" t="s">
         <v>1484</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8092,7 +8066,7 @@
       <c r="J50" t="s">
         <v>1484</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8136,7 +8110,7 @@
       <c r="J51" t="s">
         <v>1484</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8183,7 +8157,7 @@
       <c r="J52" t="s">
         <v>1484</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8227,7 +8201,7 @@
       <c r="J53" t="s">
         <v>1484</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8271,7 +8245,7 @@
       <c r="J54" t="s">
         <v>1484</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8315,7 +8289,7 @@
       <c r="J55" t="s">
         <v>1484</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8365,7 +8339,7 @@
       <c r="J56" t="s">
         <v>1484</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8418,7 +8392,7 @@
       <c r="J57" t="s">
         <v>1484</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8468,7 +8442,7 @@
       <c r="J58" t="s">
         <v>1484</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8518,7 +8492,7 @@
       <c r="J59" t="s">
         <v>1484</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8536,7 +8510,7 @@
       <c r="R59" t="s">
         <v>1656</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8577,7 +8551,7 @@
       <c r="J60" t="s">
         <v>1484</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8621,7 +8595,7 @@
       <c r="J61" t="s">
         <v>1484</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8665,7 +8639,7 @@
       <c r="J62" t="s">
         <v>1484</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8709,7 +8683,7 @@
       <c r="J63" t="s">
         <v>1484</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8753,7 +8727,7 @@
       <c r="J64" t="s">
         <v>1484</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8797,7 +8771,7 @@
       <c r="J65" t="s">
         <v>1484</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8844,7 +8818,7 @@
       <c r="J66" t="s">
         <v>1484</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8862,7 +8836,7 @@
       <c r="R66" t="s">
         <v>1657</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8900,7 +8874,7 @@
       <c r="J67" t="s">
         <v>1484</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8944,7 +8918,7 @@
       <c r="J68" t="s">
         <v>1484</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8959,7 +8933,7 @@
       <c r="O68" t="s">
         <v>1560</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9003,7 +8977,7 @@
       <c r="J69" t="s">
         <v>1486</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9047,7 +9021,7 @@
       <c r="J70" t="s">
         <v>1484</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9091,7 +9065,7 @@
       <c r="J71" t="s">
         <v>1484</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9135,7 +9109,7 @@
       <c r="J72" t="s">
         <v>1484</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9179,7 +9153,7 @@
       <c r="J73" t="s">
         <v>1484</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9223,7 +9197,7 @@
       <c r="J74" t="s">
         <v>1484</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9267,7 +9241,7 @@
       <c r="J75" t="s">
         <v>1484</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9311,7 +9285,7 @@
       <c r="J76" t="s">
         <v>1484</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9329,7 +9303,7 @@
       <c r="R76" t="s">
         <v>1658</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9367,7 +9341,7 @@
       <c r="J77" t="s">
         <v>1484</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9385,7 +9359,7 @@
       <c r="R77" t="s">
         <v>1658</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9423,7 +9397,7 @@
       <c r="J78" t="s">
         <v>1484</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9441,7 +9415,7 @@
       <c r="R78" t="s">
         <v>1658</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9479,7 +9453,7 @@
       <c r="J79" t="s">
         <v>1484</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9497,7 +9471,7 @@
       <c r="R79" t="s">
         <v>1658</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9535,7 +9509,7 @@
       <c r="J80" t="s">
         <v>1484</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9579,7 +9553,7 @@
       <c r="J81" t="s">
         <v>1484</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9623,7 +9597,7 @@
       <c r="J82" t="s">
         <v>1484</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9667,7 +9641,7 @@
       <c r="J83" t="s">
         <v>1484</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9711,7 +9685,7 @@
       <c r="J84" t="s">
         <v>1484</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9755,7 +9729,7 @@
       <c r="J85" t="s">
         <v>1484</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9773,7 +9747,7 @@
       <c r="R85" t="s">
         <v>1659</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9811,7 +9785,7 @@
       <c r="J86" t="s">
         <v>1484</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9855,7 +9829,7 @@
       <c r="J87" t="s">
         <v>1484</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9873,7 +9847,7 @@
       <c r="R87" t="s">
         <v>1660</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9911,7 +9885,7 @@
       <c r="J88" t="s">
         <v>1484</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9955,7 +9929,7 @@
       <c r="J89" t="s">
         <v>1484</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9973,7 +9947,7 @@
       <c r="R89" t="s">
         <v>1661</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10008,7 +9982,7 @@
       <c r="J90" t="s">
         <v>1484</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10026,7 +10000,7 @@
       <c r="R90" t="s">
         <v>1662</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10061,7 +10035,7 @@
       <c r="J91" t="s">
         <v>1484</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10079,7 +10053,7 @@
       <c r="R91" t="s">
         <v>1646</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10117,7 +10091,7 @@
       <c r="J92" t="s">
         <v>1484</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10138,7 +10112,7 @@
       <c r="R92" t="s">
         <v>1646</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10179,7 +10153,7 @@
       <c r="J93" t="s">
         <v>1484</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10220,7 +10194,7 @@
       <c r="J94" t="s">
         <v>1484</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10264,7 +10238,7 @@
       <c r="J95" t="s">
         <v>1484</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10308,7 +10282,7 @@
       <c r="J96" t="s">
         <v>1484</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10326,7 +10300,7 @@
       <c r="R96" t="s">
         <v>1663</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10364,7 +10338,7 @@
       <c r="J97" t="s">
         <v>1484</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10379,7 +10353,7 @@
       <c r="R97" t="s">
         <v>1663</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10420,7 +10394,7 @@
       <c r="J98" t="s">
         <v>1484</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10438,7 +10412,7 @@
       <c r="R98" t="s">
         <v>1664</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10476,7 +10450,7 @@
       <c r="J99" t="s">
         <v>1484</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10494,7 +10468,7 @@
       <c r="R99" t="s">
         <v>1665</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10532,7 +10506,7 @@
       <c r="J100" t="s">
         <v>1484</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10573,7 +10547,7 @@
       <c r="J101" t="s">
         <v>1484</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10614,7 +10588,7 @@
       <c r="J102" t="s">
         <v>1484</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10655,7 +10629,7 @@
       <c r="J103" t="s">
         <v>1484</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10696,7 +10670,7 @@
       <c r="J104" t="s">
         <v>1484</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10737,7 +10711,7 @@
       <c r="J105" t="s">
         <v>1484</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10778,7 +10752,7 @@
       <c r="J106" t="s">
         <v>1484</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10819,7 +10793,7 @@
       <c r="J107" t="s">
         <v>1484</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10860,7 +10834,7 @@
       <c r="J108" t="s">
         <v>1484</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10901,7 +10875,7 @@
       <c r="J109" t="s">
         <v>1484</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10954,7 +10928,7 @@
       <c r="J110" t="s">
         <v>1484</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11010,7 +10984,7 @@
       <c r="J111" t="s">
         <v>1484</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11028,7 +11002,7 @@
       <c r="R111" t="s">
         <v>1667</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11066,7 +11040,7 @@
       <c r="J112" t="s">
         <v>1484</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11125,7 +11099,7 @@
       <c r="J113" t="s">
         <v>1484</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11169,7 +11143,7 @@
       <c r="J114" t="s">
         <v>1484</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11213,7 +11187,7 @@
       <c r="J115" t="s">
         <v>1484</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11231,7 +11205,7 @@
       <c r="R115" t="s">
         <v>1669</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11269,7 +11243,7 @@
       <c r="J116" t="s">
         <v>1484</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11328,7 +11302,7 @@
       <c r="J117" t="s">
         <v>1484</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11372,7 +11346,7 @@
       <c r="J118" t="s">
         <v>1484</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11419,7 +11393,7 @@
       <c r="J119" t="s">
         <v>1484</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11460,7 +11434,7 @@
       <c r="J120" t="s">
         <v>1484</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11504,7 +11478,7 @@
       <c r="J121" t="s">
         <v>1484</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11551,7 +11525,7 @@
       <c r="J122" t="s">
         <v>1484</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11601,7 +11575,7 @@
       <c r="J123" t="s">
         <v>1484</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11645,7 +11619,7 @@
       <c r="J124" t="s">
         <v>1484</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11689,7 +11663,7 @@
       <c r="J125" t="s">
         <v>1484</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11707,7 +11681,7 @@
       <c r="R125" t="s">
         <v>1671</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11742,7 +11716,7 @@
       <c r="J126" t="s">
         <v>1484</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11760,7 +11734,7 @@
       <c r="R126" t="s">
         <v>1672</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11795,7 +11769,7 @@
       <c r="J127" t="s">
         <v>1484</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11851,7 +11825,7 @@
       <c r="J128" t="s">
         <v>1484</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11892,7 +11866,7 @@
       <c r="J129" t="s">
         <v>1484</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11933,7 +11907,7 @@
       <c r="J130" t="s">
         <v>1484</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11974,7 +11948,7 @@
       <c r="J131" t="s">
         <v>1484</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12018,7 +11992,7 @@
       <c r="J132" t="s">
         <v>1484</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12059,7 +12033,7 @@
       <c r="J133" t="s">
         <v>1484</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12077,7 +12051,7 @@
       <c r="R133" t="s">
         <v>1658</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12112,7 +12086,7 @@
       <c r="J134" t="s">
         <v>1484</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12130,7 +12104,7 @@
       <c r="R134" t="s">
         <v>1658</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12165,7 +12139,7 @@
       <c r="J135" t="s">
         <v>1484</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12206,7 +12180,7 @@
       <c r="J136" t="s">
         <v>1484</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12247,7 +12221,7 @@
       <c r="J137" t="s">
         <v>1484</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12288,7 +12262,7 @@
       <c r="J138" t="s">
         <v>1484</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12329,7 +12303,7 @@
       <c r="J139" t="s">
         <v>1484</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12376,7 +12350,7 @@
       <c r="J140" t="s">
         <v>1484</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12417,7 +12391,7 @@
       <c r="J141" t="s">
         <v>1484</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12458,7 +12432,7 @@
       <c r="J142" t="s">
         <v>1484</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12502,7 +12476,7 @@
       <c r="J143" t="s">
         <v>1484</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12520,7 +12494,7 @@
       <c r="R143" t="s">
         <v>1658</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12555,7 +12529,7 @@
       <c r="J144" t="s">
         <v>1484</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12573,7 +12547,7 @@
       <c r="R144" t="s">
         <v>1658</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12608,7 +12582,7 @@
       <c r="J145" t="s">
         <v>1484</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12626,7 +12600,7 @@
       <c r="R145" t="s">
         <v>1658</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12661,7 +12635,7 @@
       <c r="J146" t="s">
         <v>1484</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12679,7 +12653,7 @@
       <c r="R146" t="s">
         <v>1666</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12714,7 +12688,7 @@
       <c r="J147" t="s">
         <v>1484</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12732,7 +12706,7 @@
       <c r="R147" t="s">
         <v>1673</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12767,7 +12741,7 @@
       <c r="J148" t="s">
         <v>1484</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12808,7 +12782,7 @@
       <c r="J149" t="s">
         <v>1484</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12826,7 +12800,7 @@
       <c r="R149" t="s">
         <v>1658</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12861,7 +12835,7 @@
       <c r="J150" t="s">
         <v>1484</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12879,7 +12853,7 @@
       <c r="R150" t="s">
         <v>1658</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12914,7 +12888,7 @@
       <c r="J151" t="s">
         <v>1484</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12932,7 +12906,7 @@
       <c r="R151" t="s">
         <v>1674</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12967,7 +12941,7 @@
       <c r="J152" t="s">
         <v>1484</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12985,7 +12959,7 @@
       <c r="R152" t="s">
         <v>1675</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13020,7 +12994,7 @@
       <c r="J153" t="s">
         <v>1484</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13029,7 +13003,7 @@
       <c r="M153" t="s">
         <v>1551</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13070,7 +13044,7 @@
       <c r="J154" t="s">
         <v>1484</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13111,7 +13085,7 @@
       <c r="J155" t="s">
         <v>1484</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13152,7 +13126,7 @@
       <c r="J156" t="s">
         <v>1484</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13193,7 +13167,7 @@
       <c r="J157" t="s">
         <v>1484</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13234,7 +13208,7 @@
       <c r="J158" t="s">
         <v>1484</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13275,7 +13249,7 @@
       <c r="J159" t="s">
         <v>1484</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13316,7 +13290,7 @@
       <c r="J160" t="s">
         <v>1484</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13357,7 +13331,7 @@
       <c r="J161" t="s">
         <v>1484</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13398,7 +13372,7 @@
       <c r="J162" t="s">
         <v>1484</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13416,7 +13390,7 @@
       <c r="R162" t="s">
         <v>1661</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13451,7 +13425,7 @@
       <c r="J163" t="s">
         <v>1484</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13469,7 +13443,7 @@
       <c r="R163" t="s">
         <v>1658</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13504,7 +13478,7 @@
       <c r="J164" t="s">
         <v>1484</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13548,7 +13522,7 @@
       <c r="J165" t="s">
         <v>1484</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13589,7 +13563,7 @@
       <c r="J166" t="s">
         <v>1484</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13607,7 +13581,7 @@
       <c r="R166" t="s">
         <v>1676</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13642,7 +13616,7 @@
       <c r="J167" t="s">
         <v>1484</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13686,7 +13660,7 @@
       <c r="J168" t="s">
         <v>1484</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13730,7 +13704,7 @@
       <c r="J169" t="s">
         <v>1484</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13771,7 +13745,7 @@
       <c r="J170" t="s">
         <v>1484</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13812,7 +13786,7 @@
       <c r="J171" t="s">
         <v>1484</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13853,7 +13827,7 @@
       <c r="J172" t="s">
         <v>1484</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13894,7 +13868,7 @@
       <c r="J173" t="s">
         <v>1484</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13935,7 +13909,7 @@
       <c r="J174" t="s">
         <v>1484</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13976,7 +13950,7 @@
       <c r="J175" t="s">
         <v>1484</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14017,7 +13991,7 @@
       <c r="J176" t="s">
         <v>1484</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14058,7 +14032,7 @@
       <c r="J177" t="s">
         <v>1484</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14099,7 +14073,7 @@
       <c r="J178" t="s">
         <v>1484</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14117,7 +14091,7 @@
       <c r="R178" t="s">
         <v>1674</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14152,7 +14126,7 @@
       <c r="J179" t="s">
         <v>1484</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14161,7 +14135,7 @@
       <c r="M179" t="s">
         <v>1548</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14202,7 +14176,7 @@
       <c r="J180" t="s">
         <v>1484</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14243,7 +14217,7 @@
       <c r="J181" t="s">
         <v>1484</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14261,7 +14235,7 @@
       <c r="R181" t="s">
         <v>1658</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14296,7 +14270,7 @@
       <c r="J182" t="s">
         <v>1484</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14337,7 +14311,7 @@
       <c r="J183" t="s">
         <v>1484</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14378,7 +14352,7 @@
       <c r="J184" t="s">
         <v>1484</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14419,7 +14393,7 @@
       <c r="J185" t="s">
         <v>1484</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14460,7 +14434,7 @@
       <c r="J186" t="s">
         <v>1484</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14501,7 +14475,7 @@
       <c r="J187" t="s">
         <v>1484</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14542,7 +14516,7 @@
       <c r="J188" t="s">
         <v>1484</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14583,7 +14557,7 @@
       <c r="J189" t="s">
         <v>1484</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14624,7 +14598,7 @@
       <c r="J190" t="s">
         <v>1484</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14665,7 +14639,7 @@
       <c r="J191" t="s">
         <v>1484</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14706,7 +14680,7 @@
       <c r="J192" t="s">
         <v>1484</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14747,7 +14721,7 @@
       <c r="J193" t="s">
         <v>1484</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14788,7 +14762,7 @@
       <c r="J194" t="s">
         <v>1484</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14829,7 +14803,7 @@
       <c r="J195" t="s">
         <v>1484</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14847,7 +14821,7 @@
       <c r="R195" t="s">
         <v>1667</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14885,7 +14859,7 @@
       <c r="J196" t="s">
         <v>1484</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14903,7 +14877,7 @@
       <c r="R196" t="s">
         <v>1673</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14941,7 +14915,7 @@
       <c r="J197" t="s">
         <v>1484</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14982,7 +14956,7 @@
       <c r="J198" t="s">
         <v>1486</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15023,7 +14997,7 @@
       <c r="J199" t="s">
         <v>1485</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15064,7 +15038,7 @@
       <c r="J200" t="s">
         <v>1484</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15105,7 +15079,7 @@
       <c r="J201" t="s">
         <v>1484</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15146,7 +15120,7 @@
       <c r="J202" t="s">
         <v>1484</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15164,7 +15138,7 @@
       <c r="R202" t="s">
         <v>1658</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15199,7 +15173,7 @@
       <c r="J203" t="s">
         <v>1484</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15217,7 +15191,7 @@
       <c r="R203" t="s">
         <v>1666</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15252,7 +15226,7 @@
       <c r="J204" t="s">
         <v>1484</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15267,7 +15241,7 @@
       <c r="R204" t="s">
         <v>1677</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15305,7 +15279,7 @@
       <c r="J205" t="s">
         <v>1484</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15323,7 +15297,7 @@
       <c r="R205" t="s">
         <v>1678</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15361,7 +15335,7 @@
       <c r="J206" t="s">
         <v>1484</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15379,7 +15353,7 @@
       <c r="R206" t="s">
         <v>1646</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15414,7 +15388,7 @@
       <c r="J207" t="s">
         <v>1484</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15455,7 +15429,7 @@
       <c r="J208" t="s">
         <v>1484</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15496,7 +15470,7 @@
       <c r="J209" t="s">
         <v>1484</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15537,7 +15511,7 @@
       <c r="J210" t="s">
         <v>1484</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15578,7 +15552,7 @@
       <c r="J211" t="s">
         <v>1484</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15619,7 +15593,7 @@
       <c r="J212" t="s">
         <v>1484</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15660,7 +15634,7 @@
       <c r="J213" t="s">
         <v>1484</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15701,7 +15675,7 @@
       <c r="J214" t="s">
         <v>1484</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15719,7 +15693,7 @@
       <c r="R214" t="s">
         <v>1679</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15754,7 +15728,7 @@
       <c r="J215" t="s">
         <v>1484</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15795,7 +15769,7 @@
       <c r="J216" t="s">
         <v>1484</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15836,7 +15810,7 @@
       <c r="J217" t="s">
         <v>1484</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15877,7 +15851,7 @@
       <c r="J218" t="s">
         <v>1484</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15918,7 +15892,7 @@
       <c r="J219" t="s">
         <v>1484</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15959,7 +15933,7 @@
       <c r="J220" t="s">
         <v>1484</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16000,7 +15974,7 @@
       <c r="J221" t="s">
         <v>1484</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16041,7 +16015,7 @@
       <c r="J222" t="s">
         <v>1484</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16082,7 +16056,7 @@
       <c r="J223" t="s">
         <v>1484</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16123,7 +16097,7 @@
       <c r="J224" t="s">
         <v>1484</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16164,7 +16138,7 @@
       <c r="J225" t="s">
         <v>1484</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16205,7 +16179,7 @@
       <c r="J226" t="s">
         <v>1484</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16246,7 +16220,7 @@
       <c r="J227" t="s">
         <v>1484</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16287,7 +16261,7 @@
       <c r="J228" t="s">
         <v>1484</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16328,7 +16302,7 @@
       <c r="J229" t="s">
         <v>1484</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16369,7 +16343,7 @@
       <c r="J230" t="s">
         <v>1484</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16410,7 +16384,7 @@
       <c r="J231" t="s">
         <v>1484</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16451,7 +16425,7 @@
       <c r="J232" t="s">
         <v>1484</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16492,7 +16466,7 @@
       <c r="J233" t="s">
         <v>1484</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16533,7 +16507,7 @@
       <c r="J234" t="s">
         <v>1484</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16574,7 +16548,7 @@
       <c r="J235" t="s">
         <v>1484</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16615,7 +16589,7 @@
       <c r="J236" t="s">
         <v>1484</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16656,7 +16630,7 @@
       <c r="J237" t="s">
         <v>1484</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16697,7 +16671,7 @@
       <c r="J238" t="s">
         <v>1484</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16738,7 +16712,7 @@
       <c r="J239" t="s">
         <v>1484</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16756,7 +16730,7 @@
       <c r="R239" t="s">
         <v>1673</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16791,7 +16765,7 @@
       <c r="J240" t="s">
         <v>1484</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16832,7 +16806,7 @@
       <c r="J241" t="s">
         <v>1484</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16873,7 +16847,7 @@
       <c r="J242" t="s">
         <v>1484</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16891,7 +16865,7 @@
       <c r="R242" t="s">
         <v>1666</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16926,7 +16900,7 @@
       <c r="J243" t="s">
         <v>1484</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16967,7 +16941,7 @@
       <c r="J244" t="s">
         <v>1484</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17008,7 +16982,7 @@
       <c r="J245" t="s">
         <v>1484</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17049,7 +17023,7 @@
       <c r="J246" t="s">
         <v>1484</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17067,7 +17041,7 @@
       <c r="R246" t="s">
         <v>1646</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17102,7 +17076,7 @@
       <c r="J247" t="s">
         <v>1484</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17143,7 +17117,7 @@
       <c r="J248" t="s">
         <v>1484</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17184,7 +17158,7 @@
       <c r="J249" t="s">
         <v>1484</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17225,7 +17199,7 @@
       <c r="J250" t="s">
         <v>1484</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17266,7 +17240,7 @@
       <c r="J251" t="s">
         <v>1484</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17307,7 +17281,7 @@
       <c r="J252" t="s">
         <v>1484</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17348,7 +17322,7 @@
       <c r="J253" t="s">
         <v>1484</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17366,7 +17340,7 @@
       <c r="R253" t="s">
         <v>1676</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17404,7 +17378,7 @@
       <c r="J254" t="s">
         <v>1484</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17445,7 +17419,7 @@
       <c r="J255" t="s">
         <v>1484</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17486,7 +17460,7 @@
       <c r="J256" t="s">
         <v>1484</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17495,7 +17469,7 @@
       <c r="M256" t="s">
         <v>1547</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17533,7 +17507,7 @@
       <c r="J257" t="s">
         <v>1484</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17542,7 +17516,7 @@
       <c r="M257" t="s">
         <v>1548</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17586,7 +17560,7 @@
       <c r="J258" t="s">
         <v>1484</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17604,7 +17578,7 @@
       <c r="R258" t="s">
         <v>1658</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17642,7 +17616,7 @@
       <c r="J259" t="s">
         <v>1484</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17660,7 +17634,7 @@
       <c r="R259" t="s">
         <v>1674</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17698,7 +17672,7 @@
       <c r="J260" t="s">
         <v>1484</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17707,7 +17681,7 @@
       <c r="M260" t="s">
         <v>1542</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17751,7 +17725,7 @@
       <c r="J261" t="s">
         <v>1484</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17769,7 +17743,7 @@
       <c r="R261" t="s">
         <v>1680</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17807,7 +17781,7 @@
       <c r="J262" t="s">
         <v>1484</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17825,7 +17799,7 @@
       <c r="R262" t="s">
         <v>1674</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17863,7 +17837,7 @@
       <c r="J263" t="s">
         <v>1484</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17872,7 +17846,7 @@
       <c r="M263" t="s">
         <v>1542</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17916,7 +17890,7 @@
       <c r="J264" t="s">
         <v>1484</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17957,7 +17931,7 @@
       <c r="J265" t="s">
         <v>1484</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17998,7 +17972,7 @@
       <c r="J266" t="s">
         <v>1484</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18039,7 +18013,7 @@
       <c r="J267" t="s">
         <v>1484</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18083,7 +18057,7 @@
       <c r="J268" t="s">
         <v>1484</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18124,7 +18098,7 @@
       <c r="J269" t="s">
         <v>1484</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18165,7 +18139,7 @@
       <c r="J270" t="s">
         <v>1484</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18206,7 +18180,7 @@
       <c r="J271" t="s">
         <v>1484</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18247,7 +18221,7 @@
       <c r="J272" t="s">
         <v>1484</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18265,7 +18239,7 @@
       <c r="R272" t="s">
         <v>1681</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18303,7 +18277,7 @@
       <c r="J273" t="s">
         <v>1484</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18347,7 +18321,7 @@
       <c r="J274" t="s">
         <v>1484</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18388,7 +18362,7 @@
       <c r="J275" t="s">
         <v>1484</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18429,7 +18403,7 @@
       <c r="J276" t="s">
         <v>1484</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18470,7 +18444,7 @@
       <c r="J277" t="s">
         <v>1484</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18511,7 +18485,7 @@
       <c r="J278" t="s">
         <v>1484</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18552,7 +18526,7 @@
       <c r="J279" t="s">
         <v>1484</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18593,7 +18567,7 @@
       <c r="J280" t="s">
         <v>1484</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18634,7 +18608,7 @@
       <c r="J281" t="s">
         <v>1484</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18675,7 +18649,7 @@
       <c r="J282" t="s">
         <v>1484</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18716,7 +18690,7 @@
       <c r="J283" t="s">
         <v>1484</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18757,7 +18731,7 @@
       <c r="J284" t="s">
         <v>1484</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18798,7 +18772,7 @@
       <c r="J285" t="s">
         <v>1484</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18839,7 +18813,7 @@
       <c r="J286" t="s">
         <v>1484</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18880,7 +18854,7 @@
       <c r="J287" t="s">
         <v>1484</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18921,7 +18895,7 @@
       <c r="J288" t="s">
         <v>1484</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18962,7 +18936,7 @@
       <c r="J289" t="s">
         <v>1484</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19003,7 +18977,7 @@
       <c r="J290" t="s">
         <v>1484</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19044,7 +19018,7 @@
       <c r="J291" t="s">
         <v>1484</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19085,7 +19059,7 @@
       <c r="J292" t="s">
         <v>1484</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19126,7 +19100,7 @@
       <c r="J293" t="s">
         <v>1484</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19167,7 +19141,7 @@
       <c r="J294" t="s">
         <v>1484</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19208,7 +19182,7 @@
       <c r="J295" t="s">
         <v>1484</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19226,7 +19200,7 @@
       <c r="R295" t="s">
         <v>1682</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19264,7 +19238,7 @@
       <c r="J296" t="s">
         <v>1484</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19282,7 +19256,7 @@
       <c r="R296" t="s">
         <v>1658</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19320,7 +19294,7 @@
       <c r="J297" t="s">
         <v>1484</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19361,7 +19335,7 @@
       <c r="J298" t="s">
         <v>1484</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19402,7 +19376,7 @@
       <c r="J299" t="s">
         <v>1485</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19443,7 +19417,7 @@
       <c r="J300" t="s">
         <v>1484</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19484,7 +19458,7 @@
       <c r="J301" t="s">
         <v>1484</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20322,7 +20296,7 @@
       <c r="R321" t="s">
         <v>1644</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20542,7 +20516,7 @@
       <c r="R326" t="s">
         <v>1683</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21377,7 +21351,7 @@
       <c r="R346" t="s">
         <v>1684</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (19/08/2026 13:08)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5181,8 +5181,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5198,7 +5206,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5206,12 +5214,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5511,73 +5537,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="J2" t="s">
         <v>1484</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5656,7 +5682,7 @@
       <c r="J3" t="s">
         <v>1484</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5700,7 +5726,7 @@
       <c r="J4" t="s">
         <v>1484</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5718,7 +5744,7 @@
       <c r="R4" t="s">
         <v>1641</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5756,7 +5782,7 @@
       <c r="J5" t="s">
         <v>1485</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5806,7 +5832,7 @@
       <c r="J6" t="s">
         <v>1484</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5853,7 +5879,7 @@
       <c r="J7" t="s">
         <v>1484</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5900,7 +5926,7 @@
       <c r="J8" t="s">
         <v>1484</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5947,7 +5973,7 @@
       <c r="J9" t="s">
         <v>1484</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5994,7 +6020,7 @@
       <c r="J10" t="s">
         <v>1484</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6041,7 +6067,7 @@
       <c r="J11" t="s">
         <v>1484</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6088,7 +6114,7 @@
       <c r="J12" t="s">
         <v>1484</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6132,7 +6158,7 @@
       <c r="J13" t="s">
         <v>1484</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6150,7 +6176,7 @@
       <c r="R13" t="s">
         <v>1642</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6188,7 +6214,7 @@
       <c r="J14" t="s">
         <v>1484</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6206,7 +6232,7 @@
       <c r="R14" t="s">
         <v>1643</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6244,7 +6270,7 @@
       <c r="J15" t="s">
         <v>1484</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6262,7 +6288,7 @@
       <c r="R15" t="s">
         <v>1643</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6300,7 +6326,7 @@
       <c r="J16" t="s">
         <v>1484</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6344,7 +6370,7 @@
       <c r="J17" t="s">
         <v>1484</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6388,7 +6414,7 @@
       <c r="J18" t="s">
         <v>1484</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6406,7 +6432,7 @@
       <c r="R18" t="s">
         <v>1644</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6447,7 +6473,7 @@
       <c r="J19" t="s">
         <v>1484</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6491,7 +6517,7 @@
       <c r="J20" t="s">
         <v>1484</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6535,7 +6561,7 @@
       <c r="J21" t="s">
         <v>1484</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6553,7 +6579,7 @@
       <c r="R21" t="s">
         <v>1643</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6594,7 +6620,7 @@
       <c r="J22" t="s">
         <v>1484</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6612,7 +6638,7 @@
       <c r="R22" t="s">
         <v>1645</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6653,7 +6679,7 @@
       <c r="J23" t="s">
         <v>1484</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6671,7 +6697,7 @@
       <c r="R23" t="s">
         <v>1646</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6712,7 +6738,7 @@
       <c r="J24" t="s">
         <v>1484</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6756,7 +6782,7 @@
       <c r="J25" t="s">
         <v>1484</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6797,7 +6823,7 @@
       <c r="J26" t="s">
         <v>1486</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6815,7 +6841,7 @@
       <c r="R26" t="s">
         <v>1647</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6850,7 +6876,7 @@
       <c r="J27" t="s">
         <v>1484</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6868,7 +6894,7 @@
       <c r="R27" t="s">
         <v>1648</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6909,7 +6935,7 @@
       <c r="J28" t="s">
         <v>1484</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6953,7 +6979,7 @@
       <c r="J29" t="s">
         <v>1484</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6997,7 +7023,7 @@
       <c r="J30" t="s">
         <v>1484</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7041,7 +7067,7 @@
       <c r="J31" t="s">
         <v>1484</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7059,7 +7085,7 @@
       <c r="R31" t="s">
         <v>1649</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7100,7 +7126,7 @@
       <c r="J32" t="s">
         <v>1484</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7144,7 +7170,7 @@
       <c r="J33" t="s">
         <v>1484</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7162,7 +7188,7 @@
       <c r="R33" t="s">
         <v>1650</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7203,7 +7229,7 @@
       <c r="J34" t="s">
         <v>1484</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7247,7 +7273,7 @@
       <c r="J35" t="s">
         <v>1484</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7265,7 +7291,7 @@
       <c r="R35" t="s">
         <v>1651</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7306,7 +7332,7 @@
       <c r="J36" t="s">
         <v>1484</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7324,7 +7350,7 @@
       <c r="R36" t="s">
         <v>1651</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7365,7 +7391,7 @@
       <c r="J37" t="s">
         <v>1484</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7383,7 +7409,7 @@
       <c r="R37" t="s">
         <v>1651</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7424,7 +7450,7 @@
       <c r="J38" t="s">
         <v>1484</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7442,7 +7468,7 @@
       <c r="R38" t="s">
         <v>1651</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7483,7 +7509,7 @@
       <c r="J39" t="s">
         <v>1484</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7501,7 +7527,7 @@
       <c r="R39" t="s">
         <v>1651</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7542,7 +7568,7 @@
       <c r="J40" t="s">
         <v>1484</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7560,7 +7586,7 @@
       <c r="R40" t="s">
         <v>1652</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7601,7 +7627,7 @@
       <c r="J41" t="s">
         <v>1484</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7619,7 +7645,7 @@
       <c r="R41" t="s">
         <v>1643</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7657,7 +7683,7 @@
       <c r="J42" t="s">
         <v>1484</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7675,7 +7701,7 @@
       <c r="R42" t="s">
         <v>1651</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7716,7 +7742,7 @@
       <c r="J43" t="s">
         <v>1484</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7760,7 +7786,7 @@
       <c r="J44" t="s">
         <v>1484</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7778,7 +7804,7 @@
       <c r="R44" t="s">
         <v>1653</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7819,7 +7845,7 @@
       <c r="J45" t="s">
         <v>1484</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7837,7 +7863,7 @@
       <c r="R45" t="s">
         <v>1654</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7875,7 +7901,7 @@
       <c r="J46" t="s">
         <v>1484</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7919,7 +7945,7 @@
       <c r="J47" t="s">
         <v>1484</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7937,7 +7963,7 @@
       <c r="R47" t="s">
         <v>1655</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7978,7 +8004,7 @@
       <c r="J48" t="s">
         <v>1484</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8022,7 +8048,7 @@
       <c r="J49" t="s">
         <v>1484</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8066,7 +8092,7 @@
       <c r="J50" t="s">
         <v>1484</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8110,7 +8136,7 @@
       <c r="J51" t="s">
         <v>1484</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8157,7 +8183,7 @@
       <c r="J52" t="s">
         <v>1484</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8201,7 +8227,7 @@
       <c r="J53" t="s">
         <v>1484</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8245,7 +8271,7 @@
       <c r="J54" t="s">
         <v>1484</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8289,7 +8315,7 @@
       <c r="J55" t="s">
         <v>1484</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8339,7 +8365,7 @@
       <c r="J56" t="s">
         <v>1484</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8392,7 +8418,7 @@
       <c r="J57" t="s">
         <v>1484</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8442,7 +8468,7 @@
       <c r="J58" t="s">
         <v>1484</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8492,7 +8518,7 @@
       <c r="J59" t="s">
         <v>1484</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8510,7 +8536,7 @@
       <c r="R59" t="s">
         <v>1656</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8551,7 +8577,7 @@
       <c r="J60" t="s">
         <v>1484</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8595,7 +8621,7 @@
       <c r="J61" t="s">
         <v>1484</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8639,7 +8665,7 @@
       <c r="J62" t="s">
         <v>1484</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8683,7 +8709,7 @@
       <c r="J63" t="s">
         <v>1484</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8727,7 +8753,7 @@
       <c r="J64" t="s">
         <v>1484</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8771,7 +8797,7 @@
       <c r="J65" t="s">
         <v>1484</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8818,7 +8844,7 @@
       <c r="J66" t="s">
         <v>1484</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8836,7 +8862,7 @@
       <c r="R66" t="s">
         <v>1657</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8874,7 +8900,7 @@
       <c r="J67" t="s">
         <v>1484</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8918,7 +8944,7 @@
       <c r="J68" t="s">
         <v>1484</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8933,7 +8959,7 @@
       <c r="O68" t="s">
         <v>1560</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8977,7 +9003,7 @@
       <c r="J69" t="s">
         <v>1486</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9021,7 +9047,7 @@
       <c r="J70" t="s">
         <v>1484</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9065,7 +9091,7 @@
       <c r="J71" t="s">
         <v>1484</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9109,7 +9135,7 @@
       <c r="J72" t="s">
         <v>1484</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9153,7 +9179,7 @@
       <c r="J73" t="s">
         <v>1484</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9197,7 +9223,7 @@
       <c r="J74" t="s">
         <v>1484</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9241,7 +9267,7 @@
       <c r="J75" t="s">
         <v>1484</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9285,7 +9311,7 @@
       <c r="J76" t="s">
         <v>1484</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9303,7 +9329,7 @@
       <c r="R76" t="s">
         <v>1658</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9341,7 +9367,7 @@
       <c r="J77" t="s">
         <v>1484</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9359,7 +9385,7 @@
       <c r="R77" t="s">
         <v>1658</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9397,7 +9423,7 @@
       <c r="J78" t="s">
         <v>1484</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9415,7 +9441,7 @@
       <c r="R78" t="s">
         <v>1658</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9453,7 +9479,7 @@
       <c r="J79" t="s">
         <v>1484</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9471,7 +9497,7 @@
       <c r="R79" t="s">
         <v>1658</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9509,7 +9535,7 @@
       <c r="J80" t="s">
         <v>1484</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9553,7 +9579,7 @@
       <c r="J81" t="s">
         <v>1484</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9597,7 +9623,7 @@
       <c r="J82" t="s">
         <v>1484</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9641,7 +9667,7 @@
       <c r="J83" t="s">
         <v>1484</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9685,7 +9711,7 @@
       <c r="J84" t="s">
         <v>1484</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9729,7 +9755,7 @@
       <c r="J85" t="s">
         <v>1484</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9747,7 +9773,7 @@
       <c r="R85" t="s">
         <v>1659</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9785,7 +9811,7 @@
       <c r="J86" t="s">
         <v>1484</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9829,7 +9855,7 @@
       <c r="J87" t="s">
         <v>1484</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9847,7 +9873,7 @@
       <c r="R87" t="s">
         <v>1660</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9885,7 +9911,7 @@
       <c r="J88" t="s">
         <v>1484</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9929,7 +9955,7 @@
       <c r="J89" t="s">
         <v>1484</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9947,7 +9973,7 @@
       <c r="R89" t="s">
         <v>1661</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -9982,7 +10008,7 @@
       <c r="J90" t="s">
         <v>1484</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10000,7 +10026,7 @@
       <c r="R90" t="s">
         <v>1662</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10035,7 +10061,7 @@
       <c r="J91" t="s">
         <v>1484</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10053,7 +10079,7 @@
       <c r="R91" t="s">
         <v>1646</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10091,7 +10117,7 @@
       <c r="J92" t="s">
         <v>1484</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10112,7 +10138,7 @@
       <c r="R92" t="s">
         <v>1646</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10153,7 +10179,7 @@
       <c r="J93" t="s">
         <v>1484</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10194,7 +10220,7 @@
       <c r="J94" t="s">
         <v>1484</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10238,7 +10264,7 @@
       <c r="J95" t="s">
         <v>1484</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10282,7 +10308,7 @@
       <c r="J96" t="s">
         <v>1484</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10300,7 +10326,7 @@
       <c r="R96" t="s">
         <v>1663</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10338,7 +10364,7 @@
       <c r="J97" t="s">
         <v>1484</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10353,7 +10379,7 @@
       <c r="R97" t="s">
         <v>1663</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10394,7 +10420,7 @@
       <c r="J98" t="s">
         <v>1484</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10412,7 +10438,7 @@
       <c r="R98" t="s">
         <v>1664</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10450,7 +10476,7 @@
       <c r="J99" t="s">
         <v>1484</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10468,7 +10494,7 @@
       <c r="R99" t="s">
         <v>1665</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10506,7 +10532,7 @@
       <c r="J100" t="s">
         <v>1484</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10547,7 +10573,7 @@
       <c r="J101" t="s">
         <v>1484</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10588,7 +10614,7 @@
       <c r="J102" t="s">
         <v>1484</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10629,7 +10655,7 @@
       <c r="J103" t="s">
         <v>1484</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10670,7 +10696,7 @@
       <c r="J104" t="s">
         <v>1484</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10711,7 +10737,7 @@
       <c r="J105" t="s">
         <v>1484</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10752,7 +10778,7 @@
       <c r="J106" t="s">
         <v>1484</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10793,7 +10819,7 @@
       <c r="J107" t="s">
         <v>1484</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10834,7 +10860,7 @@
       <c r="J108" t="s">
         <v>1484</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10875,7 +10901,7 @@
       <c r="J109" t="s">
         <v>1484</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10928,7 +10954,7 @@
       <c r="J110" t="s">
         <v>1484</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10984,7 +11010,7 @@
       <c r="J111" t="s">
         <v>1484</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11002,7 +11028,7 @@
       <c r="R111" t="s">
         <v>1667</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11040,7 +11066,7 @@
       <c r="J112" t="s">
         <v>1484</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11099,7 +11125,7 @@
       <c r="J113" t="s">
         <v>1484</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11143,7 +11169,7 @@
       <c r="J114" t="s">
         <v>1484</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11187,7 +11213,7 @@
       <c r="J115" t="s">
         <v>1484</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11205,7 +11231,7 @@
       <c r="R115" t="s">
         <v>1669</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11243,7 +11269,7 @@
       <c r="J116" t="s">
         <v>1484</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11302,7 +11328,7 @@
       <c r="J117" t="s">
         <v>1484</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11346,7 +11372,7 @@
       <c r="J118" t="s">
         <v>1484</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11393,7 +11419,7 @@
       <c r="J119" t="s">
         <v>1484</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11434,7 +11460,7 @@
       <c r="J120" t="s">
         <v>1484</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11478,7 +11504,7 @@
       <c r="J121" t="s">
         <v>1484</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11525,7 +11551,7 @@
       <c r="J122" t="s">
         <v>1484</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11575,7 +11601,7 @@
       <c r="J123" t="s">
         <v>1484</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11619,7 +11645,7 @@
       <c r="J124" t="s">
         <v>1484</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11663,7 +11689,7 @@
       <c r="J125" t="s">
         <v>1484</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11681,7 +11707,7 @@
       <c r="R125" t="s">
         <v>1671</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11716,7 +11742,7 @@
       <c r="J126" t="s">
         <v>1484</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11734,7 +11760,7 @@
       <c r="R126" t="s">
         <v>1672</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11769,7 +11795,7 @@
       <c r="J127" t="s">
         <v>1484</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11825,7 +11851,7 @@
       <c r="J128" t="s">
         <v>1484</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11866,7 +11892,7 @@
       <c r="J129" t="s">
         <v>1484</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11907,7 +11933,7 @@
       <c r="J130" t="s">
         <v>1484</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11948,7 +11974,7 @@
       <c r="J131" t="s">
         <v>1484</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11992,7 +12018,7 @@
       <c r="J132" t="s">
         <v>1484</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12033,7 +12059,7 @@
       <c r="J133" t="s">
         <v>1484</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12051,7 +12077,7 @@
       <c r="R133" t="s">
         <v>1658</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12086,7 +12112,7 @@
       <c r="J134" t="s">
         <v>1484</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12104,7 +12130,7 @@
       <c r="R134" t="s">
         <v>1658</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12139,7 +12165,7 @@
       <c r="J135" t="s">
         <v>1484</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12180,7 +12206,7 @@
       <c r="J136" t="s">
         <v>1484</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12221,7 +12247,7 @@
       <c r="J137" t="s">
         <v>1484</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12262,7 +12288,7 @@
       <c r="J138" t="s">
         <v>1484</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12303,7 +12329,7 @@
       <c r="J139" t="s">
         <v>1484</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12350,7 +12376,7 @@
       <c r="J140" t="s">
         <v>1484</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12391,7 +12417,7 @@
       <c r="J141" t="s">
         <v>1484</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12432,7 +12458,7 @@
       <c r="J142" t="s">
         <v>1484</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12476,7 +12502,7 @@
       <c r="J143" t="s">
         <v>1484</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12494,7 +12520,7 @@
       <c r="R143" t="s">
         <v>1658</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12529,7 +12555,7 @@
       <c r="J144" t="s">
         <v>1484</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12547,7 +12573,7 @@
       <c r="R144" t="s">
         <v>1658</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12582,7 +12608,7 @@
       <c r="J145" t="s">
         <v>1484</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12600,7 +12626,7 @@
       <c r="R145" t="s">
         <v>1658</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12635,7 +12661,7 @@
       <c r="J146" t="s">
         <v>1484</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12653,7 +12679,7 @@
       <c r="R146" t="s">
         <v>1666</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12688,7 +12714,7 @@
       <c r="J147" t="s">
         <v>1484</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12706,7 +12732,7 @@
       <c r="R147" t="s">
         <v>1673</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12741,7 +12767,7 @@
       <c r="J148" t="s">
         <v>1484</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12782,7 +12808,7 @@
       <c r="J149" t="s">
         <v>1484</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12800,7 +12826,7 @@
       <c r="R149" t="s">
         <v>1658</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12835,7 +12861,7 @@
       <c r="J150" t="s">
         <v>1484</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12853,7 +12879,7 @@
       <c r="R150" t="s">
         <v>1658</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12888,7 +12914,7 @@
       <c r="J151" t="s">
         <v>1484</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12906,7 +12932,7 @@
       <c r="R151" t="s">
         <v>1674</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12941,7 +12967,7 @@
       <c r="J152" t="s">
         <v>1484</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12959,7 +12985,7 @@
       <c r="R152" t="s">
         <v>1675</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -12994,7 +13020,7 @@
       <c r="J153" t="s">
         <v>1484</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13003,7 +13029,7 @@
       <c r="M153" t="s">
         <v>1551</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13044,7 +13070,7 @@
       <c r="J154" t="s">
         <v>1484</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13085,7 +13111,7 @@
       <c r="J155" t="s">
         <v>1484</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13126,7 +13152,7 @@
       <c r="J156" t="s">
         <v>1484</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13167,7 +13193,7 @@
       <c r="J157" t="s">
         <v>1484</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13208,7 +13234,7 @@
       <c r="J158" t="s">
         <v>1484</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13249,7 +13275,7 @@
       <c r="J159" t="s">
         <v>1484</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13290,7 +13316,7 @@
       <c r="J160" t="s">
         <v>1484</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13331,7 +13357,7 @@
       <c r="J161" t="s">
         <v>1484</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13372,7 +13398,7 @@
       <c r="J162" t="s">
         <v>1484</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13390,7 +13416,7 @@
       <c r="R162" t="s">
         <v>1661</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13425,7 +13451,7 @@
       <c r="J163" t="s">
         <v>1484</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13443,7 +13469,7 @@
       <c r="R163" t="s">
         <v>1658</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13478,7 +13504,7 @@
       <c r="J164" t="s">
         <v>1484</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13522,7 +13548,7 @@
       <c r="J165" t="s">
         <v>1484</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13563,7 +13589,7 @@
       <c r="J166" t="s">
         <v>1484</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13581,7 +13607,7 @@
       <c r="R166" t="s">
         <v>1676</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13616,7 +13642,7 @@
       <c r="J167" t="s">
         <v>1484</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13660,7 +13686,7 @@
       <c r="J168" t="s">
         <v>1484</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13704,7 +13730,7 @@
       <c r="J169" t="s">
         <v>1484</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13745,7 +13771,7 @@
       <c r="J170" t="s">
         <v>1484</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13786,7 +13812,7 @@
       <c r="J171" t="s">
         <v>1484</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13827,7 +13853,7 @@
       <c r="J172" t="s">
         <v>1484</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13868,7 +13894,7 @@
       <c r="J173" t="s">
         <v>1484</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13909,7 +13935,7 @@
       <c r="J174" t="s">
         <v>1484</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13950,7 +13976,7 @@
       <c r="J175" t="s">
         <v>1484</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -13991,7 +14017,7 @@
       <c r="J176" t="s">
         <v>1484</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14032,7 +14058,7 @@
       <c r="J177" t="s">
         <v>1484</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14073,7 +14099,7 @@
       <c r="J178" t="s">
         <v>1484</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14091,7 +14117,7 @@
       <c r="R178" t="s">
         <v>1674</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14126,7 +14152,7 @@
       <c r="J179" t="s">
         <v>1484</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14135,7 +14161,7 @@
       <c r="M179" t="s">
         <v>1548</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14176,7 +14202,7 @@
       <c r="J180" t="s">
         <v>1484</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14217,7 +14243,7 @@
       <c r="J181" t="s">
         <v>1484</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14235,7 +14261,7 @@
       <c r="R181" t="s">
         <v>1658</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14270,7 +14296,7 @@
       <c r="J182" t="s">
         <v>1484</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14311,7 +14337,7 @@
       <c r="J183" t="s">
         <v>1484</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14352,7 +14378,7 @@
       <c r="J184" t="s">
         <v>1484</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14393,7 +14419,7 @@
       <c r="J185" t="s">
         <v>1484</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14434,7 +14460,7 @@
       <c r="J186" t="s">
         <v>1484</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14475,7 +14501,7 @@
       <c r="J187" t="s">
         <v>1484</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14516,7 +14542,7 @@
       <c r="J188" t="s">
         <v>1484</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14557,7 +14583,7 @@
       <c r="J189" t="s">
         <v>1484</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14598,7 +14624,7 @@
       <c r="J190" t="s">
         <v>1484</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14639,7 +14665,7 @@
       <c r="J191" t="s">
         <v>1484</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14680,7 +14706,7 @@
       <c r="J192" t="s">
         <v>1484</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14721,7 +14747,7 @@
       <c r="J193" t="s">
         <v>1484</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14762,7 +14788,7 @@
       <c r="J194" t="s">
         <v>1484</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14803,7 +14829,7 @@
       <c r="J195" t="s">
         <v>1484</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14821,7 +14847,7 @@
       <c r="R195" t="s">
         <v>1667</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14859,7 +14885,7 @@
       <c r="J196" t="s">
         <v>1484</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14877,7 +14903,7 @@
       <c r="R196" t="s">
         <v>1673</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14915,7 +14941,7 @@
       <c r="J197" t="s">
         <v>1484</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14956,7 +14982,7 @@
       <c r="J198" t="s">
         <v>1486</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -14997,7 +15023,7 @@
       <c r="J199" t="s">
         <v>1485</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15038,7 +15064,7 @@
       <c r="J200" t="s">
         <v>1484</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15079,7 +15105,7 @@
       <c r="J201" t="s">
         <v>1484</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15120,7 +15146,7 @@
       <c r="J202" t="s">
         <v>1484</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15138,7 +15164,7 @@
       <c r="R202" t="s">
         <v>1658</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15173,7 +15199,7 @@
       <c r="J203" t="s">
         <v>1484</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15191,7 +15217,7 @@
       <c r="R203" t="s">
         <v>1666</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15226,7 +15252,7 @@
       <c r="J204" t="s">
         <v>1484</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15241,7 +15267,7 @@
       <c r="R204" t="s">
         <v>1677</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15279,7 +15305,7 @@
       <c r="J205" t="s">
         <v>1484</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15297,7 +15323,7 @@
       <c r="R205" t="s">
         <v>1678</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15335,7 +15361,7 @@
       <c r="J206" t="s">
         <v>1484</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15353,7 +15379,7 @@
       <c r="R206" t="s">
         <v>1646</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15388,7 +15414,7 @@
       <c r="J207" t="s">
         <v>1484</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15429,7 +15455,7 @@
       <c r="J208" t="s">
         <v>1484</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15470,7 +15496,7 @@
       <c r="J209" t="s">
         <v>1484</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15511,7 +15537,7 @@
       <c r="J210" t="s">
         <v>1484</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15552,7 +15578,7 @@
       <c r="J211" t="s">
         <v>1484</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15593,7 +15619,7 @@
       <c r="J212" t="s">
         <v>1484</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15634,7 +15660,7 @@
       <c r="J213" t="s">
         <v>1484</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15675,7 +15701,7 @@
       <c r="J214" t="s">
         <v>1484</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15693,7 +15719,7 @@
       <c r="R214" t="s">
         <v>1679</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15728,7 +15754,7 @@
       <c r="J215" t="s">
         <v>1484</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15769,7 +15795,7 @@
       <c r="J216" t="s">
         <v>1484</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15810,7 +15836,7 @@
       <c r="J217" t="s">
         <v>1484</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15851,7 +15877,7 @@
       <c r="J218" t="s">
         <v>1484</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15892,7 +15918,7 @@
       <c r="J219" t="s">
         <v>1484</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15933,7 +15959,7 @@
       <c r="J220" t="s">
         <v>1484</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -15974,7 +16000,7 @@
       <c r="J221" t="s">
         <v>1484</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16015,7 +16041,7 @@
       <c r="J222" t="s">
         <v>1484</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16056,7 +16082,7 @@
       <c r="J223" t="s">
         <v>1484</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16097,7 +16123,7 @@
       <c r="J224" t="s">
         <v>1484</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16138,7 +16164,7 @@
       <c r="J225" t="s">
         <v>1484</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16179,7 +16205,7 @@
       <c r="J226" t="s">
         <v>1484</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16220,7 +16246,7 @@
       <c r="J227" t="s">
         <v>1484</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16261,7 +16287,7 @@
       <c r="J228" t="s">
         <v>1484</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16302,7 +16328,7 @@
       <c r="J229" t="s">
         <v>1484</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16343,7 +16369,7 @@
       <c r="J230" t="s">
         <v>1484</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16384,7 +16410,7 @@
       <c r="J231" t="s">
         <v>1484</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16425,7 +16451,7 @@
       <c r="J232" t="s">
         <v>1484</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16466,7 +16492,7 @@
       <c r="J233" t="s">
         <v>1484</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16507,7 +16533,7 @@
       <c r="J234" t="s">
         <v>1484</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16548,7 +16574,7 @@
       <c r="J235" t="s">
         <v>1484</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16589,7 +16615,7 @@
       <c r="J236" t="s">
         <v>1484</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16630,7 +16656,7 @@
       <c r="J237" t="s">
         <v>1484</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16671,7 +16697,7 @@
       <c r="J238" t="s">
         <v>1484</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16712,7 +16738,7 @@
       <c r="J239" t="s">
         <v>1484</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16730,7 +16756,7 @@
       <c r="R239" t="s">
         <v>1673</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16765,7 +16791,7 @@
       <c r="J240" t="s">
         <v>1484</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16806,7 +16832,7 @@
       <c r="J241" t="s">
         <v>1484</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16847,7 +16873,7 @@
       <c r="J242" t="s">
         <v>1484</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16865,7 +16891,7 @@
       <c r="R242" t="s">
         <v>1666</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16900,7 +16926,7 @@
       <c r="J243" t="s">
         <v>1484</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16941,7 +16967,7 @@
       <c r="J244" t="s">
         <v>1484</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -16982,7 +17008,7 @@
       <c r="J245" t="s">
         <v>1484</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17023,7 +17049,7 @@
       <c r="J246" t="s">
         <v>1484</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17041,7 +17067,7 @@
       <c r="R246" t="s">
         <v>1646</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17076,7 +17102,7 @@
       <c r="J247" t="s">
         <v>1484</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17117,7 +17143,7 @@
       <c r="J248" t="s">
         <v>1484</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17158,7 +17184,7 @@
       <c r="J249" t="s">
         <v>1484</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17199,7 +17225,7 @@
       <c r="J250" t="s">
         <v>1484</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17240,7 +17266,7 @@
       <c r="J251" t="s">
         <v>1484</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17281,7 +17307,7 @@
       <c r="J252" t="s">
         <v>1484</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17322,7 +17348,7 @@
       <c r="J253" t="s">
         <v>1484</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17340,7 +17366,7 @@
       <c r="R253" t="s">
         <v>1676</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17378,7 +17404,7 @@
       <c r="J254" t="s">
         <v>1484</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17419,7 +17445,7 @@
       <c r="J255" t="s">
         <v>1484</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17460,7 +17486,7 @@
       <c r="J256" t="s">
         <v>1484</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17469,7 +17495,7 @@
       <c r="M256" t="s">
         <v>1547</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17507,7 +17533,7 @@
       <c r="J257" t="s">
         <v>1484</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17516,7 +17542,7 @@
       <c r="M257" t="s">
         <v>1548</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17560,7 +17586,7 @@
       <c r="J258" t="s">
         <v>1484</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17578,7 +17604,7 @@
       <c r="R258" t="s">
         <v>1658</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17616,7 +17642,7 @@
       <c r="J259" t="s">
         <v>1484</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17634,7 +17660,7 @@
       <c r="R259" t="s">
         <v>1674</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17672,7 +17698,7 @@
       <c r="J260" t="s">
         <v>1484</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17681,7 +17707,7 @@
       <c r="M260" t="s">
         <v>1542</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17725,7 +17751,7 @@
       <c r="J261" t="s">
         <v>1484</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17743,7 +17769,7 @@
       <c r="R261" t="s">
         <v>1680</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17781,7 +17807,7 @@
       <c r="J262" t="s">
         <v>1484</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17799,7 +17825,7 @@
       <c r="R262" t="s">
         <v>1674</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17837,7 +17863,7 @@
       <c r="J263" t="s">
         <v>1484</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17846,7 +17872,7 @@
       <c r="M263" t="s">
         <v>1542</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17890,7 +17916,7 @@
       <c r="J264" t="s">
         <v>1484</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17931,7 +17957,7 @@
       <c r="J265" t="s">
         <v>1484</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17972,7 +17998,7 @@
       <c r="J266" t="s">
         <v>1484</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18013,7 +18039,7 @@
       <c r="J267" t="s">
         <v>1484</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18057,7 +18083,7 @@
       <c r="J268" t="s">
         <v>1484</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18098,7 +18124,7 @@
       <c r="J269" t="s">
         <v>1484</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18139,7 +18165,7 @@
       <c r="J270" t="s">
         <v>1484</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18180,7 +18206,7 @@
       <c r="J271" t="s">
         <v>1484</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18221,7 +18247,7 @@
       <c r="J272" t="s">
         <v>1484</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18239,7 +18265,7 @@
       <c r="R272" t="s">
         <v>1681</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18277,7 +18303,7 @@
       <c r="J273" t="s">
         <v>1484</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18321,7 +18347,7 @@
       <c r="J274" t="s">
         <v>1484</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18362,7 +18388,7 @@
       <c r="J275" t="s">
         <v>1484</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18403,7 +18429,7 @@
       <c r="J276" t="s">
         <v>1484</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18444,7 +18470,7 @@
       <c r="J277" t="s">
         <v>1484</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18485,7 +18511,7 @@
       <c r="J278" t="s">
         <v>1484</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18526,7 +18552,7 @@
       <c r="J279" t="s">
         <v>1484</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18567,7 +18593,7 @@
       <c r="J280" t="s">
         <v>1484</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18608,7 +18634,7 @@
       <c r="J281" t="s">
         <v>1484</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18649,7 +18675,7 @@
       <c r="J282" t="s">
         <v>1484</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18690,7 +18716,7 @@
       <c r="J283" t="s">
         <v>1484</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18731,7 +18757,7 @@
       <c r="J284" t="s">
         <v>1484</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18772,7 +18798,7 @@
       <c r="J285" t="s">
         <v>1484</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18813,7 +18839,7 @@
       <c r="J286" t="s">
         <v>1484</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18854,7 +18880,7 @@
       <c r="J287" t="s">
         <v>1484</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18895,7 +18921,7 @@
       <c r="J288" t="s">
         <v>1484</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18936,7 +18962,7 @@
       <c r="J289" t="s">
         <v>1484</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -18977,7 +19003,7 @@
       <c r="J290" t="s">
         <v>1484</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19018,7 +19044,7 @@
       <c r="J291" t="s">
         <v>1484</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19059,7 +19085,7 @@
       <c r="J292" t="s">
         <v>1484</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19100,7 +19126,7 @@
       <c r="J293" t="s">
         <v>1484</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19141,7 +19167,7 @@
       <c r="J294" t="s">
         <v>1484</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19182,7 +19208,7 @@
       <c r="J295" t="s">
         <v>1484</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19200,7 +19226,7 @@
       <c r="R295" t="s">
         <v>1682</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19238,7 +19264,7 @@
       <c r="J296" t="s">
         <v>1484</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19256,7 +19282,7 @@
       <c r="R296" t="s">
         <v>1658</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19294,7 +19320,7 @@
       <c r="J297" t="s">
         <v>1484</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19335,7 +19361,7 @@
       <c r="J298" t="s">
         <v>1484</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19376,7 +19402,7 @@
       <c r="J299" t="s">
         <v>1485</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19417,7 +19443,7 @@
       <c r="J300" t="s">
         <v>1484</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19458,7 +19484,7 @@
       <c r="J301" t="s">
         <v>1484</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20296,7 +20322,7 @@
       <c r="R321" t="s">
         <v>1644</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20516,7 +20542,7 @@
       <c r="R326" t="s">
         <v>1683</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21351,7 +21377,7 @@
       <c r="R346" t="s">
         <v>1684</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (19/08/2026 14:35)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5181,16 +5181,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5206,7 +5198,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5214,30 +5206,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5537,73 +5511,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5638,7 +5612,7 @@
       <c r="J2" t="s">
         <v>1484</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5682,7 +5656,7 @@
       <c r="J3" t="s">
         <v>1484</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5726,7 +5700,7 @@
       <c r="J4" t="s">
         <v>1484</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5744,7 +5718,7 @@
       <c r="R4" t="s">
         <v>1641</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5782,7 +5756,7 @@
       <c r="J5" t="s">
         <v>1485</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5832,7 +5806,7 @@
       <c r="J6" t="s">
         <v>1484</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5879,7 +5853,7 @@
       <c r="J7" t="s">
         <v>1484</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5926,7 +5900,7 @@
       <c r="J8" t="s">
         <v>1484</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5973,7 +5947,7 @@
       <c r="J9" t="s">
         <v>1484</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6020,7 +5994,7 @@
       <c r="J10" t="s">
         <v>1484</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6067,7 +6041,7 @@
       <c r="J11" t="s">
         <v>1484</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6114,7 +6088,7 @@
       <c r="J12" t="s">
         <v>1484</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6158,7 +6132,7 @@
       <c r="J13" t="s">
         <v>1484</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6176,7 +6150,7 @@
       <c r="R13" t="s">
         <v>1642</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6214,7 +6188,7 @@
       <c r="J14" t="s">
         <v>1484</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6232,7 +6206,7 @@
       <c r="R14" t="s">
         <v>1643</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6270,7 +6244,7 @@
       <c r="J15" t="s">
         <v>1484</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6288,7 +6262,7 @@
       <c r="R15" t="s">
         <v>1643</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6326,7 +6300,7 @@
       <c r="J16" t="s">
         <v>1484</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6370,7 +6344,7 @@
       <c r="J17" t="s">
         <v>1484</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6414,7 +6388,7 @@
       <c r="J18" t="s">
         <v>1484</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6432,7 +6406,7 @@
       <c r="R18" t="s">
         <v>1644</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6473,7 +6447,7 @@
       <c r="J19" t="s">
         <v>1484</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6517,7 +6491,7 @@
       <c r="J20" t="s">
         <v>1484</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6561,7 +6535,7 @@
       <c r="J21" t="s">
         <v>1484</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6579,7 +6553,7 @@
       <c r="R21" t="s">
         <v>1643</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6620,7 +6594,7 @@
       <c r="J22" t="s">
         <v>1484</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6638,7 +6612,7 @@
       <c r="R22" t="s">
         <v>1645</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6679,7 +6653,7 @@
       <c r="J23" t="s">
         <v>1484</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6697,7 +6671,7 @@
       <c r="R23" t="s">
         <v>1646</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6738,7 +6712,7 @@
       <c r="J24" t="s">
         <v>1484</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6782,7 +6756,7 @@
       <c r="J25" t="s">
         <v>1484</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6823,7 +6797,7 @@
       <c r="J26" t="s">
         <v>1486</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6841,7 +6815,7 @@
       <c r="R26" t="s">
         <v>1647</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6876,7 +6850,7 @@
       <c r="J27" t="s">
         <v>1484</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6894,7 +6868,7 @@
       <c r="R27" t="s">
         <v>1648</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6935,7 +6909,7 @@
       <c r="J28" t="s">
         <v>1484</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6979,7 +6953,7 @@
       <c r="J29" t="s">
         <v>1484</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7023,7 +6997,7 @@
       <c r="J30" t="s">
         <v>1484</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7067,7 +7041,7 @@
       <c r="J31" t="s">
         <v>1484</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7085,7 +7059,7 @@
       <c r="R31" t="s">
         <v>1649</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7126,7 +7100,7 @@
       <c r="J32" t="s">
         <v>1484</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7170,7 +7144,7 @@
       <c r="J33" t="s">
         <v>1484</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7188,7 +7162,7 @@
       <c r="R33" t="s">
         <v>1650</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7229,7 +7203,7 @@
       <c r="J34" t="s">
         <v>1484</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7273,7 +7247,7 @@
       <c r="J35" t="s">
         <v>1484</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7291,7 +7265,7 @@
       <c r="R35" t="s">
         <v>1651</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7332,7 +7306,7 @@
       <c r="J36" t="s">
         <v>1484</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7350,7 +7324,7 @@
       <c r="R36" t="s">
         <v>1651</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7391,7 +7365,7 @@
       <c r="J37" t="s">
         <v>1484</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7409,7 +7383,7 @@
       <c r="R37" t="s">
         <v>1651</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7450,7 +7424,7 @@
       <c r="J38" t="s">
         <v>1484</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7468,7 +7442,7 @@
       <c r="R38" t="s">
         <v>1651</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7509,7 +7483,7 @@
       <c r="J39" t="s">
         <v>1484</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7527,7 +7501,7 @@
       <c r="R39" t="s">
         <v>1651</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7568,7 +7542,7 @@
       <c r="J40" t="s">
         <v>1484</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7586,7 +7560,7 @@
       <c r="R40" t="s">
         <v>1652</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7627,7 +7601,7 @@
       <c r="J41" t="s">
         <v>1484</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7645,7 +7619,7 @@
       <c r="R41" t="s">
         <v>1643</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7683,7 +7657,7 @@
       <c r="J42" t="s">
         <v>1484</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7701,7 +7675,7 @@
       <c r="R42" t="s">
         <v>1651</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7742,7 +7716,7 @@
       <c r="J43" t="s">
         <v>1484</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7786,7 +7760,7 @@
       <c r="J44" t="s">
         <v>1484</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7804,7 +7778,7 @@
       <c r="R44" t="s">
         <v>1653</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7845,7 +7819,7 @@
       <c r="J45" t="s">
         <v>1484</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7863,7 +7837,7 @@
       <c r="R45" t="s">
         <v>1654</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7901,7 +7875,7 @@
       <c r="J46" t="s">
         <v>1484</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7945,7 +7919,7 @@
       <c r="J47" t="s">
         <v>1484</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7963,7 +7937,7 @@
       <c r="R47" t="s">
         <v>1655</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8004,7 +7978,7 @@
       <c r="J48" t="s">
         <v>1484</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8048,7 +8022,7 @@
       <c r="J49" t="s">
         <v>1484</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8092,7 +8066,7 @@
       <c r="J50" t="s">
         <v>1484</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8136,7 +8110,7 @@
       <c r="J51" t="s">
         <v>1484</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8183,7 +8157,7 @@
       <c r="J52" t="s">
         <v>1484</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8227,7 +8201,7 @@
       <c r="J53" t="s">
         <v>1484</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8271,7 +8245,7 @@
       <c r="J54" t="s">
         <v>1484</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8315,7 +8289,7 @@
       <c r="J55" t="s">
         <v>1484</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8365,7 +8339,7 @@
       <c r="J56" t="s">
         <v>1484</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8418,7 +8392,7 @@
       <c r="J57" t="s">
         <v>1484</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8468,7 +8442,7 @@
       <c r="J58" t="s">
         <v>1484</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8518,7 +8492,7 @@
       <c r="J59" t="s">
         <v>1484</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8536,7 +8510,7 @@
       <c r="R59" t="s">
         <v>1656</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8577,7 +8551,7 @@
       <c r="J60" t="s">
         <v>1484</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8621,7 +8595,7 @@
       <c r="J61" t="s">
         <v>1484</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8665,7 +8639,7 @@
       <c r="J62" t="s">
         <v>1484</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8709,7 +8683,7 @@
       <c r="J63" t="s">
         <v>1484</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8753,7 +8727,7 @@
       <c r="J64" t="s">
         <v>1484</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8797,7 +8771,7 @@
       <c r="J65" t="s">
         <v>1484</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8844,7 +8818,7 @@
       <c r="J66" t="s">
         <v>1484</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8862,7 +8836,7 @@
       <c r="R66" t="s">
         <v>1657</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8900,7 +8874,7 @@
       <c r="J67" t="s">
         <v>1484</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8944,7 +8918,7 @@
       <c r="J68" t="s">
         <v>1484</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8959,7 +8933,7 @@
       <c r="O68" t="s">
         <v>1560</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9003,7 +8977,7 @@
       <c r="J69" t="s">
         <v>1486</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9047,7 +9021,7 @@
       <c r="J70" t="s">
         <v>1484</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9091,7 +9065,7 @@
       <c r="J71" t="s">
         <v>1484</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9135,7 +9109,7 @@
       <c r="J72" t="s">
         <v>1484</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9179,7 +9153,7 @@
       <c r="J73" t="s">
         <v>1484</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9223,7 +9197,7 @@
       <c r="J74" t="s">
         <v>1484</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9267,7 +9241,7 @@
       <c r="J75" t="s">
         <v>1484</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9311,7 +9285,7 @@
       <c r="J76" t="s">
         <v>1484</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9329,7 +9303,7 @@
       <c r="R76" t="s">
         <v>1658</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9367,7 +9341,7 @@
       <c r="J77" t="s">
         <v>1484</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9385,7 +9359,7 @@
       <c r="R77" t="s">
         <v>1658</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9423,7 +9397,7 @@
       <c r="J78" t="s">
         <v>1484</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9441,7 +9415,7 @@
       <c r="R78" t="s">
         <v>1658</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9479,7 +9453,7 @@
       <c r="J79" t="s">
         <v>1484</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9497,7 +9471,7 @@
       <c r="R79" t="s">
         <v>1658</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9535,7 +9509,7 @@
       <c r="J80" t="s">
         <v>1484</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9579,7 +9553,7 @@
       <c r="J81" t="s">
         <v>1484</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9623,7 +9597,7 @@
       <c r="J82" t="s">
         <v>1484</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9667,7 +9641,7 @@
       <c r="J83" t="s">
         <v>1484</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9711,7 +9685,7 @@
       <c r="J84" t="s">
         <v>1484</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9755,7 +9729,7 @@
       <c r="J85" t="s">
         <v>1484</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9773,7 +9747,7 @@
       <c r="R85" t="s">
         <v>1659</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9811,7 +9785,7 @@
       <c r="J86" t="s">
         <v>1484</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9855,7 +9829,7 @@
       <c r="J87" t="s">
         <v>1484</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9873,7 +9847,7 @@
       <c r="R87" t="s">
         <v>1660</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9911,7 +9885,7 @@
       <c r="J88" t="s">
         <v>1484</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9955,7 +9929,7 @@
       <c r="J89" t="s">
         <v>1484</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9973,7 +9947,7 @@
       <c r="R89" t="s">
         <v>1661</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10008,7 +9982,7 @@
       <c r="J90" t="s">
         <v>1484</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10026,7 +10000,7 @@
       <c r="R90" t="s">
         <v>1662</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10061,7 +10035,7 @@
       <c r="J91" t="s">
         <v>1484</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10079,7 +10053,7 @@
       <c r="R91" t="s">
         <v>1646</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10117,7 +10091,7 @@
       <c r="J92" t="s">
         <v>1484</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10138,7 +10112,7 @@
       <c r="R92" t="s">
         <v>1646</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10179,7 +10153,7 @@
       <c r="J93" t="s">
         <v>1484</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10220,7 +10194,7 @@
       <c r="J94" t="s">
         <v>1484</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10264,7 +10238,7 @@
       <c r="J95" t="s">
         <v>1484</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10308,7 +10282,7 @@
       <c r="J96" t="s">
         <v>1484</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10326,7 +10300,7 @@
       <c r="R96" t="s">
         <v>1663</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10364,7 +10338,7 @@
       <c r="J97" t="s">
         <v>1484</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10379,7 +10353,7 @@
       <c r="R97" t="s">
         <v>1663</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10420,7 +10394,7 @@
       <c r="J98" t="s">
         <v>1484</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10438,7 +10412,7 @@
       <c r="R98" t="s">
         <v>1664</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10476,7 +10450,7 @@
       <c r="J99" t="s">
         <v>1484</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10494,7 +10468,7 @@
       <c r="R99" t="s">
         <v>1665</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10532,7 +10506,7 @@
       <c r="J100" t="s">
         <v>1484</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10573,7 +10547,7 @@
       <c r="J101" t="s">
         <v>1484</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10614,7 +10588,7 @@
       <c r="J102" t="s">
         <v>1484</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10655,7 +10629,7 @@
       <c r="J103" t="s">
         <v>1484</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10696,7 +10670,7 @@
       <c r="J104" t="s">
         <v>1484</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10737,7 +10711,7 @@
       <c r="J105" t="s">
         <v>1484</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10778,7 +10752,7 @@
       <c r="J106" t="s">
         <v>1484</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10819,7 +10793,7 @@
       <c r="J107" t="s">
         <v>1484</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10860,7 +10834,7 @@
       <c r="J108" t="s">
         <v>1484</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10901,7 +10875,7 @@
       <c r="J109" t="s">
         <v>1484</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10954,7 +10928,7 @@
       <c r="J110" t="s">
         <v>1484</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11010,7 +10984,7 @@
       <c r="J111" t="s">
         <v>1484</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11028,7 +11002,7 @@
       <c r="R111" t="s">
         <v>1667</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11066,7 +11040,7 @@
       <c r="J112" t="s">
         <v>1484</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11125,7 +11099,7 @@
       <c r="J113" t="s">
         <v>1484</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11169,7 +11143,7 @@
       <c r="J114" t="s">
         <v>1484</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11213,7 +11187,7 @@
       <c r="J115" t="s">
         <v>1484</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11231,7 +11205,7 @@
       <c r="R115" t="s">
         <v>1669</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11269,7 +11243,7 @@
       <c r="J116" t="s">
         <v>1484</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11328,7 +11302,7 @@
       <c r="J117" t="s">
         <v>1484</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11372,7 +11346,7 @@
       <c r="J118" t="s">
         <v>1484</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11419,7 +11393,7 @@
       <c r="J119" t="s">
         <v>1484</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11460,7 +11434,7 @@
       <c r="J120" t="s">
         <v>1484</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11504,7 +11478,7 @@
       <c r="J121" t="s">
         <v>1484</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11551,7 +11525,7 @@
       <c r="J122" t="s">
         <v>1484</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11601,7 +11575,7 @@
       <c r="J123" t="s">
         <v>1484</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11645,7 +11619,7 @@
       <c r="J124" t="s">
         <v>1484</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11689,7 +11663,7 @@
       <c r="J125" t="s">
         <v>1484</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11707,7 +11681,7 @@
       <c r="R125" t="s">
         <v>1671</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11742,7 +11716,7 @@
       <c r="J126" t="s">
         <v>1484</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11760,7 +11734,7 @@
       <c r="R126" t="s">
         <v>1672</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11795,7 +11769,7 @@
       <c r="J127" t="s">
         <v>1484</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11851,7 +11825,7 @@
       <c r="J128" t="s">
         <v>1484</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11892,7 +11866,7 @@
       <c r="J129" t="s">
         <v>1484</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11933,7 +11907,7 @@
       <c r="J130" t="s">
         <v>1484</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11974,7 +11948,7 @@
       <c r="J131" t="s">
         <v>1484</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12018,7 +11992,7 @@
       <c r="J132" t="s">
         <v>1484</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12059,7 +12033,7 @@
       <c r="J133" t="s">
         <v>1484</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12077,7 +12051,7 @@
       <c r="R133" t="s">
         <v>1658</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12112,7 +12086,7 @@
       <c r="J134" t="s">
         <v>1484</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12130,7 +12104,7 @@
       <c r="R134" t="s">
         <v>1658</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12165,7 +12139,7 @@
       <c r="J135" t="s">
         <v>1484</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12206,7 +12180,7 @@
       <c r="J136" t="s">
         <v>1484</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12247,7 +12221,7 @@
       <c r="J137" t="s">
         <v>1484</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12288,7 +12262,7 @@
       <c r="J138" t="s">
         <v>1484</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12329,7 +12303,7 @@
       <c r="J139" t="s">
         <v>1484</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12376,7 +12350,7 @@
       <c r="J140" t="s">
         <v>1484</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12417,7 +12391,7 @@
       <c r="J141" t="s">
         <v>1484</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12458,7 +12432,7 @@
       <c r="J142" t="s">
         <v>1484</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12502,7 +12476,7 @@
       <c r="J143" t="s">
         <v>1484</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12520,7 +12494,7 @@
       <c r="R143" t="s">
         <v>1658</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12555,7 +12529,7 @@
       <c r="J144" t="s">
         <v>1484</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12573,7 +12547,7 @@
       <c r="R144" t="s">
         <v>1658</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12608,7 +12582,7 @@
       <c r="J145" t="s">
         <v>1484</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12626,7 +12600,7 @@
       <c r="R145" t="s">
         <v>1658</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12661,7 +12635,7 @@
       <c r="J146" t="s">
         <v>1484</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12679,7 +12653,7 @@
       <c r="R146" t="s">
         <v>1666</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12714,7 +12688,7 @@
       <c r="J147" t="s">
         <v>1484</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12732,7 +12706,7 @@
       <c r="R147" t="s">
         <v>1673</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12767,7 +12741,7 @@
       <c r="J148" t="s">
         <v>1484</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12808,7 +12782,7 @@
       <c r="J149" t="s">
         <v>1484</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12826,7 +12800,7 @@
       <c r="R149" t="s">
         <v>1658</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12861,7 +12835,7 @@
       <c r="J150" t="s">
         <v>1484</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12879,7 +12853,7 @@
       <c r="R150" t="s">
         <v>1658</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12914,7 +12888,7 @@
       <c r="J151" t="s">
         <v>1484</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12932,7 +12906,7 @@
       <c r="R151" t="s">
         <v>1674</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12967,7 +12941,7 @@
       <c r="J152" t="s">
         <v>1484</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12985,7 +12959,7 @@
       <c r="R152" t="s">
         <v>1675</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13020,7 +12994,7 @@
       <c r="J153" t="s">
         <v>1484</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13029,7 +13003,7 @@
       <c r="M153" t="s">
         <v>1551</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13070,7 +13044,7 @@
       <c r="J154" t="s">
         <v>1484</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13111,7 +13085,7 @@
       <c r="J155" t="s">
         <v>1484</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13152,7 +13126,7 @@
       <c r="J156" t="s">
         <v>1484</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13193,7 +13167,7 @@
       <c r="J157" t="s">
         <v>1484</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13234,7 +13208,7 @@
       <c r="J158" t="s">
         <v>1484</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13275,7 +13249,7 @@
       <c r="J159" t="s">
         <v>1484</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13316,7 +13290,7 @@
       <c r="J160" t="s">
         <v>1484</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13357,7 +13331,7 @@
       <c r="J161" t="s">
         <v>1484</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13398,7 +13372,7 @@
       <c r="J162" t="s">
         <v>1484</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13416,7 +13390,7 @@
       <c r="R162" t="s">
         <v>1661</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13451,7 +13425,7 @@
       <c r="J163" t="s">
         <v>1484</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13469,7 +13443,7 @@
       <c r="R163" t="s">
         <v>1658</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13504,7 +13478,7 @@
       <c r="J164" t="s">
         <v>1484</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13548,7 +13522,7 @@
       <c r="J165" t="s">
         <v>1484</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13589,7 +13563,7 @@
       <c r="J166" t="s">
         <v>1484</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13607,7 +13581,7 @@
       <c r="R166" t="s">
         <v>1676</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13642,7 +13616,7 @@
       <c r="J167" t="s">
         <v>1484</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13686,7 +13660,7 @@
       <c r="J168" t="s">
         <v>1484</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13730,7 +13704,7 @@
       <c r="J169" t="s">
         <v>1484</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13771,7 +13745,7 @@
       <c r="J170" t="s">
         <v>1484</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13812,7 +13786,7 @@
       <c r="J171" t="s">
         <v>1484</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13853,7 +13827,7 @@
       <c r="J172" t="s">
         <v>1484</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13894,7 +13868,7 @@
       <c r="J173" t="s">
         <v>1484</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13935,7 +13909,7 @@
       <c r="J174" t="s">
         <v>1484</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13976,7 +13950,7 @@
       <c r="J175" t="s">
         <v>1484</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14017,7 +13991,7 @@
       <c r="J176" t="s">
         <v>1484</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14058,7 +14032,7 @@
       <c r="J177" t="s">
         <v>1484</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14099,7 +14073,7 @@
       <c r="J178" t="s">
         <v>1484</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14117,7 +14091,7 @@
       <c r="R178" t="s">
         <v>1674</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14152,7 +14126,7 @@
       <c r="J179" t="s">
         <v>1484</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14161,7 +14135,7 @@
       <c r="M179" t="s">
         <v>1548</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14202,7 +14176,7 @@
       <c r="J180" t="s">
         <v>1484</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14243,7 +14217,7 @@
       <c r="J181" t="s">
         <v>1484</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14261,7 +14235,7 @@
       <c r="R181" t="s">
         <v>1658</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14296,7 +14270,7 @@
       <c r="J182" t="s">
         <v>1484</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14337,7 +14311,7 @@
       <c r="J183" t="s">
         <v>1484</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14378,7 +14352,7 @@
       <c r="J184" t="s">
         <v>1484</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14419,7 +14393,7 @@
       <c r="J185" t="s">
         <v>1484</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14460,7 +14434,7 @@
       <c r="J186" t="s">
         <v>1484</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14501,7 +14475,7 @@
       <c r="J187" t="s">
         <v>1484</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14542,7 +14516,7 @@
       <c r="J188" t="s">
         <v>1484</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14583,7 +14557,7 @@
       <c r="J189" t="s">
         <v>1484</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14624,7 +14598,7 @@
       <c r="J190" t="s">
         <v>1484</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14665,7 +14639,7 @@
       <c r="J191" t="s">
         <v>1484</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14706,7 +14680,7 @@
       <c r="J192" t="s">
         <v>1484</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14747,7 +14721,7 @@
       <c r="J193" t="s">
         <v>1484</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14788,7 +14762,7 @@
       <c r="J194" t="s">
         <v>1484</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14829,7 +14803,7 @@
       <c r="J195" t="s">
         <v>1484</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14847,7 +14821,7 @@
       <c r="R195" t="s">
         <v>1667</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14885,7 +14859,7 @@
       <c r="J196" t="s">
         <v>1484</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14903,7 +14877,7 @@
       <c r="R196" t="s">
         <v>1673</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14941,7 +14915,7 @@
       <c r="J197" t="s">
         <v>1484</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14982,7 +14956,7 @@
       <c r="J198" t="s">
         <v>1486</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15023,7 +14997,7 @@
       <c r="J199" t="s">
         <v>1485</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15064,7 +15038,7 @@
       <c r="J200" t="s">
         <v>1484</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15105,7 +15079,7 @@
       <c r="J201" t="s">
         <v>1484</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15146,7 +15120,7 @@
       <c r="J202" t="s">
         <v>1484</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15164,7 +15138,7 @@
       <c r="R202" t="s">
         <v>1658</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15199,7 +15173,7 @@
       <c r="J203" t="s">
         <v>1484</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15217,7 +15191,7 @@
       <c r="R203" t="s">
         <v>1666</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15252,7 +15226,7 @@
       <c r="J204" t="s">
         <v>1484</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15267,7 +15241,7 @@
       <c r="R204" t="s">
         <v>1677</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15305,7 +15279,7 @@
       <c r="J205" t="s">
         <v>1484</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15323,7 +15297,7 @@
       <c r="R205" t="s">
         <v>1678</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15361,7 +15335,7 @@
       <c r="J206" t="s">
         <v>1484</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15379,7 +15353,7 @@
       <c r="R206" t="s">
         <v>1646</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15414,7 +15388,7 @@
       <c r="J207" t="s">
         <v>1484</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15455,7 +15429,7 @@
       <c r="J208" t="s">
         <v>1484</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15496,7 +15470,7 @@
       <c r="J209" t="s">
         <v>1484</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15537,7 +15511,7 @@
       <c r="J210" t="s">
         <v>1484</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15578,7 +15552,7 @@
       <c r="J211" t="s">
         <v>1484</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15619,7 +15593,7 @@
       <c r="J212" t="s">
         <v>1484</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15660,7 +15634,7 @@
       <c r="J213" t="s">
         <v>1484</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15701,7 +15675,7 @@
       <c r="J214" t="s">
         <v>1484</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15719,7 +15693,7 @@
       <c r="R214" t="s">
         <v>1679</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15754,7 +15728,7 @@
       <c r="J215" t="s">
         <v>1484</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15795,7 +15769,7 @@
       <c r="J216" t="s">
         <v>1484</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15836,7 +15810,7 @@
       <c r="J217" t="s">
         <v>1484</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15877,7 +15851,7 @@
       <c r="J218" t="s">
         <v>1484</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15918,7 +15892,7 @@
       <c r="J219" t="s">
         <v>1484</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15959,7 +15933,7 @@
       <c r="J220" t="s">
         <v>1484</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16000,7 +15974,7 @@
       <c r="J221" t="s">
         <v>1484</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16041,7 +16015,7 @@
       <c r="J222" t="s">
         <v>1484</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16082,7 +16056,7 @@
       <c r="J223" t="s">
         <v>1484</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16123,7 +16097,7 @@
       <c r="J224" t="s">
         <v>1484</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16164,7 +16138,7 @@
       <c r="J225" t="s">
         <v>1484</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16205,7 +16179,7 @@
       <c r="J226" t="s">
         <v>1484</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16246,7 +16220,7 @@
       <c r="J227" t="s">
         <v>1484</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16287,7 +16261,7 @@
       <c r="J228" t="s">
         <v>1484</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16328,7 +16302,7 @@
       <c r="J229" t="s">
         <v>1484</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16369,7 +16343,7 @@
       <c r="J230" t="s">
         <v>1484</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16410,7 +16384,7 @@
       <c r="J231" t="s">
         <v>1484</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16451,7 +16425,7 @@
       <c r="J232" t="s">
         <v>1484</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16492,7 +16466,7 @@
       <c r="J233" t="s">
         <v>1484</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16533,7 +16507,7 @@
       <c r="J234" t="s">
         <v>1484</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16574,7 +16548,7 @@
       <c r="J235" t="s">
         <v>1484</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16615,7 +16589,7 @@
       <c r="J236" t="s">
         <v>1484</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16656,7 +16630,7 @@
       <c r="J237" t="s">
         <v>1484</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16697,7 +16671,7 @@
       <c r="J238" t="s">
         <v>1484</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16738,7 +16712,7 @@
       <c r="J239" t="s">
         <v>1484</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16756,7 +16730,7 @@
       <c r="R239" t="s">
         <v>1673</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16791,7 +16765,7 @@
       <c r="J240" t="s">
         <v>1484</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16832,7 +16806,7 @@
       <c r="J241" t="s">
         <v>1484</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16873,7 +16847,7 @@
       <c r="J242" t="s">
         <v>1484</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16891,7 +16865,7 @@
       <c r="R242" t="s">
         <v>1666</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16926,7 +16900,7 @@
       <c r="J243" t="s">
         <v>1484</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16967,7 +16941,7 @@
       <c r="J244" t="s">
         <v>1484</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17008,7 +16982,7 @@
       <c r="J245" t="s">
         <v>1484</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17049,7 +17023,7 @@
       <c r="J246" t="s">
         <v>1484</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17067,7 +17041,7 @@
       <c r="R246" t="s">
         <v>1646</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17102,7 +17076,7 @@
       <c r="J247" t="s">
         <v>1484</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17143,7 +17117,7 @@
       <c r="J248" t="s">
         <v>1484</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17184,7 +17158,7 @@
       <c r="J249" t="s">
         <v>1484</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17225,7 +17199,7 @@
       <c r="J250" t="s">
         <v>1484</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17266,7 +17240,7 @@
       <c r="J251" t="s">
         <v>1484</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17307,7 +17281,7 @@
       <c r="J252" t="s">
         <v>1484</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17348,7 +17322,7 @@
       <c r="J253" t="s">
         <v>1484</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17366,7 +17340,7 @@
       <c r="R253" t="s">
         <v>1676</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17404,7 +17378,7 @@
       <c r="J254" t="s">
         <v>1484</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17445,7 +17419,7 @@
       <c r="J255" t="s">
         <v>1484</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17486,7 +17460,7 @@
       <c r="J256" t="s">
         <v>1484</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17495,7 +17469,7 @@
       <c r="M256" t="s">
         <v>1547</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17533,7 +17507,7 @@
       <c r="J257" t="s">
         <v>1484</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17542,7 +17516,7 @@
       <c r="M257" t="s">
         <v>1548</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17586,7 +17560,7 @@
       <c r="J258" t="s">
         <v>1484</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17604,7 +17578,7 @@
       <c r="R258" t="s">
         <v>1658</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17642,7 +17616,7 @@
       <c r="J259" t="s">
         <v>1484</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17660,7 +17634,7 @@
       <c r="R259" t="s">
         <v>1674</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17698,7 +17672,7 @@
       <c r="J260" t="s">
         <v>1484</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17707,7 +17681,7 @@
       <c r="M260" t="s">
         <v>1542</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17751,7 +17725,7 @@
       <c r="J261" t="s">
         <v>1484</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17769,7 +17743,7 @@
       <c r="R261" t="s">
         <v>1680</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17807,7 +17781,7 @@
       <c r="J262" t="s">
         <v>1484</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17825,7 +17799,7 @@
       <c r="R262" t="s">
         <v>1674</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17863,7 +17837,7 @@
       <c r="J263" t="s">
         <v>1484</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17872,7 +17846,7 @@
       <c r="M263" t="s">
         <v>1542</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17916,7 +17890,7 @@
       <c r="J264" t="s">
         <v>1484</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17957,7 +17931,7 @@
       <c r="J265" t="s">
         <v>1484</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17998,7 +17972,7 @@
       <c r="J266" t="s">
         <v>1484</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18039,7 +18013,7 @@
       <c r="J267" t="s">
         <v>1484</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18083,7 +18057,7 @@
       <c r="J268" t="s">
         <v>1484</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18124,7 +18098,7 @@
       <c r="J269" t="s">
         <v>1484</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18165,7 +18139,7 @@
       <c r="J270" t="s">
         <v>1484</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18206,7 +18180,7 @@
       <c r="J271" t="s">
         <v>1484</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18247,7 +18221,7 @@
       <c r="J272" t="s">
         <v>1484</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18265,7 +18239,7 @@
       <c r="R272" t="s">
         <v>1681</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18303,7 +18277,7 @@
       <c r="J273" t="s">
         <v>1484</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18347,7 +18321,7 @@
       <c r="J274" t="s">
         <v>1484</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18388,7 +18362,7 @@
       <c r="J275" t="s">
         <v>1484</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18429,7 +18403,7 @@
       <c r="J276" t="s">
         <v>1484</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18470,7 +18444,7 @@
       <c r="J277" t="s">
         <v>1484</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18511,7 +18485,7 @@
       <c r="J278" t="s">
         <v>1484</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18552,7 +18526,7 @@
       <c r="J279" t="s">
         <v>1484</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18593,7 +18567,7 @@
       <c r="J280" t="s">
         <v>1484</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18634,7 +18608,7 @@
       <c r="J281" t="s">
         <v>1484</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18675,7 +18649,7 @@
       <c r="J282" t="s">
         <v>1484</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18716,7 +18690,7 @@
       <c r="J283" t="s">
         <v>1484</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18757,7 +18731,7 @@
       <c r="J284" t="s">
         <v>1484</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18798,7 +18772,7 @@
       <c r="J285" t="s">
         <v>1484</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18839,7 +18813,7 @@
       <c r="J286" t="s">
         <v>1484</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18880,7 +18854,7 @@
       <c r="J287" t="s">
         <v>1484</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18921,7 +18895,7 @@
       <c r="J288" t="s">
         <v>1484</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18962,7 +18936,7 @@
       <c r="J289" t="s">
         <v>1484</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19003,7 +18977,7 @@
       <c r="J290" t="s">
         <v>1484</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19044,7 +19018,7 @@
       <c r="J291" t="s">
         <v>1484</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19085,7 +19059,7 @@
       <c r="J292" t="s">
         <v>1484</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19126,7 +19100,7 @@
       <c r="J293" t="s">
         <v>1484</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19167,7 +19141,7 @@
       <c r="J294" t="s">
         <v>1484</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19208,7 +19182,7 @@
       <c r="J295" t="s">
         <v>1484</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19226,7 +19200,7 @@
       <c r="R295" t="s">
         <v>1682</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19264,7 +19238,7 @@
       <c r="J296" t="s">
         <v>1484</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19282,7 +19256,7 @@
       <c r="R296" t="s">
         <v>1658</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19320,7 +19294,7 @@
       <c r="J297" t="s">
         <v>1484</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19361,7 +19335,7 @@
       <c r="J298" t="s">
         <v>1484</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19402,7 +19376,7 @@
       <c r="J299" t="s">
         <v>1485</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19443,7 +19417,7 @@
       <c r="J300" t="s">
         <v>1484</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19484,7 +19458,7 @@
       <c r="J301" t="s">
         <v>1484</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20322,7 +20296,7 @@
       <c r="R321" t="s">
         <v>1644</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20542,7 +20516,7 @@
       <c r="R326" t="s">
         <v>1683</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21377,7 +21351,7 @@
       <c r="R346" t="s">
         <v>1684</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (21/08/2026 09:07)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5181,8 +5181,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5198,7 +5206,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5206,12 +5214,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5511,73 +5537,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5612,7 +5638,7 @@
       <c r="J2" t="s">
         <v>1484</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5656,7 +5682,7 @@
       <c r="J3" t="s">
         <v>1484</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5700,7 +5726,7 @@
       <c r="J4" t="s">
         <v>1484</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5718,7 +5744,7 @@
       <c r="R4" t="s">
         <v>1641</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5756,7 +5782,7 @@
       <c r="J5" t="s">
         <v>1485</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5806,7 +5832,7 @@
       <c r="J6" t="s">
         <v>1484</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5853,7 +5879,7 @@
       <c r="J7" t="s">
         <v>1484</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5900,7 +5926,7 @@
       <c r="J8" t="s">
         <v>1484</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5947,7 +5973,7 @@
       <c r="J9" t="s">
         <v>1484</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -5994,7 +6020,7 @@
       <c r="J10" t="s">
         <v>1484</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6041,7 +6067,7 @@
       <c r="J11" t="s">
         <v>1484</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6088,7 +6114,7 @@
       <c r="J12" t="s">
         <v>1484</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6132,7 +6158,7 @@
       <c r="J13" t="s">
         <v>1484</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6150,7 +6176,7 @@
       <c r="R13" t="s">
         <v>1642</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6188,7 +6214,7 @@
       <c r="J14" t="s">
         <v>1484</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6206,7 +6232,7 @@
       <c r="R14" t="s">
         <v>1643</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6244,7 +6270,7 @@
       <c r="J15" t="s">
         <v>1484</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6262,7 +6288,7 @@
       <c r="R15" t="s">
         <v>1643</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6300,7 +6326,7 @@
       <c r="J16" t="s">
         <v>1484</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6344,7 +6370,7 @@
       <c r="J17" t="s">
         <v>1484</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6388,7 +6414,7 @@
       <c r="J18" t="s">
         <v>1484</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6406,7 +6432,7 @@
       <c r="R18" t="s">
         <v>1644</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6447,7 +6473,7 @@
       <c r="J19" t="s">
         <v>1484</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6491,7 +6517,7 @@
       <c r="J20" t="s">
         <v>1484</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6535,7 +6561,7 @@
       <c r="J21" t="s">
         <v>1484</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6553,7 +6579,7 @@
       <c r="R21" t="s">
         <v>1643</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6594,7 +6620,7 @@
       <c r="J22" t="s">
         <v>1484</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6612,7 +6638,7 @@
       <c r="R22" t="s">
         <v>1645</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6653,7 +6679,7 @@
       <c r="J23" t="s">
         <v>1484</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6671,7 +6697,7 @@
       <c r="R23" t="s">
         <v>1646</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6712,7 +6738,7 @@
       <c r="J24" t="s">
         <v>1484</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6756,7 +6782,7 @@
       <c r="J25" t="s">
         <v>1484</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6797,7 +6823,7 @@
       <c r="J26" t="s">
         <v>1486</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6815,7 +6841,7 @@
       <c r="R26" t="s">
         <v>1647</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6850,7 +6876,7 @@
       <c r="J27" t="s">
         <v>1484</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6868,7 +6894,7 @@
       <c r="R27" t="s">
         <v>1648</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6909,7 +6935,7 @@
       <c r="J28" t="s">
         <v>1484</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6953,7 +6979,7 @@
       <c r="J29" t="s">
         <v>1484</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -6997,7 +7023,7 @@
       <c r="J30" t="s">
         <v>1484</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7041,7 +7067,7 @@
       <c r="J31" t="s">
         <v>1484</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7059,7 +7085,7 @@
       <c r="R31" t="s">
         <v>1649</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7100,7 +7126,7 @@
       <c r="J32" t="s">
         <v>1484</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7144,7 +7170,7 @@
       <c r="J33" t="s">
         <v>1484</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7162,7 +7188,7 @@
       <c r="R33" t="s">
         <v>1650</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7203,7 +7229,7 @@
       <c r="J34" t="s">
         <v>1484</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7247,7 +7273,7 @@
       <c r="J35" t="s">
         <v>1484</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7265,7 +7291,7 @@
       <c r="R35" t="s">
         <v>1651</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7306,7 +7332,7 @@
       <c r="J36" t="s">
         <v>1484</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7324,7 +7350,7 @@
       <c r="R36" t="s">
         <v>1651</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7365,7 +7391,7 @@
       <c r="J37" t="s">
         <v>1484</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7383,7 +7409,7 @@
       <c r="R37" t="s">
         <v>1651</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7424,7 +7450,7 @@
       <c r="J38" t="s">
         <v>1484</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7442,7 +7468,7 @@
       <c r="R38" t="s">
         <v>1651</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7483,7 +7509,7 @@
       <c r="J39" t="s">
         <v>1484</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7501,7 +7527,7 @@
       <c r="R39" t="s">
         <v>1651</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7542,7 +7568,7 @@
       <c r="J40" t="s">
         <v>1484</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7560,7 +7586,7 @@
       <c r="R40" t="s">
         <v>1652</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7601,7 +7627,7 @@
       <c r="J41" t="s">
         <v>1484</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7619,7 +7645,7 @@
       <c r="R41" t="s">
         <v>1643</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7657,7 +7683,7 @@
       <c r="J42" t="s">
         <v>1484</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7675,7 +7701,7 @@
       <c r="R42" t="s">
         <v>1651</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7716,7 +7742,7 @@
       <c r="J43" t="s">
         <v>1484</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7760,7 +7786,7 @@
       <c r="J44" t="s">
         <v>1484</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7778,7 +7804,7 @@
       <c r="R44" t="s">
         <v>1653</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7819,7 +7845,7 @@
       <c r="J45" t="s">
         <v>1484</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7837,7 +7863,7 @@
       <c r="R45" t="s">
         <v>1654</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7875,7 +7901,7 @@
       <c r="J46" t="s">
         <v>1484</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7919,7 +7945,7 @@
       <c r="J47" t="s">
         <v>1484</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7937,7 +7963,7 @@
       <c r="R47" t="s">
         <v>1655</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7978,7 +8004,7 @@
       <c r="J48" t="s">
         <v>1484</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8022,7 +8048,7 @@
       <c r="J49" t="s">
         <v>1484</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8066,7 +8092,7 @@
       <c r="J50" t="s">
         <v>1484</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8110,7 +8136,7 @@
       <c r="J51" t="s">
         <v>1484</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8157,7 +8183,7 @@
       <c r="J52" t="s">
         <v>1484</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8201,7 +8227,7 @@
       <c r="J53" t="s">
         <v>1484</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8245,7 +8271,7 @@
       <c r="J54" t="s">
         <v>1484</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8289,7 +8315,7 @@
       <c r="J55" t="s">
         <v>1484</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8339,7 +8365,7 @@
       <c r="J56" t="s">
         <v>1484</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8392,7 +8418,7 @@
       <c r="J57" t="s">
         <v>1484</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8442,7 +8468,7 @@
       <c r="J58" t="s">
         <v>1484</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8492,7 +8518,7 @@
       <c r="J59" t="s">
         <v>1484</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8510,7 +8536,7 @@
       <c r="R59" t="s">
         <v>1656</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8551,7 +8577,7 @@
       <c r="J60" t="s">
         <v>1484</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8595,7 +8621,7 @@
       <c r="J61" t="s">
         <v>1484</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8639,7 +8665,7 @@
       <c r="J62" t="s">
         <v>1484</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8683,7 +8709,7 @@
       <c r="J63" t="s">
         <v>1484</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8727,7 +8753,7 @@
       <c r="J64" t="s">
         <v>1484</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8771,7 +8797,7 @@
       <c r="J65" t="s">
         <v>1484</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8818,7 +8844,7 @@
       <c r="J66" t="s">
         <v>1484</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8836,7 +8862,7 @@
       <c r="R66" t="s">
         <v>1657</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8874,7 +8900,7 @@
       <c r="J67" t="s">
         <v>1484</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8918,7 +8944,7 @@
       <c r="J68" t="s">
         <v>1484</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8933,7 +8959,7 @@
       <c r="O68" t="s">
         <v>1560</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8977,7 +9003,7 @@
       <c r="J69" t="s">
         <v>1486</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9021,7 +9047,7 @@
       <c r="J70" t="s">
         <v>1484</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9065,7 +9091,7 @@
       <c r="J71" t="s">
         <v>1484</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9109,7 +9135,7 @@
       <c r="J72" t="s">
         <v>1484</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9153,7 +9179,7 @@
       <c r="J73" t="s">
         <v>1484</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9197,7 +9223,7 @@
       <c r="J74" t="s">
         <v>1484</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9241,7 +9267,7 @@
       <c r="J75" t="s">
         <v>1484</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9285,7 +9311,7 @@
       <c r="J76" t="s">
         <v>1484</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9303,7 +9329,7 @@
       <c r="R76" t="s">
         <v>1658</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9341,7 +9367,7 @@
       <c r="J77" t="s">
         <v>1484</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9359,7 +9385,7 @@
       <c r="R77" t="s">
         <v>1658</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9397,7 +9423,7 @@
       <c r="J78" t="s">
         <v>1484</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9415,7 +9441,7 @@
       <c r="R78" t="s">
         <v>1658</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9453,7 +9479,7 @@
       <c r="J79" t="s">
         <v>1484</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9471,7 +9497,7 @@
       <c r="R79" t="s">
         <v>1658</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9509,7 +9535,7 @@
       <c r="J80" t="s">
         <v>1484</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9553,7 +9579,7 @@
       <c r="J81" t="s">
         <v>1484</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9597,7 +9623,7 @@
       <c r="J82" t="s">
         <v>1484</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9641,7 +9667,7 @@
       <c r="J83" t="s">
         <v>1484</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9685,7 +9711,7 @@
       <c r="J84" t="s">
         <v>1484</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9729,7 +9755,7 @@
       <c r="J85" t="s">
         <v>1484</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9747,7 +9773,7 @@
       <c r="R85" t="s">
         <v>1659</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9785,7 +9811,7 @@
       <c r="J86" t="s">
         <v>1484</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9829,7 +9855,7 @@
       <c r="J87" t="s">
         <v>1484</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9847,7 +9873,7 @@
       <c r="R87" t="s">
         <v>1660</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9885,7 +9911,7 @@
       <c r="J88" t="s">
         <v>1484</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9929,7 +9955,7 @@
       <c r="J89" t="s">
         <v>1484</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9947,7 +9973,7 @@
       <c r="R89" t="s">
         <v>1661</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -9982,7 +10008,7 @@
       <c r="J90" t="s">
         <v>1484</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10000,7 +10026,7 @@
       <c r="R90" t="s">
         <v>1662</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10035,7 +10061,7 @@
       <c r="J91" t="s">
         <v>1484</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10053,7 +10079,7 @@
       <c r="R91" t="s">
         <v>1646</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10091,7 +10117,7 @@
       <c r="J92" t="s">
         <v>1484</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10112,7 +10138,7 @@
       <c r="R92" t="s">
         <v>1646</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10153,7 +10179,7 @@
       <c r="J93" t="s">
         <v>1484</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10194,7 +10220,7 @@
       <c r="J94" t="s">
         <v>1484</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10238,7 +10264,7 @@
       <c r="J95" t="s">
         <v>1484</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10282,7 +10308,7 @@
       <c r="J96" t="s">
         <v>1484</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10300,7 +10326,7 @@
       <c r="R96" t="s">
         <v>1663</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10338,7 +10364,7 @@
       <c r="J97" t="s">
         <v>1484</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10353,7 +10379,7 @@
       <c r="R97" t="s">
         <v>1663</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10394,7 +10420,7 @@
       <c r="J98" t="s">
         <v>1484</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10412,7 +10438,7 @@
       <c r="R98" t="s">
         <v>1664</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10450,7 +10476,7 @@
       <c r="J99" t="s">
         <v>1484</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10468,7 +10494,7 @@
       <c r="R99" t="s">
         <v>1665</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10506,7 +10532,7 @@
       <c r="J100" t="s">
         <v>1484</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10547,7 +10573,7 @@
       <c r="J101" t="s">
         <v>1484</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10588,7 +10614,7 @@
       <c r="J102" t="s">
         <v>1484</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10629,7 +10655,7 @@
       <c r="J103" t="s">
         <v>1484</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10670,7 +10696,7 @@
       <c r="J104" t="s">
         <v>1484</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10711,7 +10737,7 @@
       <c r="J105" t="s">
         <v>1484</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10752,7 +10778,7 @@
       <c r="J106" t="s">
         <v>1484</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10793,7 +10819,7 @@
       <c r="J107" t="s">
         <v>1484</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10834,7 +10860,7 @@
       <c r="J108" t="s">
         <v>1484</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10875,7 +10901,7 @@
       <c r="J109" t="s">
         <v>1484</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10928,7 +10954,7 @@
       <c r="J110" t="s">
         <v>1484</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10984,7 +11010,7 @@
       <c r="J111" t="s">
         <v>1484</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11002,7 +11028,7 @@
       <c r="R111" t="s">
         <v>1667</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11040,7 +11066,7 @@
       <c r="J112" t="s">
         <v>1484</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11099,7 +11125,7 @@
       <c r="J113" t="s">
         <v>1484</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11143,7 +11169,7 @@
       <c r="J114" t="s">
         <v>1484</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11187,7 +11213,7 @@
       <c r="J115" t="s">
         <v>1484</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11205,7 +11231,7 @@
       <c r="R115" t="s">
         <v>1669</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11243,7 +11269,7 @@
       <c r="J116" t="s">
         <v>1484</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11302,7 +11328,7 @@
       <c r="J117" t="s">
         <v>1484</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11346,7 +11372,7 @@
       <c r="J118" t="s">
         <v>1484</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11393,7 +11419,7 @@
       <c r="J119" t="s">
         <v>1484</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11434,7 +11460,7 @@
       <c r="J120" t="s">
         <v>1484</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11478,7 +11504,7 @@
       <c r="J121" t="s">
         <v>1484</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11525,7 +11551,7 @@
       <c r="J122" t="s">
         <v>1484</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11575,7 +11601,7 @@
       <c r="J123" t="s">
         <v>1484</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11619,7 +11645,7 @@
       <c r="J124" t="s">
         <v>1484</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11663,7 +11689,7 @@
       <c r="J125" t="s">
         <v>1484</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11681,7 +11707,7 @@
       <c r="R125" t="s">
         <v>1671</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11716,7 +11742,7 @@
       <c r="J126" t="s">
         <v>1484</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11734,7 +11760,7 @@
       <c r="R126" t="s">
         <v>1672</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11769,7 +11795,7 @@
       <c r="J127" t="s">
         <v>1484</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11825,7 +11851,7 @@
       <c r="J128" t="s">
         <v>1484</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11866,7 +11892,7 @@
       <c r="J129" t="s">
         <v>1484</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11907,7 +11933,7 @@
       <c r="J130" t="s">
         <v>1484</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11948,7 +11974,7 @@
       <c r="J131" t="s">
         <v>1484</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -11992,7 +12018,7 @@
       <c r="J132" t="s">
         <v>1484</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12033,7 +12059,7 @@
       <c r="J133" t="s">
         <v>1484</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12051,7 +12077,7 @@
       <c r="R133" t="s">
         <v>1658</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12086,7 +12112,7 @@
       <c r="J134" t="s">
         <v>1484</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12104,7 +12130,7 @@
       <c r="R134" t="s">
         <v>1658</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12139,7 +12165,7 @@
       <c r="J135" t="s">
         <v>1484</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12180,7 +12206,7 @@
       <c r="J136" t="s">
         <v>1484</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12221,7 +12247,7 @@
       <c r="J137" t="s">
         <v>1484</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12262,7 +12288,7 @@
       <c r="J138" t="s">
         <v>1484</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12303,7 +12329,7 @@
       <c r="J139" t="s">
         <v>1484</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12350,7 +12376,7 @@
       <c r="J140" t="s">
         <v>1484</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12391,7 +12417,7 @@
       <c r="J141" t="s">
         <v>1484</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12432,7 +12458,7 @@
       <c r="J142" t="s">
         <v>1484</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12476,7 +12502,7 @@
       <c r="J143" t="s">
         <v>1484</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12494,7 +12520,7 @@
       <c r="R143" t="s">
         <v>1658</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12529,7 +12555,7 @@
       <c r="J144" t="s">
         <v>1484</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12547,7 +12573,7 @@
       <c r="R144" t="s">
         <v>1658</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12582,7 +12608,7 @@
       <c r="J145" t="s">
         <v>1484</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12600,7 +12626,7 @@
       <c r="R145" t="s">
         <v>1658</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12635,7 +12661,7 @@
       <c r="J146" t="s">
         <v>1484</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12653,7 +12679,7 @@
       <c r="R146" t="s">
         <v>1666</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12688,7 +12714,7 @@
       <c r="J147" t="s">
         <v>1484</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12706,7 +12732,7 @@
       <c r="R147" t="s">
         <v>1673</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12741,7 +12767,7 @@
       <c r="J148" t="s">
         <v>1484</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12782,7 +12808,7 @@
       <c r="J149" t="s">
         <v>1484</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12800,7 +12826,7 @@
       <c r="R149" t="s">
         <v>1658</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12835,7 +12861,7 @@
       <c r="J150" t="s">
         <v>1484</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12853,7 +12879,7 @@
       <c r="R150" t="s">
         <v>1658</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12888,7 +12914,7 @@
       <c r="J151" t="s">
         <v>1484</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12906,7 +12932,7 @@
       <c r="R151" t="s">
         <v>1674</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12941,7 +12967,7 @@
       <c r="J152" t="s">
         <v>1484</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12959,7 +12985,7 @@
       <c r="R152" t="s">
         <v>1675</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -12994,7 +13020,7 @@
       <c r="J153" t="s">
         <v>1484</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13003,7 +13029,7 @@
       <c r="M153" t="s">
         <v>1551</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13044,7 +13070,7 @@
       <c r="J154" t="s">
         <v>1484</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13085,7 +13111,7 @@
       <c r="J155" t="s">
         <v>1484</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13126,7 +13152,7 @@
       <c r="J156" t="s">
         <v>1484</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13167,7 +13193,7 @@
       <c r="J157" t="s">
         <v>1484</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13208,7 +13234,7 @@
       <c r="J158" t="s">
         <v>1484</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13249,7 +13275,7 @@
       <c r="J159" t="s">
         <v>1484</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13290,7 +13316,7 @@
       <c r="J160" t="s">
         <v>1484</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13331,7 +13357,7 @@
       <c r="J161" t="s">
         <v>1484</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13372,7 +13398,7 @@
       <c r="J162" t="s">
         <v>1484</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13390,7 +13416,7 @@
       <c r="R162" t="s">
         <v>1661</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13425,7 +13451,7 @@
       <c r="J163" t="s">
         <v>1484</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13443,7 +13469,7 @@
       <c r="R163" t="s">
         <v>1658</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13478,7 +13504,7 @@
       <c r="J164" t="s">
         <v>1484</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13522,7 +13548,7 @@
       <c r="J165" t="s">
         <v>1484</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13563,7 +13589,7 @@
       <c r="J166" t="s">
         <v>1484</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13581,7 +13607,7 @@
       <c r="R166" t="s">
         <v>1676</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13616,7 +13642,7 @@
       <c r="J167" t="s">
         <v>1484</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13660,7 +13686,7 @@
       <c r="J168" t="s">
         <v>1484</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13704,7 +13730,7 @@
       <c r="J169" t="s">
         <v>1484</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13745,7 +13771,7 @@
       <c r="J170" t="s">
         <v>1484</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13786,7 +13812,7 @@
       <c r="J171" t="s">
         <v>1484</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13827,7 +13853,7 @@
       <c r="J172" t="s">
         <v>1484</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13868,7 +13894,7 @@
       <c r="J173" t="s">
         <v>1484</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13909,7 +13935,7 @@
       <c r="J174" t="s">
         <v>1484</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13950,7 +13976,7 @@
       <c r="J175" t="s">
         <v>1484</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -13991,7 +14017,7 @@
       <c r="J176" t="s">
         <v>1484</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14032,7 +14058,7 @@
       <c r="J177" t="s">
         <v>1484</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14073,7 +14099,7 @@
       <c r="J178" t="s">
         <v>1484</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14091,7 +14117,7 @@
       <c r="R178" t="s">
         <v>1674</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14126,7 +14152,7 @@
       <c r="J179" t="s">
         <v>1484</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14135,7 +14161,7 @@
       <c r="M179" t="s">
         <v>1548</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14176,7 +14202,7 @@
       <c r="J180" t="s">
         <v>1484</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14217,7 +14243,7 @@
       <c r="J181" t="s">
         <v>1484</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14235,7 +14261,7 @@
       <c r="R181" t="s">
         <v>1658</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14270,7 +14296,7 @@
       <c r="J182" t="s">
         <v>1484</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14311,7 +14337,7 @@
       <c r="J183" t="s">
         <v>1484</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14352,7 +14378,7 @@
       <c r="J184" t="s">
         <v>1484</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14393,7 +14419,7 @@
       <c r="J185" t="s">
         <v>1484</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14434,7 +14460,7 @@
       <c r="J186" t="s">
         <v>1484</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14475,7 +14501,7 @@
       <c r="J187" t="s">
         <v>1484</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14516,7 +14542,7 @@
       <c r="J188" t="s">
         <v>1484</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14557,7 +14583,7 @@
       <c r="J189" t="s">
         <v>1484</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14598,7 +14624,7 @@
       <c r="J190" t="s">
         <v>1484</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14639,7 +14665,7 @@
       <c r="J191" t="s">
         <v>1484</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14680,7 +14706,7 @@
       <c r="J192" t="s">
         <v>1484</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14721,7 +14747,7 @@
       <c r="J193" t="s">
         <v>1484</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14762,7 +14788,7 @@
       <c r="J194" t="s">
         <v>1484</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14803,7 +14829,7 @@
       <c r="J195" t="s">
         <v>1484</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14821,7 +14847,7 @@
       <c r="R195" t="s">
         <v>1667</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14859,7 +14885,7 @@
       <c r="J196" t="s">
         <v>1484</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14877,7 +14903,7 @@
       <c r="R196" t="s">
         <v>1673</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14915,7 +14941,7 @@
       <c r="J197" t="s">
         <v>1484</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14956,7 +14982,7 @@
       <c r="J198" t="s">
         <v>1486</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -14997,7 +15023,7 @@
       <c r="J199" t="s">
         <v>1485</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15038,7 +15064,7 @@
       <c r="J200" t="s">
         <v>1484</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15079,7 +15105,7 @@
       <c r="J201" t="s">
         <v>1484</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15120,7 +15146,7 @@
       <c r="J202" t="s">
         <v>1484</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15138,7 +15164,7 @@
       <c r="R202" t="s">
         <v>1658</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15173,7 +15199,7 @@
       <c r="J203" t="s">
         <v>1484</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15191,7 +15217,7 @@
       <c r="R203" t="s">
         <v>1666</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15226,7 +15252,7 @@
       <c r="J204" t="s">
         <v>1484</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15241,7 +15267,7 @@
       <c r="R204" t="s">
         <v>1677</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15279,7 +15305,7 @@
       <c r="J205" t="s">
         <v>1484</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15297,7 +15323,7 @@
       <c r="R205" t="s">
         <v>1678</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15335,7 +15361,7 @@
       <c r="J206" t="s">
         <v>1484</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15353,7 +15379,7 @@
       <c r="R206" t="s">
         <v>1646</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15388,7 +15414,7 @@
       <c r="J207" t="s">
         <v>1484</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15429,7 +15455,7 @@
       <c r="J208" t="s">
         <v>1484</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15470,7 +15496,7 @@
       <c r="J209" t="s">
         <v>1484</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15511,7 +15537,7 @@
       <c r="J210" t="s">
         <v>1484</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15552,7 +15578,7 @@
       <c r="J211" t="s">
         <v>1484</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15593,7 +15619,7 @@
       <c r="J212" t="s">
         <v>1484</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15634,7 +15660,7 @@
       <c r="J213" t="s">
         <v>1484</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15675,7 +15701,7 @@
       <c r="J214" t="s">
         <v>1484</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15693,7 +15719,7 @@
       <c r="R214" t="s">
         <v>1679</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15728,7 +15754,7 @@
       <c r="J215" t="s">
         <v>1484</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15769,7 +15795,7 @@
       <c r="J216" t="s">
         <v>1484</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15810,7 +15836,7 @@
       <c r="J217" t="s">
         <v>1484</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15851,7 +15877,7 @@
       <c r="J218" t="s">
         <v>1484</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15892,7 +15918,7 @@
       <c r="J219" t="s">
         <v>1484</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15933,7 +15959,7 @@
       <c r="J220" t="s">
         <v>1484</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -15974,7 +16000,7 @@
       <c r="J221" t="s">
         <v>1484</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16015,7 +16041,7 @@
       <c r="J222" t="s">
         <v>1484</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16056,7 +16082,7 @@
       <c r="J223" t="s">
         <v>1484</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16097,7 +16123,7 @@
       <c r="J224" t="s">
         <v>1484</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16138,7 +16164,7 @@
       <c r="J225" t="s">
         <v>1484</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16179,7 +16205,7 @@
       <c r="J226" t="s">
         <v>1484</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16220,7 +16246,7 @@
       <c r="J227" t="s">
         <v>1484</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16261,7 +16287,7 @@
       <c r="J228" t="s">
         <v>1484</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16302,7 +16328,7 @@
       <c r="J229" t="s">
         <v>1484</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16343,7 +16369,7 @@
       <c r="J230" t="s">
         <v>1484</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16384,7 +16410,7 @@
       <c r="J231" t="s">
         <v>1484</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16425,7 +16451,7 @@
       <c r="J232" t="s">
         <v>1484</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16466,7 +16492,7 @@
       <c r="J233" t="s">
         <v>1484</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16507,7 +16533,7 @@
       <c r="J234" t="s">
         <v>1484</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16548,7 +16574,7 @@
       <c r="J235" t="s">
         <v>1484</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16589,7 +16615,7 @@
       <c r="J236" t="s">
         <v>1484</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16630,7 +16656,7 @@
       <c r="J237" t="s">
         <v>1484</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16671,7 +16697,7 @@
       <c r="J238" t="s">
         <v>1484</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16712,7 +16738,7 @@
       <c r="J239" t="s">
         <v>1484</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16730,7 +16756,7 @@
       <c r="R239" t="s">
         <v>1673</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16765,7 +16791,7 @@
       <c r="J240" t="s">
         <v>1484</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16806,7 +16832,7 @@
       <c r="J241" t="s">
         <v>1484</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16847,7 +16873,7 @@
       <c r="J242" t="s">
         <v>1484</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16865,7 +16891,7 @@
       <c r="R242" t="s">
         <v>1666</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16900,7 +16926,7 @@
       <c r="J243" t="s">
         <v>1484</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16941,7 +16967,7 @@
       <c r="J244" t="s">
         <v>1484</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -16982,7 +17008,7 @@
       <c r="J245" t="s">
         <v>1484</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17023,7 +17049,7 @@
       <c r="J246" t="s">
         <v>1484</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17041,7 +17067,7 @@
       <c r="R246" t="s">
         <v>1646</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17076,7 +17102,7 @@
       <c r="J247" t="s">
         <v>1484</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17117,7 +17143,7 @@
       <c r="J248" t="s">
         <v>1484</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17158,7 +17184,7 @@
       <c r="J249" t="s">
         <v>1484</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17199,7 +17225,7 @@
       <c r="J250" t="s">
         <v>1484</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17240,7 +17266,7 @@
       <c r="J251" t="s">
         <v>1484</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17281,7 +17307,7 @@
       <c r="J252" t="s">
         <v>1484</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17322,7 +17348,7 @@
       <c r="J253" t="s">
         <v>1484</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17340,7 +17366,7 @@
       <c r="R253" t="s">
         <v>1676</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17378,7 +17404,7 @@
       <c r="J254" t="s">
         <v>1484</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17419,7 +17445,7 @@
       <c r="J255" t="s">
         <v>1484</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17460,7 +17486,7 @@
       <c r="J256" t="s">
         <v>1484</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17469,7 +17495,7 @@
       <c r="M256" t="s">
         <v>1547</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17507,7 +17533,7 @@
       <c r="J257" t="s">
         <v>1484</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17516,7 +17542,7 @@
       <c r="M257" t="s">
         <v>1548</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17560,7 +17586,7 @@
       <c r="J258" t="s">
         <v>1484</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17578,7 +17604,7 @@
       <c r="R258" t="s">
         <v>1658</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17616,7 +17642,7 @@
       <c r="J259" t="s">
         <v>1484</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17634,7 +17660,7 @@
       <c r="R259" t="s">
         <v>1674</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17672,7 +17698,7 @@
       <c r="J260" t="s">
         <v>1484</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17681,7 +17707,7 @@
       <c r="M260" t="s">
         <v>1542</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17725,7 +17751,7 @@
       <c r="J261" t="s">
         <v>1484</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17743,7 +17769,7 @@
       <c r="R261" t="s">
         <v>1680</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17781,7 +17807,7 @@
       <c r="J262" t="s">
         <v>1484</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17799,7 +17825,7 @@
       <c r="R262" t="s">
         <v>1674</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17837,7 +17863,7 @@
       <c r="J263" t="s">
         <v>1484</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17846,7 +17872,7 @@
       <c r="M263" t="s">
         <v>1542</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17890,7 +17916,7 @@
       <c r="J264" t="s">
         <v>1484</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17931,7 +17957,7 @@
       <c r="J265" t="s">
         <v>1484</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17972,7 +17998,7 @@
       <c r="J266" t="s">
         <v>1484</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18013,7 +18039,7 @@
       <c r="J267" t="s">
         <v>1484</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18057,7 +18083,7 @@
       <c r="J268" t="s">
         <v>1484</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18098,7 +18124,7 @@
       <c r="J269" t="s">
         <v>1484</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18139,7 +18165,7 @@
       <c r="J270" t="s">
         <v>1484</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18180,7 +18206,7 @@
       <c r="J271" t="s">
         <v>1484</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18221,7 +18247,7 @@
       <c r="J272" t="s">
         <v>1484</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18239,7 +18265,7 @@
       <c r="R272" t="s">
         <v>1681</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18277,7 +18303,7 @@
       <c r="J273" t="s">
         <v>1484</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18321,7 +18347,7 @@
       <c r="J274" t="s">
         <v>1484</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18362,7 +18388,7 @@
       <c r="J275" t="s">
         <v>1484</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18403,7 +18429,7 @@
       <c r="J276" t="s">
         <v>1484</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18444,7 +18470,7 @@
       <c r="J277" t="s">
         <v>1484</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18485,7 +18511,7 @@
       <c r="J278" t="s">
         <v>1484</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18526,7 +18552,7 @@
       <c r="J279" t="s">
         <v>1484</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18567,7 +18593,7 @@
       <c r="J280" t="s">
         <v>1484</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18608,7 +18634,7 @@
       <c r="J281" t="s">
         <v>1484</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18649,7 +18675,7 @@
       <c r="J282" t="s">
         <v>1484</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18690,7 +18716,7 @@
       <c r="J283" t="s">
         <v>1484</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18731,7 +18757,7 @@
       <c r="J284" t="s">
         <v>1484</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18772,7 +18798,7 @@
       <c r="J285" t="s">
         <v>1484</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18813,7 +18839,7 @@
       <c r="J286" t="s">
         <v>1484</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18854,7 +18880,7 @@
       <c r="J287" t="s">
         <v>1484</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18895,7 +18921,7 @@
       <c r="J288" t="s">
         <v>1484</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18936,7 +18962,7 @@
       <c r="J289" t="s">
         <v>1484</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -18977,7 +19003,7 @@
       <c r="J290" t="s">
         <v>1484</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19018,7 +19044,7 @@
       <c r="J291" t="s">
         <v>1484</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19059,7 +19085,7 @@
       <c r="J292" t="s">
         <v>1484</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19100,7 +19126,7 @@
       <c r="J293" t="s">
         <v>1484</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19141,7 +19167,7 @@
       <c r="J294" t="s">
         <v>1484</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19182,7 +19208,7 @@
       <c r="J295" t="s">
         <v>1484</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19200,7 +19226,7 @@
       <c r="R295" t="s">
         <v>1682</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19238,7 +19264,7 @@
       <c r="J296" t="s">
         <v>1484</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19256,7 +19282,7 @@
       <c r="R296" t="s">
         <v>1658</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19294,7 +19320,7 @@
       <c r="J297" t="s">
         <v>1484</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19335,7 +19361,7 @@
       <c r="J298" t="s">
         <v>1484</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19376,7 +19402,7 @@
       <c r="J299" t="s">
         <v>1485</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19417,7 +19443,7 @@
       <c r="J300" t="s">
         <v>1484</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19458,7 +19484,7 @@
       <c r="J301" t="s">
         <v>1484</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20296,7 +20322,7 @@
       <c r="R321" t="s">
         <v>1644</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20516,7 +20542,7 @@
       <c r="R326" t="s">
         <v>1683</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21351,7 +21377,7 @@
       <c r="R346" t="s">
         <v>1684</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (25/08/2026 08:32)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5193,8 +5193,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5210,7 +5218,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5218,12 +5226,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5523,73 +5549,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5624,7 +5650,7 @@
       <c r="J2" t="s">
         <v>1487</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5668,7 +5694,7 @@
       <c r="J3" t="s">
         <v>1487</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5712,7 +5738,7 @@
       <c r="J4" t="s">
         <v>1487</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5730,7 +5756,7 @@
       <c r="R4" t="s">
         <v>1645</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5768,7 +5794,7 @@
       <c r="J5" t="s">
         <v>1488</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5818,7 +5844,7 @@
       <c r="J6" t="s">
         <v>1487</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5865,7 +5891,7 @@
       <c r="J7" t="s">
         <v>1487</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5912,7 +5938,7 @@
       <c r="J8" t="s">
         <v>1487</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5959,7 +5985,7 @@
       <c r="J9" t="s">
         <v>1487</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6006,7 +6032,7 @@
       <c r="J10" t="s">
         <v>1487</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6053,7 +6079,7 @@
       <c r="J11" t="s">
         <v>1487</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6100,7 +6126,7 @@
       <c r="J12" t="s">
         <v>1487</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6144,7 +6170,7 @@
       <c r="J13" t="s">
         <v>1487</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6162,7 +6188,7 @@
       <c r="R13" t="s">
         <v>1646</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6200,7 +6226,7 @@
       <c r="J14" t="s">
         <v>1487</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6218,7 +6244,7 @@
       <c r="R14" t="s">
         <v>1647</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6256,7 +6282,7 @@
       <c r="J15" t="s">
         <v>1487</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6274,7 +6300,7 @@
       <c r="R15" t="s">
         <v>1647</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6312,7 +6338,7 @@
       <c r="J16" t="s">
         <v>1487</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6356,7 +6382,7 @@
       <c r="J17" t="s">
         <v>1487</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6400,7 +6426,7 @@
       <c r="J18" t="s">
         <v>1487</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6418,7 +6444,7 @@
       <c r="R18" t="s">
         <v>1648</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6459,7 +6485,7 @@
       <c r="J19" t="s">
         <v>1487</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6503,7 +6529,7 @@
       <c r="J20" t="s">
         <v>1487</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6547,7 +6573,7 @@
       <c r="J21" t="s">
         <v>1487</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6565,7 +6591,7 @@
       <c r="R21" t="s">
         <v>1647</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6606,7 +6632,7 @@
       <c r="J22" t="s">
         <v>1487</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6624,7 +6650,7 @@
       <c r="R22" t="s">
         <v>1649</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6665,7 +6691,7 @@
       <c r="J23" t="s">
         <v>1487</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6683,7 +6709,7 @@
       <c r="R23" t="s">
         <v>1650</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6724,7 +6750,7 @@
       <c r="J24" t="s">
         <v>1487</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6768,7 +6794,7 @@
       <c r="J25" t="s">
         <v>1487</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6809,7 +6835,7 @@
       <c r="J26" t="s">
         <v>1489</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6827,7 +6853,7 @@
       <c r="R26" t="s">
         <v>1651</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6862,7 +6888,7 @@
       <c r="J27" t="s">
         <v>1487</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6880,7 +6906,7 @@
       <c r="R27" t="s">
         <v>1652</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6921,7 +6947,7 @@
       <c r="J28" t="s">
         <v>1487</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6965,7 +6991,7 @@
       <c r="J29" t="s">
         <v>1487</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7009,7 +7035,7 @@
       <c r="J30" t="s">
         <v>1487</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7053,7 +7079,7 @@
       <c r="J31" t="s">
         <v>1487</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7071,7 +7097,7 @@
       <c r="R31" t="s">
         <v>1653</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7112,7 +7138,7 @@
       <c r="J32" t="s">
         <v>1487</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7156,7 +7182,7 @@
       <c r="J33" t="s">
         <v>1487</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7174,7 +7200,7 @@
       <c r="R33" t="s">
         <v>1654</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7215,7 +7241,7 @@
       <c r="J34" t="s">
         <v>1487</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7259,7 +7285,7 @@
       <c r="J35" t="s">
         <v>1487</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7277,7 +7303,7 @@
       <c r="R35" t="s">
         <v>1655</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7318,7 +7344,7 @@
       <c r="J36" t="s">
         <v>1487</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7336,7 +7362,7 @@
       <c r="R36" t="s">
         <v>1655</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7377,7 +7403,7 @@
       <c r="J37" t="s">
         <v>1487</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7395,7 +7421,7 @@
       <c r="R37" t="s">
         <v>1655</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7436,7 +7462,7 @@
       <c r="J38" t="s">
         <v>1487</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7454,7 +7480,7 @@
       <c r="R38" t="s">
         <v>1655</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7495,7 +7521,7 @@
       <c r="J39" t="s">
         <v>1487</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7513,7 +7539,7 @@
       <c r="R39" t="s">
         <v>1655</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7554,7 +7580,7 @@
       <c r="J40" t="s">
         <v>1487</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7572,7 +7598,7 @@
       <c r="R40" t="s">
         <v>1656</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7613,7 +7639,7 @@
       <c r="J41" t="s">
         <v>1487</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7631,7 +7657,7 @@
       <c r="R41" t="s">
         <v>1647</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7669,7 +7695,7 @@
       <c r="J42" t="s">
         <v>1487</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7687,7 +7713,7 @@
       <c r="R42" t="s">
         <v>1655</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7728,7 +7754,7 @@
       <c r="J43" t="s">
         <v>1487</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7772,7 +7798,7 @@
       <c r="J44" t="s">
         <v>1487</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7790,7 +7816,7 @@
       <c r="R44" t="s">
         <v>1657</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7831,7 +7857,7 @@
       <c r="J45" t="s">
         <v>1487</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7849,7 +7875,7 @@
       <c r="R45" t="s">
         <v>1658</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7887,7 +7913,7 @@
       <c r="J46" t="s">
         <v>1487</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7931,7 +7957,7 @@
       <c r="J47" t="s">
         <v>1487</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7949,7 +7975,7 @@
       <c r="R47" t="s">
         <v>1659</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -7990,7 +8016,7 @@
       <c r="J48" t="s">
         <v>1487</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8034,7 +8060,7 @@
       <c r="J49" t="s">
         <v>1487</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8078,7 +8104,7 @@
       <c r="J50" t="s">
         <v>1487</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8122,7 +8148,7 @@
       <c r="J51" t="s">
         <v>1487</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8169,7 +8195,7 @@
       <c r="J52" t="s">
         <v>1487</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8213,7 +8239,7 @@
       <c r="J53" t="s">
         <v>1487</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8257,7 +8283,7 @@
       <c r="J54" t="s">
         <v>1487</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8301,7 +8327,7 @@
       <c r="J55" t="s">
         <v>1487</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8351,7 +8377,7 @@
       <c r="J56" t="s">
         <v>1487</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8404,7 +8430,7 @@
       <c r="J57" t="s">
         <v>1487</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8454,7 +8480,7 @@
       <c r="J58" t="s">
         <v>1487</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8504,7 +8530,7 @@
       <c r="J59" t="s">
         <v>1487</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8522,7 +8548,7 @@
       <c r="R59" t="s">
         <v>1660</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8563,7 +8589,7 @@
       <c r="J60" t="s">
         <v>1487</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8607,7 +8633,7 @@
       <c r="J61" t="s">
         <v>1487</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8651,7 +8677,7 @@
       <c r="J62" t="s">
         <v>1487</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8695,7 +8721,7 @@
       <c r="J63" t="s">
         <v>1487</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8739,7 +8765,7 @@
       <c r="J64" t="s">
         <v>1487</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8783,7 +8809,7 @@
       <c r="J65" t="s">
         <v>1487</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8830,7 +8856,7 @@
       <c r="J66" t="s">
         <v>1487</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8848,7 +8874,7 @@
       <c r="R66" t="s">
         <v>1661</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8886,7 +8912,7 @@
       <c r="J67" t="s">
         <v>1487</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8930,7 +8956,7 @@
       <c r="J68" t="s">
         <v>1487</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8945,7 +8971,7 @@
       <c r="O68" t="s">
         <v>1564</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -8989,7 +9015,7 @@
       <c r="J69" t="s">
         <v>1489</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9033,7 +9059,7 @@
       <c r="J70" t="s">
         <v>1487</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9077,7 +9103,7 @@
       <c r="J71" t="s">
         <v>1487</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9121,7 +9147,7 @@
       <c r="J72" t="s">
         <v>1487</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9165,7 +9191,7 @@
       <c r="J73" t="s">
         <v>1487</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9209,7 +9235,7 @@
       <c r="J74" t="s">
         <v>1487</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9253,7 +9279,7 @@
       <c r="J75" t="s">
         <v>1487</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9297,7 +9323,7 @@
       <c r="J76" t="s">
         <v>1487</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9315,7 +9341,7 @@
       <c r="R76" t="s">
         <v>1662</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9353,7 +9379,7 @@
       <c r="J77" t="s">
         <v>1487</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9371,7 +9397,7 @@
       <c r="R77" t="s">
         <v>1662</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9409,7 +9435,7 @@
       <c r="J78" t="s">
         <v>1487</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9427,7 +9453,7 @@
       <c r="R78" t="s">
         <v>1662</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9465,7 +9491,7 @@
       <c r="J79" t="s">
         <v>1487</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9483,7 +9509,7 @@
       <c r="R79" t="s">
         <v>1662</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9521,7 +9547,7 @@
       <c r="J80" t="s">
         <v>1487</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9565,7 +9591,7 @@
       <c r="J81" t="s">
         <v>1487</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9609,7 +9635,7 @@
       <c r="J82" t="s">
         <v>1487</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9653,7 +9679,7 @@
       <c r="J83" t="s">
         <v>1487</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9697,7 +9723,7 @@
       <c r="J84" t="s">
         <v>1487</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9741,7 +9767,7 @@
       <c r="J85" t="s">
         <v>1487</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9759,7 +9785,7 @@
       <c r="R85" t="s">
         <v>1663</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9797,7 +9823,7 @@
       <c r="J86" t="s">
         <v>1487</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9841,7 +9867,7 @@
       <c r="J87" t="s">
         <v>1487</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9859,7 +9885,7 @@
       <c r="R87" t="s">
         <v>1664</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9897,7 +9923,7 @@
       <c r="J88" t="s">
         <v>1487</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9941,7 +9967,7 @@
       <c r="J89" t="s">
         <v>1487</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9959,7 +9985,7 @@
       <c r="R89" t="s">
         <v>1665</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -9994,7 +10020,7 @@
       <c r="J90" t="s">
         <v>1487</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10012,7 +10038,7 @@
       <c r="R90" t="s">
         <v>1666</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10047,7 +10073,7 @@
       <c r="J91" t="s">
         <v>1487</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10065,7 +10091,7 @@
       <c r="R91" t="s">
         <v>1650</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10103,7 +10129,7 @@
       <c r="J92" t="s">
         <v>1487</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10124,7 +10150,7 @@
       <c r="R92" t="s">
         <v>1650</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10165,7 +10191,7 @@
       <c r="J93" t="s">
         <v>1487</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10206,7 +10232,7 @@
       <c r="J94" t="s">
         <v>1487</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10250,7 +10276,7 @@
       <c r="J95" t="s">
         <v>1487</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10294,7 +10320,7 @@
       <c r="J96" t="s">
         <v>1487</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10312,7 +10338,7 @@
       <c r="R96" t="s">
         <v>1667</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10350,7 +10376,7 @@
       <c r="J97" t="s">
         <v>1487</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10365,7 +10391,7 @@
       <c r="R97" t="s">
         <v>1667</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10406,7 +10432,7 @@
       <c r="J98" t="s">
         <v>1487</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10424,7 +10450,7 @@
       <c r="R98" t="s">
         <v>1668</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10462,7 +10488,7 @@
       <c r="J99" t="s">
         <v>1487</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10480,7 +10506,7 @@
       <c r="R99" t="s">
         <v>1669</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10518,7 +10544,7 @@
       <c r="J100" t="s">
         <v>1487</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10559,7 +10585,7 @@
       <c r="J101" t="s">
         <v>1487</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10600,7 +10626,7 @@
       <c r="J102" t="s">
         <v>1487</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10641,7 +10667,7 @@
       <c r="J103" t="s">
         <v>1487</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10682,7 +10708,7 @@
       <c r="J104" t="s">
         <v>1487</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10723,7 +10749,7 @@
       <c r="J105" t="s">
         <v>1487</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10764,7 +10790,7 @@
       <c r="J106" t="s">
         <v>1487</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10805,7 +10831,7 @@
       <c r="J107" t="s">
         <v>1487</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10846,7 +10872,7 @@
       <c r="J108" t="s">
         <v>1487</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10887,7 +10913,7 @@
       <c r="J109" t="s">
         <v>1487</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10940,7 +10966,7 @@
       <c r="J110" t="s">
         <v>1487</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -10996,7 +11022,7 @@
       <c r="J111" t="s">
         <v>1487</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11014,7 +11040,7 @@
       <c r="R111" t="s">
         <v>1671</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11052,7 +11078,7 @@
       <c r="J112" t="s">
         <v>1487</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11111,7 +11137,7 @@
       <c r="J113" t="s">
         <v>1487</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11155,7 +11181,7 @@
       <c r="J114" t="s">
         <v>1487</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11199,7 +11225,7 @@
       <c r="J115" t="s">
         <v>1487</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11217,7 +11243,7 @@
       <c r="R115" t="s">
         <v>1673</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11255,7 +11281,7 @@
       <c r="J116" t="s">
         <v>1487</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11314,7 +11340,7 @@
       <c r="J117" t="s">
         <v>1487</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11358,7 +11384,7 @@
       <c r="J118" t="s">
         <v>1487</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11405,7 +11431,7 @@
       <c r="J119" t="s">
         <v>1487</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11446,7 +11472,7 @@
       <c r="J120" t="s">
         <v>1487</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11490,7 +11516,7 @@
       <c r="J121" t="s">
         <v>1487</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11537,7 +11563,7 @@
       <c r="J122" t="s">
         <v>1487</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11587,7 +11613,7 @@
       <c r="J123" t="s">
         <v>1487</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11631,7 +11657,7 @@
       <c r="J124" t="s">
         <v>1487</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11675,7 +11701,7 @@
       <c r="J125" t="s">
         <v>1487</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11693,7 +11719,7 @@
       <c r="R125" t="s">
         <v>1675</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11728,7 +11754,7 @@
       <c r="J126" t="s">
         <v>1487</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11746,7 +11772,7 @@
       <c r="R126" t="s">
         <v>1676</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11781,7 +11807,7 @@
       <c r="J127" t="s">
         <v>1487</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11837,7 +11863,7 @@
       <c r="J128" t="s">
         <v>1487</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11878,7 +11904,7 @@
       <c r="J129" t="s">
         <v>1487</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11919,7 +11945,7 @@
       <c r="J130" t="s">
         <v>1487</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11960,7 +11986,7 @@
       <c r="J131" t="s">
         <v>1487</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12004,7 +12030,7 @@
       <c r="J132" t="s">
         <v>1487</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12045,7 +12071,7 @@
       <c r="J133" t="s">
         <v>1487</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12063,7 +12089,7 @@
       <c r="R133" t="s">
         <v>1662</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12098,7 +12124,7 @@
       <c r="J134" t="s">
         <v>1487</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12116,7 +12142,7 @@
       <c r="R134" t="s">
         <v>1662</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12151,7 +12177,7 @@
       <c r="J135" t="s">
         <v>1487</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12192,7 +12218,7 @@
       <c r="J136" t="s">
         <v>1487</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12233,7 +12259,7 @@
       <c r="J137" t="s">
         <v>1487</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12274,7 +12300,7 @@
       <c r="J138" t="s">
         <v>1487</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12315,7 +12341,7 @@
       <c r="J139" t="s">
         <v>1487</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12362,7 +12388,7 @@
       <c r="J140" t="s">
         <v>1487</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12403,7 +12429,7 @@
       <c r="J141" t="s">
         <v>1487</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12444,7 +12470,7 @@
       <c r="J142" t="s">
         <v>1487</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12488,7 +12514,7 @@
       <c r="J143" t="s">
         <v>1487</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12506,7 +12532,7 @@
       <c r="R143" t="s">
         <v>1662</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12541,7 +12567,7 @@
       <c r="J144" t="s">
         <v>1487</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12559,7 +12585,7 @@
       <c r="R144" t="s">
         <v>1662</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12594,7 +12620,7 @@
       <c r="J145" t="s">
         <v>1487</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12612,7 +12638,7 @@
       <c r="R145" t="s">
         <v>1662</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12647,7 +12673,7 @@
       <c r="J146" t="s">
         <v>1487</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12665,7 +12691,7 @@
       <c r="R146" t="s">
         <v>1670</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12700,7 +12726,7 @@
       <c r="J147" t="s">
         <v>1487</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12718,7 +12744,7 @@
       <c r="R147" t="s">
         <v>1677</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12753,7 +12779,7 @@
       <c r="J148" t="s">
         <v>1487</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12794,7 +12820,7 @@
       <c r="J149" t="s">
         <v>1487</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12812,7 +12838,7 @@
       <c r="R149" t="s">
         <v>1662</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12847,7 +12873,7 @@
       <c r="J150" t="s">
         <v>1487</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12865,7 +12891,7 @@
       <c r="R150" t="s">
         <v>1662</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12900,7 +12926,7 @@
       <c r="J151" t="s">
         <v>1487</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12918,7 +12944,7 @@
       <c r="R151" t="s">
         <v>1678</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12953,7 +12979,7 @@
       <c r="J152" t="s">
         <v>1487</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12971,7 +12997,7 @@
       <c r="R152" t="s">
         <v>1679</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13006,7 +13032,7 @@
       <c r="J153" t="s">
         <v>1487</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13015,7 +13041,7 @@
       <c r="M153" t="s">
         <v>1555</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13056,7 +13082,7 @@
       <c r="J154" t="s">
         <v>1487</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13097,7 +13123,7 @@
       <c r="J155" t="s">
         <v>1487</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13138,7 +13164,7 @@
       <c r="J156" t="s">
         <v>1487</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13179,7 +13205,7 @@
       <c r="J157" t="s">
         <v>1487</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13220,7 +13246,7 @@
       <c r="J158" t="s">
         <v>1487</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13261,7 +13287,7 @@
       <c r="J159" t="s">
         <v>1487</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13302,7 +13328,7 @@
       <c r="J160" t="s">
         <v>1487</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13343,7 +13369,7 @@
       <c r="J161" t="s">
         <v>1487</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13384,7 +13410,7 @@
       <c r="J162" t="s">
         <v>1487</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13402,7 +13428,7 @@
       <c r="R162" t="s">
         <v>1665</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13437,7 +13463,7 @@
       <c r="J163" t="s">
         <v>1487</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13455,7 +13481,7 @@
       <c r="R163" t="s">
         <v>1662</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13490,7 +13516,7 @@
       <c r="J164" t="s">
         <v>1487</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13534,7 +13560,7 @@
       <c r="J165" t="s">
         <v>1487</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13575,7 +13601,7 @@
       <c r="J166" t="s">
         <v>1487</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13593,7 +13619,7 @@
       <c r="R166" t="s">
         <v>1680</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13628,7 +13654,7 @@
       <c r="J167" t="s">
         <v>1487</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13672,7 +13698,7 @@
       <c r="J168" t="s">
         <v>1487</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13716,7 +13742,7 @@
       <c r="J169" t="s">
         <v>1487</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13757,7 +13783,7 @@
       <c r="J170" t="s">
         <v>1487</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13798,7 +13824,7 @@
       <c r="J171" t="s">
         <v>1487</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13839,7 +13865,7 @@
       <c r="J172" t="s">
         <v>1487</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13880,7 +13906,7 @@
       <c r="J173" t="s">
         <v>1487</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13921,7 +13947,7 @@
       <c r="J174" t="s">
         <v>1487</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13962,7 +13988,7 @@
       <c r="J175" t="s">
         <v>1487</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14003,7 +14029,7 @@
       <c r="J176" t="s">
         <v>1487</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14044,7 +14070,7 @@
       <c r="J177" t="s">
         <v>1487</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14085,7 +14111,7 @@
       <c r="J178" t="s">
         <v>1487</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14103,7 +14129,7 @@
       <c r="R178" t="s">
         <v>1678</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14138,7 +14164,7 @@
       <c r="J179" t="s">
         <v>1487</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14147,7 +14173,7 @@
       <c r="M179" t="s">
         <v>1552</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14188,7 +14214,7 @@
       <c r="J180" t="s">
         <v>1487</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14229,7 +14255,7 @@
       <c r="J181" t="s">
         <v>1487</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14247,7 +14273,7 @@
       <c r="R181" t="s">
         <v>1662</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14282,7 +14308,7 @@
       <c r="J182" t="s">
         <v>1487</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14323,7 +14349,7 @@
       <c r="J183" t="s">
         <v>1487</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14364,7 +14390,7 @@
       <c r="J184" t="s">
         <v>1487</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14405,7 +14431,7 @@
       <c r="J185" t="s">
         <v>1487</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14446,7 +14472,7 @@
       <c r="J186" t="s">
         <v>1487</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14487,7 +14513,7 @@
       <c r="J187" t="s">
         <v>1487</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14528,7 +14554,7 @@
       <c r="J188" t="s">
         <v>1487</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14569,7 +14595,7 @@
       <c r="J189" t="s">
         <v>1487</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14610,7 +14636,7 @@
       <c r="J190" t="s">
         <v>1487</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14651,7 +14677,7 @@
       <c r="J191" t="s">
         <v>1487</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14692,7 +14718,7 @@
       <c r="J192" t="s">
         <v>1487</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14733,7 +14759,7 @@
       <c r="J193" t="s">
         <v>1487</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14774,7 +14800,7 @@
       <c r="J194" t="s">
         <v>1487</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14815,7 +14841,7 @@
       <c r="J195" t="s">
         <v>1487</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14833,7 +14859,7 @@
       <c r="R195" t="s">
         <v>1671</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14871,7 +14897,7 @@
       <c r="J196" t="s">
         <v>1487</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14889,7 +14915,7 @@
       <c r="R196" t="s">
         <v>1677</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14927,7 +14953,7 @@
       <c r="J197" t="s">
         <v>1487</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14968,7 +14994,7 @@
       <c r="J198" t="s">
         <v>1489</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15009,7 +15035,7 @@
       <c r="J199" t="s">
         <v>1488</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15050,7 +15076,7 @@
       <c r="J200" t="s">
         <v>1487</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15091,7 +15117,7 @@
       <c r="J201" t="s">
         <v>1487</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15132,7 +15158,7 @@
       <c r="J202" t="s">
         <v>1487</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15150,7 +15176,7 @@
       <c r="R202" t="s">
         <v>1662</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15185,7 +15211,7 @@
       <c r="J203" t="s">
         <v>1487</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15203,7 +15229,7 @@
       <c r="R203" t="s">
         <v>1670</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15238,7 +15264,7 @@
       <c r="J204" t="s">
         <v>1487</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15253,7 +15279,7 @@
       <c r="R204" t="s">
         <v>1681</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15291,7 +15317,7 @@
       <c r="J205" t="s">
         <v>1487</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15309,7 +15335,7 @@
       <c r="R205" t="s">
         <v>1682</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15347,7 +15373,7 @@
       <c r="J206" t="s">
         <v>1487</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15365,7 +15391,7 @@
       <c r="R206" t="s">
         <v>1650</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15400,7 +15426,7 @@
       <c r="J207" t="s">
         <v>1487</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15441,7 +15467,7 @@
       <c r="J208" t="s">
         <v>1487</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15482,7 +15508,7 @@
       <c r="J209" t="s">
         <v>1487</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15523,7 +15549,7 @@
       <c r="J210" t="s">
         <v>1487</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15564,7 +15590,7 @@
       <c r="J211" t="s">
         <v>1487</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15605,7 +15631,7 @@
       <c r="J212" t="s">
         <v>1487</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15646,7 +15672,7 @@
       <c r="J213" t="s">
         <v>1487</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15687,7 +15713,7 @@
       <c r="J214" t="s">
         <v>1487</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15705,7 +15731,7 @@
       <c r="R214" t="s">
         <v>1683</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15740,7 +15766,7 @@
       <c r="J215" t="s">
         <v>1487</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15781,7 +15807,7 @@
       <c r="J216" t="s">
         <v>1487</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15822,7 +15848,7 @@
       <c r="J217" t="s">
         <v>1487</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15863,7 +15889,7 @@
       <c r="J218" t="s">
         <v>1487</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15904,7 +15930,7 @@
       <c r="J219" t="s">
         <v>1487</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15945,7 +15971,7 @@
       <c r="J220" t="s">
         <v>1487</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -15986,7 +16012,7 @@
       <c r="J221" t="s">
         <v>1487</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16027,7 +16053,7 @@
       <c r="J222" t="s">
         <v>1487</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16068,7 +16094,7 @@
       <c r="J223" t="s">
         <v>1487</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16109,7 +16135,7 @@
       <c r="J224" t="s">
         <v>1487</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16150,7 +16176,7 @@
       <c r="J225" t="s">
         <v>1487</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16191,7 +16217,7 @@
       <c r="J226" t="s">
         <v>1487</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16232,7 +16258,7 @@
       <c r="J227" t="s">
         <v>1487</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16273,7 +16299,7 @@
       <c r="J228" t="s">
         <v>1487</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16314,7 +16340,7 @@
       <c r="J229" t="s">
         <v>1487</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16355,7 +16381,7 @@
       <c r="J230" t="s">
         <v>1487</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16396,7 +16422,7 @@
       <c r="J231" t="s">
         <v>1487</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16437,7 +16463,7 @@
       <c r="J232" t="s">
         <v>1487</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16478,7 +16504,7 @@
       <c r="J233" t="s">
         <v>1487</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16519,7 +16545,7 @@
       <c r="J234" t="s">
         <v>1487</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16560,7 +16586,7 @@
       <c r="J235" t="s">
         <v>1487</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16601,7 +16627,7 @@
       <c r="J236" t="s">
         <v>1487</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16642,7 +16668,7 @@
       <c r="J237" t="s">
         <v>1487</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16683,7 +16709,7 @@
       <c r="J238" t="s">
         <v>1487</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16724,7 +16750,7 @@
       <c r="J239" t="s">
         <v>1487</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16742,7 +16768,7 @@
       <c r="R239" t="s">
         <v>1677</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16777,7 +16803,7 @@
       <c r="J240" t="s">
         <v>1487</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16818,7 +16844,7 @@
       <c r="J241" t="s">
         <v>1487</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16859,7 +16885,7 @@
       <c r="J242" t="s">
         <v>1487</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16877,7 +16903,7 @@
       <c r="R242" t="s">
         <v>1670</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16912,7 +16938,7 @@
       <c r="J243" t="s">
         <v>1487</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16953,7 +16979,7 @@
       <c r="J244" t="s">
         <v>1487</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -16994,7 +17020,7 @@
       <c r="J245" t="s">
         <v>1487</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17035,7 +17061,7 @@
       <c r="J246" t="s">
         <v>1487</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17053,7 +17079,7 @@
       <c r="R246" t="s">
         <v>1650</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17088,7 +17114,7 @@
       <c r="J247" t="s">
         <v>1487</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17129,7 +17155,7 @@
       <c r="J248" t="s">
         <v>1487</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17170,7 +17196,7 @@
       <c r="J249" t="s">
         <v>1487</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17211,7 +17237,7 @@
       <c r="J250" t="s">
         <v>1487</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17252,7 +17278,7 @@
       <c r="J251" t="s">
         <v>1487</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17293,7 +17319,7 @@
       <c r="J252" t="s">
         <v>1487</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17334,7 +17360,7 @@
       <c r="J253" t="s">
         <v>1487</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17352,7 +17378,7 @@
       <c r="R253" t="s">
         <v>1680</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17390,7 +17416,7 @@
       <c r="J254" t="s">
         <v>1487</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17431,7 +17457,7 @@
       <c r="J255" t="s">
         <v>1487</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17472,7 +17498,7 @@
       <c r="J256" t="s">
         <v>1487</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17481,7 +17507,7 @@
       <c r="M256" t="s">
         <v>1551</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17519,7 +17545,7 @@
       <c r="J257" t="s">
         <v>1487</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17528,7 +17554,7 @@
       <c r="M257" t="s">
         <v>1552</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17572,7 +17598,7 @@
       <c r="J258" t="s">
         <v>1487</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17590,7 +17616,7 @@
       <c r="R258" t="s">
         <v>1662</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17628,7 +17654,7 @@
       <c r="J259" t="s">
         <v>1487</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17646,7 +17672,7 @@
       <c r="R259" t="s">
         <v>1678</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17684,7 +17710,7 @@
       <c r="J260" t="s">
         <v>1487</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17693,7 +17719,7 @@
       <c r="M260" t="s">
         <v>1546</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17737,7 +17763,7 @@
       <c r="J261" t="s">
         <v>1487</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17755,7 +17781,7 @@
       <c r="R261" t="s">
         <v>1684</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17793,7 +17819,7 @@
       <c r="J262" t="s">
         <v>1487</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17811,7 +17837,7 @@
       <c r="R262" t="s">
         <v>1678</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17849,7 +17875,7 @@
       <c r="J263" t="s">
         <v>1487</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17858,7 +17884,7 @@
       <c r="M263" t="s">
         <v>1546</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17902,7 +17928,7 @@
       <c r="J264" t="s">
         <v>1487</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17943,7 +17969,7 @@
       <c r="J265" t="s">
         <v>1487</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -17984,7 +18010,7 @@
       <c r="J266" t="s">
         <v>1487</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18025,7 +18051,7 @@
       <c r="J267" t="s">
         <v>1487</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18069,7 +18095,7 @@
       <c r="J268" t="s">
         <v>1487</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18110,7 +18136,7 @@
       <c r="J269" t="s">
         <v>1487</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18151,7 +18177,7 @@
       <c r="J270" t="s">
         <v>1487</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18192,7 +18218,7 @@
       <c r="J271" t="s">
         <v>1487</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18233,7 +18259,7 @@
       <c r="J272" t="s">
         <v>1487</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18251,7 +18277,7 @@
       <c r="R272" t="s">
         <v>1685</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18289,7 +18315,7 @@
       <c r="J273" t="s">
         <v>1487</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18333,7 +18359,7 @@
       <c r="J274" t="s">
         <v>1487</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18374,7 +18400,7 @@
       <c r="J275" t="s">
         <v>1487</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18415,7 +18441,7 @@
       <c r="J276" t="s">
         <v>1487</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18456,7 +18482,7 @@
       <c r="J277" t="s">
         <v>1487</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18497,7 +18523,7 @@
       <c r="J278" t="s">
         <v>1487</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18538,7 +18564,7 @@
       <c r="J279" t="s">
         <v>1487</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18579,7 +18605,7 @@
       <c r="J280" t="s">
         <v>1487</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18620,7 +18646,7 @@
       <c r="J281" t="s">
         <v>1487</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18661,7 +18687,7 @@
       <c r="J282" t="s">
         <v>1487</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18702,7 +18728,7 @@
       <c r="J283" t="s">
         <v>1487</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18743,7 +18769,7 @@
       <c r="J284" t="s">
         <v>1487</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18784,7 +18810,7 @@
       <c r="J285" t="s">
         <v>1487</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18825,7 +18851,7 @@
       <c r="J286" t="s">
         <v>1487</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18866,7 +18892,7 @@
       <c r="J287" t="s">
         <v>1487</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18907,7 +18933,7 @@
       <c r="J288" t="s">
         <v>1487</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18948,7 +18974,7 @@
       <c r="J289" t="s">
         <v>1487</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -18989,7 +19015,7 @@
       <c r="J290" t="s">
         <v>1487</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19030,7 +19056,7 @@
       <c r="J291" t="s">
         <v>1487</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19071,7 +19097,7 @@
       <c r="J292" t="s">
         <v>1487</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19112,7 +19138,7 @@
       <c r="J293" t="s">
         <v>1487</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19153,7 +19179,7 @@
       <c r="J294" t="s">
         <v>1487</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19194,7 +19220,7 @@
       <c r="J295" t="s">
         <v>1487</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19212,7 +19238,7 @@
       <c r="R295" t="s">
         <v>1686</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19250,7 +19276,7 @@
       <c r="J296" t="s">
         <v>1487</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19268,7 +19294,7 @@
       <c r="R296" t="s">
         <v>1662</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19306,7 +19332,7 @@
       <c r="J297" t="s">
         <v>1487</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19347,7 +19373,7 @@
       <c r="J298" t="s">
         <v>1487</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19388,7 +19414,7 @@
       <c r="J299" t="s">
         <v>1488</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19429,7 +19455,7 @@
       <c r="J300" t="s">
         <v>1487</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19470,7 +19496,7 @@
       <c r="J301" t="s">
         <v>1487</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20308,7 +20334,7 @@
       <c r="R321" t="s">
         <v>1648</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20528,7 +20554,7 @@
       <c r="R326" t="s">
         <v>1687</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21363,7 +21389,7 @@
       <c r="R346" t="s">
         <v>1688</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (25/08/2026 08:37)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5193,16 +5193,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5218,7 +5210,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5226,30 +5218,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5549,73 +5523,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5650,7 +5624,7 @@
       <c r="J2" t="s">
         <v>1487</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5694,7 +5668,7 @@
       <c r="J3" t="s">
         <v>1487</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5738,7 +5712,7 @@
       <c r="J4" t="s">
         <v>1487</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5756,7 +5730,7 @@
       <c r="R4" t="s">
         <v>1645</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5794,7 +5768,7 @@
       <c r="J5" t="s">
         <v>1488</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5844,7 +5818,7 @@
       <c r="J6" t="s">
         <v>1487</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5891,7 +5865,7 @@
       <c r="J7" t="s">
         <v>1487</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5938,7 +5912,7 @@
       <c r="J8" t="s">
         <v>1487</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -5985,7 +5959,7 @@
       <c r="J9" t="s">
         <v>1487</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6032,7 +6006,7 @@
       <c r="J10" t="s">
         <v>1487</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6079,7 +6053,7 @@
       <c r="J11" t="s">
         <v>1487</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6126,7 +6100,7 @@
       <c r="J12" t="s">
         <v>1487</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6170,7 +6144,7 @@
       <c r="J13" t="s">
         <v>1487</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6188,7 +6162,7 @@
       <c r="R13" t="s">
         <v>1646</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6226,7 +6200,7 @@
       <c r="J14" t="s">
         <v>1487</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6244,7 +6218,7 @@
       <c r="R14" t="s">
         <v>1647</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6282,7 +6256,7 @@
       <c r="J15" t="s">
         <v>1487</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6300,7 +6274,7 @@
       <c r="R15" t="s">
         <v>1647</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6338,7 +6312,7 @@
       <c r="J16" t="s">
         <v>1487</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6382,7 +6356,7 @@
       <c r="J17" t="s">
         <v>1487</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6426,7 +6400,7 @@
       <c r="J18" t="s">
         <v>1487</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6444,7 +6418,7 @@
       <c r="R18" t="s">
         <v>1648</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6485,7 +6459,7 @@
       <c r="J19" t="s">
         <v>1487</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6529,7 +6503,7 @@
       <c r="J20" t="s">
         <v>1487</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6573,7 +6547,7 @@
       <c r="J21" t="s">
         <v>1487</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6591,7 +6565,7 @@
       <c r="R21" t="s">
         <v>1647</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6632,7 +6606,7 @@
       <c r="J22" t="s">
         <v>1487</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6650,7 +6624,7 @@
       <c r="R22" t="s">
         <v>1649</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6691,7 +6665,7 @@
       <c r="J23" t="s">
         <v>1487</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6709,7 +6683,7 @@
       <c r="R23" t="s">
         <v>1650</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6750,7 +6724,7 @@
       <c r="J24" t="s">
         <v>1487</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6794,7 +6768,7 @@
       <c r="J25" t="s">
         <v>1487</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6835,7 +6809,7 @@
       <c r="J26" t="s">
         <v>1489</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6853,7 +6827,7 @@
       <c r="R26" t="s">
         <v>1651</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6888,7 +6862,7 @@
       <c r="J27" t="s">
         <v>1487</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6906,7 +6880,7 @@
       <c r="R27" t="s">
         <v>1652</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6947,7 +6921,7 @@
       <c r="J28" t="s">
         <v>1487</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -6991,7 +6965,7 @@
       <c r="J29" t="s">
         <v>1487</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7035,7 +7009,7 @@
       <c r="J30" t="s">
         <v>1487</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7079,7 +7053,7 @@
       <c r="J31" t="s">
         <v>1487</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7097,7 +7071,7 @@
       <c r="R31" t="s">
         <v>1653</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7138,7 +7112,7 @@
       <c r="J32" t="s">
         <v>1487</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7182,7 +7156,7 @@
       <c r="J33" t="s">
         <v>1487</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7200,7 +7174,7 @@
       <c r="R33" t="s">
         <v>1654</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7241,7 +7215,7 @@
       <c r="J34" t="s">
         <v>1487</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7285,7 +7259,7 @@
       <c r="J35" t="s">
         <v>1487</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7303,7 +7277,7 @@
       <c r="R35" t="s">
         <v>1655</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7344,7 +7318,7 @@
       <c r="J36" t="s">
         <v>1487</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7362,7 +7336,7 @@
       <c r="R36" t="s">
         <v>1655</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7403,7 +7377,7 @@
       <c r="J37" t="s">
         <v>1487</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7421,7 +7395,7 @@
       <c r="R37" t="s">
         <v>1655</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7462,7 +7436,7 @@
       <c r="J38" t="s">
         <v>1487</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7480,7 +7454,7 @@
       <c r="R38" t="s">
         <v>1655</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7521,7 +7495,7 @@
       <c r="J39" t="s">
         <v>1487</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7539,7 +7513,7 @@
       <c r="R39" t="s">
         <v>1655</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7580,7 +7554,7 @@
       <c r="J40" t="s">
         <v>1487</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7598,7 +7572,7 @@
       <c r="R40" t="s">
         <v>1656</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7639,7 +7613,7 @@
       <c r="J41" t="s">
         <v>1487</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7657,7 +7631,7 @@
       <c r="R41" t="s">
         <v>1647</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7695,7 +7669,7 @@
       <c r="J42" t="s">
         <v>1487</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7713,7 +7687,7 @@
       <c r="R42" t="s">
         <v>1655</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7754,7 +7728,7 @@
       <c r="J43" t="s">
         <v>1487</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7798,7 +7772,7 @@
       <c r="J44" t="s">
         <v>1487</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7816,7 +7790,7 @@
       <c r="R44" t="s">
         <v>1657</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7857,7 +7831,7 @@
       <c r="J45" t="s">
         <v>1487</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7875,7 +7849,7 @@
       <c r="R45" t="s">
         <v>1658</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7913,7 +7887,7 @@
       <c r="J46" t="s">
         <v>1487</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7957,7 +7931,7 @@
       <c r="J47" t="s">
         <v>1487</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -7975,7 +7949,7 @@
       <c r="R47" t="s">
         <v>1659</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8016,7 +7990,7 @@
       <c r="J48" t="s">
         <v>1487</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8060,7 +8034,7 @@
       <c r="J49" t="s">
         <v>1487</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8104,7 +8078,7 @@
       <c r="J50" t="s">
         <v>1487</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8148,7 +8122,7 @@
       <c r="J51" t="s">
         <v>1487</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8195,7 +8169,7 @@
       <c r="J52" t="s">
         <v>1487</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8239,7 +8213,7 @@
       <c r="J53" t="s">
         <v>1487</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8283,7 +8257,7 @@
       <c r="J54" t="s">
         <v>1487</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8327,7 +8301,7 @@
       <c r="J55" t="s">
         <v>1487</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8377,7 +8351,7 @@
       <c r="J56" t="s">
         <v>1487</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8430,7 +8404,7 @@
       <c r="J57" t="s">
         <v>1487</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8480,7 +8454,7 @@
       <c r="J58" t="s">
         <v>1487</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8530,7 +8504,7 @@
       <c r="J59" t="s">
         <v>1487</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8548,7 +8522,7 @@
       <c r="R59" t="s">
         <v>1660</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8589,7 +8563,7 @@
       <c r="J60" t="s">
         <v>1487</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8633,7 +8607,7 @@
       <c r="J61" t="s">
         <v>1487</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8677,7 +8651,7 @@
       <c r="J62" t="s">
         <v>1487</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8721,7 +8695,7 @@
       <c r="J63" t="s">
         <v>1487</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8765,7 +8739,7 @@
       <c r="J64" t="s">
         <v>1487</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8809,7 +8783,7 @@
       <c r="J65" t="s">
         <v>1487</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8856,7 +8830,7 @@
       <c r="J66" t="s">
         <v>1487</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8874,7 +8848,7 @@
       <c r="R66" t="s">
         <v>1661</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8912,7 +8886,7 @@
       <c r="J67" t="s">
         <v>1487</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8956,7 +8930,7 @@
       <c r="J68" t="s">
         <v>1487</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8971,7 +8945,7 @@
       <c r="O68" t="s">
         <v>1564</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9015,7 +8989,7 @@
       <c r="J69" t="s">
         <v>1489</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9059,7 +9033,7 @@
       <c r="J70" t="s">
         <v>1487</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9103,7 +9077,7 @@
       <c r="J71" t="s">
         <v>1487</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9147,7 +9121,7 @@
       <c r="J72" t="s">
         <v>1487</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9191,7 +9165,7 @@
       <c r="J73" t="s">
         <v>1487</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9235,7 +9209,7 @@
       <c r="J74" t="s">
         <v>1487</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9279,7 +9253,7 @@
       <c r="J75" t="s">
         <v>1487</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9323,7 +9297,7 @@
       <c r="J76" t="s">
         <v>1487</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9341,7 +9315,7 @@
       <c r="R76" t="s">
         <v>1662</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9379,7 +9353,7 @@
       <c r="J77" t="s">
         <v>1487</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9397,7 +9371,7 @@
       <c r="R77" t="s">
         <v>1662</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9435,7 +9409,7 @@
       <c r="J78" t="s">
         <v>1487</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9453,7 +9427,7 @@
       <c r="R78" t="s">
         <v>1662</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9491,7 +9465,7 @@
       <c r="J79" t="s">
         <v>1487</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9509,7 +9483,7 @@
       <c r="R79" t="s">
         <v>1662</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9547,7 +9521,7 @@
       <c r="J80" t="s">
         <v>1487</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9591,7 +9565,7 @@
       <c r="J81" t="s">
         <v>1487</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9635,7 +9609,7 @@
       <c r="J82" t="s">
         <v>1487</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9679,7 +9653,7 @@
       <c r="J83" t="s">
         <v>1487</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9723,7 +9697,7 @@
       <c r="J84" t="s">
         <v>1487</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9767,7 +9741,7 @@
       <c r="J85" t="s">
         <v>1487</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9785,7 +9759,7 @@
       <c r="R85" t="s">
         <v>1663</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9823,7 +9797,7 @@
       <c r="J86" t="s">
         <v>1487</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9867,7 +9841,7 @@
       <c r="J87" t="s">
         <v>1487</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9885,7 +9859,7 @@
       <c r="R87" t="s">
         <v>1664</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9923,7 +9897,7 @@
       <c r="J88" t="s">
         <v>1487</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9967,7 +9941,7 @@
       <c r="J89" t="s">
         <v>1487</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -9985,7 +9959,7 @@
       <c r="R89" t="s">
         <v>1665</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10020,7 +9994,7 @@
       <c r="J90" t="s">
         <v>1487</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10038,7 +10012,7 @@
       <c r="R90" t="s">
         <v>1666</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10073,7 +10047,7 @@
       <c r="J91" t="s">
         <v>1487</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10091,7 +10065,7 @@
       <c r="R91" t="s">
         <v>1650</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10129,7 +10103,7 @@
       <c r="J92" t="s">
         <v>1487</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10150,7 +10124,7 @@
       <c r="R92" t="s">
         <v>1650</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10191,7 +10165,7 @@
       <c r="J93" t="s">
         <v>1487</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10232,7 +10206,7 @@
       <c r="J94" t="s">
         <v>1487</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10276,7 +10250,7 @@
       <c r="J95" t="s">
         <v>1487</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10320,7 +10294,7 @@
       <c r="J96" t="s">
         <v>1487</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10338,7 +10312,7 @@
       <c r="R96" t="s">
         <v>1667</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10376,7 +10350,7 @@
       <c r="J97" t="s">
         <v>1487</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10391,7 +10365,7 @@
       <c r="R97" t="s">
         <v>1667</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10432,7 +10406,7 @@
       <c r="J98" t="s">
         <v>1487</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10450,7 +10424,7 @@
       <c r="R98" t="s">
         <v>1668</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10488,7 +10462,7 @@
       <c r="J99" t="s">
         <v>1487</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10506,7 +10480,7 @@
       <c r="R99" t="s">
         <v>1669</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10544,7 +10518,7 @@
       <c r="J100" t="s">
         <v>1487</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10585,7 +10559,7 @@
       <c r="J101" t="s">
         <v>1487</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10626,7 +10600,7 @@
       <c r="J102" t="s">
         <v>1487</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10667,7 +10641,7 @@
       <c r="J103" t="s">
         <v>1487</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10708,7 +10682,7 @@
       <c r="J104" t="s">
         <v>1487</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10749,7 +10723,7 @@
       <c r="J105" t="s">
         <v>1487</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10790,7 +10764,7 @@
       <c r="J106" t="s">
         <v>1487</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10831,7 +10805,7 @@
       <c r="J107" t="s">
         <v>1487</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10872,7 +10846,7 @@
       <c r="J108" t="s">
         <v>1487</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10913,7 +10887,7 @@
       <c r="J109" t="s">
         <v>1487</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10966,7 +10940,7 @@
       <c r="J110" t="s">
         <v>1487</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11022,7 +10996,7 @@
       <c r="J111" t="s">
         <v>1487</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11040,7 +11014,7 @@
       <c r="R111" t="s">
         <v>1671</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11078,7 +11052,7 @@
       <c r="J112" t="s">
         <v>1487</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11137,7 +11111,7 @@
       <c r="J113" t="s">
         <v>1487</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11181,7 +11155,7 @@
       <c r="J114" t="s">
         <v>1487</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11225,7 +11199,7 @@
       <c r="J115" t="s">
         <v>1487</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11243,7 +11217,7 @@
       <c r="R115" t="s">
         <v>1673</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11281,7 +11255,7 @@
       <c r="J116" t="s">
         <v>1487</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11340,7 +11314,7 @@
       <c r="J117" t="s">
         <v>1487</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11384,7 +11358,7 @@
       <c r="J118" t="s">
         <v>1487</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11431,7 +11405,7 @@
       <c r="J119" t="s">
         <v>1487</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11472,7 +11446,7 @@
       <c r="J120" t="s">
         <v>1487</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11516,7 +11490,7 @@
       <c r="J121" t="s">
         <v>1487</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11563,7 +11537,7 @@
       <c r="J122" t="s">
         <v>1487</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11613,7 +11587,7 @@
       <c r="J123" t="s">
         <v>1487</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11657,7 +11631,7 @@
       <c r="J124" t="s">
         <v>1487</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11701,7 +11675,7 @@
       <c r="J125" t="s">
         <v>1487</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11719,7 +11693,7 @@
       <c r="R125" t="s">
         <v>1675</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11754,7 +11728,7 @@
       <c r="J126" t="s">
         <v>1487</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11772,7 +11746,7 @@
       <c r="R126" t="s">
         <v>1676</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11807,7 +11781,7 @@
       <c r="J127" t="s">
         <v>1487</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11863,7 +11837,7 @@
       <c r="J128" t="s">
         <v>1487</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11904,7 +11878,7 @@
       <c r="J129" t="s">
         <v>1487</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11945,7 +11919,7 @@
       <c r="J130" t="s">
         <v>1487</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -11986,7 +11960,7 @@
       <c r="J131" t="s">
         <v>1487</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12030,7 +12004,7 @@
       <c r="J132" t="s">
         <v>1487</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12071,7 +12045,7 @@
       <c r="J133" t="s">
         <v>1487</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12089,7 +12063,7 @@
       <c r="R133" t="s">
         <v>1662</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12124,7 +12098,7 @@
       <c r="J134" t="s">
         <v>1487</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12142,7 +12116,7 @@
       <c r="R134" t="s">
         <v>1662</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12177,7 +12151,7 @@
       <c r="J135" t="s">
         <v>1487</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12218,7 +12192,7 @@
       <c r="J136" t="s">
         <v>1487</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12259,7 +12233,7 @@
       <c r="J137" t="s">
         <v>1487</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12300,7 +12274,7 @@
       <c r="J138" t="s">
         <v>1487</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12341,7 +12315,7 @@
       <c r="J139" t="s">
         <v>1487</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12388,7 +12362,7 @@
       <c r="J140" t="s">
         <v>1487</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12429,7 +12403,7 @@
       <c r="J141" t="s">
         <v>1487</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12470,7 +12444,7 @@
       <c r="J142" t="s">
         <v>1487</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12514,7 +12488,7 @@
       <c r="J143" t="s">
         <v>1487</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12532,7 +12506,7 @@
       <c r="R143" t="s">
         <v>1662</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12567,7 +12541,7 @@
       <c r="J144" t="s">
         <v>1487</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12585,7 +12559,7 @@
       <c r="R144" t="s">
         <v>1662</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12620,7 +12594,7 @@
       <c r="J145" t="s">
         <v>1487</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12638,7 +12612,7 @@
       <c r="R145" t="s">
         <v>1662</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12673,7 +12647,7 @@
       <c r="J146" t="s">
         <v>1487</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12691,7 +12665,7 @@
       <c r="R146" t="s">
         <v>1670</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12726,7 +12700,7 @@
       <c r="J147" t="s">
         <v>1487</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12744,7 +12718,7 @@
       <c r="R147" t="s">
         <v>1677</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12779,7 +12753,7 @@
       <c r="J148" t="s">
         <v>1487</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12820,7 +12794,7 @@
       <c r="J149" t="s">
         <v>1487</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12838,7 +12812,7 @@
       <c r="R149" t="s">
         <v>1662</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12873,7 +12847,7 @@
       <c r="J150" t="s">
         <v>1487</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12891,7 +12865,7 @@
       <c r="R150" t="s">
         <v>1662</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12926,7 +12900,7 @@
       <c r="J151" t="s">
         <v>1487</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12944,7 +12918,7 @@
       <c r="R151" t="s">
         <v>1678</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -12979,7 +12953,7 @@
       <c r="J152" t="s">
         <v>1487</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -12997,7 +12971,7 @@
       <c r="R152" t="s">
         <v>1679</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13032,7 +13006,7 @@
       <c r="J153" t="s">
         <v>1487</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13041,7 +13015,7 @@
       <c r="M153" t="s">
         <v>1555</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13082,7 +13056,7 @@
       <c r="J154" t="s">
         <v>1487</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13123,7 +13097,7 @@
       <c r="J155" t="s">
         <v>1487</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13164,7 +13138,7 @@
       <c r="J156" t="s">
         <v>1487</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13205,7 +13179,7 @@
       <c r="J157" t="s">
         <v>1487</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13246,7 +13220,7 @@
       <c r="J158" t="s">
         <v>1487</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13287,7 +13261,7 @@
       <c r="J159" t="s">
         <v>1487</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13328,7 +13302,7 @@
       <c r="J160" t="s">
         <v>1487</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13369,7 +13343,7 @@
       <c r="J161" t="s">
         <v>1487</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13410,7 +13384,7 @@
       <c r="J162" t="s">
         <v>1487</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13428,7 +13402,7 @@
       <c r="R162" t="s">
         <v>1665</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13463,7 +13437,7 @@
       <c r="J163" t="s">
         <v>1487</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13481,7 +13455,7 @@
       <c r="R163" t="s">
         <v>1662</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13516,7 +13490,7 @@
       <c r="J164" t="s">
         <v>1487</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13560,7 +13534,7 @@
       <c r="J165" t="s">
         <v>1487</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13601,7 +13575,7 @@
       <c r="J166" t="s">
         <v>1487</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13619,7 +13593,7 @@
       <c r="R166" t="s">
         <v>1680</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13654,7 +13628,7 @@
       <c r="J167" t="s">
         <v>1487</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13698,7 +13672,7 @@
       <c r="J168" t="s">
         <v>1487</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13742,7 +13716,7 @@
       <c r="J169" t="s">
         <v>1487</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13783,7 +13757,7 @@
       <c r="J170" t="s">
         <v>1487</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13824,7 +13798,7 @@
       <c r="J171" t="s">
         <v>1487</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13865,7 +13839,7 @@
       <c r="J172" t="s">
         <v>1487</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13906,7 +13880,7 @@
       <c r="J173" t="s">
         <v>1487</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13947,7 +13921,7 @@
       <c r="J174" t="s">
         <v>1487</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -13988,7 +13962,7 @@
       <c r="J175" t="s">
         <v>1487</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14029,7 +14003,7 @@
       <c r="J176" t="s">
         <v>1487</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14070,7 +14044,7 @@
       <c r="J177" t="s">
         <v>1487</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14111,7 +14085,7 @@
       <c r="J178" t="s">
         <v>1487</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14129,7 +14103,7 @@
       <c r="R178" t="s">
         <v>1678</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14164,7 +14138,7 @@
       <c r="J179" t="s">
         <v>1487</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14173,7 +14147,7 @@
       <c r="M179" t="s">
         <v>1552</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14214,7 +14188,7 @@
       <c r="J180" t="s">
         <v>1487</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14255,7 +14229,7 @@
       <c r="J181" t="s">
         <v>1487</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14273,7 +14247,7 @@
       <c r="R181" t="s">
         <v>1662</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14308,7 +14282,7 @@
       <c r="J182" t="s">
         <v>1487</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14349,7 +14323,7 @@
       <c r="J183" t="s">
         <v>1487</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14390,7 +14364,7 @@
       <c r="J184" t="s">
         <v>1487</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14431,7 +14405,7 @@
       <c r="J185" t="s">
         <v>1487</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14472,7 +14446,7 @@
       <c r="J186" t="s">
         <v>1487</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14513,7 +14487,7 @@
       <c r="J187" t="s">
         <v>1487</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14554,7 +14528,7 @@
       <c r="J188" t="s">
         <v>1487</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14595,7 +14569,7 @@
       <c r="J189" t="s">
         <v>1487</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14636,7 +14610,7 @@
       <c r="J190" t="s">
         <v>1487</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14677,7 +14651,7 @@
       <c r="J191" t="s">
         <v>1487</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14718,7 +14692,7 @@
       <c r="J192" t="s">
         <v>1487</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14759,7 +14733,7 @@
       <c r="J193" t="s">
         <v>1487</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14800,7 +14774,7 @@
       <c r="J194" t="s">
         <v>1487</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14841,7 +14815,7 @@
       <c r="J195" t="s">
         <v>1487</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14859,7 +14833,7 @@
       <c r="R195" t="s">
         <v>1671</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14897,7 +14871,7 @@
       <c r="J196" t="s">
         <v>1487</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14915,7 +14889,7 @@
       <c r="R196" t="s">
         <v>1677</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14953,7 +14927,7 @@
       <c r="J197" t="s">
         <v>1487</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -14994,7 +14968,7 @@
       <c r="J198" t="s">
         <v>1489</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15035,7 +15009,7 @@
       <c r="J199" t="s">
         <v>1488</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15076,7 +15050,7 @@
       <c r="J200" t="s">
         <v>1487</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15117,7 +15091,7 @@
       <c r="J201" t="s">
         <v>1487</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15158,7 +15132,7 @@
       <c r="J202" t="s">
         <v>1487</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15176,7 +15150,7 @@
       <c r="R202" t="s">
         <v>1662</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15211,7 +15185,7 @@
       <c r="J203" t="s">
         <v>1487</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15229,7 +15203,7 @@
       <c r="R203" t="s">
         <v>1670</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15264,7 +15238,7 @@
       <c r="J204" t="s">
         <v>1487</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15279,7 +15253,7 @@
       <c r="R204" t="s">
         <v>1681</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15317,7 +15291,7 @@
       <c r="J205" t="s">
         <v>1487</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15335,7 +15309,7 @@
       <c r="R205" t="s">
         <v>1682</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15373,7 +15347,7 @@
       <c r="J206" t="s">
         <v>1487</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15391,7 +15365,7 @@
       <c r="R206" t="s">
         <v>1650</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15426,7 +15400,7 @@
       <c r="J207" t="s">
         <v>1487</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15467,7 +15441,7 @@
       <c r="J208" t="s">
         <v>1487</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15508,7 +15482,7 @@
       <c r="J209" t="s">
         <v>1487</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15549,7 +15523,7 @@
       <c r="J210" t="s">
         <v>1487</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15590,7 +15564,7 @@
       <c r="J211" t="s">
         <v>1487</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15631,7 +15605,7 @@
       <c r="J212" t="s">
         <v>1487</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15672,7 +15646,7 @@
       <c r="J213" t="s">
         <v>1487</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15713,7 +15687,7 @@
       <c r="J214" t="s">
         <v>1487</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15731,7 +15705,7 @@
       <c r="R214" t="s">
         <v>1683</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15766,7 +15740,7 @@
       <c r="J215" t="s">
         <v>1487</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15807,7 +15781,7 @@
       <c r="J216" t="s">
         <v>1487</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15848,7 +15822,7 @@
       <c r="J217" t="s">
         <v>1487</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15889,7 +15863,7 @@
       <c r="J218" t="s">
         <v>1487</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15930,7 +15904,7 @@
       <c r="J219" t="s">
         <v>1487</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15971,7 +15945,7 @@
       <c r="J220" t="s">
         <v>1487</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16012,7 +15986,7 @@
       <c r="J221" t="s">
         <v>1487</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16053,7 +16027,7 @@
       <c r="J222" t="s">
         <v>1487</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16094,7 +16068,7 @@
       <c r="J223" t="s">
         <v>1487</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16135,7 +16109,7 @@
       <c r="J224" t="s">
         <v>1487</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16176,7 +16150,7 @@
       <c r="J225" t="s">
         <v>1487</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16217,7 +16191,7 @@
       <c r="J226" t="s">
         <v>1487</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16258,7 +16232,7 @@
       <c r="J227" t="s">
         <v>1487</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16299,7 +16273,7 @@
       <c r="J228" t="s">
         <v>1487</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16340,7 +16314,7 @@
       <c r="J229" t="s">
         <v>1487</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16381,7 +16355,7 @@
       <c r="J230" t="s">
         <v>1487</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16422,7 +16396,7 @@
       <c r="J231" t="s">
         <v>1487</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16463,7 +16437,7 @@
       <c r="J232" t="s">
         <v>1487</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16504,7 +16478,7 @@
       <c r="J233" t="s">
         <v>1487</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16545,7 +16519,7 @@
       <c r="J234" t="s">
         <v>1487</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16586,7 +16560,7 @@
       <c r="J235" t="s">
         <v>1487</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16627,7 +16601,7 @@
       <c r="J236" t="s">
         <v>1487</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16668,7 +16642,7 @@
       <c r="J237" t="s">
         <v>1487</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16709,7 +16683,7 @@
       <c r="J238" t="s">
         <v>1487</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16750,7 +16724,7 @@
       <c r="J239" t="s">
         <v>1487</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16768,7 +16742,7 @@
       <c r="R239" t="s">
         <v>1677</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16803,7 +16777,7 @@
       <c r="J240" t="s">
         <v>1487</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16844,7 +16818,7 @@
       <c r="J241" t="s">
         <v>1487</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16885,7 +16859,7 @@
       <c r="J242" t="s">
         <v>1487</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16903,7 +16877,7 @@
       <c r="R242" t="s">
         <v>1670</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16938,7 +16912,7 @@
       <c r="J243" t="s">
         <v>1487</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -16979,7 +16953,7 @@
       <c r="J244" t="s">
         <v>1487</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17020,7 +16994,7 @@
       <c r="J245" t="s">
         <v>1487</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17061,7 +17035,7 @@
       <c r="J246" t="s">
         <v>1487</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17079,7 +17053,7 @@
       <c r="R246" t="s">
         <v>1650</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17114,7 +17088,7 @@
       <c r="J247" t="s">
         <v>1487</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17155,7 +17129,7 @@
       <c r="J248" t="s">
         <v>1487</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17196,7 +17170,7 @@
       <c r="J249" t="s">
         <v>1487</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17237,7 +17211,7 @@
       <c r="J250" t="s">
         <v>1487</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17278,7 +17252,7 @@
       <c r="J251" t="s">
         <v>1487</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17319,7 +17293,7 @@
       <c r="J252" t="s">
         <v>1487</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17360,7 +17334,7 @@
       <c r="J253" t="s">
         <v>1487</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17378,7 +17352,7 @@
       <c r="R253" t="s">
         <v>1680</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17416,7 +17390,7 @@
       <c r="J254" t="s">
         <v>1487</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17457,7 +17431,7 @@
       <c r="J255" t="s">
         <v>1487</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17498,7 +17472,7 @@
       <c r="J256" t="s">
         <v>1487</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17507,7 +17481,7 @@
       <c r="M256" t="s">
         <v>1551</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17545,7 +17519,7 @@
       <c r="J257" t="s">
         <v>1487</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17554,7 +17528,7 @@
       <c r="M257" t="s">
         <v>1552</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17598,7 +17572,7 @@
       <c r="J258" t="s">
         <v>1487</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17616,7 +17590,7 @@
       <c r="R258" t="s">
         <v>1662</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17654,7 +17628,7 @@
       <c r="J259" t="s">
         <v>1487</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17672,7 +17646,7 @@
       <c r="R259" t="s">
         <v>1678</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17710,7 +17684,7 @@
       <c r="J260" t="s">
         <v>1487</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17719,7 +17693,7 @@
       <c r="M260" t="s">
         <v>1546</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17763,7 +17737,7 @@
       <c r="J261" t="s">
         <v>1487</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17781,7 +17755,7 @@
       <c r="R261" t="s">
         <v>1684</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17819,7 +17793,7 @@
       <c r="J262" t="s">
         <v>1487</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17837,7 +17811,7 @@
       <c r="R262" t="s">
         <v>1678</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17875,7 +17849,7 @@
       <c r="J263" t="s">
         <v>1487</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17884,7 +17858,7 @@
       <c r="M263" t="s">
         <v>1546</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17928,7 +17902,7 @@
       <c r="J264" t="s">
         <v>1487</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17969,7 +17943,7 @@
       <c r="J265" t="s">
         <v>1487</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18010,7 +17984,7 @@
       <c r="J266" t="s">
         <v>1487</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18051,7 +18025,7 @@
       <c r="J267" t="s">
         <v>1487</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18095,7 +18069,7 @@
       <c r="J268" t="s">
         <v>1487</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18136,7 +18110,7 @@
       <c r="J269" t="s">
         <v>1487</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18177,7 +18151,7 @@
       <c r="J270" t="s">
         <v>1487</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18218,7 +18192,7 @@
       <c r="J271" t="s">
         <v>1487</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18259,7 +18233,7 @@
       <c r="J272" t="s">
         <v>1487</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18277,7 +18251,7 @@
       <c r="R272" t="s">
         <v>1685</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18315,7 +18289,7 @@
       <c r="J273" t="s">
         <v>1487</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18359,7 +18333,7 @@
       <c r="J274" t="s">
         <v>1487</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18400,7 +18374,7 @@
       <c r="J275" t="s">
         <v>1487</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18441,7 +18415,7 @@
       <c r="J276" t="s">
         <v>1487</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18482,7 +18456,7 @@
       <c r="J277" t="s">
         <v>1487</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18523,7 +18497,7 @@
       <c r="J278" t="s">
         <v>1487</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18564,7 +18538,7 @@
       <c r="J279" t="s">
         <v>1487</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18605,7 +18579,7 @@
       <c r="J280" t="s">
         <v>1487</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18646,7 +18620,7 @@
       <c r="J281" t="s">
         <v>1487</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18687,7 +18661,7 @@
       <c r="J282" t="s">
         <v>1487</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18728,7 +18702,7 @@
       <c r="J283" t="s">
         <v>1487</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18769,7 +18743,7 @@
       <c r="J284" t="s">
         <v>1487</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18810,7 +18784,7 @@
       <c r="J285" t="s">
         <v>1487</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18851,7 +18825,7 @@
       <c r="J286" t="s">
         <v>1487</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18892,7 +18866,7 @@
       <c r="J287" t="s">
         <v>1487</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18933,7 +18907,7 @@
       <c r="J288" t="s">
         <v>1487</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18974,7 +18948,7 @@
       <c r="J289" t="s">
         <v>1487</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19015,7 +18989,7 @@
       <c r="J290" t="s">
         <v>1487</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19056,7 +19030,7 @@
       <c r="J291" t="s">
         <v>1487</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19097,7 +19071,7 @@
       <c r="J292" t="s">
         <v>1487</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19138,7 +19112,7 @@
       <c r="J293" t="s">
         <v>1487</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19179,7 +19153,7 @@
       <c r="J294" t="s">
         <v>1487</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19220,7 +19194,7 @@
       <c r="J295" t="s">
         <v>1487</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19238,7 +19212,7 @@
       <c r="R295" t="s">
         <v>1686</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19276,7 +19250,7 @@
       <c r="J296" t="s">
         <v>1487</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19294,7 +19268,7 @@
       <c r="R296" t="s">
         <v>1662</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19332,7 +19306,7 @@
       <c r="J297" t="s">
         <v>1487</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19373,7 +19347,7 @@
       <c r="J298" t="s">
         <v>1487</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19414,7 +19388,7 @@
       <c r="J299" t="s">
         <v>1488</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19455,7 +19429,7 @@
       <c r="J300" t="s">
         <v>1487</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19496,7 +19470,7 @@
       <c r="J301" t="s">
         <v>1487</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20334,7 +20308,7 @@
       <c r="R321" t="s">
         <v>1648</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20554,7 +20528,7 @@
       <c r="R326" t="s">
         <v>1687</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21389,7 +21363,7 @@
       <c r="R346" t="s">
         <v>1688</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (01/09/2026 11:16)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5244,8 +5244,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5261,7 +5269,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5269,12 +5277,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5574,73 +5600,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5675,7 +5701,7 @@
       <c r="J2" t="s">
         <v>1500</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5719,7 +5745,7 @@
       <c r="J3" t="s">
         <v>1500</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5763,7 +5789,7 @@
       <c r="J4" t="s">
         <v>1500</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5781,7 +5807,7 @@
       <c r="R4" t="s">
         <v>1661</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5819,7 +5845,7 @@
       <c r="J5" t="s">
         <v>1501</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5869,7 +5895,7 @@
       <c r="J6" t="s">
         <v>1500</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5916,7 +5942,7 @@
       <c r="J7" t="s">
         <v>1500</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5963,7 +5989,7 @@
       <c r="J8" t="s">
         <v>1500</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6010,7 +6036,7 @@
       <c r="J9" t="s">
         <v>1500</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6057,7 +6083,7 @@
       <c r="J10" t="s">
         <v>1500</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6104,7 +6130,7 @@
       <c r="J11" t="s">
         <v>1500</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6151,7 +6177,7 @@
       <c r="J12" t="s">
         <v>1500</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6195,7 +6221,7 @@
       <c r="J13" t="s">
         <v>1500</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6213,7 +6239,7 @@
       <c r="R13" t="s">
         <v>1662</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6251,7 +6277,7 @@
       <c r="J14" t="s">
         <v>1500</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6269,7 +6295,7 @@
       <c r="R14" t="s">
         <v>1663</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6307,7 +6333,7 @@
       <c r="J15" t="s">
         <v>1500</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6325,7 +6351,7 @@
       <c r="R15" t="s">
         <v>1663</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6363,7 +6389,7 @@
       <c r="J16" t="s">
         <v>1500</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6407,7 +6433,7 @@
       <c r="J17" t="s">
         <v>1500</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6451,7 +6477,7 @@
       <c r="J18" t="s">
         <v>1500</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6469,7 +6495,7 @@
       <c r="R18" t="s">
         <v>1664</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6510,7 +6536,7 @@
       <c r="J19" t="s">
         <v>1500</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6554,7 +6580,7 @@
       <c r="J20" t="s">
         <v>1500</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6598,7 +6624,7 @@
       <c r="J21" t="s">
         <v>1500</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6616,7 +6642,7 @@
       <c r="R21" t="s">
         <v>1663</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6657,7 +6683,7 @@
       <c r="J22" t="s">
         <v>1500</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6675,7 +6701,7 @@
       <c r="R22" t="s">
         <v>1665</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6716,7 +6742,7 @@
       <c r="J23" t="s">
         <v>1500</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6734,7 +6760,7 @@
       <c r="R23" t="s">
         <v>1666</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6775,7 +6801,7 @@
       <c r="J24" t="s">
         <v>1500</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6819,7 +6845,7 @@
       <c r="J25" t="s">
         <v>1500</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6860,7 +6886,7 @@
       <c r="J26" t="s">
         <v>1502</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6878,7 +6904,7 @@
       <c r="R26" t="s">
         <v>1667</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6913,7 +6939,7 @@
       <c r="J27" t="s">
         <v>1500</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6931,7 +6957,7 @@
       <c r="R27" t="s">
         <v>1668</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6972,7 +6998,7 @@
       <c r="J28" t="s">
         <v>1500</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7016,7 +7042,7 @@
       <c r="J29" t="s">
         <v>1500</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7060,7 +7086,7 @@
       <c r="J30" t="s">
         <v>1500</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7104,7 +7130,7 @@
       <c r="J31" t="s">
         <v>1500</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7122,7 +7148,7 @@
       <c r="R31" t="s">
         <v>1669</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7163,7 +7189,7 @@
       <c r="J32" t="s">
         <v>1500</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7207,7 +7233,7 @@
       <c r="J33" t="s">
         <v>1500</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7225,7 +7251,7 @@
       <c r="R33" t="s">
         <v>1670</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7266,7 +7292,7 @@
       <c r="J34" t="s">
         <v>1500</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7310,7 +7336,7 @@
       <c r="J35" t="s">
         <v>1500</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7328,7 +7354,7 @@
       <c r="R35" t="s">
         <v>1671</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7369,7 +7395,7 @@
       <c r="J36" t="s">
         <v>1500</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7387,7 +7413,7 @@
       <c r="R36" t="s">
         <v>1671</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7428,7 +7454,7 @@
       <c r="J37" t="s">
         <v>1500</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7446,7 +7472,7 @@
       <c r="R37" t="s">
         <v>1671</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7487,7 +7513,7 @@
       <c r="J38" t="s">
         <v>1500</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7505,7 +7531,7 @@
       <c r="R38" t="s">
         <v>1671</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7546,7 +7572,7 @@
       <c r="J39" t="s">
         <v>1500</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7564,7 +7590,7 @@
       <c r="R39" t="s">
         <v>1671</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7605,7 +7631,7 @@
       <c r="J40" t="s">
         <v>1500</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7623,7 +7649,7 @@
       <c r="R40" t="s">
         <v>1672</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7664,7 +7690,7 @@
       <c r="J41" t="s">
         <v>1500</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7682,7 +7708,7 @@
       <c r="R41" t="s">
         <v>1663</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7720,7 +7746,7 @@
       <c r="J42" t="s">
         <v>1500</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7738,7 +7764,7 @@
       <c r="R42" t="s">
         <v>1671</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7779,7 +7805,7 @@
       <c r="J43" t="s">
         <v>1500</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7823,7 +7849,7 @@
       <c r="J44" t="s">
         <v>1500</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7841,7 +7867,7 @@
       <c r="R44" t="s">
         <v>1673</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7882,7 +7908,7 @@
       <c r="J45" t="s">
         <v>1500</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7900,7 +7926,7 @@
       <c r="R45" t="s">
         <v>1674</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7938,7 +7964,7 @@
       <c r="J46" t="s">
         <v>1500</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7982,7 +8008,7 @@
       <c r="J47" t="s">
         <v>1500</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8000,7 +8026,7 @@
       <c r="R47" t="s">
         <v>1675</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8041,7 +8067,7 @@
       <c r="J48" t="s">
         <v>1500</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8085,7 +8111,7 @@
       <c r="J49" t="s">
         <v>1500</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8129,7 +8155,7 @@
       <c r="J50" t="s">
         <v>1500</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8173,7 +8199,7 @@
       <c r="J51" t="s">
         <v>1500</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8220,7 +8246,7 @@
       <c r="J52" t="s">
         <v>1500</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8264,7 +8290,7 @@
       <c r="J53" t="s">
         <v>1500</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8308,7 +8334,7 @@
       <c r="J54" t="s">
         <v>1500</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8352,7 +8378,7 @@
       <c r="J55" t="s">
         <v>1500</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8402,7 +8428,7 @@
       <c r="J56" t="s">
         <v>1500</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8455,7 +8481,7 @@
       <c r="J57" t="s">
         <v>1500</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8505,7 +8531,7 @@
       <c r="J58" t="s">
         <v>1500</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8555,7 +8581,7 @@
       <c r="J59" t="s">
         <v>1500</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8573,7 +8599,7 @@
       <c r="R59" t="s">
         <v>1676</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8614,7 +8640,7 @@
       <c r="J60" t="s">
         <v>1500</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8658,7 +8684,7 @@
       <c r="J61" t="s">
         <v>1500</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8702,7 +8728,7 @@
       <c r="J62" t="s">
         <v>1500</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8746,7 +8772,7 @@
       <c r="J63" t="s">
         <v>1500</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8790,7 +8816,7 @@
       <c r="J64" t="s">
         <v>1500</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8834,7 +8860,7 @@
       <c r="J65" t="s">
         <v>1500</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8881,7 +8907,7 @@
       <c r="J66" t="s">
         <v>1500</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8899,7 +8925,7 @@
       <c r="R66" t="s">
         <v>1677</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8937,7 +8963,7 @@
       <c r="J67" t="s">
         <v>1500</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8981,7 +9007,7 @@
       <c r="J68" t="s">
         <v>1500</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8996,7 +9022,7 @@
       <c r="O68" t="s">
         <v>1580</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9040,7 +9066,7 @@
       <c r="J69" t="s">
         <v>1502</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9084,7 +9110,7 @@
       <c r="J70" t="s">
         <v>1500</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9128,7 +9154,7 @@
       <c r="J71" t="s">
         <v>1500</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9172,7 +9198,7 @@
       <c r="J72" t="s">
         <v>1500</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9216,7 +9242,7 @@
       <c r="J73" t="s">
         <v>1500</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9260,7 +9286,7 @@
       <c r="J74" t="s">
         <v>1500</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9304,7 +9330,7 @@
       <c r="J75" t="s">
         <v>1500</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9348,7 +9374,7 @@
       <c r="J76" t="s">
         <v>1500</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9366,7 +9392,7 @@
       <c r="R76" t="s">
         <v>1678</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9404,7 +9430,7 @@
       <c r="J77" t="s">
         <v>1500</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9422,7 +9448,7 @@
       <c r="R77" t="s">
         <v>1678</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9460,7 +9486,7 @@
       <c r="J78" t="s">
         <v>1500</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9478,7 +9504,7 @@
       <c r="R78" t="s">
         <v>1678</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9516,7 +9542,7 @@
       <c r="J79" t="s">
         <v>1500</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9534,7 +9560,7 @@
       <c r="R79" t="s">
         <v>1678</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9572,7 +9598,7 @@
       <c r="J80" t="s">
         <v>1500</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9616,7 +9642,7 @@
       <c r="J81" t="s">
         <v>1500</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9660,7 +9686,7 @@
       <c r="J82" t="s">
         <v>1500</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9704,7 +9730,7 @@
       <c r="J83" t="s">
         <v>1500</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9748,7 +9774,7 @@
       <c r="J84" t="s">
         <v>1500</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9792,7 +9818,7 @@
       <c r="J85" t="s">
         <v>1500</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9810,7 +9836,7 @@
       <c r="R85" t="s">
         <v>1679</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9848,7 +9874,7 @@
       <c r="J86" t="s">
         <v>1500</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9892,7 +9918,7 @@
       <c r="J87" t="s">
         <v>1500</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9910,7 +9936,7 @@
       <c r="R87" t="s">
         <v>1680</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9948,7 +9974,7 @@
       <c r="J88" t="s">
         <v>1500</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9992,7 +10018,7 @@
       <c r="J89" t="s">
         <v>1500</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10010,7 +10036,7 @@
       <c r="R89" t="s">
         <v>1681</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10045,7 +10071,7 @@
       <c r="J90" t="s">
         <v>1500</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10063,7 +10089,7 @@
       <c r="R90" t="s">
         <v>1682</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10098,7 +10124,7 @@
       <c r="J91" t="s">
         <v>1500</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10116,7 +10142,7 @@
       <c r="R91" t="s">
         <v>1666</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10154,7 +10180,7 @@
       <c r="J92" t="s">
         <v>1500</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10175,7 +10201,7 @@
       <c r="R92" t="s">
         <v>1666</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10216,7 +10242,7 @@
       <c r="J93" t="s">
         <v>1500</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10257,7 +10283,7 @@
       <c r="J94" t="s">
         <v>1500</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10301,7 +10327,7 @@
       <c r="J95" t="s">
         <v>1500</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10345,7 +10371,7 @@
       <c r="J96" t="s">
         <v>1500</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10363,7 +10389,7 @@
       <c r="R96" t="s">
         <v>1683</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10401,7 +10427,7 @@
       <c r="J97" t="s">
         <v>1500</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10416,7 +10442,7 @@
       <c r="R97" t="s">
         <v>1683</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10457,7 +10483,7 @@
       <c r="J98" t="s">
         <v>1500</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10475,7 +10501,7 @@
       <c r="R98" t="s">
         <v>1684</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10513,7 +10539,7 @@
       <c r="J99" t="s">
         <v>1500</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10531,7 +10557,7 @@
       <c r="R99" t="s">
         <v>1685</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10569,7 +10595,7 @@
       <c r="J100" t="s">
         <v>1500</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10610,7 +10636,7 @@
       <c r="J101" t="s">
         <v>1500</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10651,7 +10677,7 @@
       <c r="J102" t="s">
         <v>1500</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10692,7 +10718,7 @@
       <c r="J103" t="s">
         <v>1500</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10733,7 +10759,7 @@
       <c r="J104" t="s">
         <v>1500</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10774,7 +10800,7 @@
       <c r="J105" t="s">
         <v>1500</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10815,7 +10841,7 @@
       <c r="J106" t="s">
         <v>1500</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10856,7 +10882,7 @@
       <c r="J107" t="s">
         <v>1500</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10897,7 +10923,7 @@
       <c r="J108" t="s">
         <v>1500</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10938,7 +10964,7 @@
       <c r="J109" t="s">
         <v>1500</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10991,7 +11017,7 @@
       <c r="J110" t="s">
         <v>1500</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11047,7 +11073,7 @@
       <c r="J111" t="s">
         <v>1500</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11065,7 +11091,7 @@
       <c r="R111" t="s">
         <v>1687</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11103,7 +11129,7 @@
       <c r="J112" t="s">
         <v>1500</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11162,7 +11188,7 @@
       <c r="J113" t="s">
         <v>1500</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11206,7 +11232,7 @@
       <c r="J114" t="s">
         <v>1500</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11250,7 +11276,7 @@
       <c r="J115" t="s">
         <v>1500</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11268,7 +11294,7 @@
       <c r="R115" t="s">
         <v>1689</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11306,7 +11332,7 @@
       <c r="J116" t="s">
         <v>1500</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11365,7 +11391,7 @@
       <c r="J117" t="s">
         <v>1500</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11409,7 +11435,7 @@
       <c r="J118" t="s">
         <v>1500</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11456,7 +11482,7 @@
       <c r="J119" t="s">
         <v>1500</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11497,7 +11523,7 @@
       <c r="J120" t="s">
         <v>1500</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11541,7 +11567,7 @@
       <c r="J121" t="s">
         <v>1500</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11588,7 +11614,7 @@
       <c r="J122" t="s">
         <v>1500</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11638,7 +11664,7 @@
       <c r="J123" t="s">
         <v>1500</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11682,7 +11708,7 @@
       <c r="J124" t="s">
         <v>1500</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11726,7 +11752,7 @@
       <c r="J125" t="s">
         <v>1500</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11744,7 +11770,7 @@
       <c r="R125" t="s">
         <v>1691</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11779,7 +11805,7 @@
       <c r="J126" t="s">
         <v>1500</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11797,7 +11823,7 @@
       <c r="R126" t="s">
         <v>1692</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11832,7 +11858,7 @@
       <c r="J127" t="s">
         <v>1500</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11888,7 +11914,7 @@
       <c r="J128" t="s">
         <v>1500</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11929,7 +11955,7 @@
       <c r="J129" t="s">
         <v>1500</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11970,7 +11996,7 @@
       <c r="J130" t="s">
         <v>1500</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12011,7 +12037,7 @@
       <c r="J131" t="s">
         <v>1500</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12055,7 +12081,7 @@
       <c r="J132" t="s">
         <v>1500</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12096,7 +12122,7 @@
       <c r="J133" t="s">
         <v>1500</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12114,7 +12140,7 @@
       <c r="R133" t="s">
         <v>1678</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12149,7 +12175,7 @@
       <c r="J134" t="s">
         <v>1500</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12167,7 +12193,7 @@
       <c r="R134" t="s">
         <v>1678</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12202,7 +12228,7 @@
       <c r="J135" t="s">
         <v>1500</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12243,7 +12269,7 @@
       <c r="J136" t="s">
         <v>1500</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12284,7 +12310,7 @@
       <c r="J137" t="s">
         <v>1500</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12325,7 +12351,7 @@
       <c r="J138" t="s">
         <v>1500</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12366,7 +12392,7 @@
       <c r="J139" t="s">
         <v>1500</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12413,7 +12439,7 @@
       <c r="J140" t="s">
         <v>1500</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12454,7 +12480,7 @@
       <c r="J141" t="s">
         <v>1500</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12495,7 +12521,7 @@
       <c r="J142" t="s">
         <v>1500</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12539,7 +12565,7 @@
       <c r="J143" t="s">
         <v>1500</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12557,7 +12583,7 @@
       <c r="R143" t="s">
         <v>1678</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12592,7 +12618,7 @@
       <c r="J144" t="s">
         <v>1500</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12610,7 +12636,7 @@
       <c r="R144" t="s">
         <v>1678</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12645,7 +12671,7 @@
       <c r="J145" t="s">
         <v>1500</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12663,7 +12689,7 @@
       <c r="R145" t="s">
         <v>1678</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12698,7 +12724,7 @@
       <c r="J146" t="s">
         <v>1500</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12716,7 +12742,7 @@
       <c r="R146" t="s">
         <v>1686</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12751,7 +12777,7 @@
       <c r="J147" t="s">
         <v>1500</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12769,7 +12795,7 @@
       <c r="R147" t="s">
         <v>1693</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12804,7 +12830,7 @@
       <c r="J148" t="s">
         <v>1500</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12845,7 +12871,7 @@
       <c r="J149" t="s">
         <v>1500</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12863,7 +12889,7 @@
       <c r="R149" t="s">
         <v>1678</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12898,7 +12924,7 @@
       <c r="J150" t="s">
         <v>1500</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12916,7 +12942,7 @@
       <c r="R150" t="s">
         <v>1678</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12951,7 +12977,7 @@
       <c r="J151" t="s">
         <v>1500</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12969,7 +12995,7 @@
       <c r="R151" t="s">
         <v>1694</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13004,7 +13030,7 @@
       <c r="J152" t="s">
         <v>1500</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13022,7 +13048,7 @@
       <c r="R152" t="s">
         <v>1695</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13057,7 +13083,7 @@
       <c r="J153" t="s">
         <v>1500</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13066,7 +13092,7 @@
       <c r="M153" t="s">
         <v>1571</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13107,7 +13133,7 @@
       <c r="J154" t="s">
         <v>1500</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13148,7 +13174,7 @@
       <c r="J155" t="s">
         <v>1500</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13189,7 +13215,7 @@
       <c r="J156" t="s">
         <v>1500</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13230,7 +13256,7 @@
       <c r="J157" t="s">
         <v>1500</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13271,7 +13297,7 @@
       <c r="J158" t="s">
         <v>1500</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13312,7 +13338,7 @@
       <c r="J159" t="s">
         <v>1500</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13353,7 +13379,7 @@
       <c r="J160" t="s">
         <v>1500</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13394,7 +13420,7 @@
       <c r="J161" t="s">
         <v>1500</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13435,7 +13461,7 @@
       <c r="J162" t="s">
         <v>1500</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13453,7 +13479,7 @@
       <c r="R162" t="s">
         <v>1681</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13488,7 +13514,7 @@
       <c r="J163" t="s">
         <v>1500</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13506,7 +13532,7 @@
       <c r="R163" t="s">
         <v>1678</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13541,7 +13567,7 @@
       <c r="J164" t="s">
         <v>1500</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13585,7 +13611,7 @@
       <c r="J165" t="s">
         <v>1500</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13626,7 +13652,7 @@
       <c r="J166" t="s">
         <v>1500</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13644,7 +13670,7 @@
       <c r="R166" t="s">
         <v>1696</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13679,7 +13705,7 @@
       <c r="J167" t="s">
         <v>1500</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13723,7 +13749,7 @@
       <c r="J168" t="s">
         <v>1500</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13767,7 +13793,7 @@
       <c r="J169" t="s">
         <v>1500</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13808,7 +13834,7 @@
       <c r="J170" t="s">
         <v>1500</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13849,7 +13875,7 @@
       <c r="J171" t="s">
         <v>1500</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13890,7 +13916,7 @@
       <c r="J172" t="s">
         <v>1500</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13931,7 +13957,7 @@
       <c r="J173" t="s">
         <v>1500</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13972,7 +13998,7 @@
       <c r="J174" t="s">
         <v>1500</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14013,7 +14039,7 @@
       <c r="J175" t="s">
         <v>1500</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14054,7 +14080,7 @@
       <c r="J176" t="s">
         <v>1500</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14095,7 +14121,7 @@
       <c r="J177" t="s">
         <v>1500</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14136,7 +14162,7 @@
       <c r="J178" t="s">
         <v>1500</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14154,7 +14180,7 @@
       <c r="R178" t="s">
         <v>1694</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14189,7 +14215,7 @@
       <c r="J179" t="s">
         <v>1500</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14198,7 +14224,7 @@
       <c r="M179" t="s">
         <v>1568</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14239,7 +14265,7 @@
       <c r="J180" t="s">
         <v>1500</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14280,7 +14306,7 @@
       <c r="J181" t="s">
         <v>1500</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14298,7 +14324,7 @@
       <c r="R181" t="s">
         <v>1678</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14333,7 +14359,7 @@
       <c r="J182" t="s">
         <v>1500</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14374,7 +14400,7 @@
       <c r="J183" t="s">
         <v>1500</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14415,7 +14441,7 @@
       <c r="J184" t="s">
         <v>1500</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14456,7 +14482,7 @@
       <c r="J185" t="s">
         <v>1500</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14497,7 +14523,7 @@
       <c r="J186" t="s">
         <v>1500</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14538,7 +14564,7 @@
       <c r="J187" t="s">
         <v>1500</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14579,7 +14605,7 @@
       <c r="J188" t="s">
         <v>1500</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14620,7 +14646,7 @@
       <c r="J189" t="s">
         <v>1500</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14661,7 +14687,7 @@
       <c r="J190" t="s">
         <v>1500</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14702,7 +14728,7 @@
       <c r="J191" t="s">
         <v>1500</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14743,7 +14769,7 @@
       <c r="J192" t="s">
         <v>1500</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14784,7 +14810,7 @@
       <c r="J193" t="s">
         <v>1500</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14825,7 +14851,7 @@
       <c r="J194" t="s">
         <v>1500</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14866,7 +14892,7 @@
       <c r="J195" t="s">
         <v>1500</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14884,7 +14910,7 @@
       <c r="R195" t="s">
         <v>1687</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14922,7 +14948,7 @@
       <c r="J196" t="s">
         <v>1500</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14940,7 +14966,7 @@
       <c r="R196" t="s">
         <v>1693</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14978,7 +15004,7 @@
       <c r="J197" t="s">
         <v>1500</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15019,7 +15045,7 @@
       <c r="J198" t="s">
         <v>1502</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15060,7 +15086,7 @@
       <c r="J199" t="s">
         <v>1501</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15101,7 +15127,7 @@
       <c r="J200" t="s">
         <v>1500</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15142,7 +15168,7 @@
       <c r="J201" t="s">
         <v>1500</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15183,7 +15209,7 @@
       <c r="J202" t="s">
         <v>1500</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15201,7 +15227,7 @@
       <c r="R202" t="s">
         <v>1678</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15236,7 +15262,7 @@
       <c r="J203" t="s">
         <v>1500</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15254,7 +15280,7 @@
       <c r="R203" t="s">
         <v>1686</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15289,7 +15315,7 @@
       <c r="J204" t="s">
         <v>1500</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15304,7 +15330,7 @@
       <c r="R204" t="s">
         <v>1697</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15342,7 +15368,7 @@
       <c r="J205" t="s">
         <v>1500</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15360,7 +15386,7 @@
       <c r="R205" t="s">
         <v>1698</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15398,7 +15424,7 @@
       <c r="J206" t="s">
         <v>1500</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15416,7 +15442,7 @@
       <c r="R206" t="s">
         <v>1666</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15451,7 +15477,7 @@
       <c r="J207" t="s">
         <v>1500</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15492,7 +15518,7 @@
       <c r="J208" t="s">
         <v>1500</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15533,7 +15559,7 @@
       <c r="J209" t="s">
         <v>1500</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15574,7 +15600,7 @@
       <c r="J210" t="s">
         <v>1500</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15615,7 +15641,7 @@
       <c r="J211" t="s">
         <v>1500</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15656,7 +15682,7 @@
       <c r="J212" t="s">
         <v>1500</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15697,7 +15723,7 @@
       <c r="J213" t="s">
         <v>1500</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15738,7 +15764,7 @@
       <c r="J214" t="s">
         <v>1500</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15756,7 +15782,7 @@
       <c r="R214" t="s">
         <v>1699</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15791,7 +15817,7 @@
       <c r="J215" t="s">
         <v>1500</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15832,7 +15858,7 @@
       <c r="J216" t="s">
         <v>1500</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15873,7 +15899,7 @@
       <c r="J217" t="s">
         <v>1500</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15914,7 +15940,7 @@
       <c r="J218" t="s">
         <v>1500</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15955,7 +15981,7 @@
       <c r="J219" t="s">
         <v>1500</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15996,7 +16022,7 @@
       <c r="J220" t="s">
         <v>1500</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16037,7 +16063,7 @@
       <c r="J221" t="s">
         <v>1500</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16078,7 +16104,7 @@
       <c r="J222" t="s">
         <v>1500</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16119,7 +16145,7 @@
       <c r="J223" t="s">
         <v>1500</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16160,7 +16186,7 @@
       <c r="J224" t="s">
         <v>1500</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16201,7 +16227,7 @@
       <c r="J225" t="s">
         <v>1500</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16242,7 +16268,7 @@
       <c r="J226" t="s">
         <v>1500</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16283,7 +16309,7 @@
       <c r="J227" t="s">
         <v>1500</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16324,7 +16350,7 @@
       <c r="J228" t="s">
         <v>1500</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16365,7 +16391,7 @@
       <c r="J229" t="s">
         <v>1500</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16406,7 +16432,7 @@
       <c r="J230" t="s">
         <v>1500</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16447,7 +16473,7 @@
       <c r="J231" t="s">
         <v>1500</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16488,7 +16514,7 @@
       <c r="J232" t="s">
         <v>1500</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16529,7 +16555,7 @@
       <c r="J233" t="s">
         <v>1500</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16570,7 +16596,7 @@
       <c r="J234" t="s">
         <v>1500</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16611,7 +16637,7 @@
       <c r="J235" t="s">
         <v>1500</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16652,7 +16678,7 @@
       <c r="J236" t="s">
         <v>1500</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16693,7 +16719,7 @@
       <c r="J237" t="s">
         <v>1500</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16734,7 +16760,7 @@
       <c r="J238" t="s">
         <v>1500</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16775,7 +16801,7 @@
       <c r="J239" t="s">
         <v>1500</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16793,7 +16819,7 @@
       <c r="R239" t="s">
         <v>1693</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16828,7 +16854,7 @@
       <c r="J240" t="s">
         <v>1500</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16869,7 +16895,7 @@
       <c r="J241" t="s">
         <v>1500</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16910,7 +16936,7 @@
       <c r="J242" t="s">
         <v>1500</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16928,7 +16954,7 @@
       <c r="R242" t="s">
         <v>1686</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16963,7 +16989,7 @@
       <c r="J243" t="s">
         <v>1500</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17004,7 +17030,7 @@
       <c r="J244" t="s">
         <v>1500</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17045,7 +17071,7 @@
       <c r="J245" t="s">
         <v>1500</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17086,7 +17112,7 @@
       <c r="J246" t="s">
         <v>1500</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17104,7 +17130,7 @@
       <c r="R246" t="s">
         <v>1666</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17139,7 +17165,7 @@
       <c r="J247" t="s">
         <v>1500</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17180,7 +17206,7 @@
       <c r="J248" t="s">
         <v>1500</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17221,7 +17247,7 @@
       <c r="J249" t="s">
         <v>1500</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17262,7 +17288,7 @@
       <c r="J250" t="s">
         <v>1500</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17303,7 +17329,7 @@
       <c r="J251" t="s">
         <v>1500</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17344,7 +17370,7 @@
       <c r="J252" t="s">
         <v>1500</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17385,7 +17411,7 @@
       <c r="J253" t="s">
         <v>1500</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17403,7 +17429,7 @@
       <c r="R253" t="s">
         <v>1696</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17441,7 +17467,7 @@
       <c r="J254" t="s">
         <v>1500</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17482,7 +17508,7 @@
       <c r="J255" t="s">
         <v>1500</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17523,7 +17549,7 @@
       <c r="J256" t="s">
         <v>1500</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17532,7 +17558,7 @@
       <c r="M256" t="s">
         <v>1567</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17570,7 +17596,7 @@
       <c r="J257" t="s">
         <v>1500</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17579,7 +17605,7 @@
       <c r="M257" t="s">
         <v>1568</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17623,7 +17649,7 @@
       <c r="J258" t="s">
         <v>1500</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17641,7 +17667,7 @@
       <c r="R258" t="s">
         <v>1678</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17679,7 +17705,7 @@
       <c r="J259" t="s">
         <v>1500</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17697,7 +17723,7 @@
       <c r="R259" t="s">
         <v>1694</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17735,7 +17761,7 @@
       <c r="J260" t="s">
         <v>1500</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17744,7 +17770,7 @@
       <c r="M260" t="s">
         <v>1562</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17788,7 +17814,7 @@
       <c r="J261" t="s">
         <v>1500</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17806,7 +17832,7 @@
       <c r="R261" t="s">
         <v>1700</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17844,7 +17870,7 @@
       <c r="J262" t="s">
         <v>1500</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17862,7 +17888,7 @@
       <c r="R262" t="s">
         <v>1694</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17900,7 +17926,7 @@
       <c r="J263" t="s">
         <v>1500</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17909,7 +17935,7 @@
       <c r="M263" t="s">
         <v>1562</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17953,7 +17979,7 @@
       <c r="J264" t="s">
         <v>1500</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17994,7 +18020,7 @@
       <c r="J265" t="s">
         <v>1500</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18035,7 +18061,7 @@
       <c r="J266" t="s">
         <v>1500</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18076,7 +18102,7 @@
       <c r="J267" t="s">
         <v>1500</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18120,7 +18146,7 @@
       <c r="J268" t="s">
         <v>1500</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18161,7 +18187,7 @@
       <c r="J269" t="s">
         <v>1500</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18202,7 +18228,7 @@
       <c r="J270" t="s">
         <v>1500</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18243,7 +18269,7 @@
       <c r="J271" t="s">
         <v>1500</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18284,7 +18310,7 @@
       <c r="J272" t="s">
         <v>1500</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18302,7 +18328,7 @@
       <c r="R272" t="s">
         <v>1701</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18340,7 +18366,7 @@
       <c r="J273" t="s">
         <v>1500</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18384,7 +18410,7 @@
       <c r="J274" t="s">
         <v>1500</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18425,7 +18451,7 @@
       <c r="J275" t="s">
         <v>1500</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18466,7 +18492,7 @@
       <c r="J276" t="s">
         <v>1500</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18507,7 +18533,7 @@
       <c r="J277" t="s">
         <v>1500</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18548,7 +18574,7 @@
       <c r="J278" t="s">
         <v>1500</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18589,7 +18615,7 @@
       <c r="J279" t="s">
         <v>1500</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18630,7 +18656,7 @@
       <c r="J280" t="s">
         <v>1500</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18671,7 +18697,7 @@
       <c r="J281" t="s">
         <v>1500</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18712,7 +18738,7 @@
       <c r="J282" t="s">
         <v>1500</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18753,7 +18779,7 @@
       <c r="J283" t="s">
         <v>1500</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18794,7 +18820,7 @@
       <c r="J284" t="s">
         <v>1500</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18835,7 +18861,7 @@
       <c r="J285" t="s">
         <v>1500</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18876,7 +18902,7 @@
       <c r="J286" t="s">
         <v>1500</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18917,7 +18943,7 @@
       <c r="J287" t="s">
         <v>1500</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18958,7 +18984,7 @@
       <c r="J288" t="s">
         <v>1500</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18999,7 +19025,7 @@
       <c r="J289" t="s">
         <v>1500</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19040,7 +19066,7 @@
       <c r="J290" t="s">
         <v>1500</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19081,7 +19107,7 @@
       <c r="J291" t="s">
         <v>1500</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19122,7 +19148,7 @@
       <c r="J292" t="s">
         <v>1500</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19163,7 +19189,7 @@
       <c r="J293" t="s">
         <v>1500</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19204,7 +19230,7 @@
       <c r="J294" t="s">
         <v>1500</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19245,7 +19271,7 @@
       <c r="J295" t="s">
         <v>1500</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19263,7 +19289,7 @@
       <c r="R295" t="s">
         <v>1702</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19301,7 +19327,7 @@
       <c r="J296" t="s">
         <v>1500</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19319,7 +19345,7 @@
       <c r="R296" t="s">
         <v>1678</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19357,7 +19383,7 @@
       <c r="J297" t="s">
         <v>1500</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19398,7 +19424,7 @@
       <c r="J298" t="s">
         <v>1500</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19439,7 +19465,7 @@
       <c r="J299" t="s">
         <v>1501</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19480,7 +19506,7 @@
       <c r="J300" t="s">
         <v>1500</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19521,7 +19547,7 @@
       <c r="J301" t="s">
         <v>1500</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20359,7 +20385,7 @@
       <c r="R321" t="s">
         <v>1664</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20579,7 +20605,7 @@
       <c r="R326" t="s">
         <v>1703</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21414,7 +21440,7 @@
       <c r="R346" t="s">
         <v>1704</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (01/09/2026 12:29)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5244,16 +5244,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5269,7 +5261,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5277,30 +5269,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5600,73 +5574,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5701,7 +5675,7 @@
       <c r="J2" t="s">
         <v>1500</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5745,7 +5719,7 @@
       <c r="J3" t="s">
         <v>1500</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5789,7 +5763,7 @@
       <c r="J4" t="s">
         <v>1500</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5807,7 +5781,7 @@
       <c r="R4" t="s">
         <v>1661</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5845,7 +5819,7 @@
       <c r="J5" t="s">
         <v>1501</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5895,7 +5869,7 @@
       <c r="J6" t="s">
         <v>1500</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5942,7 +5916,7 @@
       <c r="J7" t="s">
         <v>1500</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5989,7 +5963,7 @@
       <c r="J8" t="s">
         <v>1500</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6036,7 +6010,7 @@
       <c r="J9" t="s">
         <v>1500</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6083,7 +6057,7 @@
       <c r="J10" t="s">
         <v>1500</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6130,7 +6104,7 @@
       <c r="J11" t="s">
         <v>1500</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6177,7 +6151,7 @@
       <c r="J12" t="s">
         <v>1500</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6221,7 +6195,7 @@
       <c r="J13" t="s">
         <v>1500</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6239,7 +6213,7 @@
       <c r="R13" t="s">
         <v>1662</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6277,7 +6251,7 @@
       <c r="J14" t="s">
         <v>1500</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6295,7 +6269,7 @@
       <c r="R14" t="s">
         <v>1663</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6333,7 +6307,7 @@
       <c r="J15" t="s">
         <v>1500</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6351,7 +6325,7 @@
       <c r="R15" t="s">
         <v>1663</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6389,7 +6363,7 @@
       <c r="J16" t="s">
         <v>1500</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6433,7 +6407,7 @@
       <c r="J17" t="s">
         <v>1500</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6477,7 +6451,7 @@
       <c r="J18" t="s">
         <v>1500</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6495,7 +6469,7 @@
       <c r="R18" t="s">
         <v>1664</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6536,7 +6510,7 @@
       <c r="J19" t="s">
         <v>1500</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6580,7 +6554,7 @@
       <c r="J20" t="s">
         <v>1500</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6624,7 +6598,7 @@
       <c r="J21" t="s">
         <v>1500</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6642,7 +6616,7 @@
       <c r="R21" t="s">
         <v>1663</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6683,7 +6657,7 @@
       <c r="J22" t="s">
         <v>1500</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6701,7 +6675,7 @@
       <c r="R22" t="s">
         <v>1665</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6742,7 +6716,7 @@
       <c r="J23" t="s">
         <v>1500</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6760,7 +6734,7 @@
       <c r="R23" t="s">
         <v>1666</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6801,7 +6775,7 @@
       <c r="J24" t="s">
         <v>1500</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6845,7 +6819,7 @@
       <c r="J25" t="s">
         <v>1500</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6886,7 +6860,7 @@
       <c r="J26" t="s">
         <v>1502</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6904,7 +6878,7 @@
       <c r="R26" t="s">
         <v>1667</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6939,7 +6913,7 @@
       <c r="J27" t="s">
         <v>1500</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6957,7 +6931,7 @@
       <c r="R27" t="s">
         <v>1668</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6998,7 +6972,7 @@
       <c r="J28" t="s">
         <v>1500</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7042,7 +7016,7 @@
       <c r="J29" t="s">
         <v>1500</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7086,7 +7060,7 @@
       <c r="J30" t="s">
         <v>1500</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7130,7 +7104,7 @@
       <c r="J31" t="s">
         <v>1500</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7148,7 +7122,7 @@
       <c r="R31" t="s">
         <v>1669</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7189,7 +7163,7 @@
       <c r="J32" t="s">
         <v>1500</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7233,7 +7207,7 @@
       <c r="J33" t="s">
         <v>1500</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7251,7 +7225,7 @@
       <c r="R33" t="s">
         <v>1670</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7292,7 +7266,7 @@
       <c r="J34" t="s">
         <v>1500</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7336,7 +7310,7 @@
       <c r="J35" t="s">
         <v>1500</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7354,7 +7328,7 @@
       <c r="R35" t="s">
         <v>1671</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7395,7 +7369,7 @@
       <c r="J36" t="s">
         <v>1500</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7413,7 +7387,7 @@
       <c r="R36" t="s">
         <v>1671</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7454,7 +7428,7 @@
       <c r="J37" t="s">
         <v>1500</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7472,7 +7446,7 @@
       <c r="R37" t="s">
         <v>1671</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7513,7 +7487,7 @@
       <c r="J38" t="s">
         <v>1500</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7531,7 +7505,7 @@
       <c r="R38" t="s">
         <v>1671</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7572,7 +7546,7 @@
       <c r="J39" t="s">
         <v>1500</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7590,7 +7564,7 @@
       <c r="R39" t="s">
         <v>1671</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7631,7 +7605,7 @@
       <c r="J40" t="s">
         <v>1500</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7649,7 +7623,7 @@
       <c r="R40" t="s">
         <v>1672</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7690,7 +7664,7 @@
       <c r="J41" t="s">
         <v>1500</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7708,7 +7682,7 @@
       <c r="R41" t="s">
         <v>1663</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7746,7 +7720,7 @@
       <c r="J42" t="s">
         <v>1500</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7764,7 +7738,7 @@
       <c r="R42" t="s">
         <v>1671</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7805,7 +7779,7 @@
       <c r="J43" t="s">
         <v>1500</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7849,7 +7823,7 @@
       <c r="J44" t="s">
         <v>1500</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7867,7 +7841,7 @@
       <c r="R44" t="s">
         <v>1673</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7908,7 +7882,7 @@
       <c r="J45" t="s">
         <v>1500</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7926,7 +7900,7 @@
       <c r="R45" t="s">
         <v>1674</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7964,7 +7938,7 @@
       <c r="J46" t="s">
         <v>1500</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8008,7 +7982,7 @@
       <c r="J47" t="s">
         <v>1500</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8026,7 +8000,7 @@
       <c r="R47" t="s">
         <v>1675</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8067,7 +8041,7 @@
       <c r="J48" t="s">
         <v>1500</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8111,7 +8085,7 @@
       <c r="J49" t="s">
         <v>1500</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8155,7 +8129,7 @@
       <c r="J50" t="s">
         <v>1500</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8199,7 +8173,7 @@
       <c r="J51" t="s">
         <v>1500</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8246,7 +8220,7 @@
       <c r="J52" t="s">
         <v>1500</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8290,7 +8264,7 @@
       <c r="J53" t="s">
         <v>1500</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8334,7 +8308,7 @@
       <c r="J54" t="s">
         <v>1500</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8378,7 +8352,7 @@
       <c r="J55" t="s">
         <v>1500</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8428,7 +8402,7 @@
       <c r="J56" t="s">
         <v>1500</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8481,7 +8455,7 @@
       <c r="J57" t="s">
         <v>1500</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8531,7 +8505,7 @@
       <c r="J58" t="s">
         <v>1500</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8581,7 +8555,7 @@
       <c r="J59" t="s">
         <v>1500</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8599,7 +8573,7 @@
       <c r="R59" t="s">
         <v>1676</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8640,7 +8614,7 @@
       <c r="J60" t="s">
         <v>1500</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8684,7 +8658,7 @@
       <c r="J61" t="s">
         <v>1500</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8728,7 +8702,7 @@
       <c r="J62" t="s">
         <v>1500</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8772,7 +8746,7 @@
       <c r="J63" t="s">
         <v>1500</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8816,7 +8790,7 @@
       <c r="J64" t="s">
         <v>1500</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8860,7 +8834,7 @@
       <c r="J65" t="s">
         <v>1500</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8907,7 +8881,7 @@
       <c r="J66" t="s">
         <v>1500</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8925,7 +8899,7 @@
       <c r="R66" t="s">
         <v>1677</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8963,7 +8937,7 @@
       <c r="J67" t="s">
         <v>1500</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9007,7 +8981,7 @@
       <c r="J68" t="s">
         <v>1500</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9022,7 +8996,7 @@
       <c r="O68" t="s">
         <v>1580</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9066,7 +9040,7 @@
       <c r="J69" t="s">
         <v>1502</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9110,7 +9084,7 @@
       <c r="J70" t="s">
         <v>1500</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9154,7 +9128,7 @@
       <c r="J71" t="s">
         <v>1500</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9198,7 +9172,7 @@
       <c r="J72" t="s">
         <v>1500</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9242,7 +9216,7 @@
       <c r="J73" t="s">
         <v>1500</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9286,7 +9260,7 @@
       <c r="J74" t="s">
         <v>1500</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9330,7 +9304,7 @@
       <c r="J75" t="s">
         <v>1500</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9374,7 +9348,7 @@
       <c r="J76" t="s">
         <v>1500</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9392,7 +9366,7 @@
       <c r="R76" t="s">
         <v>1678</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9430,7 +9404,7 @@
       <c r="J77" t="s">
         <v>1500</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9448,7 +9422,7 @@
       <c r="R77" t="s">
         <v>1678</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9486,7 +9460,7 @@
       <c r="J78" t="s">
         <v>1500</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9504,7 +9478,7 @@
       <c r="R78" t="s">
         <v>1678</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9542,7 +9516,7 @@
       <c r="J79" t="s">
         <v>1500</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9560,7 +9534,7 @@
       <c r="R79" t="s">
         <v>1678</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9598,7 +9572,7 @@
       <c r="J80" t="s">
         <v>1500</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9642,7 +9616,7 @@
       <c r="J81" t="s">
         <v>1500</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9686,7 +9660,7 @@
       <c r="J82" t="s">
         <v>1500</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9730,7 +9704,7 @@
       <c r="J83" t="s">
         <v>1500</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9774,7 +9748,7 @@
       <c r="J84" t="s">
         <v>1500</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9818,7 +9792,7 @@
       <c r="J85" t="s">
         <v>1500</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9836,7 +9810,7 @@
       <c r="R85" t="s">
         <v>1679</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9874,7 +9848,7 @@
       <c r="J86" t="s">
         <v>1500</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9918,7 +9892,7 @@
       <c r="J87" t="s">
         <v>1500</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9936,7 +9910,7 @@
       <c r="R87" t="s">
         <v>1680</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9974,7 +9948,7 @@
       <c r="J88" t="s">
         <v>1500</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10018,7 +9992,7 @@
       <c r="J89" t="s">
         <v>1500</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10036,7 +10010,7 @@
       <c r="R89" t="s">
         <v>1681</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10071,7 +10045,7 @@
       <c r="J90" t="s">
         <v>1500</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10089,7 +10063,7 @@
       <c r="R90" t="s">
         <v>1682</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10124,7 +10098,7 @@
       <c r="J91" t="s">
         <v>1500</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10142,7 +10116,7 @@
       <c r="R91" t="s">
         <v>1666</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10180,7 +10154,7 @@
       <c r="J92" t="s">
         <v>1500</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10201,7 +10175,7 @@
       <c r="R92" t="s">
         <v>1666</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10242,7 +10216,7 @@
       <c r="J93" t="s">
         <v>1500</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10283,7 +10257,7 @@
       <c r="J94" t="s">
         <v>1500</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10327,7 +10301,7 @@
       <c r="J95" t="s">
         <v>1500</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10371,7 +10345,7 @@
       <c r="J96" t="s">
         <v>1500</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10389,7 +10363,7 @@
       <c r="R96" t="s">
         <v>1683</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10427,7 +10401,7 @@
       <c r="J97" t="s">
         <v>1500</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10442,7 +10416,7 @@
       <c r="R97" t="s">
         <v>1683</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10483,7 +10457,7 @@
       <c r="J98" t="s">
         <v>1500</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10501,7 +10475,7 @@
       <c r="R98" t="s">
         <v>1684</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10539,7 +10513,7 @@
       <c r="J99" t="s">
         <v>1500</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10557,7 +10531,7 @@
       <c r="R99" t="s">
         <v>1685</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10595,7 +10569,7 @@
       <c r="J100" t="s">
         <v>1500</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10636,7 +10610,7 @@
       <c r="J101" t="s">
         <v>1500</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10677,7 +10651,7 @@
       <c r="J102" t="s">
         <v>1500</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10718,7 +10692,7 @@
       <c r="J103" t="s">
         <v>1500</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10759,7 +10733,7 @@
       <c r="J104" t="s">
         <v>1500</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10800,7 +10774,7 @@
       <c r="J105" t="s">
         <v>1500</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10841,7 +10815,7 @@
       <c r="J106" t="s">
         <v>1500</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10882,7 +10856,7 @@
       <c r="J107" t="s">
         <v>1500</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10923,7 +10897,7 @@
       <c r="J108" t="s">
         <v>1500</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10964,7 +10938,7 @@
       <c r="J109" t="s">
         <v>1500</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11017,7 +10991,7 @@
       <c r="J110" t="s">
         <v>1500</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11073,7 +11047,7 @@
       <c r="J111" t="s">
         <v>1500</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11091,7 +11065,7 @@
       <c r="R111" t="s">
         <v>1687</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11129,7 +11103,7 @@
       <c r="J112" t="s">
         <v>1500</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11188,7 +11162,7 @@
       <c r="J113" t="s">
         <v>1500</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11232,7 +11206,7 @@
       <c r="J114" t="s">
         <v>1500</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11276,7 +11250,7 @@
       <c r="J115" t="s">
         <v>1500</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11294,7 +11268,7 @@
       <c r="R115" t="s">
         <v>1689</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11332,7 +11306,7 @@
       <c r="J116" t="s">
         <v>1500</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11391,7 +11365,7 @@
       <c r="J117" t="s">
         <v>1500</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11435,7 +11409,7 @@
       <c r="J118" t="s">
         <v>1500</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11482,7 +11456,7 @@
       <c r="J119" t="s">
         <v>1500</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11523,7 +11497,7 @@
       <c r="J120" t="s">
         <v>1500</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11567,7 +11541,7 @@
       <c r="J121" t="s">
         <v>1500</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11614,7 +11588,7 @@
       <c r="J122" t="s">
         <v>1500</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11664,7 +11638,7 @@
       <c r="J123" t="s">
         <v>1500</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11708,7 +11682,7 @@
       <c r="J124" t="s">
         <v>1500</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11752,7 +11726,7 @@
       <c r="J125" t="s">
         <v>1500</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11770,7 +11744,7 @@
       <c r="R125" t="s">
         <v>1691</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11805,7 +11779,7 @@
       <c r="J126" t="s">
         <v>1500</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11823,7 +11797,7 @@
       <c r="R126" t="s">
         <v>1692</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11858,7 +11832,7 @@
       <c r="J127" t="s">
         <v>1500</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11914,7 +11888,7 @@
       <c r="J128" t="s">
         <v>1500</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11955,7 +11929,7 @@
       <c r="J129" t="s">
         <v>1500</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11996,7 +11970,7 @@
       <c r="J130" t="s">
         <v>1500</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12037,7 +12011,7 @@
       <c r="J131" t="s">
         <v>1500</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12081,7 +12055,7 @@
       <c r="J132" t="s">
         <v>1500</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12122,7 +12096,7 @@
       <c r="J133" t="s">
         <v>1500</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12140,7 +12114,7 @@
       <c r="R133" t="s">
         <v>1678</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12175,7 +12149,7 @@
       <c r="J134" t="s">
         <v>1500</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12193,7 +12167,7 @@
       <c r="R134" t="s">
         <v>1678</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12228,7 +12202,7 @@
       <c r="J135" t="s">
         <v>1500</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12269,7 +12243,7 @@
       <c r="J136" t="s">
         <v>1500</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12310,7 +12284,7 @@
       <c r="J137" t="s">
         <v>1500</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12351,7 +12325,7 @@
       <c r="J138" t="s">
         <v>1500</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12392,7 +12366,7 @@
       <c r="J139" t="s">
         <v>1500</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12439,7 +12413,7 @@
       <c r="J140" t="s">
         <v>1500</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12480,7 +12454,7 @@
       <c r="J141" t="s">
         <v>1500</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12521,7 +12495,7 @@
       <c r="J142" t="s">
         <v>1500</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12565,7 +12539,7 @@
       <c r="J143" t="s">
         <v>1500</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12583,7 +12557,7 @@
       <c r="R143" t="s">
         <v>1678</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12618,7 +12592,7 @@
       <c r="J144" t="s">
         <v>1500</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12636,7 +12610,7 @@
       <c r="R144" t="s">
         <v>1678</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12671,7 +12645,7 @@
       <c r="J145" t="s">
         <v>1500</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12689,7 +12663,7 @@
       <c r="R145" t="s">
         <v>1678</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12724,7 +12698,7 @@
       <c r="J146" t="s">
         <v>1500</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12742,7 +12716,7 @@
       <c r="R146" t="s">
         <v>1686</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12777,7 +12751,7 @@
       <c r="J147" t="s">
         <v>1500</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12795,7 +12769,7 @@
       <c r="R147" t="s">
         <v>1693</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12830,7 +12804,7 @@
       <c r="J148" t="s">
         <v>1500</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12871,7 +12845,7 @@
       <c r="J149" t="s">
         <v>1500</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12889,7 +12863,7 @@
       <c r="R149" t="s">
         <v>1678</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12924,7 +12898,7 @@
       <c r="J150" t="s">
         <v>1500</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12942,7 +12916,7 @@
       <c r="R150" t="s">
         <v>1678</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12977,7 +12951,7 @@
       <c r="J151" t="s">
         <v>1500</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12995,7 +12969,7 @@
       <c r="R151" t="s">
         <v>1694</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13030,7 +13004,7 @@
       <c r="J152" t="s">
         <v>1500</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13048,7 +13022,7 @@
       <c r="R152" t="s">
         <v>1695</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13083,7 +13057,7 @@
       <c r="J153" t="s">
         <v>1500</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13092,7 +13066,7 @@
       <c r="M153" t="s">
         <v>1571</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13133,7 +13107,7 @@
       <c r="J154" t="s">
         <v>1500</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13174,7 +13148,7 @@
       <c r="J155" t="s">
         <v>1500</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13215,7 +13189,7 @@
       <c r="J156" t="s">
         <v>1500</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13256,7 +13230,7 @@
       <c r="J157" t="s">
         <v>1500</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13297,7 +13271,7 @@
       <c r="J158" t="s">
         <v>1500</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13338,7 +13312,7 @@
       <c r="J159" t="s">
         <v>1500</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13379,7 +13353,7 @@
       <c r="J160" t="s">
         <v>1500</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13420,7 +13394,7 @@
       <c r="J161" t="s">
         <v>1500</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13461,7 +13435,7 @@
       <c r="J162" t="s">
         <v>1500</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13479,7 +13453,7 @@
       <c r="R162" t="s">
         <v>1681</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13514,7 +13488,7 @@
       <c r="J163" t="s">
         <v>1500</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13532,7 +13506,7 @@
       <c r="R163" t="s">
         <v>1678</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13567,7 +13541,7 @@
       <c r="J164" t="s">
         <v>1500</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13611,7 +13585,7 @@
       <c r="J165" t="s">
         <v>1500</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13652,7 +13626,7 @@
       <c r="J166" t="s">
         <v>1500</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13670,7 +13644,7 @@
       <c r="R166" t="s">
         <v>1696</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13705,7 +13679,7 @@
       <c r="J167" t="s">
         <v>1500</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13749,7 +13723,7 @@
       <c r="J168" t="s">
         <v>1500</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13793,7 +13767,7 @@
       <c r="J169" t="s">
         <v>1500</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13834,7 +13808,7 @@
       <c r="J170" t="s">
         <v>1500</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13875,7 +13849,7 @@
       <c r="J171" t="s">
         <v>1500</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13916,7 +13890,7 @@
       <c r="J172" t="s">
         <v>1500</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13957,7 +13931,7 @@
       <c r="J173" t="s">
         <v>1500</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13998,7 +13972,7 @@
       <c r="J174" t="s">
         <v>1500</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14039,7 +14013,7 @@
       <c r="J175" t="s">
         <v>1500</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14080,7 +14054,7 @@
       <c r="J176" t="s">
         <v>1500</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14121,7 +14095,7 @@
       <c r="J177" t="s">
         <v>1500</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14162,7 +14136,7 @@
       <c r="J178" t="s">
         <v>1500</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14180,7 +14154,7 @@
       <c r="R178" t="s">
         <v>1694</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14215,7 +14189,7 @@
       <c r="J179" t="s">
         <v>1500</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14224,7 +14198,7 @@
       <c r="M179" t="s">
         <v>1568</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14265,7 +14239,7 @@
       <c r="J180" t="s">
         <v>1500</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14306,7 +14280,7 @@
       <c r="J181" t="s">
         <v>1500</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14324,7 +14298,7 @@
       <c r="R181" t="s">
         <v>1678</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14359,7 +14333,7 @@
       <c r="J182" t="s">
         <v>1500</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14400,7 +14374,7 @@
       <c r="J183" t="s">
         <v>1500</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14441,7 +14415,7 @@
       <c r="J184" t="s">
         <v>1500</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14482,7 +14456,7 @@
       <c r="J185" t="s">
         <v>1500</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14523,7 +14497,7 @@
       <c r="J186" t="s">
         <v>1500</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14564,7 +14538,7 @@
       <c r="J187" t="s">
         <v>1500</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14605,7 +14579,7 @@
       <c r="J188" t="s">
         <v>1500</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14646,7 +14620,7 @@
       <c r="J189" t="s">
         <v>1500</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14687,7 +14661,7 @@
       <c r="J190" t="s">
         <v>1500</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14728,7 +14702,7 @@
       <c r="J191" t="s">
         <v>1500</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14769,7 +14743,7 @@
       <c r="J192" t="s">
         <v>1500</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14810,7 +14784,7 @@
       <c r="J193" t="s">
         <v>1500</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14851,7 +14825,7 @@
       <c r="J194" t="s">
         <v>1500</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14892,7 +14866,7 @@
       <c r="J195" t="s">
         <v>1500</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14910,7 +14884,7 @@
       <c r="R195" t="s">
         <v>1687</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14948,7 +14922,7 @@
       <c r="J196" t="s">
         <v>1500</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14966,7 +14940,7 @@
       <c r="R196" t="s">
         <v>1693</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15004,7 +14978,7 @@
       <c r="J197" t="s">
         <v>1500</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15045,7 +15019,7 @@
       <c r="J198" t="s">
         <v>1502</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15086,7 +15060,7 @@
       <c r="J199" t="s">
         <v>1501</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15127,7 +15101,7 @@
       <c r="J200" t="s">
         <v>1500</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15168,7 +15142,7 @@
       <c r="J201" t="s">
         <v>1500</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15209,7 +15183,7 @@
       <c r="J202" t="s">
         <v>1500</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15227,7 +15201,7 @@
       <c r="R202" t="s">
         <v>1678</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15262,7 +15236,7 @@
       <c r="J203" t="s">
         <v>1500</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15280,7 +15254,7 @@
       <c r="R203" t="s">
         <v>1686</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15315,7 +15289,7 @@
       <c r="J204" t="s">
         <v>1500</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15330,7 +15304,7 @@
       <c r="R204" t="s">
         <v>1697</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15368,7 +15342,7 @@
       <c r="J205" t="s">
         <v>1500</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15386,7 +15360,7 @@
       <c r="R205" t="s">
         <v>1698</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15424,7 +15398,7 @@
       <c r="J206" t="s">
         <v>1500</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15442,7 +15416,7 @@
       <c r="R206" t="s">
         <v>1666</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15477,7 +15451,7 @@
       <c r="J207" t="s">
         <v>1500</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15518,7 +15492,7 @@
       <c r="J208" t="s">
         <v>1500</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15559,7 +15533,7 @@
       <c r="J209" t="s">
         <v>1500</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15600,7 +15574,7 @@
       <c r="J210" t="s">
         <v>1500</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15641,7 +15615,7 @@
       <c r="J211" t="s">
         <v>1500</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15682,7 +15656,7 @@
       <c r="J212" t="s">
         <v>1500</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15723,7 +15697,7 @@
       <c r="J213" t="s">
         <v>1500</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15764,7 +15738,7 @@
       <c r="J214" t="s">
         <v>1500</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15782,7 +15756,7 @@
       <c r="R214" t="s">
         <v>1699</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15817,7 +15791,7 @@
       <c r="J215" t="s">
         <v>1500</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15858,7 +15832,7 @@
       <c r="J216" t="s">
         <v>1500</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15899,7 +15873,7 @@
       <c r="J217" t="s">
         <v>1500</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15940,7 +15914,7 @@
       <c r="J218" t="s">
         <v>1500</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15981,7 +15955,7 @@
       <c r="J219" t="s">
         <v>1500</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16022,7 +15996,7 @@
       <c r="J220" t="s">
         <v>1500</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16063,7 +16037,7 @@
       <c r="J221" t="s">
         <v>1500</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16104,7 +16078,7 @@
       <c r="J222" t="s">
         <v>1500</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16145,7 +16119,7 @@
       <c r="J223" t="s">
         <v>1500</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16186,7 +16160,7 @@
       <c r="J224" t="s">
         <v>1500</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16227,7 +16201,7 @@
       <c r="J225" t="s">
         <v>1500</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16268,7 +16242,7 @@
       <c r="J226" t="s">
         <v>1500</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16309,7 +16283,7 @@
       <c r="J227" t="s">
         <v>1500</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16350,7 +16324,7 @@
       <c r="J228" t="s">
         <v>1500</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16391,7 +16365,7 @@
       <c r="J229" t="s">
         <v>1500</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16432,7 +16406,7 @@
       <c r="J230" t="s">
         <v>1500</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16473,7 +16447,7 @@
       <c r="J231" t="s">
         <v>1500</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16514,7 +16488,7 @@
       <c r="J232" t="s">
         <v>1500</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16555,7 +16529,7 @@
       <c r="J233" t="s">
         <v>1500</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16596,7 +16570,7 @@
       <c r="J234" t="s">
         <v>1500</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16637,7 +16611,7 @@
       <c r="J235" t="s">
         <v>1500</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16678,7 +16652,7 @@
       <c r="J236" t="s">
         <v>1500</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16719,7 +16693,7 @@
       <c r="J237" t="s">
         <v>1500</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16760,7 +16734,7 @@
       <c r="J238" t="s">
         <v>1500</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16801,7 +16775,7 @@
       <c r="J239" t="s">
         <v>1500</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16819,7 +16793,7 @@
       <c r="R239" t="s">
         <v>1693</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16854,7 +16828,7 @@
       <c r="J240" t="s">
         <v>1500</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16895,7 +16869,7 @@
       <c r="J241" t="s">
         <v>1500</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16936,7 +16910,7 @@
       <c r="J242" t="s">
         <v>1500</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16954,7 +16928,7 @@
       <c r="R242" t="s">
         <v>1686</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16989,7 +16963,7 @@
       <c r="J243" t="s">
         <v>1500</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17030,7 +17004,7 @@
       <c r="J244" t="s">
         <v>1500</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17071,7 +17045,7 @@
       <c r="J245" t="s">
         <v>1500</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17112,7 +17086,7 @@
       <c r="J246" t="s">
         <v>1500</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17130,7 +17104,7 @@
       <c r="R246" t="s">
         <v>1666</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17165,7 +17139,7 @@
       <c r="J247" t="s">
         <v>1500</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17206,7 +17180,7 @@
       <c r="J248" t="s">
         <v>1500</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17247,7 +17221,7 @@
       <c r="J249" t="s">
         <v>1500</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17288,7 +17262,7 @@
       <c r="J250" t="s">
         <v>1500</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17329,7 +17303,7 @@
       <c r="J251" t="s">
         <v>1500</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17370,7 +17344,7 @@
       <c r="J252" t="s">
         <v>1500</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17411,7 +17385,7 @@
       <c r="J253" t="s">
         <v>1500</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17429,7 +17403,7 @@
       <c r="R253" t="s">
         <v>1696</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17467,7 +17441,7 @@
       <c r="J254" t="s">
         <v>1500</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17508,7 +17482,7 @@
       <c r="J255" t="s">
         <v>1500</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17549,7 +17523,7 @@
       <c r="J256" t="s">
         <v>1500</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17558,7 +17532,7 @@
       <c r="M256" t="s">
         <v>1567</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17596,7 +17570,7 @@
       <c r="J257" t="s">
         <v>1500</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17605,7 +17579,7 @@
       <c r="M257" t="s">
         <v>1568</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17649,7 +17623,7 @@
       <c r="J258" t="s">
         <v>1500</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17667,7 +17641,7 @@
       <c r="R258" t="s">
         <v>1678</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17705,7 +17679,7 @@
       <c r="J259" t="s">
         <v>1500</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17723,7 +17697,7 @@
       <c r="R259" t="s">
         <v>1694</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17761,7 +17735,7 @@
       <c r="J260" t="s">
         <v>1500</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17770,7 +17744,7 @@
       <c r="M260" t="s">
         <v>1562</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17814,7 +17788,7 @@
       <c r="J261" t="s">
         <v>1500</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17832,7 +17806,7 @@
       <c r="R261" t="s">
         <v>1700</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17870,7 +17844,7 @@
       <c r="J262" t="s">
         <v>1500</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17888,7 +17862,7 @@
       <c r="R262" t="s">
         <v>1694</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17926,7 +17900,7 @@
       <c r="J263" t="s">
         <v>1500</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17935,7 +17909,7 @@
       <c r="M263" t="s">
         <v>1562</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17979,7 +17953,7 @@
       <c r="J264" t="s">
         <v>1500</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18020,7 +17994,7 @@
       <c r="J265" t="s">
         <v>1500</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18061,7 +18035,7 @@
       <c r="J266" t="s">
         <v>1500</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18102,7 +18076,7 @@
       <c r="J267" t="s">
         <v>1500</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18146,7 +18120,7 @@
       <c r="J268" t="s">
         <v>1500</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18187,7 +18161,7 @@
       <c r="J269" t="s">
         <v>1500</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18228,7 +18202,7 @@
       <c r="J270" t="s">
         <v>1500</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18269,7 +18243,7 @@
       <c r="J271" t="s">
         <v>1500</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18310,7 +18284,7 @@
       <c r="J272" t="s">
         <v>1500</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18328,7 +18302,7 @@
       <c r="R272" t="s">
         <v>1701</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18366,7 +18340,7 @@
       <c r="J273" t="s">
         <v>1500</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18410,7 +18384,7 @@
       <c r="J274" t="s">
         <v>1500</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18451,7 +18425,7 @@
       <c r="J275" t="s">
         <v>1500</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18492,7 +18466,7 @@
       <c r="J276" t="s">
         <v>1500</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18533,7 +18507,7 @@
       <c r="J277" t="s">
         <v>1500</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18574,7 +18548,7 @@
       <c r="J278" t="s">
         <v>1500</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18615,7 +18589,7 @@
       <c r="J279" t="s">
         <v>1500</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18656,7 +18630,7 @@
       <c r="J280" t="s">
         <v>1500</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18697,7 +18671,7 @@
       <c r="J281" t="s">
         <v>1500</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18738,7 +18712,7 @@
       <c r="J282" t="s">
         <v>1500</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18779,7 +18753,7 @@
       <c r="J283" t="s">
         <v>1500</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18820,7 +18794,7 @@
       <c r="J284" t="s">
         <v>1500</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18861,7 +18835,7 @@
       <c r="J285" t="s">
         <v>1500</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18902,7 +18876,7 @@
       <c r="J286" t="s">
         <v>1500</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18943,7 +18917,7 @@
       <c r="J287" t="s">
         <v>1500</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18984,7 +18958,7 @@
       <c r="J288" t="s">
         <v>1500</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19025,7 +18999,7 @@
       <c r="J289" t="s">
         <v>1500</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19066,7 +19040,7 @@
       <c r="J290" t="s">
         <v>1500</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19107,7 +19081,7 @@
       <c r="J291" t="s">
         <v>1500</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19148,7 +19122,7 @@
       <c r="J292" t="s">
         <v>1500</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19189,7 +19163,7 @@
       <c r="J293" t="s">
         <v>1500</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19230,7 +19204,7 @@
       <c r="J294" t="s">
         <v>1500</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19271,7 +19245,7 @@
       <c r="J295" t="s">
         <v>1500</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19289,7 +19263,7 @@
       <c r="R295" t="s">
         <v>1702</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19327,7 +19301,7 @@
       <c r="J296" t="s">
         <v>1500</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19345,7 +19319,7 @@
       <c r="R296" t="s">
         <v>1678</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19383,7 +19357,7 @@
       <c r="J297" t="s">
         <v>1500</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19424,7 +19398,7 @@
       <c r="J298" t="s">
         <v>1500</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19465,7 +19439,7 @@
       <c r="J299" t="s">
         <v>1501</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19506,7 +19480,7 @@
       <c r="J300" t="s">
         <v>1500</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19547,7 +19521,7 @@
       <c r="J301" t="s">
         <v>1500</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20385,7 +20359,7 @@
       <c r="R321" t="s">
         <v>1664</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20605,7 +20579,7 @@
       <c r="R326" t="s">
         <v>1703</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21440,7 +21414,7 @@
       <c r="R346" t="s">
         <v>1704</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (02/09/2026 09:39)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5244,8 +5244,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5261,7 +5269,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5269,12 +5277,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5574,73 +5600,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5675,7 +5701,7 @@
       <c r="J2" t="s">
         <v>1500</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5719,7 +5745,7 @@
       <c r="J3" t="s">
         <v>1500</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5763,7 +5789,7 @@
       <c r="J4" t="s">
         <v>1500</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5781,7 +5807,7 @@
       <c r="R4" t="s">
         <v>1661</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5819,7 +5845,7 @@
       <c r="J5" t="s">
         <v>1501</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5869,7 +5895,7 @@
       <c r="J6" t="s">
         <v>1500</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5916,7 +5942,7 @@
       <c r="J7" t="s">
         <v>1500</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5963,7 +5989,7 @@
       <c r="J8" t="s">
         <v>1500</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6010,7 +6036,7 @@
       <c r="J9" t="s">
         <v>1500</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6057,7 +6083,7 @@
       <c r="J10" t="s">
         <v>1500</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6104,7 +6130,7 @@
       <c r="J11" t="s">
         <v>1500</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6151,7 +6177,7 @@
       <c r="J12" t="s">
         <v>1500</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6195,7 +6221,7 @@
       <c r="J13" t="s">
         <v>1500</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6213,7 +6239,7 @@
       <c r="R13" t="s">
         <v>1662</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6251,7 +6277,7 @@
       <c r="J14" t="s">
         <v>1500</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6269,7 +6295,7 @@
       <c r="R14" t="s">
         <v>1663</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6307,7 +6333,7 @@
       <c r="J15" t="s">
         <v>1500</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6325,7 +6351,7 @@
       <c r="R15" t="s">
         <v>1663</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6363,7 +6389,7 @@
       <c r="J16" t="s">
         <v>1500</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6407,7 +6433,7 @@
       <c r="J17" t="s">
         <v>1500</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6451,7 +6477,7 @@
       <c r="J18" t="s">
         <v>1500</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6469,7 +6495,7 @@
       <c r="R18" t="s">
         <v>1664</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6510,7 +6536,7 @@
       <c r="J19" t="s">
         <v>1500</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6554,7 +6580,7 @@
       <c r="J20" t="s">
         <v>1500</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6598,7 +6624,7 @@
       <c r="J21" t="s">
         <v>1500</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6616,7 +6642,7 @@
       <c r="R21" t="s">
         <v>1663</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6657,7 +6683,7 @@
       <c r="J22" t="s">
         <v>1500</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6675,7 +6701,7 @@
       <c r="R22" t="s">
         <v>1665</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6716,7 +6742,7 @@
       <c r="J23" t="s">
         <v>1500</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6734,7 +6760,7 @@
       <c r="R23" t="s">
         <v>1666</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6775,7 +6801,7 @@
       <c r="J24" t="s">
         <v>1500</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6819,7 +6845,7 @@
       <c r="J25" t="s">
         <v>1500</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6860,7 +6886,7 @@
       <c r="J26" t="s">
         <v>1502</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6878,7 +6904,7 @@
       <c r="R26" t="s">
         <v>1667</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6913,7 +6939,7 @@
       <c r="J27" t="s">
         <v>1500</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6931,7 +6957,7 @@
       <c r="R27" t="s">
         <v>1668</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6972,7 +6998,7 @@
       <c r="J28" t="s">
         <v>1500</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7016,7 +7042,7 @@
       <c r="J29" t="s">
         <v>1500</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7060,7 +7086,7 @@
       <c r="J30" t="s">
         <v>1500</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7104,7 +7130,7 @@
       <c r="J31" t="s">
         <v>1500</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7122,7 +7148,7 @@
       <c r="R31" t="s">
         <v>1669</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7163,7 +7189,7 @@
       <c r="J32" t="s">
         <v>1500</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7207,7 +7233,7 @@
       <c r="J33" t="s">
         <v>1500</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7225,7 +7251,7 @@
       <c r="R33" t="s">
         <v>1670</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7266,7 +7292,7 @@
       <c r="J34" t="s">
         <v>1500</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7310,7 +7336,7 @@
       <c r="J35" t="s">
         <v>1500</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7328,7 +7354,7 @@
       <c r="R35" t="s">
         <v>1671</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7369,7 +7395,7 @@
       <c r="J36" t="s">
         <v>1500</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7387,7 +7413,7 @@
       <c r="R36" t="s">
         <v>1671</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7428,7 +7454,7 @@
       <c r="J37" t="s">
         <v>1500</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7446,7 +7472,7 @@
       <c r="R37" t="s">
         <v>1671</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7487,7 +7513,7 @@
       <c r="J38" t="s">
         <v>1500</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7505,7 +7531,7 @@
       <c r="R38" t="s">
         <v>1671</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7546,7 +7572,7 @@
       <c r="J39" t="s">
         <v>1500</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7564,7 +7590,7 @@
       <c r="R39" t="s">
         <v>1671</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7605,7 +7631,7 @@
       <c r="J40" t="s">
         <v>1500</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7623,7 +7649,7 @@
       <c r="R40" t="s">
         <v>1672</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7664,7 +7690,7 @@
       <c r="J41" t="s">
         <v>1500</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7682,7 +7708,7 @@
       <c r="R41" t="s">
         <v>1663</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7720,7 +7746,7 @@
       <c r="J42" t="s">
         <v>1500</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7738,7 +7764,7 @@
       <c r="R42" t="s">
         <v>1671</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7779,7 +7805,7 @@
       <c r="J43" t="s">
         <v>1500</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7823,7 +7849,7 @@
       <c r="J44" t="s">
         <v>1500</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7841,7 +7867,7 @@
       <c r="R44" t="s">
         <v>1673</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7882,7 +7908,7 @@
       <c r="J45" t="s">
         <v>1500</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7900,7 +7926,7 @@
       <c r="R45" t="s">
         <v>1674</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7938,7 +7964,7 @@
       <c r="J46" t="s">
         <v>1500</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -7982,7 +8008,7 @@
       <c r="J47" t="s">
         <v>1500</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8000,7 +8026,7 @@
       <c r="R47" t="s">
         <v>1675</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8041,7 +8067,7 @@
       <c r="J48" t="s">
         <v>1500</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8085,7 +8111,7 @@
       <c r="J49" t="s">
         <v>1500</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8129,7 +8155,7 @@
       <c r="J50" t="s">
         <v>1500</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8173,7 +8199,7 @@
       <c r="J51" t="s">
         <v>1500</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8220,7 +8246,7 @@
       <c r="J52" t="s">
         <v>1500</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8264,7 +8290,7 @@
       <c r="J53" t="s">
         <v>1500</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8308,7 +8334,7 @@
       <c r="J54" t="s">
         <v>1500</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8352,7 +8378,7 @@
       <c r="J55" t="s">
         <v>1500</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8402,7 +8428,7 @@
       <c r="J56" t="s">
         <v>1500</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8455,7 +8481,7 @@
       <c r="J57" t="s">
         <v>1500</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8505,7 +8531,7 @@
       <c r="J58" t="s">
         <v>1500</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8555,7 +8581,7 @@
       <c r="J59" t="s">
         <v>1500</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8573,7 +8599,7 @@
       <c r="R59" t="s">
         <v>1676</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8614,7 +8640,7 @@
       <c r="J60" t="s">
         <v>1500</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8658,7 +8684,7 @@
       <c r="J61" t="s">
         <v>1500</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8702,7 +8728,7 @@
       <c r="J62" t="s">
         <v>1500</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8746,7 +8772,7 @@
       <c r="J63" t="s">
         <v>1500</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8790,7 +8816,7 @@
       <c r="J64" t="s">
         <v>1500</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8834,7 +8860,7 @@
       <c r="J65" t="s">
         <v>1500</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8881,7 +8907,7 @@
       <c r="J66" t="s">
         <v>1500</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8899,7 +8925,7 @@
       <c r="R66" t="s">
         <v>1677</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8937,7 +8963,7 @@
       <c r="J67" t="s">
         <v>1500</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8981,7 +9007,7 @@
       <c r="J68" t="s">
         <v>1500</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -8996,7 +9022,7 @@
       <c r="O68" t="s">
         <v>1580</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9040,7 +9066,7 @@
       <c r="J69" t="s">
         <v>1502</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9084,7 +9110,7 @@
       <c r="J70" t="s">
         <v>1500</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9128,7 +9154,7 @@
       <c r="J71" t="s">
         <v>1500</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9172,7 +9198,7 @@
       <c r="J72" t="s">
         <v>1500</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9216,7 +9242,7 @@
       <c r="J73" t="s">
         <v>1500</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9260,7 +9286,7 @@
       <c r="J74" t="s">
         <v>1500</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9304,7 +9330,7 @@
       <c r="J75" t="s">
         <v>1500</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9348,7 +9374,7 @@
       <c r="J76" t="s">
         <v>1500</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9366,7 +9392,7 @@
       <c r="R76" t="s">
         <v>1678</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9404,7 +9430,7 @@
       <c r="J77" t="s">
         <v>1500</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9422,7 +9448,7 @@
       <c r="R77" t="s">
         <v>1678</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9460,7 +9486,7 @@
       <c r="J78" t="s">
         <v>1500</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9478,7 +9504,7 @@
       <c r="R78" t="s">
         <v>1678</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9516,7 +9542,7 @@
       <c r="J79" t="s">
         <v>1500</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9534,7 +9560,7 @@
       <c r="R79" t="s">
         <v>1678</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9572,7 +9598,7 @@
       <c r="J80" t="s">
         <v>1500</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9616,7 +9642,7 @@
       <c r="J81" t="s">
         <v>1500</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9660,7 +9686,7 @@
       <c r="J82" t="s">
         <v>1500</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9704,7 +9730,7 @@
       <c r="J83" t="s">
         <v>1500</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9748,7 +9774,7 @@
       <c r="J84" t="s">
         <v>1500</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9792,7 +9818,7 @@
       <c r="J85" t="s">
         <v>1500</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9810,7 +9836,7 @@
       <c r="R85" t="s">
         <v>1679</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9848,7 +9874,7 @@
       <c r="J86" t="s">
         <v>1500</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9892,7 +9918,7 @@
       <c r="J87" t="s">
         <v>1500</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9910,7 +9936,7 @@
       <c r="R87" t="s">
         <v>1680</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9948,7 +9974,7 @@
       <c r="J88" t="s">
         <v>1500</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -9992,7 +10018,7 @@
       <c r="J89" t="s">
         <v>1500</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10010,7 +10036,7 @@
       <c r="R89" t="s">
         <v>1681</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10045,7 +10071,7 @@
       <c r="J90" t="s">
         <v>1500</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10063,7 +10089,7 @@
       <c r="R90" t="s">
         <v>1682</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10098,7 +10124,7 @@
       <c r="J91" t="s">
         <v>1500</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10116,7 +10142,7 @@
       <c r="R91" t="s">
         <v>1666</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10154,7 +10180,7 @@
       <c r="J92" t="s">
         <v>1500</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10175,7 +10201,7 @@
       <c r="R92" t="s">
         <v>1666</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10216,7 +10242,7 @@
       <c r="J93" t="s">
         <v>1500</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10257,7 +10283,7 @@
       <c r="J94" t="s">
         <v>1500</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10301,7 +10327,7 @@
       <c r="J95" t="s">
         <v>1500</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10345,7 +10371,7 @@
       <c r="J96" t="s">
         <v>1500</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10363,7 +10389,7 @@
       <c r="R96" t="s">
         <v>1683</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10401,7 +10427,7 @@
       <c r="J97" t="s">
         <v>1500</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10416,7 +10442,7 @@
       <c r="R97" t="s">
         <v>1683</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10457,7 +10483,7 @@
       <c r="J98" t="s">
         <v>1500</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10475,7 +10501,7 @@
       <c r="R98" t="s">
         <v>1684</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10513,7 +10539,7 @@
       <c r="J99" t="s">
         <v>1500</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10531,7 +10557,7 @@
       <c r="R99" t="s">
         <v>1685</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10569,7 +10595,7 @@
       <c r="J100" t="s">
         <v>1500</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10610,7 +10636,7 @@
       <c r="J101" t="s">
         <v>1500</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10651,7 +10677,7 @@
       <c r="J102" t="s">
         <v>1500</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10692,7 +10718,7 @@
       <c r="J103" t="s">
         <v>1500</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10733,7 +10759,7 @@
       <c r="J104" t="s">
         <v>1500</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10774,7 +10800,7 @@
       <c r="J105" t="s">
         <v>1500</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10815,7 +10841,7 @@
       <c r="J106" t="s">
         <v>1500</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10856,7 +10882,7 @@
       <c r="J107" t="s">
         <v>1500</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10897,7 +10923,7 @@
       <c r="J108" t="s">
         <v>1500</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10938,7 +10964,7 @@
       <c r="J109" t="s">
         <v>1500</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -10991,7 +11017,7 @@
       <c r="J110" t="s">
         <v>1500</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11047,7 +11073,7 @@
       <c r="J111" t="s">
         <v>1500</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11065,7 +11091,7 @@
       <c r="R111" t="s">
         <v>1687</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11103,7 +11129,7 @@
       <c r="J112" t="s">
         <v>1500</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11162,7 +11188,7 @@
       <c r="J113" t="s">
         <v>1500</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11206,7 +11232,7 @@
       <c r="J114" t="s">
         <v>1500</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11250,7 +11276,7 @@
       <c r="J115" t="s">
         <v>1500</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11268,7 +11294,7 @@
       <c r="R115" t="s">
         <v>1689</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11306,7 +11332,7 @@
       <c r="J116" t="s">
         <v>1500</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11365,7 +11391,7 @@
       <c r="J117" t="s">
         <v>1500</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11409,7 +11435,7 @@
       <c r="J118" t="s">
         <v>1500</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11456,7 +11482,7 @@
       <c r="J119" t="s">
         <v>1500</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11497,7 +11523,7 @@
       <c r="J120" t="s">
         <v>1500</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11541,7 +11567,7 @@
       <c r="J121" t="s">
         <v>1500</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11588,7 +11614,7 @@
       <c r="J122" t="s">
         <v>1500</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11638,7 +11664,7 @@
       <c r="J123" t="s">
         <v>1500</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11682,7 +11708,7 @@
       <c r="J124" t="s">
         <v>1500</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11726,7 +11752,7 @@
       <c r="J125" t="s">
         <v>1500</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11744,7 +11770,7 @@
       <c r="R125" t="s">
         <v>1691</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11779,7 +11805,7 @@
       <c r="J126" t="s">
         <v>1500</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11797,7 +11823,7 @@
       <c r="R126" t="s">
         <v>1692</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11832,7 +11858,7 @@
       <c r="J127" t="s">
         <v>1500</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11888,7 +11914,7 @@
       <c r="J128" t="s">
         <v>1500</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11929,7 +11955,7 @@
       <c r="J129" t="s">
         <v>1500</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11970,7 +11996,7 @@
       <c r="J130" t="s">
         <v>1500</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12011,7 +12037,7 @@
       <c r="J131" t="s">
         <v>1500</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12055,7 +12081,7 @@
       <c r="J132" t="s">
         <v>1500</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12096,7 +12122,7 @@
       <c r="J133" t="s">
         <v>1500</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12114,7 +12140,7 @@
       <c r="R133" t="s">
         <v>1678</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12149,7 +12175,7 @@
       <c r="J134" t="s">
         <v>1500</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12167,7 +12193,7 @@
       <c r="R134" t="s">
         <v>1678</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12202,7 +12228,7 @@
       <c r="J135" t="s">
         <v>1500</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12243,7 +12269,7 @@
       <c r="J136" t="s">
         <v>1500</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12284,7 +12310,7 @@
       <c r="J137" t="s">
         <v>1500</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12325,7 +12351,7 @@
       <c r="J138" t="s">
         <v>1500</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12366,7 +12392,7 @@
       <c r="J139" t="s">
         <v>1500</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12413,7 +12439,7 @@
       <c r="J140" t="s">
         <v>1500</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12454,7 +12480,7 @@
       <c r="J141" t="s">
         <v>1500</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12495,7 +12521,7 @@
       <c r="J142" t="s">
         <v>1500</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12539,7 +12565,7 @@
       <c r="J143" t="s">
         <v>1500</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12557,7 +12583,7 @@
       <c r="R143" t="s">
         <v>1678</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12592,7 +12618,7 @@
       <c r="J144" t="s">
         <v>1500</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12610,7 +12636,7 @@
       <c r="R144" t="s">
         <v>1678</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12645,7 +12671,7 @@
       <c r="J145" t="s">
         <v>1500</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12663,7 +12689,7 @@
       <c r="R145" t="s">
         <v>1678</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12698,7 +12724,7 @@
       <c r="J146" t="s">
         <v>1500</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12716,7 +12742,7 @@
       <c r="R146" t="s">
         <v>1686</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12751,7 +12777,7 @@
       <c r="J147" t="s">
         <v>1500</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12769,7 +12795,7 @@
       <c r="R147" t="s">
         <v>1693</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12804,7 +12830,7 @@
       <c r="J148" t="s">
         <v>1500</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12845,7 +12871,7 @@
       <c r="J149" t="s">
         <v>1500</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12863,7 +12889,7 @@
       <c r="R149" t="s">
         <v>1678</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12898,7 +12924,7 @@
       <c r="J150" t="s">
         <v>1500</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12916,7 +12942,7 @@
       <c r="R150" t="s">
         <v>1678</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12951,7 +12977,7 @@
       <c r="J151" t="s">
         <v>1500</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12969,7 +12995,7 @@
       <c r="R151" t="s">
         <v>1694</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13004,7 +13030,7 @@
       <c r="J152" t="s">
         <v>1500</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13022,7 +13048,7 @@
       <c r="R152" t="s">
         <v>1695</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13057,7 +13083,7 @@
       <c r="J153" t="s">
         <v>1500</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13066,7 +13092,7 @@
       <c r="M153" t="s">
         <v>1571</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13107,7 +13133,7 @@
       <c r="J154" t="s">
         <v>1500</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13148,7 +13174,7 @@
       <c r="J155" t="s">
         <v>1500</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13189,7 +13215,7 @@
       <c r="J156" t="s">
         <v>1500</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13230,7 +13256,7 @@
       <c r="J157" t="s">
         <v>1500</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13271,7 +13297,7 @@
       <c r="J158" t="s">
         <v>1500</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13312,7 +13338,7 @@
       <c r="J159" t="s">
         <v>1500</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13353,7 +13379,7 @@
       <c r="J160" t="s">
         <v>1500</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13394,7 +13420,7 @@
       <c r="J161" t="s">
         <v>1500</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13435,7 +13461,7 @@
       <c r="J162" t="s">
         <v>1500</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13453,7 +13479,7 @@
       <c r="R162" t="s">
         <v>1681</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13488,7 +13514,7 @@
       <c r="J163" t="s">
         <v>1500</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13506,7 +13532,7 @@
       <c r="R163" t="s">
         <v>1678</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13541,7 +13567,7 @@
       <c r="J164" t="s">
         <v>1500</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13585,7 +13611,7 @@
       <c r="J165" t="s">
         <v>1500</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13626,7 +13652,7 @@
       <c r="J166" t="s">
         <v>1500</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13644,7 +13670,7 @@
       <c r="R166" t="s">
         <v>1696</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13679,7 +13705,7 @@
       <c r="J167" t="s">
         <v>1500</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13723,7 +13749,7 @@
       <c r="J168" t="s">
         <v>1500</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13767,7 +13793,7 @@
       <c r="J169" t="s">
         <v>1500</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13808,7 +13834,7 @@
       <c r="J170" t="s">
         <v>1500</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13849,7 +13875,7 @@
       <c r="J171" t="s">
         <v>1500</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13890,7 +13916,7 @@
       <c r="J172" t="s">
         <v>1500</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13931,7 +13957,7 @@
       <c r="J173" t="s">
         <v>1500</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13972,7 +13998,7 @@
       <c r="J174" t="s">
         <v>1500</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14013,7 +14039,7 @@
       <c r="J175" t="s">
         <v>1500</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14054,7 +14080,7 @@
       <c r="J176" t="s">
         <v>1500</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14095,7 +14121,7 @@
       <c r="J177" t="s">
         <v>1500</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14136,7 +14162,7 @@
       <c r="J178" t="s">
         <v>1500</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14154,7 +14180,7 @@
       <c r="R178" t="s">
         <v>1694</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14189,7 +14215,7 @@
       <c r="J179" t="s">
         <v>1500</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14198,7 +14224,7 @@
       <c r="M179" t="s">
         <v>1568</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14239,7 +14265,7 @@
       <c r="J180" t="s">
         <v>1500</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14280,7 +14306,7 @@
       <c r="J181" t="s">
         <v>1500</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14298,7 +14324,7 @@
       <c r="R181" t="s">
         <v>1678</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14333,7 +14359,7 @@
       <c r="J182" t="s">
         <v>1500</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14374,7 +14400,7 @@
       <c r="J183" t="s">
         <v>1500</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14415,7 +14441,7 @@
       <c r="J184" t="s">
         <v>1500</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14456,7 +14482,7 @@
       <c r="J185" t="s">
         <v>1500</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14497,7 +14523,7 @@
       <c r="J186" t="s">
         <v>1500</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14538,7 +14564,7 @@
       <c r="J187" t="s">
         <v>1500</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14579,7 +14605,7 @@
       <c r="J188" t="s">
         <v>1500</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14620,7 +14646,7 @@
       <c r="J189" t="s">
         <v>1500</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14661,7 +14687,7 @@
       <c r="J190" t="s">
         <v>1500</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14702,7 +14728,7 @@
       <c r="J191" t="s">
         <v>1500</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14743,7 +14769,7 @@
       <c r="J192" t="s">
         <v>1500</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14784,7 +14810,7 @@
       <c r="J193" t="s">
         <v>1500</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14825,7 +14851,7 @@
       <c r="J194" t="s">
         <v>1500</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14866,7 +14892,7 @@
       <c r="J195" t="s">
         <v>1500</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14884,7 +14910,7 @@
       <c r="R195" t="s">
         <v>1687</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14922,7 +14948,7 @@
       <c r="J196" t="s">
         <v>1500</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14940,7 +14966,7 @@
       <c r="R196" t="s">
         <v>1693</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14978,7 +15004,7 @@
       <c r="J197" t="s">
         <v>1500</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15019,7 +15045,7 @@
       <c r="J198" t="s">
         <v>1502</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15060,7 +15086,7 @@
       <c r="J199" t="s">
         <v>1501</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15101,7 +15127,7 @@
       <c r="J200" t="s">
         <v>1500</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15142,7 +15168,7 @@
       <c r="J201" t="s">
         <v>1500</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15183,7 +15209,7 @@
       <c r="J202" t="s">
         <v>1500</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15201,7 +15227,7 @@
       <c r="R202" t="s">
         <v>1678</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15236,7 +15262,7 @@
       <c r="J203" t="s">
         <v>1500</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15254,7 +15280,7 @@
       <c r="R203" t="s">
         <v>1686</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15289,7 +15315,7 @@
       <c r="J204" t="s">
         <v>1500</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15304,7 +15330,7 @@
       <c r="R204" t="s">
         <v>1697</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15342,7 +15368,7 @@
       <c r="J205" t="s">
         <v>1500</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15360,7 +15386,7 @@
       <c r="R205" t="s">
         <v>1698</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15398,7 +15424,7 @@
       <c r="J206" t="s">
         <v>1500</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15416,7 +15442,7 @@
       <c r="R206" t="s">
         <v>1666</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15451,7 +15477,7 @@
       <c r="J207" t="s">
         <v>1500</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15492,7 +15518,7 @@
       <c r="J208" t="s">
         <v>1500</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15533,7 +15559,7 @@
       <c r="J209" t="s">
         <v>1500</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15574,7 +15600,7 @@
       <c r="J210" t="s">
         <v>1500</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15615,7 +15641,7 @@
       <c r="J211" t="s">
         <v>1500</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15656,7 +15682,7 @@
       <c r="J212" t="s">
         <v>1500</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15697,7 +15723,7 @@
       <c r="J213" t="s">
         <v>1500</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15738,7 +15764,7 @@
       <c r="J214" t="s">
         <v>1500</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15756,7 +15782,7 @@
       <c r="R214" t="s">
         <v>1699</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15791,7 +15817,7 @@
       <c r="J215" t="s">
         <v>1500</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15832,7 +15858,7 @@
       <c r="J216" t="s">
         <v>1500</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15873,7 +15899,7 @@
       <c r="J217" t="s">
         <v>1500</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15914,7 +15940,7 @@
       <c r="J218" t="s">
         <v>1500</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15955,7 +15981,7 @@
       <c r="J219" t="s">
         <v>1500</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -15996,7 +16022,7 @@
       <c r="J220" t="s">
         <v>1500</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16037,7 +16063,7 @@
       <c r="J221" t="s">
         <v>1500</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16078,7 +16104,7 @@
       <c r="J222" t="s">
         <v>1500</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16119,7 +16145,7 @@
       <c r="J223" t="s">
         <v>1500</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16160,7 +16186,7 @@
       <c r="J224" t="s">
         <v>1500</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16201,7 +16227,7 @@
       <c r="J225" t="s">
         <v>1500</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16242,7 +16268,7 @@
       <c r="J226" t="s">
         <v>1500</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16283,7 +16309,7 @@
       <c r="J227" t="s">
         <v>1500</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16324,7 +16350,7 @@
       <c r="J228" t="s">
         <v>1500</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16365,7 +16391,7 @@
       <c r="J229" t="s">
         <v>1500</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16406,7 +16432,7 @@
       <c r="J230" t="s">
         <v>1500</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16447,7 +16473,7 @@
       <c r="J231" t="s">
         <v>1500</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16488,7 +16514,7 @@
       <c r="J232" t="s">
         <v>1500</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16529,7 +16555,7 @@
       <c r="J233" t="s">
         <v>1500</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16570,7 +16596,7 @@
       <c r="J234" t="s">
         <v>1500</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16611,7 +16637,7 @@
       <c r="J235" t="s">
         <v>1500</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16652,7 +16678,7 @@
       <c r="J236" t="s">
         <v>1500</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16693,7 +16719,7 @@
       <c r="J237" t="s">
         <v>1500</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16734,7 +16760,7 @@
       <c r="J238" t="s">
         <v>1500</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16775,7 +16801,7 @@
       <c r="J239" t="s">
         <v>1500</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16793,7 +16819,7 @@
       <c r="R239" t="s">
         <v>1693</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16828,7 +16854,7 @@
       <c r="J240" t="s">
         <v>1500</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16869,7 +16895,7 @@
       <c r="J241" t="s">
         <v>1500</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16910,7 +16936,7 @@
       <c r="J242" t="s">
         <v>1500</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16928,7 +16954,7 @@
       <c r="R242" t="s">
         <v>1686</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16963,7 +16989,7 @@
       <c r="J243" t="s">
         <v>1500</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17004,7 +17030,7 @@
       <c r="J244" t="s">
         <v>1500</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17045,7 +17071,7 @@
       <c r="J245" t="s">
         <v>1500</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17086,7 +17112,7 @@
       <c r="J246" t="s">
         <v>1500</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17104,7 +17130,7 @@
       <c r="R246" t="s">
         <v>1666</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17139,7 +17165,7 @@
       <c r="J247" t="s">
         <v>1500</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17180,7 +17206,7 @@
       <c r="J248" t="s">
         <v>1500</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17221,7 +17247,7 @@
       <c r="J249" t="s">
         <v>1500</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17262,7 +17288,7 @@
       <c r="J250" t="s">
         <v>1500</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17303,7 +17329,7 @@
       <c r="J251" t="s">
         <v>1500</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17344,7 +17370,7 @@
       <c r="J252" t="s">
         <v>1500</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17385,7 +17411,7 @@
       <c r="J253" t="s">
         <v>1500</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17403,7 +17429,7 @@
       <c r="R253" t="s">
         <v>1696</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17441,7 +17467,7 @@
       <c r="J254" t="s">
         <v>1500</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17482,7 +17508,7 @@
       <c r="J255" t="s">
         <v>1500</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17523,7 +17549,7 @@
       <c r="J256" t="s">
         <v>1500</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17532,7 +17558,7 @@
       <c r="M256" t="s">
         <v>1567</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17570,7 +17596,7 @@
       <c r="J257" t="s">
         <v>1500</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17579,7 +17605,7 @@
       <c r="M257" t="s">
         <v>1568</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17623,7 +17649,7 @@
       <c r="J258" t="s">
         <v>1500</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17641,7 +17667,7 @@
       <c r="R258" t="s">
         <v>1678</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17679,7 +17705,7 @@
       <c r="J259" t="s">
         <v>1500</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17697,7 +17723,7 @@
       <c r="R259" t="s">
         <v>1694</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17735,7 +17761,7 @@
       <c r="J260" t="s">
         <v>1500</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17744,7 +17770,7 @@
       <c r="M260" t="s">
         <v>1562</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17788,7 +17814,7 @@
       <c r="J261" t="s">
         <v>1500</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17806,7 +17832,7 @@
       <c r="R261" t="s">
         <v>1700</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17844,7 +17870,7 @@
       <c r="J262" t="s">
         <v>1500</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17862,7 +17888,7 @@
       <c r="R262" t="s">
         <v>1694</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17900,7 +17926,7 @@
       <c r="J263" t="s">
         <v>1500</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17909,7 +17935,7 @@
       <c r="M263" t="s">
         <v>1562</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17953,7 +17979,7 @@
       <c r="J264" t="s">
         <v>1500</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -17994,7 +18020,7 @@
       <c r="J265" t="s">
         <v>1500</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18035,7 +18061,7 @@
       <c r="J266" t="s">
         <v>1500</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18076,7 +18102,7 @@
       <c r="J267" t="s">
         <v>1500</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18120,7 +18146,7 @@
       <c r="J268" t="s">
         <v>1500</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18161,7 +18187,7 @@
       <c r="J269" t="s">
         <v>1500</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18202,7 +18228,7 @@
       <c r="J270" t="s">
         <v>1500</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18243,7 +18269,7 @@
       <c r="J271" t="s">
         <v>1500</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18284,7 +18310,7 @@
       <c r="J272" t="s">
         <v>1500</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18302,7 +18328,7 @@
       <c r="R272" t="s">
         <v>1701</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18340,7 +18366,7 @@
       <c r="J273" t="s">
         <v>1500</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18384,7 +18410,7 @@
       <c r="J274" t="s">
         <v>1500</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18425,7 +18451,7 @@
       <c r="J275" t="s">
         <v>1500</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18466,7 +18492,7 @@
       <c r="J276" t="s">
         <v>1500</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18507,7 +18533,7 @@
       <c r="J277" t="s">
         <v>1500</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18548,7 +18574,7 @@
       <c r="J278" t="s">
         <v>1500</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18589,7 +18615,7 @@
       <c r="J279" t="s">
         <v>1500</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18630,7 +18656,7 @@
       <c r="J280" t="s">
         <v>1500</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18671,7 +18697,7 @@
       <c r="J281" t="s">
         <v>1500</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18712,7 +18738,7 @@
       <c r="J282" t="s">
         <v>1500</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18753,7 +18779,7 @@
       <c r="J283" t="s">
         <v>1500</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18794,7 +18820,7 @@
       <c r="J284" t="s">
         <v>1500</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18835,7 +18861,7 @@
       <c r="J285" t="s">
         <v>1500</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18876,7 +18902,7 @@
       <c r="J286" t="s">
         <v>1500</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18917,7 +18943,7 @@
       <c r="J287" t="s">
         <v>1500</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18958,7 +18984,7 @@
       <c r="J288" t="s">
         <v>1500</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -18999,7 +19025,7 @@
       <c r="J289" t="s">
         <v>1500</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19040,7 +19066,7 @@
       <c r="J290" t="s">
         <v>1500</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19081,7 +19107,7 @@
       <c r="J291" t="s">
         <v>1500</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19122,7 +19148,7 @@
       <c r="J292" t="s">
         <v>1500</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19163,7 +19189,7 @@
       <c r="J293" t="s">
         <v>1500</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19204,7 +19230,7 @@
       <c r="J294" t="s">
         <v>1500</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19245,7 +19271,7 @@
       <c r="J295" t="s">
         <v>1500</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19263,7 +19289,7 @@
       <c r="R295" t="s">
         <v>1702</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19301,7 +19327,7 @@
       <c r="J296" t="s">
         <v>1500</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19319,7 +19345,7 @@
       <c r="R296" t="s">
         <v>1678</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19357,7 +19383,7 @@
       <c r="J297" t="s">
         <v>1500</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19398,7 +19424,7 @@
       <c r="J298" t="s">
         <v>1500</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19439,7 +19465,7 @@
       <c r="J299" t="s">
         <v>1501</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19480,7 +19506,7 @@
       <c r="J300" t="s">
         <v>1500</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19521,7 +19547,7 @@
       <c r="J301" t="s">
         <v>1500</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20359,7 +20385,7 @@
       <c r="R321" t="s">
         <v>1664</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20579,7 +20605,7 @@
       <c r="R326" t="s">
         <v>1703</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21414,7 +21440,7 @@
       <c r="R346" t="s">
         <v>1704</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (02/09/2026 12:06)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5244,16 +5244,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5269,7 +5261,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5277,30 +5269,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5600,73 +5574,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5701,7 +5675,7 @@
       <c r="J2" t="s">
         <v>1500</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5745,7 +5719,7 @@
       <c r="J3" t="s">
         <v>1500</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5789,7 +5763,7 @@
       <c r="J4" t="s">
         <v>1500</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5807,7 +5781,7 @@
       <c r="R4" t="s">
         <v>1661</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5845,7 +5819,7 @@
       <c r="J5" t="s">
         <v>1501</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5895,7 +5869,7 @@
       <c r="J6" t="s">
         <v>1500</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5942,7 +5916,7 @@
       <c r="J7" t="s">
         <v>1500</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5989,7 +5963,7 @@
       <c r="J8" t="s">
         <v>1500</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6036,7 +6010,7 @@
       <c r="J9" t="s">
         <v>1500</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6083,7 +6057,7 @@
       <c r="J10" t="s">
         <v>1500</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6130,7 +6104,7 @@
       <c r="J11" t="s">
         <v>1500</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6177,7 +6151,7 @@
       <c r="J12" t="s">
         <v>1500</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6221,7 +6195,7 @@
       <c r="J13" t="s">
         <v>1500</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6239,7 +6213,7 @@
       <c r="R13" t="s">
         <v>1662</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6277,7 +6251,7 @@
       <c r="J14" t="s">
         <v>1500</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6295,7 +6269,7 @@
       <c r="R14" t="s">
         <v>1663</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6333,7 +6307,7 @@
       <c r="J15" t="s">
         <v>1500</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6351,7 +6325,7 @@
       <c r="R15" t="s">
         <v>1663</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6389,7 +6363,7 @@
       <c r="J16" t="s">
         <v>1500</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6433,7 +6407,7 @@
       <c r="J17" t="s">
         <v>1500</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6477,7 +6451,7 @@
       <c r="J18" t="s">
         <v>1500</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6495,7 +6469,7 @@
       <c r="R18" t="s">
         <v>1664</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6536,7 +6510,7 @@
       <c r="J19" t="s">
         <v>1500</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6580,7 +6554,7 @@
       <c r="J20" t="s">
         <v>1500</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6624,7 +6598,7 @@
       <c r="J21" t="s">
         <v>1500</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6642,7 +6616,7 @@
       <c r="R21" t="s">
         <v>1663</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6683,7 +6657,7 @@
       <c r="J22" t="s">
         <v>1500</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6701,7 +6675,7 @@
       <c r="R22" t="s">
         <v>1665</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6742,7 +6716,7 @@
       <c r="J23" t="s">
         <v>1500</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6760,7 +6734,7 @@
       <c r="R23" t="s">
         <v>1666</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6801,7 +6775,7 @@
       <c r="J24" t="s">
         <v>1500</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6845,7 +6819,7 @@
       <c r="J25" t="s">
         <v>1500</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6886,7 +6860,7 @@
       <c r="J26" t="s">
         <v>1502</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6904,7 +6878,7 @@
       <c r="R26" t="s">
         <v>1667</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6939,7 +6913,7 @@
       <c r="J27" t="s">
         <v>1500</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6957,7 +6931,7 @@
       <c r="R27" t="s">
         <v>1668</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6998,7 +6972,7 @@
       <c r="J28" t="s">
         <v>1500</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7042,7 +7016,7 @@
       <c r="J29" t="s">
         <v>1500</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7086,7 +7060,7 @@
       <c r="J30" t="s">
         <v>1500</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7130,7 +7104,7 @@
       <c r="J31" t="s">
         <v>1500</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7148,7 +7122,7 @@
       <c r="R31" t="s">
         <v>1669</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7189,7 +7163,7 @@
       <c r="J32" t="s">
         <v>1500</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7233,7 +7207,7 @@
       <c r="J33" t="s">
         <v>1500</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7251,7 +7225,7 @@
       <c r="R33" t="s">
         <v>1670</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7292,7 +7266,7 @@
       <c r="J34" t="s">
         <v>1500</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7336,7 +7310,7 @@
       <c r="J35" t="s">
         <v>1500</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7354,7 +7328,7 @@
       <c r="R35" t="s">
         <v>1671</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7395,7 +7369,7 @@
       <c r="J36" t="s">
         <v>1500</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7413,7 +7387,7 @@
       <c r="R36" t="s">
         <v>1671</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7454,7 +7428,7 @@
       <c r="J37" t="s">
         <v>1500</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7472,7 +7446,7 @@
       <c r="R37" t="s">
         <v>1671</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7513,7 +7487,7 @@
       <c r="J38" t="s">
         <v>1500</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7531,7 +7505,7 @@
       <c r="R38" t="s">
         <v>1671</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7572,7 +7546,7 @@
       <c r="J39" t="s">
         <v>1500</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7590,7 +7564,7 @@
       <c r="R39" t="s">
         <v>1671</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7631,7 +7605,7 @@
       <c r="J40" t="s">
         <v>1500</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7649,7 +7623,7 @@
       <c r="R40" t="s">
         <v>1672</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7690,7 +7664,7 @@
       <c r="J41" t="s">
         <v>1500</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7708,7 +7682,7 @@
       <c r="R41" t="s">
         <v>1663</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7746,7 +7720,7 @@
       <c r="J42" t="s">
         <v>1500</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7764,7 +7738,7 @@
       <c r="R42" t="s">
         <v>1671</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7805,7 +7779,7 @@
       <c r="J43" t="s">
         <v>1500</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7849,7 +7823,7 @@
       <c r="J44" t="s">
         <v>1500</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7867,7 +7841,7 @@
       <c r="R44" t="s">
         <v>1673</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7908,7 +7882,7 @@
       <c r="J45" t="s">
         <v>1500</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7926,7 +7900,7 @@
       <c r="R45" t="s">
         <v>1674</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7964,7 +7938,7 @@
       <c r="J46" t="s">
         <v>1500</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8008,7 +7982,7 @@
       <c r="J47" t="s">
         <v>1500</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8026,7 +8000,7 @@
       <c r="R47" t="s">
         <v>1675</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8067,7 +8041,7 @@
       <c r="J48" t="s">
         <v>1500</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8111,7 +8085,7 @@
       <c r="J49" t="s">
         <v>1500</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8155,7 +8129,7 @@
       <c r="J50" t="s">
         <v>1500</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8199,7 +8173,7 @@
       <c r="J51" t="s">
         <v>1500</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8246,7 +8220,7 @@
       <c r="J52" t="s">
         <v>1500</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8290,7 +8264,7 @@
       <c r="J53" t="s">
         <v>1500</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8334,7 +8308,7 @@
       <c r="J54" t="s">
         <v>1500</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8378,7 +8352,7 @@
       <c r="J55" t="s">
         <v>1500</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8428,7 +8402,7 @@
       <c r="J56" t="s">
         <v>1500</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8481,7 +8455,7 @@
       <c r="J57" t="s">
         <v>1500</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8531,7 +8505,7 @@
       <c r="J58" t="s">
         <v>1500</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8581,7 +8555,7 @@
       <c r="J59" t="s">
         <v>1500</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8599,7 +8573,7 @@
       <c r="R59" t="s">
         <v>1676</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8640,7 +8614,7 @@
       <c r="J60" t="s">
         <v>1500</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8684,7 +8658,7 @@
       <c r="J61" t="s">
         <v>1500</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8728,7 +8702,7 @@
       <c r="J62" t="s">
         <v>1500</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8772,7 +8746,7 @@
       <c r="J63" t="s">
         <v>1500</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8816,7 +8790,7 @@
       <c r="J64" t="s">
         <v>1500</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8860,7 +8834,7 @@
       <c r="J65" t="s">
         <v>1500</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8907,7 +8881,7 @@
       <c r="J66" t="s">
         <v>1500</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8925,7 +8899,7 @@
       <c r="R66" t="s">
         <v>1677</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8963,7 +8937,7 @@
       <c r="J67" t="s">
         <v>1500</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9007,7 +8981,7 @@
       <c r="J68" t="s">
         <v>1500</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9022,7 +8996,7 @@
       <c r="O68" t="s">
         <v>1580</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9066,7 +9040,7 @@
       <c r="J69" t="s">
         <v>1502</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9110,7 +9084,7 @@
       <c r="J70" t="s">
         <v>1500</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9154,7 +9128,7 @@
       <c r="J71" t="s">
         <v>1500</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9198,7 +9172,7 @@
       <c r="J72" t="s">
         <v>1500</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9242,7 +9216,7 @@
       <c r="J73" t="s">
         <v>1500</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9286,7 +9260,7 @@
       <c r="J74" t="s">
         <v>1500</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9330,7 +9304,7 @@
       <c r="J75" t="s">
         <v>1500</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9374,7 +9348,7 @@
       <c r="J76" t="s">
         <v>1500</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9392,7 +9366,7 @@
       <c r="R76" t="s">
         <v>1678</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9430,7 +9404,7 @@
       <c r="J77" t="s">
         <v>1500</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9448,7 +9422,7 @@
       <c r="R77" t="s">
         <v>1678</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9486,7 +9460,7 @@
       <c r="J78" t="s">
         <v>1500</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9504,7 +9478,7 @@
       <c r="R78" t="s">
         <v>1678</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9542,7 +9516,7 @@
       <c r="J79" t="s">
         <v>1500</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9560,7 +9534,7 @@
       <c r="R79" t="s">
         <v>1678</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9598,7 +9572,7 @@
       <c r="J80" t="s">
         <v>1500</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9642,7 +9616,7 @@
       <c r="J81" t="s">
         <v>1500</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9686,7 +9660,7 @@
       <c r="J82" t="s">
         <v>1500</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9730,7 +9704,7 @@
       <c r="J83" t="s">
         <v>1500</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9774,7 +9748,7 @@
       <c r="J84" t="s">
         <v>1500</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9818,7 +9792,7 @@
       <c r="J85" t="s">
         <v>1500</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9836,7 +9810,7 @@
       <c r="R85" t="s">
         <v>1679</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9874,7 +9848,7 @@
       <c r="J86" t="s">
         <v>1500</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9918,7 +9892,7 @@
       <c r="J87" t="s">
         <v>1500</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9936,7 +9910,7 @@
       <c r="R87" t="s">
         <v>1680</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9974,7 +9948,7 @@
       <c r="J88" t="s">
         <v>1500</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10018,7 +9992,7 @@
       <c r="J89" t="s">
         <v>1500</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10036,7 +10010,7 @@
       <c r="R89" t="s">
         <v>1681</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10071,7 +10045,7 @@
       <c r="J90" t="s">
         <v>1500</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10089,7 +10063,7 @@
       <c r="R90" t="s">
         <v>1682</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10124,7 +10098,7 @@
       <c r="J91" t="s">
         <v>1500</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10142,7 +10116,7 @@
       <c r="R91" t="s">
         <v>1666</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10180,7 +10154,7 @@
       <c r="J92" t="s">
         <v>1500</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10201,7 +10175,7 @@
       <c r="R92" t="s">
         <v>1666</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10242,7 +10216,7 @@
       <c r="J93" t="s">
         <v>1500</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10283,7 +10257,7 @@
       <c r="J94" t="s">
         <v>1500</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10327,7 +10301,7 @@
       <c r="J95" t="s">
         <v>1500</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10371,7 +10345,7 @@
       <c r="J96" t="s">
         <v>1500</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10389,7 +10363,7 @@
       <c r="R96" t="s">
         <v>1683</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10427,7 +10401,7 @@
       <c r="J97" t="s">
         <v>1500</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10442,7 +10416,7 @@
       <c r="R97" t="s">
         <v>1683</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10483,7 +10457,7 @@
       <c r="J98" t="s">
         <v>1500</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10501,7 +10475,7 @@
       <c r="R98" t="s">
         <v>1684</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10539,7 +10513,7 @@
       <c r="J99" t="s">
         <v>1500</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10557,7 +10531,7 @@
       <c r="R99" t="s">
         <v>1685</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10595,7 +10569,7 @@
       <c r="J100" t="s">
         <v>1500</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10636,7 +10610,7 @@
       <c r="J101" t="s">
         <v>1500</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10677,7 +10651,7 @@
       <c r="J102" t="s">
         <v>1500</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10718,7 +10692,7 @@
       <c r="J103" t="s">
         <v>1500</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10759,7 +10733,7 @@
       <c r="J104" t="s">
         <v>1500</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10800,7 +10774,7 @@
       <c r="J105" t="s">
         <v>1500</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10841,7 +10815,7 @@
       <c r="J106" t="s">
         <v>1500</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10882,7 +10856,7 @@
       <c r="J107" t="s">
         <v>1500</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10923,7 +10897,7 @@
       <c r="J108" t="s">
         <v>1500</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10964,7 +10938,7 @@
       <c r="J109" t="s">
         <v>1500</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11017,7 +10991,7 @@
       <c r="J110" t="s">
         <v>1500</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11073,7 +11047,7 @@
       <c r="J111" t="s">
         <v>1500</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11091,7 +11065,7 @@
       <c r="R111" t="s">
         <v>1687</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11129,7 +11103,7 @@
       <c r="J112" t="s">
         <v>1500</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11188,7 +11162,7 @@
       <c r="J113" t="s">
         <v>1500</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11232,7 +11206,7 @@
       <c r="J114" t="s">
         <v>1500</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11276,7 +11250,7 @@
       <c r="J115" t="s">
         <v>1500</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11294,7 +11268,7 @@
       <c r="R115" t="s">
         <v>1689</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11332,7 +11306,7 @@
       <c r="J116" t="s">
         <v>1500</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11391,7 +11365,7 @@
       <c r="J117" t="s">
         <v>1500</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11435,7 +11409,7 @@
       <c r="J118" t="s">
         <v>1500</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11482,7 +11456,7 @@
       <c r="J119" t="s">
         <v>1500</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11523,7 +11497,7 @@
       <c r="J120" t="s">
         <v>1500</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11567,7 +11541,7 @@
       <c r="J121" t="s">
         <v>1500</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11614,7 +11588,7 @@
       <c r="J122" t="s">
         <v>1500</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11664,7 +11638,7 @@
       <c r="J123" t="s">
         <v>1500</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11708,7 +11682,7 @@
       <c r="J124" t="s">
         <v>1500</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11752,7 +11726,7 @@
       <c r="J125" t="s">
         <v>1500</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11770,7 +11744,7 @@
       <c r="R125" t="s">
         <v>1691</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11805,7 +11779,7 @@
       <c r="J126" t="s">
         <v>1500</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11823,7 +11797,7 @@
       <c r="R126" t="s">
         <v>1692</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11858,7 +11832,7 @@
       <c r="J127" t="s">
         <v>1500</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11914,7 +11888,7 @@
       <c r="J128" t="s">
         <v>1500</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11955,7 +11929,7 @@
       <c r="J129" t="s">
         <v>1500</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11996,7 +11970,7 @@
       <c r="J130" t="s">
         <v>1500</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12037,7 +12011,7 @@
       <c r="J131" t="s">
         <v>1500</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12081,7 +12055,7 @@
       <c r="J132" t="s">
         <v>1500</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12122,7 +12096,7 @@
       <c r="J133" t="s">
         <v>1500</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12140,7 +12114,7 @@
       <c r="R133" t="s">
         <v>1678</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12175,7 +12149,7 @@
       <c r="J134" t="s">
         <v>1500</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12193,7 +12167,7 @@
       <c r="R134" t="s">
         <v>1678</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12228,7 +12202,7 @@
       <c r="J135" t="s">
         <v>1500</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12269,7 +12243,7 @@
       <c r="J136" t="s">
         <v>1500</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12310,7 +12284,7 @@
       <c r="J137" t="s">
         <v>1500</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12351,7 +12325,7 @@
       <c r="J138" t="s">
         <v>1500</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12392,7 +12366,7 @@
       <c r="J139" t="s">
         <v>1500</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12439,7 +12413,7 @@
       <c r="J140" t="s">
         <v>1500</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12480,7 +12454,7 @@
       <c r="J141" t="s">
         <v>1500</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12521,7 +12495,7 @@
       <c r="J142" t="s">
         <v>1500</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12565,7 +12539,7 @@
       <c r="J143" t="s">
         <v>1500</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12583,7 +12557,7 @@
       <c r="R143" t="s">
         <v>1678</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12618,7 +12592,7 @@
       <c r="J144" t="s">
         <v>1500</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12636,7 +12610,7 @@
       <c r="R144" t="s">
         <v>1678</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12671,7 +12645,7 @@
       <c r="J145" t="s">
         <v>1500</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12689,7 +12663,7 @@
       <c r="R145" t="s">
         <v>1678</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12724,7 +12698,7 @@
       <c r="J146" t="s">
         <v>1500</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12742,7 +12716,7 @@
       <c r="R146" t="s">
         <v>1686</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12777,7 +12751,7 @@
       <c r="J147" t="s">
         <v>1500</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12795,7 +12769,7 @@
       <c r="R147" t="s">
         <v>1693</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12830,7 +12804,7 @@
       <c r="J148" t="s">
         <v>1500</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12871,7 +12845,7 @@
       <c r="J149" t="s">
         <v>1500</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12889,7 +12863,7 @@
       <c r="R149" t="s">
         <v>1678</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12924,7 +12898,7 @@
       <c r="J150" t="s">
         <v>1500</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12942,7 +12916,7 @@
       <c r="R150" t="s">
         <v>1678</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12977,7 +12951,7 @@
       <c r="J151" t="s">
         <v>1500</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12995,7 +12969,7 @@
       <c r="R151" t="s">
         <v>1694</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13030,7 +13004,7 @@
       <c r="J152" t="s">
         <v>1500</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13048,7 +13022,7 @@
       <c r="R152" t="s">
         <v>1695</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13083,7 +13057,7 @@
       <c r="J153" t="s">
         <v>1500</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13092,7 +13066,7 @@
       <c r="M153" t="s">
         <v>1571</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13133,7 +13107,7 @@
       <c r="J154" t="s">
         <v>1500</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13174,7 +13148,7 @@
       <c r="J155" t="s">
         <v>1500</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13215,7 +13189,7 @@
       <c r="J156" t="s">
         <v>1500</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13256,7 +13230,7 @@
       <c r="J157" t="s">
         <v>1500</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13297,7 +13271,7 @@
       <c r="J158" t="s">
         <v>1500</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13338,7 +13312,7 @@
       <c r="J159" t="s">
         <v>1500</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13379,7 +13353,7 @@
       <c r="J160" t="s">
         <v>1500</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13420,7 +13394,7 @@
       <c r="J161" t="s">
         <v>1500</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13461,7 +13435,7 @@
       <c r="J162" t="s">
         <v>1500</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13479,7 +13453,7 @@
       <c r="R162" t="s">
         <v>1681</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13514,7 +13488,7 @@
       <c r="J163" t="s">
         <v>1500</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13532,7 +13506,7 @@
       <c r="R163" t="s">
         <v>1678</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13567,7 +13541,7 @@
       <c r="J164" t="s">
         <v>1500</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13611,7 +13585,7 @@
       <c r="J165" t="s">
         <v>1500</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13652,7 +13626,7 @@
       <c r="J166" t="s">
         <v>1500</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13670,7 +13644,7 @@
       <c r="R166" t="s">
         <v>1696</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13705,7 +13679,7 @@
       <c r="J167" t="s">
         <v>1500</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13749,7 +13723,7 @@
       <c r="J168" t="s">
         <v>1500</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13793,7 +13767,7 @@
       <c r="J169" t="s">
         <v>1500</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13834,7 +13808,7 @@
       <c r="J170" t="s">
         <v>1500</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13875,7 +13849,7 @@
       <c r="J171" t="s">
         <v>1500</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13916,7 +13890,7 @@
       <c r="J172" t="s">
         <v>1500</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13957,7 +13931,7 @@
       <c r="J173" t="s">
         <v>1500</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13998,7 +13972,7 @@
       <c r="J174" t="s">
         <v>1500</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14039,7 +14013,7 @@
       <c r="J175" t="s">
         <v>1500</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14080,7 +14054,7 @@
       <c r="J176" t="s">
         <v>1500</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14121,7 +14095,7 @@
       <c r="J177" t="s">
         <v>1500</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14162,7 +14136,7 @@
       <c r="J178" t="s">
         <v>1500</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14180,7 +14154,7 @@
       <c r="R178" t="s">
         <v>1694</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14215,7 +14189,7 @@
       <c r="J179" t="s">
         <v>1500</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14224,7 +14198,7 @@
       <c r="M179" t="s">
         <v>1568</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14265,7 +14239,7 @@
       <c r="J180" t="s">
         <v>1500</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14306,7 +14280,7 @@
       <c r="J181" t="s">
         <v>1500</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14324,7 +14298,7 @@
       <c r="R181" t="s">
         <v>1678</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14359,7 +14333,7 @@
       <c r="J182" t="s">
         <v>1500</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14400,7 +14374,7 @@
       <c r="J183" t="s">
         <v>1500</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14441,7 +14415,7 @@
       <c r="J184" t="s">
         <v>1500</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14482,7 +14456,7 @@
       <c r="J185" t="s">
         <v>1500</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14523,7 +14497,7 @@
       <c r="J186" t="s">
         <v>1500</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14564,7 +14538,7 @@
       <c r="J187" t="s">
         <v>1500</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14605,7 +14579,7 @@
       <c r="J188" t="s">
         <v>1500</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14646,7 +14620,7 @@
       <c r="J189" t="s">
         <v>1500</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14687,7 +14661,7 @@
       <c r="J190" t="s">
         <v>1500</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14728,7 +14702,7 @@
       <c r="J191" t="s">
         <v>1500</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14769,7 +14743,7 @@
       <c r="J192" t="s">
         <v>1500</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14810,7 +14784,7 @@
       <c r="J193" t="s">
         <v>1500</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14851,7 +14825,7 @@
       <c r="J194" t="s">
         <v>1500</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14892,7 +14866,7 @@
       <c r="J195" t="s">
         <v>1500</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14910,7 +14884,7 @@
       <c r="R195" t="s">
         <v>1687</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14948,7 +14922,7 @@
       <c r="J196" t="s">
         <v>1500</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14966,7 +14940,7 @@
       <c r="R196" t="s">
         <v>1693</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15004,7 +14978,7 @@
       <c r="J197" t="s">
         <v>1500</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15045,7 +15019,7 @@
       <c r="J198" t="s">
         <v>1502</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15086,7 +15060,7 @@
       <c r="J199" t="s">
         <v>1501</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15127,7 +15101,7 @@
       <c r="J200" t="s">
         <v>1500</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15168,7 +15142,7 @@
       <c r="J201" t="s">
         <v>1500</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15209,7 +15183,7 @@
       <c r="J202" t="s">
         <v>1500</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15227,7 +15201,7 @@
       <c r="R202" t="s">
         <v>1678</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15262,7 +15236,7 @@
       <c r="J203" t="s">
         <v>1500</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15280,7 +15254,7 @@
       <c r="R203" t="s">
         <v>1686</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15315,7 +15289,7 @@
       <c r="J204" t="s">
         <v>1500</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15330,7 +15304,7 @@
       <c r="R204" t="s">
         <v>1697</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15368,7 +15342,7 @@
       <c r="J205" t="s">
         <v>1500</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15386,7 +15360,7 @@
       <c r="R205" t="s">
         <v>1698</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15424,7 +15398,7 @@
       <c r="J206" t="s">
         <v>1500</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15442,7 +15416,7 @@
       <c r="R206" t="s">
         <v>1666</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15477,7 +15451,7 @@
       <c r="J207" t="s">
         <v>1500</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15518,7 +15492,7 @@
       <c r="J208" t="s">
         <v>1500</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15559,7 +15533,7 @@
       <c r="J209" t="s">
         <v>1500</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15600,7 +15574,7 @@
       <c r="J210" t="s">
         <v>1500</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15641,7 +15615,7 @@
       <c r="J211" t="s">
         <v>1500</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15682,7 +15656,7 @@
       <c r="J212" t="s">
         <v>1500</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15723,7 +15697,7 @@
       <c r="J213" t="s">
         <v>1500</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15764,7 +15738,7 @@
       <c r="J214" t="s">
         <v>1500</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15782,7 +15756,7 @@
       <c r="R214" t="s">
         <v>1699</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15817,7 +15791,7 @@
       <c r="J215" t="s">
         <v>1500</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15858,7 +15832,7 @@
       <c r="J216" t="s">
         <v>1500</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15899,7 +15873,7 @@
       <c r="J217" t="s">
         <v>1500</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15940,7 +15914,7 @@
       <c r="J218" t="s">
         <v>1500</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15981,7 +15955,7 @@
       <c r="J219" t="s">
         <v>1500</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16022,7 +15996,7 @@
       <c r="J220" t="s">
         <v>1500</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16063,7 +16037,7 @@
       <c r="J221" t="s">
         <v>1500</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16104,7 +16078,7 @@
       <c r="J222" t="s">
         <v>1500</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16145,7 +16119,7 @@
       <c r="J223" t="s">
         <v>1500</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16186,7 +16160,7 @@
       <c r="J224" t="s">
         <v>1500</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16227,7 +16201,7 @@
       <c r="J225" t="s">
         <v>1500</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16268,7 +16242,7 @@
       <c r="J226" t="s">
         <v>1500</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16309,7 +16283,7 @@
       <c r="J227" t="s">
         <v>1500</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16350,7 +16324,7 @@
       <c r="J228" t="s">
         <v>1500</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16391,7 +16365,7 @@
       <c r="J229" t="s">
         <v>1500</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16432,7 +16406,7 @@
       <c r="J230" t="s">
         <v>1500</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16473,7 +16447,7 @@
       <c r="J231" t="s">
         <v>1500</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16514,7 +16488,7 @@
       <c r="J232" t="s">
         <v>1500</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16555,7 +16529,7 @@
       <c r="J233" t="s">
         <v>1500</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16596,7 +16570,7 @@
       <c r="J234" t="s">
         <v>1500</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16637,7 +16611,7 @@
       <c r="J235" t="s">
         <v>1500</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16678,7 +16652,7 @@
       <c r="J236" t="s">
         <v>1500</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16719,7 +16693,7 @@
       <c r="J237" t="s">
         <v>1500</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16760,7 +16734,7 @@
       <c r="J238" t="s">
         <v>1500</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16801,7 +16775,7 @@
       <c r="J239" t="s">
         <v>1500</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16819,7 +16793,7 @@
       <c r="R239" t="s">
         <v>1693</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16854,7 +16828,7 @@
       <c r="J240" t="s">
         <v>1500</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16895,7 +16869,7 @@
       <c r="J241" t="s">
         <v>1500</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16936,7 +16910,7 @@
       <c r="J242" t="s">
         <v>1500</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16954,7 +16928,7 @@
       <c r="R242" t="s">
         <v>1686</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16989,7 +16963,7 @@
       <c r="J243" t="s">
         <v>1500</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17030,7 +17004,7 @@
       <c r="J244" t="s">
         <v>1500</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17071,7 +17045,7 @@
       <c r="J245" t="s">
         <v>1500</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17112,7 +17086,7 @@
       <c r="J246" t="s">
         <v>1500</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17130,7 +17104,7 @@
       <c r="R246" t="s">
         <v>1666</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17165,7 +17139,7 @@
       <c r="J247" t="s">
         <v>1500</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17206,7 +17180,7 @@
       <c r="J248" t="s">
         <v>1500</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17247,7 +17221,7 @@
       <c r="J249" t="s">
         <v>1500</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17288,7 +17262,7 @@
       <c r="J250" t="s">
         <v>1500</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17329,7 +17303,7 @@
       <c r="J251" t="s">
         <v>1500</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17370,7 +17344,7 @@
       <c r="J252" t="s">
         <v>1500</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17411,7 +17385,7 @@
       <c r="J253" t="s">
         <v>1500</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17429,7 +17403,7 @@
       <c r="R253" t="s">
         <v>1696</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17467,7 +17441,7 @@
       <c r="J254" t="s">
         <v>1500</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17508,7 +17482,7 @@
       <c r="J255" t="s">
         <v>1500</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17549,7 +17523,7 @@
       <c r="J256" t="s">
         <v>1500</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17558,7 +17532,7 @@
       <c r="M256" t="s">
         <v>1567</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17596,7 +17570,7 @@
       <c r="J257" t="s">
         <v>1500</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17605,7 +17579,7 @@
       <c r="M257" t="s">
         <v>1568</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17649,7 +17623,7 @@
       <c r="J258" t="s">
         <v>1500</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17667,7 +17641,7 @@
       <c r="R258" t="s">
         <v>1678</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17705,7 +17679,7 @@
       <c r="J259" t="s">
         <v>1500</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17723,7 +17697,7 @@
       <c r="R259" t="s">
         <v>1694</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17761,7 +17735,7 @@
       <c r="J260" t="s">
         <v>1500</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17770,7 +17744,7 @@
       <c r="M260" t="s">
         <v>1562</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17814,7 +17788,7 @@
       <c r="J261" t="s">
         <v>1500</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17832,7 +17806,7 @@
       <c r="R261" t="s">
         <v>1700</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17870,7 +17844,7 @@
       <c r="J262" t="s">
         <v>1500</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17888,7 +17862,7 @@
       <c r="R262" t="s">
         <v>1694</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17926,7 +17900,7 @@
       <c r="J263" t="s">
         <v>1500</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17935,7 +17909,7 @@
       <c r="M263" t="s">
         <v>1562</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17979,7 +17953,7 @@
       <c r="J264" t="s">
         <v>1500</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18020,7 +17994,7 @@
       <c r="J265" t="s">
         <v>1500</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18061,7 +18035,7 @@
       <c r="J266" t="s">
         <v>1500</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18102,7 +18076,7 @@
       <c r="J267" t="s">
         <v>1500</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18146,7 +18120,7 @@
       <c r="J268" t="s">
         <v>1500</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18187,7 +18161,7 @@
       <c r="J269" t="s">
         <v>1500</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18228,7 +18202,7 @@
       <c r="J270" t="s">
         <v>1500</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18269,7 +18243,7 @@
       <c r="J271" t="s">
         <v>1500</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18310,7 +18284,7 @@
       <c r="J272" t="s">
         <v>1500</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18328,7 +18302,7 @@
       <c r="R272" t="s">
         <v>1701</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18366,7 +18340,7 @@
       <c r="J273" t="s">
         <v>1500</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18410,7 +18384,7 @@
       <c r="J274" t="s">
         <v>1500</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18451,7 +18425,7 @@
       <c r="J275" t="s">
         <v>1500</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18492,7 +18466,7 @@
       <c r="J276" t="s">
         <v>1500</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18533,7 +18507,7 @@
       <c r="J277" t="s">
         <v>1500</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18574,7 +18548,7 @@
       <c r="J278" t="s">
         <v>1500</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18615,7 +18589,7 @@
       <c r="J279" t="s">
         <v>1500</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18656,7 +18630,7 @@
       <c r="J280" t="s">
         <v>1500</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18697,7 +18671,7 @@
       <c r="J281" t="s">
         <v>1500</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18738,7 +18712,7 @@
       <c r="J282" t="s">
         <v>1500</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18779,7 +18753,7 @@
       <c r="J283" t="s">
         <v>1500</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18820,7 +18794,7 @@
       <c r="J284" t="s">
         <v>1500</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18861,7 +18835,7 @@
       <c r="J285" t="s">
         <v>1500</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18902,7 +18876,7 @@
       <c r="J286" t="s">
         <v>1500</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18943,7 +18917,7 @@
       <c r="J287" t="s">
         <v>1500</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18984,7 +18958,7 @@
       <c r="J288" t="s">
         <v>1500</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19025,7 +18999,7 @@
       <c r="J289" t="s">
         <v>1500</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19066,7 +19040,7 @@
       <c r="J290" t="s">
         <v>1500</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19107,7 +19081,7 @@
       <c r="J291" t="s">
         <v>1500</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19148,7 +19122,7 @@
       <c r="J292" t="s">
         <v>1500</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19189,7 +19163,7 @@
       <c r="J293" t="s">
         <v>1500</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19230,7 +19204,7 @@
       <c r="J294" t="s">
         <v>1500</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19271,7 +19245,7 @@
       <c r="J295" t="s">
         <v>1500</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19289,7 +19263,7 @@
       <c r="R295" t="s">
         <v>1702</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19327,7 +19301,7 @@
       <c r="J296" t="s">
         <v>1500</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19345,7 +19319,7 @@
       <c r="R296" t="s">
         <v>1678</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19383,7 +19357,7 @@
       <c r="J297" t="s">
         <v>1500</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19424,7 +19398,7 @@
       <c r="J298" t="s">
         <v>1500</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19465,7 +19439,7 @@
       <c r="J299" t="s">
         <v>1501</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19506,7 +19480,7 @@
       <c r="J300" t="s">
         <v>1500</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19547,7 +19521,7 @@
       <c r="J301" t="s">
         <v>1500</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20385,7 +20359,7 @@
       <c r="R321" t="s">
         <v>1664</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20605,7 +20579,7 @@
       <c r="R326" t="s">
         <v>1703</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21440,7 +21414,7 @@
       <c r="R346" t="s">
         <v>1704</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (03/09/2026 13:44)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5262,8 +5262,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5279,7 +5287,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5287,12 +5295,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5592,73 +5618,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5693,7 +5719,7 @@
       <c r="J2" t="s">
         <v>1504</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5737,7 +5763,7 @@
       <c r="J3" t="s">
         <v>1504</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5781,7 +5807,7 @@
       <c r="J4" t="s">
         <v>1504</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5799,7 +5825,7 @@
       <c r="R4" t="s">
         <v>1666</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5837,7 +5863,7 @@
       <c r="J5" t="s">
         <v>1505</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5887,7 +5913,7 @@
       <c r="J6" t="s">
         <v>1504</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5934,7 +5960,7 @@
       <c r="J7" t="s">
         <v>1504</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5981,7 +6007,7 @@
       <c r="J8" t="s">
         <v>1504</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6028,7 +6054,7 @@
       <c r="J9" t="s">
         <v>1504</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6075,7 +6101,7 @@
       <c r="J10" t="s">
         <v>1504</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6122,7 +6148,7 @@
       <c r="J11" t="s">
         <v>1504</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6169,7 +6195,7 @@
       <c r="J12" t="s">
         <v>1504</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6213,7 +6239,7 @@
       <c r="J13" t="s">
         <v>1504</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6231,7 +6257,7 @@
       <c r="R13" t="s">
         <v>1667</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6269,7 +6295,7 @@
       <c r="J14" t="s">
         <v>1504</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6287,7 +6313,7 @@
       <c r="R14" t="s">
         <v>1668</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6325,7 +6351,7 @@
       <c r="J15" t="s">
         <v>1504</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6343,7 +6369,7 @@
       <c r="R15" t="s">
         <v>1668</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6381,7 +6407,7 @@
       <c r="J16" t="s">
         <v>1504</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6425,7 +6451,7 @@
       <c r="J17" t="s">
         <v>1504</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6469,7 +6495,7 @@
       <c r="J18" t="s">
         <v>1504</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6487,7 +6513,7 @@
       <c r="R18" t="s">
         <v>1669</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6528,7 +6554,7 @@
       <c r="J19" t="s">
         <v>1504</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6572,7 +6598,7 @@
       <c r="J20" t="s">
         <v>1504</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6616,7 +6642,7 @@
       <c r="J21" t="s">
         <v>1504</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6634,7 +6660,7 @@
       <c r="R21" t="s">
         <v>1668</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6675,7 +6701,7 @@
       <c r="J22" t="s">
         <v>1504</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6693,7 +6719,7 @@
       <c r="R22" t="s">
         <v>1670</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6734,7 +6760,7 @@
       <c r="J23" t="s">
         <v>1504</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6752,7 +6778,7 @@
       <c r="R23" t="s">
         <v>1671</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6793,7 +6819,7 @@
       <c r="J24" t="s">
         <v>1504</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6837,7 +6863,7 @@
       <c r="J25" t="s">
         <v>1504</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J26" t="s">
         <v>1506</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6896,7 +6922,7 @@
       <c r="R26" t="s">
         <v>1672</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6931,7 +6957,7 @@
       <c r="J27" t="s">
         <v>1504</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6949,7 +6975,7 @@
       <c r="R27" t="s">
         <v>1673</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6990,7 +7016,7 @@
       <c r="J28" t="s">
         <v>1504</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7034,7 +7060,7 @@
       <c r="J29" t="s">
         <v>1504</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7078,7 +7104,7 @@
       <c r="J30" t="s">
         <v>1504</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7122,7 +7148,7 @@
       <c r="J31" t="s">
         <v>1504</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7140,7 +7166,7 @@
       <c r="R31" t="s">
         <v>1674</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7181,7 +7207,7 @@
       <c r="J32" t="s">
         <v>1504</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7225,7 +7251,7 @@
       <c r="J33" t="s">
         <v>1504</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7243,7 +7269,7 @@
       <c r="R33" t="s">
         <v>1675</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7284,7 +7310,7 @@
       <c r="J34" t="s">
         <v>1504</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7328,7 +7354,7 @@
       <c r="J35" t="s">
         <v>1504</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7346,7 +7372,7 @@
       <c r="R35" t="s">
         <v>1676</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7387,7 +7413,7 @@
       <c r="J36" t="s">
         <v>1504</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7405,7 +7431,7 @@
       <c r="R36" t="s">
         <v>1676</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7446,7 +7472,7 @@
       <c r="J37" t="s">
         <v>1504</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7464,7 +7490,7 @@
       <c r="R37" t="s">
         <v>1676</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7505,7 +7531,7 @@
       <c r="J38" t="s">
         <v>1504</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7523,7 +7549,7 @@
       <c r="R38" t="s">
         <v>1676</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7564,7 +7590,7 @@
       <c r="J39" t="s">
         <v>1504</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7582,7 +7608,7 @@
       <c r="R39" t="s">
         <v>1676</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7623,7 +7649,7 @@
       <c r="J40" t="s">
         <v>1504</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7641,7 +7667,7 @@
       <c r="R40" t="s">
         <v>1677</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7682,7 +7708,7 @@
       <c r="J41" t="s">
         <v>1504</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7700,7 +7726,7 @@
       <c r="R41" t="s">
         <v>1668</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7738,7 +7764,7 @@
       <c r="J42" t="s">
         <v>1504</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7756,7 +7782,7 @@
       <c r="R42" t="s">
         <v>1676</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7797,7 +7823,7 @@
       <c r="J43" t="s">
         <v>1504</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7841,7 +7867,7 @@
       <c r="J44" t="s">
         <v>1504</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7859,7 +7885,7 @@
       <c r="R44" t="s">
         <v>1678</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7900,7 +7926,7 @@
       <c r="J45" t="s">
         <v>1504</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7918,7 +7944,7 @@
       <c r="R45" t="s">
         <v>1679</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7956,7 +7982,7 @@
       <c r="J46" t="s">
         <v>1504</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8000,7 +8026,7 @@
       <c r="J47" t="s">
         <v>1504</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8018,7 +8044,7 @@
       <c r="R47" t="s">
         <v>1680</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8059,7 +8085,7 @@
       <c r="J48" t="s">
         <v>1504</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8103,7 +8129,7 @@
       <c r="J49" t="s">
         <v>1504</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8147,7 +8173,7 @@
       <c r="J50" t="s">
         <v>1504</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8191,7 +8217,7 @@
       <c r="J51" t="s">
         <v>1504</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8238,7 +8264,7 @@
       <c r="J52" t="s">
         <v>1504</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8282,7 +8308,7 @@
       <c r="J53" t="s">
         <v>1504</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8326,7 +8352,7 @@
       <c r="J54" t="s">
         <v>1504</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8370,7 +8396,7 @@
       <c r="J55" t="s">
         <v>1504</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8420,7 +8446,7 @@
       <c r="J56" t="s">
         <v>1504</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8473,7 +8499,7 @@
       <c r="J57" t="s">
         <v>1504</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8523,7 +8549,7 @@
       <c r="J58" t="s">
         <v>1504</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8573,7 +8599,7 @@
       <c r="J59" t="s">
         <v>1504</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8591,7 +8617,7 @@
       <c r="R59" t="s">
         <v>1681</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8632,7 +8658,7 @@
       <c r="J60" t="s">
         <v>1504</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8676,7 +8702,7 @@
       <c r="J61" t="s">
         <v>1504</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8720,7 +8746,7 @@
       <c r="J62" t="s">
         <v>1504</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8764,7 +8790,7 @@
       <c r="J63" t="s">
         <v>1504</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8808,7 +8834,7 @@
       <c r="J64" t="s">
         <v>1504</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8852,7 +8878,7 @@
       <c r="J65" t="s">
         <v>1504</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8899,7 +8925,7 @@
       <c r="J66" t="s">
         <v>1504</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8917,7 +8943,7 @@
       <c r="R66" t="s">
         <v>1682</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8955,7 +8981,7 @@
       <c r="J67" t="s">
         <v>1504</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8999,7 +9025,7 @@
       <c r="J68" t="s">
         <v>1504</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9014,7 +9040,7 @@
       <c r="O68" t="s">
         <v>1585</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9058,7 +9084,7 @@
       <c r="J69" t="s">
         <v>1506</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9102,7 +9128,7 @@
       <c r="J70" t="s">
         <v>1504</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9146,7 +9172,7 @@
       <c r="J71" t="s">
         <v>1504</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9190,7 +9216,7 @@
       <c r="J72" t="s">
         <v>1504</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9234,7 +9260,7 @@
       <c r="J73" t="s">
         <v>1504</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9278,7 +9304,7 @@
       <c r="J74" t="s">
         <v>1504</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9322,7 +9348,7 @@
       <c r="J75" t="s">
         <v>1504</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9366,7 +9392,7 @@
       <c r="J76" t="s">
         <v>1504</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9384,7 +9410,7 @@
       <c r="R76" t="s">
         <v>1683</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9422,7 +9448,7 @@
       <c r="J77" t="s">
         <v>1504</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9440,7 +9466,7 @@
       <c r="R77" t="s">
         <v>1683</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9478,7 +9504,7 @@
       <c r="J78" t="s">
         <v>1504</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9496,7 +9522,7 @@
       <c r="R78" t="s">
         <v>1683</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9534,7 +9560,7 @@
       <c r="J79" t="s">
         <v>1504</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9552,7 +9578,7 @@
       <c r="R79" t="s">
         <v>1683</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9590,7 +9616,7 @@
       <c r="J80" t="s">
         <v>1504</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9634,7 +9660,7 @@
       <c r="J81" t="s">
         <v>1504</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9678,7 +9704,7 @@
       <c r="J82" t="s">
         <v>1504</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9722,7 +9748,7 @@
       <c r="J83" t="s">
         <v>1504</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9766,7 +9792,7 @@
       <c r="J84" t="s">
         <v>1504</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9810,7 +9836,7 @@
       <c r="J85" t="s">
         <v>1504</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9828,7 +9854,7 @@
       <c r="R85" t="s">
         <v>1684</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9866,7 +9892,7 @@
       <c r="J86" t="s">
         <v>1504</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9910,7 +9936,7 @@
       <c r="J87" t="s">
         <v>1504</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9928,7 +9954,7 @@
       <c r="R87" t="s">
         <v>1685</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9966,7 +9992,7 @@
       <c r="J88" t="s">
         <v>1504</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10010,7 +10036,7 @@
       <c r="J89" t="s">
         <v>1504</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10028,7 +10054,7 @@
       <c r="R89" t="s">
         <v>1686</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10063,7 +10089,7 @@
       <c r="J90" t="s">
         <v>1504</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10081,7 +10107,7 @@
       <c r="R90" t="s">
         <v>1687</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10116,7 +10142,7 @@
       <c r="J91" t="s">
         <v>1504</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10134,7 +10160,7 @@
       <c r="R91" t="s">
         <v>1671</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10172,7 +10198,7 @@
       <c r="J92" t="s">
         <v>1504</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10193,7 +10219,7 @@
       <c r="R92" t="s">
         <v>1671</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10234,7 +10260,7 @@
       <c r="J93" t="s">
         <v>1504</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10275,7 +10301,7 @@
       <c r="J94" t="s">
         <v>1504</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10319,7 +10345,7 @@
       <c r="J95" t="s">
         <v>1504</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10363,7 +10389,7 @@
       <c r="J96" t="s">
         <v>1504</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10381,7 +10407,7 @@
       <c r="R96" t="s">
         <v>1688</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10419,7 +10445,7 @@
       <c r="J97" t="s">
         <v>1504</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10434,7 +10460,7 @@
       <c r="R97" t="s">
         <v>1688</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10475,7 +10501,7 @@
       <c r="J98" t="s">
         <v>1504</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10493,7 +10519,7 @@
       <c r="R98" t="s">
         <v>1689</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10531,7 +10557,7 @@
       <c r="J99" t="s">
         <v>1504</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10549,7 +10575,7 @@
       <c r="R99" t="s">
         <v>1690</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10587,7 +10613,7 @@
       <c r="J100" t="s">
         <v>1504</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10628,7 +10654,7 @@
       <c r="J101" t="s">
         <v>1504</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10669,7 +10695,7 @@
       <c r="J102" t="s">
         <v>1504</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10710,7 +10736,7 @@
       <c r="J103" t="s">
         <v>1504</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10751,7 +10777,7 @@
       <c r="J104" t="s">
         <v>1504</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10792,7 +10818,7 @@
       <c r="J105" t="s">
         <v>1504</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10833,7 +10859,7 @@
       <c r="J106" t="s">
         <v>1504</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10874,7 +10900,7 @@
       <c r="J107" t="s">
         <v>1504</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10915,7 +10941,7 @@
       <c r="J108" t="s">
         <v>1504</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10956,7 +10982,7 @@
       <c r="J109" t="s">
         <v>1504</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11009,7 +11035,7 @@
       <c r="J110" t="s">
         <v>1504</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11065,7 +11091,7 @@
       <c r="J111" t="s">
         <v>1504</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11083,7 +11109,7 @@
       <c r="R111" t="s">
         <v>1692</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11121,7 +11147,7 @@
       <c r="J112" t="s">
         <v>1504</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11180,7 +11206,7 @@
       <c r="J113" t="s">
         <v>1504</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11224,7 +11250,7 @@
       <c r="J114" t="s">
         <v>1504</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11268,7 +11294,7 @@
       <c r="J115" t="s">
         <v>1504</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11286,7 +11312,7 @@
       <c r="R115" t="s">
         <v>1694</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11324,7 +11350,7 @@
       <c r="J116" t="s">
         <v>1504</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11383,7 +11409,7 @@
       <c r="J117" t="s">
         <v>1504</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11427,7 +11453,7 @@
       <c r="J118" t="s">
         <v>1504</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11474,7 +11500,7 @@
       <c r="J119" t="s">
         <v>1504</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J120" t="s">
         <v>1504</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11559,7 +11585,7 @@
       <c r="J121" t="s">
         <v>1504</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11606,7 +11632,7 @@
       <c r="J122" t="s">
         <v>1504</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11656,7 +11682,7 @@
       <c r="J123" t="s">
         <v>1504</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11700,7 +11726,7 @@
       <c r="J124" t="s">
         <v>1504</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11744,7 +11770,7 @@
       <c r="J125" t="s">
         <v>1504</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11762,7 +11788,7 @@
       <c r="R125" t="s">
         <v>1696</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11797,7 +11823,7 @@
       <c r="J126" t="s">
         <v>1504</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11815,7 +11841,7 @@
       <c r="R126" t="s">
         <v>1697</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11850,7 +11876,7 @@
       <c r="J127" t="s">
         <v>1504</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11906,7 +11932,7 @@
       <c r="J128" t="s">
         <v>1504</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11947,7 +11973,7 @@
       <c r="J129" t="s">
         <v>1504</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11988,7 +12014,7 @@
       <c r="J130" t="s">
         <v>1504</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12029,7 +12055,7 @@
       <c r="J131" t="s">
         <v>1504</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12073,7 +12099,7 @@
       <c r="J132" t="s">
         <v>1504</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12114,7 +12140,7 @@
       <c r="J133" t="s">
         <v>1504</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12132,7 +12158,7 @@
       <c r="R133" t="s">
         <v>1683</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12167,7 +12193,7 @@
       <c r="J134" t="s">
         <v>1504</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12185,7 +12211,7 @@
       <c r="R134" t="s">
         <v>1683</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12220,7 +12246,7 @@
       <c r="J135" t="s">
         <v>1504</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12261,7 +12287,7 @@
       <c r="J136" t="s">
         <v>1504</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12302,7 +12328,7 @@
       <c r="J137" t="s">
         <v>1504</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12343,7 +12369,7 @@
       <c r="J138" t="s">
         <v>1504</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12384,7 +12410,7 @@
       <c r="J139" t="s">
         <v>1504</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12431,7 +12457,7 @@
       <c r="J140" t="s">
         <v>1504</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12472,7 +12498,7 @@
       <c r="J141" t="s">
         <v>1504</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12513,7 +12539,7 @@
       <c r="J142" t="s">
         <v>1504</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12557,7 +12583,7 @@
       <c r="J143" t="s">
         <v>1504</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12575,7 +12601,7 @@
       <c r="R143" t="s">
         <v>1683</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12610,7 +12636,7 @@
       <c r="J144" t="s">
         <v>1504</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12628,7 +12654,7 @@
       <c r="R144" t="s">
         <v>1683</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12663,7 +12689,7 @@
       <c r="J145" t="s">
         <v>1504</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12681,7 +12707,7 @@
       <c r="R145" t="s">
         <v>1683</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12716,7 +12742,7 @@
       <c r="J146" t="s">
         <v>1504</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12734,7 +12760,7 @@
       <c r="R146" t="s">
         <v>1691</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12769,7 +12795,7 @@
       <c r="J147" t="s">
         <v>1504</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12787,7 +12813,7 @@
       <c r="R147" t="s">
         <v>1698</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12822,7 +12848,7 @@
       <c r="J148" t="s">
         <v>1504</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12863,7 +12889,7 @@
       <c r="J149" t="s">
         <v>1504</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12881,7 +12907,7 @@
       <c r="R149" t="s">
         <v>1683</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12916,7 +12942,7 @@
       <c r="J150" t="s">
         <v>1504</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12934,7 +12960,7 @@
       <c r="R150" t="s">
         <v>1683</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12969,7 +12995,7 @@
       <c r="J151" t="s">
         <v>1504</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12987,7 +13013,7 @@
       <c r="R151" t="s">
         <v>1699</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13022,7 +13048,7 @@
       <c r="J152" t="s">
         <v>1504</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13040,7 +13066,7 @@
       <c r="R152" t="s">
         <v>1700</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13075,7 +13101,7 @@
       <c r="J153" t="s">
         <v>1504</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13084,7 +13110,7 @@
       <c r="M153" t="s">
         <v>1576</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13125,7 +13151,7 @@
       <c r="J154" t="s">
         <v>1504</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13166,7 +13192,7 @@
       <c r="J155" t="s">
         <v>1504</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13207,7 +13233,7 @@
       <c r="J156" t="s">
         <v>1504</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13248,7 +13274,7 @@
       <c r="J157" t="s">
         <v>1504</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13289,7 +13315,7 @@
       <c r="J158" t="s">
         <v>1504</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13330,7 +13356,7 @@
       <c r="J159" t="s">
         <v>1504</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13371,7 +13397,7 @@
       <c r="J160" t="s">
         <v>1504</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13412,7 +13438,7 @@
       <c r="J161" t="s">
         <v>1504</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13453,7 +13479,7 @@
       <c r="J162" t="s">
         <v>1504</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13471,7 +13497,7 @@
       <c r="R162" t="s">
         <v>1686</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13506,7 +13532,7 @@
       <c r="J163" t="s">
         <v>1504</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13524,7 +13550,7 @@
       <c r="R163" t="s">
         <v>1683</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13559,7 +13585,7 @@
       <c r="J164" t="s">
         <v>1504</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13603,7 +13629,7 @@
       <c r="J165" t="s">
         <v>1504</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13644,7 +13670,7 @@
       <c r="J166" t="s">
         <v>1504</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13662,7 +13688,7 @@
       <c r="R166" t="s">
         <v>1701</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13697,7 +13723,7 @@
       <c r="J167" t="s">
         <v>1504</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13741,7 +13767,7 @@
       <c r="J168" t="s">
         <v>1504</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13785,7 +13811,7 @@
       <c r="J169" t="s">
         <v>1504</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13826,7 +13852,7 @@
       <c r="J170" t="s">
         <v>1504</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13867,7 +13893,7 @@
       <c r="J171" t="s">
         <v>1504</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13908,7 +13934,7 @@
       <c r="J172" t="s">
         <v>1504</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13949,7 +13975,7 @@
       <c r="J173" t="s">
         <v>1504</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13990,7 +14016,7 @@
       <c r="J174" t="s">
         <v>1504</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14031,7 +14057,7 @@
       <c r="J175" t="s">
         <v>1504</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14072,7 +14098,7 @@
       <c r="J176" t="s">
         <v>1504</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14113,7 +14139,7 @@
       <c r="J177" t="s">
         <v>1504</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14154,7 +14180,7 @@
       <c r="J178" t="s">
         <v>1504</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14172,7 +14198,7 @@
       <c r="R178" t="s">
         <v>1699</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14207,7 +14233,7 @@
       <c r="J179" t="s">
         <v>1504</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14216,7 +14242,7 @@
       <c r="M179" t="s">
         <v>1573</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14257,7 +14283,7 @@
       <c r="J180" t="s">
         <v>1504</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14298,7 +14324,7 @@
       <c r="J181" t="s">
         <v>1504</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14316,7 +14342,7 @@
       <c r="R181" t="s">
         <v>1683</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14351,7 +14377,7 @@
       <c r="J182" t="s">
         <v>1504</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14392,7 +14418,7 @@
       <c r="J183" t="s">
         <v>1504</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14433,7 +14459,7 @@
       <c r="J184" t="s">
         <v>1504</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14474,7 +14500,7 @@
       <c r="J185" t="s">
         <v>1504</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14515,7 +14541,7 @@
       <c r="J186" t="s">
         <v>1504</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14556,7 +14582,7 @@
       <c r="J187" t="s">
         <v>1504</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14597,7 +14623,7 @@
       <c r="J188" t="s">
         <v>1504</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14638,7 +14664,7 @@
       <c r="J189" t="s">
         <v>1504</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14679,7 +14705,7 @@
       <c r="J190" t="s">
         <v>1504</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14720,7 +14746,7 @@
       <c r="J191" t="s">
         <v>1504</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14761,7 +14787,7 @@
       <c r="J192" t="s">
         <v>1504</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14802,7 +14828,7 @@
       <c r="J193" t="s">
         <v>1504</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14843,7 +14869,7 @@
       <c r="J194" t="s">
         <v>1504</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14884,7 +14910,7 @@
       <c r="J195" t="s">
         <v>1504</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14902,7 +14928,7 @@
       <c r="R195" t="s">
         <v>1692</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14940,7 +14966,7 @@
       <c r="J196" t="s">
         <v>1504</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14958,7 +14984,7 @@
       <c r="R196" t="s">
         <v>1698</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14996,7 +15022,7 @@
       <c r="J197" t="s">
         <v>1504</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15037,7 +15063,7 @@
       <c r="J198" t="s">
         <v>1506</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15078,7 +15104,7 @@
       <c r="J199" t="s">
         <v>1505</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15119,7 +15145,7 @@
       <c r="J200" t="s">
         <v>1504</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15160,7 +15186,7 @@
       <c r="J201" t="s">
         <v>1504</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15201,7 +15227,7 @@
       <c r="J202" t="s">
         <v>1504</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15219,7 +15245,7 @@
       <c r="R202" t="s">
         <v>1683</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15254,7 +15280,7 @@
       <c r="J203" t="s">
         <v>1504</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15272,7 +15298,7 @@
       <c r="R203" t="s">
         <v>1691</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15307,7 +15333,7 @@
       <c r="J204" t="s">
         <v>1504</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15322,7 +15348,7 @@
       <c r="R204" t="s">
         <v>1702</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15360,7 +15386,7 @@
       <c r="J205" t="s">
         <v>1504</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15378,7 +15404,7 @@
       <c r="R205" t="s">
         <v>1703</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15416,7 +15442,7 @@
       <c r="J206" t="s">
         <v>1504</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15434,7 +15460,7 @@
       <c r="R206" t="s">
         <v>1671</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15469,7 +15495,7 @@
       <c r="J207" t="s">
         <v>1504</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15510,7 +15536,7 @@
       <c r="J208" t="s">
         <v>1504</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15551,7 +15577,7 @@
       <c r="J209" t="s">
         <v>1504</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15592,7 +15618,7 @@
       <c r="J210" t="s">
         <v>1504</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15633,7 +15659,7 @@
       <c r="J211" t="s">
         <v>1504</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15674,7 +15700,7 @@
       <c r="J212" t="s">
         <v>1504</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15715,7 +15741,7 @@
       <c r="J213" t="s">
         <v>1504</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15756,7 +15782,7 @@
       <c r="J214" t="s">
         <v>1504</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15774,7 +15800,7 @@
       <c r="R214" t="s">
         <v>1704</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15809,7 +15835,7 @@
       <c r="J215" t="s">
         <v>1504</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15850,7 +15876,7 @@
       <c r="J216" t="s">
         <v>1504</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15891,7 +15917,7 @@
       <c r="J217" t="s">
         <v>1504</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15932,7 +15958,7 @@
       <c r="J218" t="s">
         <v>1504</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15973,7 +15999,7 @@
       <c r="J219" t="s">
         <v>1504</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16014,7 +16040,7 @@
       <c r="J220" t="s">
         <v>1504</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16055,7 +16081,7 @@
       <c r="J221" t="s">
         <v>1504</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16096,7 +16122,7 @@
       <c r="J222" t="s">
         <v>1504</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16137,7 +16163,7 @@
       <c r="J223" t="s">
         <v>1504</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16178,7 +16204,7 @@
       <c r="J224" t="s">
         <v>1504</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16219,7 +16245,7 @@
       <c r="J225" t="s">
         <v>1504</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16260,7 +16286,7 @@
       <c r="J226" t="s">
         <v>1504</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16301,7 +16327,7 @@
       <c r="J227" t="s">
         <v>1504</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J228" t="s">
         <v>1504</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J229" t="s">
         <v>1504</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J230" t="s">
         <v>1504</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J231" t="s">
         <v>1504</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J232" t="s">
         <v>1504</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J233" t="s">
         <v>1504</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J234" t="s">
         <v>1504</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J235" t="s">
         <v>1504</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J236" t="s">
         <v>1504</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J237" t="s">
         <v>1504</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J238" t="s">
         <v>1504</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J239" t="s">
         <v>1504</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16811,7 +16837,7 @@
       <c r="R239" t="s">
         <v>1698</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16846,7 +16872,7 @@
       <c r="J240" t="s">
         <v>1504</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16887,7 +16913,7 @@
       <c r="J241" t="s">
         <v>1504</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16928,7 +16954,7 @@
       <c r="J242" t="s">
         <v>1504</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16946,7 +16972,7 @@
       <c r="R242" t="s">
         <v>1691</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16981,7 +17007,7 @@
       <c r="J243" t="s">
         <v>1504</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17022,7 +17048,7 @@
       <c r="J244" t="s">
         <v>1504</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17063,7 +17089,7 @@
       <c r="J245" t="s">
         <v>1504</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17104,7 +17130,7 @@
       <c r="J246" t="s">
         <v>1504</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17122,7 +17148,7 @@
       <c r="R246" t="s">
         <v>1671</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17157,7 +17183,7 @@
       <c r="J247" t="s">
         <v>1504</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17198,7 +17224,7 @@
       <c r="J248" t="s">
         <v>1504</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17239,7 +17265,7 @@
       <c r="J249" t="s">
         <v>1504</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17280,7 +17306,7 @@
       <c r="J250" t="s">
         <v>1504</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17321,7 +17347,7 @@
       <c r="J251" t="s">
         <v>1504</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17362,7 +17388,7 @@
       <c r="J252" t="s">
         <v>1504</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17403,7 +17429,7 @@
       <c r="J253" t="s">
         <v>1504</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17421,7 +17447,7 @@
       <c r="R253" t="s">
         <v>1701</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17459,7 +17485,7 @@
       <c r="J254" t="s">
         <v>1504</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17500,7 +17526,7 @@
       <c r="J255" t="s">
         <v>1504</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17541,7 +17567,7 @@
       <c r="J256" t="s">
         <v>1504</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17550,7 +17576,7 @@
       <c r="M256" t="s">
         <v>1572</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17588,7 +17614,7 @@
       <c r="J257" t="s">
         <v>1504</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17597,7 +17623,7 @@
       <c r="M257" t="s">
         <v>1573</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17641,7 +17667,7 @@
       <c r="J258" t="s">
         <v>1504</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17659,7 +17685,7 @@
       <c r="R258" t="s">
         <v>1683</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17697,7 +17723,7 @@
       <c r="J259" t="s">
         <v>1504</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17715,7 +17741,7 @@
       <c r="R259" t="s">
         <v>1699</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17753,7 +17779,7 @@
       <c r="J260" t="s">
         <v>1504</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17762,7 +17788,7 @@
       <c r="M260" t="s">
         <v>1567</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17806,7 +17832,7 @@
       <c r="J261" t="s">
         <v>1504</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17824,7 +17850,7 @@
       <c r="R261" t="s">
         <v>1705</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17862,7 +17888,7 @@
       <c r="J262" t="s">
         <v>1504</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17880,7 +17906,7 @@
       <c r="R262" t="s">
         <v>1699</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17918,7 +17944,7 @@
       <c r="J263" t="s">
         <v>1504</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17927,7 +17953,7 @@
       <c r="M263" t="s">
         <v>1567</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17971,7 +17997,7 @@
       <c r="J264" t="s">
         <v>1504</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18012,7 +18038,7 @@
       <c r="J265" t="s">
         <v>1504</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18053,7 +18079,7 @@
       <c r="J266" t="s">
         <v>1504</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18094,7 +18120,7 @@
       <c r="J267" t="s">
         <v>1504</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18138,7 +18164,7 @@
       <c r="J268" t="s">
         <v>1504</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18179,7 +18205,7 @@
       <c r="J269" t="s">
         <v>1504</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18220,7 +18246,7 @@
       <c r="J270" t="s">
         <v>1504</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18261,7 +18287,7 @@
       <c r="J271" t="s">
         <v>1504</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18302,7 +18328,7 @@
       <c r="J272" t="s">
         <v>1504</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18320,7 +18346,7 @@
       <c r="R272" t="s">
         <v>1706</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18358,7 +18384,7 @@
       <c r="J273" t="s">
         <v>1504</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18402,7 +18428,7 @@
       <c r="J274" t="s">
         <v>1504</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18443,7 +18469,7 @@
       <c r="J275" t="s">
         <v>1504</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18484,7 +18510,7 @@
       <c r="J276" t="s">
         <v>1504</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18525,7 +18551,7 @@
       <c r="J277" t="s">
         <v>1504</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18566,7 +18592,7 @@
       <c r="J278" t="s">
         <v>1504</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18607,7 +18633,7 @@
       <c r="J279" t="s">
         <v>1504</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18648,7 +18674,7 @@
       <c r="J280" t="s">
         <v>1504</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18689,7 +18715,7 @@
       <c r="J281" t="s">
         <v>1504</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18730,7 +18756,7 @@
       <c r="J282" t="s">
         <v>1504</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18771,7 +18797,7 @@
       <c r="J283" t="s">
         <v>1504</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18812,7 +18838,7 @@
       <c r="J284" t="s">
         <v>1504</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18853,7 +18879,7 @@
       <c r="J285" t="s">
         <v>1504</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18894,7 +18920,7 @@
       <c r="J286" t="s">
         <v>1504</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18935,7 +18961,7 @@
       <c r="J287" t="s">
         <v>1504</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18976,7 +19002,7 @@
       <c r="J288" t="s">
         <v>1504</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19017,7 +19043,7 @@
       <c r="J289" t="s">
         <v>1504</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19058,7 +19084,7 @@
       <c r="J290" t="s">
         <v>1504</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19099,7 +19125,7 @@
       <c r="J291" t="s">
         <v>1504</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19140,7 +19166,7 @@
       <c r="J292" t="s">
         <v>1504</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19181,7 +19207,7 @@
       <c r="J293" t="s">
         <v>1504</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19222,7 +19248,7 @@
       <c r="J294" t="s">
         <v>1504</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19263,7 +19289,7 @@
       <c r="J295" t="s">
         <v>1504</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19281,7 +19307,7 @@
       <c r="R295" t="s">
         <v>1707</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19319,7 +19345,7 @@
       <c r="J296" t="s">
         <v>1504</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19337,7 +19363,7 @@
       <c r="R296" t="s">
         <v>1683</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19375,7 +19401,7 @@
       <c r="J297" t="s">
         <v>1504</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19416,7 +19442,7 @@
       <c r="J298" t="s">
         <v>1504</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19457,7 +19483,7 @@
       <c r="J299" t="s">
         <v>1505</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19498,7 +19524,7 @@
       <c r="J300" t="s">
         <v>1504</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19539,7 +19565,7 @@
       <c r="J301" t="s">
         <v>1504</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20377,7 +20403,7 @@
       <c r="R321" t="s">
         <v>1669</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20597,7 +20623,7 @@
       <c r="R326" t="s">
         <v>1708</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21432,7 +21458,7 @@
       <c r="R346" t="s">
         <v>1709</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (04/09/2026 11:56)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5262,16 +5262,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5287,7 +5279,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5295,30 +5287,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5618,73 +5592,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5719,7 +5693,7 @@
       <c r="J2" t="s">
         <v>1504</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5763,7 +5737,7 @@
       <c r="J3" t="s">
         <v>1504</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5807,7 +5781,7 @@
       <c r="J4" t="s">
         <v>1504</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5825,7 +5799,7 @@
       <c r="R4" t="s">
         <v>1666</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5863,7 +5837,7 @@
       <c r="J5" t="s">
         <v>1505</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5913,7 +5887,7 @@
       <c r="J6" t="s">
         <v>1504</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5960,7 +5934,7 @@
       <c r="J7" t="s">
         <v>1504</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6007,7 +5981,7 @@
       <c r="J8" t="s">
         <v>1504</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6054,7 +6028,7 @@
       <c r="J9" t="s">
         <v>1504</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6101,7 +6075,7 @@
       <c r="J10" t="s">
         <v>1504</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6148,7 +6122,7 @@
       <c r="J11" t="s">
         <v>1504</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6195,7 +6169,7 @@
       <c r="J12" t="s">
         <v>1504</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6239,7 +6213,7 @@
       <c r="J13" t="s">
         <v>1504</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6257,7 +6231,7 @@
       <c r="R13" t="s">
         <v>1667</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6295,7 +6269,7 @@
       <c r="J14" t="s">
         <v>1504</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6313,7 +6287,7 @@
       <c r="R14" t="s">
         <v>1668</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6351,7 +6325,7 @@
       <c r="J15" t="s">
         <v>1504</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6369,7 +6343,7 @@
       <c r="R15" t="s">
         <v>1668</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6407,7 +6381,7 @@
       <c r="J16" t="s">
         <v>1504</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6451,7 +6425,7 @@
       <c r="J17" t="s">
         <v>1504</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6495,7 +6469,7 @@
       <c r="J18" t="s">
         <v>1504</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6513,7 +6487,7 @@
       <c r="R18" t="s">
         <v>1669</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6554,7 +6528,7 @@
       <c r="J19" t="s">
         <v>1504</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6598,7 +6572,7 @@
       <c r="J20" t="s">
         <v>1504</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6642,7 +6616,7 @@
       <c r="J21" t="s">
         <v>1504</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6660,7 +6634,7 @@
       <c r="R21" t="s">
         <v>1668</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6701,7 +6675,7 @@
       <c r="J22" t="s">
         <v>1504</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6719,7 +6693,7 @@
       <c r="R22" t="s">
         <v>1670</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6760,7 +6734,7 @@
       <c r="J23" t="s">
         <v>1504</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6778,7 +6752,7 @@
       <c r="R23" t="s">
         <v>1671</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6819,7 +6793,7 @@
       <c r="J24" t="s">
         <v>1504</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6863,7 +6837,7 @@
       <c r="J25" t="s">
         <v>1504</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6904,7 +6878,7 @@
       <c r="J26" t="s">
         <v>1506</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6922,7 +6896,7 @@
       <c r="R26" t="s">
         <v>1672</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6957,7 +6931,7 @@
       <c r="J27" t="s">
         <v>1504</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6975,7 +6949,7 @@
       <c r="R27" t="s">
         <v>1673</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7016,7 +6990,7 @@
       <c r="J28" t="s">
         <v>1504</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7060,7 +7034,7 @@
       <c r="J29" t="s">
         <v>1504</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7104,7 +7078,7 @@
       <c r="J30" t="s">
         <v>1504</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7148,7 +7122,7 @@
       <c r="J31" t="s">
         <v>1504</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7166,7 +7140,7 @@
       <c r="R31" t="s">
         <v>1674</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7207,7 +7181,7 @@
       <c r="J32" t="s">
         <v>1504</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7251,7 +7225,7 @@
       <c r="J33" t="s">
         <v>1504</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7269,7 +7243,7 @@
       <c r="R33" t="s">
         <v>1675</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7310,7 +7284,7 @@
       <c r="J34" t="s">
         <v>1504</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7354,7 +7328,7 @@
       <c r="J35" t="s">
         <v>1504</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7372,7 +7346,7 @@
       <c r="R35" t="s">
         <v>1676</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7413,7 +7387,7 @@
       <c r="J36" t="s">
         <v>1504</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7431,7 +7405,7 @@
       <c r="R36" t="s">
         <v>1676</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7472,7 +7446,7 @@
       <c r="J37" t="s">
         <v>1504</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7490,7 +7464,7 @@
       <c r="R37" t="s">
         <v>1676</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7531,7 +7505,7 @@
       <c r="J38" t="s">
         <v>1504</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7549,7 +7523,7 @@
       <c r="R38" t="s">
         <v>1676</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7590,7 +7564,7 @@
       <c r="J39" t="s">
         <v>1504</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7608,7 +7582,7 @@
       <c r="R39" t="s">
         <v>1676</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7649,7 +7623,7 @@
       <c r="J40" t="s">
         <v>1504</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7667,7 +7641,7 @@
       <c r="R40" t="s">
         <v>1677</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7708,7 +7682,7 @@
       <c r="J41" t="s">
         <v>1504</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7726,7 +7700,7 @@
       <c r="R41" t="s">
         <v>1668</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7764,7 +7738,7 @@
       <c r="J42" t="s">
         <v>1504</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7782,7 +7756,7 @@
       <c r="R42" t="s">
         <v>1676</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7823,7 +7797,7 @@
       <c r="J43" t="s">
         <v>1504</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7867,7 +7841,7 @@
       <c r="J44" t="s">
         <v>1504</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7885,7 +7859,7 @@
       <c r="R44" t="s">
         <v>1678</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7926,7 +7900,7 @@
       <c r="J45" t="s">
         <v>1504</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7944,7 +7918,7 @@
       <c r="R45" t="s">
         <v>1679</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7982,7 +7956,7 @@
       <c r="J46" t="s">
         <v>1504</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8026,7 +8000,7 @@
       <c r="J47" t="s">
         <v>1504</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8044,7 +8018,7 @@
       <c r="R47" t="s">
         <v>1680</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8085,7 +8059,7 @@
       <c r="J48" t="s">
         <v>1504</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8129,7 +8103,7 @@
       <c r="J49" t="s">
         <v>1504</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8173,7 +8147,7 @@
       <c r="J50" t="s">
         <v>1504</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8217,7 +8191,7 @@
       <c r="J51" t="s">
         <v>1504</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8264,7 +8238,7 @@
       <c r="J52" t="s">
         <v>1504</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8308,7 +8282,7 @@
       <c r="J53" t="s">
         <v>1504</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8352,7 +8326,7 @@
       <c r="J54" t="s">
         <v>1504</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8396,7 +8370,7 @@
       <c r="J55" t="s">
         <v>1504</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8446,7 +8420,7 @@
       <c r="J56" t="s">
         <v>1504</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8499,7 +8473,7 @@
       <c r="J57" t="s">
         <v>1504</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8549,7 +8523,7 @@
       <c r="J58" t="s">
         <v>1504</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8599,7 +8573,7 @@
       <c r="J59" t="s">
         <v>1504</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8617,7 +8591,7 @@
       <c r="R59" t="s">
         <v>1681</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8658,7 +8632,7 @@
       <c r="J60" t="s">
         <v>1504</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8702,7 +8676,7 @@
       <c r="J61" t="s">
         <v>1504</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8746,7 +8720,7 @@
       <c r="J62" t="s">
         <v>1504</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8790,7 +8764,7 @@
       <c r="J63" t="s">
         <v>1504</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8834,7 +8808,7 @@
       <c r="J64" t="s">
         <v>1504</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8878,7 +8852,7 @@
       <c r="J65" t="s">
         <v>1504</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8925,7 +8899,7 @@
       <c r="J66" t="s">
         <v>1504</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8943,7 +8917,7 @@
       <c r="R66" t="s">
         <v>1682</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8981,7 +8955,7 @@
       <c r="J67" t="s">
         <v>1504</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9025,7 +8999,7 @@
       <c r="J68" t="s">
         <v>1504</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9040,7 +9014,7 @@
       <c r="O68" t="s">
         <v>1585</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9084,7 +9058,7 @@
       <c r="J69" t="s">
         <v>1506</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9128,7 +9102,7 @@
       <c r="J70" t="s">
         <v>1504</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9172,7 +9146,7 @@
       <c r="J71" t="s">
         <v>1504</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9216,7 +9190,7 @@
       <c r="J72" t="s">
         <v>1504</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9260,7 +9234,7 @@
       <c r="J73" t="s">
         <v>1504</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9304,7 +9278,7 @@
       <c r="J74" t="s">
         <v>1504</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9348,7 +9322,7 @@
       <c r="J75" t="s">
         <v>1504</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9392,7 +9366,7 @@
       <c r="J76" t="s">
         <v>1504</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9410,7 +9384,7 @@
       <c r="R76" t="s">
         <v>1683</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9448,7 +9422,7 @@
       <c r="J77" t="s">
         <v>1504</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9466,7 +9440,7 @@
       <c r="R77" t="s">
         <v>1683</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9504,7 +9478,7 @@
       <c r="J78" t="s">
         <v>1504</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9522,7 +9496,7 @@
       <c r="R78" t="s">
         <v>1683</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9560,7 +9534,7 @@
       <c r="J79" t="s">
         <v>1504</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9578,7 +9552,7 @@
       <c r="R79" t="s">
         <v>1683</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9616,7 +9590,7 @@
       <c r="J80" t="s">
         <v>1504</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9660,7 +9634,7 @@
       <c r="J81" t="s">
         <v>1504</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9704,7 +9678,7 @@
       <c r="J82" t="s">
         <v>1504</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9748,7 +9722,7 @@
       <c r="J83" t="s">
         <v>1504</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9792,7 +9766,7 @@
       <c r="J84" t="s">
         <v>1504</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9836,7 +9810,7 @@
       <c r="J85" t="s">
         <v>1504</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9854,7 +9828,7 @@
       <c r="R85" t="s">
         <v>1684</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9892,7 +9866,7 @@
       <c r="J86" t="s">
         <v>1504</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9936,7 +9910,7 @@
       <c r="J87" t="s">
         <v>1504</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9954,7 +9928,7 @@
       <c r="R87" t="s">
         <v>1685</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9992,7 +9966,7 @@
       <c r="J88" t="s">
         <v>1504</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10036,7 +10010,7 @@
       <c r="J89" t="s">
         <v>1504</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10054,7 +10028,7 @@
       <c r="R89" t="s">
         <v>1686</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10089,7 +10063,7 @@
       <c r="J90" t="s">
         <v>1504</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10107,7 +10081,7 @@
       <c r="R90" t="s">
         <v>1687</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10142,7 +10116,7 @@
       <c r="J91" t="s">
         <v>1504</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10160,7 +10134,7 @@
       <c r="R91" t="s">
         <v>1671</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10198,7 +10172,7 @@
       <c r="J92" t="s">
         <v>1504</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10219,7 +10193,7 @@
       <c r="R92" t="s">
         <v>1671</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10260,7 +10234,7 @@
       <c r="J93" t="s">
         <v>1504</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10301,7 +10275,7 @@
       <c r="J94" t="s">
         <v>1504</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10345,7 +10319,7 @@
       <c r="J95" t="s">
         <v>1504</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10389,7 +10363,7 @@
       <c r="J96" t="s">
         <v>1504</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10407,7 +10381,7 @@
       <c r="R96" t="s">
         <v>1688</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10445,7 +10419,7 @@
       <c r="J97" t="s">
         <v>1504</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10460,7 +10434,7 @@
       <c r="R97" t="s">
         <v>1688</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10501,7 +10475,7 @@
       <c r="J98" t="s">
         <v>1504</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10519,7 +10493,7 @@
       <c r="R98" t="s">
         <v>1689</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10557,7 +10531,7 @@
       <c r="J99" t="s">
         <v>1504</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10575,7 +10549,7 @@
       <c r="R99" t="s">
         <v>1690</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10613,7 +10587,7 @@
       <c r="J100" t="s">
         <v>1504</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10654,7 +10628,7 @@
       <c r="J101" t="s">
         <v>1504</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10695,7 +10669,7 @@
       <c r="J102" t="s">
         <v>1504</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10736,7 +10710,7 @@
       <c r="J103" t="s">
         <v>1504</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10777,7 +10751,7 @@
       <c r="J104" t="s">
         <v>1504</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10818,7 +10792,7 @@
       <c r="J105" t="s">
         <v>1504</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10859,7 +10833,7 @@
       <c r="J106" t="s">
         <v>1504</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10900,7 +10874,7 @@
       <c r="J107" t="s">
         <v>1504</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10941,7 +10915,7 @@
       <c r="J108" t="s">
         <v>1504</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10982,7 +10956,7 @@
       <c r="J109" t="s">
         <v>1504</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11035,7 +11009,7 @@
       <c r="J110" t="s">
         <v>1504</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11091,7 +11065,7 @@
       <c r="J111" t="s">
         <v>1504</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11109,7 +11083,7 @@
       <c r="R111" t="s">
         <v>1692</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11147,7 +11121,7 @@
       <c r="J112" t="s">
         <v>1504</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11206,7 +11180,7 @@
       <c r="J113" t="s">
         <v>1504</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11250,7 +11224,7 @@
       <c r="J114" t="s">
         <v>1504</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11294,7 +11268,7 @@
       <c r="J115" t="s">
         <v>1504</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11312,7 +11286,7 @@
       <c r="R115" t="s">
         <v>1694</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11350,7 +11324,7 @@
       <c r="J116" t="s">
         <v>1504</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11409,7 +11383,7 @@
       <c r="J117" t="s">
         <v>1504</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11453,7 +11427,7 @@
       <c r="J118" t="s">
         <v>1504</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11500,7 +11474,7 @@
       <c r="J119" t="s">
         <v>1504</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11541,7 +11515,7 @@
       <c r="J120" t="s">
         <v>1504</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11585,7 +11559,7 @@
       <c r="J121" t="s">
         <v>1504</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11632,7 +11606,7 @@
       <c r="J122" t="s">
         <v>1504</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11682,7 +11656,7 @@
       <c r="J123" t="s">
         <v>1504</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11726,7 +11700,7 @@
       <c r="J124" t="s">
         <v>1504</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11770,7 +11744,7 @@
       <c r="J125" t="s">
         <v>1504</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11788,7 +11762,7 @@
       <c r="R125" t="s">
         <v>1696</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11823,7 +11797,7 @@
       <c r="J126" t="s">
         <v>1504</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11841,7 +11815,7 @@
       <c r="R126" t="s">
         <v>1697</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11876,7 +11850,7 @@
       <c r="J127" t="s">
         <v>1504</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11932,7 +11906,7 @@
       <c r="J128" t="s">
         <v>1504</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11973,7 +11947,7 @@
       <c r="J129" t="s">
         <v>1504</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12014,7 +11988,7 @@
       <c r="J130" t="s">
         <v>1504</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12055,7 +12029,7 @@
       <c r="J131" t="s">
         <v>1504</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12099,7 +12073,7 @@
       <c r="J132" t="s">
         <v>1504</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12140,7 +12114,7 @@
       <c r="J133" t="s">
         <v>1504</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12158,7 +12132,7 @@
       <c r="R133" t="s">
         <v>1683</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12193,7 +12167,7 @@
       <c r="J134" t="s">
         <v>1504</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12211,7 +12185,7 @@
       <c r="R134" t="s">
         <v>1683</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12246,7 +12220,7 @@
       <c r="J135" t="s">
         <v>1504</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12287,7 +12261,7 @@
       <c r="J136" t="s">
         <v>1504</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12328,7 +12302,7 @@
       <c r="J137" t="s">
         <v>1504</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12369,7 +12343,7 @@
       <c r="J138" t="s">
         <v>1504</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12410,7 +12384,7 @@
       <c r="J139" t="s">
         <v>1504</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12457,7 +12431,7 @@
       <c r="J140" t="s">
         <v>1504</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12498,7 +12472,7 @@
       <c r="J141" t="s">
         <v>1504</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12539,7 +12513,7 @@
       <c r="J142" t="s">
         <v>1504</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12583,7 +12557,7 @@
       <c r="J143" t="s">
         <v>1504</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12601,7 +12575,7 @@
       <c r="R143" t="s">
         <v>1683</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12636,7 +12610,7 @@
       <c r="J144" t="s">
         <v>1504</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12654,7 +12628,7 @@
       <c r="R144" t="s">
         <v>1683</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12689,7 +12663,7 @@
       <c r="J145" t="s">
         <v>1504</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12707,7 +12681,7 @@
       <c r="R145" t="s">
         <v>1683</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12742,7 +12716,7 @@
       <c r="J146" t="s">
         <v>1504</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12760,7 +12734,7 @@
       <c r="R146" t="s">
         <v>1691</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12795,7 +12769,7 @@
       <c r="J147" t="s">
         <v>1504</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12813,7 +12787,7 @@
       <c r="R147" t="s">
         <v>1698</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12848,7 +12822,7 @@
       <c r="J148" t="s">
         <v>1504</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12889,7 +12863,7 @@
       <c r="J149" t="s">
         <v>1504</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12907,7 +12881,7 @@
       <c r="R149" t="s">
         <v>1683</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12942,7 +12916,7 @@
       <c r="J150" t="s">
         <v>1504</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12960,7 +12934,7 @@
       <c r="R150" t="s">
         <v>1683</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12995,7 +12969,7 @@
       <c r="J151" t="s">
         <v>1504</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13013,7 +12987,7 @@
       <c r="R151" t="s">
         <v>1699</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13048,7 +13022,7 @@
       <c r="J152" t="s">
         <v>1504</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13066,7 +13040,7 @@
       <c r="R152" t="s">
         <v>1700</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13101,7 +13075,7 @@
       <c r="J153" t="s">
         <v>1504</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13110,7 +13084,7 @@
       <c r="M153" t="s">
         <v>1576</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13151,7 +13125,7 @@
       <c r="J154" t="s">
         <v>1504</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13192,7 +13166,7 @@
       <c r="J155" t="s">
         <v>1504</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13233,7 +13207,7 @@
       <c r="J156" t="s">
         <v>1504</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13274,7 +13248,7 @@
       <c r="J157" t="s">
         <v>1504</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13315,7 +13289,7 @@
       <c r="J158" t="s">
         <v>1504</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13356,7 +13330,7 @@
       <c r="J159" t="s">
         <v>1504</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13397,7 +13371,7 @@
       <c r="J160" t="s">
         <v>1504</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13438,7 +13412,7 @@
       <c r="J161" t="s">
         <v>1504</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13479,7 +13453,7 @@
       <c r="J162" t="s">
         <v>1504</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13497,7 +13471,7 @@
       <c r="R162" t="s">
         <v>1686</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13532,7 +13506,7 @@
       <c r="J163" t="s">
         <v>1504</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13550,7 +13524,7 @@
       <c r="R163" t="s">
         <v>1683</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13585,7 +13559,7 @@
       <c r="J164" t="s">
         <v>1504</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13629,7 +13603,7 @@
       <c r="J165" t="s">
         <v>1504</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13670,7 +13644,7 @@
       <c r="J166" t="s">
         <v>1504</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13688,7 +13662,7 @@
       <c r="R166" t="s">
         <v>1701</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13723,7 +13697,7 @@
       <c r="J167" t="s">
         <v>1504</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13767,7 +13741,7 @@
       <c r="J168" t="s">
         <v>1504</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13811,7 +13785,7 @@
       <c r="J169" t="s">
         <v>1504</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13852,7 +13826,7 @@
       <c r="J170" t="s">
         <v>1504</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13893,7 +13867,7 @@
       <c r="J171" t="s">
         <v>1504</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13934,7 +13908,7 @@
       <c r="J172" t="s">
         <v>1504</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13975,7 +13949,7 @@
       <c r="J173" t="s">
         <v>1504</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14016,7 +13990,7 @@
       <c r="J174" t="s">
         <v>1504</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14057,7 +14031,7 @@
       <c r="J175" t="s">
         <v>1504</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14098,7 +14072,7 @@
       <c r="J176" t="s">
         <v>1504</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14139,7 +14113,7 @@
       <c r="J177" t="s">
         <v>1504</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14180,7 +14154,7 @@
       <c r="J178" t="s">
         <v>1504</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14198,7 +14172,7 @@
       <c r="R178" t="s">
         <v>1699</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14233,7 +14207,7 @@
       <c r="J179" t="s">
         <v>1504</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14242,7 +14216,7 @@
       <c r="M179" t="s">
         <v>1573</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14283,7 +14257,7 @@
       <c r="J180" t="s">
         <v>1504</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14324,7 +14298,7 @@
       <c r="J181" t="s">
         <v>1504</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14342,7 +14316,7 @@
       <c r="R181" t="s">
         <v>1683</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14377,7 +14351,7 @@
       <c r="J182" t="s">
         <v>1504</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14418,7 +14392,7 @@
       <c r="J183" t="s">
         <v>1504</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14459,7 +14433,7 @@
       <c r="J184" t="s">
         <v>1504</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14500,7 +14474,7 @@
       <c r="J185" t="s">
         <v>1504</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14541,7 +14515,7 @@
       <c r="J186" t="s">
         <v>1504</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14582,7 +14556,7 @@
       <c r="J187" t="s">
         <v>1504</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14623,7 +14597,7 @@
       <c r="J188" t="s">
         <v>1504</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14664,7 +14638,7 @@
       <c r="J189" t="s">
         <v>1504</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14705,7 +14679,7 @@
       <c r="J190" t="s">
         <v>1504</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14746,7 +14720,7 @@
       <c r="J191" t="s">
         <v>1504</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14787,7 +14761,7 @@
       <c r="J192" t="s">
         <v>1504</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14828,7 +14802,7 @@
       <c r="J193" t="s">
         <v>1504</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14869,7 +14843,7 @@
       <c r="J194" t="s">
         <v>1504</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14910,7 +14884,7 @@
       <c r="J195" t="s">
         <v>1504</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14928,7 +14902,7 @@
       <c r="R195" t="s">
         <v>1692</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14966,7 +14940,7 @@
       <c r="J196" t="s">
         <v>1504</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14984,7 +14958,7 @@
       <c r="R196" t="s">
         <v>1698</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15022,7 +14996,7 @@
       <c r="J197" t="s">
         <v>1504</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15063,7 +15037,7 @@
       <c r="J198" t="s">
         <v>1506</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15104,7 +15078,7 @@
       <c r="J199" t="s">
         <v>1505</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15145,7 +15119,7 @@
       <c r="J200" t="s">
         <v>1504</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15186,7 +15160,7 @@
       <c r="J201" t="s">
         <v>1504</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15227,7 +15201,7 @@
       <c r="J202" t="s">
         <v>1504</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15245,7 +15219,7 @@
       <c r="R202" t="s">
         <v>1683</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15280,7 +15254,7 @@
       <c r="J203" t="s">
         <v>1504</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15298,7 +15272,7 @@
       <c r="R203" t="s">
         <v>1691</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15333,7 +15307,7 @@
       <c r="J204" t="s">
         <v>1504</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15348,7 +15322,7 @@
       <c r="R204" t="s">
         <v>1702</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15386,7 +15360,7 @@
       <c r="J205" t="s">
         <v>1504</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15404,7 +15378,7 @@
       <c r="R205" t="s">
         <v>1703</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15442,7 +15416,7 @@
       <c r="J206" t="s">
         <v>1504</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15460,7 +15434,7 @@
       <c r="R206" t="s">
         <v>1671</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15495,7 +15469,7 @@
       <c r="J207" t="s">
         <v>1504</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15536,7 +15510,7 @@
       <c r="J208" t="s">
         <v>1504</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15577,7 +15551,7 @@
       <c r="J209" t="s">
         <v>1504</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15618,7 +15592,7 @@
       <c r="J210" t="s">
         <v>1504</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15659,7 +15633,7 @@
       <c r="J211" t="s">
         <v>1504</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15700,7 +15674,7 @@
       <c r="J212" t="s">
         <v>1504</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15741,7 +15715,7 @@
       <c r="J213" t="s">
         <v>1504</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15782,7 +15756,7 @@
       <c r="J214" t="s">
         <v>1504</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15800,7 +15774,7 @@
       <c r="R214" t="s">
         <v>1704</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15835,7 +15809,7 @@
       <c r="J215" t="s">
         <v>1504</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15876,7 +15850,7 @@
       <c r="J216" t="s">
         <v>1504</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15917,7 +15891,7 @@
       <c r="J217" t="s">
         <v>1504</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15958,7 +15932,7 @@
       <c r="J218" t="s">
         <v>1504</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15999,7 +15973,7 @@
       <c r="J219" t="s">
         <v>1504</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16040,7 +16014,7 @@
       <c r="J220" t="s">
         <v>1504</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16081,7 +16055,7 @@
       <c r="J221" t="s">
         <v>1504</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16122,7 +16096,7 @@
       <c r="J222" t="s">
         <v>1504</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16163,7 +16137,7 @@
       <c r="J223" t="s">
         <v>1504</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16204,7 +16178,7 @@
       <c r="J224" t="s">
         <v>1504</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16245,7 +16219,7 @@
       <c r="J225" t="s">
         <v>1504</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16286,7 +16260,7 @@
       <c r="J226" t="s">
         <v>1504</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16327,7 +16301,7 @@
       <c r="J227" t="s">
         <v>1504</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16368,7 +16342,7 @@
       <c r="J228" t="s">
         <v>1504</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16409,7 +16383,7 @@
       <c r="J229" t="s">
         <v>1504</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16450,7 +16424,7 @@
       <c r="J230" t="s">
         <v>1504</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16491,7 +16465,7 @@
       <c r="J231" t="s">
         <v>1504</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16532,7 +16506,7 @@
       <c r="J232" t="s">
         <v>1504</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16573,7 +16547,7 @@
       <c r="J233" t="s">
         <v>1504</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16614,7 +16588,7 @@
       <c r="J234" t="s">
         <v>1504</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16655,7 +16629,7 @@
       <c r="J235" t="s">
         <v>1504</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16696,7 +16670,7 @@
       <c r="J236" t="s">
         <v>1504</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16737,7 +16711,7 @@
       <c r="J237" t="s">
         <v>1504</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16778,7 +16752,7 @@
       <c r="J238" t="s">
         <v>1504</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16819,7 +16793,7 @@
       <c r="J239" t="s">
         <v>1504</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16837,7 +16811,7 @@
       <c r="R239" t="s">
         <v>1698</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16872,7 +16846,7 @@
       <c r="J240" t="s">
         <v>1504</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16913,7 +16887,7 @@
       <c r="J241" t="s">
         <v>1504</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16954,7 +16928,7 @@
       <c r="J242" t="s">
         <v>1504</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16972,7 +16946,7 @@
       <c r="R242" t="s">
         <v>1691</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17007,7 +16981,7 @@
       <c r="J243" t="s">
         <v>1504</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17048,7 +17022,7 @@
       <c r="J244" t="s">
         <v>1504</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17089,7 +17063,7 @@
       <c r="J245" t="s">
         <v>1504</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17130,7 +17104,7 @@
       <c r="J246" t="s">
         <v>1504</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17148,7 +17122,7 @@
       <c r="R246" t="s">
         <v>1671</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17183,7 +17157,7 @@
       <c r="J247" t="s">
         <v>1504</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17224,7 +17198,7 @@
       <c r="J248" t="s">
         <v>1504</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17265,7 +17239,7 @@
       <c r="J249" t="s">
         <v>1504</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17306,7 +17280,7 @@
       <c r="J250" t="s">
         <v>1504</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17347,7 +17321,7 @@
       <c r="J251" t="s">
         <v>1504</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17388,7 +17362,7 @@
       <c r="J252" t="s">
         <v>1504</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17429,7 +17403,7 @@
       <c r="J253" t="s">
         <v>1504</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17447,7 +17421,7 @@
       <c r="R253" t="s">
         <v>1701</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17485,7 +17459,7 @@
       <c r="J254" t="s">
         <v>1504</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17526,7 +17500,7 @@
       <c r="J255" t="s">
         <v>1504</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17567,7 +17541,7 @@
       <c r="J256" t="s">
         <v>1504</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17576,7 +17550,7 @@
       <c r="M256" t="s">
         <v>1572</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17614,7 +17588,7 @@
       <c r="J257" t="s">
         <v>1504</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17623,7 +17597,7 @@
       <c r="M257" t="s">
         <v>1573</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17667,7 +17641,7 @@
       <c r="J258" t="s">
         <v>1504</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17685,7 +17659,7 @@
       <c r="R258" t="s">
         <v>1683</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17723,7 +17697,7 @@
       <c r="J259" t="s">
         <v>1504</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17741,7 +17715,7 @@
       <c r="R259" t="s">
         <v>1699</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17779,7 +17753,7 @@
       <c r="J260" t="s">
         <v>1504</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17788,7 +17762,7 @@
       <c r="M260" t="s">
         <v>1567</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17832,7 +17806,7 @@
       <c r="J261" t="s">
         <v>1504</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17850,7 +17824,7 @@
       <c r="R261" t="s">
         <v>1705</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17888,7 +17862,7 @@
       <c r="J262" t="s">
         <v>1504</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17906,7 +17880,7 @@
       <c r="R262" t="s">
         <v>1699</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17944,7 +17918,7 @@
       <c r="J263" t="s">
         <v>1504</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17953,7 +17927,7 @@
       <c r="M263" t="s">
         <v>1567</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17997,7 +17971,7 @@
       <c r="J264" t="s">
         <v>1504</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18038,7 +18012,7 @@
       <c r="J265" t="s">
         <v>1504</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18079,7 +18053,7 @@
       <c r="J266" t="s">
         <v>1504</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18120,7 +18094,7 @@
       <c r="J267" t="s">
         <v>1504</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18164,7 +18138,7 @@
       <c r="J268" t="s">
         <v>1504</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18205,7 +18179,7 @@
       <c r="J269" t="s">
         <v>1504</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18246,7 +18220,7 @@
       <c r="J270" t="s">
         <v>1504</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18287,7 +18261,7 @@
       <c r="J271" t="s">
         <v>1504</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18328,7 +18302,7 @@
       <c r="J272" t="s">
         <v>1504</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18346,7 +18320,7 @@
       <c r="R272" t="s">
         <v>1706</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18384,7 +18358,7 @@
       <c r="J273" t="s">
         <v>1504</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18428,7 +18402,7 @@
       <c r="J274" t="s">
         <v>1504</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18469,7 +18443,7 @@
       <c r="J275" t="s">
         <v>1504</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18510,7 +18484,7 @@
       <c r="J276" t="s">
         <v>1504</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18551,7 +18525,7 @@
       <c r="J277" t="s">
         <v>1504</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18592,7 +18566,7 @@
       <c r="J278" t="s">
         <v>1504</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18633,7 +18607,7 @@
       <c r="J279" t="s">
         <v>1504</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18674,7 +18648,7 @@
       <c r="J280" t="s">
         <v>1504</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18715,7 +18689,7 @@
       <c r="J281" t="s">
         <v>1504</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18756,7 +18730,7 @@
       <c r="J282" t="s">
         <v>1504</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18797,7 +18771,7 @@
       <c r="J283" t="s">
         <v>1504</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18838,7 +18812,7 @@
       <c r="J284" t="s">
         <v>1504</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18879,7 +18853,7 @@
       <c r="J285" t="s">
         <v>1504</v>
       </c>
-      <c r="K285" s="2">
+      <c r="K285" s="1">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18920,7 +18894,7 @@
       <c r="J286" t="s">
         <v>1504</v>
       </c>
-      <c r="K286" s="2">
+      <c r="K286" s="1">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18961,7 +18935,7 @@
       <c r="J287" t="s">
         <v>1504</v>
       </c>
-      <c r="K287" s="2">
+      <c r="K287" s="1">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -19002,7 +18976,7 @@
       <c r="J288" t="s">
         <v>1504</v>
       </c>
-      <c r="K288" s="2">
+      <c r="K288" s="1">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19043,7 +19017,7 @@
       <c r="J289" t="s">
         <v>1504</v>
       </c>
-      <c r="K289" s="2">
+      <c r="K289" s="1">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19084,7 +19058,7 @@
       <c r="J290" t="s">
         <v>1504</v>
       </c>
-      <c r="K290" s="2">
+      <c r="K290" s="1">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19125,7 +19099,7 @@
       <c r="J291" t="s">
         <v>1504</v>
       </c>
-      <c r="K291" s="2">
+      <c r="K291" s="1">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19166,7 +19140,7 @@
       <c r="J292" t="s">
         <v>1504</v>
       </c>
-      <c r="K292" s="2">
+      <c r="K292" s="1">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19207,7 +19181,7 @@
       <c r="J293" t="s">
         <v>1504</v>
       </c>
-      <c r="K293" s="2">
+      <c r="K293" s="1">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19248,7 +19222,7 @@
       <c r="J294" t="s">
         <v>1504</v>
       </c>
-      <c r="K294" s="2">
+      <c r="K294" s="1">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19289,7 +19263,7 @@
       <c r="J295" t="s">
         <v>1504</v>
       </c>
-      <c r="K295" s="2">
+      <c r="K295" s="1">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19307,7 +19281,7 @@
       <c r="R295" t="s">
         <v>1707</v>
       </c>
-      <c r="T295" s="2">
+      <c r="T295" s="1">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19345,7 +19319,7 @@
       <c r="J296" t="s">
         <v>1504</v>
       </c>
-      <c r="K296" s="2">
+      <c r="K296" s="1">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19363,7 +19337,7 @@
       <c r="R296" t="s">
         <v>1683</v>
       </c>
-      <c r="T296" s="2">
+      <c r="T296" s="1">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19401,7 +19375,7 @@
       <c r="J297" t="s">
         <v>1504</v>
       </c>
-      <c r="K297" s="2">
+      <c r="K297" s="1">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19442,7 +19416,7 @@
       <c r="J298" t="s">
         <v>1504</v>
       </c>
-      <c r="K298" s="2">
+      <c r="K298" s="1">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19483,7 +19457,7 @@
       <c r="J299" t="s">
         <v>1505</v>
       </c>
-      <c r="K299" s="2">
+      <c r="K299" s="1">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19524,7 +19498,7 @@
       <c r="J300" t="s">
         <v>1504</v>
       </c>
-      <c r="K300" s="2">
+      <c r="K300" s="1">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19565,7 +19539,7 @@
       <c r="J301" t="s">
         <v>1504</v>
       </c>
-      <c r="K301" s="2">
+      <c r="K301" s="1">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20403,7 +20377,7 @@
       <c r="R321" t="s">
         <v>1669</v>
       </c>
-      <c r="T321" s="2">
+      <c r="T321" s="1">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20623,7 +20597,7 @@
       <c r="R326" t="s">
         <v>1708</v>
       </c>
-      <c r="T326" s="2">
+      <c r="T326" s="1">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21458,7 +21432,7 @@
       <c r="R346" t="s">
         <v>1709</v>
       </c>
-      <c r="T346" s="2">
+      <c r="T346" s="1">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (08/09/2026 08:24)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5262,8 +5262,16 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="1">
+  <fonts count="2">
     <font>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5279,7 +5287,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="1">
+  <borders count="2">
     <border>
       <left/>
       <right/>
@@ -5287,12 +5295,30 @@
       <bottom/>
       <diagonal/>
     </border>
+    <border>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="3">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="top"/>
+    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5592,73 +5618,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" t="s">
+      <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" t="s">
+      <c r="B1" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" t="s">
+      <c r="D1" s="1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" t="s">
+      <c r="E1" s="1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" t="s">
+      <c r="F1" s="1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" t="s">
+      <c r="G1" s="1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" t="s">
+      <c r="H1" s="1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" t="s">
+      <c r="I1" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" t="s">
+      <c r="J1" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" t="s">
+      <c r="K1" s="1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" t="s">
+      <c r="L1" s="1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" t="s">
+      <c r="M1" s="1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" t="s">
+      <c r="N1" s="1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" t="s">
+      <c r="O1" s="1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" t="s">
+      <c r="P1" s="1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" t="s">
+      <c r="Q1" s="1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" t="s">
+      <c r="R1" s="1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" t="s">
+      <c r="S1" s="1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" t="s">
+      <c r="T1" s="1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" t="s">
+      <c r="U1" s="1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" t="s">
+      <c r="V1" s="1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" t="s">
+      <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5693,7 +5719,7 @@
       <c r="J2" t="s">
         <v>1504</v>
       </c>
-      <c r="K2" s="1">
+      <c r="K2" s="2">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5737,7 +5763,7 @@
       <c r="J3" t="s">
         <v>1504</v>
       </c>
-      <c r="K3" s="1">
+      <c r="K3" s="2">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5781,7 +5807,7 @@
       <c r="J4" t="s">
         <v>1504</v>
       </c>
-      <c r="K4" s="1">
+      <c r="K4" s="2">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5799,7 +5825,7 @@
       <c r="R4" t="s">
         <v>1666</v>
       </c>
-      <c r="T4" s="1">
+      <c r="T4" s="2">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5837,7 +5863,7 @@
       <c r="J5" t="s">
         <v>1505</v>
       </c>
-      <c r="K5" s="1">
+      <c r="K5" s="2">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5887,7 +5913,7 @@
       <c r="J6" t="s">
         <v>1504</v>
       </c>
-      <c r="K6" s="1">
+      <c r="K6" s="2">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5934,7 +5960,7 @@
       <c r="J7" t="s">
         <v>1504</v>
       </c>
-      <c r="K7" s="1">
+      <c r="K7" s="2">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -5981,7 +6007,7 @@
       <c r="J8" t="s">
         <v>1504</v>
       </c>
-      <c r="K8" s="1">
+      <c r="K8" s="2">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6028,7 +6054,7 @@
       <c r="J9" t="s">
         <v>1504</v>
       </c>
-      <c r="K9" s="1">
+      <c r="K9" s="2">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6075,7 +6101,7 @@
       <c r="J10" t="s">
         <v>1504</v>
       </c>
-      <c r="K10" s="1">
+      <c r="K10" s="2">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6122,7 +6148,7 @@
       <c r="J11" t="s">
         <v>1504</v>
       </c>
-      <c r="K11" s="1">
+      <c r="K11" s="2">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6169,7 +6195,7 @@
       <c r="J12" t="s">
         <v>1504</v>
       </c>
-      <c r="K12" s="1">
+      <c r="K12" s="2">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6213,7 +6239,7 @@
       <c r="J13" t="s">
         <v>1504</v>
       </c>
-      <c r="K13" s="1">
+      <c r="K13" s="2">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6231,7 +6257,7 @@
       <c r="R13" t="s">
         <v>1667</v>
       </c>
-      <c r="T13" s="1">
+      <c r="T13" s="2">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6269,7 +6295,7 @@
       <c r="J14" t="s">
         <v>1504</v>
       </c>
-      <c r="K14" s="1">
+      <c r="K14" s="2">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6287,7 +6313,7 @@
       <c r="R14" t="s">
         <v>1668</v>
       </c>
-      <c r="T14" s="1">
+      <c r="T14" s="2">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6325,7 +6351,7 @@
       <c r="J15" t="s">
         <v>1504</v>
       </c>
-      <c r="K15" s="1">
+      <c r="K15" s="2">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6343,7 +6369,7 @@
       <c r="R15" t="s">
         <v>1668</v>
       </c>
-      <c r="T15" s="1">
+      <c r="T15" s="2">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6381,7 +6407,7 @@
       <c r="J16" t="s">
         <v>1504</v>
       </c>
-      <c r="K16" s="1">
+      <c r="K16" s="2">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6425,7 +6451,7 @@
       <c r="J17" t="s">
         <v>1504</v>
       </c>
-      <c r="K17" s="1">
+      <c r="K17" s="2">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6469,7 +6495,7 @@
       <c r="J18" t="s">
         <v>1504</v>
       </c>
-      <c r="K18" s="1">
+      <c r="K18" s="2">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6487,7 +6513,7 @@
       <c r="R18" t="s">
         <v>1669</v>
       </c>
-      <c r="T18" s="1">
+      <c r="T18" s="2">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6528,7 +6554,7 @@
       <c r="J19" t="s">
         <v>1504</v>
       </c>
-      <c r="K19" s="1">
+      <c r="K19" s="2">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6572,7 +6598,7 @@
       <c r="J20" t="s">
         <v>1504</v>
       </c>
-      <c r="K20" s="1">
+      <c r="K20" s="2">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6616,7 +6642,7 @@
       <c r="J21" t="s">
         <v>1504</v>
       </c>
-      <c r="K21" s="1">
+      <c r="K21" s="2">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6634,7 +6660,7 @@
       <c r="R21" t="s">
         <v>1668</v>
       </c>
-      <c r="T21" s="1">
+      <c r="T21" s="2">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6675,7 +6701,7 @@
       <c r="J22" t="s">
         <v>1504</v>
       </c>
-      <c r="K22" s="1">
+      <c r="K22" s="2">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6693,7 +6719,7 @@
       <c r="R22" t="s">
         <v>1670</v>
       </c>
-      <c r="T22" s="1">
+      <c r="T22" s="2">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6734,7 +6760,7 @@
       <c r="J23" t="s">
         <v>1504</v>
       </c>
-      <c r="K23" s="1">
+      <c r="K23" s="2">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6752,7 +6778,7 @@
       <c r="R23" t="s">
         <v>1671</v>
       </c>
-      <c r="T23" s="1">
+      <c r="T23" s="2">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6793,7 +6819,7 @@
       <c r="J24" t="s">
         <v>1504</v>
       </c>
-      <c r="K24" s="1">
+      <c r="K24" s="2">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6837,7 +6863,7 @@
       <c r="J25" t="s">
         <v>1504</v>
       </c>
-      <c r="K25" s="1">
+      <c r="K25" s="2">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6878,7 +6904,7 @@
       <c r="J26" t="s">
         <v>1506</v>
       </c>
-      <c r="K26" s="1">
+      <c r="K26" s="2">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6896,7 +6922,7 @@
       <c r="R26" t="s">
         <v>1672</v>
       </c>
-      <c r="T26" s="1">
+      <c r="T26" s="2">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6931,7 +6957,7 @@
       <c r="J27" t="s">
         <v>1504</v>
       </c>
-      <c r="K27" s="1">
+      <c r="K27" s="2">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6949,7 +6975,7 @@
       <c r="R27" t="s">
         <v>1673</v>
       </c>
-      <c r="T27" s="1">
+      <c r="T27" s="2">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -6990,7 +7016,7 @@
       <c r="J28" t="s">
         <v>1504</v>
       </c>
-      <c r="K28" s="1">
+      <c r="K28" s="2">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7034,7 +7060,7 @@
       <c r="J29" t="s">
         <v>1504</v>
       </c>
-      <c r="K29" s="1">
+      <c r="K29" s="2">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7078,7 +7104,7 @@
       <c r="J30" t="s">
         <v>1504</v>
       </c>
-      <c r="K30" s="1">
+      <c r="K30" s="2">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7122,7 +7148,7 @@
       <c r="J31" t="s">
         <v>1504</v>
       </c>
-      <c r="K31" s="1">
+      <c r="K31" s="2">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7140,7 +7166,7 @@
       <c r="R31" t="s">
         <v>1674</v>
       </c>
-      <c r="T31" s="1">
+      <c r="T31" s="2">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7181,7 +7207,7 @@
       <c r="J32" t="s">
         <v>1504</v>
       </c>
-      <c r="K32" s="1">
+      <c r="K32" s="2">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7225,7 +7251,7 @@
       <c r="J33" t="s">
         <v>1504</v>
       </c>
-      <c r="K33" s="1">
+      <c r="K33" s="2">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7243,7 +7269,7 @@
       <c r="R33" t="s">
         <v>1675</v>
       </c>
-      <c r="T33" s="1">
+      <c r="T33" s="2">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7284,7 +7310,7 @@
       <c r="J34" t="s">
         <v>1504</v>
       </c>
-      <c r="K34" s="1">
+      <c r="K34" s="2">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7328,7 +7354,7 @@
       <c r="J35" t="s">
         <v>1504</v>
       </c>
-      <c r="K35" s="1">
+      <c r="K35" s="2">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7346,7 +7372,7 @@
       <c r="R35" t="s">
         <v>1676</v>
       </c>
-      <c r="T35" s="1">
+      <c r="T35" s="2">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7387,7 +7413,7 @@
       <c r="J36" t="s">
         <v>1504</v>
       </c>
-      <c r="K36" s="1">
+      <c r="K36" s="2">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7405,7 +7431,7 @@
       <c r="R36" t="s">
         <v>1676</v>
       </c>
-      <c r="T36" s="1">
+      <c r="T36" s="2">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7446,7 +7472,7 @@
       <c r="J37" t="s">
         <v>1504</v>
       </c>
-      <c r="K37" s="1">
+      <c r="K37" s="2">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7464,7 +7490,7 @@
       <c r="R37" t="s">
         <v>1676</v>
       </c>
-      <c r="T37" s="1">
+      <c r="T37" s="2">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7505,7 +7531,7 @@
       <c r="J38" t="s">
         <v>1504</v>
       </c>
-      <c r="K38" s="1">
+      <c r="K38" s="2">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7523,7 +7549,7 @@
       <c r="R38" t="s">
         <v>1676</v>
       </c>
-      <c r="T38" s="1">
+      <c r="T38" s="2">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7564,7 +7590,7 @@
       <c r="J39" t="s">
         <v>1504</v>
       </c>
-      <c r="K39" s="1">
+      <c r="K39" s="2">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7582,7 +7608,7 @@
       <c r="R39" t="s">
         <v>1676</v>
       </c>
-      <c r="T39" s="1">
+      <c r="T39" s="2">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7623,7 +7649,7 @@
       <c r="J40" t="s">
         <v>1504</v>
       </c>
-      <c r="K40" s="1">
+      <c r="K40" s="2">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7641,7 +7667,7 @@
       <c r="R40" t="s">
         <v>1677</v>
       </c>
-      <c r="T40" s="1">
+      <c r="T40" s="2">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7682,7 +7708,7 @@
       <c r="J41" t="s">
         <v>1504</v>
       </c>
-      <c r="K41" s="1">
+      <c r="K41" s="2">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7700,7 +7726,7 @@
       <c r="R41" t="s">
         <v>1668</v>
       </c>
-      <c r="T41" s="1">
+      <c r="T41" s="2">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7738,7 +7764,7 @@
       <c r="J42" t="s">
         <v>1504</v>
       </c>
-      <c r="K42" s="1">
+      <c r="K42" s="2">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7756,7 +7782,7 @@
       <c r="R42" t="s">
         <v>1676</v>
       </c>
-      <c r="T42" s="1">
+      <c r="T42" s="2">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7797,7 +7823,7 @@
       <c r="J43" t="s">
         <v>1504</v>
       </c>
-      <c r="K43" s="1">
+      <c r="K43" s="2">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7841,7 +7867,7 @@
       <c r="J44" t="s">
         <v>1504</v>
       </c>
-      <c r="K44" s="1">
+      <c r="K44" s="2">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7859,7 +7885,7 @@
       <c r="R44" t="s">
         <v>1678</v>
       </c>
-      <c r="T44" s="1">
+      <c r="T44" s="2">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7900,7 +7926,7 @@
       <c r="J45" t="s">
         <v>1504</v>
       </c>
-      <c r="K45" s="1">
+      <c r="K45" s="2">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7918,7 +7944,7 @@
       <c r="R45" t="s">
         <v>1679</v>
       </c>
-      <c r="T45" s="1">
+      <c r="T45" s="2">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7956,7 +7982,7 @@
       <c r="J46" t="s">
         <v>1504</v>
       </c>
-      <c r="K46" s="1">
+      <c r="K46" s="2">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8000,7 +8026,7 @@
       <c r="J47" t="s">
         <v>1504</v>
       </c>
-      <c r="K47" s="1">
+      <c r="K47" s="2">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8018,7 +8044,7 @@
       <c r="R47" t="s">
         <v>1680</v>
       </c>
-      <c r="T47" s="1">
+      <c r="T47" s="2">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8059,7 +8085,7 @@
       <c r="J48" t="s">
         <v>1504</v>
       </c>
-      <c r="K48" s="1">
+      <c r="K48" s="2">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8103,7 +8129,7 @@
       <c r="J49" t="s">
         <v>1504</v>
       </c>
-      <c r="K49" s="1">
+      <c r="K49" s="2">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8147,7 +8173,7 @@
       <c r="J50" t="s">
         <v>1504</v>
       </c>
-      <c r="K50" s="1">
+      <c r="K50" s="2">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8191,7 +8217,7 @@
       <c r="J51" t="s">
         <v>1504</v>
       </c>
-      <c r="K51" s="1">
+      <c r="K51" s="2">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8238,7 +8264,7 @@
       <c r="J52" t="s">
         <v>1504</v>
       </c>
-      <c r="K52" s="1">
+      <c r="K52" s="2">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8282,7 +8308,7 @@
       <c r="J53" t="s">
         <v>1504</v>
       </c>
-      <c r="K53" s="1">
+      <c r="K53" s="2">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8326,7 +8352,7 @@
       <c r="J54" t="s">
         <v>1504</v>
       </c>
-      <c r="K54" s="1">
+      <c r="K54" s="2">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8370,7 +8396,7 @@
       <c r="J55" t="s">
         <v>1504</v>
       </c>
-      <c r="K55" s="1">
+      <c r="K55" s="2">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8420,7 +8446,7 @@
       <c r="J56" t="s">
         <v>1504</v>
       </c>
-      <c r="K56" s="1">
+      <c r="K56" s="2">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8473,7 +8499,7 @@
       <c r="J57" t="s">
         <v>1504</v>
       </c>
-      <c r="K57" s="1">
+      <c r="K57" s="2">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8523,7 +8549,7 @@
       <c r="J58" t="s">
         <v>1504</v>
       </c>
-      <c r="K58" s="1">
+      <c r="K58" s="2">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8573,7 +8599,7 @@
       <c r="J59" t="s">
         <v>1504</v>
       </c>
-      <c r="K59" s="1">
+      <c r="K59" s="2">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8591,7 +8617,7 @@
       <c r="R59" t="s">
         <v>1681</v>
       </c>
-      <c r="T59" s="1">
+      <c r="T59" s="2">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8632,7 +8658,7 @@
       <c r="J60" t="s">
         <v>1504</v>
       </c>
-      <c r="K60" s="1">
+      <c r="K60" s="2">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8676,7 +8702,7 @@
       <c r="J61" t="s">
         <v>1504</v>
       </c>
-      <c r="K61" s="1">
+      <c r="K61" s="2">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8720,7 +8746,7 @@
       <c r="J62" t="s">
         <v>1504</v>
       </c>
-      <c r="K62" s="1">
+      <c r="K62" s="2">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8764,7 +8790,7 @@
       <c r="J63" t="s">
         <v>1504</v>
       </c>
-      <c r="K63" s="1">
+      <c r="K63" s="2">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8808,7 +8834,7 @@
       <c r="J64" t="s">
         <v>1504</v>
       </c>
-      <c r="K64" s="1">
+      <c r="K64" s="2">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8852,7 +8878,7 @@
       <c r="J65" t="s">
         <v>1504</v>
       </c>
-      <c r="K65" s="1">
+      <c r="K65" s="2">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8899,7 +8925,7 @@
       <c r="J66" t="s">
         <v>1504</v>
       </c>
-      <c r="K66" s="1">
+      <c r="K66" s="2">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8917,7 +8943,7 @@
       <c r="R66" t="s">
         <v>1682</v>
       </c>
-      <c r="T66" s="1">
+      <c r="T66" s="2">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8955,7 +8981,7 @@
       <c r="J67" t="s">
         <v>1504</v>
       </c>
-      <c r="K67" s="1">
+      <c r="K67" s="2">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -8999,7 +9025,7 @@
       <c r="J68" t="s">
         <v>1504</v>
       </c>
-      <c r="K68" s="1">
+      <c r="K68" s="2">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9014,7 +9040,7 @@
       <c r="O68" t="s">
         <v>1585</v>
       </c>
-      <c r="T68" s="1">
+      <c r="T68" s="2">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9058,7 +9084,7 @@
       <c r="J69" t="s">
         <v>1506</v>
       </c>
-      <c r="K69" s="1">
+      <c r="K69" s="2">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9102,7 +9128,7 @@
       <c r="J70" t="s">
         <v>1504</v>
       </c>
-      <c r="K70" s="1">
+      <c r="K70" s="2">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9146,7 +9172,7 @@
       <c r="J71" t="s">
         <v>1504</v>
       </c>
-      <c r="K71" s="1">
+      <c r="K71" s="2">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9190,7 +9216,7 @@
       <c r="J72" t="s">
         <v>1504</v>
       </c>
-      <c r="K72" s="1">
+      <c r="K72" s="2">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9234,7 +9260,7 @@
       <c r="J73" t="s">
         <v>1504</v>
       </c>
-      <c r="K73" s="1">
+      <c r="K73" s="2">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9278,7 +9304,7 @@
       <c r="J74" t="s">
         <v>1504</v>
       </c>
-      <c r="K74" s="1">
+      <c r="K74" s="2">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9322,7 +9348,7 @@
       <c r="J75" t="s">
         <v>1504</v>
       </c>
-      <c r="K75" s="1">
+      <c r="K75" s="2">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9366,7 +9392,7 @@
       <c r="J76" t="s">
         <v>1504</v>
       </c>
-      <c r="K76" s="1">
+      <c r="K76" s="2">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9384,7 +9410,7 @@
       <c r="R76" t="s">
         <v>1683</v>
       </c>
-      <c r="T76" s="1">
+      <c r="T76" s="2">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9422,7 +9448,7 @@
       <c r="J77" t="s">
         <v>1504</v>
       </c>
-      <c r="K77" s="1">
+      <c r="K77" s="2">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9440,7 +9466,7 @@
       <c r="R77" t="s">
         <v>1683</v>
       </c>
-      <c r="T77" s="1">
+      <c r="T77" s="2">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9478,7 +9504,7 @@
       <c r="J78" t="s">
         <v>1504</v>
       </c>
-      <c r="K78" s="1">
+      <c r="K78" s="2">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9496,7 +9522,7 @@
       <c r="R78" t="s">
         <v>1683</v>
       </c>
-      <c r="T78" s="1">
+      <c r="T78" s="2">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9534,7 +9560,7 @@
       <c r="J79" t="s">
         <v>1504</v>
       </c>
-      <c r="K79" s="1">
+      <c r="K79" s="2">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9552,7 +9578,7 @@
       <c r="R79" t="s">
         <v>1683</v>
       </c>
-      <c r="T79" s="1">
+      <c r="T79" s="2">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9590,7 +9616,7 @@
       <c r="J80" t="s">
         <v>1504</v>
       </c>
-      <c r="K80" s="1">
+      <c r="K80" s="2">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9634,7 +9660,7 @@
       <c r="J81" t="s">
         <v>1504</v>
       </c>
-      <c r="K81" s="1">
+      <c r="K81" s="2">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9678,7 +9704,7 @@
       <c r="J82" t="s">
         <v>1504</v>
       </c>
-      <c r="K82" s="1">
+      <c r="K82" s="2">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9722,7 +9748,7 @@
       <c r="J83" t="s">
         <v>1504</v>
       </c>
-      <c r="K83" s="1">
+      <c r="K83" s="2">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9766,7 +9792,7 @@
       <c r="J84" t="s">
         <v>1504</v>
       </c>
-      <c r="K84" s="1">
+      <c r="K84" s="2">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9810,7 +9836,7 @@
       <c r="J85" t="s">
         <v>1504</v>
       </c>
-      <c r="K85" s="1">
+      <c r="K85" s="2">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9828,7 +9854,7 @@
       <c r="R85" t="s">
         <v>1684</v>
       </c>
-      <c r="T85" s="1">
+      <c r="T85" s="2">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9866,7 +9892,7 @@
       <c r="J86" t="s">
         <v>1504</v>
       </c>
-      <c r="K86" s="1">
+      <c r="K86" s="2">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9910,7 +9936,7 @@
       <c r="J87" t="s">
         <v>1504</v>
       </c>
-      <c r="K87" s="1">
+      <c r="K87" s="2">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9928,7 +9954,7 @@
       <c r="R87" t="s">
         <v>1685</v>
       </c>
-      <c r="T87" s="1">
+      <c r="T87" s="2">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9966,7 +9992,7 @@
       <c r="J88" t="s">
         <v>1504</v>
       </c>
-      <c r="K88" s="1">
+      <c r="K88" s="2">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10010,7 +10036,7 @@
       <c r="J89" t="s">
         <v>1504</v>
       </c>
-      <c r="K89" s="1">
+      <c r="K89" s="2">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10028,7 +10054,7 @@
       <c r="R89" t="s">
         <v>1686</v>
       </c>
-      <c r="T89" s="1">
+      <c r="T89" s="2">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10063,7 +10089,7 @@
       <c r="J90" t="s">
         <v>1504</v>
       </c>
-      <c r="K90" s="1">
+      <c r="K90" s="2">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10081,7 +10107,7 @@
       <c r="R90" t="s">
         <v>1687</v>
       </c>
-      <c r="T90" s="1">
+      <c r="T90" s="2">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10116,7 +10142,7 @@
       <c r="J91" t="s">
         <v>1504</v>
       </c>
-      <c r="K91" s="1">
+      <c r="K91" s="2">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10134,7 +10160,7 @@
       <c r="R91" t="s">
         <v>1671</v>
       </c>
-      <c r="T91" s="1">
+      <c r="T91" s="2">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10172,7 +10198,7 @@
       <c r="J92" t="s">
         <v>1504</v>
       </c>
-      <c r="K92" s="1">
+      <c r="K92" s="2">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10193,7 +10219,7 @@
       <c r="R92" t="s">
         <v>1671</v>
       </c>
-      <c r="T92" s="1">
+      <c r="T92" s="2">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10234,7 +10260,7 @@
       <c r="J93" t="s">
         <v>1504</v>
       </c>
-      <c r="K93" s="1">
+      <c r="K93" s="2">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10275,7 +10301,7 @@
       <c r="J94" t="s">
         <v>1504</v>
       </c>
-      <c r="K94" s="1">
+      <c r="K94" s="2">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10319,7 +10345,7 @@
       <c r="J95" t="s">
         <v>1504</v>
       </c>
-      <c r="K95" s="1">
+      <c r="K95" s="2">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10363,7 +10389,7 @@
       <c r="J96" t="s">
         <v>1504</v>
       </c>
-      <c r="K96" s="1">
+      <c r="K96" s="2">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10381,7 +10407,7 @@
       <c r="R96" t="s">
         <v>1688</v>
       </c>
-      <c r="T96" s="1">
+      <c r="T96" s="2">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10419,7 +10445,7 @@
       <c r="J97" t="s">
         <v>1504</v>
       </c>
-      <c r="K97" s="1">
+      <c r="K97" s="2">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10434,7 +10460,7 @@
       <c r="R97" t="s">
         <v>1688</v>
       </c>
-      <c r="T97" s="1">
+      <c r="T97" s="2">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10475,7 +10501,7 @@
       <c r="J98" t="s">
         <v>1504</v>
       </c>
-      <c r="K98" s="1">
+      <c r="K98" s="2">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10493,7 +10519,7 @@
       <c r="R98" t="s">
         <v>1689</v>
       </c>
-      <c r="T98" s="1">
+      <c r="T98" s="2">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10531,7 +10557,7 @@
       <c r="J99" t="s">
         <v>1504</v>
       </c>
-      <c r="K99" s="1">
+      <c r="K99" s="2">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10549,7 +10575,7 @@
       <c r="R99" t="s">
         <v>1690</v>
       </c>
-      <c r="T99" s="1">
+      <c r="T99" s="2">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10587,7 +10613,7 @@
       <c r="J100" t="s">
         <v>1504</v>
       </c>
-      <c r="K100" s="1">
+      <c r="K100" s="2">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10628,7 +10654,7 @@
       <c r="J101" t="s">
         <v>1504</v>
       </c>
-      <c r="K101" s="1">
+      <c r="K101" s="2">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10669,7 +10695,7 @@
       <c r="J102" t="s">
         <v>1504</v>
       </c>
-      <c r="K102" s="1">
+      <c r="K102" s="2">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10710,7 +10736,7 @@
       <c r="J103" t="s">
         <v>1504</v>
       </c>
-      <c r="K103" s="1">
+      <c r="K103" s="2">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10751,7 +10777,7 @@
       <c r="J104" t="s">
         <v>1504</v>
       </c>
-      <c r="K104" s="1">
+      <c r="K104" s="2">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10792,7 +10818,7 @@
       <c r="J105" t="s">
         <v>1504</v>
       </c>
-      <c r="K105" s="1">
+      <c r="K105" s="2">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10833,7 +10859,7 @@
       <c r="J106" t="s">
         <v>1504</v>
       </c>
-      <c r="K106" s="1">
+      <c r="K106" s="2">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10874,7 +10900,7 @@
       <c r="J107" t="s">
         <v>1504</v>
       </c>
-      <c r="K107" s="1">
+      <c r="K107" s="2">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10915,7 +10941,7 @@
       <c r="J108" t="s">
         <v>1504</v>
       </c>
-      <c r="K108" s="1">
+      <c r="K108" s="2">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10956,7 +10982,7 @@
       <c r="J109" t="s">
         <v>1504</v>
       </c>
-      <c r="K109" s="1">
+      <c r="K109" s="2">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11009,7 +11035,7 @@
       <c r="J110" t="s">
         <v>1504</v>
       </c>
-      <c r="K110" s="1">
+      <c r="K110" s="2">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11065,7 +11091,7 @@
       <c r="J111" t="s">
         <v>1504</v>
       </c>
-      <c r="K111" s="1">
+      <c r="K111" s="2">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11083,7 +11109,7 @@
       <c r="R111" t="s">
         <v>1692</v>
       </c>
-      <c r="T111" s="1">
+      <c r="T111" s="2">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11121,7 +11147,7 @@
       <c r="J112" t="s">
         <v>1504</v>
       </c>
-      <c r="K112" s="1">
+      <c r="K112" s="2">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11180,7 +11206,7 @@
       <c r="J113" t="s">
         <v>1504</v>
       </c>
-      <c r="K113" s="1">
+      <c r="K113" s="2">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11224,7 +11250,7 @@
       <c r="J114" t="s">
         <v>1504</v>
       </c>
-      <c r="K114" s="1">
+      <c r="K114" s="2">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11268,7 +11294,7 @@
       <c r="J115" t="s">
         <v>1504</v>
       </c>
-      <c r="K115" s="1">
+      <c r="K115" s="2">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11286,7 +11312,7 @@
       <c r="R115" t="s">
         <v>1694</v>
       </c>
-      <c r="T115" s="1">
+      <c r="T115" s="2">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11324,7 +11350,7 @@
       <c r="J116" t="s">
         <v>1504</v>
       </c>
-      <c r="K116" s="1">
+      <c r="K116" s="2">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11383,7 +11409,7 @@
       <c r="J117" t="s">
         <v>1504</v>
       </c>
-      <c r="K117" s="1">
+      <c r="K117" s="2">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11427,7 +11453,7 @@
       <c r="J118" t="s">
         <v>1504</v>
       </c>
-      <c r="K118" s="1">
+      <c r="K118" s="2">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11474,7 +11500,7 @@
       <c r="J119" t="s">
         <v>1504</v>
       </c>
-      <c r="K119" s="1">
+      <c r="K119" s="2">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11515,7 +11541,7 @@
       <c r="J120" t="s">
         <v>1504</v>
       </c>
-      <c r="K120" s="1">
+      <c r="K120" s="2">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11559,7 +11585,7 @@
       <c r="J121" t="s">
         <v>1504</v>
       </c>
-      <c r="K121" s="1">
+      <c r="K121" s="2">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11606,7 +11632,7 @@
       <c r="J122" t="s">
         <v>1504</v>
       </c>
-      <c r="K122" s="1">
+      <c r="K122" s="2">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11656,7 +11682,7 @@
       <c r="J123" t="s">
         <v>1504</v>
       </c>
-      <c r="K123" s="1">
+      <c r="K123" s="2">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11700,7 +11726,7 @@
       <c r="J124" t="s">
         <v>1504</v>
       </c>
-      <c r="K124" s="1">
+      <c r="K124" s="2">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11744,7 +11770,7 @@
       <c r="J125" t="s">
         <v>1504</v>
       </c>
-      <c r="K125" s="1">
+      <c r="K125" s="2">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11762,7 +11788,7 @@
       <c r="R125" t="s">
         <v>1696</v>
       </c>
-      <c r="T125" s="1">
+      <c r="T125" s="2">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11797,7 +11823,7 @@
       <c r="J126" t="s">
         <v>1504</v>
       </c>
-      <c r="K126" s="1">
+      <c r="K126" s="2">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11815,7 +11841,7 @@
       <c r="R126" t="s">
         <v>1697</v>
       </c>
-      <c r="T126" s="1">
+      <c r="T126" s="2">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11850,7 +11876,7 @@
       <c r="J127" t="s">
         <v>1504</v>
       </c>
-      <c r="K127" s="1">
+      <c r="K127" s="2">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11906,7 +11932,7 @@
       <c r="J128" t="s">
         <v>1504</v>
       </c>
-      <c r="K128" s="1">
+      <c r="K128" s="2">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11947,7 +11973,7 @@
       <c r="J129" t="s">
         <v>1504</v>
       </c>
-      <c r="K129" s="1">
+      <c r="K129" s="2">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -11988,7 +12014,7 @@
       <c r="J130" t="s">
         <v>1504</v>
       </c>
-      <c r="K130" s="1">
+      <c r="K130" s="2">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12029,7 +12055,7 @@
       <c r="J131" t="s">
         <v>1504</v>
       </c>
-      <c r="K131" s="1">
+      <c r="K131" s="2">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12073,7 +12099,7 @@
       <c r="J132" t="s">
         <v>1504</v>
       </c>
-      <c r="K132" s="1">
+      <c r="K132" s="2">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12114,7 +12140,7 @@
       <c r="J133" t="s">
         <v>1504</v>
       </c>
-      <c r="K133" s="1">
+      <c r="K133" s="2">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12132,7 +12158,7 @@
       <c r="R133" t="s">
         <v>1683</v>
       </c>
-      <c r="T133" s="1">
+      <c r="T133" s="2">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12167,7 +12193,7 @@
       <c r="J134" t="s">
         <v>1504</v>
       </c>
-      <c r="K134" s="1">
+      <c r="K134" s="2">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12185,7 +12211,7 @@
       <c r="R134" t="s">
         <v>1683</v>
       </c>
-      <c r="T134" s="1">
+      <c r="T134" s="2">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12220,7 +12246,7 @@
       <c r="J135" t="s">
         <v>1504</v>
       </c>
-      <c r="K135" s="1">
+      <c r="K135" s="2">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12261,7 +12287,7 @@
       <c r="J136" t="s">
         <v>1504</v>
       </c>
-      <c r="K136" s="1">
+      <c r="K136" s="2">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12302,7 +12328,7 @@
       <c r="J137" t="s">
         <v>1504</v>
       </c>
-      <c r="K137" s="1">
+      <c r="K137" s="2">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12343,7 +12369,7 @@
       <c r="J138" t="s">
         <v>1504</v>
       </c>
-      <c r="K138" s="1">
+      <c r="K138" s="2">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12384,7 +12410,7 @@
       <c r="J139" t="s">
         <v>1504</v>
       </c>
-      <c r="K139" s="1">
+      <c r="K139" s="2">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12431,7 +12457,7 @@
       <c r="J140" t="s">
         <v>1504</v>
       </c>
-      <c r="K140" s="1">
+      <c r="K140" s="2">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12472,7 +12498,7 @@
       <c r="J141" t="s">
         <v>1504</v>
       </c>
-      <c r="K141" s="1">
+      <c r="K141" s="2">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12513,7 +12539,7 @@
       <c r="J142" t="s">
         <v>1504</v>
       </c>
-      <c r="K142" s="1">
+      <c r="K142" s="2">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12557,7 +12583,7 @@
       <c r="J143" t="s">
         <v>1504</v>
       </c>
-      <c r="K143" s="1">
+      <c r="K143" s="2">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12575,7 +12601,7 @@
       <c r="R143" t="s">
         <v>1683</v>
       </c>
-      <c r="T143" s="1">
+      <c r="T143" s="2">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12610,7 +12636,7 @@
       <c r="J144" t="s">
         <v>1504</v>
       </c>
-      <c r="K144" s="1">
+      <c r="K144" s="2">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12628,7 +12654,7 @@
       <c r="R144" t="s">
         <v>1683</v>
       </c>
-      <c r="T144" s="1">
+      <c r="T144" s="2">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12663,7 +12689,7 @@
       <c r="J145" t="s">
         <v>1504</v>
       </c>
-      <c r="K145" s="1">
+      <c r="K145" s="2">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12681,7 +12707,7 @@
       <c r="R145" t="s">
         <v>1683</v>
       </c>
-      <c r="T145" s="1">
+      <c r="T145" s="2">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12716,7 +12742,7 @@
       <c r="J146" t="s">
         <v>1504</v>
       </c>
-      <c r="K146" s="1">
+      <c r="K146" s="2">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12734,7 +12760,7 @@
       <c r="R146" t="s">
         <v>1691</v>
       </c>
-      <c r="T146" s="1">
+      <c r="T146" s="2">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12769,7 +12795,7 @@
       <c r="J147" t="s">
         <v>1504</v>
       </c>
-      <c r="K147" s="1">
+      <c r="K147" s="2">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12787,7 +12813,7 @@
       <c r="R147" t="s">
         <v>1698</v>
       </c>
-      <c r="T147" s="1">
+      <c r="T147" s="2">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12822,7 +12848,7 @@
       <c r="J148" t="s">
         <v>1504</v>
       </c>
-      <c r="K148" s="1">
+      <c r="K148" s="2">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12863,7 +12889,7 @@
       <c r="J149" t="s">
         <v>1504</v>
       </c>
-      <c r="K149" s="1">
+      <c r="K149" s="2">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12881,7 +12907,7 @@
       <c r="R149" t="s">
         <v>1683</v>
       </c>
-      <c r="T149" s="1">
+      <c r="T149" s="2">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12916,7 +12942,7 @@
       <c r="J150" t="s">
         <v>1504</v>
       </c>
-      <c r="K150" s="1">
+      <c r="K150" s="2">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12934,7 +12960,7 @@
       <c r="R150" t="s">
         <v>1683</v>
       </c>
-      <c r="T150" s="1">
+      <c r="T150" s="2">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12969,7 +12995,7 @@
       <c r="J151" t="s">
         <v>1504</v>
       </c>
-      <c r="K151" s="1">
+      <c r="K151" s="2">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -12987,7 +13013,7 @@
       <c r="R151" t="s">
         <v>1699</v>
       </c>
-      <c r="T151" s="1">
+      <c r="T151" s="2">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13022,7 +13048,7 @@
       <c r="J152" t="s">
         <v>1504</v>
       </c>
-      <c r="K152" s="1">
+      <c r="K152" s="2">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13040,7 +13066,7 @@
       <c r="R152" t="s">
         <v>1700</v>
       </c>
-      <c r="T152" s="1">
+      <c r="T152" s="2">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13075,7 +13101,7 @@
       <c r="J153" t="s">
         <v>1504</v>
       </c>
-      <c r="K153" s="1">
+      <c r="K153" s="2">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13084,7 +13110,7 @@
       <c r="M153" t="s">
         <v>1576</v>
       </c>
-      <c r="T153" s="1">
+      <c r="T153" s="2">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13125,7 +13151,7 @@
       <c r="J154" t="s">
         <v>1504</v>
       </c>
-      <c r="K154" s="1">
+      <c r="K154" s="2">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13166,7 +13192,7 @@
       <c r="J155" t="s">
         <v>1504</v>
       </c>
-      <c r="K155" s="1">
+      <c r="K155" s="2">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13207,7 +13233,7 @@
       <c r="J156" t="s">
         <v>1504</v>
       </c>
-      <c r="K156" s="1">
+      <c r="K156" s="2">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13248,7 +13274,7 @@
       <c r="J157" t="s">
         <v>1504</v>
       </c>
-      <c r="K157" s="1">
+      <c r="K157" s="2">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13289,7 +13315,7 @@
       <c r="J158" t="s">
         <v>1504</v>
       </c>
-      <c r="K158" s="1">
+      <c r="K158" s="2">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13330,7 +13356,7 @@
       <c r="J159" t="s">
         <v>1504</v>
       </c>
-      <c r="K159" s="1">
+      <c r="K159" s="2">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13371,7 +13397,7 @@
       <c r="J160" t="s">
         <v>1504</v>
       </c>
-      <c r="K160" s="1">
+      <c r="K160" s="2">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13412,7 +13438,7 @@
       <c r="J161" t="s">
         <v>1504</v>
       </c>
-      <c r="K161" s="1">
+      <c r="K161" s="2">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13453,7 +13479,7 @@
       <c r="J162" t="s">
         <v>1504</v>
       </c>
-      <c r="K162" s="1">
+      <c r="K162" s="2">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13471,7 +13497,7 @@
       <c r="R162" t="s">
         <v>1686</v>
       </c>
-      <c r="T162" s="1">
+      <c r="T162" s="2">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13506,7 +13532,7 @@
       <c r="J163" t="s">
         <v>1504</v>
       </c>
-      <c r="K163" s="1">
+      <c r="K163" s="2">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13524,7 +13550,7 @@
       <c r="R163" t="s">
         <v>1683</v>
       </c>
-      <c r="T163" s="1">
+      <c r="T163" s="2">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13559,7 +13585,7 @@
       <c r="J164" t="s">
         <v>1504</v>
       </c>
-      <c r="K164" s="1">
+      <c r="K164" s="2">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13603,7 +13629,7 @@
       <c r="J165" t="s">
         <v>1504</v>
       </c>
-      <c r="K165" s="1">
+      <c r="K165" s="2">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13644,7 +13670,7 @@
       <c r="J166" t="s">
         <v>1504</v>
       </c>
-      <c r="K166" s="1">
+      <c r="K166" s="2">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13662,7 +13688,7 @@
       <c r="R166" t="s">
         <v>1701</v>
       </c>
-      <c r="T166" s="1">
+      <c r="T166" s="2">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13697,7 +13723,7 @@
       <c r="J167" t="s">
         <v>1504</v>
       </c>
-      <c r="K167" s="1">
+      <c r="K167" s="2">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13741,7 +13767,7 @@
       <c r="J168" t="s">
         <v>1504</v>
       </c>
-      <c r="K168" s="1">
+      <c r="K168" s="2">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13785,7 +13811,7 @@
       <c r="J169" t="s">
         <v>1504</v>
       </c>
-      <c r="K169" s="1">
+      <c r="K169" s="2">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13826,7 +13852,7 @@
       <c r="J170" t="s">
         <v>1504</v>
       </c>
-      <c r="K170" s="1">
+      <c r="K170" s="2">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13867,7 +13893,7 @@
       <c r="J171" t="s">
         <v>1504</v>
       </c>
-      <c r="K171" s="1">
+      <c r="K171" s="2">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13908,7 +13934,7 @@
       <c r="J172" t="s">
         <v>1504</v>
       </c>
-      <c r="K172" s="1">
+      <c r="K172" s="2">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13949,7 +13975,7 @@
       <c r="J173" t="s">
         <v>1504</v>
       </c>
-      <c r="K173" s="1">
+      <c r="K173" s="2">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -13990,7 +14016,7 @@
       <c r="J174" t="s">
         <v>1504</v>
       </c>
-      <c r="K174" s="1">
+      <c r="K174" s="2">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14031,7 +14057,7 @@
       <c r="J175" t="s">
         <v>1504</v>
       </c>
-      <c r="K175" s="1">
+      <c r="K175" s="2">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14072,7 +14098,7 @@
       <c r="J176" t="s">
         <v>1504</v>
       </c>
-      <c r="K176" s="1">
+      <c r="K176" s="2">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14113,7 +14139,7 @@
       <c r="J177" t="s">
         <v>1504</v>
       </c>
-      <c r="K177" s="1">
+      <c r="K177" s="2">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14154,7 +14180,7 @@
       <c r="J178" t="s">
         <v>1504</v>
       </c>
-      <c r="K178" s="1">
+      <c r="K178" s="2">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14172,7 +14198,7 @@
       <c r="R178" t="s">
         <v>1699</v>
       </c>
-      <c r="T178" s="1">
+      <c r="T178" s="2">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14207,7 +14233,7 @@
       <c r="J179" t="s">
         <v>1504</v>
       </c>
-      <c r="K179" s="1">
+      <c r="K179" s="2">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14216,7 +14242,7 @@
       <c r="M179" t="s">
         <v>1573</v>
       </c>
-      <c r="T179" s="1">
+      <c r="T179" s="2">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14257,7 +14283,7 @@
       <c r="J180" t="s">
         <v>1504</v>
       </c>
-      <c r="K180" s="1">
+      <c r="K180" s="2">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14298,7 +14324,7 @@
       <c r="J181" t="s">
         <v>1504</v>
       </c>
-      <c r="K181" s="1">
+      <c r="K181" s="2">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14316,7 +14342,7 @@
       <c r="R181" t="s">
         <v>1683</v>
       </c>
-      <c r="T181" s="1">
+      <c r="T181" s="2">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14351,7 +14377,7 @@
       <c r="J182" t="s">
         <v>1504</v>
       </c>
-      <c r="K182" s="1">
+      <c r="K182" s="2">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14392,7 +14418,7 @@
       <c r="J183" t="s">
         <v>1504</v>
       </c>
-      <c r="K183" s="1">
+      <c r="K183" s="2">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14433,7 +14459,7 @@
       <c r="J184" t="s">
         <v>1504</v>
       </c>
-      <c r="K184" s="1">
+      <c r="K184" s="2">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14474,7 +14500,7 @@
       <c r="J185" t="s">
         <v>1504</v>
       </c>
-      <c r="K185" s="1">
+      <c r="K185" s="2">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14515,7 +14541,7 @@
       <c r="J186" t="s">
         <v>1504</v>
       </c>
-      <c r="K186" s="1">
+      <c r="K186" s="2">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14556,7 +14582,7 @@
       <c r="J187" t="s">
         <v>1504</v>
       </c>
-      <c r="K187" s="1">
+      <c r="K187" s="2">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14597,7 +14623,7 @@
       <c r="J188" t="s">
         <v>1504</v>
       </c>
-      <c r="K188" s="1">
+      <c r="K188" s="2">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14638,7 +14664,7 @@
       <c r="J189" t="s">
         <v>1504</v>
       </c>
-      <c r="K189" s="1">
+      <c r="K189" s="2">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14679,7 +14705,7 @@
       <c r="J190" t="s">
         <v>1504</v>
       </c>
-      <c r="K190" s="1">
+      <c r="K190" s="2">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14720,7 +14746,7 @@
       <c r="J191" t="s">
         <v>1504</v>
       </c>
-      <c r="K191" s="1">
+      <c r="K191" s="2">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14761,7 +14787,7 @@
       <c r="J192" t="s">
         <v>1504</v>
       </c>
-      <c r="K192" s="1">
+      <c r="K192" s="2">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14802,7 +14828,7 @@
       <c r="J193" t="s">
         <v>1504</v>
       </c>
-      <c r="K193" s="1">
+      <c r="K193" s="2">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14843,7 +14869,7 @@
       <c r="J194" t="s">
         <v>1504</v>
       </c>
-      <c r="K194" s="1">
+      <c r="K194" s="2">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14884,7 +14910,7 @@
       <c r="J195" t="s">
         <v>1504</v>
       </c>
-      <c r="K195" s="1">
+      <c r="K195" s="2">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14902,7 +14928,7 @@
       <c r="R195" t="s">
         <v>1692</v>
       </c>
-      <c r="T195" s="1">
+      <c r="T195" s="2">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14940,7 +14966,7 @@
       <c r="J196" t="s">
         <v>1504</v>
       </c>
-      <c r="K196" s="1">
+      <c r="K196" s="2">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14958,7 +14984,7 @@
       <c r="R196" t="s">
         <v>1698</v>
       </c>
-      <c r="T196" s="1">
+      <c r="T196" s="2">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -14996,7 +15022,7 @@
       <c r="J197" t="s">
         <v>1504</v>
       </c>
-      <c r="K197" s="1">
+      <c r="K197" s="2">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15037,7 +15063,7 @@
       <c r="J198" t="s">
         <v>1506</v>
       </c>
-      <c r="K198" s="1">
+      <c r="K198" s="2">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15078,7 +15104,7 @@
       <c r="J199" t="s">
         <v>1505</v>
       </c>
-      <c r="K199" s="1">
+      <c r="K199" s="2">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15119,7 +15145,7 @@
       <c r="J200" t="s">
         <v>1504</v>
       </c>
-      <c r="K200" s="1">
+      <c r="K200" s="2">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15160,7 +15186,7 @@
       <c r="J201" t="s">
         <v>1504</v>
       </c>
-      <c r="K201" s="1">
+      <c r="K201" s="2">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15201,7 +15227,7 @@
       <c r="J202" t="s">
         <v>1504</v>
       </c>
-      <c r="K202" s="1">
+      <c r="K202" s="2">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15219,7 +15245,7 @@
       <c r="R202" t="s">
         <v>1683</v>
       </c>
-      <c r="T202" s="1">
+      <c r="T202" s="2">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15254,7 +15280,7 @@
       <c r="J203" t="s">
         <v>1504</v>
       </c>
-      <c r="K203" s="1">
+      <c r="K203" s="2">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15272,7 +15298,7 @@
       <c r="R203" t="s">
         <v>1691</v>
       </c>
-      <c r="T203" s="1">
+      <c r="T203" s="2">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15307,7 +15333,7 @@
       <c r="J204" t="s">
         <v>1504</v>
       </c>
-      <c r="K204" s="1">
+      <c r="K204" s="2">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15322,7 +15348,7 @@
       <c r="R204" t="s">
         <v>1702</v>
       </c>
-      <c r="T204" s="1">
+      <c r="T204" s="2">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15360,7 +15386,7 @@
       <c r="J205" t="s">
         <v>1504</v>
       </c>
-      <c r="K205" s="1">
+      <c r="K205" s="2">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15378,7 +15404,7 @@
       <c r="R205" t="s">
         <v>1703</v>
       </c>
-      <c r="T205" s="1">
+      <c r="T205" s="2">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15416,7 +15442,7 @@
       <c r="J206" t="s">
         <v>1504</v>
       </c>
-      <c r="K206" s="1">
+      <c r="K206" s="2">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15434,7 +15460,7 @@
       <c r="R206" t="s">
         <v>1671</v>
       </c>
-      <c r="T206" s="1">
+      <c r="T206" s="2">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15469,7 +15495,7 @@
       <c r="J207" t="s">
         <v>1504</v>
       </c>
-      <c r="K207" s="1">
+      <c r="K207" s="2">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15510,7 +15536,7 @@
       <c r="J208" t="s">
         <v>1504</v>
       </c>
-      <c r="K208" s="1">
+      <c r="K208" s="2">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15551,7 +15577,7 @@
       <c r="J209" t="s">
         <v>1504</v>
       </c>
-      <c r="K209" s="1">
+      <c r="K209" s="2">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15592,7 +15618,7 @@
       <c r="J210" t="s">
         <v>1504</v>
       </c>
-      <c r="K210" s="1">
+      <c r="K210" s="2">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15633,7 +15659,7 @@
       <c r="J211" t="s">
         <v>1504</v>
       </c>
-      <c r="K211" s="1">
+      <c r="K211" s="2">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15674,7 +15700,7 @@
       <c r="J212" t="s">
         <v>1504</v>
       </c>
-      <c r="K212" s="1">
+      <c r="K212" s="2">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15715,7 +15741,7 @@
       <c r="J213" t="s">
         <v>1504</v>
       </c>
-      <c r="K213" s="1">
+      <c r="K213" s="2">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15756,7 +15782,7 @@
       <c r="J214" t="s">
         <v>1504</v>
       </c>
-      <c r="K214" s="1">
+      <c r="K214" s="2">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15774,7 +15800,7 @@
       <c r="R214" t="s">
         <v>1704</v>
       </c>
-      <c r="T214" s="1">
+      <c r="T214" s="2">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15809,7 +15835,7 @@
       <c r="J215" t="s">
         <v>1504</v>
       </c>
-      <c r="K215" s="1">
+      <c r="K215" s="2">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15850,7 +15876,7 @@
       <c r="J216" t="s">
         <v>1504</v>
       </c>
-      <c r="K216" s="1">
+      <c r="K216" s="2">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15891,7 +15917,7 @@
       <c r="J217" t="s">
         <v>1504</v>
       </c>
-      <c r="K217" s="1">
+      <c r="K217" s="2">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15932,7 +15958,7 @@
       <c r="J218" t="s">
         <v>1504</v>
       </c>
-      <c r="K218" s="1">
+      <c r="K218" s="2">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15973,7 +15999,7 @@
       <c r="J219" t="s">
         <v>1504</v>
       </c>
-      <c r="K219" s="1">
+      <c r="K219" s="2">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16014,7 +16040,7 @@
       <c r="J220" t="s">
         <v>1504</v>
       </c>
-      <c r="K220" s="1">
+      <c r="K220" s="2">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16055,7 +16081,7 @@
       <c r="J221" t="s">
         <v>1504</v>
       </c>
-      <c r="K221" s="1">
+      <c r="K221" s="2">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16096,7 +16122,7 @@
       <c r="J222" t="s">
         <v>1504</v>
       </c>
-      <c r="K222" s="1">
+      <c r="K222" s="2">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16137,7 +16163,7 @@
       <c r="J223" t="s">
         <v>1504</v>
       </c>
-      <c r="K223" s="1">
+      <c r="K223" s="2">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16178,7 +16204,7 @@
       <c r="J224" t="s">
         <v>1504</v>
       </c>
-      <c r="K224" s="1">
+      <c r="K224" s="2">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16219,7 +16245,7 @@
       <c r="J225" t="s">
         <v>1504</v>
       </c>
-      <c r="K225" s="1">
+      <c r="K225" s="2">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16260,7 +16286,7 @@
       <c r="J226" t="s">
         <v>1504</v>
       </c>
-      <c r="K226" s="1">
+      <c r="K226" s="2">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16301,7 +16327,7 @@
       <c r="J227" t="s">
         <v>1504</v>
       </c>
-      <c r="K227" s="1">
+      <c r="K227" s="2">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16342,7 +16368,7 @@
       <c r="J228" t="s">
         <v>1504</v>
       </c>
-      <c r="K228" s="1">
+      <c r="K228" s="2">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16383,7 +16409,7 @@
       <c r="J229" t="s">
         <v>1504</v>
       </c>
-      <c r="K229" s="1">
+      <c r="K229" s="2">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16424,7 +16450,7 @@
       <c r="J230" t="s">
         <v>1504</v>
       </c>
-      <c r="K230" s="1">
+      <c r="K230" s="2">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16465,7 +16491,7 @@
       <c r="J231" t="s">
         <v>1504</v>
       </c>
-      <c r="K231" s="1">
+      <c r="K231" s="2">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16506,7 +16532,7 @@
       <c r="J232" t="s">
         <v>1504</v>
       </c>
-      <c r="K232" s="1">
+      <c r="K232" s="2">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16547,7 +16573,7 @@
       <c r="J233" t="s">
         <v>1504</v>
       </c>
-      <c r="K233" s="1">
+      <c r="K233" s="2">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16588,7 +16614,7 @@
       <c r="J234" t="s">
         <v>1504</v>
       </c>
-      <c r="K234" s="1">
+      <c r="K234" s="2">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16629,7 +16655,7 @@
       <c r="J235" t="s">
         <v>1504</v>
       </c>
-      <c r="K235" s="1">
+      <c r="K235" s="2">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16670,7 +16696,7 @@
       <c r="J236" t="s">
         <v>1504</v>
       </c>
-      <c r="K236" s="1">
+      <c r="K236" s="2">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16711,7 +16737,7 @@
       <c r="J237" t="s">
         <v>1504</v>
       </c>
-      <c r="K237" s="1">
+      <c r="K237" s="2">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16752,7 +16778,7 @@
       <c r="J238" t="s">
         <v>1504</v>
       </c>
-      <c r="K238" s="1">
+      <c r="K238" s="2">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16793,7 +16819,7 @@
       <c r="J239" t="s">
         <v>1504</v>
       </c>
-      <c r="K239" s="1">
+      <c r="K239" s="2">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16811,7 +16837,7 @@
       <c r="R239" t="s">
         <v>1698</v>
       </c>
-      <c r="T239" s="1">
+      <c r="T239" s="2">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16846,7 +16872,7 @@
       <c r="J240" t="s">
         <v>1504</v>
       </c>
-      <c r="K240" s="1">
+      <c r="K240" s="2">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16887,7 +16913,7 @@
       <c r="J241" t="s">
         <v>1504</v>
       </c>
-      <c r="K241" s="1">
+      <c r="K241" s="2">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16928,7 +16954,7 @@
       <c r="J242" t="s">
         <v>1504</v>
       </c>
-      <c r="K242" s="1">
+      <c r="K242" s="2">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16946,7 +16972,7 @@
       <c r="R242" t="s">
         <v>1691</v>
       </c>
-      <c r="T242" s="1">
+      <c r="T242" s="2">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -16981,7 +17007,7 @@
       <c r="J243" t="s">
         <v>1504</v>
       </c>
-      <c r="K243" s="1">
+      <c r="K243" s="2">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17022,7 +17048,7 @@
       <c r="J244" t="s">
         <v>1504</v>
       </c>
-      <c r="K244" s="1">
+      <c r="K244" s="2">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17063,7 +17089,7 @@
       <c r="J245" t="s">
         <v>1504</v>
       </c>
-      <c r="K245" s="1">
+      <c r="K245" s="2">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17104,7 +17130,7 @@
       <c r="J246" t="s">
         <v>1504</v>
       </c>
-      <c r="K246" s="1">
+      <c r="K246" s="2">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17122,7 +17148,7 @@
       <c r="R246" t="s">
         <v>1671</v>
       </c>
-      <c r="T246" s="1">
+      <c r="T246" s="2">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17157,7 +17183,7 @@
       <c r="J247" t="s">
         <v>1504</v>
       </c>
-      <c r="K247" s="1">
+      <c r="K247" s="2">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17198,7 +17224,7 @@
       <c r="J248" t="s">
         <v>1504</v>
       </c>
-      <c r="K248" s="1">
+      <c r="K248" s="2">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17239,7 +17265,7 @@
       <c r="J249" t="s">
         <v>1504</v>
       </c>
-      <c r="K249" s="1">
+      <c r="K249" s="2">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17280,7 +17306,7 @@
       <c r="J250" t="s">
         <v>1504</v>
       </c>
-      <c r="K250" s="1">
+      <c r="K250" s="2">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17321,7 +17347,7 @@
       <c r="J251" t="s">
         <v>1504</v>
       </c>
-      <c r="K251" s="1">
+      <c r="K251" s="2">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17362,7 +17388,7 @@
       <c r="J252" t="s">
         <v>1504</v>
       </c>
-      <c r="K252" s="1">
+      <c r="K252" s="2">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17403,7 +17429,7 @@
       <c r="J253" t="s">
         <v>1504</v>
       </c>
-      <c r="K253" s="1">
+      <c r="K253" s="2">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17421,7 +17447,7 @@
       <c r="R253" t="s">
         <v>1701</v>
       </c>
-      <c r="T253" s="1">
+      <c r="T253" s="2">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17459,7 +17485,7 @@
       <c r="J254" t="s">
         <v>1504</v>
       </c>
-      <c r="K254" s="1">
+      <c r="K254" s="2">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17500,7 +17526,7 @@
       <c r="J255" t="s">
         <v>1504</v>
       </c>
-      <c r="K255" s="1">
+      <c r="K255" s="2">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17541,7 +17567,7 @@
       <c r="J256" t="s">
         <v>1504</v>
       </c>
-      <c r="K256" s="1">
+      <c r="K256" s="2">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17550,7 +17576,7 @@
       <c r="M256" t="s">
         <v>1572</v>
       </c>
-      <c r="T256" s="1">
+      <c r="T256" s="2">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17588,7 +17614,7 @@
       <c r="J257" t="s">
         <v>1504</v>
       </c>
-      <c r="K257" s="1">
+      <c r="K257" s="2">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17597,7 +17623,7 @@
       <c r="M257" t="s">
         <v>1573</v>
       </c>
-      <c r="T257" s="1">
+      <c r="T257" s="2">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17641,7 +17667,7 @@
       <c r="J258" t="s">
         <v>1504</v>
       </c>
-      <c r="K258" s="1">
+      <c r="K258" s="2">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17659,7 +17685,7 @@
       <c r="R258" t="s">
         <v>1683</v>
       </c>
-      <c r="T258" s="1">
+      <c r="T258" s="2">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17697,7 +17723,7 @@
       <c r="J259" t="s">
         <v>1504</v>
       </c>
-      <c r="K259" s="1">
+      <c r="K259" s="2">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17715,7 +17741,7 @@
       <c r="R259" t="s">
         <v>1699</v>
       </c>
-      <c r="T259" s="1">
+      <c r="T259" s="2">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17753,7 +17779,7 @@
       <c r="J260" t="s">
         <v>1504</v>
       </c>
-      <c r="K260" s="1">
+      <c r="K260" s="2">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17762,7 +17788,7 @@
       <c r="M260" t="s">
         <v>1567</v>
       </c>
-      <c r="T260" s="1">
+      <c r="T260" s="2">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17806,7 +17832,7 @@
       <c r="J261" t="s">
         <v>1504</v>
       </c>
-      <c r="K261" s="1">
+      <c r="K261" s="2">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17824,7 +17850,7 @@
       <c r="R261" t="s">
         <v>1705</v>
       </c>
-      <c r="T261" s="1">
+      <c r="T261" s="2">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17862,7 +17888,7 @@
       <c r="J262" t="s">
         <v>1504</v>
       </c>
-      <c r="K262" s="1">
+      <c r="K262" s="2">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17880,7 +17906,7 @@
       <c r="R262" t="s">
         <v>1699</v>
       </c>
-      <c r="T262" s="1">
+      <c r="T262" s="2">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17918,7 +17944,7 @@
       <c r="J263" t="s">
         <v>1504</v>
       </c>
-      <c r="K263" s="1">
+      <c r="K263" s="2">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17927,7 +17953,7 @@
       <c r="M263" t="s">
         <v>1567</v>
       </c>
-      <c r="T263" s="1">
+      <c r="T263" s="2">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17971,7 +17997,7 @@
       <c r="J264" t="s">
         <v>1504</v>
       </c>
-      <c r="K264" s="1">
+      <c r="K264" s="2">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18012,7 +18038,7 @@
       <c r="J265" t="s">
         <v>1504</v>
       </c>
-      <c r="K265" s="1">
+      <c r="K265" s="2">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18053,7 +18079,7 @@
       <c r="J266" t="s">
         <v>1504</v>
       </c>
-      <c r="K266" s="1">
+      <c r="K266" s="2">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18094,7 +18120,7 @@
       <c r="J267" t="s">
         <v>1504</v>
       </c>
-      <c r="K267" s="1">
+      <c r="K267" s="2">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18138,7 +18164,7 @@
       <c r="J268" t="s">
         <v>1504</v>
       </c>
-      <c r="K268" s="1">
+      <c r="K268" s="2">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18179,7 +18205,7 @@
       <c r="J269" t="s">
         <v>1504</v>
       </c>
-      <c r="K269" s="1">
+      <c r="K269" s="2">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18220,7 +18246,7 @@
       <c r="J270" t="s">
         <v>1504</v>
       </c>
-      <c r="K270" s="1">
+      <c r="K270" s="2">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18261,7 +18287,7 @@
       <c r="J271" t="s">
         <v>1504</v>
       </c>
-      <c r="K271" s="1">
+      <c r="K271" s="2">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18302,7 +18328,7 @@
       <c r="J272" t="s">
         <v>1504</v>
       </c>
-      <c r="K272" s="1">
+      <c r="K272" s="2">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18320,7 +18346,7 @@
       <c r="R272" t="s">
         <v>1706</v>
       </c>
-      <c r="T272" s="1">
+      <c r="T272" s="2">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18358,7 +18384,7 @@
       <c r="J273" t="s">
         <v>1504</v>
       </c>
-      <c r="K273" s="1">
+      <c r="K273" s="2">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18402,7 +18428,7 @@
       <c r="J274" t="s">
         <v>1504</v>
       </c>
-      <c r="K274" s="1">
+      <c r="K274" s="2">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18443,7 +18469,7 @@
       <c r="J275" t="s">
         <v>1504</v>
       </c>
-      <c r="K275" s="1">
+      <c r="K275" s="2">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18484,7 +18510,7 @@
       <c r="J276" t="s">
         <v>1504</v>
       </c>
-      <c r="K276" s="1">
+      <c r="K276" s="2">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18525,7 +18551,7 @@
       <c r="J277" t="s">
         <v>1504</v>
       </c>
-      <c r="K277" s="1">
+      <c r="K277" s="2">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18566,7 +18592,7 @@
       <c r="J278" t="s">
         <v>1504</v>
       </c>
-      <c r="K278" s="1">
+      <c r="K278" s="2">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18607,7 +18633,7 @@
       <c r="J279" t="s">
         <v>1504</v>
       </c>
-      <c r="K279" s="1">
+      <c r="K279" s="2">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18648,7 +18674,7 @@
       <c r="J280" t="s">
         <v>1504</v>
       </c>
-      <c r="K280" s="1">
+      <c r="K280" s="2">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18689,7 +18715,7 @@
       <c r="J281" t="s">
         <v>1504</v>
       </c>
-      <c r="K281" s="1">
+      <c r="K281" s="2">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18730,7 +18756,7 @@
       <c r="J282" t="s">
         <v>1504</v>
       </c>
-      <c r="K282" s="1">
+      <c r="K282" s="2">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18771,7 +18797,7 @@
       <c r="J283" t="s">
         <v>1504</v>
       </c>
-      <c r="K283" s="1">
+      <c r="K283" s="2">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18812,7 +18838,7 @@
       <c r="J284" t="s">
         <v>1504</v>
       </c>
-      <c r="K284" s="1">
+      <c r="K284" s="2">
         <v>46174</v>
       </c>
       <c r="L284" t="s">
@@ -18853,7 +18879,7 @@
       <c r="J285" t="s">
         <v>1504</v>
       </c>
-      <c r="K285" s="1">
+      <c r="K285" s="2">
         <v>46174</v>
       </c>
       <c r="L285" t="s">
@@ -18894,7 +18920,7 @@
       <c r="J286" t="s">
         <v>1504</v>
       </c>
-      <c r="K286" s="1">
+      <c r="K286" s="2">
         <v>46174</v>
       </c>
       <c r="L286" t="s">
@@ -18935,7 +18961,7 @@
       <c r="J287" t="s">
         <v>1504</v>
       </c>
-      <c r="K287" s="1">
+      <c r="K287" s="2">
         <v>46174</v>
       </c>
       <c r="L287" t="s">
@@ -18976,7 +19002,7 @@
       <c r="J288" t="s">
         <v>1504</v>
       </c>
-      <c r="K288" s="1">
+      <c r="K288" s="2">
         <v>46176</v>
       </c>
       <c r="L288" t="s">
@@ -19017,7 +19043,7 @@
       <c r="J289" t="s">
         <v>1504</v>
       </c>
-      <c r="K289" s="1">
+      <c r="K289" s="2">
         <v>46182</v>
       </c>
       <c r="L289" t="s">
@@ -19058,7 +19084,7 @@
       <c r="J290" t="s">
         <v>1504</v>
       </c>
-      <c r="K290" s="1">
+      <c r="K290" s="2">
         <v>46182</v>
       </c>
       <c r="L290" t="s">
@@ -19099,7 +19125,7 @@
       <c r="J291" t="s">
         <v>1504</v>
       </c>
-      <c r="K291" s="1">
+      <c r="K291" s="2">
         <v>46183</v>
       </c>
       <c r="L291" t="s">
@@ -19140,7 +19166,7 @@
       <c r="J292" t="s">
         <v>1504</v>
       </c>
-      <c r="K292" s="1">
+      <c r="K292" s="2">
         <v>46185</v>
       </c>
       <c r="L292" t="s">
@@ -19181,7 +19207,7 @@
       <c r="J293" t="s">
         <v>1504</v>
       </c>
-      <c r="K293" s="1">
+      <c r="K293" s="2">
         <v>46192</v>
       </c>
       <c r="L293" t="s">
@@ -19222,7 +19248,7 @@
       <c r="J294" t="s">
         <v>1504</v>
       </c>
-      <c r="K294" s="1">
+      <c r="K294" s="2">
         <v>46192</v>
       </c>
       <c r="L294" t="s">
@@ -19263,7 +19289,7 @@
       <c r="J295" t="s">
         <v>1504</v>
       </c>
-      <c r="K295" s="1">
+      <c r="K295" s="2">
         <v>46192</v>
       </c>
       <c r="L295" t="s">
@@ -19281,7 +19307,7 @@
       <c r="R295" t="s">
         <v>1707</v>
       </c>
-      <c r="T295" s="1">
+      <c r="T295" s="2">
         <v>45912</v>
       </c>
       <c r="W295" t="s">
@@ -19319,7 +19345,7 @@
       <c r="J296" t="s">
         <v>1504</v>
       </c>
-      <c r="K296" s="1">
+      <c r="K296" s="2">
         <v>46192</v>
       </c>
       <c r="L296" t="s">
@@ -19337,7 +19363,7 @@
       <c r="R296" t="s">
         <v>1683</v>
       </c>
-      <c r="T296" s="1">
+      <c r="T296" s="2">
         <v>46230</v>
       </c>
       <c r="W296" t="s">
@@ -19375,7 +19401,7 @@
       <c r="J297" t="s">
         <v>1504</v>
       </c>
-      <c r="K297" s="1">
+      <c r="K297" s="2">
         <v>46192</v>
       </c>
       <c r="L297" t="s">
@@ -19416,7 +19442,7 @@
       <c r="J298" t="s">
         <v>1504</v>
       </c>
-      <c r="K298" s="1">
+      <c r="K298" s="2">
         <v>46192</v>
       </c>
       <c r="L298" t="s">
@@ -19457,7 +19483,7 @@
       <c r="J299" t="s">
         <v>1505</v>
       </c>
-      <c r="K299" s="1">
+      <c r="K299" s="2">
         <v>46192</v>
       </c>
       <c r="L299" t="s">
@@ -19498,7 +19524,7 @@
       <c r="J300" t="s">
         <v>1504</v>
       </c>
-      <c r="K300" s="1">
+      <c r="K300" s="2">
         <v>46192</v>
       </c>
       <c r="L300" t="s">
@@ -19539,7 +19565,7 @@
       <c r="J301" t="s">
         <v>1504</v>
       </c>
-      <c r="K301" s="1">
+      <c r="K301" s="2">
         <v>46192</v>
       </c>
       <c r="L301" t="s">
@@ -20377,7 +20403,7 @@
       <c r="R321" t="s">
         <v>1669</v>
       </c>
-      <c r="T321" s="1">
+      <c r="T321" s="2">
         <v>45845</v>
       </c>
       <c r="W321" t="s">
@@ -20597,7 +20623,7 @@
       <c r="R326" t="s">
         <v>1708</v>
       </c>
-      <c r="T326" s="1">
+      <c r="T326" s="2">
         <v>45848</v>
       </c>
       <c r="W326" t="s">
@@ -21432,7 +21458,7 @@
       <c r="R346" t="s">
         <v>1709</v>
       </c>
-      <c r="T346" s="1">
+      <c r="T346" s="2">
         <v>46234</v>
       </c>
       <c r="W346" t="s">

</xml_diff>

<commit_message>
Atualização automática: devolucoes (08/09/2026 12:05)
</commit_message>
<xml_diff>
--- a/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
+++ b/Contrato 005/Dashboard/02_Dados_Tratados/base_devolucoes_tratada.xlsx
@@ -5262,16 +5262,8 @@
   <numFmts count="1">
     <numFmt numFmtId="164" formatCode="YYYY-MM-DD HH:MM:SS"/>
   </numFmts>
-  <fonts count="2">
+  <fonts count="1">
     <font>
-      <sz val="11"/>
-      <color theme="1"/>
-      <name val="Calibri"/>
-      <family val="2"/>
-      <scheme val="minor"/>
-    </font>
-    <font>
-      <b/>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Calibri"/>
@@ -5287,7 +5279,7 @@
       <patternFill patternType="gray125"/>
     </fill>
   </fills>
-  <borders count="2">
+  <borders count="1">
     <border>
       <left/>
       <right/>
@@ -5295,30 +5287,12 @@
       <bottom/>
       <diagonal/>
     </border>
-    <border>
-      <left style="thin">
-        <color auto="1"/>
-      </left>
-      <right style="thin">
-        <color auto="1"/>
-      </right>
-      <top style="thin">
-        <color auto="1"/>
-      </top>
-      <bottom style="thin">
-        <color auto="1"/>
-      </bottom>
-      <diagonal/>
-    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="3">
+  <cellXfs count="2">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="top"/>
-    </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
   </cellXfs>
   <cellStyles count="1">
@@ -5618,73 +5592,73 @@
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:23">
-      <c r="A1" s="1" t="s">
+      <c r="A1" t="s">
         <v>0</v>
       </c>
-      <c r="B1" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C1" s="1" t="s">
+      <c r="B1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C1" t="s">
         <v>2</v>
       </c>
-      <c r="D1" s="1" t="s">
+      <c r="D1" t="s">
         <v>3</v>
       </c>
-      <c r="E1" s="1" t="s">
+      <c r="E1" t="s">
         <v>4</v>
       </c>
-      <c r="F1" s="1" t="s">
+      <c r="F1" t="s">
         <v>5</v>
       </c>
-      <c r="G1" s="1" t="s">
+      <c r="G1" t="s">
         <v>6</v>
       </c>
-      <c r="H1" s="1" t="s">
+      <c r="H1" t="s">
         <v>7</v>
       </c>
-      <c r="I1" s="1" t="s">
+      <c r="I1" t="s">
         <v>8</v>
       </c>
-      <c r="J1" s="1" t="s">
+      <c r="J1" t="s">
         <v>9</v>
       </c>
-      <c r="K1" s="1" t="s">
+      <c r="K1" t="s">
         <v>10</v>
       </c>
-      <c r="L1" s="1" t="s">
+      <c r="L1" t="s">
         <v>11</v>
       </c>
-      <c r="M1" s="1" t="s">
+      <c r="M1" t="s">
         <v>12</v>
       </c>
-      <c r="N1" s="1" t="s">
+      <c r="N1" t="s">
         <v>13</v>
       </c>
-      <c r="O1" s="1" t="s">
+      <c r="O1" t="s">
         <v>14</v>
       </c>
-      <c r="P1" s="1" t="s">
+      <c r="P1" t="s">
         <v>15</v>
       </c>
-      <c r="Q1" s="1" t="s">
+      <c r="Q1" t="s">
         <v>16</v>
       </c>
-      <c r="R1" s="1" t="s">
+      <c r="R1" t="s">
         <v>17</v>
       </c>
-      <c r="S1" s="1" t="s">
+      <c r="S1" t="s">
         <v>18</v>
       </c>
-      <c r="T1" s="1" t="s">
+      <c r="T1" t="s">
         <v>19</v>
       </c>
-      <c r="U1" s="1" t="s">
+      <c r="U1" t="s">
         <v>20</v>
       </c>
-      <c r="V1" s="1" t="s">
+      <c r="V1" t="s">
         <v>21</v>
       </c>
-      <c r="W1" s="1" t="s">
+      <c r="W1" t="s">
         <v>22</v>
       </c>
     </row>
@@ -5719,7 +5693,7 @@
       <c r="J2" t="s">
         <v>1504</v>
       </c>
-      <c r="K2" s="2">
+      <c r="K2" s="1">
         <v>45730</v>
       </c>
       <c r="L2" t="s">
@@ -5763,7 +5737,7 @@
       <c r="J3" t="s">
         <v>1504</v>
       </c>
-      <c r="K3" s="2">
+      <c r="K3" s="1">
         <v>45735</v>
       </c>
       <c r="L3" t="s">
@@ -5807,7 +5781,7 @@
       <c r="J4" t="s">
         <v>1504</v>
       </c>
-      <c r="K4" s="2">
+      <c r="K4" s="1">
         <v>45737</v>
       </c>
       <c r="L4" t="s">
@@ -5825,7 +5799,7 @@
       <c r="R4" t="s">
         <v>1666</v>
       </c>
-      <c r="T4" s="2">
+      <c r="T4" s="1">
         <v>46227</v>
       </c>
       <c r="W4" t="s">
@@ -5863,7 +5837,7 @@
       <c r="J5" t="s">
         <v>1505</v>
       </c>
-      <c r="K5" s="2">
+      <c r="K5" s="1">
         <v>45747</v>
       </c>
       <c r="L5" t="s">
@@ -5913,7 +5887,7 @@
       <c r="J6" t="s">
         <v>1504</v>
       </c>
-      <c r="K6" s="2">
+      <c r="K6" s="1">
         <v>45747</v>
       </c>
       <c r="L6" t="s">
@@ -5960,7 +5934,7 @@
       <c r="J7" t="s">
         <v>1504</v>
       </c>
-      <c r="K7" s="2">
+      <c r="K7" s="1">
         <v>45747</v>
       </c>
       <c r="L7" t="s">
@@ -6007,7 +5981,7 @@
       <c r="J8" t="s">
         <v>1504</v>
       </c>
-      <c r="K8" s="2">
+      <c r="K8" s="1">
         <v>45747</v>
       </c>
       <c r="L8" t="s">
@@ -6054,7 +6028,7 @@
       <c r="J9" t="s">
         <v>1504</v>
       </c>
-      <c r="K9" s="2">
+      <c r="K9" s="1">
         <v>45747</v>
       </c>
       <c r="L9" t="s">
@@ -6101,7 +6075,7 @@
       <c r="J10" t="s">
         <v>1504</v>
       </c>
-      <c r="K10" s="2">
+      <c r="K10" s="1">
         <v>45747</v>
       </c>
       <c r="L10" t="s">
@@ -6148,7 +6122,7 @@
       <c r="J11" t="s">
         <v>1504</v>
       </c>
-      <c r="K11" s="2">
+      <c r="K11" s="1">
         <v>45747</v>
       </c>
       <c r="L11" t="s">
@@ -6195,7 +6169,7 @@
       <c r="J12" t="s">
         <v>1504</v>
       </c>
-      <c r="K12" s="2">
+      <c r="K12" s="1">
         <v>45747</v>
       </c>
       <c r="L12" t="s">
@@ -6239,7 +6213,7 @@
       <c r="J13" t="s">
         <v>1504</v>
       </c>
-      <c r="K13" s="2">
+      <c r="K13" s="1">
         <v>45762</v>
       </c>
       <c r="L13" t="s">
@@ -6257,7 +6231,7 @@
       <c r="R13" t="s">
         <v>1667</v>
       </c>
-      <c r="T13" s="2">
+      <c r="T13" s="1">
         <v>46080</v>
       </c>
       <c r="W13" t="s">
@@ -6295,7 +6269,7 @@
       <c r="J14" t="s">
         <v>1504</v>
       </c>
-      <c r="K14" s="2">
+      <c r="K14" s="1">
         <v>45763</v>
       </c>
       <c r="L14" t="s">
@@ -6313,7 +6287,7 @@
       <c r="R14" t="s">
         <v>1668</v>
       </c>
-      <c r="T14" s="2">
+      <c r="T14" s="1">
         <v>45938</v>
       </c>
       <c r="W14" t="s">
@@ -6351,7 +6325,7 @@
       <c r="J15" t="s">
         <v>1504</v>
       </c>
-      <c r="K15" s="2">
+      <c r="K15" s="1">
         <v>45763</v>
       </c>
       <c r="L15" t="s">
@@ -6369,7 +6343,7 @@
       <c r="R15" t="s">
         <v>1668</v>
       </c>
-      <c r="T15" s="2">
+      <c r="T15" s="1">
         <v>45938</v>
       </c>
       <c r="W15" t="s">
@@ -6407,7 +6381,7 @@
       <c r="J16" t="s">
         <v>1504</v>
       </c>
-      <c r="K16" s="2">
+      <c r="K16" s="1">
         <v>45783</v>
       </c>
       <c r="L16" t="s">
@@ -6451,7 +6425,7 @@
       <c r="J17" t="s">
         <v>1504</v>
       </c>
-      <c r="K17" s="2">
+      <c r="K17" s="1">
         <v>45783</v>
       </c>
       <c r="L17" t="s">
@@ -6495,7 +6469,7 @@
       <c r="J18" t="s">
         <v>1504</v>
       </c>
-      <c r="K18" s="2">
+      <c r="K18" s="1">
         <v>45784</v>
       </c>
       <c r="L18" t="s">
@@ -6513,7 +6487,7 @@
       <c r="R18" t="s">
         <v>1669</v>
       </c>
-      <c r="T18" s="2">
+      <c r="T18" s="1">
         <v>45845</v>
       </c>
       <c r="U18" t="s">
@@ -6554,7 +6528,7 @@
       <c r="J19" t="s">
         <v>1504</v>
       </c>
-      <c r="K19" s="2">
+      <c r="K19" s="1">
         <v>45784</v>
       </c>
       <c r="L19" t="s">
@@ -6598,7 +6572,7 @@
       <c r="J20" t="s">
         <v>1504</v>
       </c>
-      <c r="K20" s="2">
+      <c r="K20" s="1">
         <v>45784</v>
       </c>
       <c r="L20" t="s">
@@ -6642,7 +6616,7 @@
       <c r="J21" t="s">
         <v>1504</v>
       </c>
-      <c r="K21" s="2">
+      <c r="K21" s="1">
         <v>45784</v>
       </c>
       <c r="L21" t="s">
@@ -6660,7 +6634,7 @@
       <c r="R21" t="s">
         <v>1668</v>
       </c>
-      <c r="T21" s="2">
+      <c r="T21" s="1">
         <v>45938</v>
       </c>
       <c r="U21" t="s">
@@ -6701,7 +6675,7 @@
       <c r="J22" t="s">
         <v>1504</v>
       </c>
-      <c r="K22" s="2">
+      <c r="K22" s="1">
         <v>45789</v>
       </c>
       <c r="L22" t="s">
@@ -6719,7 +6693,7 @@
       <c r="R22" t="s">
         <v>1670</v>
       </c>
-      <c r="T22" s="2">
+      <c r="T22" s="1">
         <v>45868</v>
       </c>
       <c r="U22" t="s">
@@ -6760,7 +6734,7 @@
       <c r="J23" t="s">
         <v>1504</v>
       </c>
-      <c r="K23" s="2">
+      <c r="K23" s="1">
         <v>45789</v>
       </c>
       <c r="L23" t="s">
@@ -6778,7 +6752,7 @@
       <c r="R23" t="s">
         <v>1671</v>
       </c>
-      <c r="T23" s="2">
+      <c r="T23" s="1">
         <v>45982</v>
       </c>
       <c r="U23" t="s">
@@ -6819,7 +6793,7 @@
       <c r="J24" t="s">
         <v>1504</v>
       </c>
-      <c r="K24" s="2">
+      <c r="K24" s="1">
         <v>45791</v>
       </c>
       <c r="L24" t="s">
@@ -6863,7 +6837,7 @@
       <c r="J25" t="s">
         <v>1504</v>
       </c>
-      <c r="K25" s="2">
+      <c r="K25" s="1">
         <v>45814</v>
       </c>
       <c r="L25" t="s">
@@ -6904,7 +6878,7 @@
       <c r="J26" t="s">
         <v>1506</v>
       </c>
-      <c r="K26" s="2">
+      <c r="K26" s="1">
         <v>45819</v>
       </c>
       <c r="L26" t="s">
@@ -6922,7 +6896,7 @@
       <c r="R26" t="s">
         <v>1672</v>
       </c>
-      <c r="T26" s="2">
+      <c r="T26" s="1">
         <v>46185</v>
       </c>
       <c r="W26" t="s">
@@ -6957,7 +6931,7 @@
       <c r="J27" t="s">
         <v>1504</v>
       </c>
-      <c r="K27" s="2">
+      <c r="K27" s="1">
         <v>45821</v>
       </c>
       <c r="L27" t="s">
@@ -6975,7 +6949,7 @@
       <c r="R27" t="s">
         <v>1673</v>
       </c>
-      <c r="T27" s="2">
+      <c r="T27" s="1">
         <v>45876</v>
       </c>
       <c r="U27" t="s">
@@ -7016,7 +6990,7 @@
       <c r="J28" t="s">
         <v>1504</v>
       </c>
-      <c r="K28" s="2">
+      <c r="K28" s="1">
         <v>45824</v>
       </c>
       <c r="L28" t="s">
@@ -7060,7 +7034,7 @@
       <c r="J29" t="s">
         <v>1504</v>
       </c>
-      <c r="K29" s="2">
+      <c r="K29" s="1">
         <v>45825</v>
       </c>
       <c r="L29" t="s">
@@ -7104,7 +7078,7 @@
       <c r="J30" t="s">
         <v>1504</v>
       </c>
-      <c r="K30" s="2">
+      <c r="K30" s="1">
         <v>45836</v>
       </c>
       <c r="L30" t="s">
@@ -7148,7 +7122,7 @@
       <c r="J31" t="s">
         <v>1504</v>
       </c>
-      <c r="K31" s="2">
+      <c r="K31" s="1">
         <v>45839</v>
       </c>
       <c r="L31" t="s">
@@ -7166,7 +7140,7 @@
       <c r="R31" t="s">
         <v>1674</v>
       </c>
-      <c r="T31" s="2">
+      <c r="T31" s="1">
         <v>45912</v>
       </c>
       <c r="U31" t="s">
@@ -7207,7 +7181,7 @@
       <c r="J32" t="s">
         <v>1504</v>
       </c>
-      <c r="K32" s="2">
+      <c r="K32" s="1">
         <v>45839</v>
       </c>
       <c r="L32" t="s">
@@ -7251,7 +7225,7 @@
       <c r="J33" t="s">
         <v>1504</v>
       </c>
-      <c r="K33" s="2">
+      <c r="K33" s="1">
         <v>45845</v>
       </c>
       <c r="L33" t="s">
@@ -7269,7 +7243,7 @@
       <c r="R33" t="s">
         <v>1675</v>
       </c>
-      <c r="T33" s="2">
+      <c r="T33" s="1">
         <v>45912</v>
       </c>
       <c r="U33" t="s">
@@ -7310,7 +7284,7 @@
       <c r="J34" t="s">
         <v>1504</v>
       </c>
-      <c r="K34" s="2">
+      <c r="K34" s="1">
         <v>45856</v>
       </c>
       <c r="L34" t="s">
@@ -7354,7 +7328,7 @@
       <c r="J35" t="s">
         <v>1504</v>
       </c>
-      <c r="K35" s="2">
+      <c r="K35" s="1">
         <v>45856</v>
       </c>
       <c r="L35" t="s">
@@ -7372,7 +7346,7 @@
       <c r="R35" t="s">
         <v>1676</v>
       </c>
-      <c r="T35" s="2">
+      <c r="T35" s="1">
         <v>45912</v>
       </c>
       <c r="U35" t="s">
@@ -7413,7 +7387,7 @@
       <c r="J36" t="s">
         <v>1504</v>
       </c>
-      <c r="K36" s="2">
+      <c r="K36" s="1">
         <v>45856</v>
       </c>
       <c r="L36" t="s">
@@ -7431,7 +7405,7 @@
       <c r="R36" t="s">
         <v>1676</v>
       </c>
-      <c r="T36" s="2">
+      <c r="T36" s="1">
         <v>45912</v>
       </c>
       <c r="U36" t="s">
@@ -7472,7 +7446,7 @@
       <c r="J37" t="s">
         <v>1504</v>
       </c>
-      <c r="K37" s="2">
+      <c r="K37" s="1">
         <v>45856</v>
       </c>
       <c r="L37" t="s">
@@ -7490,7 +7464,7 @@
       <c r="R37" t="s">
         <v>1676</v>
       </c>
-      <c r="T37" s="2">
+      <c r="T37" s="1">
         <v>45912</v>
       </c>
       <c r="U37" t="s">
@@ -7531,7 +7505,7 @@
       <c r="J38" t="s">
         <v>1504</v>
       </c>
-      <c r="K38" s="2">
+      <c r="K38" s="1">
         <v>45856</v>
       </c>
       <c r="L38" t="s">
@@ -7549,7 +7523,7 @@
       <c r="R38" t="s">
         <v>1676</v>
       </c>
-      <c r="T38" s="2">
+      <c r="T38" s="1">
         <v>45912</v>
       </c>
       <c r="U38" t="s">
@@ -7590,7 +7564,7 @@
       <c r="J39" t="s">
         <v>1504</v>
       </c>
-      <c r="K39" s="2">
+      <c r="K39" s="1">
         <v>45856</v>
       </c>
       <c r="L39" t="s">
@@ -7608,7 +7582,7 @@
       <c r="R39" t="s">
         <v>1676</v>
       </c>
-      <c r="T39" s="2">
+      <c r="T39" s="1">
         <v>45912</v>
       </c>
       <c r="U39" t="s">
@@ -7649,7 +7623,7 @@
       <c r="J40" t="s">
         <v>1504</v>
       </c>
-      <c r="K40" s="2">
+      <c r="K40" s="1">
         <v>45866</v>
       </c>
       <c r="L40" t="s">
@@ -7667,7 +7641,7 @@
       <c r="R40" t="s">
         <v>1677</v>
       </c>
-      <c r="T40" s="2">
+      <c r="T40" s="1">
         <v>45916</v>
       </c>
       <c r="U40" t="s">
@@ -7708,7 +7682,7 @@
       <c r="J41" t="s">
         <v>1504</v>
       </c>
-      <c r="K41" s="2">
+      <c r="K41" s="1">
         <v>45866</v>
       </c>
       <c r="L41" t="s">
@@ -7726,7 +7700,7 @@
       <c r="R41" t="s">
         <v>1668</v>
       </c>
-      <c r="T41" s="2">
+      <c r="T41" s="1">
         <v>45938</v>
       </c>
       <c r="W41" t="s">
@@ -7764,7 +7738,7 @@
       <c r="J42" t="s">
         <v>1504</v>
       </c>
-      <c r="K42" s="2">
+      <c r="K42" s="1">
         <v>45866</v>
       </c>
       <c r="L42" t="s">
@@ -7782,7 +7756,7 @@
       <c r="R42" t="s">
         <v>1676</v>
       </c>
-      <c r="T42" s="2">
+      <c r="T42" s="1">
         <v>45912</v>
       </c>
       <c r="U42" t="s">
@@ -7823,7 +7797,7 @@
       <c r="J43" t="s">
         <v>1504</v>
       </c>
-      <c r="K43" s="2">
+      <c r="K43" s="1">
         <v>45866</v>
       </c>
       <c r="L43" t="s">
@@ -7867,7 +7841,7 @@
       <c r="J44" t="s">
         <v>1504</v>
       </c>
-      <c r="K44" s="2">
+      <c r="K44" s="1">
         <v>45866</v>
       </c>
       <c r="L44" t="s">
@@ -7885,7 +7859,7 @@
       <c r="R44" t="s">
         <v>1678</v>
       </c>
-      <c r="T44" s="2">
+      <c r="T44" s="1">
         <v>46002</v>
       </c>
       <c r="U44" t="s">
@@ -7926,7 +7900,7 @@
       <c r="J45" t="s">
         <v>1504</v>
       </c>
-      <c r="K45" s="2">
+      <c r="K45" s="1">
         <v>45882</v>
       </c>
       <c r="L45" t="s">
@@ -7944,7 +7918,7 @@
       <c r="R45" t="s">
         <v>1679</v>
       </c>
-      <c r="T45" s="2">
+      <c r="T45" s="1">
         <v>46112</v>
       </c>
       <c r="W45" t="s">
@@ -7982,7 +7956,7 @@
       <c r="J46" t="s">
         <v>1504</v>
       </c>
-      <c r="K46" s="2">
+      <c r="K46" s="1">
         <v>45882</v>
       </c>
       <c r="L46" t="s">
@@ -8026,7 +8000,7 @@
       <c r="J47" t="s">
         <v>1504</v>
       </c>
-      <c r="K47" s="2">
+      <c r="K47" s="1">
         <v>45890</v>
       </c>
       <c r="L47" t="s">
@@ -8044,7 +8018,7 @@
       <c r="R47" t="s">
         <v>1680</v>
       </c>
-      <c r="T47" s="2">
+      <c r="T47" s="1">
         <v>45944</v>
       </c>
       <c r="U47" t="s">
@@ -8085,7 +8059,7 @@
       <c r="J48" t="s">
         <v>1504</v>
       </c>
-      <c r="K48" s="2">
+      <c r="K48" s="1">
         <v>45903</v>
       </c>
       <c r="L48" t="s">
@@ -8129,7 +8103,7 @@
       <c r="J49" t="s">
         <v>1504</v>
       </c>
-      <c r="K49" s="2">
+      <c r="K49" s="1">
         <v>45904</v>
       </c>
       <c r="L49" t="s">
@@ -8173,7 +8147,7 @@
       <c r="J50" t="s">
         <v>1504</v>
       </c>
-      <c r="K50" s="2">
+      <c r="K50" s="1">
         <v>45912</v>
       </c>
       <c r="L50" t="s">
@@ -8217,7 +8191,7 @@
       <c r="J51" t="s">
         <v>1504</v>
       </c>
-      <c r="K51" s="2">
+      <c r="K51" s="1">
         <v>45925</v>
       </c>
       <c r="L51" t="s">
@@ -8264,7 +8238,7 @@
       <c r="J52" t="s">
         <v>1504</v>
       </c>
-      <c r="K52" s="2">
+      <c r="K52" s="1">
         <v>45924</v>
       </c>
       <c r="L52" t="s">
@@ -8308,7 +8282,7 @@
       <c r="J53" t="s">
         <v>1504</v>
       </c>
-      <c r="K53" s="2">
+      <c r="K53" s="1">
         <v>45930</v>
       </c>
       <c r="L53" t="s">
@@ -8352,7 +8326,7 @@
       <c r="J54" t="s">
         <v>1504</v>
       </c>
-      <c r="K54" s="2">
+      <c r="K54" s="1">
         <v>45930</v>
       </c>
       <c r="L54" t="s">
@@ -8396,7 +8370,7 @@
       <c r="J55" t="s">
         <v>1504</v>
       </c>
-      <c r="K55" s="2">
+      <c r="K55" s="1">
         <v>45931</v>
       </c>
       <c r="L55" t="s">
@@ -8446,7 +8420,7 @@
       <c r="J56" t="s">
         <v>1504</v>
       </c>
-      <c r="K56" s="2">
+      <c r="K56" s="1">
         <v>45931</v>
       </c>
       <c r="L56" t="s">
@@ -8499,7 +8473,7 @@
       <c r="J57" t="s">
         <v>1504</v>
       </c>
-      <c r="K57" s="2">
+      <c r="K57" s="1">
         <v>45931</v>
       </c>
       <c r="L57" t="s">
@@ -8549,7 +8523,7 @@
       <c r="J58" t="s">
         <v>1504</v>
       </c>
-      <c r="K58" s="2">
+      <c r="K58" s="1">
         <v>45931</v>
       </c>
       <c r="L58" t="s">
@@ -8599,7 +8573,7 @@
       <c r="J59" t="s">
         <v>1504</v>
       </c>
-      <c r="K59" s="2">
+      <c r="K59" s="1">
         <v>45937</v>
       </c>
       <c r="L59" t="s">
@@ -8617,7 +8591,7 @@
       <c r="R59" t="s">
         <v>1681</v>
       </c>
-      <c r="T59" s="2">
+      <c r="T59" s="1">
         <v>45965</v>
       </c>
       <c r="U59" t="s">
@@ -8658,7 +8632,7 @@
       <c r="J60" t="s">
         <v>1504</v>
       </c>
-      <c r="K60" s="2">
+      <c r="K60" s="1">
         <v>45938</v>
       </c>
       <c r="L60" t="s">
@@ -8702,7 +8676,7 @@
       <c r="J61" t="s">
         <v>1504</v>
       </c>
-      <c r="K61" s="2">
+      <c r="K61" s="1">
         <v>45939</v>
       </c>
       <c r="L61" t="s">
@@ -8746,7 +8720,7 @@
       <c r="J62" t="s">
         <v>1504</v>
       </c>
-      <c r="K62" s="2">
+      <c r="K62" s="1">
         <v>45939</v>
       </c>
       <c r="L62" t="s">
@@ -8790,7 +8764,7 @@
       <c r="J63" t="s">
         <v>1504</v>
       </c>
-      <c r="K63" s="2">
+      <c r="K63" s="1">
         <v>45939</v>
       </c>
       <c r="L63" t="s">
@@ -8834,7 +8808,7 @@
       <c r="J64" t="s">
         <v>1504</v>
       </c>
-      <c r="K64" s="2">
+      <c r="K64" s="1">
         <v>45940</v>
       </c>
       <c r="L64" t="s">
@@ -8878,7 +8852,7 @@
       <c r="J65" t="s">
         <v>1504</v>
       </c>
-      <c r="K65" s="2">
+      <c r="K65" s="1">
         <v>45943</v>
       </c>
       <c r="L65" t="s">
@@ -8925,7 +8899,7 @@
       <c r="J66" t="s">
         <v>1504</v>
       </c>
-      <c r="K66" s="2">
+      <c r="K66" s="1">
         <v>45943</v>
       </c>
       <c r="L66" t="s">
@@ -8943,7 +8917,7 @@
       <c r="R66" t="s">
         <v>1682</v>
       </c>
-      <c r="T66" s="2">
+      <c r="T66" s="1">
         <v>46191</v>
       </c>
       <c r="W66" t="s">
@@ -8981,7 +8955,7 @@
       <c r="J67" t="s">
         <v>1504</v>
       </c>
-      <c r="K67" s="2">
+      <c r="K67" s="1">
         <v>45943</v>
       </c>
       <c r="L67" t="s">
@@ -9025,7 +8999,7 @@
       <c r="J68" t="s">
         <v>1504</v>
       </c>
-      <c r="K68" s="2">
+      <c r="K68" s="1">
         <v>45961</v>
       </c>
       <c r="L68" t="s">
@@ -9040,7 +9014,7 @@
       <c r="O68" t="s">
         <v>1585</v>
       </c>
-      <c r="T68" s="2">
+      <c r="T68" s="1">
         <v>46176</v>
       </c>
       <c r="U68" t="s">
@@ -9084,7 +9058,7 @@
       <c r="J69" t="s">
         <v>1506</v>
       </c>
-      <c r="K69" s="2">
+      <c r="K69" s="1">
         <v>45965</v>
       </c>
       <c r="L69" t="s">
@@ -9128,7 +9102,7 @@
       <c r="J70" t="s">
         <v>1504</v>
       </c>
-      <c r="K70" s="2">
+      <c r="K70" s="1">
         <v>45965</v>
       </c>
       <c r="L70" t="s">
@@ -9172,7 +9146,7 @@
       <c r="J71" t="s">
         <v>1504</v>
       </c>
-      <c r="K71" s="2">
+      <c r="K71" s="1">
         <v>45965</v>
       </c>
       <c r="L71" t="s">
@@ -9216,7 +9190,7 @@
       <c r="J72" t="s">
         <v>1504</v>
       </c>
-      <c r="K72" s="2">
+      <c r="K72" s="1">
         <v>45967</v>
       </c>
       <c r="L72" t="s">
@@ -9260,7 +9234,7 @@
       <c r="J73" t="s">
         <v>1504</v>
       </c>
-      <c r="K73" s="2">
+      <c r="K73" s="1">
         <v>45967</v>
       </c>
       <c r="L73" t="s">
@@ -9304,7 +9278,7 @@
       <c r="J74" t="s">
         <v>1504</v>
       </c>
-      <c r="K74" s="2">
+      <c r="K74" s="1">
         <v>45967</v>
       </c>
       <c r="L74" t="s">
@@ -9348,7 +9322,7 @@
       <c r="J75" t="s">
         <v>1504</v>
       </c>
-      <c r="K75" s="2">
+      <c r="K75" s="1">
         <v>45967</v>
       </c>
       <c r="L75" t="s">
@@ -9392,7 +9366,7 @@
       <c r="J76" t="s">
         <v>1504</v>
       </c>
-      <c r="K76" s="2">
+      <c r="K76" s="1">
         <v>45968</v>
       </c>
       <c r="L76" t="s">
@@ -9410,7 +9384,7 @@
       <c r="R76" t="s">
         <v>1683</v>
       </c>
-      <c r="T76" s="2">
+      <c r="T76" s="1">
         <v>46230</v>
       </c>
       <c r="W76" t="s">
@@ -9448,7 +9422,7 @@
       <c r="J77" t="s">
         <v>1504</v>
       </c>
-      <c r="K77" s="2">
+      <c r="K77" s="1">
         <v>45968</v>
       </c>
       <c r="L77" t="s">
@@ -9466,7 +9440,7 @@
       <c r="R77" t="s">
         <v>1683</v>
       </c>
-      <c r="T77" s="2">
+      <c r="T77" s="1">
         <v>46230</v>
       </c>
       <c r="W77" t="s">
@@ -9504,7 +9478,7 @@
       <c r="J78" t="s">
         <v>1504</v>
       </c>
-      <c r="K78" s="2">
+      <c r="K78" s="1">
         <v>45968</v>
       </c>
       <c r="L78" t="s">
@@ -9522,7 +9496,7 @@
       <c r="R78" t="s">
         <v>1683</v>
       </c>
-      <c r="T78" s="2">
+      <c r="T78" s="1">
         <v>46230</v>
       </c>
       <c r="W78" t="s">
@@ -9560,7 +9534,7 @@
       <c r="J79" t="s">
         <v>1504</v>
       </c>
-      <c r="K79" s="2">
+      <c r="K79" s="1">
         <v>45968</v>
       </c>
       <c r="L79" t="s">
@@ -9578,7 +9552,7 @@
       <c r="R79" t="s">
         <v>1683</v>
       </c>
-      <c r="T79" s="2">
+      <c r="T79" s="1">
         <v>46230</v>
       </c>
       <c r="W79" t="s">
@@ -9616,7 +9590,7 @@
       <c r="J80" t="s">
         <v>1504</v>
       </c>
-      <c r="K80" s="2">
+      <c r="K80" s="1">
         <v>45968</v>
       </c>
       <c r="L80" t="s">
@@ -9660,7 +9634,7 @@
       <c r="J81" t="s">
         <v>1504</v>
       </c>
-      <c r="K81" s="2">
+      <c r="K81" s="1">
         <v>45973</v>
       </c>
       <c r="L81" t="s">
@@ -9704,7 +9678,7 @@
       <c r="J82" t="s">
         <v>1504</v>
       </c>
-      <c r="K82" s="2">
+      <c r="K82" s="1">
         <v>45974</v>
       </c>
       <c r="L82" t="s">
@@ -9748,7 +9722,7 @@
       <c r="J83" t="s">
         <v>1504</v>
       </c>
-      <c r="K83" s="2">
+      <c r="K83" s="1">
         <v>45975</v>
       </c>
       <c r="L83" t="s">
@@ -9792,7 +9766,7 @@
       <c r="J84" t="s">
         <v>1504</v>
       </c>
-      <c r="K84" s="2">
+      <c r="K84" s="1">
         <v>45975</v>
       </c>
       <c r="L84" t="s">
@@ -9836,7 +9810,7 @@
       <c r="J85" t="s">
         <v>1504</v>
       </c>
-      <c r="K85" s="2">
+      <c r="K85" s="1">
         <v>45982</v>
       </c>
       <c r="L85" t="s">
@@ -9854,7 +9828,7 @@
       <c r="R85" t="s">
         <v>1684</v>
       </c>
-      <c r="T85" s="2">
+      <c r="T85" s="1">
         <v>45989</v>
       </c>
       <c r="W85" t="s">
@@ -9892,7 +9866,7 @@
       <c r="J86" t="s">
         <v>1504</v>
       </c>
-      <c r="K86" s="2">
+      <c r="K86" s="1">
         <v>45982</v>
       </c>
       <c r="L86" t="s">
@@ -9936,7 +9910,7 @@
       <c r="J87" t="s">
         <v>1504</v>
       </c>
-      <c r="K87" s="2">
+      <c r="K87" s="1">
         <v>45985</v>
       </c>
       <c r="L87" t="s">
@@ -9954,7 +9928,7 @@
       <c r="R87" t="s">
         <v>1685</v>
       </c>
-      <c r="T87" s="2">
+      <c r="T87" s="1">
         <v>46001</v>
       </c>
       <c r="W87" t="s">
@@ -9992,7 +9966,7 @@
       <c r="J88" t="s">
         <v>1504</v>
       </c>
-      <c r="K88" s="2">
+      <c r="K88" s="1">
         <v>45985</v>
       </c>
       <c r="L88" t="s">
@@ -10036,7 +10010,7 @@
       <c r="J89" t="s">
         <v>1504</v>
       </c>
-      <c r="K89" s="2">
+      <c r="K89" s="1">
         <v>45986</v>
       </c>
       <c r="L89" t="s">
@@ -10054,7 +10028,7 @@
       <c r="R89" t="s">
         <v>1686</v>
       </c>
-      <c r="T89" s="2">
+      <c r="T89" s="1">
         <v>46006</v>
       </c>
       <c r="W89" t="s">
@@ -10089,7 +10063,7 @@
       <c r="J90" t="s">
         <v>1504</v>
       </c>
-      <c r="K90" s="2">
+      <c r="K90" s="1">
         <v>45992</v>
       </c>
       <c r="L90" t="s">
@@ -10107,7 +10081,7 @@
       <c r="R90" t="s">
         <v>1687</v>
       </c>
-      <c r="T90" s="2">
+      <c r="T90" s="1">
         <v>46007</v>
       </c>
       <c r="W90" t="s">
@@ -10142,7 +10116,7 @@
       <c r="J91" t="s">
         <v>1504</v>
       </c>
-      <c r="K91" s="2">
+      <c r="K91" s="1">
         <v>45992</v>
       </c>
       <c r="L91" t="s">
@@ -10160,7 +10134,7 @@
       <c r="R91" t="s">
         <v>1671</v>
       </c>
-      <c r="T91" s="2">
+      <c r="T91" s="1">
         <v>45979</v>
       </c>
       <c r="W91" t="s">
@@ -10198,7 +10172,7 @@
       <c r="J92" t="s">
         <v>1504</v>
       </c>
-      <c r="K92" s="2">
+      <c r="K92" s="1">
         <v>45996</v>
       </c>
       <c r="L92" t="s">
@@ -10219,7 +10193,7 @@
       <c r="R92" t="s">
         <v>1671</v>
       </c>
-      <c r="T92" s="2">
+      <c r="T92" s="1">
         <v>45979</v>
       </c>
       <c r="U92" t="s">
@@ -10260,7 +10234,7 @@
       <c r="J93" t="s">
         <v>1504</v>
       </c>
-      <c r="K93" s="2">
+      <c r="K93" s="1">
         <v>46002</v>
       </c>
       <c r="L93" t="s">
@@ -10301,7 +10275,7 @@
       <c r="J94" t="s">
         <v>1504</v>
       </c>
-      <c r="K94" s="2">
+      <c r="K94" s="1">
         <v>46007</v>
       </c>
       <c r="L94" t="s">
@@ -10345,7 +10319,7 @@
       <c r="J95" t="s">
         <v>1504</v>
       </c>
-      <c r="K95" s="2">
+      <c r="K95" s="1">
         <v>46007</v>
       </c>
       <c r="L95" t="s">
@@ -10389,7 +10363,7 @@
       <c r="J96" t="s">
         <v>1504</v>
       </c>
-      <c r="K96" s="2">
+      <c r="K96" s="1">
         <v>46008</v>
       </c>
       <c r="L96" t="s">
@@ -10407,7 +10381,7 @@
       <c r="R96" t="s">
         <v>1688</v>
       </c>
-      <c r="T96" s="2">
+      <c r="T96" s="1">
         <v>46030</v>
       </c>
       <c r="W96" t="s">
@@ -10445,7 +10419,7 @@
       <c r="J97" t="s">
         <v>1504</v>
       </c>
-      <c r="K97" s="2">
+      <c r="K97" s="1">
         <v>46029</v>
       </c>
       <c r="L97" t="s">
@@ -10460,7 +10434,7 @@
       <c r="R97" t="s">
         <v>1688</v>
       </c>
-      <c r="T97" s="2">
+      <c r="T97" s="1">
         <v>46030</v>
       </c>
       <c r="U97" t="s">
@@ -10501,7 +10475,7 @@
       <c r="J98" t="s">
         <v>1504</v>
       </c>
-      <c r="K98" s="2">
+      <c r="K98" s="1">
         <v>46029</v>
       </c>
       <c r="L98" t="s">
@@ -10519,7 +10493,7 @@
       <c r="R98" t="s">
         <v>1689</v>
       </c>
-      <c r="T98" s="2">
+      <c r="T98" s="1">
         <v>46050</v>
       </c>
       <c r="W98" t="s">
@@ -10557,7 +10531,7 @@
       <c r="J99" t="s">
         <v>1504</v>
       </c>
-      <c r="K99" s="2">
+      <c r="K99" s="1">
         <v>46034</v>
       </c>
       <c r="L99" t="s">
@@ -10575,7 +10549,7 @@
       <c r="R99" t="s">
         <v>1690</v>
       </c>
-      <c r="T99" s="2">
+      <c r="T99" s="1">
         <v>45869</v>
       </c>
       <c r="W99" t="s">
@@ -10613,7 +10587,7 @@
       <c r="J100" t="s">
         <v>1504</v>
       </c>
-      <c r="K100" s="2">
+      <c r="K100" s="1">
         <v>46034</v>
       </c>
       <c r="L100" t="s">
@@ -10654,7 +10628,7 @@
       <c r="J101" t="s">
         <v>1504</v>
       </c>
-      <c r="K101" s="2">
+      <c r="K101" s="1">
         <v>46035</v>
       </c>
       <c r="L101" t="s">
@@ -10695,7 +10669,7 @@
       <c r="J102" t="s">
         <v>1504</v>
       </c>
-      <c r="K102" s="2">
+      <c r="K102" s="1">
         <v>46036</v>
       </c>
       <c r="L102" t="s">
@@ -10736,7 +10710,7 @@
       <c r="J103" t="s">
         <v>1504</v>
       </c>
-      <c r="K103" s="2">
+      <c r="K103" s="1">
         <v>46036</v>
       </c>
       <c r="L103" t="s">
@@ -10777,7 +10751,7 @@
       <c r="J104" t="s">
         <v>1504</v>
       </c>
-      <c r="K104" s="2">
+      <c r="K104" s="1">
         <v>46036</v>
       </c>
       <c r="L104" t="s">
@@ -10818,7 +10792,7 @@
       <c r="J105" t="s">
         <v>1504</v>
       </c>
-      <c r="K105" s="2">
+      <c r="K105" s="1">
         <v>46036</v>
       </c>
       <c r="L105" t="s">
@@ -10859,7 +10833,7 @@
       <c r="J106" t="s">
         <v>1504</v>
       </c>
-      <c r="K106" s="2">
+      <c r="K106" s="1">
         <v>46036</v>
       </c>
       <c r="L106" t="s">
@@ -10900,7 +10874,7 @@
       <c r="J107" t="s">
         <v>1504</v>
       </c>
-      <c r="K107" s="2">
+      <c r="K107" s="1">
         <v>46036</v>
       </c>
       <c r="L107" t="s">
@@ -10941,7 +10915,7 @@
       <c r="J108" t="s">
         <v>1504</v>
       </c>
-      <c r="K108" s="2">
+      <c r="K108" s="1">
         <v>46043</v>
       </c>
       <c r="L108" t="s">
@@ -10982,7 +10956,7 @@
       <c r="J109" t="s">
         <v>1504</v>
       </c>
-      <c r="K109" s="2">
+      <c r="K109" s="1">
         <v>46043</v>
       </c>
       <c r="L109" t="s">
@@ -11035,7 +11009,7 @@
       <c r="J110" t="s">
         <v>1504</v>
       </c>
-      <c r="K110" s="2">
+      <c r="K110" s="1">
         <v>46043</v>
       </c>
       <c r="L110" t="s">
@@ -11091,7 +11065,7 @@
       <c r="J111" t="s">
         <v>1504</v>
       </c>
-      <c r="K111" s="2">
+      <c r="K111" s="1">
         <v>46043</v>
       </c>
       <c r="L111" t="s">
@@ -11109,7 +11083,7 @@
       <c r="R111" t="s">
         <v>1692</v>
       </c>
-      <c r="T111" s="2">
+      <c r="T111" s="1">
         <v>45959</v>
       </c>
       <c r="U111" t="s">
@@ -11147,7 +11121,7 @@
       <c r="J112" t="s">
         <v>1504</v>
       </c>
-      <c r="K112" s="2">
+      <c r="K112" s="1">
         <v>46044</v>
       </c>
       <c r="L112" t="s">
@@ -11206,7 +11180,7 @@
       <c r="J113" t="s">
         <v>1504</v>
       </c>
-      <c r="K113" s="2">
+      <c r="K113" s="1">
         <v>46049</v>
       </c>
       <c r="L113" t="s">
@@ -11250,7 +11224,7 @@
       <c r="J114" t="s">
         <v>1504</v>
       </c>
-      <c r="K114" s="2">
+      <c r="K114" s="1">
         <v>46049</v>
       </c>
       <c r="L114" t="s">
@@ -11294,7 +11268,7 @@
       <c r="J115" t="s">
         <v>1504</v>
       </c>
-      <c r="K115" s="2">
+      <c r="K115" s="1">
         <v>46050</v>
       </c>
       <c r="L115" t="s">
@@ -11312,7 +11286,7 @@
       <c r="R115" t="s">
         <v>1694</v>
       </c>
-      <c r="T115" s="2">
+      <c r="T115" s="1">
         <v>46048</v>
       </c>
       <c r="W115" t="s">
@@ -11350,7 +11324,7 @@
       <c r="J116" t="s">
         <v>1504</v>
       </c>
-      <c r="K116" s="2">
+      <c r="K116" s="1">
         <v>46050</v>
       </c>
       <c r="L116" t="s">
@@ -11409,7 +11383,7 @@
       <c r="J117" t="s">
         <v>1504</v>
       </c>
-      <c r="K117" s="2">
+      <c r="K117" s="1">
         <v>46050</v>
       </c>
       <c r="L117" t="s">
@@ -11453,7 +11427,7 @@
       <c r="J118" t="s">
         <v>1504</v>
       </c>
-      <c r="K118" s="2">
+      <c r="K118" s="1">
         <v>46063</v>
       </c>
       <c r="L118" t="s">
@@ -11500,7 +11474,7 @@
       <c r="J119" t="s">
         <v>1504</v>
       </c>
-      <c r="K119" s="2">
+      <c r="K119" s="1">
         <v>46028</v>
       </c>
       <c r="L119" t="s">
@@ -11541,7 +11515,7 @@
       <c r="J120" t="s">
         <v>1504</v>
       </c>
-      <c r="K120" s="2">
+      <c r="K120" s="1">
         <v>46062</v>
       </c>
       <c r="L120" t="s">
@@ -11585,7 +11559,7 @@
       <c r="J121" t="s">
         <v>1504</v>
       </c>
-      <c r="K121" s="2">
+      <c r="K121" s="1">
         <v>46065</v>
       </c>
       <c r="L121" t="s">
@@ -11632,7 +11606,7 @@
       <c r="J122" t="s">
         <v>1504</v>
       </c>
-      <c r="K122" s="2">
+      <c r="K122" s="1">
         <v>46065</v>
       </c>
       <c r="L122" t="s">
@@ -11682,7 +11656,7 @@
       <c r="J123" t="s">
         <v>1504</v>
       </c>
-      <c r="K123" s="2">
+      <c r="K123" s="1">
         <v>46065</v>
       </c>
       <c r="L123" t="s">
@@ -11726,7 +11700,7 @@
       <c r="J124" t="s">
         <v>1504</v>
       </c>
-      <c r="K124" s="2">
+      <c r="K124" s="1">
         <v>46065</v>
       </c>
       <c r="L124" t="s">
@@ -11770,7 +11744,7 @@
       <c r="J125" t="s">
         <v>1504</v>
       </c>
-      <c r="K125" s="2">
+      <c r="K125" s="1">
         <v>46066</v>
       </c>
       <c r="L125" t="s">
@@ -11788,7 +11762,7 @@
       <c r="R125" t="s">
         <v>1696</v>
       </c>
-      <c r="T125" s="2">
+      <c r="T125" s="1">
         <v>45800</v>
       </c>
       <c r="W125" t="s">
@@ -11823,7 +11797,7 @@
       <c r="J126" t="s">
         <v>1504</v>
       </c>
-      <c r="K126" s="2">
+      <c r="K126" s="1">
         <v>46073</v>
       </c>
       <c r="L126" t="s">
@@ -11841,7 +11815,7 @@
       <c r="R126" t="s">
         <v>1697</v>
       </c>
-      <c r="T126" s="2">
+      <c r="T126" s="1">
         <v>45889</v>
       </c>
       <c r="W126" t="s">
@@ -11876,7 +11850,7 @@
       <c r="J127" t="s">
         <v>1504</v>
       </c>
-      <c r="K127" s="2">
+      <c r="K127" s="1">
         <v>46073</v>
       </c>
       <c r="L127" t="s">
@@ -11932,7 +11906,7 @@
       <c r="J128" t="s">
         <v>1504</v>
       </c>
-      <c r="K128" s="2">
+      <c r="K128" s="1">
         <v>46073</v>
       </c>
       <c r="L128" t="s">
@@ -11973,7 +11947,7 @@
       <c r="J129" t="s">
         <v>1504</v>
       </c>
-      <c r="K129" s="2">
+      <c r="K129" s="1">
         <v>46073</v>
       </c>
       <c r="L129" t="s">
@@ -12014,7 +11988,7 @@
       <c r="J130" t="s">
         <v>1504</v>
       </c>
-      <c r="K130" s="2">
+      <c r="K130" s="1">
         <v>46073</v>
       </c>
       <c r="L130" t="s">
@@ -12055,7 +12029,7 @@
       <c r="J131" t="s">
         <v>1504</v>
       </c>
-      <c r="K131" s="2">
+      <c r="K131" s="1">
         <v>46073</v>
       </c>
       <c r="L131" t="s">
@@ -12099,7 +12073,7 @@
       <c r="J132" t="s">
         <v>1504</v>
       </c>
-      <c r="K132" s="2">
+      <c r="K132" s="1">
         <v>46077</v>
       </c>
       <c r="L132" t="s">
@@ -12140,7 +12114,7 @@
       <c r="J133" t="s">
         <v>1504</v>
       </c>
-      <c r="K133" s="2">
+      <c r="K133" s="1">
         <v>46079</v>
       </c>
       <c r="L133" t="s">
@@ -12158,7 +12132,7 @@
       <c r="R133" t="s">
         <v>1683</v>
       </c>
-      <c r="T133" s="2">
+      <c r="T133" s="1">
         <v>46230</v>
       </c>
       <c r="W133" t="s">
@@ -12193,7 +12167,7 @@
       <c r="J134" t="s">
         <v>1504</v>
       </c>
-      <c r="K134" s="2">
+      <c r="K134" s="1">
         <v>46080</v>
       </c>
       <c r="L134" t="s">
@@ -12211,7 +12185,7 @@
       <c r="R134" t="s">
         <v>1683</v>
       </c>
-      <c r="T134" s="2">
+      <c r="T134" s="1">
         <v>46230</v>
       </c>
       <c r="W134" t="s">
@@ -12246,7 +12220,7 @@
       <c r="J135" t="s">
         <v>1504</v>
       </c>
-      <c r="K135" s="2">
+      <c r="K135" s="1">
         <v>46080</v>
       </c>
       <c r="L135" t="s">
@@ -12287,7 +12261,7 @@
       <c r="J136" t="s">
         <v>1504</v>
       </c>
-      <c r="K136" s="2">
+      <c r="K136" s="1">
         <v>46080</v>
       </c>
       <c r="L136" t="s">
@@ -12328,7 +12302,7 @@
       <c r="J137" t="s">
         <v>1504</v>
       </c>
-      <c r="K137" s="2">
+      <c r="K137" s="1">
         <v>46080</v>
       </c>
       <c r="L137" t="s">
@@ -12369,7 +12343,7 @@
       <c r="J138" t="s">
         <v>1504</v>
       </c>
-      <c r="K138" s="2">
+      <c r="K138" s="1">
         <v>46080</v>
       </c>
       <c r="L138" t="s">
@@ -12410,7 +12384,7 @@
       <c r="J139" t="s">
         <v>1504</v>
       </c>
-      <c r="K139" s="2">
+      <c r="K139" s="1">
         <v>46078</v>
       </c>
       <c r="L139" t="s">
@@ -12457,7 +12431,7 @@
       <c r="J140" t="s">
         <v>1504</v>
       </c>
-      <c r="K140" s="2">
+      <c r="K140" s="1">
         <v>46092</v>
       </c>
       <c r="L140" t="s">
@@ -12498,7 +12472,7 @@
       <c r="J141" t="s">
         <v>1504</v>
       </c>
-      <c r="K141" s="2">
+      <c r="K141" s="1">
         <v>46092</v>
       </c>
       <c r="L141" t="s">
@@ -12539,7 +12513,7 @@
       <c r="J142" t="s">
         <v>1504</v>
       </c>
-      <c r="K142" s="2">
+      <c r="K142" s="1">
         <v>46092</v>
       </c>
       <c r="L142" t="s">
@@ -12583,7 +12557,7 @@
       <c r="J143" t="s">
         <v>1504</v>
       </c>
-      <c r="K143" s="2">
+      <c r="K143" s="1">
         <v>46092</v>
       </c>
       <c r="L143" t="s">
@@ -12601,7 +12575,7 @@
       <c r="R143" t="s">
         <v>1683</v>
       </c>
-      <c r="T143" s="2">
+      <c r="T143" s="1">
         <v>46230</v>
       </c>
       <c r="W143" t="s">
@@ -12636,7 +12610,7 @@
       <c r="J144" t="s">
         <v>1504</v>
       </c>
-      <c r="K144" s="2">
+      <c r="K144" s="1">
         <v>46090</v>
       </c>
       <c r="L144" t="s">
@@ -12654,7 +12628,7 @@
       <c r="R144" t="s">
         <v>1683</v>
       </c>
-      <c r="T144" s="2">
+      <c r="T144" s="1">
         <v>46230</v>
       </c>
       <c r="W144" t="s">
@@ -12689,7 +12663,7 @@
       <c r="J145" t="s">
         <v>1504</v>
       </c>
-      <c r="K145" s="2">
+      <c r="K145" s="1">
         <v>46094</v>
       </c>
       <c r="L145" t="s">
@@ -12707,7 +12681,7 @@
       <c r="R145" t="s">
         <v>1683</v>
       </c>
-      <c r="T145" s="2">
+      <c r="T145" s="1">
         <v>46230</v>
       </c>
       <c r="W145" t="s">
@@ -12742,7 +12716,7 @@
       <c r="J146" t="s">
         <v>1504</v>
       </c>
-      <c r="K146" s="2">
+      <c r="K146" s="1">
         <v>46094</v>
       </c>
       <c r="L146" t="s">
@@ -12760,7 +12734,7 @@
       <c r="R146" t="s">
         <v>1691</v>
       </c>
-      <c r="T146" s="2">
+      <c r="T146" s="1">
         <v>45805</v>
       </c>
       <c r="W146" t="s">
@@ -12795,7 +12769,7 @@
       <c r="J147" t="s">
         <v>1504</v>
       </c>
-      <c r="K147" s="2">
+      <c r="K147" s="1">
         <v>46094</v>
       </c>
       <c r="L147" t="s">
@@ -12813,7 +12787,7 @@
       <c r="R147" t="s">
         <v>1698</v>
       </c>
-      <c r="T147" s="2">
+      <c r="T147" s="1">
         <v>45971</v>
       </c>
       <c r="W147" t="s">
@@ -12848,7 +12822,7 @@
       <c r="J148" t="s">
         <v>1504</v>
       </c>
-      <c r="K148" s="2">
+      <c r="K148" s="1">
         <v>46097</v>
       </c>
       <c r="L148" t="s">
@@ -12889,7 +12863,7 @@
       <c r="J149" t="s">
         <v>1504</v>
       </c>
-      <c r="K149" s="2">
+      <c r="K149" s="1">
         <v>46097</v>
       </c>
       <c r="L149" t="s">
@@ -12907,7 +12881,7 @@
       <c r="R149" t="s">
         <v>1683</v>
       </c>
-      <c r="T149" s="2">
+      <c r="T149" s="1">
         <v>46230</v>
       </c>
       <c r="W149" t="s">
@@ -12942,7 +12916,7 @@
       <c r="J150" t="s">
         <v>1504</v>
       </c>
-      <c r="K150" s="2">
+      <c r="K150" s="1">
         <v>46098</v>
       </c>
       <c r="L150" t="s">
@@ -12960,7 +12934,7 @@
       <c r="R150" t="s">
         <v>1683</v>
       </c>
-      <c r="T150" s="2">
+      <c r="T150" s="1">
         <v>46230</v>
       </c>
       <c r="W150" t="s">
@@ -12995,7 +12969,7 @@
       <c r="J151" t="s">
         <v>1504</v>
       </c>
-      <c r="K151" s="2">
+      <c r="K151" s="1">
         <v>46100</v>
       </c>
       <c r="L151" t="s">
@@ -13013,7 +12987,7 @@
       <c r="R151" t="s">
         <v>1699</v>
       </c>
-      <c r="T151" s="2">
+      <c r="T151" s="1">
         <v>46176</v>
       </c>
       <c r="W151" t="s">
@@ -13048,7 +13022,7 @@
       <c r="J152" t="s">
         <v>1504</v>
       </c>
-      <c r="K152" s="2">
+      <c r="K152" s="1">
         <v>46100</v>
       </c>
       <c r="L152" t="s">
@@ -13066,7 +13040,7 @@
       <c r="R152" t="s">
         <v>1700</v>
       </c>
-      <c r="T152" s="2">
+      <c r="T152" s="1">
         <v>45769</v>
       </c>
       <c r="W152" t="s">
@@ -13101,7 +13075,7 @@
       <c r="J153" t="s">
         <v>1504</v>
       </c>
-      <c r="K153" s="2">
+      <c r="K153" s="1">
         <v>46100</v>
       </c>
       <c r="L153" t="s">
@@ -13110,7 +13084,7 @@
       <c r="M153" t="s">
         <v>1576</v>
       </c>
-      <c r="T153" s="2">
+      <c r="T153" s="1">
         <v>46176</v>
       </c>
       <c r="U153" t="s">
@@ -13151,7 +13125,7 @@
       <c r="J154" t="s">
         <v>1504</v>
       </c>
-      <c r="K154" s="2">
+      <c r="K154" s="1">
         <v>46101</v>
       </c>
       <c r="L154" t="s">
@@ -13192,7 +13166,7 @@
       <c r="J155" t="s">
         <v>1504</v>
       </c>
-      <c r="K155" s="2">
+      <c r="K155" s="1">
         <v>46101</v>
       </c>
       <c r="L155" t="s">
@@ -13233,7 +13207,7 @@
       <c r="J156" t="s">
         <v>1504</v>
       </c>
-      <c r="K156" s="2">
+      <c r="K156" s="1">
         <v>46101</v>
       </c>
       <c r="L156" t="s">
@@ -13274,7 +13248,7 @@
       <c r="J157" t="s">
         <v>1504</v>
       </c>
-      <c r="K157" s="2">
+      <c r="K157" s="1">
         <v>46101</v>
       </c>
       <c r="L157" t="s">
@@ -13315,7 +13289,7 @@
       <c r="J158" t="s">
         <v>1504</v>
       </c>
-      <c r="K158" s="2">
+      <c r="K158" s="1">
         <v>46101</v>
       </c>
       <c r="L158" t="s">
@@ -13356,7 +13330,7 @@
       <c r="J159" t="s">
         <v>1504</v>
       </c>
-      <c r="K159" s="2">
+      <c r="K159" s="1">
         <v>46101</v>
       </c>
       <c r="L159" t="s">
@@ -13397,7 +13371,7 @@
       <c r="J160" t="s">
         <v>1504</v>
       </c>
-      <c r="K160" s="2">
+      <c r="K160" s="1">
         <v>46101</v>
       </c>
       <c r="L160" t="s">
@@ -13438,7 +13412,7 @@
       <c r="J161" t="s">
         <v>1504</v>
       </c>
-      <c r="K161" s="2">
+      <c r="K161" s="1">
         <v>46101</v>
       </c>
       <c r="L161" t="s">
@@ -13479,7 +13453,7 @@
       <c r="J162" t="s">
         <v>1504</v>
       </c>
-      <c r="K162" s="2">
+      <c r="K162" s="1">
         <v>46113</v>
       </c>
       <c r="L162" t="s">
@@ -13497,7 +13471,7 @@
       <c r="R162" t="s">
         <v>1686</v>
       </c>
-      <c r="T162" s="2">
+      <c r="T162" s="1">
         <v>46006</v>
       </c>
       <c r="W162" t="s">
@@ -13532,7 +13506,7 @@
       <c r="J163" t="s">
         <v>1504</v>
       </c>
-      <c r="K163" s="2">
+      <c r="K163" s="1">
         <v>46119</v>
       </c>
       <c r="L163" t="s">
@@ -13550,7 +13524,7 @@
       <c r="R163" t="s">
         <v>1683</v>
       </c>
-      <c r="T163" s="2">
+      <c r="T163" s="1">
         <v>46230</v>
       </c>
       <c r="W163" t="s">
@@ -13585,7 +13559,7 @@
       <c r="J164" t="s">
         <v>1504</v>
       </c>
-      <c r="K164" s="2">
+      <c r="K164" s="1">
         <v>46119</v>
       </c>
       <c r="L164" t="s">
@@ -13629,7 +13603,7 @@
       <c r="J165" t="s">
         <v>1504</v>
       </c>
-      <c r="K165" s="2">
+      <c r="K165" s="1">
         <v>46119</v>
       </c>
       <c r="L165" t="s">
@@ -13670,7 +13644,7 @@
       <c r="J166" t="s">
         <v>1504</v>
       </c>
-      <c r="K166" s="2">
+      <c r="K166" s="1">
         <v>46119</v>
       </c>
       <c r="L166" t="s">
@@ -13688,7 +13662,7 @@
       <c r="R166" t="s">
         <v>1701</v>
       </c>
-      <c r="T166" s="2">
+      <c r="T166" s="1">
         <v>45817</v>
       </c>
       <c r="W166" t="s">
@@ -13723,7 +13697,7 @@
       <c r="J167" t="s">
         <v>1504</v>
       </c>
-      <c r="K167" s="2">
+      <c r="K167" s="1">
         <v>46119</v>
       </c>
       <c r="L167" t="s">
@@ -13767,7 +13741,7 @@
       <c r="J168" t="s">
         <v>1504</v>
       </c>
-      <c r="K168" s="2">
+      <c r="K168" s="1">
         <v>46120</v>
       </c>
       <c r="L168" t="s">
@@ -13811,7 +13785,7 @@
       <c r="J169" t="s">
         <v>1504</v>
       </c>
-      <c r="K169" s="2">
+      <c r="K169" s="1">
         <v>46120</v>
       </c>
       <c r="L169" t="s">
@@ -13852,7 +13826,7 @@
       <c r="J170" t="s">
         <v>1504</v>
       </c>
-      <c r="K170" s="2">
+      <c r="K170" s="1">
         <v>46120</v>
       </c>
       <c r="L170" t="s">
@@ -13893,7 +13867,7 @@
       <c r="J171" t="s">
         <v>1504</v>
       </c>
-      <c r="K171" s="2">
+      <c r="K171" s="1">
         <v>46120</v>
       </c>
       <c r="L171" t="s">
@@ -13934,7 +13908,7 @@
       <c r="J172" t="s">
         <v>1504</v>
       </c>
-      <c r="K172" s="2">
+      <c r="K172" s="1">
         <v>46120</v>
       </c>
       <c r="L172" t="s">
@@ -13975,7 +13949,7 @@
       <c r="J173" t="s">
         <v>1504</v>
       </c>
-      <c r="K173" s="2">
+      <c r="K173" s="1">
         <v>46120</v>
       </c>
       <c r="L173" t="s">
@@ -14016,7 +13990,7 @@
       <c r="J174" t="s">
         <v>1504</v>
       </c>
-      <c r="K174" s="2">
+      <c r="K174" s="1">
         <v>46120</v>
       </c>
       <c r="L174" t="s">
@@ -14057,7 +14031,7 @@
       <c r="J175" t="s">
         <v>1504</v>
       </c>
-      <c r="K175" s="2">
+      <c r="K175" s="1">
         <v>46120</v>
       </c>
       <c r="L175" t="s">
@@ -14098,7 +14072,7 @@
       <c r="J176" t="s">
         <v>1504</v>
       </c>
-      <c r="K176" s="2">
+      <c r="K176" s="1">
         <v>46120</v>
       </c>
       <c r="L176" t="s">
@@ -14139,7 +14113,7 @@
       <c r="J177" t="s">
         <v>1504</v>
       </c>
-      <c r="K177" s="2">
+      <c r="K177" s="1">
         <v>46120</v>
       </c>
       <c r="L177" t="s">
@@ -14180,7 +14154,7 @@
       <c r="J178" t="s">
         <v>1504</v>
       </c>
-      <c r="K178" s="2">
+      <c r="K178" s="1">
         <v>46120</v>
       </c>
       <c r="L178" t="s">
@@ -14198,7 +14172,7 @@
       <c r="R178" t="s">
         <v>1699</v>
       </c>
-      <c r="T178" s="2">
+      <c r="T178" s="1">
         <v>46176</v>
       </c>
       <c r="W178" t="s">
@@ -14233,7 +14207,7 @@
       <c r="J179" t="s">
         <v>1504</v>
       </c>
-      <c r="K179" s="2">
+      <c r="K179" s="1">
         <v>46121</v>
       </c>
       <c r="L179" t="s">
@@ -14242,7 +14216,7 @@
       <c r="M179" t="s">
         <v>1573</v>
       </c>
-      <c r="T179" s="2">
+      <c r="T179" s="1">
         <v>46176</v>
       </c>
       <c r="U179" t="s">
@@ -14283,7 +14257,7 @@
       <c r="J180" t="s">
         <v>1504</v>
       </c>
-      <c r="K180" s="2">
+      <c r="K180" s="1">
         <v>46121</v>
       </c>
       <c r="L180" t="s">
@@ -14324,7 +14298,7 @@
       <c r="J181" t="s">
         <v>1504</v>
       </c>
-      <c r="K181" s="2">
+      <c r="K181" s="1">
         <v>46121</v>
       </c>
       <c r="L181" t="s">
@@ -14342,7 +14316,7 @@
       <c r="R181" t="s">
         <v>1683</v>
       </c>
-      <c r="T181" s="2">
+      <c r="T181" s="1">
         <v>46230</v>
       </c>
       <c r="W181" t="s">
@@ -14377,7 +14351,7 @@
       <c r="J182" t="s">
         <v>1504</v>
       </c>
-      <c r="K182" s="2">
+      <c r="K182" s="1">
         <v>46121</v>
       </c>
       <c r="L182" t="s">
@@ -14418,7 +14392,7 @@
       <c r="J183" t="s">
         <v>1504</v>
       </c>
-      <c r="K183" s="2">
+      <c r="K183" s="1">
         <v>46121</v>
       </c>
       <c r="L183" t="s">
@@ -14459,7 +14433,7 @@
       <c r="J184" t="s">
         <v>1504</v>
       </c>
-      <c r="K184" s="2">
+      <c r="K184" s="1">
         <v>46122</v>
       </c>
       <c r="L184" t="s">
@@ -14500,7 +14474,7 @@
       <c r="J185" t="s">
         <v>1504</v>
       </c>
-      <c r="K185" s="2">
+      <c r="K185" s="1">
         <v>46122</v>
       </c>
       <c r="L185" t="s">
@@ -14541,7 +14515,7 @@
       <c r="J186" t="s">
         <v>1504</v>
       </c>
-      <c r="K186" s="2">
+      <c r="K186" s="1">
         <v>46122</v>
       </c>
       <c r="L186" t="s">
@@ -14582,7 +14556,7 @@
       <c r="J187" t="s">
         <v>1504</v>
       </c>
-      <c r="K187" s="2">
+      <c r="K187" s="1">
         <v>46122</v>
       </c>
       <c r="L187" t="s">
@@ -14623,7 +14597,7 @@
       <c r="J188" t="s">
         <v>1504</v>
       </c>
-      <c r="K188" s="2">
+      <c r="K188" s="1">
         <v>46122</v>
       </c>
       <c r="L188" t="s">
@@ -14664,7 +14638,7 @@
       <c r="J189" t="s">
         <v>1504</v>
       </c>
-      <c r="K189" s="2">
+      <c r="K189" s="1">
         <v>46122</v>
       </c>
       <c r="L189" t="s">
@@ -14705,7 +14679,7 @@
       <c r="J190" t="s">
         <v>1504</v>
       </c>
-      <c r="K190" s="2">
+      <c r="K190" s="1">
         <v>46122</v>
       </c>
       <c r="L190" t="s">
@@ -14746,7 +14720,7 @@
       <c r="J191" t="s">
         <v>1504</v>
       </c>
-      <c r="K191" s="2">
+      <c r="K191" s="1">
         <v>46122</v>
       </c>
       <c r="L191" t="s">
@@ -14787,7 +14761,7 @@
       <c r="J192" t="s">
         <v>1504</v>
       </c>
-      <c r="K192" s="2">
+      <c r="K192" s="1">
         <v>46122</v>
       </c>
       <c r="L192" t="s">
@@ -14828,7 +14802,7 @@
       <c r="J193" t="s">
         <v>1504</v>
       </c>
-      <c r="K193" s="2">
+      <c r="K193" s="1">
         <v>46122</v>
       </c>
       <c r="L193" t="s">
@@ -14869,7 +14843,7 @@
       <c r="J194" t="s">
         <v>1504</v>
       </c>
-      <c r="K194" s="2">
+      <c r="K194" s="1">
         <v>46122</v>
       </c>
       <c r="L194" t="s">
@@ -14910,7 +14884,7 @@
       <c r="J195" t="s">
         <v>1504</v>
       </c>
-      <c r="K195" s="2">
+      <c r="K195" s="1">
         <v>46126</v>
       </c>
       <c r="L195" t="s">
@@ -14928,7 +14902,7 @@
       <c r="R195" t="s">
         <v>1692</v>
       </c>
-      <c r="T195" s="2">
+      <c r="T195" s="1">
         <v>45959</v>
       </c>
       <c r="W195" t="s">
@@ -14966,7 +14940,7 @@
       <c r="J196" t="s">
         <v>1504</v>
       </c>
-      <c r="K196" s="2">
+      <c r="K196" s="1">
         <v>46128</v>
       </c>
       <c r="L196" t="s">
@@ -14984,7 +14958,7 @@
       <c r="R196" t="s">
         <v>1698</v>
       </c>
-      <c r="T196" s="2">
+      <c r="T196" s="1">
         <v>45971</v>
       </c>
       <c r="W196" t="s">
@@ -15022,7 +14996,7 @@
       <c r="J197" t="s">
         <v>1504</v>
       </c>
-      <c r="K197" s="2">
+      <c r="K197" s="1">
         <v>46128</v>
       </c>
       <c r="L197" t="s">
@@ -15063,7 +15037,7 @@
       <c r="J198" t="s">
         <v>1506</v>
       </c>
-      <c r="K198" s="2">
+      <c r="K198" s="1">
         <v>46128</v>
       </c>
       <c r="L198" t="s">
@@ -15104,7 +15078,7 @@
       <c r="J199" t="s">
         <v>1505</v>
       </c>
-      <c r="K199" s="2">
+      <c r="K199" s="1">
         <v>46129</v>
       </c>
       <c r="L199" t="s">
@@ -15145,7 +15119,7 @@
       <c r="J200" t="s">
         <v>1504</v>
       </c>
-      <c r="K200" s="2">
+      <c r="K200" s="1">
         <v>46135</v>
       </c>
       <c r="L200" t="s">
@@ -15186,7 +15160,7 @@
       <c r="J201" t="s">
         <v>1504</v>
       </c>
-      <c r="K201" s="2">
+      <c r="K201" s="1">
         <v>46139</v>
       </c>
       <c r="L201" t="s">
@@ -15227,7 +15201,7 @@
       <c r="J202" t="s">
         <v>1504</v>
       </c>
-      <c r="K202" s="2">
+      <c r="K202" s="1">
         <v>46139</v>
       </c>
       <c r="L202" t="s">
@@ -15245,7 +15219,7 @@
       <c r="R202" t="s">
         <v>1683</v>
       </c>
-      <c r="T202" s="2">
+      <c r="T202" s="1">
         <v>46230</v>
       </c>
       <c r="W202" t="s">
@@ -15280,7 +15254,7 @@
       <c r="J203" t="s">
         <v>1504</v>
       </c>
-      <c r="K203" s="2">
+      <c r="K203" s="1">
         <v>46139</v>
       </c>
       <c r="L203" t="s">
@@ -15298,7 +15272,7 @@
       <c r="R203" t="s">
         <v>1691</v>
       </c>
-      <c r="T203" s="2">
+      <c r="T203" s="1">
         <v>45805</v>
       </c>
       <c r="W203" t="s">
@@ -15333,7 +15307,7 @@
       <c r="J204" t="s">
         <v>1504</v>
       </c>
-      <c r="K204" s="2">
+      <c r="K204" s="1">
         <v>46139</v>
       </c>
       <c r="L204" t="s">
@@ -15348,7 +15322,7 @@
       <c r="R204" t="s">
         <v>1702</v>
       </c>
-      <c r="T204" s="2">
+      <c r="T204" s="1">
         <v>45889</v>
       </c>
       <c r="W204" t="s">
@@ -15386,7 +15360,7 @@
       <c r="J205" t="s">
         <v>1504</v>
       </c>
-      <c r="K205" s="2">
+      <c r="K205" s="1">
         <v>46139</v>
       </c>
       <c r="L205" t="s">
@@ -15404,7 +15378,7 @@
       <c r="R205" t="s">
         <v>1703</v>
       </c>
-      <c r="T205" s="2">
+      <c r="T205" s="1">
         <v>45762</v>
       </c>
       <c r="W205" t="s">
@@ -15442,7 +15416,7 @@
       <c r="J206" t="s">
         <v>1504</v>
       </c>
-      <c r="K206" s="2">
+      <c r="K206" s="1">
         <v>46141</v>
       </c>
       <c r="L206" t="s">
@@ -15460,7 +15434,7 @@
       <c r="R206" t="s">
         <v>1671</v>
       </c>
-      <c r="T206" s="2">
+      <c r="T206" s="1">
         <v>45979</v>
       </c>
       <c r="W206" t="s">
@@ -15495,7 +15469,7 @@
       <c r="J207" t="s">
         <v>1504</v>
       </c>
-      <c r="K207" s="2">
+      <c r="K207" s="1">
         <v>46141</v>
       </c>
       <c r="L207" t="s">
@@ -15536,7 +15510,7 @@
       <c r="J208" t="s">
         <v>1504</v>
       </c>
-      <c r="K208" s="2">
+      <c r="K208" s="1">
         <v>46141</v>
       </c>
       <c r="L208" t="s">
@@ -15577,7 +15551,7 @@
       <c r="J209" t="s">
         <v>1504</v>
       </c>
-      <c r="K209" s="2">
+      <c r="K209" s="1">
         <v>46141</v>
       </c>
       <c r="L209" t="s">
@@ -15618,7 +15592,7 @@
       <c r="J210" t="s">
         <v>1504</v>
       </c>
-      <c r="K210" s="2">
+      <c r="K210" s="1">
         <v>46141</v>
       </c>
       <c r="L210" t="s">
@@ -15659,7 +15633,7 @@
       <c r="J211" t="s">
         <v>1504</v>
       </c>
-      <c r="K211" s="2">
+      <c r="K211" s="1">
         <v>46141</v>
       </c>
       <c r="L211" t="s">
@@ -15700,7 +15674,7 @@
       <c r="J212" t="s">
         <v>1504</v>
       </c>
-      <c r="K212" s="2">
+      <c r="K212" s="1">
         <v>46141</v>
       </c>
       <c r="L212" t="s">
@@ -15741,7 +15715,7 @@
       <c r="J213" t="s">
         <v>1504</v>
       </c>
-      <c r="K213" s="2">
+      <c r="K213" s="1">
         <v>46141</v>
       </c>
       <c r="L213" t="s">
@@ -15782,7 +15756,7 @@
       <c r="J214" t="s">
         <v>1504</v>
       </c>
-      <c r="K214" s="2">
+      <c r="K214" s="1">
         <v>46141</v>
       </c>
       <c r="L214" t="s">
@@ -15800,7 +15774,7 @@
       <c r="R214" t="s">
         <v>1704</v>
       </c>
-      <c r="T214" s="2">
+      <c r="T214" s="1">
         <v>46216</v>
       </c>
       <c r="W214" t="s">
@@ -15835,7 +15809,7 @@
       <c r="J215" t="s">
         <v>1504</v>
       </c>
-      <c r="K215" s="2">
+      <c r="K215" s="1">
         <v>46142</v>
       </c>
       <c r="L215" t="s">
@@ -15876,7 +15850,7 @@
       <c r="J216" t="s">
         <v>1504</v>
       </c>
-      <c r="K216" s="2">
+      <c r="K216" s="1">
         <v>46146</v>
       </c>
       <c r="L216" t="s">
@@ -15917,7 +15891,7 @@
       <c r="J217" t="s">
         <v>1504</v>
       </c>
-      <c r="K217" s="2">
+      <c r="K217" s="1">
         <v>46148</v>
       </c>
       <c r="L217" t="s">
@@ -15958,7 +15932,7 @@
       <c r="J218" t="s">
         <v>1504</v>
       </c>
-      <c r="K218" s="2">
+      <c r="K218" s="1">
         <v>46148</v>
       </c>
       <c r="L218" t="s">
@@ -15999,7 +15973,7 @@
       <c r="J219" t="s">
         <v>1504</v>
       </c>
-      <c r="K219" s="2">
+      <c r="K219" s="1">
         <v>46148</v>
       </c>
       <c r="L219" t="s">
@@ -16040,7 +16014,7 @@
       <c r="J220" t="s">
         <v>1504</v>
       </c>
-      <c r="K220" s="2">
+      <c r="K220" s="1">
         <v>46148</v>
       </c>
       <c r="L220" t="s">
@@ -16081,7 +16055,7 @@
       <c r="J221" t="s">
         <v>1504</v>
       </c>
-      <c r="K221" s="2">
+      <c r="K221" s="1">
         <v>46148</v>
       </c>
       <c r="L221" t="s">
@@ -16122,7 +16096,7 @@
       <c r="J222" t="s">
         <v>1504</v>
       </c>
-      <c r="K222" s="2">
+      <c r="K222" s="1">
         <v>46148</v>
       </c>
       <c r="L222" t="s">
@@ -16163,7 +16137,7 @@
       <c r="J223" t="s">
         <v>1504</v>
       </c>
-      <c r="K223" s="2">
+      <c r="K223" s="1">
         <v>46148</v>
       </c>
       <c r="L223" t="s">
@@ -16204,7 +16178,7 @@
       <c r="J224" t="s">
         <v>1504</v>
       </c>
-      <c r="K224" s="2">
+      <c r="K224" s="1">
         <v>46148</v>
       </c>
       <c r="L224" t="s">
@@ -16245,7 +16219,7 @@
       <c r="J225" t="s">
         <v>1504</v>
       </c>
-      <c r="K225" s="2">
+      <c r="K225" s="1">
         <v>46148</v>
       </c>
       <c r="L225" t="s">
@@ -16286,7 +16260,7 @@
       <c r="J226" t="s">
         <v>1504</v>
       </c>
-      <c r="K226" s="2">
+      <c r="K226" s="1">
         <v>46148</v>
       </c>
       <c r="L226" t="s">
@@ -16327,7 +16301,7 @@
       <c r="J227" t="s">
         <v>1504</v>
       </c>
-      <c r="K227" s="2">
+      <c r="K227" s="1">
         <v>46148</v>
       </c>
       <c r="L227" t="s">
@@ -16368,7 +16342,7 @@
       <c r="J228" t="s">
         <v>1504</v>
       </c>
-      <c r="K228" s="2">
+      <c r="K228" s="1">
         <v>46148</v>
       </c>
       <c r="L228" t="s">
@@ -16409,7 +16383,7 @@
       <c r="J229" t="s">
         <v>1504</v>
       </c>
-      <c r="K229" s="2">
+      <c r="K229" s="1">
         <v>46148</v>
       </c>
       <c r="L229" t="s">
@@ -16450,7 +16424,7 @@
       <c r="J230" t="s">
         <v>1504</v>
       </c>
-      <c r="K230" s="2">
+      <c r="K230" s="1">
         <v>46148</v>
       </c>
       <c r="L230" t="s">
@@ -16491,7 +16465,7 @@
       <c r="J231" t="s">
         <v>1504</v>
       </c>
-      <c r="K231" s="2">
+      <c r="K231" s="1">
         <v>46148</v>
       </c>
       <c r="L231" t="s">
@@ -16532,7 +16506,7 @@
       <c r="J232" t="s">
         <v>1504</v>
       </c>
-      <c r="K232" s="2">
+      <c r="K232" s="1">
         <v>46148</v>
       </c>
       <c r="L232" t="s">
@@ -16573,7 +16547,7 @@
       <c r="J233" t="s">
         <v>1504</v>
       </c>
-      <c r="K233" s="2">
+      <c r="K233" s="1">
         <v>46148</v>
       </c>
       <c r="L233" t="s">
@@ -16614,7 +16588,7 @@
       <c r="J234" t="s">
         <v>1504</v>
       </c>
-      <c r="K234" s="2">
+      <c r="K234" s="1">
         <v>46149</v>
       </c>
       <c r="L234" t="s">
@@ -16655,7 +16629,7 @@
       <c r="J235" t="s">
         <v>1504</v>
       </c>
-      <c r="K235" s="2">
+      <c r="K235" s="1">
         <v>46149</v>
       </c>
       <c r="L235" t="s">
@@ -16696,7 +16670,7 @@
       <c r="J236" t="s">
         <v>1504</v>
       </c>
-      <c r="K236" s="2">
+      <c r="K236" s="1">
         <v>46149</v>
       </c>
       <c r="L236" t="s">
@@ -16737,7 +16711,7 @@
       <c r="J237" t="s">
         <v>1504</v>
       </c>
-      <c r="K237" s="2">
+      <c r="K237" s="1">
         <v>46149</v>
       </c>
       <c r="L237" t="s">
@@ -16778,7 +16752,7 @@
       <c r="J238" t="s">
         <v>1504</v>
       </c>
-      <c r="K238" s="2">
+      <c r="K238" s="1">
         <v>46149</v>
       </c>
       <c r="L238" t="s">
@@ -16819,7 +16793,7 @@
       <c r="J239" t="s">
         <v>1504</v>
       </c>
-      <c r="K239" s="2">
+      <c r="K239" s="1">
         <v>46149</v>
       </c>
       <c r="L239" t="s">
@@ -16837,7 +16811,7 @@
       <c r="R239" t="s">
         <v>1698</v>
       </c>
-      <c r="T239" s="2">
+      <c r="T239" s="1">
         <v>45971</v>
       </c>
       <c r="W239" t="s">
@@ -16872,7 +16846,7 @@
       <c r="J240" t="s">
         <v>1504</v>
       </c>
-      <c r="K240" s="2">
+      <c r="K240" s="1">
         <v>46149</v>
       </c>
       <c r="L240" t="s">
@@ -16913,7 +16887,7 @@
       <c r="J241" t="s">
         <v>1504</v>
       </c>
-      <c r="K241" s="2">
+      <c r="K241" s="1">
         <v>46149</v>
       </c>
       <c r="L241" t="s">
@@ -16954,7 +16928,7 @@
       <c r="J242" t="s">
         <v>1504</v>
       </c>
-      <c r="K242" s="2">
+      <c r="K242" s="1">
         <v>46149</v>
       </c>
       <c r="L242" t="s">
@@ -16972,7 +16946,7 @@
       <c r="R242" t="s">
         <v>1691</v>
       </c>
-      <c r="T242" s="2">
+      <c r="T242" s="1">
         <v>45805</v>
       </c>
       <c r="W242" t="s">
@@ -17007,7 +16981,7 @@
       <c r="J243" t="s">
         <v>1504</v>
       </c>
-      <c r="K243" s="2">
+      <c r="K243" s="1">
         <v>46149</v>
       </c>
       <c r="L243" t="s">
@@ -17048,7 +17022,7 @@
       <c r="J244" t="s">
         <v>1504</v>
       </c>
-      <c r="K244" s="2">
+      <c r="K244" s="1">
         <v>46149</v>
       </c>
       <c r="L244" t="s">
@@ -17089,7 +17063,7 @@
       <c r="J245" t="s">
         <v>1504</v>
       </c>
-      <c r="K245" s="2">
+      <c r="K245" s="1">
         <v>46149</v>
       </c>
       <c r="L245" t="s">
@@ -17130,7 +17104,7 @@
       <c r="J246" t="s">
         <v>1504</v>
       </c>
-      <c r="K246" s="2">
+      <c r="K246" s="1">
         <v>46149</v>
       </c>
       <c r="L246" t="s">
@@ -17148,7 +17122,7 @@
       <c r="R246" t="s">
         <v>1671</v>
       </c>
-      <c r="T246" s="2">
+      <c r="T246" s="1">
         <v>45979</v>
       </c>
       <c r="W246" t="s">
@@ -17183,7 +17157,7 @@
       <c r="J247" t="s">
         <v>1504</v>
       </c>
-      <c r="K247" s="2">
+      <c r="K247" s="1">
         <v>46149</v>
       </c>
       <c r="L247" t="s">
@@ -17224,7 +17198,7 @@
       <c r="J248" t="s">
         <v>1504</v>
       </c>
-      <c r="K248" s="2">
+      <c r="K248" s="1">
         <v>46149</v>
       </c>
       <c r="L248" t="s">
@@ -17265,7 +17239,7 @@
       <c r="J249" t="s">
         <v>1504</v>
       </c>
-      <c r="K249" s="2">
+      <c r="K249" s="1">
         <v>46150</v>
       </c>
       <c r="L249" t="s">
@@ -17306,7 +17280,7 @@
       <c r="J250" t="s">
         <v>1504</v>
       </c>
-      <c r="K250" s="2">
+      <c r="K250" s="1">
         <v>46155</v>
       </c>
       <c r="L250" t="s">
@@ -17347,7 +17321,7 @@
       <c r="J251" t="s">
         <v>1504</v>
       </c>
-      <c r="K251" s="2">
+      <c r="K251" s="1">
         <v>46161</v>
       </c>
       <c r="L251" t="s">
@@ -17388,7 +17362,7 @@
       <c r="J252" t="s">
         <v>1504</v>
       </c>
-      <c r="K252" s="2">
+      <c r="K252" s="1">
         <v>46161</v>
       </c>
       <c r="L252" t="s">
@@ -17429,7 +17403,7 @@
       <c r="J253" t="s">
         <v>1504</v>
       </c>
-      <c r="K253" s="2">
+      <c r="K253" s="1">
         <v>46162</v>
       </c>
       <c r="L253" t="s">
@@ -17447,7 +17421,7 @@
       <c r="R253" t="s">
         <v>1701</v>
       </c>
-      <c r="T253" s="2">
+      <c r="T253" s="1">
         <v>45817</v>
       </c>
       <c r="W253" t="s">
@@ -17485,7 +17459,7 @@
       <c r="J254" t="s">
         <v>1504</v>
       </c>
-      <c r="K254" s="2">
+      <c r="K254" s="1">
         <v>46162</v>
       </c>
       <c r="L254" t="s">
@@ -17526,7 +17500,7 @@
       <c r="J255" t="s">
         <v>1504</v>
       </c>
-      <c r="K255" s="2">
+      <c r="K255" s="1">
         <v>46163</v>
       </c>
       <c r="L255" t="s">
@@ -17567,7 +17541,7 @@
       <c r="J256" t="s">
         <v>1504</v>
       </c>
-      <c r="K256" s="2">
+      <c r="K256" s="1">
         <v>46163</v>
       </c>
       <c r="L256" t="s">
@@ -17576,7 +17550,7 @@
       <c r="M256" t="s">
         <v>1572</v>
       </c>
-      <c r="T256" s="2">
+      <c r="T256" s="1">
         <v>46176</v>
       </c>
       <c r="W256" t="s">
@@ -17614,7 +17588,7 @@
       <c r="J257" t="s">
         <v>1504</v>
       </c>
-      <c r="K257" s="2">
+      <c r="K257" s="1">
         <v>46170</v>
       </c>
       <c r="L257" t="s">
@@ -17623,7 +17597,7 @@
       <c r="M257" t="s">
         <v>1573</v>
       </c>
-      <c r="T257" s="2">
+      <c r="T257" s="1">
         <v>46176</v>
       </c>
       <c r="U257" t="s">
@@ -17667,7 +17641,7 @@
       <c r="J258" t="s">
         <v>1504</v>
       </c>
-      <c r="K258" s="2">
+      <c r="K258" s="1">
         <v>46170</v>
       </c>
       <c r="L258" t="s">
@@ -17685,7 +17659,7 @@
       <c r="R258" t="s">
         <v>1683</v>
       </c>
-      <c r="T258" s="2">
+      <c r="T258" s="1">
         <v>46230</v>
       </c>
       <c r="W258" t="s">
@@ -17723,7 +17697,7 @@
       <c r="J259" t="s">
         <v>1504</v>
       </c>
-      <c r="K259" s="2">
+      <c r="K259" s="1">
         <v>46171</v>
       </c>
       <c r="L259" t="s">
@@ -17741,7 +17715,7 @@
       <c r="R259" t="s">
         <v>1699</v>
       </c>
-      <c r="T259" s="2">
+      <c r="T259" s="1">
         <v>46176</v>
       </c>
       <c r="W259" t="s">
@@ -17779,7 +17753,7 @@
       <c r="J260" t="s">
         <v>1504</v>
       </c>
-      <c r="K260" s="2">
+      <c r="K260" s="1">
         <v>46171</v>
       </c>
       <c r="L260" t="s">
@@ -17788,7 +17762,7 @@
       <c r="M260" t="s">
         <v>1567</v>
       </c>
-      <c r="T260" s="2">
+      <c r="T260" s="1">
         <v>46176</v>
       </c>
       <c r="U260" t="s">
@@ -17832,7 +17806,7 @@
       <c r="J261" t="s">
         <v>1504</v>
       </c>
-      <c r="K261" s="2">
+      <c r="K261" s="1">
         <v>46171</v>
       </c>
       <c r="L261" t="s">
@@ -17850,7 +17824,7 @@
       <c r="R261" t="s">
         <v>1705</v>
       </c>
-      <c r="T261" s="2">
+      <c r="T261" s="1">
         <v>46094</v>
       </c>
       <c r="W261" t="s">
@@ -17888,7 +17862,7 @@
       <c r="J262" t="s">
         <v>1504</v>
       </c>
-      <c r="K262" s="2">
+      <c r="K262" s="1">
         <v>46171</v>
       </c>
       <c r="L262" t="s">
@@ -17906,7 +17880,7 @@
       <c r="R262" t="s">
         <v>1699</v>
       </c>
-      <c r="T262" s="2">
+      <c r="T262" s="1">
         <v>46176</v>
       </c>
       <c r="W262" t="s">
@@ -17944,7 +17918,7 @@
       <c r="J263" t="s">
         <v>1504</v>
       </c>
-      <c r="K263" s="2">
+      <c r="K263" s="1">
         <v>46171</v>
       </c>
       <c r="L263" t="s">
@@ -17953,7 +17927,7 @@
       <c r="M263" t="s">
         <v>1567</v>
       </c>
-      <c r="T263" s="2">
+      <c r="T263" s="1">
         <v>46176</v>
       </c>
       <c r="U263" t="s">
@@ -17997,7 +17971,7 @@
       <c r="J264" t="s">
         <v>1504</v>
       </c>
-      <c r="K264" s="2">
+      <c r="K264" s="1">
         <v>46174</v>
       </c>
       <c r="L264" t="s">
@@ -18038,7 +18012,7 @@
       <c r="J265" t="s">
         <v>1504</v>
       </c>
-      <c r="K265" s="2">
+      <c r="K265" s="1">
         <v>46174</v>
       </c>
       <c r="L265" t="s">
@@ -18079,7 +18053,7 @@
       <c r="J266" t="s">
         <v>1504</v>
       </c>
-      <c r="K266" s="2">
+      <c r="K266" s="1">
         <v>46174</v>
       </c>
       <c r="L266" t="s">
@@ -18120,7 +18094,7 @@
       <c r="J267" t="s">
         <v>1504</v>
       </c>
-      <c r="K267" s="2">
+      <c r="K267" s="1">
         <v>46174</v>
       </c>
       <c r="L267" t="s">
@@ -18164,7 +18138,7 @@
       <c r="J268" t="s">
         <v>1504</v>
       </c>
-      <c r="K268" s="2">
+      <c r="K268" s="1">
         <v>46174</v>
       </c>
       <c r="L268" t="s">
@@ -18205,7 +18179,7 @@
       <c r="J269" t="s">
         <v>1504</v>
       </c>
-      <c r="K269" s="2">
+      <c r="K269" s="1">
         <v>46174</v>
       </c>
       <c r="L269" t="s">
@@ -18246,7 +18220,7 @@
       <c r="J270" t="s">
         <v>1504</v>
       </c>
-      <c r="K270" s="2">
+      <c r="K270" s="1">
         <v>46174</v>
       </c>
       <c r="L270" t="s">
@@ -18287,7 +18261,7 @@
       <c r="J271" t="s">
         <v>1504</v>
       </c>
-      <c r="K271" s="2">
+      <c r="K271" s="1">
         <v>46174</v>
       </c>
       <c r="L271" t="s">
@@ -18328,7 +18302,7 @@
       <c r="J272" t="s">
         <v>1504</v>
       </c>
-      <c r="K272" s="2">
+      <c r="K272" s="1">
         <v>46174</v>
       </c>
       <c r="L272" t="s">
@@ -18346,7 +18320,7 @@
       <c r="R272" t="s">
         <v>1706</v>
       </c>
-      <c r="T272" s="2">
+      <c r="T272" s="1">
         <v>46168</v>
       </c>
       <c r="W272" t="s">
@@ -18384,7 +18358,7 @@
       <c r="J273" t="s">
         <v>1504</v>
       </c>
-      <c r="K273" s="2">
+      <c r="K273" s="1">
         <v>46174</v>
       </c>
       <c r="L273" t="s">
@@ -18428,7 +18402,7 @@
       <c r="J274" t="s">
         <v>1504</v>
       </c>
-      <c r="K274" s="2">
+      <c r="K274" s="1">
         <v>46174</v>
       </c>
       <c r="L274" t="s">
@@ -18469,7 +18443,7 @@
       <c r="J275" t="s">
         <v>1504</v>
       </c>
-      <c r="K275" s="2">
+      <c r="K275" s="1">
         <v>46174</v>
       </c>
       <c r="L275" t="s">
@@ -18510,7 +18484,7 @@
       <c r="J276" t="s">
         <v>1504</v>
       </c>
-      <c r="K276" s="2">
+      <c r="K276" s="1">
         <v>46174</v>
       </c>
       <c r="L276" t="s">
@@ -18551,7 +18525,7 @@
       <c r="J277" t="s">
         <v>1504</v>
       </c>
-      <c r="K277" s="2">
+      <c r="K277" s="1">
         <v>46174</v>
       </c>
       <c r="L277" t="s">
@@ -18592,7 +18566,7 @@
       <c r="J278" t="s">
         <v>1504</v>
       </c>
-      <c r="K278" s="2">
+      <c r="K278" s="1">
         <v>46174</v>
       </c>
       <c r="L278" t="s">
@@ -18633,7 +18607,7 @@
       <c r="J279" t="s">
         <v>1504</v>
       </c>
-      <c r="K279" s="2">
+      <c r="K279" s="1">
         <v>46174</v>
       </c>
       <c r="L279" t="s">
@@ -18674,7 +18648,7 @@
       <c r="J280" t="s">
         <v>1504</v>
       </c>
-      <c r="K280" s="2">
+      <c r="K280" s="1">
         <v>46174</v>
       </c>
       <c r="L280" t="s">
@@ -18715,7 +18689,7 @@
       <c r="J281" t="s">
         <v>1504</v>
       </c>
-      <c r="K281" s="2">
+      <c r="K281" s="1">
         <v>46174</v>
       </c>
       <c r="L281" t="s">
@@ -18756,7 +18730,7 @@
       <c r="J282" t="s">
         <v>1504</v>
       </c>
-      <c r="K282" s="2">
+      <c r="K282" s="1">
         <v>46174</v>
       </c>
       <c r="L282" t="s">
@@ -18797,7 +18771,7 @@
       <c r="J283" t="s">
         <v>1504</v>
       </c>
-      <c r="K283" s="2">
+      <c r="K283" s="1">
         <v>46174</v>
       </c>
       <c r="L283" t="s">
@@ -18838,7 +18812,7 @@
       <c r="J284" t="s">
         <v>1504</v>
       </c>
-      <c r="K284" s="2">
+      <c r="K284" s="1">
         <v>46174</v>
       </c>
       <c r="L284" t=